<commit_message>
Split other-business forecast periods
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -1265,13 +1265,13 @@
         <v>131.15</v>
       </c>
       <c r="H5" s="2">
-        <v>149.51999999999998</v>
+        <v>149.38</v>
       </c>
       <c r="I5" s="2">
-        <v>171.4</v>
+        <v>171.12</v>
       </c>
       <c r="J5" s="2">
-        <v>197.52</v>
+        <v>197.08</v>
       </c>
     </row>
     <row r="6">
@@ -1333,13 +1333,13 @@
         <v>67.59</v>
       </c>
       <c r="H7" s="4">
-        <v>77.57</v>
+        <v>77.70999999999998</v>
       </c>
       <c r="I7" s="4">
-        <v>89.46000000000001</v>
+        <v>89.74000000000001</v>
       </c>
       <c r="J7" s="4">
-        <v>103.63999999999996</v>
+        <v>104.07999999999996</v>
       </c>
     </row>
     <row r="8">
@@ -1367,13 +1367,13 @@
         <v>34.009258327463016</v>
       </c>
       <c r="H8" s="2">
-        <v>34.158263243647895</v>
+        <v>34.21991280989916</v>
       </c>
       <c r="I8" s="2">
-        <v>34.29425745610673</v>
+        <v>34.40159472513992</v>
       </c>
       <c r="J8" s="2">
-        <v>34.41360074379067</v>
+        <v>34.559702483729566</v>
       </c>
     </row>
     <row r="9">
@@ -1392,19 +1392,19 @@
         <v>36.5</v>
       </c>
       <c r="E9" s="2">
-        <v>28.43</v>
+        <v>28.419999999999998</v>
       </c>
       <c r="F9" s="2">
-        <v>38.800000000000004</v>
+        <v>38.78</v>
       </c>
       <c r="G9" s="2">
-        <v>49.17</v>
+        <v>49.15</v>
       </c>
       <c r="H9" s="2">
-        <v>53.1</v>
+        <v>53.08</v>
       </c>
       <c r="I9" s="2">
-        <v>57.48</v>
+        <v>57.47</v>
       </c>
       <c r="J9" s="2">
         <v>62.43</v>
@@ -1698,22 +1698,22 @@
         <v>11.5</v>
       </c>
       <c r="E18" s="4">
-        <v>8.990000000000002</v>
+        <v>9.000000000000004</v>
       </c>
       <c r="F18" s="4">
-        <v>13.679999999999993</v>
+        <v>13.699999999999996</v>
       </c>
       <c r="G18" s="4">
-        <v>18.42</v>
+        <v>18.440000000000005</v>
       </c>
       <c r="H18" s="4">
-        <v>24.469999999999985</v>
+        <v>24.629999999999974</v>
       </c>
       <c r="I18" s="4">
-        <v>31.980000000000004</v>
+        <v>32.27</v>
       </c>
       <c r="J18" s="4">
-        <v>41.20999999999996</v>
+        <v>41.649999999999956</v>
       </c>
     </row>
     <row r="19">
@@ -1732,22 +1732,22 @@
         <v>7.666666666666666</v>
       </c>
       <c r="E19" s="2">
-        <v>7.969858156028371</v>
+        <v>7.978723404255322</v>
       </c>
       <c r="F19" s="2">
-        <v>8.785562905401061</v>
+        <v>8.79840729561364</v>
       </c>
       <c r="G19" s="2">
-        <v>9.26839086243333</v>
+        <v>9.278454261849655</v>
       </c>
       <c r="H19" s="2">
-        <v>10.77546347263199</v>
+        <v>10.84592011977629</v>
       </c>
       <c r="I19" s="2">
-        <v>12.259449513148816</v>
+        <v>12.370620256076057</v>
       </c>
       <c r="J19" s="2">
-        <v>13.683756142914053</v>
+        <v>13.829857882852956</v>
       </c>
     </row>
     <row r="20">
@@ -1766,22 +1766,22 @@
         <v>11.5</v>
       </c>
       <c r="E20" s="4">
-        <v>8.990000000000002</v>
+        <v>9.000000000000004</v>
       </c>
       <c r="F20" s="4">
-        <v>13.679999999999993</v>
+        <v>13.699999999999996</v>
       </c>
       <c r="G20" s="4">
-        <v>18.42</v>
+        <v>18.440000000000005</v>
       </c>
       <c r="H20" s="4">
-        <v>24.469999999999985</v>
+        <v>24.629999999999974</v>
       </c>
       <c r="I20" s="4">
-        <v>31.980000000000004</v>
+        <v>32.27</v>
       </c>
       <c r="J20" s="4">
-        <v>41.20999999999996</v>
+        <v>41.649999999999956</v>
       </c>
     </row>
   </sheetData>
@@ -2959,17 +2959,17 @@
       </c>
       <c r="J5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 65.84 % / 補助 65 % / 他 67.33 %</t>
+          <t xml:space="preserve">全社 65.78 % / 補助 65 % / 他 67.16 %</t>
         </is>
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 65.71 % / 補助 65 % / 他 67.16 %</t>
+          <t xml:space="preserve">全社 65.6 % / 補助 65 % / 他 66.83 %</t>
         </is>
       </c>
       <c r="L5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 65.59 % / 補助 65 % / 他 67 %</t>
+          <t xml:space="preserve">全社 65.44 % / 補助 65 % / 他 66.5 %</t>
         </is>
       </c>
     </row>
@@ -3021,17 +3021,17 @@
       </c>
       <c r="J6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 34.16 % / 補助 35 % / 他 32.67 %</t>
+          <t xml:space="preserve">全社 34.22 % / 補助 35 % / 他 32.84 %</t>
         </is>
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 34.29 % / 補助 35 % / 他 32.84 %</t>
+          <t xml:space="preserve">全社 34.4 % / 補助 35 % / 他 33.17 %</t>
         </is>
       </c>
       <c r="L6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 34.41 % / 補助 35 % / 他 33 %</t>
+          <t xml:space="preserve">全社 34.56 % / 補助 35 % / 他 33.5 %</t>
         </is>
       </c>
     </row>
@@ -3068,27 +3068,27 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 25.2 % / 補助 24.25 % / 他 25.73 %</t>
+          <t xml:space="preserve">全社 25.2 % / 補助 24.25 % / 他 25.71 %</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.92 % / 補助 24.25 % / 他 25.62 %</t>
+          <t xml:space="preserve">全社 24.91 % / 補助 24.25 % / 他 25.6 %</t>
         </is>
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.74 % / 補助 24.25 % / 他 25.49 %</t>
+          <t xml:space="preserve">全社 24.73 % / 補助 24.25 % / 他 25.46 %</t>
         </is>
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 23.38 % / 補助 22.25 % / 他 25.39 %</t>
+          <t xml:space="preserve">全社 23.37 % / 補助 22.25 % / 他 25.36 %</t>
         </is>
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 22.03 % / 補助 20.46 % / 他 25.28 %</t>
+          <t xml:space="preserve">全社 22.03 % / 補助 20.46 % / 他 25.27 %</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
@@ -3130,32 +3130,32 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.97 % / 補助 10.75 % / 他 6.44 %</t>
+          <t xml:space="preserve">全社 7.98 % / 補助 10.75 % / 他 6.46 %</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.79 % / 補助 10.75 % / 他 6.71 %</t>
+          <t xml:space="preserve">全社 8.8 % / 補助 10.75 % / 他 6.74 %</t>
         </is>
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.27 % / 補助 10.75 % / 他 7.01 %</t>
+          <t xml:space="preserve">全社 9.28 % / 補助 10.75 % / 他 7.04 %</t>
         </is>
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.78 % / 補助 12.75 % / 他 7.28 %</t>
+          <t xml:space="preserve">全社 10.85 % / 補助 12.75 % / 他 7.47 %</t>
         </is>
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.26 % / 補助 14.54 % / 他 7.56 %</t>
+          <t xml:space="preserve">全社 12.37 % / 補助 14.54 % / 他 7.9 %</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.68 % / 補助 16.13 % / 他 7.81 %</t>
+          <t xml:space="preserve">全社 13.83 % / 補助 16.13 % / 他 8.31 %</t>
         </is>
       </c>
     </row>
@@ -3192,32 +3192,32 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.22 % / 補助 16.18 % / 他 8.5 %</t>
+          <t xml:space="preserve">全社 11.23 % / 補助 16.18 % / 他 8.52 %</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.53 % / 補助 16.16 % / 他 8.69 %</t>
+          <t xml:space="preserve">全社 12.54 % / 補助 16.16 % / 他 8.72 %</t>
         </is>
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.29 % / 補助 16.17 % / 他 8.92 %</t>
+          <t xml:space="preserve">全社 13.3 % / 補助 16.17 % / 他 8.94 %</t>
         </is>
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 14.3 % / 補助 17.22 % / 他 9.11 %</t>
+          <t xml:space="preserve">全社 14.37 % / 補助 17.22 % / 他 9.31 %</t>
         </is>
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.33 % / 補助 18.24 % / 他 9.32 %</t>
+          <t xml:space="preserve">全社 15.44 % / 補助 18.24 % / 他 9.66 %</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 16.34 % / 補助 19.19 % / 他 9.51 %</t>
+          <t xml:space="preserve">全社 16.49 % / 補助 19.19 % / 他 10 %</t>
         </is>
       </c>
     </row>
@@ -3254,27 +3254,27 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.82 % / 補助 10 % / 他 11.28 %</t>
+          <t xml:space="preserve">全社 10.82 % / 補助 10 % / 他 11.26 %</t>
         </is>
       </c>
       <c r="H10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.55 % / 補助 10 % / 他 11.12 %</t>
+          <t xml:space="preserve">全社 10.53 % / 補助 10 % / 他 11.09 %</t>
         </is>
       </c>
       <c r="I10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.38 % / 補助 10 % / 他 10.96 %</t>
+          <t xml:space="preserve">全社 10.37 % / 補助 10 % / 他 10.93 %</t>
         </is>
       </c>
       <c r="J10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.08 % / 補助 9.67 % / 他 10.81 %</t>
+          <t xml:space="preserve">全社 10.07 % / 補助 9.67 % / 他 10.78 %</t>
         </is>
       </c>
       <c r="K10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.76 % / 補助 9.33 % / 他 10.65 %</t>
+          <t xml:space="preserve">全社 9.76 % / 補助 9.33 % / 他 10.64 %</t>
         </is>
       </c>
       <c r="L10" s="0" t="inlineStr">
@@ -3750,32 +3750,32 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 49.78 % / 補助 35.3 % / 他 59.3 %</t>
+          <t xml:space="preserve">全社 49.76 % / 補助 35.3 % / 他 59.26 %</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 45.9 % / 補助 35.35 % / 他 59.03 %</t>
+          <t xml:space="preserve">全社 45.87 % / 補助 35.35 % / 他 58.96 %</t>
         </is>
       </c>
       <c r="I18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 43.74 % / 補助 35.33 % / 他 58.61 %</t>
+          <t xml:space="preserve">全社 43.72 % / 補助 35.33 % / 他 58.54 %</t>
         </is>
       </c>
       <c r="J18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 40.62 % / 補助 32 % / 他 58.32 %</t>
+          <t xml:space="preserve">全社 40.5 % / 補助 32 % / 他 57.81 %</t>
         </is>
       </c>
       <c r="K18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 37.52 % / 補助 28.94 % / 他 57.99 %</t>
+          <t xml:space="preserve">全社 37.35 % / 補助 28.94 % / 他 57.11 %</t>
         </is>
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 34.57 % / 補助 26.21 % / 他 57.75 %</t>
+          <t xml:space="preserve">全社 34.37 % / 補助 26.21 % / 他 56.5 %</t>
         </is>
       </c>
     </row>
@@ -3951,17 +3951,17 @@
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.096 億円/人 / 補助 0.155 億円/人 / 他 0.044 億円/人</t>
+          <t xml:space="preserve">全社 0.097 億円/人 / 補助 0.155 億円/人 / 他 0.045 億円/人</t>
         </is>
       </c>
       <c r="K21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.123 億円/人 / 補助 0.205 億円/人 / 他 0.047 億円/人</t>
+          <t xml:space="preserve">全社 0.124 億円/人 / 補助 0.205 億円/人 / 他 0.049 億円/人</t>
         </is>
       </c>
       <c r="L21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.154 億円/人 / 補助 0.265 億円/人 / 他 0.05 億円/人</t>
+          <t xml:space="preserve">全社 0.156 億円/人 / 補助 0.265 億円/人 / 他 0.053 億円/人</t>
         </is>
       </c>
     </row>
@@ -4003,7 +4003,7 @@
       </c>
       <c r="H22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.168 億円/人 / 補助 0.254 億円/人 / 他 0.118 億円/人</t>
+          <t xml:space="preserve">全社 0.168 億円/人 / 補助 0.254 億円/人 / 他 0.119 億円/人</t>
         </is>
       </c>
       <c r="I22" s="0" t="inlineStr">
@@ -4013,17 +4013,17 @@
       </c>
       <c r="J22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.21 億円/人 / 補助 0.302 億円/人 / 他 0.129 億円/人</t>
+          <t xml:space="preserve">全社 0.211 億円/人 / 補助 0.302 億円/人 / 他 0.131 億円/人</t>
         </is>
       </c>
       <c r="K22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.241 億円/人 / 補助 0.357 億円/人 / 他 0.135 億円/人</t>
+          <t xml:space="preserve">全社 0.242 億円/人 / 補助 0.357 億円/人 / 他 0.137 億円/人</t>
         </is>
       </c>
       <c r="L22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.276 億円/人 / 補助 0.421 億円/人 / 他 0.141 億円/人</t>
+          <t xml:space="preserve">全社 0.278 億円/人 / 補助 0.421 億円/人 / 他 0.144 億円/人</t>
         </is>
       </c>
     </row>
@@ -4437,27 +4437,27 @@
       </c>
       <c r="H29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.35 倍 / 補助 2.99 倍 / 他 4.39 倍</t>
+          <t xml:space="preserve">全社 3.35 倍 / 補助 2.99 倍 / 他 4.4 倍</t>
         </is>
       </c>
       <c r="I29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.3 倍 / 補助 2.98 倍 / 他 4.68 倍</t>
+          <t xml:space="preserve">全社 3.31 倍 / 補助 2.98 倍 / 他 4.69 倍</t>
         </is>
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.06 倍 / 補助 3.85 倍 / 他 4.97 倍</t>
+          <t xml:space="preserve">全社 4.08 倍 / 補助 3.85 倍 / 他 5.08 倍</t>
         </is>
       </c>
       <c r="K29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5 倍 / 補助 4.93 倍 / 他 5.29 倍</t>
+          <t xml:space="preserve">全社 5.03 倍 / 補助 4.93 倍 / 他 5.49 倍</t>
         </is>
       </c>
       <c r="L29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.15 倍 / 補助 6.28 倍 / 他 5.61 倍</t>
+          <t xml:space="preserve">全社 6.21 倍 / 補助 6.28 倍 / 他 5.91 倍</t>
         </is>
       </c>
     </row>
@@ -4757,17 +4757,17 @@
       </c>
       <c r="J34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -2.33 pt</t>
+          <t xml:space="preserve">差 -2.16 pt</t>
         </is>
       </c>
       <c r="K34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -2.16 pt</t>
+          <t xml:space="preserve">差 -1.83 pt</t>
         </is>
       </c>
       <c r="L34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -2 pt</t>
+          <t xml:space="preserve">差 -1.5 pt</t>
         </is>
       </c>
     </row>
@@ -4804,32 +4804,32 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 4.31 pt</t>
+          <t xml:space="preserve">差 4.29 pt</t>
         </is>
       </c>
       <c r="H35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 4.04 pt</t>
+          <t xml:space="preserve">差 4.01 pt</t>
         </is>
       </c>
       <c r="I35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 3.74 pt</t>
+          <t xml:space="preserve">差 3.71 pt</t>
         </is>
       </c>
       <c r="J35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 5.47 pt</t>
+          <t xml:space="preserve">差 5.27 pt</t>
         </is>
       </c>
       <c r="K35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 6.98 pt</t>
+          <t xml:space="preserve">差 6.64 pt</t>
         </is>
       </c>
       <c r="L35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 8.32 pt</t>
+          <t xml:space="preserve">差 7.82 pt</t>
         </is>
       </c>
     </row>
@@ -4990,12 +4990,12 @@
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 115.54 %</t>
+          <t xml:space="preserve">寄与率 116 %</t>
         </is>
       </c>
       <c r="H38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 91.68 %</t>
+          <t xml:space="preserve">寄与率 91.49 %</t>
         </is>
       </c>
       <c r="I38" s="0" t="inlineStr">
@@ -5005,17 +5005,17 @@
       </c>
       <c r="J38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 92.73 %</t>
+          <t xml:space="preserve">寄与率 90.63 %</t>
         </is>
       </c>
       <c r="K38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 93.61 %</t>
+          <t xml:space="preserve">寄与率 92.02 %</t>
         </is>
       </c>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 94.8 %</t>
+          <t xml:space="preserve">寄与率 93.28 %</t>
         </is>
       </c>
     </row>
@@ -5025,7 +5025,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="68" customWidth="1"/>
@@ -5193,110 +5193,110 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 売上成長率（基準年度後）</t>
+          <t xml:space="preserve">その他事業 売上成長率（設備導入期間）</t>
         </is>
       </c>
       <c r="B10" s="2">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="C10" s="2">
-        <v>-5</v>
+        <v>-10</v>
       </c>
       <c r="D10" s="2">
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">その他事業 売上成長率</t>
+          <t xml:space="preserve">その他事業 原価率改善ポイント（設備導入期間）</t>
         </is>
       </c>
       <c r="B11" s="2">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="C11" s="2">
-        <v>-10</v>
+        <v>-15</v>
       </c>
       <c r="D11" s="2">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 原価率改善ポイント（基準年度後）</t>
+          <t xml:space="preserve">その他事業1人当たり給与支給総額の年平均上昇率（設備導入期間）</t>
         </is>
       </c>
       <c r="B12" s="2">
+        <v>4</v>
+      </c>
+      <c r="C12" s="2">
         <v>0</v>
       </c>
-      <c r="C12" s="2">
-        <v>-15</v>
-      </c>
       <c r="D12" s="2">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">その他事業 原価率改善ポイント</t>
+          <t xml:space="preserve">その他事業 常時使用する従業員数の成長率（設備導入期間）</t>
         </is>
       </c>
       <c r="B13" s="2">
         <v>1</v>
       </c>
       <c r="C13" s="2">
-        <v>-15</v>
+        <v>-5</v>
       </c>
       <c r="D13" s="2">
-        <v>25</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業1人当たり給与支給総額の年平均上昇率</t>
+          <t xml:space="preserve">その他事業 その他販管費率改善ポイント（設備導入期間）</t>
         </is>
       </c>
       <c r="B14" s="2">
-        <v>7.000000000000001</v>
+        <v>0.5</v>
       </c>
       <c r="C14" s="2">
-        <v>4.5</v>
+        <v>-15</v>
       </c>
       <c r="D14" s="2">
-        <v>10</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">その他事業1人当たり給与支給総額の年平均上昇率</t>
+          <t xml:space="preserve">補助事業 売上成長率（基準年度後）</t>
         </is>
       </c>
       <c r="B15" s="2">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="C15" s="2">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="D15" s="2">
-        <v>8</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 常時使用する従業員数の成長率</t>
+          <t xml:space="preserve">その他事業 売上成長率（基準年度後）</t>
         </is>
       </c>
       <c r="B16" s="2">
         <v>4</v>
       </c>
       <c r="C16" s="2">
-        <v>-3</v>
+        <v>-10</v>
       </c>
       <c r="D16" s="2">
         <v>20</v>
@@ -5305,30 +5305,30 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">その他事業 常時使用する従業員数の成長率</t>
+          <t xml:space="preserve">補助事業 原価率改善ポイント（基準年度後）</t>
         </is>
       </c>
       <c r="B17" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C17" s="2">
-        <v>-5</v>
+        <v>-15</v>
       </c>
       <c r="D17" s="2">
-        <v>10</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 その他販管費率（事業化報告3年目）</t>
+          <t xml:space="preserve">その他事業 原価率改善ポイント（基準年度後）</t>
         </is>
       </c>
       <c r="B18" s="2">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C18" s="2">
-        <v>4</v>
+        <v>-15</v>
       </c>
       <c r="D18" s="2">
         <v>25</v>
@@ -5337,104 +5337,184 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">その他事業 その他販管費率（事業化報告3年目）</t>
+          <t xml:space="preserve">補助事業1人当たり給与支給総額の年平均上昇率</t>
         </is>
       </c>
       <c r="B19" s="2">
-        <v>10.5</v>
+        <v>7.000000000000001</v>
       </c>
       <c r="C19" s="2">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="D19" s="2">
-        <v>25</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">役員1人当たり給与支給総額の年平均上昇率</t>
+          <t xml:space="preserve">その他事業1人当たり給与支給総額の年平均上昇率（基準年度後）</t>
         </is>
       </c>
       <c r="B20" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C20" s="2">
         <v>0</v>
       </c>
       <c r="D20" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">新規投資の耐用年数</t>
+          <t xml:space="preserve">補助事業 常時使用する従業員数の成長率</t>
         </is>
       </c>
       <c r="B21" s="2">
-        <v>10</v>
-      </c>
-      <c r="C21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+        <v>4</v>
+      </c>
+      <c r="C21" s="2">
+        <v>-3</v>
+      </c>
+      <c r="D21" s="2">
+        <v>20</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業投資額</t>
+          <t xml:space="preserve">その他事業 常時使用する従業員数の成長率（基準年度後）</t>
         </is>
       </c>
       <c r="B22" s="2">
-        <v>45</v>
-      </c>
-      <c r="C22" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D22" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="C22" s="2">
+        <v>-5</v>
+      </c>
+      <c r="D22" s="2">
+        <v>10</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">申請補助金額</t>
+          <t xml:space="preserve">補助事業 その他販管費率（事業化報告3年目）</t>
         </is>
       </c>
       <c r="B23" s="2">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C23" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D23" s="2">
-        <v>50</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">その他事業 その他販管費率（事業化報告3年目）</t>
+        </is>
+      </c>
+      <c r="B24" s="2">
+        <v>10.5</v>
+      </c>
+      <c r="C24" s="2">
+        <v>4</v>
+      </c>
+      <c r="D24" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">役員1人当たり給与支給総額の年平均上昇率</t>
+        </is>
+      </c>
+      <c r="B25" s="2">
+        <v>6</v>
+      </c>
+      <c r="C25" s="2">
+        <v>0</v>
+      </c>
+      <c r="D25" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">新規投資の耐用年数</t>
+        </is>
+      </c>
+      <c r="B26" s="2">
+        <v>10</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">補助事業投資額</t>
+        </is>
+      </c>
+      <c r="B27" s="2">
+        <v>45</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">申請補助金額</t>
+        </is>
+      </c>
+      <c r="B28" s="2">
+        <v>15</v>
+      </c>
+      <c r="C28" s="2">
+        <v>1</v>
+      </c>
+      <c r="D28" s="2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">ローカルベンチマーク</t>
         </is>
       </c>
-      <c r="B24" s="2">
+      <c r="B29" s="2">
         <v>23</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C29" s="2">
         <v>0</v>
       </c>
-      <c r="D24" s="2">
+      <c r="D29" s="2">
         <v>100</v>
       </c>
     </row>
@@ -5460,7 +5540,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjQsIm9mZmljZXJQYXkiOjAuMzYsImRlcHJlY2lhdGlvbiI6MS44LCJvdGhlclNnYSI6OSwiaGVhZGNvdW50Ijo5MCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4zNiwib2ZmaWNlclBheSI6MC41NSwiZGVwcmVjaWF0aW9uIjoxLjM4LCJvdGhlclNnYSI6Ny4zNiwiaGVhZGNvdW50IjoxMTkuNiwib2ZmaWNlckNvdW50IjozfX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjcsIm9mZmljZXJQYXkiOjAuMzgsImRlcHJlY2lhdGlvbiI6MS45LCJvdGhlclNnYSI6OS41LCJoZWFkY291bnQiOjk1LCJvZmZpY2VyQ291bnQiOjJ9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNjgsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI0LjgsIm9mZmljZXJDb3VudCI6M319LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6Niwib2ZmaWNlclBheSI6MC40LCJkZXByZWNpYXRpb24iOjIsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsIm9mZmljZXJQYXkiOjAuNiwiZGVwcmVjaWF0aW9uIjoxLjUsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjIxLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjowLjA3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjA3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAuMDEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA2LCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjEsIm90aGVyU2FsZXNHcm93dGgiOjAuMDQsInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAsIm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAxLCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJvdGhlclBheUdyb3d0aCI6MC4wNCwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDEsInByb2plY3RTZ2FSYXRlRW5kIjowLjA5LCJvdGhlclNnYVJhdGVFbmQiOjAuMTA1LCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNiwidXNlZnVsTGlmZSI6MTAsImludmVzdG1lbnQiOjQ1LCJzdWJzaWR5IjoxNSwibG9jYWxCZW5jaG1hcmsiOjIzfSwiZHJpdmVyUmFuZ2VzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOlstMC4wNSwwLjNdLCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOlstMC4wNSwwLjRdLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjpbLTAuMTUsMC4yNV0sInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOlstMC4wNSwwLjFdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbLTAuMDMsMC4yXSwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjpbLTAuMTUsMC4yNV0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjFdLCJwcm9qZWN0U2FsZXNHcm93dGgiOlstMC4wNSwwLjRdLCJvdGhlclNhbGVzR3Jvd3RoIjpbLTAuMSwwLjJdLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjpbLTAuMTUsMC4yNV0sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbLTAuMTUsMC4yNV0sInByb2plY3RQYXlHcm93dGgiOlswLjA0NSwwLjFdLCJvdGhlclBheUdyb3d0aCI6WzAsMC4wOF0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlstMC4wMywwLjJdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6Wy0wLjA1LDAuMV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMC4wNCwwLjI1XSwib3RoZXJTZ2FSYXRlRW5kIjpbMC4wNCwwLjI1XSwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOlswLDAuMV0sInVzZWZ1bExpZmUiOls1LDIwXSwiaW52ZXN0bWVudCI6WzE1LDIwMF0sInN1YnNpZHkiOlsxLDUwXSwibG9jYWxCZW5jaG1hcmsiOlswLDEwMF19LCJ0YXJnZXRzIjp7ImNvbXBhbnlTYWxlc0NhZ3IiOnsidmFsdWUiOjIxLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjgyLjQsIm1heCI6MTUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjozLjUsIm1heCI6NywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc1NoYXJlIjp7InZhbHVlIjo3MCwibWF4Ijo5NSwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0NhZ3IiOnsidmFsdWUiOjIyLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjc0LjgsIm1heCI6MTUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MjguMSwibWF4Ijo1MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5Q2FnciI6eyJ2YWx1ZSI6NywibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5SW5jcmVhc2UiOnsidmFsdWUiOjMuOSwibWF4Ijo3LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUNhZ3IiOnsidmFsdWUiOjYsIm1heCI6MTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAuMSwibWF4IjowLjIsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJpbnZlc3RtZW50U2FsZXNSYXRpbyI6eyJ2YWx1ZSI6MzAsIm1heCI6NzAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvIjp7InZhbHVlIjoyMTMsIm1heCI6MzUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibG9jYWxCZW5jaG1hcmsiOnsidmFsdWUiOjIzLCJtYXgiOjQwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfX0sImZvcmVjYXN0T3ZlcnJpZGVzIjp7fSwiZnV0dXJlSW5wdXRCYXNpcyI6Im90aGVyIn0=</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjQsIm9mZmljZXJQYXkiOjAuMzYsImRlcHJlY2lhdGlvbiI6MS44LCJvdGhlclNnYSI6OSwiaGVhZGNvdW50Ijo5MCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4zNiwib2ZmaWNlclBheSI6MC41NSwiZGVwcmVjaWF0aW9uIjoxLjM4LCJvdGhlclNnYSI6Ny4zNiwiaGVhZGNvdW50IjoxMTkuNiwib2ZmaWNlckNvdW50IjozfX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjcsIm9mZmljZXJQYXkiOjAuMzgsImRlcHJlY2lhdGlvbiI6MS45LCJvdGhlclNnYSI6OS41LCJoZWFkY291bnQiOjk1LCJvZmZpY2VyQ291bnQiOjJ9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNjgsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI0LjgsIm9mZmljZXJDb3VudCI6M319LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6Niwib2ZmaWNlclBheSI6MC40LCJkZXByZWNpYXRpb24iOjIsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsIm9mZmljZXJQYXkiOjAuNiwiZGVwcmVjaWF0aW9uIjoxLjUsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjIxLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjowLjA3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjA3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAuMDEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA2LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wMSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMSwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNCwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MCwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDEsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjA0LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wMSwicHJvamVjdFNnYVJhdGVFbmQiOjAuMDksIm90aGVyU2dhUmF0ZUVuZCI6MC4xMDUsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA2LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6NDUsInN1YnNpZHkiOjE1LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6Wy0wLjA1LDAuNF0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlstMC4xNSwwLjI1XSwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6Wy0wLjA1LDAuMV0sInByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOlstMC4wMywwLjJdLCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlstMC4xNSwwLjI1XSwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOlswLDAuMV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlstMC4xLDAuMl0sIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjpbLTAuMTUsMC4yNV0sIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlstMC4wNSwwLjFdLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbLTAuMTUsMC4yNV0sInByb2plY3RTYWxlc0dyb3d0aCI6Wy0wLjA1LDAuNF0sIm90aGVyU2FsZXNHcm93dGgiOlstMC4xLDAuMl0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOlstMC4xNSwwLjI1XSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOlstMC4xNSwwLjI1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDQ1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMCwwLjA4XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6Wy0wLjAzLDAuMl0sIm90aGVySGVhZGNvdW50R3Jvd3RoIjpbLTAuMDUsMC4xXSwicHJvamVjdFNnYVJhdGVFbmQiOlswLjA0LDAuMjVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA0LDAuMjVdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAsMC4xXSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjEsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6ODIuNCwibWF4IjoxNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55UGF5U2NoZWR1bGUiOnsidmFsdWUiOjMuNSwibWF4Ijo3LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzU2hhcmUiOnsidmFsdWUiOjcwLCJtYXgiOjk1LCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjIsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6NzQuOCwibWF4IjoxNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsYWJvclByb2R1Y3Rpdml0eUNhZ3IiOnsidmFsdWUiOjIxLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZEluY3JlYXNlIjp7InZhbHVlIjoyOC4xLCJtYXgiOjUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6My45LCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MC4xLCJtYXgiOjAuMiwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjozMCwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnt9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIifQ==</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add synergy lift to post-base defaults
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -191,7 +191,7 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <v>14.860490791493142</v>
+        <v>15.187557062867052</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -217,7 +217,7 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <v>102.41999999999996</v>
+        <v>105</v>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
@@ -269,7 +269,7 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <v>70.59038384911676</v>
+        <v>69.99078158951735</v>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
@@ -1195,13 +1195,13 @@
         <v>198.74</v>
       </c>
       <c r="H3" s="4">
-        <v>227.08999999999997</v>
+        <v>227.88</v>
       </c>
       <c r="I3" s="4">
-        <v>260.86</v>
+        <v>262.5</v>
       </c>
       <c r="J3" s="4">
-        <v>301.15999999999997</v>
+        <v>303.74</v>
       </c>
     </row>
     <row r="4">
@@ -1231,13 +1231,13 @@
         <v>27.63470554235441</v>
       </c>
       <c r="H4" s="2">
-        <v>14.26486867263761</v>
+        <v>14.66237294958237</v>
       </c>
       <c r="I4" s="2">
-        <v>14.870756087894677</v>
+        <v>15.192206424433907</v>
       </c>
       <c r="J4" s="2">
-        <v>15.4488997929924</v>
+        <v>15.710476190476186</v>
       </c>
     </row>
     <row r="5">
@@ -1265,13 +1265,13 @@
         <v>131.15</v>
       </c>
       <c r="H5" s="2">
-        <v>149.38</v>
+        <v>149.91</v>
       </c>
       <c r="I5" s="2">
-        <v>171.12</v>
+        <v>172.22</v>
       </c>
       <c r="J5" s="2">
-        <v>197.08</v>
+        <v>198.8</v>
       </c>
     </row>
     <row r="6">
@@ -1333,13 +1333,13 @@
         <v>67.59</v>
       </c>
       <c r="H7" s="4">
-        <v>77.70999999999998</v>
+        <v>77.97</v>
       </c>
       <c r="I7" s="4">
-        <v>89.74000000000001</v>
+        <v>90.28</v>
       </c>
       <c r="J7" s="4">
-        <v>104.07999999999996</v>
+        <v>104.94</v>
       </c>
     </row>
     <row r="8">
@@ -1367,13 +1367,13 @@
         <v>34.009258327463016</v>
       </c>
       <c r="H8" s="2">
-        <v>34.21991280989916</v>
+        <v>34.215376513954716</v>
       </c>
       <c r="I8" s="2">
-        <v>34.40159472513992</v>
+        <v>34.392380952380954</v>
       </c>
       <c r="J8" s="2">
-        <v>34.559702483729566</v>
+        <v>34.549285573187596</v>
       </c>
     </row>
     <row r="9">
@@ -1401,13 +1401,13 @@
         <v>49.15</v>
       </c>
       <c r="H9" s="2">
-        <v>53.08</v>
+        <v>53.13</v>
       </c>
       <c r="I9" s="2">
-        <v>57.47</v>
+        <v>57.56999999999999</v>
       </c>
       <c r="J9" s="2">
-        <v>62.43</v>
+        <v>62.57</v>
       </c>
     </row>
     <row r="10">
@@ -1435,13 +1435,13 @@
         <v>1.27</v>
       </c>
       <c r="H10" s="2">
-        <v>1.3399999999999999</v>
+        <v>1.35</v>
       </c>
       <c r="I10" s="2">
-        <v>1.4</v>
+        <v>1.4100000000000001</v>
       </c>
       <c r="J10" s="2">
-        <v>1.47</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="11">
@@ -1469,13 +1469,13 @@
         <v>1.27</v>
       </c>
       <c r="H11" s="2">
-        <v>1.3399999999999999</v>
+        <v>1.35</v>
       </c>
       <c r="I11" s="2">
-        <v>1.4</v>
+        <v>1.4100000000000001</v>
       </c>
       <c r="J11" s="2">
-        <v>1.47</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="12">
@@ -1537,13 +1537,13 @@
         <v>19.27</v>
       </c>
       <c r="H13" s="2">
-        <v>20.87</v>
+        <v>20.96</v>
       </c>
       <c r="I13" s="2">
-        <v>22.61</v>
+        <v>22.810000000000002</v>
       </c>
       <c r="J13" s="2">
-        <v>24.53</v>
+        <v>24.84</v>
       </c>
     </row>
     <row r="14">
@@ -1571,13 +1571,13 @@
         <v>19.27</v>
       </c>
       <c r="H14" s="2">
-        <v>20.87</v>
+        <v>20.96</v>
       </c>
       <c r="I14" s="2">
-        <v>22.61</v>
+        <v>22.810000000000002</v>
       </c>
       <c r="J14" s="2">
-        <v>24.53</v>
+        <v>24.84</v>
       </c>
     </row>
     <row r="15">
@@ -1707,13 +1707,13 @@
         <v>18.440000000000005</v>
       </c>
       <c r="H18" s="4">
-        <v>24.629999999999974</v>
+        <v>24.839999999999996</v>
       </c>
       <c r="I18" s="4">
-        <v>32.27</v>
+        <v>32.71000000000001</v>
       </c>
       <c r="J18" s="4">
-        <v>41.649999999999956</v>
+        <v>42.36999999999999</v>
       </c>
     </row>
     <row r="19">
@@ -1741,13 +1741,13 @@
         <v>9.278454261849655</v>
       </c>
       <c r="H19" s="2">
-        <v>10.84592011977629</v>
+        <v>10.900473933649288</v>
       </c>
       <c r="I19" s="2">
-        <v>12.370620256076057</v>
+        <v>12.460952380952383</v>
       </c>
       <c r="J19" s="2">
-        <v>13.829857882852956</v>
+        <v>13.949430433923746</v>
       </c>
     </row>
     <row r="20">
@@ -1775,13 +1775,13 @@
         <v>18.440000000000005</v>
       </c>
       <c r="H20" s="4">
-        <v>24.629999999999974</v>
+        <v>24.839999999999996</v>
       </c>
       <c r="I20" s="4">
-        <v>32.27</v>
+        <v>32.71000000000001</v>
       </c>
       <c r="J20" s="4">
-        <v>41.649999999999956</v>
+        <v>42.36999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2013,13 +2013,13 @@
         <v>60.38039649793701</v>
       </c>
       <c r="H5" s="2">
-        <v>63.93940728345589</v>
+        <v>63.717746182201154</v>
       </c>
       <c r="I5" s="2">
-        <v>67.35030284443762</v>
+        <v>66.9295238095238</v>
       </c>
       <c r="J5" s="2">
-        <v>70.59038384911676</v>
+        <v>69.99078158951735</v>
       </c>
     </row>
     <row r="6">
@@ -2897,17 +2897,17 @@
       </c>
       <c r="J4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 14.26 % / 補助 21 % / 他 4 %</t>
+          <t xml:space="preserve">全社 14.66 % / 補助 21 % / 他 5 %</t>
         </is>
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 14.87 % / 補助 21 % / 他 4.01 %</t>
+          <t xml:space="preserve">全社 15.19 % / 補助 21 % / 他 5 %</t>
         </is>
       </c>
       <c r="L4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.45 % / 補助 21 % / 他 3.99 %</t>
+          <t xml:space="preserve">全社 15.71 % / 補助 21 % / 他 5 %</t>
         </is>
       </c>
     </row>
@@ -2964,12 +2964,12 @@
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 65.6 % / 補助 65 % / 他 66.83 %</t>
+          <t xml:space="preserve">全社 65.61 % / 補助 65 % / 他 66.84 %</t>
         </is>
       </c>
       <c r="L5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 65.44 % / 補助 65 % / 他 66.5 %</t>
+          <t xml:space="preserve">全社 65.45 % / 補助 65 % / 他 66.51 %</t>
         </is>
       </c>
     </row>
@@ -3026,12 +3026,12 @@
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 34.4 % / 補助 35 % / 他 33.17 %</t>
+          <t xml:space="preserve">全社 34.39 % / 補助 35 % / 他 33.16 %</t>
         </is>
       </c>
       <c r="L6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 34.56 % / 補助 35 % / 他 33.5 %</t>
+          <t xml:space="preserve">全社 34.55 % / 補助 35 % / 他 33.49 %</t>
         </is>
       </c>
     </row>
@@ -3083,17 +3083,17 @@
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 23.37 % / 補助 22.25 % / 他 25.36 %</t>
+          <t xml:space="preserve">全社 23.31 % / 補助 22.25 % / 他 25.18 %</t>
         </is>
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 22.03 % / 補助 20.46 % / 他 25.27 %</t>
+          <t xml:space="preserve">全社 21.93 % / 補助 20.46 % / 他 24.9 %</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 20.73 % / 補助 18.87 % / 他 25.19 %</t>
+          <t xml:space="preserve">全社 20.6 % / 補助 18.87 % / 他 24.63 %</t>
         </is>
       </c>
     </row>
@@ -3145,17 +3145,17 @@
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.85 % / 補助 12.75 % / 他 7.47 %</t>
+          <t xml:space="preserve">全社 10.9 % / 補助 12.75 % / 他 7.66 %</t>
         </is>
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.37 % / 補助 14.54 % / 他 7.9 %</t>
+          <t xml:space="preserve">全社 12.46 % / 補助 14.54 % / 他 8.26 %</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.83 % / 補助 16.13 % / 他 8.31 %</t>
+          <t xml:space="preserve">全社 13.95 % / 補助 16.13 % / 他 8.86 %</t>
         </is>
       </c>
     </row>
@@ -3207,17 +3207,17 @@
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 14.37 % / 補助 17.22 % / 他 9.31 %</t>
+          <t xml:space="preserve">全社 14.41 % / 補助 17.22 % / 他 9.47 %</t>
         </is>
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.44 % / 補助 18.24 % / 他 9.66 %</t>
+          <t xml:space="preserve">全社 15.51 % / 補助 18.24 % / 他 9.99 %</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 16.49 % / 補助 19.19 % / 他 10 %</t>
+          <t xml:space="preserve">全社 16.58 % / 補助 19.19 % / 他 10.51 %</t>
         </is>
       </c>
     </row>
@@ -3269,17 +3269,17 @@
       </c>
       <c r="J10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.07 % / 補助 9.67 % / 他 10.78 %</t>
+          <t xml:space="preserve">全社 10.01 % / 補助 9.67 % / 他 10.62 %</t>
         </is>
       </c>
       <c r="K10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.76 % / 補助 9.33 % / 他 10.64 %</t>
+          <t xml:space="preserve">全社 9.66 % / 補助 9.33 % / 他 10.31 %</t>
         </is>
       </c>
       <c r="L10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.44 % / 補助 9 % / 他 10.5 %</t>
+          <t xml:space="preserve">全社 9.3 % / 補助 9 % / 他 10.01 %</t>
         </is>
       </c>
     </row>
@@ -3393,17 +3393,17 @@
       </c>
       <c r="J12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.19 % / 補助 7.67 % / 他 11.89 %</t>
+          <t xml:space="preserve">全社 9.2 % / 補助 7.67 % / 他 11.89 %</t>
         </is>
       </c>
       <c r="K12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.67 % / 補助 7.05 % / 他 12.01 %</t>
+          <t xml:space="preserve">全社 8.69 % / 補助 7.05 % / 他 12.01 %</t>
         </is>
       </c>
       <c r="L12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.15 % / 補助 6.48 % / 他 12.14 %</t>
+          <t xml:space="preserve">全社 8.18 % / 補助 6.48 % / 他 12.13 %</t>
         </is>
       </c>
     </row>
@@ -3455,17 +3455,17 @@
       </c>
       <c r="J13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.59 % / 補助 0.44 % / 他 0.85 %</t>
+          <t xml:space="preserve">全社 0.59 % / 補助 0.44 % / 他 0.86 %</t>
         </is>
       </c>
       <c r="K13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.54 % / 補助 0.38 % / 他 0.86 %</t>
+          <t xml:space="preserve">全社 0.54 % / 補助 0.38 % / 他 0.85 %</t>
         </is>
       </c>
       <c r="L13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.49 % / 補助 0.33 % / 他 0.86 %</t>
+          <t xml:space="preserve">全社 0.49 % / 補助 0.33 % / 他 0.84 %</t>
         </is>
       </c>
     </row>
@@ -3517,17 +3517,17 @@
       </c>
       <c r="J14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.78 % / 補助 8.11 % / 他 12.75 %</t>
+          <t xml:space="preserve">全社 9.79 % / 補助 8.11 % / 他 12.75 %</t>
         </is>
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.2 % / 補助 7.43 % / 他 12.87 %</t>
+          <t xml:space="preserve">全社 9.23 % / 補助 7.43 % / 他 12.87 %</t>
         </is>
       </c>
       <c r="L14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.63 % / 補助 6.82 % / 他 13 %</t>
+          <t xml:space="preserve">全社 8.67 % / 補助 6.82 % / 他 12.98 %</t>
         </is>
       </c>
     </row>
@@ -3584,12 +3584,12 @@
       </c>
       <c r="K15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.087 億円/人 / 補助 0.1 億円/人 / 他 0.075 億円/人</t>
+          <t xml:space="preserve">全社 0.087 億円/人 / 補助 0.1 億円/人 / 他 0.076 億円/人</t>
         </is>
       </c>
       <c r="L15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.092 億円/人 / 補助 0.107 億円/人 / 他 0.078 億円/人</t>
+          <t xml:space="preserve">全社 0.092 億円/人 / 補助 0.107 億円/人 / 他 0.079 億円/人</t>
         </is>
       </c>
     </row>
@@ -3641,17 +3641,17 @@
       </c>
       <c r="J16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.268 億円/人 / 補助 0.32 億円/人 / 他 0.233 億円/人</t>
+          <t xml:space="preserve">全社 0.27 億円/人 / 補助 0.32 億円/人 / 他 0.237 億円/人</t>
         </is>
       </c>
       <c r="K16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.28 億円/人 / 補助 0.335 億円/人 / 他 0.243 億円/人</t>
+          <t xml:space="preserve">全社 0.282 億円/人 / 補助 0.335 億円/人 / 他 0.247 億円/人</t>
         </is>
       </c>
       <c r="L16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.294 億円/人 / 補助 0.355 億円/人 / 他 0.253 億円/人</t>
+          <t xml:space="preserve">全社 0.296 億円/人 / 補助 0.355 億円/人 / 他 0.257 億円/人</t>
         </is>
       </c>
     </row>
@@ -3703,17 +3703,17 @@
       </c>
       <c r="J17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5.78 % / 補助 7.02 % / 他 4.03 %</t>
+          <t xml:space="preserve">全社 5.96 % / 補助 7.02 % / 他 4.47 %</t>
         </is>
       </c>
       <c r="K17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5.79 % / 補助 6.96 % / 他 3.99 %</t>
+          <t xml:space="preserve">全社 6 % / 補助 6.96 % / 他 4.54 %</t>
         </is>
       </c>
       <c r="L17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5.92 % / 補助 7.02 % / 他 4.04 %</t>
+          <t xml:space="preserve">全社 6.05 % / 補助 7.02 % / 他 4.47 %</t>
         </is>
       </c>
     </row>
@@ -3765,17 +3765,17 @@
       </c>
       <c r="J18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 40.5 % / 補助 32 % / 他 57.81 %</t>
+          <t xml:space="preserve">全社 40.45 % / 補助 32 % / 他 57.38 %</t>
         </is>
       </c>
       <c r="K18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 37.35 % / 補助 28.94 % / 他 57.11 %</t>
+          <t xml:space="preserve">全社 37.3 % / 補助 28.94 % / 他 56.3 %</t>
         </is>
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 34.37 % / 補助 26.21 % / 他 56.5 %</t>
+          <t xml:space="preserve">全社 34.32 % / 補助 26.21 % / 他 55.25 %</t>
         </is>
       </c>
     </row>
@@ -3889,17 +3889,17 @@
       </c>
       <c r="J20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.891 億円/人 / 補助 1.214 億円/人 / 他 0.605 億円/人</t>
+          <t xml:space="preserve">全社 0.892 億円/人 / 補助 1.214 億円/人 / 他 0.608 億円/人</t>
         </is>
       </c>
       <c r="K20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.999 億円/人 / 補助 1.413 億円/人 / 他 0.623 億円/人</t>
+          <t xml:space="preserve">全社 1 億円/人 / 補助 1.413 億円/人 / 他 0.629 億円/人</t>
         </is>
       </c>
       <c r="L20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.126 億円/人 / 補助 1.643 億円/人 / 他 0.642 億円/人</t>
+          <t xml:space="preserve">全社 1.127 億円/人 / 補助 1.643 億円/人 / 他 0.651 億円/人</t>
         </is>
       </c>
     </row>
@@ -3951,17 +3951,17 @@
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.097 億円/人 / 補助 0.155 億円/人 / 他 0.045 億円/人</t>
+          <t xml:space="preserve">全社 0.097 億円/人 / 補助 0.155 億円/人 / 他 0.047 億円/人</t>
         </is>
       </c>
       <c r="K21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.124 億円/人 / 補助 0.205 億円/人 / 他 0.049 億円/人</t>
+          <t xml:space="preserve">全社 0.125 億円/人 / 補助 0.205 億円/人 / 他 0.052 億円/人</t>
         </is>
       </c>
       <c r="L21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.156 億円/人 / 補助 0.265 億円/人 / 他 0.053 億円/人</t>
+          <t xml:space="preserve">全社 0.157 億円/人 / 補助 0.265 億円/人 / 他 0.058 億円/人</t>
         </is>
       </c>
     </row>
@@ -4013,17 +4013,17 @@
       </c>
       <c r="J22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.211 億円/人 / 補助 0.302 億円/人 / 他 0.131 億円/人</t>
+          <t xml:space="preserve">全社 0.212 億円/人 / 補助 0.302 億円/人 / 他 0.132 億円/人</t>
         </is>
       </c>
       <c r="K22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.242 億円/人 / 補助 0.357 億円/人 / 他 0.137 億円/人</t>
+          <t xml:space="preserve">全社 0.243 億円/人 / 補助 0.357 億円/人 / 他 0.141 億円/人</t>
         </is>
       </c>
       <c r="L22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.278 億円/人 / 補助 0.421 億円/人 / 他 0.144 億円/人</t>
+          <t xml:space="preserve">全社 0.279 億円/人 / 補助 0.421 億円/人 / 他 0.15 億円/人</t>
         </is>
       </c>
     </row>
@@ -4075,17 +4075,17 @@
       </c>
       <c r="J23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.39 % / 補助 4 % / 他 1 %</t>
+          <t xml:space="preserve">全社 2.66 % / 補助 4 % / 他 1.5 %</t>
         </is>
       </c>
       <c r="K23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.41 % / 補助 4 % / 他 1 %</t>
+          <t xml:space="preserve">全社 2.67 % / 補助 4 % / 他 1.5 %</t>
         </is>
       </c>
       <c r="L23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.43 % / 補助 4 % / 他 1 %</t>
+          <t xml:space="preserve">全社 2.69 % / 補助 4 % / 他 1.5 %</t>
         </is>
       </c>
     </row>
@@ -4137,17 +4137,17 @@
       </c>
       <c r="J24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.88 pt / 補助 17 pt / 他 3 pt</t>
+          <t xml:space="preserve">全社 12.01 pt / 補助 17 pt / 他 3.5 pt</t>
         </is>
       </c>
       <c r="K24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.47 pt / 補助 17 pt / 他 3.01 pt</t>
+          <t xml:space="preserve">全社 12.52 pt / 補助 17 pt / 他 3.49 pt</t>
         </is>
       </c>
       <c r="L24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.02 pt / 補助 17 pt / 他 2.99 pt</t>
+          <t xml:space="preserve">全社 13.02 pt / 補助 17 pt / 他 3.5 pt</t>
         </is>
       </c>
     </row>
@@ -4261,17 +4261,17 @@
       </c>
       <c r="J26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.52 % / 補助 4.48 % / 他 1.83 %</t>
+          <t xml:space="preserve">全社 3.51 % / 補助 4.48 % / 他 1.81 %</t>
         </is>
       </c>
       <c r="K26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.07 % / 補助 3.7 % / 他 1.76 %</t>
+          <t xml:space="preserve">全社 3.05 % / 補助 3.7 % / 他 1.73 %</t>
         </is>
       </c>
       <c r="L26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.66 % / 補助 3.06 % / 他 1.69 %</t>
+          <t xml:space="preserve">全社 2.63 % / 補助 3.06 % / 他 1.65 %</t>
         </is>
       </c>
     </row>
@@ -4447,17 +4447,17 @@
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.08 倍 / 補助 3.85 倍 / 他 5.08 倍</t>
+          <t xml:space="preserve">全社 4.1 倍 / 補助 3.85 倍 / 他 5.22 倍</t>
         </is>
       </c>
       <c r="K29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5.03 倍 / 補助 4.93 倍 / 他 5.49 倍</t>
+          <t xml:space="preserve">全社 5.09 倍 / 補助 4.93 倍 / 他 5.78 倍</t>
         </is>
       </c>
       <c r="L29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.21 倍 / 補助 6.28 倍 / 他 5.91 倍</t>
+          <t xml:space="preserve">全社 6.3 倍 / 補助 6.28 倍 / 他 6.39 倍</t>
         </is>
       </c>
     </row>
@@ -4633,17 +4633,17 @@
       </c>
       <c r="J32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 63.94 %</t>
+          <t xml:space="preserve">構成比 63.72 %</t>
         </is>
       </c>
       <c r="K32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 67.35 %</t>
+          <t xml:space="preserve">構成比 66.93 %</t>
         </is>
       </c>
       <c r="L32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 70.59 %</t>
+          <t xml:space="preserve">構成比 69.99 %</t>
         </is>
       </c>
     </row>
@@ -4695,17 +4695,17 @@
       </c>
       <c r="J33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 21 % / 他 4 %</t>
+          <t xml:space="preserve">補助 21 % / 他 5 %</t>
         </is>
       </c>
       <c r="K33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 21 % / 他 4.01 %</t>
+          <t xml:space="preserve">補助 21 % / 他 5 %</t>
         </is>
       </c>
       <c r="L33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 21 % / 他 3.99 %</t>
+          <t xml:space="preserve">補助 21 % / 他 5 %</t>
         </is>
       </c>
     </row>
@@ -4767,7 +4767,7 @@
       </c>
       <c r="L34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -1.5 pt</t>
+          <t xml:space="preserve">差 -1.51 pt</t>
         </is>
       </c>
     </row>
@@ -4819,17 +4819,17 @@
       </c>
       <c r="J35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 5.27 pt</t>
+          <t xml:space="preserve">差 5.09 pt</t>
         </is>
       </c>
       <c r="K35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 6.64 pt</t>
+          <t xml:space="preserve">差 6.28 pt</t>
         </is>
       </c>
       <c r="L35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 7.82 pt</t>
+          <t xml:space="preserve">差 7.27 pt</t>
         </is>
       </c>
     </row>
@@ -4881,17 +4881,17 @@
       </c>
       <c r="J36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.214 億円/人 / 他 0.605 億円/人</t>
+          <t xml:space="preserve">補助 1.214 億円/人 / 他 0.608 億円/人</t>
         </is>
       </c>
       <c r="K36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.413 億円/人 / 他 0.623 億円/人</t>
+          <t xml:space="preserve">補助 1.413 億円/人 / 他 0.629 億円/人</t>
         </is>
       </c>
       <c r="L36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.643 億円/人 / 他 0.642 億円/人</t>
+          <t xml:space="preserve">補助 1.643 億円/人 / 他 0.651 億円/人</t>
         </is>
       </c>
     </row>
@@ -4948,12 +4948,12 @@
       </c>
       <c r="K37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.1 億円/人 / 他 0.075 億円/人</t>
+          <t xml:space="preserve">補助 0.1 億円/人 / 他 0.076 億円/人</t>
         </is>
       </c>
       <c r="L37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.107 億円/人 / 他 0.078 億円/人</t>
+          <t xml:space="preserve">補助 0.107 億円/人 / 他 0.079 億円/人</t>
         </is>
       </c>
     </row>
@@ -5005,17 +5005,17 @@
       </c>
       <c r="J38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 90.63 %</t>
+          <t xml:space="preserve">寄与率 87.66 %</t>
         </is>
       </c>
       <c r="K38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 92.02 %</t>
+          <t xml:space="preserve">寄与率 89.33 %</t>
         </is>
       </c>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 93.28 %</t>
+          <t xml:space="preserve">寄与率 90.58 %</t>
         </is>
       </c>
     </row>
@@ -5293,7 +5293,7 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C16" s="2">
         <v>-10</v>
@@ -5357,7 +5357,7 @@
         </is>
       </c>
       <c r="B20" s="2">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="C20" s="2">
         <v>0</v>
@@ -5389,7 +5389,7 @@
         </is>
       </c>
       <c r="B22" s="2">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="C22" s="2">
         <v>-5</v>
@@ -5421,7 +5421,7 @@
         </is>
       </c>
       <c r="B24" s="2">
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="C24" s="2">
         <v>4</v>
@@ -5540,7 +5540,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjQsIm9mZmljZXJQYXkiOjAuMzYsImRlcHJlY2lhdGlvbiI6MS44LCJvdGhlclNnYSI6OSwiaGVhZGNvdW50Ijo5MCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4zNiwib2ZmaWNlclBheSI6MC41NSwiZGVwcmVjaWF0aW9uIjoxLjM4LCJvdGhlclNnYSI6Ny4zNiwiaGVhZGNvdW50IjoxMTkuNiwib2ZmaWNlckNvdW50IjozfX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjcsIm9mZmljZXJQYXkiOjAuMzgsImRlcHJlY2lhdGlvbiI6MS45LCJvdGhlclNnYSI6OS41LCJoZWFkY291bnQiOjk1LCJvZmZpY2VyQ291bnQiOjJ9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNjgsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI0LjgsIm9mZmljZXJDb3VudCI6M319LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6Niwib2ZmaWNlclBheSI6MC40LCJkZXByZWNpYXRpb24iOjIsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsIm9mZmljZXJQYXkiOjAuNiwiZGVwcmVjaWF0aW9uIjoxLjUsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjIxLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjowLjA3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjA3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAuMDEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA2LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wMSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMSwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNCwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MCwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDEsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjA0LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wMSwicHJvamVjdFNnYVJhdGVFbmQiOjAuMDksIm90aGVyU2dhUmF0ZUVuZCI6MC4xMDUsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA2LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6NDUsInN1YnNpZHkiOjE1LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6Wy0wLjA1LDAuNF0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlstMC4xNSwwLjI1XSwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6Wy0wLjA1LDAuMV0sInByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOlstMC4wMywwLjJdLCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlstMC4xNSwwLjI1XSwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOlswLDAuMV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlstMC4xLDAuMl0sIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjpbLTAuMTUsMC4yNV0sIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlstMC4wNSwwLjFdLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbLTAuMTUsMC4yNV0sInByb2plY3RTYWxlc0dyb3d0aCI6Wy0wLjA1LDAuNF0sIm90aGVyU2FsZXNHcm93dGgiOlstMC4xLDAuMl0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOlstMC4xNSwwLjI1XSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOlstMC4xNSwwLjI1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDQ1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMCwwLjA4XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6Wy0wLjAzLDAuMl0sIm90aGVySGVhZGNvdW50R3Jvd3RoIjpbLTAuMDUsMC4xXSwicHJvamVjdFNnYVJhdGVFbmQiOlswLjA0LDAuMjVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA0LDAuMjVdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAsMC4xXSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjEsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6ODIuNCwibWF4IjoxNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55UGF5U2NoZWR1bGUiOnsidmFsdWUiOjMuNSwibWF4Ijo3LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzU2hhcmUiOnsidmFsdWUiOjcwLCJtYXgiOjk1LCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjIsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6NzQuOCwibWF4IjoxNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsYWJvclByb2R1Y3Rpdml0eUNhZ3IiOnsidmFsdWUiOjIxLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZEluY3JlYXNlIjp7InZhbHVlIjoyOC4xLCJtYXgiOjUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6My45LCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MC4xLCJtYXgiOjAuMiwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjozMCwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnt9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIifQ==</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjQsIm9mZmljZXJQYXkiOjAuMzYsImRlcHJlY2lhdGlvbiI6MS44LCJvdGhlclNnYSI6OSwiaGVhZGNvdW50Ijo5MCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4zNiwib2ZmaWNlclBheSI6MC41NSwiZGVwcmVjaWF0aW9uIjoxLjM4LCJvdGhlclNnYSI6Ny4zNiwiaGVhZGNvdW50IjoxMTkuNiwib2ZmaWNlckNvdW50IjozfX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjcsIm9mZmljZXJQYXkiOjAuMzgsImRlcHJlY2lhdGlvbiI6MS45LCJvdGhlclNnYSI6OS41LCJoZWFkY291bnQiOjk1LCJvZmZpY2VyQ291bnQiOjJ9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNjgsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI0LjgsIm9mZmljZXJDb3VudCI6M319LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6Niwib2ZmaWNlclBheSI6MC40LCJkZXByZWNpYXRpb24iOjIsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsIm9mZmljZXJQYXkiOjAuNiwiZGVwcmVjaWF0aW9uIjoxLjUsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjIxLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjowLjA3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjA3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAuMDEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA2LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wMSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMSwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MCwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDEsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDE1LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wOSwib3RoZXJTZ2FSYXRlRW5kIjowLjEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA2LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6NDUsInN1YnNpZHkiOjE1LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6Wy0wLjA1LDAuNF0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlstMC4xNSwwLjI1XSwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6Wy0wLjA1LDAuMV0sInByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOlstMC4wMywwLjJdLCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlstMC4xNSwwLjI1XSwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOlswLDAuMV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlstMC4xLDAuMl0sIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjpbLTAuMTUsMC4yNV0sIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlstMC4wNSwwLjFdLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbLTAuMTUsMC4yNV0sInByb2plY3RTYWxlc0dyb3d0aCI6Wy0wLjA1LDAuNF0sIm90aGVyU2FsZXNHcm93dGgiOlstMC4xLDAuMl0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOlstMC4xNSwwLjI1XSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOlstMC4xNSwwLjI1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDQ1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMCwwLjA4XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6Wy0wLjAzLDAuMl0sIm90aGVySGVhZGNvdW50R3Jvd3RoIjpbLTAuMDUsMC4xXSwicHJvamVjdFNnYVJhdGVFbmQiOlswLjA0LDAuMjVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA0LDAuMjVdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAsMC4xXSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjEsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6ODIuNCwibWF4IjoxNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55UGF5U2NoZWR1bGUiOnsidmFsdWUiOjMuNSwibWF4Ijo3LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzU2hhcmUiOnsidmFsdWUiOjcwLCJtYXgiOjk1LCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjIsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6NzQuOCwibWF4IjoxNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsYWJvclByb2R1Y3Rpdml0eUNhZ3IiOnsidmFsdWUiOjIxLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZEluY3JlYXNlIjp7InZhbHVlIjoyOC4xLCJtYXgiOjUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6My45LCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MC4xLCJtYXgiOjAuMiwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjozMCwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnt9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIifQ==</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Unify null and zero input handling
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -11,7 +11,8 @@
     <sheet name="補助事業収支" sheetId="4" r:id="rId4"/>
     <sheet name="妥当性診断" sheetId="5" r:id="rId5"/>
     <sheet name="前提・目標" sheetId="6" r:id="rId6"/>
-    <sheet name="モデルデータ" sheetId="7" state="hidden" r:id="rId7"/>
+    <sheet name="入力データ監査" sheetId="7" r:id="rId7"/>
+    <sheet name="モデルデータ" sheetId="8" state="hidden" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -198,11 +199,15 @@
           <t xml:space="preserve">%/年</t>
         </is>
       </c>
-      <c r="D7" s="2">
-        <v>21</v>
-      </c>
-      <c r="E7" s="2">
-        <v>35</v>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
@@ -224,11 +229,15 @@
           <t xml:space="preserve">億円</t>
         </is>
       </c>
-      <c r="D8" s="2">
-        <v>82.4</v>
-      </c>
-      <c r="E8" s="2">
-        <v>150</v>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
@@ -250,11 +259,15 @@
           <t xml:space="preserve">%/年</t>
         </is>
       </c>
-      <c r="D9" s="2">
-        <v>3.5</v>
-      </c>
-      <c r="E9" s="2">
-        <v>7</v>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
@@ -276,11 +289,15 @@
           <t xml:space="preserve">%</t>
         </is>
       </c>
-      <c r="D10" s="2">
-        <v>70</v>
-      </c>
-      <c r="E10" s="2">
-        <v>95</v>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
@@ -302,11 +319,15 @@
           <t xml:space="preserve">%/年</t>
         </is>
       </c>
-      <c r="D11" s="2">
-        <v>22</v>
-      </c>
-      <c r="E11" s="2">
-        <v>35</v>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
@@ -328,11 +349,15 @@
           <t xml:space="preserve">億円</t>
         </is>
       </c>
-      <c r="D12" s="2">
-        <v>74.8</v>
-      </c>
-      <c r="E12" s="2">
-        <v>150</v>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
@@ -354,11 +379,15 @@
           <t xml:space="preserve">%/年</t>
         </is>
       </c>
-      <c r="D13" s="2">
-        <v>21</v>
-      </c>
-      <c r="E13" s="2">
-        <v>35</v>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
@@ -380,11 +409,15 @@
           <t xml:space="preserve">億円</t>
         </is>
       </c>
-      <c r="D14" s="2">
-        <v>28.1</v>
-      </c>
-      <c r="E14" s="2">
-        <v>50</v>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E14" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="F14" s="0" t="inlineStr">
         <is>
@@ -406,11 +439,15 @@
           <t xml:space="preserve">%/年</t>
         </is>
       </c>
-      <c r="D15" s="2">
-        <v>7</v>
-      </c>
-      <c r="E15" s="2">
-        <v>10</v>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
@@ -432,11 +469,15 @@
           <t xml:space="preserve">億円</t>
         </is>
       </c>
-      <c r="D16" s="2">
-        <v>3.9</v>
-      </c>
-      <c r="E16" s="2">
-        <v>7</v>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
@@ -458,11 +499,15 @@
           <t xml:space="preserve">%/年</t>
         </is>
       </c>
-      <c r="D17" s="2">
-        <v>6</v>
-      </c>
-      <c r="E17" s="2">
-        <v>10</v>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="F17" s="0" t="inlineStr">
         <is>
@@ -484,11 +529,15 @@
           <t xml:space="preserve">億円</t>
         </is>
       </c>
-      <c r="D18" s="2">
-        <v>0.1</v>
-      </c>
-      <c r="E18" s="2">
-        <v>0.2</v>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
@@ -510,11 +559,15 @@
           <t xml:space="preserve">%</t>
         </is>
       </c>
-      <c r="D19" s="2">
-        <v>30</v>
-      </c>
-      <c r="E19" s="2">
-        <v>70</v>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
@@ -536,11 +589,15 @@
           <t xml:space="preserve">%</t>
         </is>
       </c>
-      <c r="D20" s="2">
-        <v>213</v>
-      </c>
-      <c r="E20" s="2">
-        <v>350</v>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
@@ -562,15 +619,19 @@
           <t xml:space="preserve">点</t>
         </is>
       </c>
-      <c r="D21" s="2">
-        <v>23</v>
-      </c>
-      <c r="E21" s="2">
-        <v>40</v>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">努力</t>
+          <t xml:space="preserve">参考</t>
         </is>
       </c>
     </row>
@@ -5025,7 +5086,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="68" customWidth="1"/>
@@ -5087,11 +5148,15 @@
       <c r="B3" s="2">
         <v>5</v>
       </c>
-      <c r="C3" s="2">
-        <v>-5</v>
-      </c>
-      <c r="D3" s="2">
-        <v>30</v>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -5120,10 +5185,10 @@
         <v>7.000000000000001</v>
       </c>
       <c r="C5" s="2">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="D5" s="2">
-        <v>25</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -5168,10 +5233,10 @@
         <v>1</v>
       </c>
       <c r="C8" s="2">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="D8" s="2">
-        <v>25</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -5216,10 +5281,10 @@
         <v>0.5</v>
       </c>
       <c r="C11" s="2">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="D11" s="2">
-        <v>25</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -5264,10 +5329,10 @@
         <v>0.5</v>
       </c>
       <c r="C14" s="2">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="D14" s="2">
-        <v>25</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -5312,10 +5377,10 @@
         <v>0</v>
       </c>
       <c r="C17" s="2">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="D17" s="2">
-        <v>25</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
@@ -5328,10 +5393,10 @@
         <v>1</v>
       </c>
       <c r="C18" s="2">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="D18" s="2">
-        <v>25</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -5500,22 +5565,6 @@
       </c>
       <c r="D28" s="2">
         <v>50</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ローカルベンチマーク</t>
-        </is>
-      </c>
-      <c r="B29" s="2">
-        <v>23</v>
-      </c>
-      <c r="C29" s="2">
-        <v>0</v>
-      </c>
-      <c r="D29" s="2">
-        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -5523,6 +5572,3219 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C213"/>
+  <sheetFormatPr defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="72" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力データ監査（Null／0区別）</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">保存値</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">状態</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力キー</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">保存値</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">状態</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:company:2023:2-1</t>
+        </is>
+      </c>
+      <c r="B3" s="2">
+        <v>136.4</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:company:2023:2-11</t>
+        </is>
+      </c>
+      <c r="B4" s="2">
+        <v>12.76</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:company:2023:2-14</t>
+        </is>
+      </c>
+      <c r="B5" s="2">
+        <v>3.18</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:company:2023:2-3</t>
+        </is>
+      </c>
+      <c r="B6" s="2">
+        <v>92.75</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:company:2023:2-7</t>
+        </is>
+      </c>
+      <c r="B7" s="2">
+        <v>33.21</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:company:2023:2-8</t>
+        </is>
+      </c>
+      <c r="B8" s="2">
+        <v>0.91</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:company:2024:2-1</t>
+        </is>
+      </c>
+      <c r="B9" s="2">
+        <v>143.2</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:company:2024:2-11</t>
+        </is>
+      </c>
+      <c r="B10" s="2">
+        <v>13.38</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:company:2024:2-14</t>
+        </is>
+      </c>
+      <c r="B11" s="2">
+        <v>3.34</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:company:2024:2-3</t>
+        </is>
+      </c>
+      <c r="B12" s="2">
+        <v>97.38</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:company:2024:2-7</t>
+        </is>
+      </c>
+      <c r="B13" s="2">
+        <v>34.86</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:company:2024:2-8</t>
+        </is>
+      </c>
+      <c r="B14" s="2">
+        <v>0.96</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:company:2025:2-1</t>
+        </is>
+      </c>
+      <c r="B15" s="2">
+        <v>150</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:company:2025:2-11</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <v>14</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:company:2025:2-14</t>
+        </is>
+      </c>
+      <c r="B17" s="2">
+        <v>3.5</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:company:2025:2-3</t>
+        </is>
+      </c>
+      <c r="B18" s="2">
+        <v>102</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:company:2025:2-7</t>
+        </is>
+      </c>
+      <c r="B19" s="2">
+        <v>36.5</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:company:2025:2-8</t>
+        </is>
+      </c>
+      <c r="B20" s="2">
+        <v>1</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2023:7-1</t>
+        </is>
+      </c>
+      <c r="B21" s="2">
+        <v>72</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2023:7-10</t>
+        </is>
+      </c>
+      <c r="B22" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2023:7-13</t>
+        </is>
+      </c>
+      <c r="B23" s="2">
+        <v>90</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2023:7-14</t>
+        </is>
+      </c>
+      <c r="B24" s="2">
+        <v>2</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2023:7-4</t>
+        </is>
+      </c>
+      <c r="B25" s="2">
+        <v>23.04</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2023:7-6</t>
+        </is>
+      </c>
+      <c r="B26" s="2">
+        <v>6.48</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2023:7-8</t>
+        </is>
+      </c>
+      <c r="B27" s="2">
+        <v>5.4</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2023:7-9</t>
+        </is>
+      </c>
+      <c r="B28" s="2">
+        <v>0.36</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2024:7-1</t>
+        </is>
+      </c>
+      <c r="B29" s="2">
+        <v>76</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2024:7-10</t>
+        </is>
+      </c>
+      <c r="B30" s="2">
+        <v>1.9</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2024:7-13</t>
+        </is>
+      </c>
+      <c r="B31" s="2">
+        <v>95</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2024:7-14</t>
+        </is>
+      </c>
+      <c r="B32" s="2">
+        <v>2</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2024:7-4</t>
+        </is>
+      </c>
+      <c r="B33" s="2">
+        <v>24.32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2024:7-6</t>
+        </is>
+      </c>
+      <c r="B34" s="2">
+        <v>6.84</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2024:7-8</t>
+        </is>
+      </c>
+      <c r="B35" s="2">
+        <v>5.7</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2024:7-9</t>
+        </is>
+      </c>
+      <c r="B36" s="2">
+        <v>0.38</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2025:7-1</t>
+        </is>
+      </c>
+      <c r="B37" s="2">
+        <v>80</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2025:7-10</t>
+        </is>
+      </c>
+      <c r="B38" s="2">
+        <v>2</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2025:7-13</t>
+        </is>
+      </c>
+      <c r="B39" s="2">
+        <v>100</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2025:7-14</t>
+        </is>
+      </c>
+      <c r="B40" s="2">
+        <v>2</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2025:7-4</t>
+        </is>
+      </c>
+      <c r="B41" s="2">
+        <v>25.6</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2025:7-6</t>
+        </is>
+      </c>
+      <c r="B42" s="2">
+        <v>7.2</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2025:7-8</t>
+        </is>
+      </c>
+      <c r="B43" s="2">
+        <v>6</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">actual:project:2025:7-9</t>
+        </is>
+      </c>
+      <c r="B44" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:assets</t>
+        </is>
+      </c>
+      <c r="B45" s="2">
+        <v>132</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:buildings</t>
+        </is>
+      </c>
+      <c r="B46" s="2">
+        <v>19</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:capex</t>
+        </is>
+      </c>
+      <c r="B47" s="2">
+        <v>5</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:capital</t>
+        </is>
+      </c>
+      <c r="B48" s="2">
+        <v>10</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:cash</t>
+        </is>
+      </c>
+      <c r="B49" s="2">
+        <v>24</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:currentAssets</t>
+        </is>
+      </c>
+      <c r="B50" s="2">
+        <v>67</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:currentLiabilities</t>
+        </is>
+      </c>
+      <c r="B51" s="2">
+        <v>39</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:fixedAssets</t>
+        </is>
+      </c>
+      <c r="B52" s="2">
+        <v>65</v>
+      </c>
+      <c r="C52" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:fixedLiabilities</t>
+        </is>
+      </c>
+      <c r="B53" s="2">
+        <v>36</v>
+      </c>
+      <c r="C53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:intangibleAssets</t>
+        </is>
+      </c>
+      <c r="B54" s="2">
+        <v>7</v>
+      </c>
+      <c r="C54" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:land</t>
+        </is>
+      </c>
+      <c r="B55" s="2">
+        <v>10</v>
+      </c>
+      <c r="C55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:liabilities</t>
+        </is>
+      </c>
+      <c r="B56" s="2">
+        <v>75</v>
+      </c>
+      <c r="C56" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:longTermDebt</t>
+        </is>
+      </c>
+      <c r="B57" s="2">
+        <v>29</v>
+      </c>
+      <c r="C57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:machinery</t>
+        </is>
+      </c>
+      <c r="B58" s="2">
+        <v>24</v>
+      </c>
+      <c r="C58" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:netAssets</t>
+        </is>
+      </c>
+      <c r="B59" s="2">
+        <v>57</v>
+      </c>
+      <c r="C59" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:shareholderEquity</t>
+        </is>
+      </c>
+      <c r="B60" s="2">
+        <v>54</v>
+      </c>
+      <c r="C60" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:shortTermDebt</t>
+        </is>
+      </c>
+      <c r="B61" s="2">
+        <v>12</v>
+      </c>
+      <c r="C61" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:software</t>
+        </is>
+      </c>
+      <c r="B62" s="2">
+        <v>5</v>
+      </c>
+      <c r="C62" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2023:tangibleAssets</t>
+        </is>
+      </c>
+      <c r="B63" s="2">
+        <v>53</v>
+      </c>
+      <c r="C63" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:assets</t>
+        </is>
+      </c>
+      <c r="B64" s="2">
+        <v>143</v>
+      </c>
+      <c r="C64" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:buildings</t>
+        </is>
+      </c>
+      <c r="B65" s="2">
+        <v>20</v>
+      </c>
+      <c r="C65" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:capex</t>
+        </is>
+      </c>
+      <c r="B66" s="2">
+        <v>8</v>
+      </c>
+      <c r="C66" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:capital</t>
+        </is>
+      </c>
+      <c r="B67" s="2">
+        <v>10</v>
+      </c>
+      <c r="C67" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:cash</t>
+        </is>
+      </c>
+      <c r="B68" s="2">
+        <v>25</v>
+      </c>
+      <c r="C68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:currentAssets</t>
+        </is>
+      </c>
+      <c r="B69" s="2">
+        <v>72</v>
+      </c>
+      <c r="C69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:currentLiabilities</t>
+        </is>
+      </c>
+      <c r="B70" s="2">
+        <v>41</v>
+      </c>
+      <c r="C70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:fixedAssets</t>
+        </is>
+      </c>
+      <c r="B71" s="2">
+        <v>71</v>
+      </c>
+      <c r="C71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:fixedLiabilities</t>
+        </is>
+      </c>
+      <c r="B72" s="2">
+        <v>38</v>
+      </c>
+      <c r="C72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:intangibleAssets</t>
+        </is>
+      </c>
+      <c r="B73" s="2">
+        <v>8</v>
+      </c>
+      <c r="C73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:land</t>
+        </is>
+      </c>
+      <c r="B74" s="2">
+        <v>10</v>
+      </c>
+      <c r="C74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:liabilities</t>
+        </is>
+      </c>
+      <c r="B75" s="2">
+        <v>79</v>
+      </c>
+      <c r="C75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:longTermDebt</t>
+        </is>
+      </c>
+      <c r="B76" s="2">
+        <v>31</v>
+      </c>
+      <c r="C76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:machinery</t>
+        </is>
+      </c>
+      <c r="B77" s="2">
+        <v>28</v>
+      </c>
+      <c r="C77" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:netAssets</t>
+        </is>
+      </c>
+      <c r="B78" s="2">
+        <v>64</v>
+      </c>
+      <c r="C78" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:shareholderEquity</t>
+        </is>
+      </c>
+      <c r="B79" s="2">
+        <v>61</v>
+      </c>
+      <c r="C79" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:shortTermDebt</t>
+        </is>
+      </c>
+      <c r="B80" s="2">
+        <v>12</v>
+      </c>
+      <c r="C80" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:software</t>
+        </is>
+      </c>
+      <c r="B81" s="2">
+        <v>6</v>
+      </c>
+      <c r="C81" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2024:tangibleAssets</t>
+        </is>
+      </c>
+      <c r="B82" s="2">
+        <v>58</v>
+      </c>
+      <c r="C82" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:assets</t>
+        </is>
+      </c>
+      <c r="B83" s="2">
+        <v>156</v>
+      </c>
+      <c r="C83" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:buildings</t>
+        </is>
+      </c>
+      <c r="B84" s="2">
+        <v>22</v>
+      </c>
+      <c r="C84" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:capex</t>
+        </is>
+      </c>
+      <c r="B85" s="2">
+        <v>10</v>
+      </c>
+      <c r="C85" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:capital</t>
+        </is>
+      </c>
+      <c r="B86" s="2">
+        <v>10</v>
+      </c>
+      <c r="C86" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:cash</t>
+        </is>
+      </c>
+      <c r="B87" s="2">
+        <v>27</v>
+      </c>
+      <c r="C87" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:currentAssets</t>
+        </is>
+      </c>
+      <c r="B88" s="2">
+        <v>78</v>
+      </c>
+      <c r="C88" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:currentLiabilities</t>
+        </is>
+      </c>
+      <c r="B89" s="2">
+        <v>43</v>
+      </c>
+      <c r="C89" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:fixedAssets</t>
+        </is>
+      </c>
+      <c r="B90" s="2">
+        <v>78</v>
+      </c>
+      <c r="C90" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:fixedLiabilities</t>
+        </is>
+      </c>
+      <c r="B91" s="2">
+        <v>40</v>
+      </c>
+      <c r="C91" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:intangibleAssets</t>
+        </is>
+      </c>
+      <c r="B92" s="2">
+        <v>9</v>
+      </c>
+      <c r="C92" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:land</t>
+        </is>
+      </c>
+      <c r="B93" s="2">
+        <v>10</v>
+      </c>
+      <c r="C93" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:liabilities</t>
+        </is>
+      </c>
+      <c r="B94" s="2">
+        <v>83</v>
+      </c>
+      <c r="C94" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:longTermDebt</t>
+        </is>
+      </c>
+      <c r="B95" s="2">
+        <v>32</v>
+      </c>
+      <c r="C95" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:machinery</t>
+        </is>
+      </c>
+      <c r="B96" s="2">
+        <v>32</v>
+      </c>
+      <c r="C96" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:netAssets</t>
+        </is>
+      </c>
+      <c r="B97" s="2">
+        <v>73</v>
+      </c>
+      <c r="C97" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:shareholderEquity</t>
+        </is>
+      </c>
+      <c r="B98" s="2">
+        <v>70</v>
+      </c>
+      <c r="C98" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:shortTermDebt</t>
+        </is>
+      </c>
+      <c r="B99" s="2">
+        <v>11</v>
+      </c>
+      <c r="C99" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:software</t>
+        </is>
+      </c>
+      <c r="B100" s="2">
+        <v>7</v>
+      </c>
+      <c r="C100" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">balance-sheet:2025:tangibleAssets</t>
+        </is>
+      </c>
+      <c r="B101" s="2">
+        <v>64</v>
+      </c>
+      <c r="C101" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:investment:0</t>
+        </is>
+      </c>
+      <c r="B102" s="2">
+        <v>15</v>
+      </c>
+      <c r="C102" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:investment:1</t>
+        </is>
+      </c>
+      <c r="B103" s="2">
+        <v>200</v>
+      </c>
+      <c r="C103" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:localBenchmark:0</t>
+        </is>
+      </c>
+      <c r="B104" s="2">
+        <v>0</v>
+      </c>
+      <c r="C104" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:localBenchmark:1</t>
+        </is>
+      </c>
+      <c r="B105" s="2">
+        <v>100</v>
+      </c>
+      <c r="C105" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherCogsImprovement:0</t>
+        </is>
+      </c>
+      <c r="B106" s="2">
+        <v>0</v>
+      </c>
+      <c r="C106" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherCogsImprovement:1</t>
+        </is>
+      </c>
+      <c r="B107" s="2">
+        <v>0.03</v>
+      </c>
+      <c r="C107" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherCogsImprovementToBase:0</t>
+        </is>
+      </c>
+      <c r="B108" s="2">
+        <v>0</v>
+      </c>
+      <c r="C108" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherCogsImprovementToBase:1</t>
+        </is>
+      </c>
+      <c r="B109" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="C109" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowth:0</t>
+        </is>
+      </c>
+      <c r="B110" s="2">
+        <v>-0.05</v>
+      </c>
+      <c r="C110" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowth:1</t>
+        </is>
+      </c>
+      <c r="B111" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C111" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowthToBase:0</t>
+        </is>
+      </c>
+      <c r="B112" s="2">
+        <v>-0.05</v>
+      </c>
+      <c r="C112" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowthToBase:1</t>
+        </is>
+      </c>
+      <c r="B113" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C113" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherPayGrowth:0</t>
+        </is>
+      </c>
+      <c r="B114" s="2">
+        <v>0</v>
+      </c>
+      <c r="C114" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherPayGrowth:1</t>
+        </is>
+      </c>
+      <c r="B115" s="2">
+        <v>0.08</v>
+      </c>
+      <c r="C115" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherPayGrowthToBase:0</t>
+        </is>
+      </c>
+      <c r="B116" s="2">
+        <v>0</v>
+      </c>
+      <c r="C116" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherPayGrowthToBase:1</t>
+        </is>
+      </c>
+      <c r="B117" s="2">
+        <v>0.08</v>
+      </c>
+      <c r="C117" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherSalesGrowth:0</t>
+        </is>
+      </c>
+      <c r="B118" s="2">
+        <v>-0.1</v>
+      </c>
+      <c r="C118" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherSalesGrowth:1</t>
+        </is>
+      </c>
+      <c r="B119" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="C119" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherSalesGrowthToBase:0</t>
+        </is>
+      </c>
+      <c r="B120" s="2">
+        <v>-0.1</v>
+      </c>
+      <c r="C120" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherSalesGrowthToBase:1</t>
+        </is>
+      </c>
+      <c r="B121" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="C121" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherSgaImprovementToBase:0</t>
+        </is>
+      </c>
+      <c r="B122" s="2">
+        <v>0</v>
+      </c>
+      <c r="C122" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherSgaImprovementToBase:1</t>
+        </is>
+      </c>
+      <c r="B123" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="C123" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherSgaRateEnd:0</t>
+        </is>
+      </c>
+      <c r="B124" s="2">
+        <v>0.04</v>
+      </c>
+      <c r="C124" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:otherSgaRateEnd:1</t>
+        </is>
+      </c>
+      <c r="B125" s="2">
+        <v>0.25</v>
+      </c>
+      <c r="C125" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectCogsImprovementAfterBase:0</t>
+        </is>
+      </c>
+      <c r="B126" s="2">
+        <v>0</v>
+      </c>
+      <c r="C126" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectCogsImprovementAfterBase:1</t>
+        </is>
+      </c>
+      <c r="B127" s="2">
+        <v>0.03</v>
+      </c>
+      <c r="C127" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectCogsImprovementToBase:0</t>
+        </is>
+      </c>
+      <c r="B128" s="2">
+        <v>0</v>
+      </c>
+      <c r="C128" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectCogsImprovementToBase:1</t>
+        </is>
+      </c>
+      <c r="B129" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="C129" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowth:0</t>
+        </is>
+      </c>
+      <c r="B130" s="2">
+        <v>-0.03</v>
+      </c>
+      <c r="C130" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowth:1</t>
+        </is>
+      </c>
+      <c r="B131" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="C131" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowthToBase:0</t>
+        </is>
+      </c>
+      <c r="B132" s="2">
+        <v>-0.03</v>
+      </c>
+      <c r="C132" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowthToBase:1</t>
+        </is>
+      </c>
+      <c r="B133" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="C133" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectMarketGrowth:0</t>
+        </is>
+      </c>
+      <c r="B134" s="2">
+        <v>-0.05</v>
+      </c>
+      <c r="C134" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectMarketGrowth:1</t>
+        </is>
+      </c>
+      <c r="B135" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="C135" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowth:0</t>
+        </is>
+      </c>
+      <c r="B136" s="2">
+        <v>0</v>
+      </c>
+      <c r="C136" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowth:1</t>
+        </is>
+      </c>
+      <c r="B137" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C137" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowthToBase:0</t>
+        </is>
+      </c>
+      <c r="B138" s="2">
+        <v>0</v>
+      </c>
+      <c r="C138" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowthToBase:1</t>
+        </is>
+      </c>
+      <c r="B139" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C139" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectPayGrowth:0</t>
+        </is>
+      </c>
+      <c r="B140" s="2">
+        <v>0.045</v>
+      </c>
+      <c r="C140" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectPayGrowth:1</t>
+        </is>
+      </c>
+      <c r="B141" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C141" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectPayGrowthToBase:0</t>
+        </is>
+      </c>
+      <c r="B142" s="2">
+        <v>-0.05</v>
+      </c>
+      <c r="C142" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectPayGrowthToBase:1</t>
+        </is>
+      </c>
+      <c r="B143" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C143" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectSalesGrowth:0</t>
+        </is>
+      </c>
+      <c r="B144" s="2">
+        <v>-0.05</v>
+      </c>
+      <c r="C144" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectSalesGrowth:1</t>
+        </is>
+      </c>
+      <c r="B145" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="C145" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectSalesGrowthToBase:0</t>
+        </is>
+      </c>
+      <c r="B146" s="2">
+        <v>-0.05</v>
+      </c>
+      <c r="C146" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectSalesGrowthToBase:1</t>
+        </is>
+      </c>
+      <c r="B147" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="C147" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectSgaImprovementToBase:0</t>
+        </is>
+      </c>
+      <c r="B148" s="2">
+        <v>0</v>
+      </c>
+      <c r="C148" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectSgaImprovementToBase:1</t>
+        </is>
+      </c>
+      <c r="B149" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="C149" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectSgaRateEnd:0</t>
+        </is>
+      </c>
+      <c r="B150" s="2">
+        <v>0.04</v>
+      </c>
+      <c r="C150" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:projectSgaRateEnd:1</t>
+        </is>
+      </c>
+      <c r="B151" s="2">
+        <v>0.25</v>
+      </c>
+      <c r="C151" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:subsidy:0</t>
+        </is>
+      </c>
+      <c r="B152" s="2">
+        <v>1</v>
+      </c>
+      <c r="C152" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:subsidy:1</t>
+        </is>
+      </c>
+      <c r="B153" s="2">
+        <v>50</v>
+      </c>
+      <c r="C153" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:usefulLife:0</t>
+        </is>
+      </c>
+      <c r="B154" s="2">
+        <v>5</v>
+      </c>
+      <c r="C154" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver-range:usefulLife:1</t>
+        </is>
+      </c>
+      <c r="B155" s="2">
+        <v>20</v>
+      </c>
+      <c r="C155" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:investment</t>
+        </is>
+      </c>
+      <c r="B156" s="2">
+        <v>45</v>
+      </c>
+      <c r="C156" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:localBenchmark</t>
+        </is>
+      </c>
+      <c r="B157" s="2">
+        <v>23</v>
+      </c>
+      <c r="C157" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:otherCogsImprovement</t>
+        </is>
+      </c>
+      <c r="B158" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="C158" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:otherCogsImprovementToBase</t>
+        </is>
+      </c>
+      <c r="B159" s="2">
+        <v>0.005</v>
+      </c>
+      <c r="C159" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:otherHeadcountGrowth</t>
+        </is>
+      </c>
+      <c r="B160" s="2">
+        <v>0.015</v>
+      </c>
+      <c r="C160" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:otherHeadcountGrowthToBase</t>
+        </is>
+      </c>
+      <c r="B161" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="C161" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:otherPayGrowth</t>
+        </is>
+      </c>
+      <c r="B162" s="2">
+        <v>0.045</v>
+      </c>
+      <c r="C162" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:otherPayGrowthToBase</t>
+        </is>
+      </c>
+      <c r="B163" s="2">
+        <v>0.04</v>
+      </c>
+      <c r="C163" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:otherSalesGrowth</t>
+        </is>
+      </c>
+      <c r="B164" s="2">
+        <v>0.05</v>
+      </c>
+      <c r="C164" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:otherSalesGrowthToBase</t>
+        </is>
+      </c>
+      <c r="B165" s="2">
+        <v>0.04</v>
+      </c>
+      <c r="C165" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:otherSgaImprovementToBase</t>
+        </is>
+      </c>
+      <c r="B166" s="2">
+        <v>0.005</v>
+      </c>
+      <c r="C166" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:otherSgaRateEnd</t>
+        </is>
+      </c>
+      <c r="B167" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C167" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:projectCogsImprovementAfterBase</t>
+        </is>
+      </c>
+      <c r="B168" s="2">
+        <v>0</v>
+      </c>
+      <c r="C168" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:projectCogsImprovementToBase</t>
+        </is>
+      </c>
+      <c r="B169" s="2">
+        <v>0.07</v>
+      </c>
+      <c r="C169" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:projectHeadcountGrowth</t>
+        </is>
+      </c>
+      <c r="B170" s="2">
+        <v>0.04</v>
+      </c>
+      <c r="C170" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:projectHeadcountGrowthToBase</t>
+        </is>
+      </c>
+      <c r="B171" s="2">
+        <v>0.04</v>
+      </c>
+      <c r="C171" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:projectMarketGrowth</t>
+        </is>
+      </c>
+      <c r="B172" s="2">
+        <v>0.05</v>
+      </c>
+      <c r="C172" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:projectOfficerPayGrowth</t>
+        </is>
+      </c>
+      <c r="B173" s="2">
+        <v>0.06</v>
+      </c>
+      <c r="C173" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:projectOfficerPayGrowthToBase</t>
+        </is>
+      </c>
+      <c r="B174" s="2">
+        <v>0.06</v>
+      </c>
+      <c r="C174" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:projectPayGrowth</t>
+        </is>
+      </c>
+      <c r="B175" s="2">
+        <v>0.07</v>
+      </c>
+      <c r="C175" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:projectPayGrowthToBase</t>
+        </is>
+      </c>
+      <c r="B176" s="2">
+        <v>0.07</v>
+      </c>
+      <c r="C176" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:projectSalesGrowth</t>
+        </is>
+      </c>
+      <c r="B177" s="2">
+        <v>0.21</v>
+      </c>
+      <c r="C177" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:projectSalesGrowthToBase</t>
+        </is>
+      </c>
+      <c r="B178" s="2">
+        <v>0.21</v>
+      </c>
+      <c r="C178" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:projectSgaImprovementToBase</t>
+        </is>
+      </c>
+      <c r="B179" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="C179" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:projectSgaRateEnd</t>
+        </is>
+      </c>
+      <c r="B180" s="2">
+        <v>0.09</v>
+      </c>
+      <c r="C180" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:subsidy</t>
+        </is>
+      </c>
+      <c r="B181" s="2">
+        <v>15</v>
+      </c>
+      <c r="C181" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:usefulLife</t>
+        </is>
+      </c>
+      <c r="B182" s="2">
+        <v>10</v>
+      </c>
+      <c r="C182" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">future-capex:2026</t>
+        </is>
+      </c>
+      <c r="B183" s="2">
+        <v>15</v>
+      </c>
+      <c r="C183" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">future-capex:2027</t>
+        </is>
+      </c>
+      <c r="B184" s="2">
+        <v>15</v>
+      </c>
+      <c r="C184" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">future-capex:2028</t>
+        </is>
+      </c>
+      <c r="B185" s="2">
+        <v>15</v>
+      </c>
+      <c r="C185" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">future-capex:2029</t>
+        </is>
+      </c>
+      <c r="B186" s="2">
+        <v>0</v>
+      </c>
+      <c r="C186" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">future-capex:2030</t>
+        </is>
+      </c>
+      <c r="B187" s="2">
+        <v>0</v>
+      </c>
+      <c r="C187" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">future-capex:2031</t>
+        </is>
+      </c>
+      <c r="B188" s="2">
+        <v>0</v>
+      </c>
+      <c r="C188" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:companyPaySchedule:max</t>
+        </is>
+      </c>
+      <c r="B189" s="2">
+        <v>7</v>
+      </c>
+      <c r="C189" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:companyPaySchedule:value</t>
+        </is>
+      </c>
+      <c r="B190" s="2">
+        <v>3.5</v>
+      </c>
+      <c r="C190" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:companySalesCagr:max</t>
+        </is>
+      </c>
+      <c r="B191" s="2">
+        <v>35</v>
+      </c>
+      <c r="C191" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:companySalesCagr:value</t>
+        </is>
+      </c>
+      <c r="B192" s="2">
+        <v>21</v>
+      </c>
+      <c r="C192" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:companySalesIncrease:value</t>
+        </is>
+      </c>
+      <c r="B193" s="2">
+        <v>0</v>
+      </c>
+      <c r="C193" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:employeePayCagr:max</t>
+        </is>
+      </c>
+      <c r="B194" s="2">
+        <v>10</v>
+      </c>
+      <c r="C194" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:employeePayCagr:value</t>
+        </is>
+      </c>
+      <c r="B195" s="2">
+        <v>7</v>
+      </c>
+      <c r="C195" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:employeePayIncrease:value</t>
+        </is>
+      </c>
+      <c r="B196" s="2">
+        <v>0</v>
+      </c>
+      <c r="C196" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:investmentSalesRatio:max</t>
+        </is>
+      </c>
+      <c r="B197" s="2">
+        <v>70</v>
+      </c>
+      <c r="C197" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:investmentSalesRatio:value</t>
+        </is>
+      </c>
+      <c r="B198" s="2">
+        <v>30</v>
+      </c>
+      <c r="C198" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:laborProductivityCagr:max</t>
+        </is>
+      </c>
+      <c r="B199" s="2">
+        <v>35</v>
+      </c>
+      <c r="C199" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:laborProductivityCagr:value</t>
+        </is>
+      </c>
+      <c r="B200" s="2">
+        <v>21</v>
+      </c>
+      <c r="C200" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:localBenchmark:max</t>
+        </is>
+      </c>
+      <c r="B201" s="2">
+        <v>40</v>
+      </c>
+      <c r="C201" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:localBenchmark:value</t>
+        </is>
+      </c>
+      <c r="B202" s="2">
+        <v>23</v>
+      </c>
+      <c r="C202" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:officerPayCagr:max</t>
+        </is>
+      </c>
+      <c r="B203" s="2">
+        <v>10</v>
+      </c>
+      <c r="C203" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:officerPayCagr:value</t>
+        </is>
+      </c>
+      <c r="B204" s="2">
+        <v>6</v>
+      </c>
+      <c r="C204" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:officerPayIncrease:value</t>
+        </is>
+      </c>
+      <c r="B205" s="2">
+        <v>0</v>
+      </c>
+      <c r="C205" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesCagr:max</t>
+        </is>
+      </c>
+      <c r="B206" s="2">
+        <v>35</v>
+      </c>
+      <c r="C206" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesCagr:value</t>
+        </is>
+      </c>
+      <c r="B207" s="2">
+        <v>22</v>
+      </c>
+      <c r="C207" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesIncrease:value</t>
+        </is>
+      </c>
+      <c r="B208" s="2">
+        <v>0</v>
+      </c>
+      <c r="C208" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesShare:max</t>
+        </is>
+      </c>
+      <c r="B209" s="2">
+        <v>95</v>
+      </c>
+      <c r="C209" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesShare:value</t>
+        </is>
+      </c>
+      <c r="B210" s="2">
+        <v>70</v>
+      </c>
+      <c r="C210" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:valueAddedIncrease:value</t>
+        </is>
+      </c>
+      <c r="B211" s="2">
+        <v>0</v>
+      </c>
+      <c r="C211" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:valueAddedSubsidyRatio:max</t>
+        </is>
+      </c>
+      <c r="B212" s="2">
+        <v>350</v>
+      </c>
+      <c r="C212" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:valueAddedSubsidyRatio:value</t>
+        </is>
+      </c>
+      <c r="B213" s="2">
+        <v>213</v>
+      </c>
+      <c r="C213" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="18"/>
@@ -5540,7 +8802,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjQsIm9mZmljZXJQYXkiOjAuMzYsImRlcHJlY2lhdGlvbiI6MS44LCJvdGhlclNnYSI6OSwiaGVhZGNvdW50Ijo5MCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4zNiwib2ZmaWNlclBheSI6MC41NSwiZGVwcmVjaWF0aW9uIjoxLjM4LCJvdGhlclNnYSI6Ny4zNiwiaGVhZGNvdW50IjoxMTkuNiwib2ZmaWNlckNvdW50IjozfX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjcsIm9mZmljZXJQYXkiOjAuMzgsImRlcHJlY2lhdGlvbiI6MS45LCJvdGhlclNnYSI6OS41LCJoZWFkY291bnQiOjk1LCJvZmZpY2VyQ291bnQiOjJ9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNjgsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI0LjgsIm9mZmljZXJDb3VudCI6M319LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6Niwib2ZmaWNlclBheSI6MC40LCJkZXByZWNpYXRpb24iOjIsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsIm9mZmljZXJQYXkiOjAuNiwiZGVwcmVjaWF0aW9uIjoxLjUsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjIxLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjowLjA3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjA3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAuMDEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA2LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wMSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMSwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MCwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDEsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDE1LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wOSwib3RoZXJTZ2FSYXRlRW5kIjowLjEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA2LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6NDUsInN1YnNpZHkiOjE1LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6Wy0wLjA1LDAuNF0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlstMC4xNSwwLjI1XSwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6Wy0wLjA1LDAuMV0sInByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOlstMC4wMywwLjJdLCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlstMC4xNSwwLjI1XSwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOlswLDAuMV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlstMC4xLDAuMl0sIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjpbLTAuMTUsMC4yNV0sIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlstMC4wNSwwLjFdLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbLTAuMTUsMC4yNV0sInByb2plY3RTYWxlc0dyb3d0aCI6Wy0wLjA1LDAuNF0sIm90aGVyU2FsZXNHcm93dGgiOlstMC4xLDAuMl0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOlstMC4xNSwwLjI1XSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOlstMC4xNSwwLjI1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDQ1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMCwwLjA4XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6Wy0wLjAzLDAuMl0sIm90aGVySGVhZGNvdW50R3Jvd3RoIjpbLTAuMDUsMC4xXSwicHJvamVjdFNnYVJhdGVFbmQiOlswLjA0LDAuMjVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA0LDAuMjVdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAsMC4xXSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjEsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6ODIuNCwibWF4IjoxNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55UGF5U2NoZWR1bGUiOnsidmFsdWUiOjMuNSwibWF4Ijo3LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzU2hhcmUiOnsidmFsdWUiOjcwLCJtYXgiOjk1LCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjIsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6NzQuOCwibWF4IjoxNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsYWJvclByb2R1Y3Rpdml0eUNhZ3IiOnsidmFsdWUiOjIxLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZEluY3JlYXNlIjp7InZhbHVlIjoyOC4xLCJtYXgiOjUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6My45LCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MC4xLCJtYXgiOjAuMiwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjozMCwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnt9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIifQ==</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjQsIm9mZmljZXJQYXkiOjAuMzYsImRlcHJlY2lhdGlvbiI6MS44LCJvdGhlclNnYSI6OSwiaGVhZGNvdW50Ijo5MCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4zNiwib2ZmaWNlclBheSI6MC41NSwiZGVwcmVjaWF0aW9uIjoxLjM4LCJvdGhlclNnYSI6Ny4zNiwiaGVhZGNvdW50IjoxMTkuNiwib2ZmaWNlckNvdW50IjozfX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjcsIm9mZmljZXJQYXkiOjAuMzgsImRlcHJlY2lhdGlvbiI6MS45LCJvdGhlclNnYSI6OS41LCJoZWFkY291bnQiOjk1LCJvZmZpY2VyQ291bnQiOjJ9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNjgsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI0LjgsIm9mZmljZXJDb3VudCI6M319LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6Niwib2ZmaWNlclBheSI6MC40LCJkZXByZWNpYXRpb24iOjIsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsIm9mZmljZXJQYXkiOjAuNiwiZGVwcmVjaWF0aW9uIjoxLjUsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjIxLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjowLjA3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjA3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAuMDEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA2LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wMSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMSwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MCwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDEsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDE1LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wOSwib3RoZXJTZ2FSYXRlRW5kIjowLjEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA2LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6NDUsInN1YnNpZHkiOjE1LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6Wy0wLjA1LDAuNF0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDJdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbLTAuMDUsMC4xXSwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6Wy0wLjAzLDAuMl0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMC4wMl0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjFdLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjpbLTAuMSwwLjJdLCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6WzAsMC4wMl0sIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlstMC4wNSwwLjFdLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAyXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbLTAuMDUsMC40XSwib3RoZXJTYWxlc0dyb3d0aCI6Wy0wLjEsMC4yXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMCwwLjAzXSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDQ1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMCwwLjA4XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6Wy0wLjAzLDAuMl0sIm90aGVySGVhZGNvdW50R3Jvd3RoIjpbLTAuMDUsMC4xXSwicHJvamVjdFNnYVJhdGVFbmQiOlswLjA0LDAuMjVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA0LDAuMjVdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAsMC4xXSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjEsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlQYXlTY2hlZHVsZSI6eyJ2YWx1ZSI6My41LCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NzAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjowLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5Q2FnciI6eyJ2YWx1ZSI6NywibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjozMCwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnt9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2LjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mi43NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMzLjIxLCJhY3R1YWw6Y29tcGFueToyMDIzOjItOCI6MC45MSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTExIjoxMi43NiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE0IjozLjE4LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMSI6NzIsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny00IjoyMy4wNCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjYuNDgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny04Ijo1LjQsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny05IjowLjM2LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTAiOjEuOCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEzIjo5MCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMSI6MTQzLjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0zIjo5Ny4zOCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTciOjM0Ljg2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItOCI6MC45NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTExIjoxMy4zOCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjozLjM0LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMSI6NzYsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny00IjoyNC4zMiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTYiOjYuODQsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny04Ijo1LjcsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTAiOjEuOSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTgiOjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMSI6MTQsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6My41LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMSI6ODAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNS42LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6Ny4yLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTkiOjAuNCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEwIjoyLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTMiOjEwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTE0IjoyLCJiYWxhbmNlLXNoZWV0OjIwMjM6YXNzZXRzIjoxMzIsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NywiYmFsYW5jZS1zaGVldDoyMDIzOmNhc2giOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRBc3NldHMiOjY1LCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzLCJiYWxhbmNlLXNoZWV0OjIwMjM6YnVpbGRpbmdzIjoxOSwiYmFsYW5jZS1zaGVldDoyMDIzOm1hY2hpbmVyeSI6MjQsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmludGFuZ2libGVBc3NldHMiOjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzb2Z0d2FyZSI6NSwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NSwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRMaWFiaWxpdGllcyI6MzksImJhbGFuY2Utc2hlZXQ6MjAyMzpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2LCJiYWxhbmNlLXNoZWV0OjIwMjM6bG9uZ1Rlcm1EZWJ0IjoyOSwiYmFsYW5jZS1zaGVldDoyMDIzOm5ldEFzc2V0cyI6NTcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGV4Ijo1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50QXNzZXRzIjo3MiwiYmFsYW5jZS1zaGVldDoyMDI0OmNhc2giOjI1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6dGFuZ2libGVBc3NldHMiOjU4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YnVpbGRpbmdzIjoyMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmludGFuZ2libGVBc3NldHMiOjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NiwiYmFsYW5jZS1zaGVldDoyMDI0OmxpYWJpbGl0aWVzIjo3OSwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRMaWFiaWxpdGllcyI6NDEsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkTGlhYmlsaXRpZXMiOjM4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bG9uZ1Rlcm1EZWJ0IjozMSwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaGFyZWhvbGRlckVxdWl0eSI6NjEsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4LCJiYWxhbmNlLXNoZWV0OjIwMjU6YXNzZXRzIjoxNTYsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50QXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3LCJiYWxhbmNlLXNoZWV0OjIwMjU6Zml4ZWRBc3NldHMiOjc4LCJiYWxhbmNlLXNoZWV0OjIwMjU6dGFuZ2libGVBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMiwiYmFsYW5jZS1zaGVldDoyMDI1Om1hY2hpbmVyeSI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjksImJhbGFuY2Utc2hlZXQ6MjAyNTpzb2Z0d2FyZSI6NywiYmFsYW5jZS1zaGVldDoyMDI1OmxpYWJpbGl0aWVzIjo4MywiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaG9ydFRlcm1EZWJ0IjoxMSwiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkTGlhYmlsaXRpZXMiOjQwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMiwiYmFsYW5jZS1zaGVldDoyMDI1Om5ldEFzc2V0cyI6NzMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaGFyZWhvbGRlckVxdWl0eSI6NzAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGV4IjoxMCwiZnV0dXJlLWNhcGV4OjIwMjYiOjE1LCJmdXR1cmUtY2FwZXg6MjAyNyI6MTUsImZ1dHVyZS1jYXBleDoyMDI4IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjkiOjAsImZ1dHVyZS1jYXBleDoyMDMwIjowLCJmdXR1cmUtY2FwZXg6MjAzMSI6MCwiZHJpdmVyOnByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDoxIjowLjMsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMjEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6LTAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC40LCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MC4wNywiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZToxIjowLjEsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjotMC4wMywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4yLCJkcml2ZXI6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLjAxLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMiwiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA2LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMSwiZHJpdmVyOm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjAiOi0wLjEsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMiwiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAyLCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjAxLCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6LTAuMDUsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZToxIjowLjEsImRyaXZlcjpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMiwiZHJpdmVyOnByb2plY3RTYWxlc0dyb3d0aCI6MC4yMSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjQsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjotMC4xLCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjIsImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZToxIjowLjAzLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDEsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MSI6MC4wMywiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDQ1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDoxIjowLjEsImRyaXZlcjpvdGhlclBheUdyb3d0aCI6MC4wNDUsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wOCwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOi0wLjAzLCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aDoxIjowLjIsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wMTUsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjA5LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MCI6MC4wNCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjEiOjAuMjUsImRyaXZlcjpvdGhlclNnYVJhdGVFbmQiOjAuMSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLjA0LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMjUsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNiwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjEsImRyaXZlcjp1c2VmdWxMaWZlIjoxMCwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MCI6NSwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MSI6MjAsImRyaXZlcjppbnZlc3RtZW50Ijo0NSwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjEiOjIwMCwiZHJpdmVyOnN1YnNpZHkiOjE1LCJkcml2ZXItcmFuZ2U6c3Vic2lkeTowIjoxLCJkcml2ZXItcmFuZ2U6c3Vic2lkeToxIjo1MCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoyMSwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjowLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjozLjUsInRhcmdldDpjb21wYW55UGF5U2NoZWR1bGU6bWF4Ijo3LCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6dmFsdWUiOjcwLCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6bWF4Ijo5NSwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6dmFsdWUiOjIyLCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6dmFsdWUiOjIxLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOm1heCI6MzUsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDplbXBsb3llZVBheUNhZ3I6dmFsdWUiOjcsInRhcmdldDplbXBsb3llZVBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MzAsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDB9fQ==</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Clarify multi-year increase comparisons
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -161,7 +161,7 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">計画値</t>
+          <t xml:space="preserve">計画値（基準年→事業化報告3年目・3年間）</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
@@ -171,12 +171,12 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">目標下限</t>
+          <t xml:space="preserve">目標下限（3年間）</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">計画上限</t>
+          <t xml:space="preserve">計画上限（3年間）</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Move officer metrics to reference rows
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -488,15 +488,15 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">年平均役員目標賃上げ率</t>
+          <t xml:space="preserve">投資額／全社売上高</t>
         </is>
       </c>
       <c r="B17" s="2">
-        <v>5.7715899735125475</v>
+        <v>30</v>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">%/年</t>
+          <t xml:space="preserve">%</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
@@ -511,22 +511,22 @@
       </c>
       <c r="F17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">努力</t>
+          <t xml:space="preserve">参考</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">役員給与支給総額の増加額</t>
+          <t xml:space="preserve">付加価値増加額／補助金額</t>
         </is>
       </c>
       <c r="B18" s="2">
-        <v>0.10999999999999999</v>
+        <v>168.5333333333333</v>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">億円</t>
+          <t xml:space="preserve">%</t>
         </is>
       </c>
       <c r="D18" s="0" t="inlineStr">
@@ -548,15 +548,15 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">投資額／全社売上高</t>
+          <t xml:space="preserve">ローカルベンチマーク財務分析結果</t>
         </is>
       </c>
       <c r="B19" s="2">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">%</t>
+          <t xml:space="preserve">点</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
@@ -578,15 +578,15 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">付加価値増加額／補助金額</t>
+          <t xml:space="preserve">年平均役員目標賃上げ率</t>
         </is>
       </c>
       <c r="B20" s="2">
-        <v>168.5333333333333</v>
+        <v>5.7715899735125475</v>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">%</t>
+          <t xml:space="preserve">%/年</t>
         </is>
       </c>
       <c r="D20" s="0" t="inlineStr">
@@ -601,22 +601,22 @@
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">努力</t>
+          <t xml:space="preserve">参考</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ローカルベンチマーク財務分析結果</t>
+          <t xml:space="preserve">役員給与支給総額の増加額</t>
         </is>
       </c>
       <c r="B21" s="2">
-        <v>23</v>
+        <v>0.10999999999999999</v>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">点</t>
+          <t xml:space="preserve">億円</t>
         </is>
       </c>
       <c r="D21" s="0" t="inlineStr">
@@ -8802,7 +8802,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjQsIm9mZmljZXJQYXkiOjAuMzYsImRlcHJlY2lhdGlvbiI6MS44LCJvdGhlclNnYSI6OSwiaGVhZGNvdW50Ijo5MCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4zNiwib2ZmaWNlclBheSI6MC41NSwiZGVwcmVjaWF0aW9uIjoxLjM4LCJvdGhlclNnYSI6Ny4zNiwiaGVhZGNvdW50IjoxMTkuNiwib2ZmaWNlckNvdW50IjozfX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjcsIm9mZmljZXJQYXkiOjAuMzgsImRlcHJlY2lhdGlvbiI6MS45LCJvdGhlclNnYSI6OS41LCJoZWFkY291bnQiOjk1LCJvZmZpY2VyQ291bnQiOjJ9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNjgsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI0LjgsIm9mZmljZXJDb3VudCI6M319LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6Niwib2ZmaWNlclBheSI6MC40LCJkZXByZWNpYXRpb24iOjIsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsIm9mZmljZXJQYXkiOjAuNiwiZGVwcmVjaWF0aW9uIjoxLjUsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjIxLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjowLjA3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjA3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAuMDEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA2LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wMSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMSwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MCwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDEsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDE1LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wOSwib3RoZXJTZ2FSYXRlRW5kIjowLjEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA2LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6NDUsInN1YnNpZHkiOjE1LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6Wy0wLjA1LDAuNF0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDJdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbLTAuMDUsMC4xXSwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6Wy0wLjAzLDAuMl0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMC4wMl0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjFdLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjpbLTAuMSwwLjJdLCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6WzAsMC4wMl0sIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlstMC4wNSwwLjFdLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAyXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbLTAuMDUsMC40XSwib3RoZXJTYWxlc0dyb3d0aCI6Wy0wLjEsMC4yXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMCwwLjAzXSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDQ1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMCwwLjA4XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6Wy0wLjAzLDAuMl0sIm90aGVySGVhZGNvdW50R3Jvd3RoIjpbLTAuMDUsMC4xXSwicHJvamVjdFNnYVJhdGVFbmQiOlswLjA0LDAuMjVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA0LDAuMjVdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAsMC4xXSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjEsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlQYXlTY2hlZHVsZSI6eyJ2YWx1ZSI6My41LCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NzAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjowLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5Q2FnciI6eyJ2YWx1ZSI6NywibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjozMCwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnt9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2LjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mi43NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMzLjIxLCJhY3R1YWw6Y29tcGFueToyMDIzOjItOCI6MC45MSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTExIjoxMi43NiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE0IjozLjE4LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMSI6NzIsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny00IjoyMy4wNCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjYuNDgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny04Ijo1LjQsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny05IjowLjM2LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTAiOjEuOCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEzIjo5MCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMSI6MTQzLjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0zIjo5Ny4zOCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTciOjM0Ljg2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItOCI6MC45NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTExIjoxMy4zOCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjozLjM0LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMSI6NzYsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny00IjoyNC4zMiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTYiOjYuODQsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny04Ijo1LjcsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTAiOjEuOSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTgiOjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMSI6MTQsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6My41LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMSI6ODAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNS42LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6Ny4yLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTkiOjAuNCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEwIjoyLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTMiOjEwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTE0IjoyLCJiYWxhbmNlLXNoZWV0OjIwMjM6YXNzZXRzIjoxMzIsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NywiYmFsYW5jZS1zaGVldDoyMDIzOmNhc2giOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRBc3NldHMiOjY1LCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzLCJiYWxhbmNlLXNoZWV0OjIwMjM6YnVpbGRpbmdzIjoxOSwiYmFsYW5jZS1zaGVldDoyMDIzOm1hY2hpbmVyeSI6MjQsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmludGFuZ2libGVBc3NldHMiOjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzb2Z0d2FyZSI6NSwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NSwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRMaWFiaWxpdGllcyI6MzksImJhbGFuY2Utc2hlZXQ6MjAyMzpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2LCJiYWxhbmNlLXNoZWV0OjIwMjM6bG9uZ1Rlcm1EZWJ0IjoyOSwiYmFsYW5jZS1zaGVldDoyMDIzOm5ldEFzc2V0cyI6NTcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGV4Ijo1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50QXNzZXRzIjo3MiwiYmFsYW5jZS1zaGVldDoyMDI0OmNhc2giOjI1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6dGFuZ2libGVBc3NldHMiOjU4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YnVpbGRpbmdzIjoyMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmludGFuZ2libGVBc3NldHMiOjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NiwiYmFsYW5jZS1zaGVldDoyMDI0OmxpYWJpbGl0aWVzIjo3OSwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRMaWFiaWxpdGllcyI6NDEsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkTGlhYmlsaXRpZXMiOjM4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bG9uZ1Rlcm1EZWJ0IjozMSwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaGFyZWhvbGRlckVxdWl0eSI6NjEsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4LCJiYWxhbmNlLXNoZWV0OjIwMjU6YXNzZXRzIjoxNTYsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50QXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3LCJiYWxhbmNlLXNoZWV0OjIwMjU6Zml4ZWRBc3NldHMiOjc4LCJiYWxhbmNlLXNoZWV0OjIwMjU6dGFuZ2libGVBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMiwiYmFsYW5jZS1zaGVldDoyMDI1Om1hY2hpbmVyeSI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjksImJhbGFuY2Utc2hlZXQ6MjAyNTpzb2Z0d2FyZSI6NywiYmFsYW5jZS1zaGVldDoyMDI1OmxpYWJpbGl0aWVzIjo4MywiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaG9ydFRlcm1EZWJ0IjoxMSwiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkTGlhYmlsaXRpZXMiOjQwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMiwiYmFsYW5jZS1zaGVldDoyMDI1Om5ldEFzc2V0cyI6NzMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaGFyZWhvbGRlckVxdWl0eSI6NzAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGV4IjoxMCwiZnV0dXJlLWNhcGV4OjIwMjYiOjE1LCJmdXR1cmUtY2FwZXg6MjAyNyI6MTUsImZ1dHVyZS1jYXBleDoyMDI4IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjkiOjAsImZ1dHVyZS1jYXBleDoyMDMwIjowLCJmdXR1cmUtY2FwZXg6MjAzMSI6MCwiZHJpdmVyOnByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDoxIjowLjMsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMjEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6LTAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC40LCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MC4wNywiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZToxIjowLjEsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjotMC4wMywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4yLCJkcml2ZXI6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLjAxLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMiwiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA2LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMSwiZHJpdmVyOm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjAiOi0wLjEsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMiwiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAyLCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjAxLCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6LTAuMDUsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZToxIjowLjEsImRyaXZlcjpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMiwiZHJpdmVyOnByb2plY3RTYWxlc0dyb3d0aCI6MC4yMSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjQsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjotMC4xLCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjIsImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZToxIjowLjAzLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDEsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MSI6MC4wMywiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDQ1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDoxIjowLjEsImRyaXZlcjpvdGhlclBheUdyb3d0aCI6MC4wNDUsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wOCwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOi0wLjAzLCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aDoxIjowLjIsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wMTUsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjA5LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MCI6MC4wNCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjEiOjAuMjUsImRyaXZlcjpvdGhlclNnYVJhdGVFbmQiOjAuMSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLjA0LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMjUsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNiwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjEsImRyaXZlcjp1c2VmdWxMaWZlIjoxMCwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MCI6NSwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MSI6MjAsImRyaXZlcjppbnZlc3RtZW50Ijo0NSwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjEiOjIwMCwiZHJpdmVyOnN1YnNpZHkiOjE1LCJkcml2ZXItcmFuZ2U6c3Vic2lkeTowIjoxLCJkcml2ZXItcmFuZ2U6c3Vic2lkeToxIjo1MCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoyMSwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjowLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjozLjUsInRhcmdldDpjb21wYW55UGF5U2NoZWR1bGU6bWF4Ijo3LCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6dmFsdWUiOjcwLCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6bWF4Ijo5NSwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6dmFsdWUiOjIyLCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6dmFsdWUiOjIxLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOm1heCI6MzUsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDplbXBsb3llZVBheUNhZ3I6dmFsdWUiOjcsInRhcmdldDplbXBsb3llZVBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MzAsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDB9LCJtZXRyaWNHcm91cEJhc2VzIjp7ImNvbXBhbnlTYWxlcyI6InJhdGUiLCJwcm9qZWN0U2FsZXMiOiJyYXRlIiwibGFib3JQcm9kdWN0aXZpdHkiOiJyYXRlIiwiZW1wbG95ZWVQYXkiOiJyYXRlIiwib2ZmaWNlclBheSI6InJhdGUifX0=</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjQsIm9mZmljZXJQYXkiOjAuMzYsImRlcHJlY2lhdGlvbiI6MS44LCJvdGhlclNnYSI6OSwiaGVhZGNvdW50Ijo5MCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4zNiwib2ZmaWNlclBheSI6MC41NSwiZGVwcmVjaWF0aW9uIjoxLjM4LCJvdGhlclNnYSI6Ny4zNiwiaGVhZGNvdW50IjoxMTkuNiwib2ZmaWNlckNvdW50IjozfX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjcsIm9mZmljZXJQYXkiOjAuMzgsImRlcHJlY2lhdGlvbiI6MS45LCJvdGhlclNnYSI6OS41LCJoZWFkY291bnQiOjk1LCJvZmZpY2VyQ291bnQiOjJ9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNjgsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI0LjgsIm9mZmljZXJDb3VudCI6M319LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6Niwib2ZmaWNlclBheSI6MC40LCJkZXByZWNpYXRpb24iOjIsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsIm9mZmljZXJQYXkiOjAuNiwiZGVwcmVjaWF0aW9uIjoxLjUsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjIxLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjowLjA3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjA3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAuMDEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA2LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wMSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMSwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MCwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDEsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDE1LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wOSwib3RoZXJTZ2FSYXRlRW5kIjowLjEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA2LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6NDUsInN1YnNpZHkiOjE1LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6Wy0wLjA1LDAuNF0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDJdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbLTAuMDUsMC4xXSwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6Wy0wLjAzLDAuMl0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMC4wMl0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjFdLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjpbLTAuMSwwLjJdLCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6WzAsMC4wMl0sIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlstMC4wNSwwLjFdLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAyXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbLTAuMDUsMC40XSwib3RoZXJTYWxlc0dyb3d0aCI6Wy0wLjEsMC4yXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMCwwLjAzXSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDQ1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMCwwLjA4XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6Wy0wLjAzLDAuMl0sIm90aGVySGVhZGNvdW50R3Jvd3RoIjpbLTAuMDUsMC4xXSwicHJvamVjdFNnYVJhdGVFbmQiOlswLjA0LDAuMjVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA0LDAuMjVdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAsMC4xXSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjEsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlQYXlTY2hlZHVsZSI6eyJ2YWx1ZSI6My41LCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NzAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjowLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5Q2FnciI6eyJ2YWx1ZSI6NywibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJpbnZlc3RtZW50U2FsZXNSYXRpbyI6eyJ2YWx1ZSI6MzAsIm1heCI6NzAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvIjp7InZhbHVlIjoyMTMsIm1heCI6MzUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibG9jYWxCZW5jaG1hcmsiOnsidmFsdWUiOjIzLCJtYXgiOjQwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUNhZ3IiOnsidmFsdWUiOjYsIm1heCI6MTAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnt9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2LjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mi43NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMzLjIxLCJhY3R1YWw6Y29tcGFueToyMDIzOjItOCI6MC45MSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTExIjoxMi43NiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE0IjozLjE4LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMSI6NzIsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny00IjoyMy4wNCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjYuNDgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny04Ijo1LjQsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny05IjowLjM2LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTAiOjEuOCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEzIjo5MCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMSI6MTQzLjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0zIjo5Ny4zOCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTciOjM0Ljg2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItOCI6MC45NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTExIjoxMy4zOCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjozLjM0LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMSI6NzYsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny00IjoyNC4zMiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTYiOjYuODQsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny04Ijo1LjcsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTAiOjEuOSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTgiOjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMSI6MTQsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6My41LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMSI6ODAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNS42LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6Ny4yLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTkiOjAuNCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEwIjoyLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTMiOjEwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTE0IjoyLCJiYWxhbmNlLXNoZWV0OjIwMjM6YXNzZXRzIjoxMzIsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NywiYmFsYW5jZS1zaGVldDoyMDIzOmNhc2giOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRBc3NldHMiOjY1LCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzLCJiYWxhbmNlLXNoZWV0OjIwMjM6YnVpbGRpbmdzIjoxOSwiYmFsYW5jZS1zaGVldDoyMDIzOm1hY2hpbmVyeSI6MjQsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmludGFuZ2libGVBc3NldHMiOjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzb2Z0d2FyZSI6NSwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NSwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRMaWFiaWxpdGllcyI6MzksImJhbGFuY2Utc2hlZXQ6MjAyMzpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2LCJiYWxhbmNlLXNoZWV0OjIwMjM6bG9uZ1Rlcm1EZWJ0IjoyOSwiYmFsYW5jZS1zaGVldDoyMDIzOm5ldEFzc2V0cyI6NTcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGV4Ijo1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50QXNzZXRzIjo3MiwiYmFsYW5jZS1zaGVldDoyMDI0OmNhc2giOjI1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6dGFuZ2libGVBc3NldHMiOjU4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YnVpbGRpbmdzIjoyMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmludGFuZ2libGVBc3NldHMiOjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NiwiYmFsYW5jZS1zaGVldDoyMDI0OmxpYWJpbGl0aWVzIjo3OSwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRMaWFiaWxpdGllcyI6NDEsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkTGlhYmlsaXRpZXMiOjM4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bG9uZ1Rlcm1EZWJ0IjozMSwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaGFyZWhvbGRlckVxdWl0eSI6NjEsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4LCJiYWxhbmNlLXNoZWV0OjIwMjU6YXNzZXRzIjoxNTYsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50QXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3LCJiYWxhbmNlLXNoZWV0OjIwMjU6Zml4ZWRBc3NldHMiOjc4LCJiYWxhbmNlLXNoZWV0OjIwMjU6dGFuZ2libGVBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMiwiYmFsYW5jZS1zaGVldDoyMDI1Om1hY2hpbmVyeSI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjksImJhbGFuY2Utc2hlZXQ6MjAyNTpzb2Z0d2FyZSI6NywiYmFsYW5jZS1zaGVldDoyMDI1OmxpYWJpbGl0aWVzIjo4MywiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaG9ydFRlcm1EZWJ0IjoxMSwiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkTGlhYmlsaXRpZXMiOjQwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMiwiYmFsYW5jZS1zaGVldDoyMDI1Om5ldEFzc2V0cyI6NzMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaGFyZWhvbGRlckVxdWl0eSI6NzAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGV4IjoxMCwiZnV0dXJlLWNhcGV4OjIwMjYiOjE1LCJmdXR1cmUtY2FwZXg6MjAyNyI6MTUsImZ1dHVyZS1jYXBleDoyMDI4IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjkiOjAsImZ1dHVyZS1jYXBleDoyMDMwIjowLCJmdXR1cmUtY2FwZXg6MjAzMSI6MCwiZHJpdmVyOnByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDoxIjowLjMsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMjEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6LTAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC40LCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MC4wNywiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZToxIjowLjEsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjotMC4wMywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4yLCJkcml2ZXI6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLjAxLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMiwiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA2LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMSwiZHJpdmVyOm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjAiOi0wLjEsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMiwiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAyLCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjAxLCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6LTAuMDUsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZToxIjowLjEsImRyaXZlcjpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMiwiZHJpdmVyOnByb2plY3RTYWxlc0dyb3d0aCI6MC4yMSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjQsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjotMC4xLCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjIsImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZToxIjowLjAzLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDEsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MSI6MC4wMywiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDQ1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDoxIjowLjEsImRyaXZlcjpvdGhlclBheUdyb3d0aCI6MC4wNDUsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wOCwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOi0wLjAzLCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aDoxIjowLjIsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wMTUsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjA5LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MCI6MC4wNCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjEiOjAuMjUsImRyaXZlcjpvdGhlclNnYVJhdGVFbmQiOjAuMSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLjA0LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMjUsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNiwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjEsImRyaXZlcjp1c2VmdWxMaWZlIjoxMCwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MCI6NSwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MSI6MjAsImRyaXZlcjppbnZlc3RtZW50Ijo0NSwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjEiOjIwMCwiZHJpdmVyOnN1YnNpZHkiOjE1LCJkcml2ZXItcmFuZ2U6c3Vic2lkeTowIjoxLCJkcml2ZXItcmFuZ2U6c3Vic2lkeToxIjo1MCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoyMSwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjowLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjozLjUsInRhcmdldDpjb21wYW55UGF5U2NoZWR1bGU6bWF4Ijo3LCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6dmFsdWUiOjcwLCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6bWF4Ijo5NSwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6dmFsdWUiOjIyLCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6dmFsdWUiOjIxLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOm1heCI6MzUsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDplbXBsb3llZVBheUNhZ3I6dmFsdWUiOjcsInRhcmdldDplbXBsb3llZVBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MzAsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjB9LCJtZXRyaWNHcm91cEJhc2VzIjp7ImNvbXBhbnlTYWxlcyI6InJhdGUiLCJwcm9qZWN0U2FsZXMiOiJyYXRlIiwibGFib3JQcm9kdWN0aXZpdHkiOiJyYXRlIiwiZW1wbG95ZWVQYXkiOiJyYXRlIn19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Show round six definition for each metric
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -156,12 +156,12 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">15指標・目標</t>
+          <t xml:space="preserve">15指標・目標（指標名に第6次定義を併記）</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">計画値（基準年→事業化報告3年目・3年間）</t>
+          <t xml:space="preserve">計画値</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
@@ -171,12 +171,12 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">目標下限（3年間）</t>
+          <t xml:space="preserve">目標下限</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">計画上限（3年間）</t>
+          <t xml:space="preserve">計画上限</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
@@ -188,7 +188,7 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社年平均売上高成長率</t>
+          <t xml:space="preserve">全社年平均売上高成長率（第6次定義：undefined）</t>
         </is>
       </c>
       <c r="B7" s="2">
@@ -218,7 +218,7 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社売上高増加額</t>
+          <t xml:space="preserve">全社売上高増加額（第6次定義：undefined）</t>
         </is>
       </c>
       <c r="B8" s="2">
@@ -248,7 +248,7 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社の従業員1人当たり給与支給総額の年平均上昇率（最新決算期→基準年度）</t>
+          <t xml:space="preserve">全社の従業員1人当たり給与支給総額の年平均上昇率（最新決算期→基準年度）（第6次定義：undefined）</t>
         </is>
       </c>
       <c r="B9" s="2">
@@ -278,7 +278,7 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業売上高／全社売上高</t>
+          <t xml:space="preserve">補助事業売上高／全社売上高（第6次定義：undefined）</t>
         </is>
       </c>
       <c r="B10" s="2">
@@ -308,7 +308,7 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業年平均売上高成長率</t>
+          <t xml:space="preserve">補助事業年平均売上高成長率（第6次定義：undefined）</t>
         </is>
       </c>
       <c r="B11" s="2">
@@ -338,7 +338,7 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業売上高増加額</t>
+          <t xml:space="preserve">補助事業売上高増加額（第6次定義：undefined）</t>
         </is>
       </c>
       <c r="B12" s="2">
@@ -368,7 +368,7 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業年平均労働生産性の伸び</t>
+          <t xml:space="preserve">補助事業年平均労働生産性の伸び（第6次定義：undefined）</t>
         </is>
       </c>
       <c r="B13" s="2">
@@ -398,7 +398,7 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業付加価値増加額</t>
+          <t xml:space="preserve">補助事業付加価値増加額（第6次定義：undefined）</t>
         </is>
       </c>
       <c r="B14" s="2">
@@ -428,7 +428,7 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業1人当たり給与支給総額の年平均上昇率</t>
+          <t xml:space="preserve">補助事業1人当たり給与支給総額の年平均上昇率（第6次定義：undefined）</t>
         </is>
       </c>
       <c r="B15" s="2">
@@ -458,7 +458,7 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業従業員給与支給総額の増加額</t>
+          <t xml:space="preserve">補助事業従業員給与支給総額の増加額（第6次定義：undefined）</t>
         </is>
       </c>
       <c r="B16" s="2">
@@ -488,7 +488,7 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">投資額／全社売上高</t>
+          <t xml:space="preserve">投資額／全社売上高（第6次定義：undefined）</t>
         </is>
       </c>
       <c r="B17" s="2">
@@ -518,7 +518,7 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">付加価値増加額／補助金額</t>
+          <t xml:space="preserve">付加価値増加額／補助金額（第6次定義：undefined）</t>
         </is>
       </c>
       <c r="B18" s="2">
@@ -548,7 +548,7 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ローカルベンチマーク財務分析結果</t>
+          <t xml:space="preserve">ローカルベンチマーク財務分析結果（第6次定義：undefined）</t>
         </is>
       </c>
       <c r="B19" s="2">
@@ -578,7 +578,7 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">年平均役員目標賃上げ率</t>
+          <t xml:space="preserve">年平均役員目標賃上げ率（第6次定義：undefined）</t>
         </is>
       </c>
       <c r="B20" s="2">
@@ -608,7 +608,7 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">役員給与支給総額の増加額</t>
+          <t xml:space="preserve">役員給与支給総額の増加額（第6次定義：undefined）</t>
         </is>
       </c>
       <c r="B21" s="2">

</xml_diff>

<commit_message>
Raise post-base other business growth default
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -192,7 +192,7 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <v>15.187557062867052</v>
+        <v>15.51906107932668</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -222,7 +222,7 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <v>105</v>
+        <v>107.63</v>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
@@ -282,7 +282,7 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <v>69.99078158951735</v>
+        <v>69.38995332441166</v>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
@@ -1256,13 +1256,13 @@
         <v>198.74</v>
       </c>
       <c r="H3" s="4">
-        <v>227.88</v>
+        <v>228.65999999999997</v>
       </c>
       <c r="I3" s="4">
-        <v>262.5</v>
+        <v>264.15999999999997</v>
       </c>
       <c r="J3" s="4">
-        <v>303.74</v>
+        <v>306.37</v>
       </c>
     </row>
     <row r="4">
@@ -1292,13 +1292,13 @@
         <v>27.63470554235441</v>
       </c>
       <c r="H4" s="2">
-        <v>14.66237294958237</v>
+        <v>15.054845526818927</v>
       </c>
       <c r="I4" s="2">
-        <v>15.192206424433907</v>
+        <v>15.525233971835917</v>
       </c>
       <c r="J4" s="2">
-        <v>15.710476190476186</v>
+        <v>15.978952150212011</v>
       </c>
     </row>
     <row r="5">
@@ -1326,13 +1326,13 @@
         <v>131.15</v>
       </c>
       <c r="H5" s="2">
-        <v>149.91</v>
+        <v>150.44</v>
       </c>
       <c r="I5" s="2">
-        <v>172.22</v>
+        <v>173.33</v>
       </c>
       <c r="J5" s="2">
-        <v>198.8</v>
+        <v>200.54000000000002</v>
       </c>
     </row>
     <row r="6">
@@ -1394,13 +1394,13 @@
         <v>67.59</v>
       </c>
       <c r="H7" s="4">
-        <v>77.97</v>
+        <v>78.21999999999997</v>
       </c>
       <c r="I7" s="4">
-        <v>90.28</v>
+        <v>90.82999999999996</v>
       </c>
       <c r="J7" s="4">
-        <v>104.94</v>
+        <v>105.82999999999998</v>
       </c>
     </row>
     <row r="8">
@@ -1428,13 +1428,13 @@
         <v>34.009258327463016</v>
       </c>
       <c r="H8" s="2">
-        <v>34.215376513954716</v>
+        <v>34.20799440216915</v>
       </c>
       <c r="I8" s="2">
-        <v>34.392380952380954</v>
+        <v>34.3844639612356</v>
       </c>
       <c r="J8" s="2">
-        <v>34.549285573187596</v>
+        <v>34.543199399419</v>
       </c>
     </row>
     <row r="9">
@@ -1462,13 +1462,13 @@
         <v>49.15</v>
       </c>
       <c r="H9" s="2">
-        <v>53.13</v>
+        <v>53.21</v>
       </c>
       <c r="I9" s="2">
-        <v>57.56999999999999</v>
+        <v>57.739999999999995</v>
       </c>
       <c r="J9" s="2">
-        <v>62.57</v>
+        <v>62.83</v>
       </c>
     </row>
     <row r="10">
@@ -1768,13 +1768,13 @@
         <v>18.440000000000005</v>
       </c>
       <c r="H18" s="4">
-        <v>24.839999999999996</v>
+        <v>25.00999999999997</v>
       </c>
       <c r="I18" s="4">
-        <v>32.71000000000001</v>
+        <v>33.08999999999996</v>
       </c>
       <c r="J18" s="4">
-        <v>42.36999999999999</v>
+        <v>42.99999999999998</v>
       </c>
     </row>
     <row r="19">
@@ -1802,13 +1802,13 @@
         <v>9.278454261849655</v>
       </c>
       <c r="H19" s="2">
-        <v>10.900473933649288</v>
+        <v>10.937636665791995</v>
       </c>
       <c r="I19" s="2">
-        <v>12.460952380952383</v>
+        <v>12.526499091459709</v>
       </c>
       <c r="J19" s="2">
-        <v>13.949430433923746</v>
+        <v>14.035316773835552</v>
       </c>
     </row>
     <row r="20">
@@ -1836,13 +1836,13 @@
         <v>18.440000000000005</v>
       </c>
       <c r="H20" s="4">
-        <v>24.839999999999996</v>
+        <v>25.00999999999997</v>
       </c>
       <c r="I20" s="4">
-        <v>32.71000000000001</v>
+        <v>33.08999999999996</v>
       </c>
       <c r="J20" s="4">
-        <v>42.36999999999999</v>
+        <v>42.99999999999998</v>
       </c>
     </row>
   </sheetData>
@@ -2074,13 +2074,13 @@
         <v>60.38039649793701</v>
       </c>
       <c r="H5" s="2">
-        <v>63.717746182201154</v>
+        <v>63.50039359748097</v>
       </c>
       <c r="I5" s="2">
-        <v>66.9295238095238</v>
+        <v>66.50893397940642</v>
       </c>
       <c r="J5" s="2">
-        <v>69.99078158951735</v>
+        <v>69.38995332441166</v>
       </c>
     </row>
     <row r="6">
@@ -2958,17 +2958,17 @@
       </c>
       <c r="J4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 14.66 % / 補助 21 % / 他 5 %</t>
+          <t xml:space="preserve">全社 15.05 % / 補助 21 % / 他 5.99 %</t>
         </is>
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.19 % / 補助 21 % / 他 5 %</t>
+          <t xml:space="preserve">全社 15.53 % / 補助 21 % / 他 6 %</t>
         </is>
       </c>
       <c r="L4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.71 % / 補助 21 % / 他 5 %</t>
+          <t xml:space="preserve">全社 15.98 % / 補助 21 % / 他 6 %</t>
         </is>
       </c>
     </row>
@@ -3020,17 +3020,17 @@
       </c>
       <c r="J5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 65.78 % / 補助 65 % / 他 67.16 %</t>
+          <t xml:space="preserve">全社 65.79 % / 補助 65 % / 他 67.17 %</t>
         </is>
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 65.61 % / 補助 65 % / 他 66.84 %</t>
+          <t xml:space="preserve">全社 65.62 % / 補助 65 % / 他 66.84 %</t>
         </is>
       </c>
       <c r="L5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 65.45 % / 補助 65 % / 他 66.51 %</t>
+          <t xml:space="preserve">全社 65.46 % / 補助 65 % / 他 66.5 %</t>
         </is>
       </c>
     </row>
@@ -3082,17 +3082,17 @@
       </c>
       <c r="J6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 34.22 % / 補助 35 % / 他 32.84 %</t>
+          <t xml:space="preserve">全社 34.21 % / 補助 35 % / 他 32.83 %</t>
         </is>
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 34.39 % / 補助 35 % / 他 33.16 %</t>
+          <t xml:space="preserve">全社 34.38 % / 補助 35 % / 他 33.16 %</t>
         </is>
       </c>
       <c r="L6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 34.55 % / 補助 35 % / 他 33.49 %</t>
+          <t xml:space="preserve">全社 34.54 % / 補助 35 % / 他 33.5 %</t>
         </is>
       </c>
     </row>
@@ -3144,17 +3144,17 @@
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 23.31 % / 補助 22.25 % / 他 25.18 %</t>
+          <t xml:space="preserve">全社 23.27 % / 補助 22.25 % / 他 25.04 %</t>
         </is>
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 21.93 % / 補助 20.46 % / 他 24.9 %</t>
+          <t xml:space="preserve">全社 21.86 % / 補助 20.46 % / 他 24.63 %</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 20.6 % / 補助 18.87 % / 他 24.63 %</t>
+          <t xml:space="preserve">全社 20.51 % / 補助 18.87 % / 他 24.22 %</t>
         </is>
       </c>
     </row>
@@ -3206,17 +3206,17 @@
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.9 % / 補助 12.75 % / 他 7.66 %</t>
+          <t xml:space="preserve">全社 10.94 % / 補助 12.75 % / 他 7.79 %</t>
         </is>
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.46 % / 補助 14.54 % / 他 8.26 %</t>
+          <t xml:space="preserve">全社 12.53 % / 補助 14.54 % / 他 8.53 %</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.95 % / 補助 16.13 % / 他 8.86 %</t>
+          <t xml:space="preserve">全社 14.04 % / 補助 16.13 % / 他 9.29 %</t>
         </is>
       </c>
     </row>
@@ -3268,17 +3268,17 @@
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 14.41 % / 補助 17.22 % / 他 9.47 %</t>
+          <t xml:space="preserve">全社 14.44 % / 補助 17.22 % / 他 9.59 %</t>
         </is>
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.51 % / 補助 18.24 % / 他 9.99 %</t>
+          <t xml:space="preserve">全社 15.55 % / 補助 18.24 % / 他 10.23 %</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 16.58 % / 補助 19.19 % / 他 10.51 %</t>
+          <t xml:space="preserve">全社 16.65 % / 補助 19.19 % / 他 10.89 %</t>
         </is>
       </c>
     </row>
@@ -3340,7 +3340,7 @@
       </c>
       <c r="L10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.3 % / 補助 9 % / 他 10.01 %</t>
+          <t xml:space="preserve">全社 9.31 % / 補助 9 % / 他 10 %</t>
         </is>
       </c>
     </row>
@@ -3454,17 +3454,17 @@
       </c>
       <c r="J12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.2 % / 補助 7.67 % / 他 11.89 %</t>
+          <t xml:space="preserve">全社 9.17 % / 補助 7.67 % / 他 11.78 %</t>
         </is>
       </c>
       <c r="K12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.69 % / 補助 7.05 % / 他 12.01 %</t>
+          <t xml:space="preserve">全社 8.63 % / 補助 7.05 % / 他 11.79 %</t>
         </is>
       </c>
       <c r="L12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.18 % / 補助 6.48 % / 他 12.13 %</t>
+          <t xml:space="preserve">全社 8.11 % / 補助 6.48 % / 他 11.79 %</t>
         </is>
       </c>
     </row>
@@ -3516,17 +3516,17 @@
       </c>
       <c r="J13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.59 % / 補助 0.44 % / 他 0.86 %</t>
+          <t xml:space="preserve">全社 0.59 % / 補助 0.44 % / 他 0.85 %</t>
         </is>
       </c>
       <c r="K13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.54 % / 補助 0.38 % / 他 0.85 %</t>
+          <t xml:space="preserve">全社 0.53 % / 補助 0.38 % / 他 0.84 %</t>
         </is>
       </c>
       <c r="L13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.49 % / 補助 0.33 % / 他 0.84 %</t>
+          <t xml:space="preserve">全社 0.48 % / 補助 0.33 % / 他 0.82 %</t>
         </is>
       </c>
     </row>
@@ -3578,17 +3578,17 @@
       </c>
       <c r="J14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.79 % / 補助 8.11 % / 他 12.75 %</t>
+          <t xml:space="preserve">全社 9.76 % / 補助 8.11 % / 他 12.63 %</t>
         </is>
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.23 % / 補助 7.43 % / 他 12.87 %</t>
+          <t xml:space="preserve">全社 9.17 % / 補助 7.43 % / 他 12.63 %</t>
         </is>
       </c>
       <c r="L14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.67 % / 補助 6.82 % / 他 12.98 %</t>
+          <t xml:space="preserve">全社 8.59 % / 補助 6.82 % / 他 12.61 %</t>
         </is>
       </c>
     </row>
@@ -3826,17 +3826,17 @@
       </c>
       <c r="J18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 40.45 % / 補助 32 % / 他 57.38 %</t>
+          <t xml:space="preserve">全社 40.33 % / 補助 32 % / 他 56.85 %</t>
         </is>
       </c>
       <c r="K18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 37.3 % / 補助 28.94 % / 他 56.3 %</t>
+          <t xml:space="preserve">全社 37.08 % / 補助 28.94 % / 他 55.24 %</t>
         </is>
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 34.32 % / 補助 26.21 % / 他 55.25 %</t>
+          <t xml:space="preserve">全社 34.04 % / 補助 26.21 % / 他 53.68 %</t>
         </is>
       </c>
     </row>
@@ -3950,17 +3950,17 @@
       </c>
       <c r="J20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.892 億円/人 / 補助 1.214 億円/人 / 他 0.608 億円/人</t>
+          <t xml:space="preserve">全社 0.895 億円/人 / 補助 1.214 億円/人 / 他 0.614 億円/人</t>
         </is>
       </c>
       <c r="K20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1 億円/人 / 補助 1.413 億円/人 / 他 0.629 億円/人</t>
+          <t xml:space="preserve">全社 1.007 億円/人 / 補助 1.413 億円/人 / 他 0.641 億円/人</t>
         </is>
       </c>
       <c r="L20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.127 億円/人 / 補助 1.643 億円/人 / 他 0.651 億円/人</t>
+          <t xml:space="preserve">全社 1.137 億円/人 / 補助 1.643 億円/人 / 他 0.67 億円/人</t>
         </is>
       </c>
     </row>
@@ -4012,17 +4012,17 @@
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.097 億円/人 / 補助 0.155 億円/人 / 他 0.047 億円/人</t>
+          <t xml:space="preserve">全社 0.098 億円/人 / 補助 0.155 億円/人 / 他 0.048 億円/人</t>
         </is>
       </c>
       <c r="K21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.125 億円/人 / 補助 0.205 億円/人 / 他 0.052 億円/人</t>
+          <t xml:space="preserve">全社 0.126 億円/人 / 補助 0.205 億円/人 / 他 0.055 億円/人</t>
         </is>
       </c>
       <c r="L21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.157 億円/人 / 補助 0.265 億円/人 / 他 0.058 億円/人</t>
+          <t xml:space="preserve">全社 0.16 億円/人 / 補助 0.265 億円/人 / 他 0.062 億円/人</t>
         </is>
       </c>
     </row>
@@ -4074,17 +4074,17 @@
       </c>
       <c r="J22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.212 億円/人 / 補助 0.302 億円/人 / 他 0.132 億円/人</t>
+          <t xml:space="preserve">全社 0.212 億円/人 / 補助 0.302 億円/人 / 他 0.133 億円/人</t>
         </is>
       </c>
       <c r="K22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.243 億円/人 / 補助 0.357 億円/人 / 他 0.141 億円/人</t>
+          <t xml:space="preserve">全社 0.244 億円/人 / 補助 0.357 億円/人 / 他 0.143 億円/人</t>
         </is>
       </c>
       <c r="L22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.279 億円/人 / 補助 0.421 億円/人 / 他 0.15 億円/人</t>
+          <t xml:space="preserve">全社 0.282 億円/人 / 補助 0.421 億円/人 / 他 0.154 億円/人</t>
         </is>
       </c>
     </row>
@@ -4198,17 +4198,17 @@
       </c>
       <c r="J24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.01 pt / 補助 17 pt / 他 3.5 pt</t>
+          <t xml:space="preserve">全社 12.4 pt / 補助 17 pt / 他 4.49 pt</t>
         </is>
       </c>
       <c r="K24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.52 pt / 補助 17 pt / 他 3.49 pt</t>
+          <t xml:space="preserve">全社 12.86 pt / 補助 17 pt / 他 4.5 pt</t>
         </is>
       </c>
       <c r="L24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.02 pt / 補助 17 pt / 他 3.5 pt</t>
+          <t xml:space="preserve">全社 13.29 pt / 補助 17 pt / 他 4.5 pt</t>
         </is>
       </c>
     </row>
@@ -4322,17 +4322,17 @@
       </c>
       <c r="J26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.51 % / 補助 4.48 % / 他 1.81 %</t>
+          <t xml:space="preserve">全社 3.5 % / 補助 4.48 % / 他 1.8 %</t>
         </is>
       </c>
       <c r="K26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.05 % / 補助 3.7 % / 他 1.73 %</t>
+          <t xml:space="preserve">全社 3.03 % / 補助 3.7 % / 他 1.7 %</t>
         </is>
       </c>
       <c r="L26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.63 % / 補助 3.06 % / 他 1.65 %</t>
+          <t xml:space="preserve">全社 2.61 % / 補助 3.06 % / 他 1.6 %</t>
         </is>
       </c>
     </row>
@@ -4508,17 +4508,17 @@
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.1 倍 / 補助 3.85 倍 / 他 5.22 倍</t>
+          <t xml:space="preserve">全社 4.13 倍 / 補助 3.85 倍 / 他 5.33 倍</t>
         </is>
       </c>
       <c r="K29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5.09 倍 / 補助 4.93 倍 / 他 5.78 倍</t>
+          <t xml:space="preserve">全社 5.14 倍 / 補助 4.93 倍 / 他 6.03 倍</t>
         </is>
       </c>
       <c r="L29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.3 倍 / 補助 6.28 倍 / 他 6.39 倍</t>
+          <t xml:space="preserve">全社 6.37 倍 / 補助 6.28 倍 / 他 6.81 倍</t>
         </is>
       </c>
     </row>
@@ -4694,17 +4694,17 @@
       </c>
       <c r="J32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 63.72 %</t>
+          <t xml:space="preserve">構成比 63.5 %</t>
         </is>
       </c>
       <c r="K32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 66.93 %</t>
+          <t xml:space="preserve">構成比 66.51 %</t>
         </is>
       </c>
       <c r="L32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 69.99 %</t>
+          <t xml:space="preserve">構成比 69.39 %</t>
         </is>
       </c>
     </row>
@@ -4756,17 +4756,17 @@
       </c>
       <c r="J33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 21 % / 他 5 %</t>
+          <t xml:space="preserve">補助 21 % / 他 5.99 %</t>
         </is>
       </c>
       <c r="K33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 21 % / 他 5 %</t>
+          <t xml:space="preserve">補助 21 % / 他 6 %</t>
         </is>
       </c>
       <c r="L33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 21 % / 他 5 %</t>
+          <t xml:space="preserve">補助 21 % / 他 6 %</t>
         </is>
       </c>
     </row>
@@ -4818,17 +4818,17 @@
       </c>
       <c r="J34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -2.16 pt</t>
+          <t xml:space="preserve">差 -2.17 pt</t>
         </is>
       </c>
       <c r="K34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -1.83 pt</t>
+          <t xml:space="preserve">差 -1.84 pt</t>
         </is>
       </c>
       <c r="L34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -1.51 pt</t>
+          <t xml:space="preserve">差 -1.5 pt</t>
         </is>
       </c>
     </row>
@@ -4880,17 +4880,17 @@
       </c>
       <c r="J35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 5.09 pt</t>
+          <t xml:space="preserve">差 4.96 pt</t>
         </is>
       </c>
       <c r="K35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 6.28 pt</t>
+          <t xml:space="preserve">差 6 pt</t>
         </is>
       </c>
       <c r="L35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 7.27 pt</t>
+          <t xml:space="preserve">差 6.84 pt</t>
         </is>
       </c>
     </row>
@@ -4942,17 +4942,17 @@
       </c>
       <c r="J36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.214 億円/人 / 他 0.608 億円/人</t>
+          <t xml:space="preserve">補助 1.214 億円/人 / 他 0.614 億円/人</t>
         </is>
       </c>
       <c r="K36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.413 億円/人 / 他 0.629 億円/人</t>
+          <t xml:space="preserve">補助 1.413 億円/人 / 他 0.641 億円/人</t>
         </is>
       </c>
       <c r="L36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.643 億円/人 / 他 0.651 億円/人</t>
+          <t xml:space="preserve">補助 1.643 億円/人 / 他 0.67 億円/人</t>
         </is>
       </c>
     </row>
@@ -5066,17 +5066,17 @@
       </c>
       <c r="J38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 87.66 %</t>
+          <t xml:space="preserve">寄与率 85.39 %</t>
         </is>
       </c>
       <c r="K38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 89.33 %</t>
+          <t xml:space="preserve">寄与率 87 %</t>
         </is>
       </c>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 90.58 %</t>
+          <t xml:space="preserve">寄与率 88.29 %</t>
         </is>
       </c>
     </row>
@@ -5358,7 +5358,7 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C16" s="2">
         <v>-10</v>
@@ -8037,7 +8037,7 @@
         </is>
       </c>
       <c r="B164" s="2">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="C164" s="0" t="inlineStr">
         <is>
@@ -8802,7 +8802,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjQsIm9mZmljZXJQYXkiOjAuMzYsImRlcHJlY2lhdGlvbiI6MS44LCJvdGhlclNnYSI6OSwiaGVhZGNvdW50Ijo5MCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4zNiwib2ZmaWNlclBheSI6MC41NSwiZGVwcmVjaWF0aW9uIjoxLjM4LCJvdGhlclNnYSI6Ny4zNiwiaGVhZGNvdW50IjoxMTkuNiwib2ZmaWNlckNvdW50IjozfX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjcsIm9mZmljZXJQYXkiOjAuMzgsImRlcHJlY2lhdGlvbiI6MS45LCJvdGhlclNnYSI6OS41LCJoZWFkY291bnQiOjk1LCJvZmZpY2VyQ291bnQiOjJ9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNjgsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI0LjgsIm9mZmljZXJDb3VudCI6M319LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6Niwib2ZmaWNlclBheSI6MC40LCJkZXByZWNpYXRpb24iOjIsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsIm9mZmljZXJQYXkiOjAuNiwiZGVwcmVjaWF0aW9uIjoxLjUsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjIxLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjowLjA3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjA3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAuMDEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA2LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wMSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMSwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MCwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDEsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDE1LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wOSwib3RoZXJTZ2FSYXRlRW5kIjowLjEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA2LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6NDUsInN1YnNpZHkiOjE1LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6Wy0wLjA1LDAuNF0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDJdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbLTAuMDUsMC4xXSwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6Wy0wLjAzLDAuMl0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMC4wMl0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjFdLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjpbLTAuMSwwLjJdLCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6WzAsMC4wMl0sIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlstMC4wNSwwLjFdLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAyXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbLTAuMDUsMC40XSwib3RoZXJTYWxlc0dyb3d0aCI6Wy0wLjEsMC4yXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMCwwLjAzXSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDQ1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMCwwLjA4XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6Wy0wLjAzLDAuMl0sIm90aGVySGVhZGNvdW50R3Jvd3RoIjpbLTAuMDUsMC4xXSwicHJvamVjdFNnYVJhdGVFbmQiOlswLjA0LDAuMjVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA0LDAuMjVdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAsMC4xXSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjEsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlQYXlTY2hlZHVsZSI6eyJ2YWx1ZSI6My41LCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NzAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjowLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5Q2FnciI6eyJ2YWx1ZSI6NywibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJpbnZlc3RtZW50U2FsZXNSYXRpbyI6eyJ2YWx1ZSI6MzAsIm1heCI6NzAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvIjp7InZhbHVlIjoyMTMsIm1heCI6MzUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibG9jYWxCZW5jaG1hcmsiOnsidmFsdWUiOjIzLCJtYXgiOjQwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUNhZ3IiOnsidmFsdWUiOjYsIm1heCI6MTAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnt9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2LjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mi43NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMzLjIxLCJhY3R1YWw6Y29tcGFueToyMDIzOjItOCI6MC45MSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTExIjoxMi43NiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE0IjozLjE4LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMSI6NzIsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny00IjoyMy4wNCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjYuNDgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny04Ijo1LjQsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny05IjowLjM2LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTAiOjEuOCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEzIjo5MCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMSI6MTQzLjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0zIjo5Ny4zOCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTciOjM0Ljg2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItOCI6MC45NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTExIjoxMy4zOCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjozLjM0LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMSI6NzYsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny00IjoyNC4zMiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTYiOjYuODQsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny04Ijo1LjcsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTAiOjEuOSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTgiOjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMSI6MTQsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6My41LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMSI6ODAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNS42LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6Ny4yLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTkiOjAuNCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEwIjoyLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTMiOjEwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTE0IjoyLCJiYWxhbmNlLXNoZWV0OjIwMjM6YXNzZXRzIjoxMzIsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NywiYmFsYW5jZS1zaGVldDoyMDIzOmNhc2giOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRBc3NldHMiOjY1LCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzLCJiYWxhbmNlLXNoZWV0OjIwMjM6YnVpbGRpbmdzIjoxOSwiYmFsYW5jZS1zaGVldDoyMDIzOm1hY2hpbmVyeSI6MjQsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmludGFuZ2libGVBc3NldHMiOjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzb2Z0d2FyZSI6NSwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NSwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRMaWFiaWxpdGllcyI6MzksImJhbGFuY2Utc2hlZXQ6MjAyMzpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2LCJiYWxhbmNlLXNoZWV0OjIwMjM6bG9uZ1Rlcm1EZWJ0IjoyOSwiYmFsYW5jZS1zaGVldDoyMDIzOm5ldEFzc2V0cyI6NTcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGV4Ijo1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50QXNzZXRzIjo3MiwiYmFsYW5jZS1zaGVldDoyMDI0OmNhc2giOjI1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6dGFuZ2libGVBc3NldHMiOjU4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YnVpbGRpbmdzIjoyMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmludGFuZ2libGVBc3NldHMiOjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NiwiYmFsYW5jZS1zaGVldDoyMDI0OmxpYWJpbGl0aWVzIjo3OSwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRMaWFiaWxpdGllcyI6NDEsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkTGlhYmlsaXRpZXMiOjM4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bG9uZ1Rlcm1EZWJ0IjozMSwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaGFyZWhvbGRlckVxdWl0eSI6NjEsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4LCJiYWxhbmNlLXNoZWV0OjIwMjU6YXNzZXRzIjoxNTYsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50QXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3LCJiYWxhbmNlLXNoZWV0OjIwMjU6Zml4ZWRBc3NldHMiOjc4LCJiYWxhbmNlLXNoZWV0OjIwMjU6dGFuZ2libGVBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMiwiYmFsYW5jZS1zaGVldDoyMDI1Om1hY2hpbmVyeSI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjksImJhbGFuY2Utc2hlZXQ6MjAyNTpzb2Z0d2FyZSI6NywiYmFsYW5jZS1zaGVldDoyMDI1OmxpYWJpbGl0aWVzIjo4MywiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaG9ydFRlcm1EZWJ0IjoxMSwiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkTGlhYmlsaXRpZXMiOjQwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMiwiYmFsYW5jZS1zaGVldDoyMDI1Om5ldEFzc2V0cyI6NzMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaGFyZWhvbGRlckVxdWl0eSI6NzAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGV4IjoxMCwiZnV0dXJlLWNhcGV4OjIwMjYiOjE1LCJmdXR1cmUtY2FwZXg6MjAyNyI6MTUsImZ1dHVyZS1jYXBleDoyMDI4IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjkiOjAsImZ1dHVyZS1jYXBleDoyMDMwIjowLCJmdXR1cmUtY2FwZXg6MjAzMSI6MCwiZHJpdmVyOnByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDoxIjowLjMsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMjEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6LTAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC40LCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MC4wNywiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZToxIjowLjEsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjotMC4wMywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4yLCJkcml2ZXI6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLjAxLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMiwiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA2LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMSwiZHJpdmVyOm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjAiOi0wLjEsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMiwiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAyLCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjAxLCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6LTAuMDUsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZToxIjowLjEsImRyaXZlcjpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMiwiZHJpdmVyOnByb2plY3RTYWxlc0dyb3d0aCI6MC4yMSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjQsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjotMC4xLCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjIsImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZToxIjowLjAzLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDEsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MSI6MC4wMywiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDQ1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDoxIjowLjEsImRyaXZlcjpvdGhlclBheUdyb3d0aCI6MC4wNDUsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wOCwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOi0wLjAzLCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aDoxIjowLjIsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wMTUsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjA5LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MCI6MC4wNCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjEiOjAuMjUsImRyaXZlcjpvdGhlclNnYVJhdGVFbmQiOjAuMSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLjA0LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMjUsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNiwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjEsImRyaXZlcjp1c2VmdWxMaWZlIjoxMCwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MCI6NSwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MSI6MjAsImRyaXZlcjppbnZlc3RtZW50Ijo0NSwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjEiOjIwMCwiZHJpdmVyOnN1YnNpZHkiOjE1LCJkcml2ZXItcmFuZ2U6c3Vic2lkeTowIjoxLCJkcml2ZXItcmFuZ2U6c3Vic2lkeToxIjo1MCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoyMSwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjowLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjozLjUsInRhcmdldDpjb21wYW55UGF5U2NoZWR1bGU6bWF4Ijo3LCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6dmFsdWUiOjcwLCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6bWF4Ijo5NSwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6dmFsdWUiOjIyLCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6dmFsdWUiOjIxLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOm1heCI6MzUsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDplbXBsb3llZVBheUNhZ3I6dmFsdWUiOjcsInRhcmdldDplbXBsb3llZVBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MzAsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjB9LCJtZXRyaWNHcm91cEJhc2VzIjp7ImNvbXBhbnlTYWxlcyI6InJhdGUiLCJwcm9qZWN0U2FsZXMiOiJyYXRlIiwibGFib3JQcm9kdWN0aXZpdHkiOiJyYXRlIiwiZW1wbG95ZWVQYXkiOiJyYXRlIn19</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjQsIm9mZmljZXJQYXkiOjAuMzYsImRlcHJlY2lhdGlvbiI6MS44LCJvdGhlclNnYSI6OSwiaGVhZGNvdW50Ijo5MCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4zNiwib2ZmaWNlclBheSI6MC41NSwiZGVwcmVjaWF0aW9uIjoxLjM4LCJvdGhlclNnYSI6Ny4zNiwiaGVhZGNvdW50IjoxMTkuNiwib2ZmaWNlckNvdW50IjozfX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjcsIm9mZmljZXJQYXkiOjAuMzgsImRlcHJlY2lhdGlvbiI6MS45LCJvdGhlclNnYSI6OS41LCJoZWFkY291bnQiOjk1LCJvZmZpY2VyQ291bnQiOjJ9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNjgsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI0LjgsIm9mZmljZXJDb3VudCI6M319LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6Niwib2ZmaWNlclBheSI6MC40LCJkZXByZWNpYXRpb24iOjIsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsIm9mZmljZXJQYXkiOjAuNiwiZGVwcmVjaWF0aW9uIjoxLjUsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjIxLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjowLjA3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjA3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAuMDEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA2LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wMSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMSwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNiwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MCwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDEsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDE1LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wOSwib3RoZXJTZ2FSYXRlRW5kIjowLjEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA2LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6NDUsInN1YnNpZHkiOjE1LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6Wy0wLjA1LDAuNF0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDJdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbLTAuMDUsMC4xXSwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6Wy0wLjAzLDAuMl0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMC4wMl0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjFdLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjpbLTAuMSwwLjJdLCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6WzAsMC4wMl0sIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlstMC4wNSwwLjFdLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAyXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbLTAuMDUsMC40XSwib3RoZXJTYWxlc0dyb3d0aCI6Wy0wLjEsMC4yXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMCwwLjAzXSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDQ1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMCwwLjA4XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6Wy0wLjAzLDAuMl0sIm90aGVySGVhZGNvdW50R3Jvd3RoIjpbLTAuMDUsMC4xXSwicHJvamVjdFNnYVJhdGVFbmQiOlswLjA0LDAuMjVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA0LDAuMjVdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAsMC4xXSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjEsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlQYXlTY2hlZHVsZSI6eyJ2YWx1ZSI6My41LCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NzAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjowLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5Q2FnciI6eyJ2YWx1ZSI6NywibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJpbnZlc3RtZW50U2FsZXNSYXRpbyI6eyJ2YWx1ZSI6MzAsIm1heCI6NzAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvIjp7InZhbHVlIjoyMTMsIm1heCI6MzUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibG9jYWxCZW5jaG1hcmsiOnsidmFsdWUiOjIzLCJtYXgiOjQwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUNhZ3IiOnsidmFsdWUiOjYsIm1heCI6MTAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnt9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2LjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mi43NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMzLjIxLCJhY3R1YWw6Y29tcGFueToyMDIzOjItOCI6MC45MSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTExIjoxMi43NiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE0IjozLjE4LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMSI6NzIsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny00IjoyMy4wNCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjYuNDgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny04Ijo1LjQsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny05IjowLjM2LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTAiOjEuOCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEzIjo5MCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMSI6MTQzLjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0zIjo5Ny4zOCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTciOjM0Ljg2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItOCI6MC45NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTExIjoxMy4zOCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjozLjM0LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMSI6NzYsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny00IjoyNC4zMiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTYiOjYuODQsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny04Ijo1LjcsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTAiOjEuOSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTgiOjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMSI6MTQsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6My41LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMSI6ODAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNS42LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6Ny4yLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTkiOjAuNCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEwIjoyLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTMiOjEwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTE0IjoyLCJiYWxhbmNlLXNoZWV0OjIwMjM6YXNzZXRzIjoxMzIsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NywiYmFsYW5jZS1zaGVldDoyMDIzOmNhc2giOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRBc3NldHMiOjY1LCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzLCJiYWxhbmNlLXNoZWV0OjIwMjM6YnVpbGRpbmdzIjoxOSwiYmFsYW5jZS1zaGVldDoyMDIzOm1hY2hpbmVyeSI6MjQsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmludGFuZ2libGVBc3NldHMiOjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzb2Z0d2FyZSI6NSwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NSwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRMaWFiaWxpdGllcyI6MzksImJhbGFuY2Utc2hlZXQ6MjAyMzpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2LCJiYWxhbmNlLXNoZWV0OjIwMjM6bG9uZ1Rlcm1EZWJ0IjoyOSwiYmFsYW5jZS1zaGVldDoyMDIzOm5ldEFzc2V0cyI6NTcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGV4Ijo1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50QXNzZXRzIjo3MiwiYmFsYW5jZS1zaGVldDoyMDI0OmNhc2giOjI1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6dGFuZ2libGVBc3NldHMiOjU4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YnVpbGRpbmdzIjoyMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmludGFuZ2libGVBc3NldHMiOjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NiwiYmFsYW5jZS1zaGVldDoyMDI0OmxpYWJpbGl0aWVzIjo3OSwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRMaWFiaWxpdGllcyI6NDEsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkTGlhYmlsaXRpZXMiOjM4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bG9uZ1Rlcm1EZWJ0IjozMSwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaGFyZWhvbGRlckVxdWl0eSI6NjEsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4LCJiYWxhbmNlLXNoZWV0OjIwMjU6YXNzZXRzIjoxNTYsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50QXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3LCJiYWxhbmNlLXNoZWV0OjIwMjU6Zml4ZWRBc3NldHMiOjc4LCJiYWxhbmNlLXNoZWV0OjIwMjU6dGFuZ2libGVBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMiwiYmFsYW5jZS1zaGVldDoyMDI1Om1hY2hpbmVyeSI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjksImJhbGFuY2Utc2hlZXQ6MjAyNTpzb2Z0d2FyZSI6NywiYmFsYW5jZS1zaGVldDoyMDI1OmxpYWJpbGl0aWVzIjo4MywiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaG9ydFRlcm1EZWJ0IjoxMSwiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkTGlhYmlsaXRpZXMiOjQwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMiwiYmFsYW5jZS1zaGVldDoyMDI1Om5ldEFzc2V0cyI6NzMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaGFyZWhvbGRlckVxdWl0eSI6NzAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGV4IjoxMCwiZnV0dXJlLWNhcGV4OjIwMjYiOjE1LCJmdXR1cmUtY2FwZXg6MjAyNyI6MTUsImZ1dHVyZS1jYXBleDoyMDI4IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjkiOjAsImZ1dHVyZS1jYXBleDoyMDMwIjowLCJmdXR1cmUtY2FwZXg6MjAzMSI6MCwiZHJpdmVyOnByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDoxIjowLjMsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMjEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6LTAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC40LCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MC4wNywiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZToxIjowLjEsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjotMC4wMywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4yLCJkcml2ZXI6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLjAxLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMiwiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA2LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMSwiZHJpdmVyOm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjAiOi0wLjEsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMiwiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAyLCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjAxLCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6LTAuMDUsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZToxIjowLjEsImRyaXZlcjpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMiwiZHJpdmVyOnByb2plY3RTYWxlc0dyb3d0aCI6MC4yMSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjQsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjotMC4xLCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjIsImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZToxIjowLjAzLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDEsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MSI6MC4wMywiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDQ1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDoxIjowLjEsImRyaXZlcjpvdGhlclBheUdyb3d0aCI6MC4wNDUsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wOCwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOi0wLjAzLCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aDoxIjowLjIsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wMTUsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjA5LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MCI6MC4wNCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjEiOjAuMjUsImRyaXZlcjpvdGhlclNnYVJhdGVFbmQiOjAuMSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLjA0LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMjUsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNiwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjEsImRyaXZlcjp1c2VmdWxMaWZlIjoxMCwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MCI6NSwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MSI6MjAsImRyaXZlcjppbnZlc3RtZW50Ijo0NSwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjEiOjIwMCwiZHJpdmVyOnN1YnNpZHkiOjE1LCJkcml2ZXItcmFuZ2U6c3Vic2lkeTowIjoxLCJkcml2ZXItcmFuZ2U6c3Vic2lkeToxIjo1MCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoyMSwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjowLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjozLjUsInRhcmdldDpjb21wYW55UGF5U2NoZWR1bGU6bWF4Ijo3LCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6dmFsdWUiOjcwLCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6bWF4Ijo5NSwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6dmFsdWUiOjIyLCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6dmFsdWUiOjIxLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOm1heCI6MzUsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDplbXBsb3llZVBheUNhZ3I6dmFsdWUiOjcsInRhcmdldDplbXBsb3llZVBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MzAsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjB9LCJtZXRyaWNHcm91cEJhc2VzIjp7ImNvbXBhbnlTYWxlcyI6InJhdGUiLCJwcm9qZWN0U2FsZXMiOiJyYXRlIiwibGFib3JQcm9kdWN0aXZpdHkiOiJyYXRlIiwiZW1wbG95ZWVQYXkiOiJyYXRlIn19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build completed standard proposal sample
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -204,7 +204,7 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <v>15.51906107932668</v>
+        <v>20.152518023637867</v>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
@@ -234,7 +234,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <v>107.63</v>
+        <v>127.10000000000002</v>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
@@ -264,7 +264,7 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <v>8.332988192871005</v>
+        <v>2.0136531491304233</v>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
@@ -294,7 +294,7 @@
         </is>
       </c>
       <c r="B11" s="2">
-        <v>69.38995332441166</v>
+        <v>67.97614287618285</v>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
@@ -324,7 +324,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>21.000508463435665</v>
+        <v>29.614246350044503</v>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
@@ -354,7 +354,7 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <v>92.59</v>
+        <v>110.32</v>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
@@ -384,7 +384,7 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <v>18.06480348374826</v>
+        <v>32.737848619973995</v>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
@@ -414,7 +414,7 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <v>25.279999999999994</v>
+        <v>28.59999999999998</v>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
@@ -444,7 +444,7 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <v>7.099090446266931</v>
+        <v>7.018093513861001</v>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B17" s="2">
-        <v>3.7799999999999994</v>
+        <v>2.3899999999999997</v>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B18" s="2">
-        <v>30</v>
+        <v>15.333333333333332</v>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <v>168.5333333333333</v>
+        <v>372.8813559322032</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B21" s="2">
-        <v>5.7715899735125475</v>
+        <v>5.379211308937237</v>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="B22" s="2">
-        <v>0.10999999999999999</v>
+        <v>0.08000000000000007</v>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
@@ -1259,22 +1259,22 @@
         <v>150</v>
       </c>
       <c r="E3" s="4">
-        <v>112.8</v>
+        <v>157.31</v>
       </c>
       <c r="F3" s="4">
-        <v>155.70999999999998</v>
+        <v>164.98000000000002</v>
       </c>
       <c r="G3" s="4">
-        <v>198.74</v>
+        <v>173.01999999999998</v>
       </c>
       <c r="H3" s="4">
-        <v>228.65999999999997</v>
+        <v>206.57</v>
       </c>
       <c r="I3" s="4">
-        <v>264.15999999999997</v>
+        <v>247.85000000000002</v>
       </c>
       <c r="J3" s="4">
-        <v>306.37</v>
+        <v>300.12</v>
       </c>
     </row>
     <row r="4">
@@ -1295,22 +1295,22 @@
         <v>4.748603351955305</v>
       </c>
       <c r="E4" s="2">
-        <v>-24.8</v>
+        <v>4.8733333333333295</v>
       </c>
       <c r="F4" s="2">
-        <v>38.04078014184395</v>
+        <v>4.875723094526752</v>
       </c>
       <c r="G4" s="2">
-        <v>27.63470554235441</v>
+        <v>4.873317977936686</v>
       </c>
       <c r="H4" s="2">
-        <v>15.054845526818927</v>
+        <v>19.39082187030401</v>
       </c>
       <c r="I4" s="2">
-        <v>15.525233971835917</v>
+        <v>19.983540688386526</v>
       </c>
       <c r="J4" s="2">
-        <v>15.978952150212011</v>
+        <v>21.089368569699406</v>
       </c>
     </row>
     <row r="5">
@@ -1329,22 +1329,22 @@
         <v>102</v>
       </c>
       <c r="E5" s="2">
-        <v>75.38</v>
+        <v>106.97</v>
       </c>
       <c r="F5" s="2">
-        <v>103.22999999999999</v>
+        <v>112.18</v>
       </c>
       <c r="G5" s="2">
-        <v>131.15</v>
+        <v>117.66</v>
       </c>
       <c r="H5" s="2">
-        <v>150.44</v>
+        <v>139.13</v>
       </c>
       <c r="I5" s="2">
-        <v>173.33</v>
+        <v>166</v>
       </c>
       <c r="J5" s="2">
-        <v>200.54000000000002</v>
+        <v>199.78000000000003</v>
       </c>
     </row>
     <row r="6">
@@ -1363,22 +1363,22 @@
         <v>0.8</v>
       </c>
       <c r="E6" s="2">
-        <v>0.3</v>
+        <v>0.99</v>
       </c>
       <c r="F6" s="2">
-        <v>0.3</v>
+        <v>1.18</v>
       </c>
       <c r="G6" s="2">
-        <v>0.3</v>
+        <v>1.37</v>
       </c>
       <c r="H6" s="2">
-        <v>0.3</v>
+        <v>1.37</v>
       </c>
       <c r="I6" s="2">
-        <v>0.3</v>
+        <v>1.37</v>
       </c>
       <c r="J6" s="2">
-        <v>0.3</v>
+        <v>1.37</v>
       </c>
     </row>
     <row r="7">
@@ -1397,22 +1397,22 @@
         <v>48</v>
       </c>
       <c r="E7" s="4">
-        <v>37.42</v>
+        <v>50.34</v>
       </c>
       <c r="F7" s="4">
-        <v>52.47999999999999</v>
+        <v>52.80000000000001</v>
       </c>
       <c r="G7" s="4">
-        <v>67.59</v>
+        <v>55.359999999999985</v>
       </c>
       <c r="H7" s="4">
-        <v>78.21999999999997</v>
+        <v>67.44</v>
       </c>
       <c r="I7" s="4">
-        <v>90.82999999999996</v>
+        <v>81.85000000000002</v>
       </c>
       <c r="J7" s="4">
-        <v>105.82999999999998</v>
+        <v>100.33999999999997</v>
       </c>
     </row>
     <row r="8">
@@ -1431,22 +1431,22 @@
         <v>32</v>
       </c>
       <c r="E8" s="2">
-        <v>33.17375886524823</v>
+        <v>32.00050854999682</v>
       </c>
       <c r="F8" s="2">
-        <v>33.703679917795895</v>
+        <v>32.00387925809189</v>
       </c>
       <c r="G8" s="2">
-        <v>34.009258327463016</v>
+        <v>31.99630100566408</v>
       </c>
       <c r="H8" s="2">
-        <v>34.20799440216915</v>
+        <v>32.64752868277097</v>
       </c>
       <c r="I8" s="2">
-        <v>34.3844639612356</v>
+        <v>33.02400645551746</v>
       </c>
       <c r="J8" s="2">
-        <v>34.543199399419</v>
+        <v>33.433293349326924</v>
       </c>
     </row>
     <row r="9">
@@ -1465,22 +1465,22 @@
         <v>36.4</v>
       </c>
       <c r="E9" s="2">
-        <v>28.43</v>
+        <v>38.87</v>
       </c>
       <c r="F9" s="2">
-        <v>38.8</v>
+        <v>41.449999999999996</v>
       </c>
       <c r="G9" s="2">
-        <v>49.19</v>
+        <v>44.19</v>
       </c>
       <c r="H9" s="2">
-        <v>53.269999999999996</v>
+        <v>48.489999999999995</v>
       </c>
       <c r="I9" s="2">
-        <v>57.82</v>
+        <v>53.92999999999999</v>
       </c>
       <c r="J9" s="2">
-        <v>62.93</v>
+        <v>60.18</v>
       </c>
     </row>
     <row r="10">
@@ -1499,22 +1499,22 @@
         <v>1</v>
       </c>
       <c r="E10" s="2">
-        <v>0.8200000000000001</v>
+        <v>1.03</v>
       </c>
       <c r="F10" s="2">
-        <v>1.05</v>
+        <v>1.06</v>
       </c>
       <c r="G10" s="2">
-        <v>1.27</v>
+        <v>1.1099999999999999</v>
       </c>
       <c r="H10" s="2">
-        <v>1.35</v>
+        <v>1.15</v>
       </c>
       <c r="I10" s="2">
-        <v>1.4100000000000001</v>
+        <v>1.19</v>
       </c>
       <c r="J10" s="2">
-        <v>1.48</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="11">
@@ -1533,22 +1533,22 @@
         <v>0.9</v>
       </c>
       <c r="E11" s="2">
-        <v>0.76</v>
+        <v>0.93</v>
       </c>
       <c r="F11" s="2">
-        <v>0.99</v>
+        <v>0.9600000000000001</v>
       </c>
       <c r="G11" s="2">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="H11" s="2">
-        <v>1.28</v>
+        <v>1.04</v>
       </c>
       <c r="I11" s="2">
-        <v>1.34</v>
+        <v>1.06</v>
       </c>
       <c r="J11" s="2">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="12">
@@ -1567,22 +1567,22 @@
         <v>0.1</v>
       </c>
       <c r="E12" s="2">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="F12" s="2">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="G12" s="2">
-        <v>0.07</v>
+        <v>0.11</v>
       </c>
       <c r="H12" s="2">
-        <v>0.07</v>
+        <v>0.11</v>
       </c>
       <c r="I12" s="2">
-        <v>0.07</v>
+        <v>0.13</v>
       </c>
       <c r="J12" s="2">
-        <v>0.08</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="13">
@@ -1601,22 +1601,22 @@
         <v>14</v>
       </c>
       <c r="E13" s="2">
-        <v>11.73</v>
+        <v>14.95</v>
       </c>
       <c r="F13" s="2">
-        <v>15.5</v>
+        <v>15.96</v>
       </c>
       <c r="G13" s="2">
-        <v>19.27</v>
+        <v>17.06</v>
       </c>
       <c r="H13" s="2">
-        <v>20.96</v>
+        <v>18.16</v>
       </c>
       <c r="I13" s="2">
-        <v>22.810000000000002</v>
+        <v>19.83</v>
       </c>
       <c r="J13" s="2">
-        <v>24.84</v>
+        <v>21.66</v>
       </c>
     </row>
     <row r="14">
@@ -1635,22 +1635,22 @@
         <v>13.3</v>
       </c>
       <c r="E14" s="2">
-        <v>11.31</v>
+        <v>14.2</v>
       </c>
       <c r="F14" s="2">
-        <v>15.06</v>
+        <v>15.16</v>
       </c>
       <c r="G14" s="2">
-        <v>18.810000000000002</v>
+        <v>16.21</v>
       </c>
       <c r="H14" s="2">
-        <v>20.47</v>
+        <v>17.7</v>
       </c>
       <c r="I14" s="2">
-        <v>22.29</v>
+        <v>19.33</v>
       </c>
       <c r="J14" s="2">
-        <v>24.29</v>
+        <v>21.12</v>
       </c>
     </row>
     <row r="15">
@@ -1669,22 +1669,22 @@
         <v>0.7</v>
       </c>
       <c r="E15" s="2">
-        <v>0.42</v>
+        <v>0.75</v>
       </c>
       <c r="F15" s="2">
-        <v>0.44</v>
+        <v>0.8</v>
       </c>
       <c r="G15" s="2">
-        <v>0.46</v>
+        <v>0.85</v>
       </c>
       <c r="H15" s="2">
-        <v>0.49</v>
+        <v>0.9199999999999999</v>
       </c>
       <c r="I15" s="2">
-        <v>0.52</v>
+        <v>1.01</v>
       </c>
       <c r="J15" s="2">
-        <v>0.55</v>
+        <v>1.1099999999999999</v>
       </c>
     </row>
     <row r="16">
@@ -1703,22 +1703,22 @@
         <v>2.7</v>
       </c>
       <c r="E16" s="2">
-        <v>3.37</v>
+        <v>3.2800000000000002</v>
       </c>
       <c r="F16" s="2">
-        <v>5.53</v>
+        <v>3.8499999999999996</v>
       </c>
       <c r="G16" s="2">
-        <v>7.7</v>
+        <v>4.43</v>
       </c>
       <c r="H16" s="2">
-        <v>7.7</v>
+        <v>4.43</v>
       </c>
       <c r="I16" s="2">
-        <v>7.7</v>
+        <v>4.43</v>
       </c>
       <c r="J16" s="2">
-        <v>7.7</v>
+        <v>4.43</v>
       </c>
     </row>
     <row r="17">
@@ -1737,22 +1737,22 @@
         <v>0.7</v>
       </c>
       <c r="E17" s="2">
-        <v>0.31</v>
+        <v>0.73</v>
       </c>
       <c r="F17" s="2">
-        <v>0.32</v>
+        <v>0.77</v>
       </c>
       <c r="G17" s="2">
-        <v>0.34</v>
+        <v>0.81</v>
       </c>
       <c r="H17" s="2">
-        <v>0.36</v>
+        <v>0.97</v>
       </c>
       <c r="I17" s="2">
-        <v>0.38</v>
+        <v>1.17</v>
       </c>
       <c r="J17" s="2">
-        <v>0.4</v>
+        <v>1.43</v>
       </c>
     </row>
     <row r="18">
@@ -1771,22 +1771,22 @@
         <v>11.600000000000001</v>
       </c>
       <c r="E18" s="4">
-        <v>8.990000000000002</v>
+        <v>11.469999999999999</v>
       </c>
       <c r="F18" s="4">
-        <v>13.679999999999993</v>
+        <v>11.350000000000009</v>
       </c>
       <c r="G18" s="4">
-        <v>18.4</v>
+        <v>11.169999999999984</v>
       </c>
       <c r="H18" s="4">
-        <v>24.949999999999967</v>
+        <v>18.950000000000003</v>
       </c>
       <c r="I18" s="4">
-        <v>33.009999999999955</v>
+        <v>27.920000000000027</v>
       </c>
       <c r="J18" s="4">
-        <v>42.89999999999997</v>
+        <v>40.159999999999975</v>
       </c>
     </row>
     <row r="19">
@@ -1805,22 +1805,22 @@
         <v>7.733333333333333</v>
       </c>
       <c r="E19" s="2">
-        <v>7.969858156028371</v>
+        <v>7.291335579429152</v>
       </c>
       <c r="F19" s="2">
-        <v>8.785562905401061</v>
+        <v>6.879621772336045</v>
       </c>
       <c r="G19" s="2">
-        <v>9.258327463017006</v>
+        <v>6.455901051901505</v>
       </c>
       <c r="H19" s="2">
-        <v>10.911396833726918</v>
+        <v>9.173645737522392</v>
       </c>
       <c r="I19" s="2">
-        <v>12.496214415505738</v>
+        <v>11.26487795037322</v>
       </c>
       <c r="J19" s="2">
-        <v>14.002676502268487</v>
+        <v>13.381314141010254</v>
       </c>
     </row>
     <row r="20">
@@ -1839,22 +1839,22 @@
         <v>11.600000000000001</v>
       </c>
       <c r="E20" s="4">
-        <v>8.990000000000002</v>
+        <v>11.469999999999999</v>
       </c>
       <c r="F20" s="4">
-        <v>13.679999999999993</v>
+        <v>11.350000000000009</v>
       </c>
       <c r="G20" s="4">
-        <v>18.4</v>
+        <v>11.169999999999984</v>
       </c>
       <c r="H20" s="4">
-        <v>24.949999999999967</v>
+        <v>18.950000000000003</v>
       </c>
       <c r="I20" s="4">
-        <v>33.009999999999955</v>
+        <v>27.920000000000027</v>
       </c>
       <c r="J20" s="4">
-        <v>42.89999999999997</v>
+        <v>40.159999999999975</v>
       </c>
     </row>
     <row r="21">
@@ -1977,22 +1977,22 @@
         <v>14</v>
       </c>
       <c r="E23" s="2">
-        <v>11.73</v>
+        <v>14.95</v>
       </c>
       <c r="F23" s="2">
-        <v>15.5</v>
+        <v>15.96</v>
       </c>
       <c r="G23" s="2">
-        <v>19.27</v>
+        <v>17.06</v>
       </c>
       <c r="H23" s="2">
-        <v>20.96</v>
+        <v>18.16</v>
       </c>
       <c r="I23" s="2">
-        <v>22.810000000000002</v>
+        <v>19.83</v>
       </c>
       <c r="J23" s="2">
-        <v>24.84</v>
+        <v>21.66</v>
       </c>
     </row>
     <row r="24">
@@ -2011,22 +2011,22 @@
         <v>1</v>
       </c>
       <c r="E24" s="2">
-        <v>0.8200000000000001</v>
+        <v>1.03</v>
       </c>
       <c r="F24" s="2">
-        <v>1.05</v>
+        <v>1.06</v>
       </c>
       <c r="G24" s="2">
-        <v>1.27</v>
+        <v>1.1099999999999999</v>
       </c>
       <c r="H24" s="2">
-        <v>1.35</v>
+        <v>1.15</v>
       </c>
       <c r="I24" s="2">
-        <v>1.4100000000000001</v>
+        <v>1.19</v>
       </c>
       <c r="J24" s="2">
-        <v>1.48</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="25">
@@ -2045,22 +2045,22 @@
         <v>3.5</v>
       </c>
       <c r="E25" s="2">
-        <v>3.67</v>
+        <v>4.27</v>
       </c>
       <c r="F25" s="2">
-        <v>5.83</v>
+        <v>5.029999999999999</v>
       </c>
       <c r="G25" s="2">
-        <v>8</v>
+        <v>5.8</v>
       </c>
       <c r="H25" s="2">
-        <v>8</v>
+        <v>5.8</v>
       </c>
       <c r="I25" s="2">
-        <v>8</v>
+        <v>5.8</v>
       </c>
       <c r="J25" s="2">
-        <v>8</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="26">
@@ -2079,22 +2079,22 @@
         <v>30.1</v>
       </c>
       <c r="E26" s="4">
-        <v>25.21</v>
+        <v>31.72</v>
       </c>
       <c r="F26" s="4">
-        <v>36.059999999999995</v>
+        <v>33.400000000000006</v>
       </c>
       <c r="G26" s="4">
-        <v>46.940000000000005</v>
+        <v>35.13999999999998</v>
       </c>
       <c r="H26" s="4">
-        <v>55.25999999999997</v>
+        <v>44.059999999999995</v>
       </c>
       <c r="I26" s="4">
-        <v>65.22999999999996</v>
+        <v>54.74000000000002</v>
       </c>
       <c r="J26" s="4">
-        <v>77.21999999999997</v>
+        <v>68.84999999999998</v>
       </c>
     </row>
     <row r="27">
@@ -2115,22 +2115,22 @@
         <v>4.768534632788035</v>
       </c>
       <c r="E27" s="2">
-        <v>-16.24584717607973</v>
+        <v>5.3820598006644405</v>
       </c>
       <c r="F27" s="2">
-        <v>43.03847679492263</v>
+        <v>5.29634300126105</v>
       </c>
       <c r="G27" s="2">
-        <v>30.17193566278429</v>
+        <v>5.20958083832328</v>
       </c>
       <c r="H27" s="2">
-        <v>17.724755006391057</v>
+        <v>25.384177575412693</v>
       </c>
       <c r="I27" s="2">
-        <v>18.041983351429593</v>
+        <v>24.23967317294604</v>
       </c>
       <c r="J27" s="2">
-        <v>18.381112984822966</v>
+        <v>25.776397515527872</v>
       </c>
     </row>
     <row r="28">
@@ -2149,22 +2149,22 @@
         <v>20.06666666666667</v>
       </c>
       <c r="E28" s="2">
-        <v>22.349290780141846</v>
+        <v>20.164007373974954</v>
       </c>
       <c r="F28" s="2">
-        <v>23.15843555327211</v>
+        <v>20.244878167050555</v>
       </c>
       <c r="G28" s="2">
-        <v>23.618798430109692</v>
+        <v>20.309790775632866</v>
       </c>
       <c r="H28" s="2">
-        <v>24.166885331933866</v>
+        <v>21.32933146149005</v>
       </c>
       <c r="I28" s="2">
-        <v>24.69336765596607</v>
+        <v>22.085939076054075</v>
       </c>
       <c r="J28" s="2">
-        <v>25.204817704083286</v>
+        <v>22.940823670531778</v>
       </c>
     </row>
     <row r="29">
@@ -2183,22 +2183,22 @@
         <v>230</v>
       </c>
       <c r="E29" s="2">
-        <v>169</v>
+        <v>240</v>
       </c>
       <c r="F29" s="2">
-        <v>210</v>
+        <v>252</v>
       </c>
       <c r="G29" s="2">
-        <v>249</v>
+        <v>264</v>
       </c>
       <c r="H29" s="2">
-        <v>256</v>
+        <v>274</v>
       </c>
       <c r="I29" s="2">
-        <v>262</v>
+        <v>284</v>
       </c>
       <c r="J29" s="2">
-        <v>269</v>
+        <v>294</v>
       </c>
     </row>
     <row r="30">
@@ -2251,22 +2251,22 @@
         <v>0.06086956521739131</v>
       </c>
       <c r="E31" s="2">
-        <v>0.06940828402366864</v>
+        <v>0.06229166666666666</v>
       </c>
       <c r="F31" s="2">
-        <v>0.07380952380952381</v>
+        <v>0.06333333333333334</v>
       </c>
       <c r="G31" s="2">
-        <v>0.07738955823293173</v>
+        <v>0.06462121212121212</v>
       </c>
       <c r="H31" s="2">
-        <v>0.081875</v>
+        <v>0.06627737226277372</v>
       </c>
       <c r="I31" s="2">
-        <v>0.08706106870229008</v>
+        <v>0.06982394366197182</v>
       </c>
       <c r="J31" s="2">
-        <v>0.09234200743494424</v>
+        <v>0.0736734693877551</v>
       </c>
     </row>
     <row r="32">
@@ -2287,22 +2287,22 @@
         <v>1.9901321235802572</v>
       </c>
       <c r="E32" s="2">
-        <v>14.027895181741323</v>
+        <v>2.336309523809521</v>
       </c>
       <c r="F32" s="2">
-        <v>6.3410871595014795</v>
+        <v>1.6722408026756064</v>
       </c>
       <c r="G32" s="2">
-        <v>4.850369218810724</v>
+        <v>2.0334928229664984</v>
       </c>
       <c r="H32" s="2">
-        <v>5.795926310326949</v>
+        <v>2.562873841572455</v>
       </c>
       <c r="I32" s="2">
-        <v>6.334129712720693</v>
+        <v>5.3511044239002326</v>
       </c>
       <c r="J32" s="2">
-        <v>6.0657867073888205</v>
+        <v>5.513188634001254</v>
       </c>
     </row>
     <row r="33">
@@ -2321,22 +2321,22 @@
         <v>0.2</v>
       </c>
       <c r="E33" s="2">
-        <v>0.164</v>
+        <v>0.20600000000000002</v>
       </c>
       <c r="F33" s="2">
-        <v>0.21000000000000002</v>
+        <v>0.21200000000000002</v>
       </c>
       <c r="G33" s="2">
-        <v>0.254</v>
+        <v>0.22199999999999998</v>
       </c>
       <c r="H33" s="2">
-        <v>0.27</v>
+        <v>0.22999999999999998</v>
       </c>
       <c r="I33" s="2">
-        <v>0.28200000000000003</v>
+        <v>0.238</v>
       </c>
       <c r="J33" s="2">
-        <v>0.296</v>
+        <v>0.246</v>
       </c>
     </row>
     <row r="34">
@@ -2357,22 +2357,22 @@
         <v>4.166666666666674</v>
       </c>
       <c r="E34" s="2">
-        <v>-18.000000000000004</v>
+        <v>3.0000000000000027</v>
       </c>
       <c r="F34" s="2">
-        <v>28.04878048780488</v>
+        <v>2.9126213592232997</v>
       </c>
       <c r="G34" s="2">
-        <v>20.952380952380945</v>
+        <v>4.7169811320754595</v>
       </c>
       <c r="H34" s="2">
-        <v>6.299212598425208</v>
+        <v>3.603603603603611</v>
       </c>
       <c r="I34" s="2">
-        <v>4.444444444444451</v>
+        <v>3.4782608695652195</v>
       </c>
       <c r="J34" s="2">
-        <v>4.964539007092172</v>
+        <v>3.3613445378151363</v>
       </c>
     </row>
     <row r="35">
@@ -2391,22 +2391,22 @@
         <v>0.12808510638297874</v>
       </c>
       <c r="E35" s="2">
-        <v>0.14488505747126437</v>
+        <v>0.12946938775510203</v>
       </c>
       <c r="F35" s="2">
-        <v>0.16772093023255813</v>
+        <v>0.12996108949416343</v>
       </c>
       <c r="G35" s="2">
-        <v>0.18480314960629923</v>
+        <v>0.13063197026022297</v>
       </c>
       <c r="H35" s="2">
-        <v>0.21172413793103437</v>
+        <v>0.157921146953405</v>
       </c>
       <c r="I35" s="2">
-        <v>0.24430711610486877</v>
+        <v>0.18941176470588245</v>
       </c>
       <c r="J35" s="2">
-        <v>0.28182481751824806</v>
+        <v>0.23026755852842803</v>
       </c>
     </row>
     <row r="36">
@@ -2425,22 +2425,22 @@
         <v>15.100000000000001</v>
       </c>
       <c r="E36" s="4">
-        <v>12.660000000000002</v>
+        <v>15.739999999999998</v>
       </c>
       <c r="F36" s="4">
-        <v>19.50999999999999</v>
+        <v>16.38000000000001</v>
       </c>
       <c r="G36" s="4">
-        <v>26.4</v>
+        <v>16.969999999999985</v>
       </c>
       <c r="H36" s="4">
-        <v>32.94999999999997</v>
+        <v>24.750000000000004</v>
       </c>
       <c r="I36" s="4">
-        <v>41.009999999999955</v>
+        <v>33.72000000000003</v>
       </c>
       <c r="J36" s="4">
-        <v>50.89999999999997</v>
+        <v>45.95999999999997</v>
       </c>
     </row>
     <row r="37">
@@ -2459,22 +2459,22 @@
         <v>10.066666666666668</v>
       </c>
       <c r="E37" s="2">
-        <v>11.223404255319151</v>
+        <v>10.005721187464243</v>
       </c>
       <c r="F37" s="2">
-        <v>12.529702652366575</v>
+        <v>9.928476178930785</v>
       </c>
       <c r="G37" s="2">
-        <v>13.28368722954614</v>
+        <v>9.808114668824405</v>
       </c>
       <c r="H37" s="2">
-        <v>14.410041109070223</v>
+        <v>11.981410659824759</v>
       </c>
       <c r="I37" s="2">
-        <v>15.524682010902469</v>
+        <v>13.605003026023816</v>
       </c>
       <c r="J37" s="2">
-        <v>16.613898227633246</v>
+        <v>15.313874450219902</v>
       </c>
     </row>
     <row r="38">
@@ -2495,22 +2495,22 @@
         <v>3.1420765027322606</v>
       </c>
       <c r="E38" s="2">
-        <v>-16.158940397350985</v>
+        <v>4.238410596026476</v>
       </c>
       <c r="F38" s="2">
-        <v>54.107424960505426</v>
+        <v>4.066073697585848</v>
       </c>
       <c r="G38" s="2">
-        <v>35.315222962583334</v>
+        <v>3.601953601953456</v>
       </c>
       <c r="H38" s="2">
-        <v>24.810606060605945</v>
+        <v>45.84560989982338</v>
       </c>
       <c r="I38" s="2">
-        <v>24.46130500758723</v>
+        <v>36.24242424242434</v>
       </c>
       <c r="J38" s="2">
-        <v>24.116069251402152</v>
+        <v>36.298932384341455</v>
       </c>
     </row>
   </sheetData>
@@ -2663,22 +2663,22 @@
         <v>80</v>
       </c>
       <c r="E3" s="4">
-        <v>40</v>
+        <v>84.33</v>
       </c>
       <c r="F3" s="4">
-        <v>80</v>
+        <v>88.89</v>
       </c>
       <c r="G3" s="4">
-        <v>120</v>
+        <v>93.69</v>
       </c>
       <c r="H3" s="4">
-        <v>145.2</v>
+        <v>121.44</v>
       </c>
       <c r="I3" s="4">
-        <v>175.69</v>
+        <v>157.4</v>
       </c>
       <c r="J3" s="4">
-        <v>212.59</v>
+        <v>204.01</v>
       </c>
     </row>
     <row r="4">
@@ -2699,22 +2699,22 @@
         <v>5.263157894736836</v>
       </c>
       <c r="E4" s="2">
-        <v>-50</v>
+        <v>5.412499999999998</v>
       </c>
       <c r="F4" s="2">
-        <v>100</v>
+        <v>5.407328352899321</v>
       </c>
       <c r="G4" s="2">
-        <v>50</v>
+        <v>5.39993250084374</v>
       </c>
       <c r="H4" s="2">
-        <v>20.999999999999996</v>
+        <v>29.618956131924424</v>
       </c>
       <c r="I4" s="2">
-        <v>20.998622589531692</v>
+        <v>29.61133069828723</v>
       </c>
       <c r="J4" s="2">
-        <v>21.002902840229964</v>
+        <v>29.61245235069885</v>
       </c>
     </row>
     <row r="5">
@@ -2733,22 +2733,22 @@
         <v>53.333333333333336</v>
       </c>
       <c r="E5" s="2">
-        <v>35.46099290780142</v>
+        <v>53.60752653995296</v>
       </c>
       <c r="F5" s="2">
-        <v>51.37756085029864</v>
+        <v>53.87925809188992</v>
       </c>
       <c r="G5" s="2">
-        <v>60.38039649793701</v>
+        <v>54.14980927060456</v>
       </c>
       <c r="H5" s="2">
-        <v>63.50039359748097</v>
+        <v>58.788788304206804</v>
       </c>
       <c r="I5" s="2">
-        <v>66.50893397940642</v>
+        <v>63.50615291506959</v>
       </c>
       <c r="J5" s="2">
-        <v>69.38995332441166</v>
+        <v>67.97614287618285</v>
       </c>
     </row>
     <row r="6">
@@ -2767,22 +2767,22 @@
         <v>25.6</v>
       </c>
       <c r="E6" s="4">
-        <v>14</v>
+        <v>26.989999999999995</v>
       </c>
       <c r="F6" s="4">
-        <v>28</v>
+        <v>28.450000000000003</v>
       </c>
       <c r="G6" s="4">
-        <v>42</v>
+        <v>29.979999999999997</v>
       </c>
       <c r="H6" s="4">
-        <v>50.81999999999999</v>
+        <v>39.489999999999995</v>
       </c>
       <c r="I6" s="4">
-        <v>61.489999999999995</v>
+        <v>52</v>
       </c>
       <c r="J6" s="4">
-        <v>74.41</v>
+        <v>68.45999999999998</v>
       </c>
     </row>
     <row r="7">
@@ -2801,22 +2801,22 @@
         <v>32</v>
       </c>
       <c r="E7" s="2">
-        <v>35</v>
+        <v>32.005217597533495</v>
       </c>
       <c r="F7" s="2">
-        <v>35</v>
+        <v>32.00584992687592</v>
       </c>
       <c r="G7" s="2">
-        <v>35</v>
+        <v>31.999146120183582</v>
       </c>
       <c r="H7" s="2">
-        <v>35</v>
+        <v>32.51811594202898</v>
       </c>
       <c r="I7" s="2">
-        <v>34.99914622346177</v>
+        <v>33.03684879288437</v>
       </c>
       <c r="J7" s="2">
-        <v>35.00164636154099</v>
+        <v>33.557178569677944</v>
       </c>
     </row>
     <row r="8">
@@ -2835,22 +2835,22 @@
         <v>7.300000000000004</v>
       </c>
       <c r="E8" s="4">
-        <v>4.300000000000001</v>
+        <v>7.079999999999991</v>
       </c>
       <c r="F8" s="4">
-        <v>8.600000000000001</v>
+        <v>6.870000000000001</v>
       </c>
       <c r="G8" s="4">
-        <v>12.899999999999999</v>
+        <v>6.629999999999999</v>
       </c>
       <c r="H8" s="4">
-        <v>18.50999999999999</v>
+        <v>12.969999999999995</v>
       </c>
       <c r="I8" s="4">
-        <v>25.539999999999992</v>
+        <v>21.26</v>
       </c>
       <c r="J8" s="4">
-        <v>34.28999999999999</v>
+        <v>32.759999999999984</v>
       </c>
     </row>
     <row r="9">
@@ -2869,22 +2869,22 @@
         <v>9.125000000000005</v>
       </c>
       <c r="E9" s="2">
-        <v>10.750000000000002</v>
+        <v>8.395588758448941</v>
       </c>
       <c r="F9" s="2">
-        <v>10.750000000000002</v>
+        <v>7.728653391832603</v>
       </c>
       <c r="G9" s="2">
-        <v>10.749999999999998</v>
+        <v>7.076528978546269</v>
       </c>
       <c r="H9" s="2">
-        <v>12.747933884297517</v>
+        <v>10.68017127799736</v>
       </c>
       <c r="I9" s="2">
-        <v>14.536968524104953</v>
+        <v>13.506988564167727</v>
       </c>
       <c r="J9" s="2">
-        <v>16.129639211628014</v>
+        <v>16.058036370766132</v>
       </c>
     </row>
     <row r="10">
@@ -2903,22 +2903,22 @@
         <v>6</v>
       </c>
       <c r="E10" s="2">
-        <v>3.33</v>
+        <v>6.45</v>
       </c>
       <c r="F10" s="2">
-        <v>6.67</v>
+        <v>6.94</v>
       </c>
       <c r="G10" s="2">
-        <v>10</v>
+        <v>7.47</v>
       </c>
       <c r="H10" s="2">
-        <v>11.13</v>
+        <v>7.89</v>
       </c>
       <c r="I10" s="2">
-        <v>12.38</v>
+        <v>8.82</v>
       </c>
       <c r="J10" s="2">
-        <v>13.78</v>
+        <v>9.86</v>
       </c>
     </row>
     <row r="11">
@@ -2937,22 +2937,22 @@
         <v>0.4</v>
       </c>
       <c r="E11" s="2">
-        <v>0.2</v>
+        <v>0.42</v>
       </c>
       <c r="F11" s="2">
-        <v>0.4</v>
+        <v>0.44</v>
       </c>
       <c r="G11" s="2">
-        <v>0.6</v>
+        <v>0.47</v>
       </c>
       <c r="H11" s="2">
-        <v>0.64</v>
+        <v>0.5</v>
       </c>
       <c r="I11" s="2">
-        <v>0.67</v>
+        <v>0.52</v>
       </c>
       <c r="J11" s="2">
-        <v>0.71</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="12">
@@ -2971,22 +2971,22 @@
         <v>2</v>
       </c>
       <c r="E12" s="2">
-        <v>2.17</v>
+        <v>2.77</v>
       </c>
       <c r="F12" s="2">
-        <v>4.33</v>
+        <v>3.53</v>
       </c>
       <c r="G12" s="2">
-        <v>6.5</v>
+        <v>4.3</v>
       </c>
       <c r="H12" s="2">
-        <v>6.5</v>
+        <v>4.3</v>
       </c>
       <c r="I12" s="2">
-        <v>6.5</v>
+        <v>4.3</v>
       </c>
       <c r="J12" s="2">
-        <v>6.5</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="13">
@@ -3005,22 +3005,22 @@
         <v>15.700000000000005</v>
       </c>
       <c r="E13" s="4">
-        <v>10</v>
+        <v>16.71999999999999</v>
       </c>
       <c r="F13" s="4">
-        <v>20</v>
+        <v>17.78</v>
       </c>
       <c r="G13" s="4">
-        <v>30</v>
+        <v>18.869999999999997</v>
       </c>
       <c r="H13" s="4">
-        <v>36.779999999999994</v>
+        <v>25.659999999999997</v>
       </c>
       <c r="I13" s="4">
-        <v>45.089999999999996</v>
+        <v>34.9</v>
       </c>
       <c r="J13" s="4">
-        <v>55.279999999999994</v>
+        <v>47.46999999999998</v>
       </c>
     </row>
     <row r="14">
@@ -3041,22 +3041,22 @@
         <v>5.2984574111334615</v>
       </c>
       <c r="E14" s="2">
-        <v>-36.305732484076444</v>
+        <v>6.496815286624114</v>
       </c>
       <c r="F14" s="2">
-        <v>100</v>
+        <v>6.339712918660356</v>
       </c>
       <c r="G14" s="2">
-        <v>50</v>
+        <v>6.13048368953879</v>
       </c>
       <c r="H14" s="2">
-        <v>22.599999999999977</v>
+        <v>35.9830418653948</v>
       </c>
       <c r="I14" s="2">
-        <v>22.59380097879282</v>
+        <v>36.00935307872175</v>
       </c>
       <c r="J14" s="2">
-        <v>22.59924595253937</v>
+        <v>36.01719197707731</v>
       </c>
     </row>
     <row r="15">
@@ -3075,22 +3075,22 @@
         <v>100</v>
       </c>
       <c r="E15" s="2">
-        <v>38</v>
+        <v>105</v>
       </c>
       <c r="F15" s="2">
-        <v>77</v>
+        <v>111</v>
       </c>
       <c r="G15" s="2">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H15" s="2">
         <v>120</v>
       </c>
       <c r="I15" s="2">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J15" s="2">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="16">
@@ -3143,22 +3143,22 @@
         <v>0.06</v>
       </c>
       <c r="E17" s="2">
-        <v>0.08763157894736842</v>
+        <v>0.06142857142857143</v>
       </c>
       <c r="F17" s="2">
-        <v>0.08662337662337662</v>
+        <v>0.06252252252252252</v>
       </c>
       <c r="G17" s="2">
-        <v>0.08695652173913043</v>
+        <v>0.06384615384615384</v>
       </c>
       <c r="H17" s="2">
-        <v>0.09275000000000001</v>
+        <v>0.06575</v>
       </c>
       <c r="I17" s="2">
-        <v>0.09983870967741935</v>
+        <v>0.07170731707317074</v>
       </c>
       <c r="J17" s="2">
-        <v>0.10682170542635658</v>
+        <v>0.07825396825396826</v>
       </c>
     </row>
     <row r="18">
@@ -3179,22 +3179,22 @@
         <v>1.9677996422182487</v>
       </c>
       <c r="E18" s="2">
-        <v>46.05263157894737</v>
+        <v>2.3809523809523947</v>
       </c>
       <c r="F18" s="2">
-        <v>-1.1505011505011598</v>
+        <v>1.780850618059926</v>
       </c>
       <c r="G18" s="2">
-        <v>0.3845903135388795</v>
+        <v>2.1170472179117716</v>
       </c>
       <c r="H18" s="2">
-        <v>6.662500000000016</v>
+        <v>2.9819277108433795</v>
       </c>
       <c r="I18" s="2">
-        <v>7.642813668376647</v>
+        <v>9.060558286191235</v>
       </c>
       <c r="J18" s="2">
-        <v>6.994276840615643</v>
+        <v>9.129683619479522</v>
       </c>
     </row>
     <row r="19">
@@ -3213,22 +3213,22 @@
         <v>0.2</v>
       </c>
       <c r="E19" s="2">
-        <v>0.1</v>
+        <v>0.21</v>
       </c>
       <c r="F19" s="2">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="G19" s="2">
-        <v>0.3</v>
+        <v>0.235</v>
       </c>
       <c r="H19" s="2">
-        <v>0.32</v>
+        <v>0.25</v>
       </c>
       <c r="I19" s="2">
-        <v>0.335</v>
+        <v>0.26</v>
       </c>
       <c r="J19" s="2">
-        <v>0.355</v>
+        <v>0.275</v>
       </c>
     </row>
     <row r="20">
@@ -3249,22 +3249,22 @@
         <v>5.263157894736836</v>
       </c>
       <c r="E20" s="2">
-        <v>-50</v>
+        <v>4.999999999999982</v>
       </c>
       <c r="F20" s="2">
-        <v>100</v>
+        <v>4.761904761904767</v>
       </c>
       <c r="G20" s="2">
-        <v>49.99999999999998</v>
+        <v>6.818181818181812</v>
       </c>
       <c r="H20" s="2">
-        <v>6.666666666666665</v>
+        <v>6.382978723404253</v>
       </c>
       <c r="I20" s="2">
-        <v>4.6875</v>
+        <v>4.0000000000000036</v>
       </c>
       <c r="J20" s="2">
-        <v>5.970149253731338</v>
+        <v>5.769230769230771</v>
       </c>
     </row>
     <row r="21">
@@ -3283,22 +3283,22 @@
         <v>0.15392156862745102</v>
       </c>
       <c r="E21" s="2">
-        <v>0.25</v>
+        <v>0.15626168224299058</v>
       </c>
       <c r="F21" s="2">
-        <v>0.25316455696202533</v>
+        <v>0.15734513274336284</v>
       </c>
       <c r="G21" s="2">
-        <v>0.2564102564102564</v>
+        <v>0.15857142857142856</v>
       </c>
       <c r="H21" s="2">
-        <v>0.3014754098360655</v>
+        <v>0.210327868852459</v>
       </c>
       <c r="I21" s="2">
-        <v>0.3578571428571428</v>
+        <v>0.2792</v>
       </c>
       <c r="J21" s="2">
-        <v>0.42198473282442744</v>
+        <v>0.3708593749999998</v>
       </c>
     </row>
     <row r="22">
@@ -3611,32 +3611,32 @@
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 -24.8 % / 補助 -50 % / 他 4 %</t>
+          <t xml:space="preserve">全社 4.87 % / 補助 5.41 % / 他 4.26 %</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 38.04 % / 補助 100 % / 他 4 %</t>
+          <t xml:space="preserve">全社 4.88 % / 補助 5.41 % / 他 4.26 %</t>
         </is>
       </c>
       <c r="I4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 27.63 % / 補助 50 % / 他 4 %</t>
+          <t xml:space="preserve">全社 4.87 % / 補助 5.4 % / 他 4.26 %</t>
         </is>
       </c>
       <c r="J4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.05 % / 補助 21 % / 他 5.99 %</t>
+          <t xml:space="preserve">全社 19.39 % / 補助 29.62 % / 他 7.31 %</t>
         </is>
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.53 % / 補助 21 % / 他 6 %</t>
+          <t xml:space="preserve">全社 19.98 % / 補助 29.61 % / 他 6.25 %</t>
         </is>
       </c>
       <c r="L4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.98 % / 補助 21 % / 他 6 %</t>
+          <t xml:space="preserve">全社 21.09 % / 補助 29.61 % / 他 6.26 %</t>
         </is>
       </c>
     </row>
@@ -3673,32 +3673,32 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 66.83 % / 補助 65 % / 他 67.83 %</t>
+          <t xml:space="preserve">全社 68 % / 補助 67.99 % / 他 68 %</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 66.3 % / 補助 65 % / 他 67.67 %</t>
+          <t xml:space="preserve">全社 68 % / 補助 67.99 % / 他 68 %</t>
         </is>
       </c>
       <c r="I5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 65.99 % / 補助 65 % / 他 67.5 %</t>
+          <t xml:space="preserve">全社 68 % / 補助 68 % / 他 68.01 %</t>
         </is>
       </c>
       <c r="J5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 65.79 % / 補助 65 % / 他 67.17 %</t>
+          <t xml:space="preserve">全社 67.35 % / 補助 67.48 % / 他 67.17 %</t>
         </is>
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 65.62 % / 補助 65 % / 他 66.84 %</t>
+          <t xml:space="preserve">全社 66.98 % / 補助 66.96 % / 他 67 %</t>
         </is>
       </c>
       <c r="L5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 65.46 % / 補助 65 % / 他 66.5 %</t>
+          <t xml:space="preserve">全社 66.57 % / 補助 66.44 % / 他 66.83 %</t>
         </is>
       </c>
     </row>
@@ -3735,32 +3735,32 @@
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 33.17 % / 補助 35 % / 他 32.17 %</t>
+          <t xml:space="preserve">全社 32 % / 補助 32.01 % / 他 32 %</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 33.7 % / 補助 35 % / 他 32.33 %</t>
+          <t xml:space="preserve">全社 32 % / 補助 32.01 % / 他 32 %</t>
         </is>
       </c>
       <c r="I6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 34.01 % / 補助 35 % / 他 32.5 %</t>
+          <t xml:space="preserve">全社 32 % / 補助 32 % / 他 31.99 %</t>
         </is>
       </c>
       <c r="J6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 34.21 % / 補助 35 % / 他 32.83 %</t>
+          <t xml:space="preserve">全社 32.65 % / 補助 32.52 % / 他 32.83 %</t>
         </is>
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 34.38 % / 補助 35 % / 他 33.16 %</t>
+          <t xml:space="preserve">全社 33.02 % / 補助 33.04 % / 他 33 %</t>
         </is>
       </c>
       <c r="L6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 34.54 % / 補助 35 % / 他 33.5 %</t>
+          <t xml:space="preserve">全社 33.43 % / 補助 33.56 % / 他 33.17 %</t>
         </is>
       </c>
     </row>
@@ -3797,32 +3797,32 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 25.2 % / 補助 24.25 % / 他 25.73 %</t>
+          <t xml:space="preserve">全社 24.71 % / 補助 23.61 % / 他 25.98 %</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.92 % / 補助 24.25 % / 他 25.62 %</t>
+          <t xml:space="preserve">全社 25.12 % / 補助 24.28 % / 他 26.11 %</t>
         </is>
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.75 % / 補助 24.25 % / 他 25.51 %</t>
+          <t xml:space="preserve">全社 25.54 % / 補助 24.92 % / 他 26.27 %</t>
         </is>
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 23.3 % / 補助 22.25 % / 他 25.11 %</t>
+          <t xml:space="preserve">全社 23.47 % / 補助 21.84 % / 他 25.81 %</t>
         </is>
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 21.89 % / 補助 20.46 % / 他 24.72 %</t>
+          <t xml:space="preserve">全社 21.76 % / 補助 19.53 % / 他 25.64 %</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 20.54 % / 補助 18.87 % / 他 24.32 %</t>
+          <t xml:space="preserve">全社 20.05 % / 補助 17.5 % / 他 25.47 %</t>
         </is>
       </c>
     </row>
@@ -3859,32 +3859,32 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.97 % / 補助 10.75 % / 他 6.44 %</t>
+          <t xml:space="preserve">全社 7.29 % / 補助 8.4 % / 他 6.02 %</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.79 % / 補助 10.75 % / 他 6.71 %</t>
+          <t xml:space="preserve">全社 6.88 % / 補助 7.73 % / 他 5.89 %</t>
         </is>
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.26 % / 補助 10.75 % / 他 6.99 %</t>
+          <t xml:space="preserve">全社 6.46 % / 補助 7.08 % / 他 5.72 %</t>
         </is>
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.91 % / 補助 12.75 % / 他 7.72 %</t>
+          <t xml:space="preserve">全社 9.17 % / 補助 10.68 % / 他 7.02 %</t>
         </is>
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.5 % / 補助 14.54 % / 他 8.44 %</t>
+          <t xml:space="preserve">全社 11.26 % / 補助 13.51 % / 他 7.36 %</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 14 % / 補助 16.13 % / 他 9.18 %</t>
+          <t xml:space="preserve">全社 13.38 % / 補助 16.06 % / 他 7.7 %</t>
         </is>
       </c>
     </row>
@@ -3921,32 +3921,32 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.22 % / 補助 16.18 % / 他 8.5 %</t>
+          <t xml:space="preserve">全社 10.01 % / 補助 11.68 % / 他 8.07 %</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.53 % / 補助 16.16 % / 他 8.69 %</t>
+          <t xml:space="preserve">全社 9.93 % / 補助 11.7 % / 他 7.86 %</t>
         </is>
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.28 % / 補助 16.17 % / 他 8.89 %</t>
+          <t xml:space="preserve">全社 9.81 % / 補助 11.67 % / 他 7.61 %</t>
         </is>
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 14.41 % / 補助 17.22 % / 他 9.51 %</t>
+          <t xml:space="preserve">全社 11.98 % / 補助 14.22 % / 他 8.79 %</t>
         </is>
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.52 % / 補助 18.24 % / 他 10.14 %</t>
+          <t xml:space="preserve">全社 13.61 % / 補助 16.24 % / 他 9.02 %</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 16.61 % / 補助 19.19 % / 他 10.78 %</t>
+          <t xml:space="preserve">全社 15.31 % / 補助 18.17 % / 他 9.26 %</t>
         </is>
       </c>
     </row>
@@ -3983,32 +3983,32 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.82 % / 補助 10 % / 他 11.26 %</t>
+          <t xml:space="preserve">全社 12 % / 補助 12.5 % / 他 11.43 %</t>
         </is>
       </c>
       <c r="H10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.53 % / 補助 10 % / 他 11.09 %</t>
+          <t xml:space="preserve">全社 12.01 % / 補助 12.5 % / 他 11.43 %</t>
         </is>
       </c>
       <c r="I10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.37 % / 補助 10 % / 他 10.93 %</t>
+          <t xml:space="preserve">全社 12.01 % / 補助 12.5 % / 他 11.43 %</t>
         </is>
       </c>
       <c r="J10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.01 % / 補助 9.67 % / 他 10.62 %</t>
+          <t xml:space="preserve">全社 11.51 % / 補助 11.77 % / 他 11.15 %</t>
         </is>
       </c>
       <c r="K10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.66 % / 補助 9.33 % / 他 10.31 %</t>
+          <t xml:space="preserve">全社 11.02 % / 補助 11.04 % / 他 10.98 %</t>
         </is>
       </c>
       <c r="L10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.31 % / 補助 9 % / 他 10 %</t>
+          <t xml:space="preserve">全社 10.47 % / 補助 10.31 % / 他 10.81 %</t>
         </is>
       </c>
     </row>
@@ -4107,32 +4107,32 @@
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.4 % / 補助 8.33 % / 他 11.54 %</t>
+          <t xml:space="preserve">全社 9.5 % / 補助 7.65 % / 他 11.65 %</t>
         </is>
       </c>
       <c r="H12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.95 % / 補助 8.34 % / 他 11.66 %</t>
+          <t xml:space="preserve">全社 9.67 % / 補助 7.81 % / 他 11.85 %</t>
         </is>
       </c>
       <c r="I12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.7 % / 補助 8.33 % / 他 11.77 %</t>
+          <t xml:space="preserve">全社 9.86 % / 補助 7.97 % / 他 12.09 %</t>
         </is>
       </c>
       <c r="J12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.17 % / 補助 7.67 % / 他 11.78 %</t>
+          <t xml:space="preserve">全社 8.79 % / 補助 6.5 % / 他 12.06 %</t>
         </is>
       </c>
       <c r="K12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.63 % / 補助 7.05 % / 他 11.79 %</t>
+          <t xml:space="preserve">全社 8 % / 補助 5.6 % / 他 12.17 %</t>
         </is>
       </c>
       <c r="L12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.11 % / 補助 6.48 % / 他 11.79 %</t>
+          <t xml:space="preserve">全社 7.22 % / 補助 4.83 % / 他 12.28 %</t>
         </is>
       </c>
     </row>
@@ -4169,32 +4169,32 @@
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.73 % / 補助 0.5 % / 他 0.85 %</t>
+          <t xml:space="preserve">全社 0.65 % / 補助 0.5 % / 他 0.84 %</t>
         </is>
       </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.67 % / 補助 0.5 % / 他 0.86 %</t>
+          <t xml:space="preserve">全社 0.64 % / 補助 0.49 % / 他 0.81 %</t>
         </is>
       </c>
       <c r="I13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.64 % / 補助 0.5 % / 他 0.85 %</t>
+          <t xml:space="preserve">全社 0.64 % / 補助 0.5 % / 他 0.81 %</t>
         </is>
       </c>
       <c r="J13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.59 % / 補助 0.44 % / 他 0.85 %</t>
+          <t xml:space="preserve">全社 0.56 % / 補助 0.41 % / 他 0.76 %</t>
         </is>
       </c>
       <c r="K13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.53 % / 補助 0.38 % / 他 0.84 %</t>
+          <t xml:space="preserve">全社 0.48 % / 補助 0.33 % / 他 0.74 %</t>
         </is>
       </c>
       <c r="L13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.48 % / 補助 0.33 % / 他 0.82 %</t>
+          <t xml:space="preserve">全社 0.41 % / 補助 0.27 % / 他 0.71 %</t>
         </is>
       </c>
     </row>
@@ -4231,32 +4231,32 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.13 % / 補助 8.83 % / 他 12.39 %</t>
+          <t xml:space="preserve">全社 10.16 % / 補助 8.15 % / 他 12.48 %</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.63 % / 補助 8.84 % / 他 12.52 %</t>
+          <t xml:space="preserve">全社 10.32 % / 補助 8.3 % / 他 12.67 %</t>
         </is>
       </c>
       <c r="I14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.34 % / 補助 8.83 % / 他 12.62 %</t>
+          <t xml:space="preserve">全社 10.5 % / 補助 8.47 % / 他 12.9 %</t>
         </is>
       </c>
       <c r="J14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.76 % / 補助 8.11 % / 他 12.63 %</t>
+          <t xml:space="preserve">全社 9.35 % / 補助 6.91 % / 他 12.83 %</t>
         </is>
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.17 % / 補助 7.43 % / 他 12.63 %</t>
+          <t xml:space="preserve">全社 8.48 % / 補助 5.93 % / 他 12.91 %</t>
         </is>
       </c>
       <c r="L14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.59 % / 補助 6.82 % / 他 12.61 %</t>
+          <t xml:space="preserve">全社 7.63 % / 補助 5.1 % / 他 12.99 %</t>
         </is>
       </c>
     </row>
@@ -4293,32 +4293,32 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.069 億円/人 / 補助 0.088 億円/人 / 他 0.064 億円/人</t>
+          <t xml:space="preserve">全社 0.062 億円/人 / 補助 0.061 億円/人 / 他 0.063 億円/人</t>
         </is>
       </c>
       <c r="H15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.074 億円/人 / 補助 0.087 億円/人 / 他 0.066 億円/人</t>
+          <t xml:space="preserve">全社 0.063 億円/人 / 補助 0.063 億円/人 / 他 0.064 億円/人</t>
         </is>
       </c>
       <c r="I15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.077 億円/人 / 補助 0.087 億円/人 / 他 0.069 億円/人</t>
+          <t xml:space="preserve">全社 0.065 億円/人 / 補助 0.064 億円/人 / 他 0.065 億円/人</t>
         </is>
       </c>
       <c r="J15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.082 億円/人 / 補助 0.093 億円/人 / 他 0.072 億円/人</t>
+          <t xml:space="preserve">全社 0.066 億円/人 / 補助 0.066 億円/人 / 他 0.067 億円/人</t>
         </is>
       </c>
       <c r="K15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.087 億円/人 / 補助 0.1 億円/人 / 他 0.076 億円/人</t>
+          <t xml:space="preserve">全社 0.07 億円/人 / 補助 0.072 億円/人 / 他 0.068 億円/人</t>
         </is>
       </c>
       <c r="L15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.092 億円/人 / 補助 0.107 億円/人 / 他 0.079 億円/人</t>
+          <t xml:space="preserve">全社 0.074 億円/人 / 補助 0.078 億円/人 / 他 0.07 億円/人</t>
         </is>
       </c>
     </row>
@@ -4355,32 +4355,32 @@
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.164 億円/人 / 補助 0.1 億円/人 / 他 0.207 億円/人</t>
+          <t xml:space="preserve">全社 0.206 億円/人 / 補助 0.21 億円/人 / 他 0.203 億円/人</t>
         </is>
       </c>
       <c r="H16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.21 億円/人 / 補助 0.2 億円/人 / 他 0.217 億円/人</t>
+          <t xml:space="preserve">全社 0.212 億円/人 / 補助 0.22 億円/人 / 他 0.207 億円/人</t>
         </is>
       </c>
       <c r="I16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.254 億円/人 / 補助 0.3 億円/人 / 他 0.223 億円/人</t>
+          <t xml:space="preserve">全社 0.222 億円/人 / 補助 0.235 億円/人 / 他 0.213 億円/人</t>
         </is>
       </c>
       <c r="J16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.27 億円/人 / 補助 0.32 億円/人 / 他 0.237 億円/人</t>
+          <t xml:space="preserve">全社 0.23 億円/人 / 補助 0.25 億円/人 / 他 0.217 億円/人</t>
         </is>
       </c>
       <c r="K16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.282 億円/人 / 補助 0.335 億円/人 / 他 0.247 億円/人</t>
+          <t xml:space="preserve">全社 0.238 億円/人 / 補助 0.26 億円/人 / 他 0.223 億円/人</t>
         </is>
       </c>
       <c r="L16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.296 億円/人 / 補助 0.355 億円/人 / 他 0.257 億円/人</t>
+          <t xml:space="preserve">全社 0.246 億円/人 / 補助 0.275 億円/人 / 他 0.227 億円/人</t>
         </is>
       </c>
     </row>
@@ -4417,32 +4417,32 @@
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 14.03 % / 補助 46.05 % / 他 4.2 %</t>
+          <t xml:space="preserve">全社 2.34 % / 補助 2.38 % / 他 2.31 %</t>
         </is>
       </c>
       <c r="H17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.34 % / 補助 -1.15 % / 他 3.54 %</t>
+          <t xml:space="preserve">全社 1.67 % / 補助 1.78 % / 他 1.6 %</t>
         </is>
       </c>
       <c r="I17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.85 % / 補助 0.38 % / 他 4.2 %</t>
+          <t xml:space="preserve">全社 2.03 % / 補助 2.12 % / 他 1.98 %</t>
         </is>
       </c>
       <c r="J17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5.8 % / 補助 6.66 % / 他 4.48 %</t>
+          <t xml:space="preserve">全社 2.56 % / 補助 2.98 % / 他 2.22 %</t>
         </is>
       </c>
       <c r="K17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.33 % / 補助 7.64 % / 他 4.57 %</t>
+          <t xml:space="preserve">全社 5.35 % / 補助 9.06 % / 他 2.54 %</t>
         </is>
       </c>
       <c r="L17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.07 % / 補助 6.99 % / 他 4.53 %</t>
+          <t xml:space="preserve">全社 5.51 % / 補助 9.13 % / 他 2.71 %</t>
         </is>
       </c>
     </row>
@@ -4479,32 +4479,32 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 49.78 % / 補助 35.3 % / 他 59.3 %</t>
+          <t xml:space="preserve">全社 50.38 % / 補助 41.09 % / 他 60.73 %</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 45.9 % / 補助 35.35 % / 他 59.03 %</t>
+          <t xml:space="preserve">全社 50.96 % / 補助 41.51 % / 他 61.72 %</t>
         </is>
       </c>
       <c r="I18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 43.76 % / 補助 35.33 % / 他 58.68 %</t>
+          <t xml:space="preserve">全社 51.71 % / 補助 42.08 % / 他 62.88 %</t>
         </is>
       </c>
       <c r="J18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 40.37 % / 補助 32 % / 他 57.03 %</t>
+          <t xml:space="preserve">全社 43.83 % / 補助 32.7 % / 他 59.35 %</t>
         </is>
       </c>
       <c r="K18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 37.13 % / 補助 28.94 % / 他 55.46 %</t>
+          <t xml:space="preserve">全社 38.4 % / 補助 26.76 % / 他 58.87 %</t>
         </is>
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 34.08 % / 補助 26.21 % / 他 53.92 %</t>
+          <t xml:space="preserve">全社 33.25 % / 補助 21.93 % / 他 58.37 %</t>
         </is>
       </c>
     </row>
@@ -4603,32 +4603,32 @@
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.667 億円/人 / 補助 1.053 億円/人 / 他 0.556 億円/人</t>
+          <t xml:space="preserve">全社 0.655 億円/人 / 補助 0.803 億円/人 / 他 0.541 億円/人</t>
         </is>
       </c>
       <c r="H20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.741 億円/人 / 補助 1.039 億円/人 / 他 0.569 億円/人</t>
+          <t xml:space="preserve">全社 0.655 億円/人 / 補助 0.801 億円/人 / 他 0.54 億円/人</t>
         </is>
       </c>
       <c r="I20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.798 億円/人 / 補助 1.043 億円/人 / 他 0.588 億円/人</t>
+          <t xml:space="preserve">全社 0.655 億円/人 / 補助 0.801 億円/人 / 他 0.54 億円/人</t>
         </is>
       </c>
       <c r="J20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.893 億円/人 / 補助 1.21 億円/人 / 他 0.614 億円/人</t>
+          <t xml:space="preserve">全社 0.754 億円/人 / 補助 1.012 億円/人 / 他 0.553 億円/人</t>
         </is>
       </c>
       <c r="K20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.008 億円/人 / 補助 1.417 億円/人 / 他 0.641 億円/人</t>
+          <t xml:space="preserve">全社 0.873 億円/人 / 補助 1.28 億円/人 / 他 0.562 億円/人</t>
         </is>
       </c>
       <c r="L20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.139 億円/人 / 補助 1.648 億円/人 / 他 0.67 億円/人</t>
+          <t xml:space="preserve">全社 1.021 億円/人 / 補助 1.619 億円/人 / 他 0.572 億円/人</t>
         </is>
       </c>
     </row>
@@ -4665,32 +4665,32 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.053 億円/人 / 補助 0.113 億円/人 / 他 0.036 億円/人</t>
+          <t xml:space="preserve">全社 0.048 億円/人 / 補助 0.067 億円/人 / 他 0.033 億円/人</t>
         </is>
       </c>
       <c r="H21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.065 億円/人 / 補助 0.112 億円/人 / 他 0.038 億円/人</t>
+          <t xml:space="preserve">全社 0.045 億円/人 / 補助 0.062 億円/人 / 他 0.032 億円/人</t>
         </is>
       </c>
       <c r="I21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.074 億円/人 / 補助 0.112 億円/人 / 他 0.041 億円/人</t>
+          <t xml:space="preserve">全社 0.042 億円/人 / 補助 0.057 億円/人 / 他 0.031 億円/人</t>
         </is>
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.097 億円/人 / 補助 0.154 億円/人 / 他 0.047 億円/人</t>
+          <t xml:space="preserve">全社 0.069 億円/人 / 補助 0.108 億円/人 / 他 0.039 億円/人</t>
         </is>
       </c>
       <c r="K21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.126 億円/人 / 補助 0.206 億円/人 / 他 0.054 億円/人</t>
+          <t xml:space="preserve">全社 0.098 億円/人 / 補助 0.173 億円/人 / 他 0.041 億円/人</t>
         </is>
       </c>
       <c r="L21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.159 億円/人 / 補助 0.266 億円/人 / 他 0.062 億円/人</t>
+          <t xml:space="preserve">全社 0.137 億円/人 / 補助 0.26 億円/人 / 他 0.044 億円/人</t>
         </is>
       </c>
     </row>
@@ -4727,32 +4727,32 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.145 億円/人 / 補助 0.25 億円/人 / 他 0.114 億円/人</t>
+          <t xml:space="preserve">全社 0.129 億円/人 / 補助 0.156 億円/人 / 他 0.109 億円/人</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.168 億円/人 / 補助 0.253 億円/人 / 他 0.118 億円/人</t>
+          <t xml:space="preserve">全社 0.13 億円/人 / 補助 0.157 億円/人 / 他 0.108 億円/人</t>
         </is>
       </c>
       <c r="I22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.185 億円/人 / 補助 0.256 億円/人 / 他 0.124 億円/人</t>
+          <t xml:space="preserve">全社 0.131 億円/人 / 補助 0.159 億円/人 / 他 0.108 億円/人</t>
         </is>
       </c>
       <c r="J22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.212 億円/人 / 補助 0.301 億円/人 / 他 0.133 億円/人</t>
+          <t xml:space="preserve">全社 0.158 億円/人 / 補助 0.21 億円/人 / 他 0.117 億円/人</t>
         </is>
       </c>
       <c r="K22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.244 億円/人 / 補助 0.358 億円/人 / 他 0.143 億円/人</t>
+          <t xml:space="preserve">全社 0.189 億円/人 / 補助 0.279 億円/人 / 他 0.121 億円/人</t>
         </is>
       </c>
       <c r="L22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.282 億円/人 / 補助 0.422 億円/人 / 他 0.153 億円/人</t>
+          <t xml:space="preserve">全社 0.23 億円/人 / 補助 0.371 億円/人 / 他 0.125 億円/人</t>
         </is>
       </c>
     </row>
@@ -4789,32 +4789,32 @@
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 -26.52 % / 補助 -62 % / 他 0.77 %</t>
+          <t xml:space="preserve">全社 4.35 % / 補助 5 % / 他 3.85 %</t>
         </is>
       </c>
       <c r="H23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.26 % / 補助 102.63 % / 他 1.53 %</t>
+          <t xml:space="preserve">全社 5 % / 補助 5.71 % / 他 4.44 %</t>
         </is>
       </c>
       <c r="I23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 18.57 % / 補助 49.35 % / 他 0.75 %</t>
+          <t xml:space="preserve">全社 4.76 % / 補助 5.41 % / 他 4.26 %</t>
         </is>
       </c>
       <c r="J23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.81 % / 補助 4.35 % / 他 1.49 %</t>
+          <t xml:space="preserve">全社 3.79 % / 補助 2.56 % / 他 4.76 %</t>
         </is>
       </c>
       <c r="K23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.34 % / 補助 3.33 % / 他 1.47 %</t>
+          <t xml:space="preserve">全社 3.65 % / 補助 2.5 % / 他 4.55 %</t>
         </is>
       </c>
       <c r="L23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.67 % / 補助 4.03 % / 他 1.45 %</t>
+          <t xml:space="preserve">全社 3.52 % / 補助 2.44 % / 他 4.35 %</t>
         </is>
       </c>
     </row>
@@ -4851,32 +4851,32 @@
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.72 pt / 補助 12 pt / 他 3.23 pt</t>
+          <t xml:space="preserve">全社 0.53 pt / 補助 0.41 pt / 他 0.41 pt</t>
         </is>
       </c>
       <c r="H24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.78 pt / 補助 -2.63 pt / 他 2.47 pt</t>
+          <t xml:space="preserve">全社 -0.12 pt / 補助 -0.31 pt / 他 -0.18 pt</t>
         </is>
       </c>
       <c r="I24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.06 pt / 補助 0.65 pt / 他 3.25 pt</t>
+          <t xml:space="preserve">全社 0.11 pt / 補助 -0.01 pt / 他 0 pt</t>
         </is>
       </c>
       <c r="J24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.24 pt / 補助 16.65 pt / 他 4.5 pt</t>
+          <t xml:space="preserve">全社 15.6 pt / 補助 27.05 pt / 他 2.55 pt</t>
         </is>
       </c>
       <c r="K24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.18 pt / 補助 17.67 pt / 他 4.53 pt</t>
+          <t xml:space="preserve">全社 16.33 pt / 補助 27.11 pt / 他 1.7 pt</t>
         </is>
       </c>
       <c r="L24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.31 pt / 補助 16.97 pt / 他 4.55 pt</t>
+          <t xml:space="preserve">全社 17.57 pt / 補助 27.17 pt / 他 1.91 pt</t>
         </is>
       </c>
     </row>
@@ -4975,32 +4975,32 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.25 % / 補助 5.43 % / 他 2.06 %</t>
+          <t xml:space="preserve">全社 2.71 % / 補助 3.28 % / 他 2.06 %</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.74 % / 補助 5.41 % / 他 1.98 %</t>
+          <t xml:space="preserve">全社 3.05 % / 補助 3.97 % / 他 1.97 %</t>
         </is>
       </c>
       <c r="I26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.03 % / 補助 5.42 % / 他 1.91 %</t>
+          <t xml:space="preserve">全社 3.35 % / 補助 4.59 % / 他 1.89 %</t>
         </is>
       </c>
       <c r="J26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.5 % / 補助 4.48 % / 他 1.8 %</t>
+          <t xml:space="preserve">全社 2.81 % / 補助 3.54 % / 他 1.76 %</t>
         </is>
       </c>
       <c r="K26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.03 % / 補助 3.7 % / 他 1.7 %</t>
+          <t xml:space="preserve">全社 2.34 % / 補助 2.73 % / 他 1.66 %</t>
         </is>
       </c>
       <c r="L26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.61 % / 補助 3.06 % / 他 1.6 %</t>
+          <t xml:space="preserve">全社 1.93 % / 補助 2.11 % / 他 1.56 %</t>
         </is>
       </c>
     </row>
@@ -5037,17 +5037,17 @@
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.3 %</t>
+          <t xml:space="preserve">全社 9.54 %</t>
         </is>
       </c>
       <c r="H27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.63 %</t>
+          <t xml:space="preserve">全社 9.09 %</t>
         </is>
       </c>
       <c r="I27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.55 %</t>
+          <t xml:space="preserve">全社 8.67 %</t>
         </is>
       </c>
       <c r="J27" s="0" t="inlineStr">
@@ -5099,17 +5099,17 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.18 倍</t>
+          <t xml:space="preserve">全社 0.95 倍</t>
         </is>
       </c>
       <c r="H28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.77 倍</t>
+          <t xml:space="preserve">全社 0.92 倍</t>
         </is>
       </c>
       <c r="I28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.57 倍</t>
+          <t xml:space="preserve">全社 0.88 倍</t>
         </is>
       </c>
       <c r="J28" s="0" t="inlineStr">
@@ -5161,32 +5161,32 @@
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.45 倍 / 補助 2.98 倍 / 他 4.13 倍</t>
+          <t xml:space="preserve">全社 3.69 倍 / 補助 3.56 倍 / 他 3.93 倍</t>
         </is>
       </c>
       <c r="H29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.35 倍 / 補助 2.99 倍 / 他 4.39 倍</t>
+          <t xml:space="preserve">全社 3.26 倍 / 補助 2.95 倍 / 他 3.99 倍</t>
         </is>
       </c>
       <c r="I29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.3 倍 / 補助 2.98 倍 / 他 4.67 倍</t>
+          <t xml:space="preserve">全社 2.93 倍 / 補助 2.54 倍 / 他 4.03 倍</t>
         </is>
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.12 倍 / 補助 3.85 倍 / 他 5.29 倍</t>
+          <t xml:space="preserve">全社 4.27 倍 / 補助 4.02 倍 / 他 4.99 倍</t>
         </is>
       </c>
       <c r="K29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5.13 倍 / 補助 4.93 倍 / 他 5.98 倍</t>
+          <t xml:space="preserve">全社 5.81 倍 / 補助 5.94 倍 / 他 5.44 倍</t>
         </is>
       </c>
       <c r="L29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.36 倍 / 補助 6.28 倍 / 他 6.74 倍</t>
+          <t xml:space="preserve">全社 7.92 倍 / 補助 8.62 倍 / 他 5.93 倍</t>
         </is>
       </c>
     </row>
@@ -5223,17 +5223,17 @@
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 -2.48 倍</t>
+          <t xml:space="preserve">全社 0.49 倍</t>
         </is>
       </c>
       <c r="H30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.86 倍</t>
+          <t xml:space="preserve">全社 0.51 倍</t>
         </is>
       </c>
       <c r="I30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.87 倍</t>
+          <t xml:space="preserve">全社 0.54 倍</t>
         </is>
       </c>
       <c r="J30" s="0" t="inlineStr">
@@ -5347,32 +5347,32 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 35.46 %</t>
+          <t xml:space="preserve">構成比 53.61 %</t>
         </is>
       </c>
       <c r="H32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 51.38 %</t>
+          <t xml:space="preserve">構成比 53.88 %</t>
         </is>
       </c>
       <c r="I32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 60.38 %</t>
+          <t xml:space="preserve">構成比 54.15 %</t>
         </is>
       </c>
       <c r="J32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 63.5 %</t>
+          <t xml:space="preserve">構成比 58.79 %</t>
         </is>
       </c>
       <c r="K32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 66.51 %</t>
+          <t xml:space="preserve">構成比 63.51 %</t>
         </is>
       </c>
       <c r="L32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 69.39 %</t>
+          <t xml:space="preserve">構成比 67.98 %</t>
         </is>
       </c>
     </row>
@@ -5409,32 +5409,32 @@
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 -50 % / 他 4 %</t>
+          <t xml:space="preserve">補助 5.41 % / 他 4.26 %</t>
         </is>
       </c>
       <c r="H33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 100 % / 他 4 %</t>
+          <t xml:space="preserve">補助 5.41 % / 他 4.26 %</t>
         </is>
       </c>
       <c r="I33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 50 % / 他 4 %</t>
+          <t xml:space="preserve">補助 5.4 % / 他 4.26 %</t>
         </is>
       </c>
       <c r="J33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 21 % / 他 5.99 %</t>
+          <t xml:space="preserve">補助 29.62 % / 他 7.31 %</t>
         </is>
       </c>
       <c r="K33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 21 % / 他 6 %</t>
+          <t xml:space="preserve">補助 29.61 % / 他 6.25 %</t>
         </is>
       </c>
       <c r="L33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 21 % / 他 6 %</t>
+          <t xml:space="preserve">補助 29.61 % / 他 6.26 %</t>
         </is>
       </c>
     </row>
@@ -5471,32 +5471,32 @@
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -2.83 pt</t>
+          <t xml:space="preserve">差 -0.01 pt</t>
         </is>
       </c>
       <c r="H34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -2.67 pt</t>
+          <t xml:space="preserve">差 -0 pt</t>
         </is>
       </c>
       <c r="I34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -2.5 pt</t>
+          <t xml:space="preserve">差 -0.01 pt</t>
         </is>
       </c>
       <c r="J34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -2.17 pt</t>
+          <t xml:space="preserve">差 0.31 pt</t>
         </is>
       </c>
       <c r="K34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -1.84 pt</t>
+          <t xml:space="preserve">差 -0.04 pt</t>
         </is>
       </c>
       <c r="L34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -1.5 pt</t>
+          <t xml:space="preserve">差 -0.39 pt</t>
         </is>
       </c>
     </row>
@@ -5533,32 +5533,32 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 4.31 pt</t>
+          <t xml:space="preserve">差 2.38 pt</t>
         </is>
       </c>
       <c r="H35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 4.04 pt</t>
+          <t xml:space="preserve">差 1.84 pt</t>
         </is>
       </c>
       <c r="I35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 3.76 pt</t>
+          <t xml:space="preserve">差 1.35 pt</t>
         </is>
       </c>
       <c r="J35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 5.03 pt</t>
+          <t xml:space="preserve">差 3.66 pt</t>
         </is>
       </c>
       <c r="K35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 6.09 pt</t>
+          <t xml:space="preserve">差 6.14 pt</t>
         </is>
       </c>
       <c r="L35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 6.95 pt</t>
+          <t xml:space="preserve">差 8.36 pt</t>
         </is>
       </c>
     </row>
@@ -5595,32 +5595,32 @@
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.053 億円/人 / 他 0.556 億円/人</t>
+          <t xml:space="preserve">補助 0.803 億円/人 / 他 0.541 億円/人</t>
         </is>
       </c>
       <c r="H36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.039 億円/人 / 他 0.569 億円/人</t>
+          <t xml:space="preserve">補助 0.801 億円/人 / 他 0.54 億円/人</t>
         </is>
       </c>
       <c r="I36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.043 億円/人 / 他 0.588 億円/人</t>
+          <t xml:space="preserve">補助 0.801 億円/人 / 他 0.54 億円/人</t>
         </is>
       </c>
       <c r="J36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.21 億円/人 / 他 0.614 億円/人</t>
+          <t xml:space="preserve">補助 1.012 億円/人 / 他 0.553 億円/人</t>
         </is>
       </c>
       <c r="K36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.417 億円/人 / 他 0.641 億円/人</t>
+          <t xml:space="preserve">補助 1.28 億円/人 / 他 0.562 億円/人</t>
         </is>
       </c>
       <c r="L36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.648 億円/人 / 他 0.67 億円/人</t>
+          <t xml:space="preserve">補助 1.619 億円/人 / 他 0.572 億円/人</t>
         </is>
       </c>
     </row>
@@ -5657,32 +5657,32 @@
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.088 億円/人 / 他 0.064 億円/人</t>
+          <t xml:space="preserve">補助 0.061 億円/人 / 他 0.063 億円/人</t>
         </is>
       </c>
       <c r="H37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.087 億円/人 / 他 0.066 億円/人</t>
+          <t xml:space="preserve">補助 0.063 億円/人 / 他 0.064 億円/人</t>
         </is>
       </c>
       <c r="I37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.087 億円/人 / 他 0.069 億円/人</t>
+          <t xml:space="preserve">補助 0.064 億円/人 / 他 0.065 億円/人</t>
         </is>
       </c>
       <c r="J37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.093 億円/人 / 他 0.072 億円/人</t>
+          <t xml:space="preserve">補助 0.066 億円/人 / 他 0.067 億円/人</t>
         </is>
       </c>
       <c r="K37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.1 億円/人 / 他 0.076 億円/人</t>
+          <t xml:space="preserve">補助 0.072 億円/人 / 他 0.068 億円/人</t>
         </is>
       </c>
       <c r="L37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.107 億円/人 / 他 0.079 億円/人</t>
+          <t xml:space="preserve">補助 0.078 億円/人 / 他 0.07 億円/人</t>
         </is>
       </c>
     </row>
@@ -5719,32 +5719,32 @@
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 114.94 %</t>
+          <t xml:space="preserve">寄与率 169.23 %</t>
         </is>
       </c>
       <c r="H38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 91.68 %</t>
+          <t xml:space="preserve">寄与率 175 %</t>
         </is>
       </c>
       <c r="I38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 91.1 %</t>
+          <t xml:space="preserve">寄与率 133.33 %</t>
         </is>
       </c>
       <c r="J38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 85.65 %</t>
+          <t xml:space="preserve">寄与率 81.49 %</t>
         </is>
       </c>
       <c r="K38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 87.22 %</t>
+          <t xml:space="preserve">寄与率 92.42 %</t>
         </is>
       </c>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 88.47 %</t>
+          <t xml:space="preserve">寄与率 93.95 %</t>
         </is>
       </c>
     </row>
@@ -5850,7 +5850,7 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <v>21</v>
+        <v>5.407072368421051</v>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
@@ -5858,10 +5858,10 @@
         </is>
       </c>
       <c r="D4" s="2">
-        <v>-5</v>
+        <v>5.116959064327475</v>
       </c>
       <c r="E4" s="2">
-        <v>40</v>
+        <v>5.701754385964919</v>
       </c>
     </row>
     <row r="5">
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <v>7.000000000000001</v>
+        <v>1.174186491064466e-14</v>
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
@@ -5882,7 +5882,7 @@
         <v>0</v>
       </c>
       <c r="E5" s="2">
-        <v>2</v>
+        <v>1.6653345369377348e-14</v>
       </c>
     </row>
     <row r="6">
@@ -5892,7 +5892,7 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <v>7.000000000000001</v>
+        <v>2.0019816287178878</v>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
@@ -5900,10 +5900,10 @@
         </is>
       </c>
       <c r="D6" s="2">
-        <v>0</v>
+        <v>1.9325330501846927</v>
       </c>
       <c r="E6" s="2">
-        <v>10</v>
+        <v>2.0735994183189166</v>
       </c>
     </row>
     <row r="7">
@@ -5913,7 +5913,7 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <v>4</v>
+        <v>5.444853630675327</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -5921,10 +5921,10 @@
         </is>
       </c>
       <c r="D7" s="2">
-        <v>-3</v>
+        <v>5.116959064327475</v>
       </c>
       <c r="E7" s="2">
-        <v>20</v>
+        <v>5.701754385964919</v>
       </c>
     </row>
     <row r="8">
@@ -5934,7 +5934,7 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
@@ -5945,7 +5945,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -5955,7 +5955,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <v>6</v>
+        <v>5.40609337027898</v>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
@@ -5963,10 +5963,10 @@
         </is>
       </c>
       <c r="D9" s="2">
-        <v>0</v>
+        <v>5.116959064327475</v>
       </c>
       <c r="E9" s="2">
-        <v>10</v>
+        <v>5.701754385964919</v>
       </c>
     </row>
     <row r="10">
@@ -5976,7 +5976,7 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <v>4</v>
+        <v>4.260731658392249</v>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
@@ -5984,10 +5984,10 @@
         </is>
       </c>
       <c r="D10" s="2">
-        <v>-10</v>
+        <v>4.076086956521719</v>
       </c>
       <c r="E10" s="2">
-        <v>20</v>
+        <v>4.438405797101453</v>
       </c>
     </row>
     <row r="11">
@@ -5997,7 +5997,7 @@
         </is>
       </c>
       <c r="B11" s="2">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
@@ -6008,7 +6008,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="2">
-        <v>2</v>
+        <v>0.013457556935819737</v>
       </c>
     </row>
     <row r="12">
@@ -6018,7 +6018,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>4</v>
+        <v>1.9809059504605664</v>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
@@ -6026,10 +6026,10 @@
         </is>
       </c>
       <c r="D12" s="2">
-        <v>0</v>
+        <v>1.9139457023717443</v>
       </c>
       <c r="E12" s="2">
-        <v>8</v>
+        <v>2.0553459914763095</v>
       </c>
     </row>
     <row r="13">
@@ -6039,7 +6039,7 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <v>1</v>
+        <v>4.149377724930645</v>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
@@ -6047,10 +6047,10 @@
         </is>
       </c>
       <c r="D13" s="2">
-        <v>-5</v>
+        <v>3.9166666666666683</v>
       </c>
       <c r="E13" s="2">
-        <v>10</v>
+        <v>4.250000000000009</v>
       </c>
     </row>
     <row r="14">
@@ -6060,7 +6060,7 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
@@ -6071,7 +6071,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -6081,7 +6081,7 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <v>21</v>
+        <v>29.61371439006574</v>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
@@ -6089,10 +6089,10 @@
         </is>
       </c>
       <c r="D15" s="2">
-        <v>-5</v>
+        <v>15</v>
       </c>
       <c r="E15" s="2">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16">
@@ -6102,7 +6102,7 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <v>6</v>
+        <v>6.249525817103336</v>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
@@ -6110,10 +6110,10 @@
         </is>
       </c>
       <c r="D16" s="2">
-        <v>-10</v>
+        <v>6.076086956521719</v>
       </c>
       <c r="E16" s="2">
-        <v>20</v>
+        <v>6.438405797101453</v>
       </c>
     </row>
     <row r="17">
@@ -6123,7 +6123,7 @@
         </is>
       </c>
       <c r="B17" s="2">
-        <v>0</v>
+        <v>1.5550427257977284</v>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
@@ -6144,7 +6144,7 @@
         </is>
       </c>
       <c r="B18" s="2">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
@@ -6152,10 +6152,10 @@
         </is>
       </c>
       <c r="D18" s="2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E18" s="2">
-        <v>3</v>
+        <v>0.5134575569358197</v>
       </c>
     </row>
     <row r="19">
@@ -6165,7 +6165,7 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <v>7.000000000000001</v>
+        <v>8.894384122463512</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
@@ -6173,7 +6173,7 @@
         </is>
       </c>
       <c r="D19" s="2">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="E19" s="2">
         <v>10</v>
@@ -6186,7 +6186,7 @@
         </is>
       </c>
       <c r="B20" s="2">
-        <v>4.5</v>
+        <v>2.484215290694131</v>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
@@ -6194,10 +6194,10 @@
         </is>
       </c>
       <c r="D20" s="2">
-        <v>0</v>
+        <v>2.4139457023717443</v>
       </c>
       <c r="E20" s="2">
-        <v>8</v>
+        <v>2.5553459914763095</v>
       </c>
     </row>
     <row r="21">
@@ -6207,7 +6207,7 @@
         </is>
       </c>
       <c r="B21" s="2">
-        <v>4</v>
+        <v>2.6240752485890892</v>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
@@ -6215,10 +6215,10 @@
         </is>
       </c>
       <c r="D21" s="2">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="E21" s="2">
-        <v>20</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22">
@@ -6228,7 +6228,7 @@
         </is>
       </c>
       <c r="B22" s="2">
-        <v>1.5</v>
+        <v>4.5872376921363385</v>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
@@ -6236,10 +6236,10 @@
         </is>
       </c>
       <c r="D22" s="2">
-        <v>-5</v>
+        <v>4.416666666666668</v>
       </c>
       <c r="E22" s="2">
-        <v>10</v>
+        <v>4.750000000000009</v>
       </c>
     </row>
     <row r="23">
@@ -6249,7 +6249,7 @@
         </is>
       </c>
       <c r="B23" s="2">
-        <v>9</v>
+        <v>10.315299543741322</v>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
@@ -6257,10 +6257,10 @@
         </is>
       </c>
       <c r="D23" s="2">
-        <v>4</v>
+        <v>8.5</v>
       </c>
       <c r="E23" s="2">
-        <v>25</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="24">
@@ -6270,7 +6270,7 @@
         </is>
       </c>
       <c r="B24" s="2">
-        <v>10</v>
+        <v>10.92261646516366</v>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
@@ -6278,10 +6278,10 @@
         </is>
       </c>
       <c r="D24" s="2">
-        <v>4</v>
+        <v>8.928571428571427</v>
       </c>
       <c r="E24" s="2">
-        <v>25</v>
+        <v>11.928571428571427</v>
       </c>
     </row>
     <row r="25">
@@ -6291,7 +6291,7 @@
         </is>
       </c>
       <c r="B25" s="2">
-        <v>6</v>
+        <v>5.371923167958349</v>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
@@ -6299,10 +6299,10 @@
         </is>
       </c>
       <c r="D25" s="2">
-        <v>0</v>
+        <v>4.263157894736836</v>
       </c>
       <c r="E25" s="2">
-        <v>10</v>
+        <v>6.555555555555557</v>
       </c>
     </row>
     <row r="26">
@@ -6337,7 +6337,7 @@
         </is>
       </c>
       <c r="B27" s="2">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
@@ -6362,11 +6362,11 @@
         </is>
       </c>
       <c r="B28" s="2">
-        <v>15</v>
+        <v>7.67</v>
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">50億円以下、かつ投資額の1/3以下（現在上限15.00億円）</t>
+          <t xml:space="preserve">50億円以下、かつ投資額の1/3以下（現在上限7.67億円）</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
@@ -6386,7 +6386,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C225"/>
+  <dimension ref="A1:C229"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="72" customWidth="1"/>
@@ -8160,11 +8160,11 @@
         </is>
       </c>
       <c r="B118" s="2">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="C118" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
@@ -8175,7 +8175,7 @@
         </is>
       </c>
       <c r="B119" s="2">
-        <v>0.03</v>
+        <v>0.0051345755693581975</v>
       </c>
       <c r="C119" s="0" t="inlineStr">
         <is>
@@ -8205,7 +8205,7 @@
         </is>
       </c>
       <c r="B121" s="2">
-        <v>0.02</v>
+        <v>0.00013457556935819737</v>
       </c>
       <c r="C121" s="0" t="inlineStr">
         <is>
@@ -8220,7 +8220,7 @@
         </is>
       </c>
       <c r="B122" s="2">
-        <v>-0.05</v>
+        <v>0.04416666666666668</v>
       </c>
       <c r="C122" s="0" t="inlineStr">
         <is>
@@ -8235,7 +8235,7 @@
         </is>
       </c>
       <c r="B123" s="2">
-        <v>0.1</v>
+        <v>0.04750000000000009</v>
       </c>
       <c r="C123" s="0" t="inlineStr">
         <is>
@@ -8250,7 +8250,7 @@
         </is>
       </c>
       <c r="B124" s="2">
-        <v>-0.05</v>
+        <v>0.03916666666666668</v>
       </c>
       <c r="C124" s="0" t="inlineStr">
         <is>
@@ -8265,7 +8265,7 @@
         </is>
       </c>
       <c r="B125" s="2">
-        <v>0.1</v>
+        <v>0.04250000000000009</v>
       </c>
       <c r="C125" s="0" t="inlineStr">
         <is>
@@ -8280,11 +8280,11 @@
         </is>
       </c>
       <c r="B126" s="2">
-        <v>0</v>
+        <v>0.024139457023717444</v>
       </c>
       <c r="C126" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
@@ -8295,7 +8295,7 @@
         </is>
       </c>
       <c r="B127" s="2">
-        <v>0.08</v>
+        <v>0.025553459914763096</v>
       </c>
       <c r="C127" s="0" t="inlineStr">
         <is>
@@ -8310,11 +8310,11 @@
         </is>
       </c>
       <c r="B128" s="2">
-        <v>0</v>
+        <v>0.019139457023717443</v>
       </c>
       <c r="C128" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
@@ -8325,7 +8325,7 @@
         </is>
       </c>
       <c r="B129" s="2">
-        <v>0.08</v>
+        <v>0.020553459914763095</v>
       </c>
       <c r="C129" s="0" t="inlineStr">
         <is>
@@ -8340,7 +8340,7 @@
         </is>
       </c>
       <c r="B130" s="2">
-        <v>-0.1</v>
+        <v>0.06076086956521719</v>
       </c>
       <c r="C130" s="0" t="inlineStr">
         <is>
@@ -8355,7 +8355,7 @@
         </is>
       </c>
       <c r="B131" s="2">
-        <v>0.2</v>
+        <v>0.06438405797101453</v>
       </c>
       <c r="C131" s="0" t="inlineStr">
         <is>
@@ -8370,7 +8370,7 @@
         </is>
       </c>
       <c r="B132" s="2">
-        <v>-0.1</v>
+        <v>0.040760869565217184</v>
       </c>
       <c r="C132" s="0" t="inlineStr">
         <is>
@@ -8385,7 +8385,7 @@
         </is>
       </c>
       <c r="B133" s="2">
-        <v>0.2</v>
+        <v>0.04438405797101452</v>
       </c>
       <c r="C133" s="0" t="inlineStr">
         <is>
@@ -8415,11 +8415,11 @@
         </is>
       </c>
       <c r="B135" s="2">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="C135" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
@@ -8430,7 +8430,7 @@
         </is>
       </c>
       <c r="B136" s="2">
-        <v>0.04</v>
+        <v>0.08928571428571427</v>
       </c>
       <c r="C136" s="0" t="inlineStr">
         <is>
@@ -8445,7 +8445,7 @@
         </is>
       </c>
       <c r="B137" s="2">
-        <v>0.25</v>
+        <v>0.11928571428571427</v>
       </c>
       <c r="C137" s="0" t="inlineStr">
         <is>
@@ -8505,7 +8505,7 @@
         </is>
       </c>
       <c r="B141" s="2">
-        <v>0.02</v>
+        <v>1.6653345369377348e-16</v>
       </c>
       <c r="C141" s="0" t="inlineStr">
         <is>
@@ -8520,11 +8520,11 @@
         </is>
       </c>
       <c r="B142" s="2">
-        <v>-0.03</v>
+        <v>0</v>
       </c>
       <c r="C142" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
@@ -8535,7 +8535,7 @@
         </is>
       </c>
       <c r="B143" s="2">
-        <v>0.2</v>
+        <v>0.08</v>
       </c>
       <c r="C143" s="0" t="inlineStr">
         <is>
@@ -8550,7 +8550,7 @@
         </is>
       </c>
       <c r="B144" s="2">
-        <v>-0.03</v>
+        <v>0.051169590643274754</v>
       </c>
       <c r="C144" s="0" t="inlineStr">
         <is>
@@ -8565,7 +8565,7 @@
         </is>
       </c>
       <c r="B145" s="2">
-        <v>0.2</v>
+        <v>0.05701754385964919</v>
       </c>
       <c r="C145" s="0" t="inlineStr">
         <is>
@@ -8610,11 +8610,11 @@
         </is>
       </c>
       <c r="B148" s="2">
-        <v>0</v>
+        <v>0.04263157894736836</v>
       </c>
       <c r="C148" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
@@ -8625,7 +8625,7 @@
         </is>
       </c>
       <c r="B149" s="2">
-        <v>0.1</v>
+        <v>0.06555555555555558</v>
       </c>
       <c r="C149" s="0" t="inlineStr">
         <is>
@@ -8640,11 +8640,11 @@
         </is>
       </c>
       <c r="B150" s="2">
-        <v>0</v>
+        <v>0.051169590643274754</v>
       </c>
       <c r="C150" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
@@ -8655,7 +8655,7 @@
         </is>
       </c>
       <c r="B151" s="2">
-        <v>0.1</v>
+        <v>0.05701754385964919</v>
       </c>
       <c r="C151" s="0" t="inlineStr">
         <is>
@@ -8670,7 +8670,7 @@
         </is>
       </c>
       <c r="B152" s="2">
-        <v>0.045</v>
+        <v>0.05</v>
       </c>
       <c r="C152" s="0" t="inlineStr">
         <is>
@@ -8700,11 +8700,11 @@
         </is>
       </c>
       <c r="B154" s="2">
-        <v>0</v>
+        <v>0.019325330501846927</v>
       </c>
       <c r="C154" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
@@ -8715,7 +8715,7 @@
         </is>
       </c>
       <c r="B155" s="2">
-        <v>0.1</v>
+        <v>0.020735994183189166</v>
       </c>
       <c r="C155" s="0" t="inlineStr">
         <is>
@@ -8730,7 +8730,7 @@
         </is>
       </c>
       <c r="B156" s="2">
-        <v>-0.05</v>
+        <v>0.15</v>
       </c>
       <c r="C156" s="0" t="inlineStr">
         <is>
@@ -8745,7 +8745,7 @@
         </is>
       </c>
       <c r="B157" s="2">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="C157" s="0" t="inlineStr">
         <is>
@@ -8760,7 +8760,7 @@
         </is>
       </c>
       <c r="B158" s="2">
-        <v>-0.05</v>
+        <v>0.051169590643274754</v>
       </c>
       <c r="C158" s="0" t="inlineStr">
         <is>
@@ -8775,7 +8775,7 @@
         </is>
       </c>
       <c r="B159" s="2">
-        <v>0.4</v>
+        <v>0.05701754385964919</v>
       </c>
       <c r="C159" s="0" t="inlineStr">
         <is>
@@ -8805,11 +8805,11 @@
         </is>
       </c>
       <c r="B161" s="2">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="C161" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
@@ -8820,7 +8820,7 @@
         </is>
       </c>
       <c r="B162" s="2">
-        <v>0.04</v>
+        <v>0.08499999999999999</v>
       </c>
       <c r="C162" s="0" t="inlineStr">
         <is>
@@ -8835,7 +8835,7 @@
         </is>
       </c>
       <c r="B163" s="2">
-        <v>0.25</v>
+        <v>0.135</v>
       </c>
       <c r="C163" s="0" t="inlineStr">
         <is>
@@ -8910,7 +8910,7 @@
         </is>
       </c>
       <c r="B168" s="2">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="C168" s="0" t="inlineStr">
         <is>
@@ -8940,7 +8940,7 @@
         </is>
       </c>
       <c r="B170" s="2">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="C170" s="0" t="inlineStr">
         <is>
@@ -8955,11 +8955,11 @@
         </is>
       </c>
       <c r="B171" s="2">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="C171" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
@@ -8970,7 +8970,7 @@
         </is>
       </c>
       <c r="B172" s="2">
-        <v>0.015</v>
+        <v>0.04587237692136338</v>
       </c>
       <c r="C172" s="0" t="inlineStr">
         <is>
@@ -8985,7 +8985,7 @@
         </is>
       </c>
       <c r="B173" s="2">
-        <v>0.01</v>
+        <v>0.041493777249306446</v>
       </c>
       <c r="C173" s="0" t="inlineStr">
         <is>
@@ -9000,7 +9000,7 @@
         </is>
       </c>
       <c r="B174" s="2">
-        <v>0.045</v>
+        <v>0.024842152906941306</v>
       </c>
       <c r="C174" s="0" t="inlineStr">
         <is>
@@ -9015,7 +9015,7 @@
         </is>
       </c>
       <c r="B175" s="2">
-        <v>0.04</v>
+        <v>0.019809059504605663</v>
       </c>
       <c r="C175" s="0" t="inlineStr">
         <is>
@@ -9030,7 +9030,7 @@
         </is>
       </c>
       <c r="B176" s="2">
-        <v>0.06</v>
+        <v>0.062495258171033366</v>
       </c>
       <c r="C176" s="0" t="inlineStr">
         <is>
@@ -9045,7 +9045,7 @@
         </is>
       </c>
       <c r="B177" s="2">
-        <v>0.04</v>
+        <v>0.04260731658392249</v>
       </c>
       <c r="C177" s="0" t="inlineStr">
         <is>
@@ -9060,11 +9060,11 @@
         </is>
       </c>
       <c r="B178" s="2">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="C178" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
@@ -9075,7 +9075,7 @@
         </is>
       </c>
       <c r="B179" s="2">
-        <v>0.1</v>
+        <v>0.10922616465163659</v>
       </c>
       <c r="C179" s="0" t="inlineStr">
         <is>
@@ -9090,11 +9090,11 @@
         </is>
       </c>
       <c r="B180" s="2">
-        <v>0</v>
+        <v>0.015550427257977284</v>
       </c>
       <c r="C180" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
@@ -9105,7 +9105,7 @@
         </is>
       </c>
       <c r="B181" s="2">
-        <v>0.07</v>
+        <v>1.174186491064466e-16</v>
       </c>
       <c r="C181" s="0" t="inlineStr">
         <is>
@@ -9120,7 +9120,7 @@
         </is>
       </c>
       <c r="B182" s="2">
-        <v>0.04</v>
+        <v>0.026240752485890893</v>
       </c>
       <c r="C182" s="0" t="inlineStr">
         <is>
@@ -9135,7 +9135,7 @@
         </is>
       </c>
       <c r="B183" s="2">
-        <v>0.04</v>
+        <v>0.054448536306753274</v>
       </c>
       <c r="C183" s="0" t="inlineStr">
         <is>
@@ -9165,7 +9165,7 @@
         </is>
       </c>
       <c r="B185" s="2">
-        <v>0.06</v>
+        <v>0.05371923167958349</v>
       </c>
       <c r="C185" s="0" t="inlineStr">
         <is>
@@ -9180,7 +9180,7 @@
         </is>
       </c>
       <c r="B186" s="2">
-        <v>0.06</v>
+        <v>0.054060933702789804</v>
       </c>
       <c r="C186" s="0" t="inlineStr">
         <is>
@@ -9195,7 +9195,7 @@
         </is>
       </c>
       <c r="B187" s="2">
-        <v>0.07</v>
+        <v>0.08894384122463511</v>
       </c>
       <c r="C187" s="0" t="inlineStr">
         <is>
@@ -9210,7 +9210,7 @@
         </is>
       </c>
       <c r="B188" s="2">
-        <v>0.07</v>
+        <v>0.020019816287178877</v>
       </c>
       <c r="C188" s="0" t="inlineStr">
         <is>
@@ -9225,7 +9225,7 @@
         </is>
       </c>
       <c r="B189" s="2">
-        <v>0.21</v>
+        <v>0.29613714390065743</v>
       </c>
       <c r="C189" s="0" t="inlineStr">
         <is>
@@ -9240,7 +9240,7 @@
         </is>
       </c>
       <c r="B190" s="2">
-        <v>0.21</v>
+        <v>0.05407072368421051</v>
       </c>
       <c r="C190" s="0" t="inlineStr">
         <is>
@@ -9255,11 +9255,11 @@
         </is>
       </c>
       <c r="B191" s="2">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="C191" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
@@ -9270,7 +9270,7 @@
         </is>
       </c>
       <c r="B192" s="2">
-        <v>0.09</v>
+        <v>0.10315299543741321</v>
       </c>
       <c r="C192" s="0" t="inlineStr">
         <is>
@@ -9285,7 +9285,7 @@
         </is>
       </c>
       <c r="B193" s="2">
-        <v>15</v>
+        <v>7.67</v>
       </c>
       <c r="C193" s="0" t="inlineStr">
         <is>
@@ -9420,7 +9420,7 @@
         </is>
       </c>
       <c r="B202" s="2">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="C202" s="0" t="inlineStr">
         <is>
@@ -9450,7 +9450,7 @@
         </is>
       </c>
       <c r="B204" s="2">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C204" s="0" t="inlineStr">
         <is>
@@ -9461,26 +9461,26 @@
     <row r="205">
       <c r="A205" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesIncrease:value</t>
+          <t xml:space="preserve">target:companySalesIncrease:max</t>
         </is>
       </c>
       <c r="B205" s="2">
-        <v>0</v>
+        <v>252.69</v>
       </c>
       <c r="C205" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayCagr:max</t>
+          <t xml:space="preserve">target:companySalesIncrease:value</t>
         </is>
       </c>
       <c r="B206" s="2">
-        <v>10</v>
+        <v>133.5</v>
       </c>
       <c r="C206" s="0" t="inlineStr">
         <is>
@@ -9491,11 +9491,11 @@
     <row r="207">
       <c r="A207" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayCagr:value</t>
+          <t xml:space="preserve">target:employeePayCagr:max</t>
         </is>
       </c>
       <c r="B207" s="2">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C207" s="0" t="inlineStr">
         <is>
@@ -9506,26 +9506,26 @@
     <row r="208">
       <c r="A208" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayIncrease:value</t>
+          <t xml:space="preserve">target:employeePayCagr:value</t>
         </is>
       </c>
       <c r="B208" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C208" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:investmentSalesRatio:max</t>
+          <t xml:space="preserve">target:employeePayIncrease:max</t>
         </is>
       </c>
       <c r="B209" s="2">
-        <v>70</v>
+        <v>3.74</v>
       </c>
       <c r="C209" s="0" t="inlineStr">
         <is>
@@ -9536,11 +9536,11 @@
     <row r="210">
       <c r="A210" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:investmentSalesRatio:value</t>
+          <t xml:space="preserve">target:employeePayIncrease:value</t>
         </is>
       </c>
       <c r="B210" s="2">
-        <v>30</v>
+        <v>2.85</v>
       </c>
       <c r="C210" s="0" t="inlineStr">
         <is>
@@ -9551,11 +9551,11 @@
     <row r="211">
       <c r="A211" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:laborProductivityCagr:max</t>
+          <t xml:space="preserve">target:investmentSalesRatio:max</t>
         </is>
       </c>
       <c r="B211" s="2">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="C211" s="0" t="inlineStr">
         <is>
@@ -9566,11 +9566,11 @@
     <row r="212">
       <c r="A212" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:laborProductivityCagr:value</t>
+          <t xml:space="preserve">target:investmentSalesRatio:value</t>
         </is>
       </c>
       <c r="B212" s="2">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="C212" s="0" t="inlineStr">
         <is>
@@ -9581,11 +9581,11 @@
     <row r="213">
       <c r="A213" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:localBenchmark:max</t>
+          <t xml:space="preserve">target:laborProductivityCagr:max</t>
         </is>
       </c>
       <c r="B213" s="2">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C213" s="0" t="inlineStr">
         <is>
@@ -9596,11 +9596,11 @@
     <row r="214">
       <c r="A214" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:localBenchmark:value</t>
+          <t xml:space="preserve">target:laborProductivityCagr:value</t>
         </is>
       </c>
       <c r="B214" s="2">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C214" s="0" t="inlineStr">
         <is>
@@ -9611,11 +9611,11 @@
     <row r="215">
       <c r="A215" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayCagr:max</t>
+          <t xml:space="preserve">target:localBenchmark:max</t>
         </is>
       </c>
       <c r="B215" s="2">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="C215" s="0" t="inlineStr">
         <is>
@@ -9626,11 +9626,11 @@
     <row r="216">
       <c r="A216" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayCagr:value</t>
+          <t xml:space="preserve">target:localBenchmark:value</t>
         </is>
       </c>
       <c r="B216" s="2">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="C216" s="0" t="inlineStr">
         <is>
@@ -9641,26 +9641,26 @@
     <row r="217">
       <c r="A217" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayIncrease:value</t>
+          <t xml:space="preserve">target:officerPayCagr:max</t>
         </is>
       </c>
       <c r="B217" s="2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C217" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesCagr:max</t>
+          <t xml:space="preserve">target:officerPayCagr:value</t>
         </is>
       </c>
       <c r="B218" s="2">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="C218" s="0" t="inlineStr">
         <is>
@@ -9671,41 +9671,41 @@
     <row r="219">
       <c r="A219" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesCagr:value</t>
+          <t xml:space="preserve">target:officerPayIncrease:value</t>
         </is>
       </c>
       <c r="B219" s="2">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="C219" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesIncrease:value</t>
+          <t xml:space="preserve">target:projectSalesCagr:max</t>
         </is>
       </c>
       <c r="B220" s="2">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="C220" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesShare:max</t>
+          <t xml:space="preserve">target:projectSalesCagr:value</t>
         </is>
       </c>
       <c r="B221" s="2">
-        <v>95</v>
+        <v>22</v>
       </c>
       <c r="C221" s="0" t="inlineStr">
         <is>
@@ -9716,11 +9716,11 @@
     <row r="222">
       <c r="A222" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesShare:value</t>
+          <t xml:space="preserve">target:projectSalesIncrease:max</t>
         </is>
       </c>
       <c r="B222" s="2">
-        <v>70</v>
+        <v>136.84</v>
       </c>
       <c r="C222" s="0" t="inlineStr">
         <is>
@@ -9731,26 +9731,26 @@
     <row r="223">
       <c r="A223" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:valueAddedIncrease:value</t>
+          <t xml:space="preserve">target:projectSalesIncrease:value</t>
         </is>
       </c>
       <c r="B223" s="2">
-        <v>0</v>
+        <v>76.44</v>
       </c>
       <c r="C223" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:valueAddedSubsidyRatio:max</t>
+          <t xml:space="preserve">target:projectSalesShare:max</t>
         </is>
       </c>
       <c r="B224" s="2">
-        <v>350</v>
+        <v>95</v>
       </c>
       <c r="C224" s="0" t="inlineStr">
         <is>
@@ -9761,13 +9761,73 @@
     <row r="225">
       <c r="A225" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">target:projectSalesShare:value</t>
+        </is>
+      </c>
+      <c r="B225" s="2">
+        <v>65</v>
+      </c>
+      <c r="C225" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:valueAddedIncrease:max</t>
+        </is>
+      </c>
+      <c r="B226" s="2">
+        <v>33.43</v>
+      </c>
+      <c r="C226" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:valueAddedIncrease:value</t>
+        </is>
+      </c>
+      <c r="B227" s="2">
+        <v>18.78</v>
+      </c>
+      <c r="C227" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:valueAddedSubsidyRatio:max</t>
+        </is>
+      </c>
+      <c r="B228" s="2">
+        <v>350</v>
+      </c>
+      <c r="C228" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">target:valueAddedSubsidyRatio:value</t>
         </is>
       </c>
-      <c r="B225" s="2">
+      <c r="B229" s="2">
         <v>213</v>
       </c>
-      <c r="C225" s="0" t="inlineStr">
+      <c r="C229" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">入力済み</t>
         </is>
@@ -9795,7 +9855,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4fX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjU5LCJvZmZpY2VyUGF5IjowLjM4LCJkZXByZWNpYXRpb24iOjEuOSwib3RoZXJTZ2EiOjkuNSwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NS4zMSwiZW1wbG95ZWVCb251cyI6MC4yOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNCwib2ZmaWNlckJvbnVzIjowLjA0LCJjb2dzRGVwcmVjaWF0aW9uIjowLjQ3LCJzZ2FEZXByZWNpYXRpb24iOjEuNDMsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMzh9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNTQsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3LjE2LCJlbXBsb3llZUJvbnVzIjowLjM4LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjUyLCJvZmZpY2VyQm9udXMiOjAuMDYsImNvZ3NEZXByZWNpYXRpb24iOjAuMjksInNnYURlcHJlY2lhdGlvbiI6MS4xNSwicmVzZWFyY2hEZXZlbG9wbWVudCI6MC4yOX19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6NiwiZW1wbG95ZWVTYWxhcnkiOjUuNywiZW1wbG95ZWVCb251cyI6MC4zLCJvZmZpY2VyUGF5IjowLjQsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzYsIm9mZmljZXJCb251cyI6MC4wNCwiZGVwcmVjaWF0aW9uIjoyLCJjb2dzRGVwcmVjaWF0aW9uIjowLjUsInNnYURlcHJlY2lhdGlvbiI6MS41LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjQsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsImVtcGxveWVlU2FsYXJ5Ijo3LjYsImVtcGxveWVlQm9udXMiOjAuNCwib2ZmaWNlclBheSI6MC42LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjU0LCJvZmZpY2VyQm9udXMiOjAuMDYsImRlcHJlY2lhdGlvbiI6MS41LCJjb2dzRGVwcmVjaWF0aW9uIjowLjMsInNnYURlcHJlY2lhdGlvbiI6MS4yLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjMsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjIxLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjowLjA3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjA3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAuMDEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA2LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wMSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MC4wMDUsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMSwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNiwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MCwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDEsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDE1LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wOSwib3RoZXJTZ2FSYXRlRW5kIjowLjEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA2LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6NDUsInN1YnNpZHkiOjE1LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6Wy0wLjA1LDAuNF0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDJdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjFdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbLTAuMDMsMC4yXSwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAyXSwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOlswLDAuMV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlstMC4xLDAuMl0sIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAyXSwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6Wy0wLjA1LDAuMV0sIm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDJdLCJwcm9qZWN0U2FsZXNHcm93dGgiOlstMC4wNSwwLjRdLCJvdGhlclNhbGVzR3Jvd3RoIjpbLTAuMSwwLjJdLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjpbMCwwLjAzXSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOlswLDAuMDNdLCJwcm9qZWN0UGF5R3Jvd3RoIjpbMC4wNDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLDAuMDhdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjpbLTAuMDMsMC4yXSwib3RoZXJIZWFkY291bnRHcm93dGgiOlstMC4wNSwwLjFdLCJwcm9qZWN0U2dhUmF0ZUVuZCI6WzAuMDQsMC4yNV0sIm90aGVyU2dhUmF0ZUVuZCI6WzAuMDQsMC4yNV0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjpbMCwwLjFdLCJ1c2VmdWxMaWZlIjpbNSwyMF0sImludmVzdG1lbnQiOlsxNSwyMDBdLCJzdWJzaWR5IjpbMSw1MF0sImxvY2FsQmVuY2htYXJrIjpbMCwxMDBdfSwidGFyZ2V0cyI6eyJjb21wYW55U2FsZXNDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlTYWxlc0luY3JlYXNlIjp7InZhbHVlIjowLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjozLjUsIm1heCI6NywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc1NoYXJlIjp7InZhbHVlIjo3MCwibWF4Ijo5NSwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0NhZ3IiOnsidmFsdWUiOjIyLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsYWJvclByb2R1Y3Rpdml0eUNhZ3IiOnsidmFsdWUiOjIxLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZEluY3JlYXNlIjp7InZhbHVlIjowLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjozMCwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX19LCJmb3JlY2FzdE92ZXJyaWRlcyI6e30sImZ1dHVyZUlucHV0QmFzaXMiOiJvdGhlciIsImlucHV0VmFsdWVzIjp7ImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xIjoxMzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTMiOjkyLjc1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6MC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMyLjY1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6MC44MiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEwIjowLjA5LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTIiOjExLjY3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjAuNjIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNCI6Mi40NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1IjowLjY0LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMSI6NzIsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny00IjoyMy4wNCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjYuNzgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny04Ijo1LjE5LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOSI6MC4zNiwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEwIjoxLjgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMyI6OTAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEiOjE0My4yLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMyI6OTcuMzgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi00IjowLjc2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNyI6MzQuNTIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi05IjowLjg2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEyIjoxMi40NywiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEzIjowLjY2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTQiOjIuNTgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNSI6MC42NywiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEiOjc2LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNCI6MjQuMzIsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny02Ijo3LjA0LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctOCI6NS41OSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTkiOjAuMzgsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xMCI6MS45LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTMiOjk1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xIjoxNTAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0zIjoxMDIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi00IjowLjgsImFjdHVhbDpjb21wYW55OjIwMjU6Mi03IjozNi40LCJhY3R1YWw6Y29tcGFueToyMDI1OjItOSI6MC45LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEyIjoxMy4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTMiOjAuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE0IjoyLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNSI6MC43LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMSI6ODAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNS42LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6Ny4zLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTkiOjAuNCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEwIjoyLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTMiOjEwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTE0IjoyLCJiYWxhbmNlLXNoZWV0OjIwMjM6YXNzZXRzIjoxMzIsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NywiYmFsYW5jZS1zaGVldDoyMDIzOmNhc2giOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRBc3NldHMiOjY1LCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzLCJiYWxhbmNlLXNoZWV0OjIwMjM6YnVpbGRpbmdzIjoxOSwiYmFsYW5jZS1zaGVldDoyMDIzOm1hY2hpbmVyeSI6MjQsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmludGFuZ2libGVBc3NldHMiOjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzb2Z0d2FyZSI6NSwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NSwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRMaWFiaWxpdGllcyI6MzksImJhbGFuY2Utc2hlZXQ6MjAyMzpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2LCJiYWxhbmNlLXNoZWV0OjIwMjM6bG9uZ1Rlcm1EZWJ0IjoyOSwiYmFsYW5jZS1zaGVldDoyMDIzOm5ldEFzc2V0cyI6NTcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGV4Ijo1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50QXNzZXRzIjo3MiwiYmFsYW5jZS1zaGVldDoyMDI0OmNhc2giOjI1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6dGFuZ2libGVBc3NldHMiOjU4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YnVpbGRpbmdzIjoyMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmludGFuZ2libGVBc3NldHMiOjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NiwiYmFsYW5jZS1zaGVldDoyMDI0OmxpYWJpbGl0aWVzIjo3OSwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRMaWFiaWxpdGllcyI6NDEsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkTGlhYmlsaXRpZXMiOjM4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bG9uZ1Rlcm1EZWJ0IjozMSwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaGFyZWhvbGRlckVxdWl0eSI6NjEsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4LCJiYWxhbmNlLXNoZWV0OjIwMjU6YXNzZXRzIjoxNTYsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50QXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3LCJiYWxhbmNlLXNoZWV0OjIwMjU6Zml4ZWRBc3NldHMiOjc4LCJiYWxhbmNlLXNoZWV0OjIwMjU6dGFuZ2libGVBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMiwiYmFsYW5jZS1zaGVldDoyMDI1Om1hY2hpbmVyeSI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjksImJhbGFuY2Utc2hlZXQ6MjAyNTpzb2Z0d2FyZSI6NywiYmFsYW5jZS1zaGVldDoyMDI1OmxpYWJpbGl0aWVzIjo4MywiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaG9ydFRlcm1EZWJ0IjoxMSwiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkTGlhYmlsaXRpZXMiOjQwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMiwiYmFsYW5jZS1zaGVldDoyMDI1Om5ldEFzc2V0cyI6NzMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaGFyZWhvbGRlckVxdWl0eSI6NzAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGV4IjoxMCwiZnV0dXJlLWNhcGV4OjIwMjYiOjE1LCJmdXR1cmUtY2FwZXg6MjAyNyI6MTUsImZ1dHVyZS1jYXBleDoyMDI4IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjkiOjAsImZ1dHVyZS1jYXBleDoyMDMwIjowLCJmdXR1cmUtY2FwZXg6MjAzMSI6MCwiZHJpdmVyOnByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDoxIjowLjMsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMjEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6LTAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC40LCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MC4wNywiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjEiOjAuMSwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjAiOi0wLjAzLCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZToxIjowLjIsImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAuMDEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLjAyLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDYsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4xLCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6LTAuMSwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4yLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjAuMDIsImRyaXZlcjpvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wNCwiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZToxIjowLjA4LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDEsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjotMC4wNSwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMSwiZHJpdmVyOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLjAyLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoIjowLjIxLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjEiOjAuNCwiZHJpdmVyOm90aGVyU2FsZXNHcm93dGgiOjAuMDYsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoOjAiOi0wLjEsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoOjEiOjAuMiwiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDoxIjowLjAzLCJkcml2ZXI6cHJvamVjdFBheUdyb3d0aCI6MC4wNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGg6MCI6MC4wNDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjA0NSwiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDoxIjowLjA4LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MCI6LTAuMDMsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjEiOjAuMiwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjAxNSwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MSI6MC4xLCJkcml2ZXI6cHJvamVjdFNnYVJhdGVFbmQiOjAuMDksImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDowIjowLjA0LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MSI6MC4yNSwiZHJpdmVyOm90aGVyU2dhUmF0ZUVuZCI6MC4xLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjAiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MSI6MC4yNSwiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA2LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOnVzZWZ1bExpZmUiOjEwLCJkcml2ZXItcmFuZ2U6dXNlZnVsTGlmZTowIjo1LCJkcml2ZXItcmFuZ2U6dXNlZnVsTGlmZToxIjoyMCwiZHJpdmVyOmludmVzdG1lbnQiOjQ1LCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDowIjoxNSwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MSI6MjAwLCJkcml2ZXI6c3Vic2lkeSI6MTUsImRyaXZlci1yYW5nZTpzdWJzaWR5OjAiOjEsImRyaXZlci1yYW5nZTpzdWJzaWR5OjEiOjUwLCJkcml2ZXI6bG9jYWxCZW5jaG1hcmsiOjIzLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MCI6MCwiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjEiOjEwMCwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6dmFsdWUiOjIxLCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55UGF5U2NoZWR1bGU6dmFsdWUiOjMuNSwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTptYXgiOjcsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTp2YWx1ZSI6NzAsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTptYXgiOjk1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2Fncjp2YWx1ZSI6MjIsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTp2YWx1ZSI6MCwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2Fncjp2YWx1ZSI6MjEsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6bWF4IjozNSwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTp2YWx1ZSI6MCwidGFyZ2V0OmVtcGxveWVlUGF5Q2Fncjp2YWx1ZSI6NywidGFyZ2V0OmVtcGxveWVlUGF5Q2FncjptYXgiOjEwLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlJbmNyZWFzZTp2YWx1ZSI6MCwidGFyZ2V0OmludmVzdG1lbnRTYWxlc1JhdGlvOnZhbHVlIjozMCwidGFyZ2V0OmludmVzdG1lbnRTYWxlc1JhdGlvOm1heCI6NzAsInRhcmdldDp2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvOnZhbHVlIjoyMTMsInRhcmdldDp2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvOm1heCI6MzUwLCJ0YXJnZXQ6bG9jYWxCZW5jaG1hcms6dmFsdWUiOjIzLCJ0YXJnZXQ6bG9jYWxCZW5jaG1hcms6bWF4Ijo0MCwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOnZhbHVlIjo2LCJ0YXJnZXQ6b2ZmaWNlclBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0Om9mZmljZXJQYXlJbmNyZWFzZTp2YWx1ZSI6MH0sIm1ldHJpY0dyb3VwQmFzZXMiOnsiY29tcGFueVNhbGVzIjoicmF0ZSIsInByb2plY3RTYWxlcyI6InJhdGUiLCJsYWJvclByb2R1Y3Rpdml0eSI6InJhdGUiLCJlbXBsb3llZVBheSI6InJhdGUifSwiYXBwbGljYXRpb25DYXRlZ29yeSI6ImdlbmVyYWwifQ==</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4fX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjU5LCJvZmZpY2VyUGF5IjowLjM4LCJkZXByZWNpYXRpb24iOjEuOSwib3RoZXJTZ2EiOjkuNSwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NS4zMSwiZW1wbG95ZWVCb251cyI6MC4yOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNCwib2ZmaWNlckJvbnVzIjowLjA0LCJjb2dzRGVwcmVjaWF0aW9uIjowLjQ3LCJzZ2FEZXByZWNpYXRpb24iOjEuNDMsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMzh9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNTQsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3LjE2LCJlbXBsb3llZUJvbnVzIjowLjM4LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjUyLCJvZmZpY2VyQm9udXMiOjAuMDYsImNvZ3NEZXByZWNpYXRpb24iOjAuMjksInNnYURlcHJlY2lhdGlvbiI6MS4xNSwicmVzZWFyY2hEZXZlbG9wbWVudCI6MC4yOX19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6NiwiZW1wbG95ZWVTYWxhcnkiOjUuNywiZW1wbG95ZWVCb251cyI6MC4zLCJvZmZpY2VyUGF5IjowLjQsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzYsIm9mZmljZXJCb251cyI6MC4wNCwiZGVwcmVjaWF0aW9uIjoyLCJjb2dzRGVwcmVjaWF0aW9uIjowLjUsInNnYURlcHJlY2lhdGlvbiI6MS41LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjQsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsImVtcGxveWVlU2FsYXJ5Ijo3LjYsImVtcGxveWVlQm9udXMiOjAuNCwib2ZmaWNlclBheSI6MC42LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjU0LCJvZmZpY2VyQm9udXMiOjAuMDYsImRlcHJlY2lhdGlvbiI6MS41LCJjb2dzRGVwcmVjaWF0aW9uIjowLjMsInNnYURlcHJlY2lhdGlvbiI6MS4yLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjMsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA3MDcyMzY4NDIxMDUxLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjoxLjE3NDE4NjQ5MTA2NDQ2NmUtMTYsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDE5ODE2Mjg3MTc4ODc3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDQ0ODUzNjMwNjc1MzI3NCwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwNjA5MzM3MDI3ODk4MDQsIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNjA3MzE2NTgzOTIyNDksIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4MDkwNTk1MDQ2MDU2NjMsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MTQ5Mzc3NzI0OTMwNjQ0Niwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjI5NjEzNzE0MzkwMDY1NzQzLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjQ5NTI1ODE3MTAzMzM2NiwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTU1NTA0MjcyNTc5NzcyODQsIm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwicHJvamVjdFBheUdyb3d0aCI6MC4wODg5NDM4NDEyMjQ2MzUxMSwib3RoZXJQYXlHcm93dGgiOjAuMDI0ODQyMTUyOTA2OTQxMzA2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjAyNjI0MDc1MjQ4NTg5MDg5Mywib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODcyMzc2OTIxMzYzMzgsInByb2plY3RTZ2FSYXRlRW5kIjowLjEwMzE1Mjk5NTQzNzQxMzIxLCJvdGhlclNnYVJhdGVFbmQiOjAuMTA5MjI2MTY0NjUxNjM2NTksInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzcxOTIzMTY3OTU4MzQ5LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6MjMsInN1YnNpZHkiOjcuNjcsImxvY2FsQmVuY2htYXJrIjoyM30sImRyaXZlclJhbmdlcyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjpbLTAuMDUsMC4zXSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDEuNjY1MzM0NTM2OTM3NzM0OGUtMTZdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkzMjUzMzA1MDE4NDY5MjcsMC4wMjA3MzU5OTQxODMxODkxNjZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlswLjA0MDc2MDg2OTU2NTIxNzE4NCwwLjA0NDM4NDA1Nzk3MTAxNDUyXSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDAwMTM0NTc1NTY5MzU4MTk3MzddLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MTM5NDU3MDIzNzE3NDQzLDAuMDIwNTUzNDU5OTE0NzYzMDk1XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjAzOTE2NjY2NjY2NjY2NjY4LDAuMDQyNTAwMDAwMDAwMDAwMDldLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbMC4xNSwwLjNdLCJvdGhlclNhbGVzR3Jvd3RoIjpbMC4wNjA3NjA4Njk1NjUyMTcxOSwwLjA2NDM4NDA1Nzk3MTAxNDUzXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMC4wMDUsMC4wMDUxMzQ1NzU1NjkzNTgxOTc1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLjAyNDEzOTQ1NzAyMzcxNzQ0NCwwLjAyNTU1MzQ1OTkxNDc2MzA5Nl0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6WzAuMDQ0MTY2NjY2NjY2NjY2NjgsMC4wNDc1MDAwMDAwMDAwMDAwOV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMC4wODQ5OTk5OTk5OTk5OTk5OSwwLjEzNV0sIm90aGVyU2dhUmF0ZUVuZCI6WzAuMDg5Mjg1NzE0Mjg1NzE0MjcsMC4xMTkyODU3MTQyODU3MTQyN10sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjpbMC4wNDI2MzE1Nzg5NDczNjgzNiwwLjA2NTU1NTU1NTU1NTU1NTU4XSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjAsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6MTMzLjUsIm1heCI6MjUyLjY5LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjoyLCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NjUsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo3Ni40NCwibWF4IjoxMzYuODQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsYWJvclByb2R1Y3Rpdml0eUNhZ3IiOnsidmFsdWUiOjIxLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZEluY3JlYXNlIjp7InZhbHVlIjoxOC43OCwibWF4IjozMy40MywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5Q2FnciI6eyJ2YWx1ZSI6NywibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5SW5jcmVhc2UiOnsidmFsdWUiOjIuODUsIm1heCI6My43NCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjoxNSwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX19LCJmb3JlY2FzdE92ZXJyaWRlcyI6eyIyMDI5Om90aGVyOnNhbGVzIjo4NS4xMywiMjAyOTpwcm9qZWN0OjctOCI6Ny44OX0sImZ1dHVyZUlucHV0QmFzaXMiOiJvdGhlciIsImlucHV0VmFsdWVzIjp7ImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xIjoxMzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTMiOjkyLjc1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6MC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMyLjY1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6MC44MiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEwIjowLjA5LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTIiOjExLjY3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjAuNjIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNCI6Mi40NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1IjowLjY0LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMSI6NzIsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny00IjoyMy4wNCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjYuNzgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny04Ijo1LjE5LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOSI6MC4zNiwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEwIjoxLjgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMyI6OTAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEiOjE0My4yLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMyI6OTcuMzgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi00IjowLjc2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNyI6MzQuNTIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi05IjowLjg2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEyIjoxMi40NywiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEzIjowLjY2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTQiOjIuNTgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNSI6MC42NywiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEiOjc2LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNCI6MjQuMzIsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny02Ijo3LjA0LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctOCI6NS41OSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTkiOjAuMzgsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xMCI6MS45LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTMiOjk1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xIjoxNTAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0zIjoxMDIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi00IjowLjgsImFjdHVhbDpjb21wYW55OjIwMjU6Mi03IjozNi40LCJhY3R1YWw6Y29tcGFueToyMDI1OjItOSI6MC45LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEyIjoxMy4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTMiOjAuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE0IjoyLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNSI6MC43LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMSI6ODAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNS42LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6Ny4zLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTkiOjAuNCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEwIjoyLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTMiOjEwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTE0IjoyLCJiYWxhbmNlLXNoZWV0OjIwMjM6YXNzZXRzIjoxMzIsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NywiYmFsYW5jZS1zaGVldDoyMDIzOmNhc2giOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRBc3NldHMiOjY1LCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzLCJiYWxhbmNlLXNoZWV0OjIwMjM6YnVpbGRpbmdzIjoxOSwiYmFsYW5jZS1zaGVldDoyMDIzOm1hY2hpbmVyeSI6MjQsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmludGFuZ2libGVBc3NldHMiOjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzb2Z0d2FyZSI6NSwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NSwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRMaWFiaWxpdGllcyI6MzksImJhbGFuY2Utc2hlZXQ6MjAyMzpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2LCJiYWxhbmNlLXNoZWV0OjIwMjM6bG9uZ1Rlcm1EZWJ0IjoyOSwiYmFsYW5jZS1zaGVldDoyMDIzOm5ldEFzc2V0cyI6NTcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGV4Ijo1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50QXNzZXRzIjo3MiwiYmFsYW5jZS1zaGVldDoyMDI0OmNhc2giOjI1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6dGFuZ2libGVBc3NldHMiOjU4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YnVpbGRpbmdzIjoyMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmludGFuZ2libGVBc3NldHMiOjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NiwiYmFsYW5jZS1zaGVldDoyMDI0OmxpYWJpbGl0aWVzIjo3OSwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRMaWFiaWxpdGllcyI6NDEsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkTGlhYmlsaXRpZXMiOjM4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bG9uZ1Rlcm1EZWJ0IjozMSwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaGFyZWhvbGRlckVxdWl0eSI6NjEsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4LCJiYWxhbmNlLXNoZWV0OjIwMjU6YXNzZXRzIjoxNTYsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50QXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3LCJiYWxhbmNlLXNoZWV0OjIwMjU6Zml4ZWRBc3NldHMiOjc4LCJiYWxhbmNlLXNoZWV0OjIwMjU6dGFuZ2libGVBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMiwiYmFsYW5jZS1zaGVldDoyMDI1Om1hY2hpbmVyeSI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjksImJhbGFuY2Utc2hlZXQ6MjAyNTpzb2Z0d2FyZSI6NywiYmFsYW5jZS1zaGVldDoyMDI1OmxpYWJpbGl0aWVzIjo4MywiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaG9ydFRlcm1EZWJ0IjoxMSwiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkTGlhYmlsaXRpZXMiOjQwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMiwiYmFsYW5jZS1zaGVldDoyMDI1Om5ldEFzc2V0cyI6NzMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaGFyZWhvbGRlckVxdWl0eSI6NzAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGV4IjoxMCwiZnV0dXJlLWNhcGV4OjIwMjYiOjE1LCJmdXR1cmUtY2FwZXg6MjAyNyI6MTUsImZ1dHVyZS1jYXBleDoyMDI4IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjkiOjAsImZ1dHVyZS1jYXBleDoyMDMwIjowLCJmdXR1cmUtY2FwZXg6MjAzMSI6MCwiZHJpdmVyOnByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDoxIjowLjMsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDcwNzIzNjg0MjEwNTEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjEuMTc0MTg2NDkxMDY0NDY2ZS0xNiwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDE5ODE2Mjg3MTc4ODc3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZTowIjowLjAxOTMyNTMzMDUwMTg0NjkyNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA3MzU5OTQxODMxODkxNjYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDQ0ODUzNjMwNjc1MzI3NCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDYwOTMzNzAyNzg5ODA0LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZToxIjowLjA1NzAxNzU0Mzg1OTY0OTE5LCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI2MDczMTY1ODM5MjI0OSwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODA5MDU5NTA0NjA1NjYzLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkxMzk0NTcwMjM3MTc0NDMsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZToxIjowLjAyMDU1MzQ1OTkxNDc2MzA5NSwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MTQ5Mzc3NzI0OTMwNjQ0NiwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjAiOjAuMDM5MTY2NjY2NjY2NjY2NjgsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZToxIjowLjA0MjUwMDAwMDAwMDAwMDA5LCJkcml2ZXI6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MCwiZHJpdmVyOnByb2plY3RTYWxlc0dyb3d0aCI6MC4yOTYxMzcxNDM5MDA2NTc0MywiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDowIjowLjE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjEiOjAuMywiZHJpdmVyOm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNDk1MjU4MTcxMDMzMzY2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTU1NTA0MjcyNTc5NzcyODQsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDg4OTQzODQxMjI0NjM1MTEsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0MjE1MjkwNjk0MTMwNiwiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjAiOjAuMDI0MTM5NDU3MDIzNzE3NDQ0LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wMjU1NTM0NTk5MTQ3NjMwOTYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjAyNjI0MDc1MjQ4NTg5MDg5MywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTg3MjM3NjkyMTM2MzM4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MCI6MC4wNDQxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjEiOjAuMDQ3NTAwMDAwMDAwMDAwMDksImRyaXZlcjpwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMDMxNTI5OTU0Mzc0MTMyMSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjAiOjAuMDg0OTk5OTk5OTk5OTk5OTksImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDoxIjowLjEzNSwiZHJpdmVyOm90aGVyU2dhUmF0ZUVuZCI6MC4xMDkyMjYxNjQ2NTE2MzY1OSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLjA4OTI4NTcxNDI4NTcxNDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMTE5Mjg1NzE0Mjg1NzE0MjcsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM3MTkyMzE2Nzk1ODM0OSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAuMDQyNjMxNTc4OTQ3MzY4MzYsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjA2NTU1NTU1NTU1NTU1NTU4LCJkcml2ZXI6dXNlZnVsTGlmZSI6MTAsImRyaXZlci1yYW5nZTp1c2VmdWxMaWZlOjAiOjUsImRyaXZlci1yYW5nZTp1c2VmdWxMaWZlOjEiOjIwLCJkcml2ZXI6aW52ZXN0bWVudCI6MjMsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjAiOjE1LCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDoxIjoyMDAsImRyaXZlcjpzdWJzaWR5Ijo3LjY3LCJkcml2ZXItcmFuZ2U6c3Vic2lkeTowIjoxLCJkcml2ZXItcmFuZ2U6c3Vic2lkeToxIjo1MCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoyMCwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjoxMzMuNSwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTp2YWx1ZSI6MiwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTptYXgiOjcsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTp2YWx1ZSI6NjUsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTptYXgiOjk1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2Fncjp2YWx1ZSI6MjIsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTp2YWx1ZSI6NzYuNDQsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6dmFsdWUiOjIxLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOm1heCI6MzUsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6dmFsdWUiOjE4Ljc4LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOnZhbHVlIjo3LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOm1heCI6MTAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOnZhbHVlIjoyLjg1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86dmFsdWUiOjE1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86bWF4Ijo3MCwidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86dmFsdWUiOjIxMywidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86bWF4IjozNTAsInRhcmdldDpsb2NhbEJlbmNobWFyazp2YWx1ZSI6MjMsInRhcmdldDpsb2NhbEJlbmNobWFyazptYXgiOjQwLCJ0YXJnZXQ6b2ZmaWNlclBheUNhZ3I6dmFsdWUiOjYsInRhcmdldDpvZmZpY2VyUGF5Q2FncjptYXgiOjEwLCJ0YXJnZXQ6b2ZmaWNlclBheUluY3JlYXNlOnZhbHVlIjowLCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6bWF4IjoyNTIuNjksInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTptYXgiOjEzNi44NCwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTptYXgiOjMzLjQzLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlJbmNyZWFzZTptYXgiOjMuNzR9LCJtZXRyaWNHcm91cEJhc2VzIjp7ImNvbXBhbnlTYWxlcyI6InJhdGUiLCJwcm9qZWN0U2FsZXMiOiJyYXRlIiwibGFib3JQcm9kdWN0aXZpdHkiOiJyYXRlIiwiZW1wbG95ZWVQYXkiOiJyYXRlIn0sImFwcGxpY2F0aW9uQ2F0ZWdvcnkiOiJnZW5lcmFsIn0=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix subsidy decimal ceiling in standard sample
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <v>372.8813559322032</v>
+        <v>373.36814621409894</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
@@ -6362,11 +6362,11 @@
         </is>
       </c>
       <c r="B28" s="2">
-        <v>7.67</v>
+        <v>7.66</v>
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">50億円以下、かつ投資額の1/3以下（現在上限7.67億円）</t>
+          <t xml:space="preserve">50億円以下、かつ投資額の1/3以下（現在上限7.66億円）</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
@@ -9285,7 +9285,7 @@
         </is>
       </c>
       <c r="B193" s="2">
-        <v>7.67</v>
+        <v>7.66</v>
       </c>
       <c r="C193" s="0" t="inlineStr">
         <is>
@@ -9855,7 +9855,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4fX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjU5LCJvZmZpY2VyUGF5IjowLjM4LCJkZXByZWNpYXRpb24iOjEuOSwib3RoZXJTZ2EiOjkuNSwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NS4zMSwiZW1wbG95ZWVCb251cyI6MC4yOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNCwib2ZmaWNlckJvbnVzIjowLjA0LCJjb2dzRGVwcmVjaWF0aW9uIjowLjQ3LCJzZ2FEZXByZWNpYXRpb24iOjEuNDMsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMzh9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNTQsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3LjE2LCJlbXBsb3llZUJvbnVzIjowLjM4LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjUyLCJvZmZpY2VyQm9udXMiOjAuMDYsImNvZ3NEZXByZWNpYXRpb24iOjAuMjksInNnYURlcHJlY2lhdGlvbiI6MS4xNSwicmVzZWFyY2hEZXZlbG9wbWVudCI6MC4yOX19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6NiwiZW1wbG95ZWVTYWxhcnkiOjUuNywiZW1wbG95ZWVCb251cyI6MC4zLCJvZmZpY2VyUGF5IjowLjQsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzYsIm9mZmljZXJCb251cyI6MC4wNCwiZGVwcmVjaWF0aW9uIjoyLCJjb2dzRGVwcmVjaWF0aW9uIjowLjUsInNnYURlcHJlY2lhdGlvbiI6MS41LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjQsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsImVtcGxveWVlU2FsYXJ5Ijo3LjYsImVtcGxveWVlQm9udXMiOjAuNCwib2ZmaWNlclBheSI6MC42LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjU0LCJvZmZpY2VyQm9udXMiOjAuMDYsImRlcHJlY2lhdGlvbiI6MS41LCJjb2dzRGVwcmVjaWF0aW9uIjowLjMsInNnYURlcHJlY2lhdGlvbiI6MS4yLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjMsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA3MDcyMzY4NDIxMDUxLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjoxLjE3NDE4NjQ5MTA2NDQ2NmUtMTYsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDE5ODE2Mjg3MTc4ODc3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDQ0ODUzNjMwNjc1MzI3NCwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwNjA5MzM3MDI3ODk4MDQsIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNjA3MzE2NTgzOTIyNDksIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4MDkwNTk1MDQ2MDU2NjMsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MTQ5Mzc3NzI0OTMwNjQ0Niwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjI5NjEzNzE0MzkwMDY1NzQzLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjQ5NTI1ODE3MTAzMzM2NiwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTU1NTA0MjcyNTc5NzcyODQsIm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwicHJvamVjdFBheUdyb3d0aCI6MC4wODg5NDM4NDEyMjQ2MzUxMSwib3RoZXJQYXlHcm93dGgiOjAuMDI0ODQyMTUyOTA2OTQxMzA2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjAyNjI0MDc1MjQ4NTg5MDg5Mywib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODcyMzc2OTIxMzYzMzgsInByb2plY3RTZ2FSYXRlRW5kIjowLjEwMzE1Mjk5NTQzNzQxMzIxLCJvdGhlclNnYVJhdGVFbmQiOjAuMTA5MjI2MTY0NjUxNjM2NTksInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzcxOTIzMTY3OTU4MzQ5LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6MjMsInN1YnNpZHkiOjcuNjcsImxvY2FsQmVuY2htYXJrIjoyM30sImRyaXZlclJhbmdlcyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjpbLTAuMDUsMC4zXSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDEuNjY1MzM0NTM2OTM3NzM0OGUtMTZdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkzMjUzMzA1MDE4NDY5MjcsMC4wMjA3MzU5OTQxODMxODkxNjZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlswLjA0MDc2MDg2OTU2NTIxNzE4NCwwLjA0NDM4NDA1Nzk3MTAxNDUyXSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDAwMTM0NTc1NTY5MzU4MTk3MzddLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MTM5NDU3MDIzNzE3NDQzLDAuMDIwNTUzNDU5OTE0NzYzMDk1XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjAzOTE2NjY2NjY2NjY2NjY4LDAuMDQyNTAwMDAwMDAwMDAwMDldLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbMC4xNSwwLjNdLCJvdGhlclNhbGVzR3Jvd3RoIjpbMC4wNjA3NjA4Njk1NjUyMTcxOSwwLjA2NDM4NDA1Nzk3MTAxNDUzXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMC4wMDUsMC4wMDUxMzQ1NzU1NjkzNTgxOTc1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLjAyNDEzOTQ1NzAyMzcxNzQ0NCwwLjAyNTU1MzQ1OTkxNDc2MzA5Nl0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6WzAuMDQ0MTY2NjY2NjY2NjY2NjgsMC4wNDc1MDAwMDAwMDAwMDAwOV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMC4wODQ5OTk5OTk5OTk5OTk5OSwwLjEzNV0sIm90aGVyU2dhUmF0ZUVuZCI6WzAuMDg5Mjg1NzE0Mjg1NzE0MjcsMC4xMTkyODU3MTQyODU3MTQyN10sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjpbMC4wNDI2MzE1Nzg5NDczNjgzNiwwLjA2NTU1NTU1NTU1NTU1NTU4XSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjAsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6MTMzLjUsIm1heCI6MjUyLjY5LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjoyLCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NjUsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo3Ni40NCwibWF4IjoxMzYuODQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsYWJvclByb2R1Y3Rpdml0eUNhZ3IiOnsidmFsdWUiOjIxLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZEluY3JlYXNlIjp7InZhbHVlIjoxOC43OCwibWF4IjozMy40MywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5Q2FnciI6eyJ2YWx1ZSI6NywibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5SW5jcmVhc2UiOnsidmFsdWUiOjIuODUsIm1heCI6My43NCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjoxNSwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX19LCJmb3JlY2FzdE92ZXJyaWRlcyI6eyIyMDI5Om90aGVyOnNhbGVzIjo4NS4xMywiMjAyOTpwcm9qZWN0OjctOCI6Ny44OX0sImZ1dHVyZUlucHV0QmFzaXMiOiJvdGhlciIsImlucHV0VmFsdWVzIjp7ImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xIjoxMzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTMiOjkyLjc1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6MC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMyLjY1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6MC44MiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEwIjowLjA5LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTIiOjExLjY3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjAuNjIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNCI6Mi40NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1IjowLjY0LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMSI6NzIsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny00IjoyMy4wNCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjYuNzgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny04Ijo1LjE5LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOSI6MC4zNiwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEwIjoxLjgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMyI6OTAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEiOjE0My4yLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMyI6OTcuMzgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi00IjowLjc2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNyI6MzQuNTIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi05IjowLjg2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEyIjoxMi40NywiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEzIjowLjY2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTQiOjIuNTgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNSI6MC42NywiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEiOjc2LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNCI6MjQuMzIsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny02Ijo3LjA0LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctOCI6NS41OSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTkiOjAuMzgsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xMCI6MS45LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTMiOjk1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xIjoxNTAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0zIjoxMDIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi00IjowLjgsImFjdHVhbDpjb21wYW55OjIwMjU6Mi03IjozNi40LCJhY3R1YWw6Y29tcGFueToyMDI1OjItOSI6MC45LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEyIjoxMy4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTMiOjAuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE0IjoyLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNSI6MC43LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMSI6ODAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNS42LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6Ny4zLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTkiOjAuNCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEwIjoyLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTMiOjEwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTE0IjoyLCJiYWxhbmNlLXNoZWV0OjIwMjM6YXNzZXRzIjoxMzIsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NywiYmFsYW5jZS1zaGVldDoyMDIzOmNhc2giOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRBc3NldHMiOjY1LCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzLCJiYWxhbmNlLXNoZWV0OjIwMjM6YnVpbGRpbmdzIjoxOSwiYmFsYW5jZS1zaGVldDoyMDIzOm1hY2hpbmVyeSI6MjQsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmludGFuZ2libGVBc3NldHMiOjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzb2Z0d2FyZSI6NSwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NSwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRMaWFiaWxpdGllcyI6MzksImJhbGFuY2Utc2hlZXQ6MjAyMzpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2LCJiYWxhbmNlLXNoZWV0OjIwMjM6bG9uZ1Rlcm1EZWJ0IjoyOSwiYmFsYW5jZS1zaGVldDoyMDIzOm5ldEFzc2V0cyI6NTcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGV4Ijo1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50QXNzZXRzIjo3MiwiYmFsYW5jZS1zaGVldDoyMDI0OmNhc2giOjI1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6dGFuZ2libGVBc3NldHMiOjU4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YnVpbGRpbmdzIjoyMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmludGFuZ2libGVBc3NldHMiOjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NiwiYmFsYW5jZS1zaGVldDoyMDI0OmxpYWJpbGl0aWVzIjo3OSwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRMaWFiaWxpdGllcyI6NDEsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkTGlhYmlsaXRpZXMiOjM4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bG9uZ1Rlcm1EZWJ0IjozMSwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaGFyZWhvbGRlckVxdWl0eSI6NjEsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4LCJiYWxhbmNlLXNoZWV0OjIwMjU6YXNzZXRzIjoxNTYsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50QXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3LCJiYWxhbmNlLXNoZWV0OjIwMjU6Zml4ZWRBc3NldHMiOjc4LCJiYWxhbmNlLXNoZWV0OjIwMjU6dGFuZ2libGVBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMiwiYmFsYW5jZS1zaGVldDoyMDI1Om1hY2hpbmVyeSI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjksImJhbGFuY2Utc2hlZXQ6MjAyNTpzb2Z0d2FyZSI6NywiYmFsYW5jZS1zaGVldDoyMDI1OmxpYWJpbGl0aWVzIjo4MywiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaG9ydFRlcm1EZWJ0IjoxMSwiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkTGlhYmlsaXRpZXMiOjQwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMiwiYmFsYW5jZS1zaGVldDoyMDI1Om5ldEFzc2V0cyI6NzMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaGFyZWhvbGRlckVxdWl0eSI6NzAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGV4IjoxMCwiZnV0dXJlLWNhcGV4OjIwMjYiOjE1LCJmdXR1cmUtY2FwZXg6MjAyNyI6MTUsImZ1dHVyZS1jYXBleDoyMDI4IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjkiOjAsImZ1dHVyZS1jYXBleDoyMDMwIjowLCJmdXR1cmUtY2FwZXg6MjAzMSI6MCwiZHJpdmVyOnByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDoxIjowLjMsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDcwNzIzNjg0MjEwNTEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjEuMTc0MTg2NDkxMDY0NDY2ZS0xNiwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDE5ODE2Mjg3MTc4ODc3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZTowIjowLjAxOTMyNTMzMDUwMTg0NjkyNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA3MzU5OTQxODMxODkxNjYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDQ0ODUzNjMwNjc1MzI3NCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDYwOTMzNzAyNzg5ODA0LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZToxIjowLjA1NzAxNzU0Mzg1OTY0OTE5LCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI2MDczMTY1ODM5MjI0OSwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODA5MDU5NTA0NjA1NjYzLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkxMzk0NTcwMjM3MTc0NDMsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZToxIjowLjAyMDU1MzQ1OTkxNDc2MzA5NSwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MTQ5Mzc3NzI0OTMwNjQ0NiwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjAiOjAuMDM5MTY2NjY2NjY2NjY2NjgsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZToxIjowLjA0MjUwMDAwMDAwMDAwMDA5LCJkcml2ZXI6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MCwiZHJpdmVyOnByb2plY3RTYWxlc0dyb3d0aCI6MC4yOTYxMzcxNDM5MDA2NTc0MywiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDowIjowLjE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjEiOjAuMywiZHJpdmVyOm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNDk1MjU4MTcxMDMzMzY2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTU1NTA0MjcyNTc5NzcyODQsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDg4OTQzODQxMjI0NjM1MTEsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0MjE1MjkwNjk0MTMwNiwiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjAiOjAuMDI0MTM5NDU3MDIzNzE3NDQ0LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wMjU1NTM0NTk5MTQ3NjMwOTYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjAyNjI0MDc1MjQ4NTg5MDg5MywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTg3MjM3NjkyMTM2MzM4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MCI6MC4wNDQxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjEiOjAuMDQ3NTAwMDAwMDAwMDAwMDksImRyaXZlcjpwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMDMxNTI5OTU0Mzc0MTMyMSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjAiOjAuMDg0OTk5OTk5OTk5OTk5OTksImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDoxIjowLjEzNSwiZHJpdmVyOm90aGVyU2dhUmF0ZUVuZCI6MC4xMDkyMjYxNjQ2NTE2MzY1OSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLjA4OTI4NTcxNDI4NTcxNDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMTE5Mjg1NzE0Mjg1NzE0MjcsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM3MTkyMzE2Nzk1ODM0OSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAuMDQyNjMxNTc4OTQ3MzY4MzYsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjA2NTU1NTU1NTU1NTU1NTU4LCJkcml2ZXI6dXNlZnVsTGlmZSI6MTAsImRyaXZlci1yYW5nZTp1c2VmdWxMaWZlOjAiOjUsImRyaXZlci1yYW5nZTp1c2VmdWxMaWZlOjEiOjIwLCJkcml2ZXI6aW52ZXN0bWVudCI6MjMsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjAiOjE1LCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDoxIjoyMDAsImRyaXZlcjpzdWJzaWR5Ijo3LjY3LCJkcml2ZXItcmFuZ2U6c3Vic2lkeTowIjoxLCJkcml2ZXItcmFuZ2U6c3Vic2lkeToxIjo1MCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoyMCwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjoxMzMuNSwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTp2YWx1ZSI6MiwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTptYXgiOjcsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTp2YWx1ZSI6NjUsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTptYXgiOjk1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2Fncjp2YWx1ZSI6MjIsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTp2YWx1ZSI6NzYuNDQsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6dmFsdWUiOjIxLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOm1heCI6MzUsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6dmFsdWUiOjE4Ljc4LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOnZhbHVlIjo3LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOm1heCI6MTAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOnZhbHVlIjoyLjg1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86dmFsdWUiOjE1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86bWF4Ijo3MCwidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86dmFsdWUiOjIxMywidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86bWF4IjozNTAsInRhcmdldDpsb2NhbEJlbmNobWFyazp2YWx1ZSI6MjMsInRhcmdldDpsb2NhbEJlbmNobWFyazptYXgiOjQwLCJ0YXJnZXQ6b2ZmaWNlclBheUNhZ3I6dmFsdWUiOjYsInRhcmdldDpvZmZpY2VyUGF5Q2FncjptYXgiOjEwLCJ0YXJnZXQ6b2ZmaWNlclBheUluY3JlYXNlOnZhbHVlIjowLCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6bWF4IjoyNTIuNjksInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTptYXgiOjEzNi44NCwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTptYXgiOjMzLjQzLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlJbmNyZWFzZTptYXgiOjMuNzR9LCJtZXRyaWNHcm91cEJhc2VzIjp7ImNvbXBhbnlTYWxlcyI6InJhdGUiLCJwcm9qZWN0U2FsZXMiOiJyYXRlIiwibGFib3JQcm9kdWN0aXZpdHkiOiJyYXRlIiwiZW1wbG95ZWVQYXkiOiJyYXRlIn0sImFwcGxpY2F0aW9uQ2F0ZWdvcnkiOiJnZW5lcmFsIn0=</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4fX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjU5LCJvZmZpY2VyUGF5IjowLjM4LCJkZXByZWNpYXRpb24iOjEuOSwib3RoZXJTZ2EiOjkuNSwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NS4zMSwiZW1wbG95ZWVCb251cyI6MC4yOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNCwib2ZmaWNlckJvbnVzIjowLjA0LCJjb2dzRGVwcmVjaWF0aW9uIjowLjQ3LCJzZ2FEZXByZWNpYXRpb24iOjEuNDMsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMzh9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNTQsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3LjE2LCJlbXBsb3llZUJvbnVzIjowLjM4LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjUyLCJvZmZpY2VyQm9udXMiOjAuMDYsImNvZ3NEZXByZWNpYXRpb24iOjAuMjksInNnYURlcHJlY2lhdGlvbiI6MS4xNSwicmVzZWFyY2hEZXZlbG9wbWVudCI6MC4yOX19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6NiwiZW1wbG95ZWVTYWxhcnkiOjUuNywiZW1wbG95ZWVCb251cyI6MC4zLCJvZmZpY2VyUGF5IjowLjQsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzYsIm9mZmljZXJCb251cyI6MC4wNCwiZGVwcmVjaWF0aW9uIjoyLCJjb2dzRGVwcmVjaWF0aW9uIjowLjUsInNnYURlcHJlY2lhdGlvbiI6MS41LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjQsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsImVtcGxveWVlU2FsYXJ5Ijo3LjYsImVtcGxveWVlQm9udXMiOjAuNCwib2ZmaWNlclBheSI6MC42LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjU0LCJvZmZpY2VyQm9udXMiOjAuMDYsImRlcHJlY2lhdGlvbiI6MS41LCJjb2dzRGVwcmVjaWF0aW9uIjowLjMsInNnYURlcHJlY2lhdGlvbiI6MS4yLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjMsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA3MDcyMzY4NDIxMDUxLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjoxLjE3NDE4NjQ5MTA2NDQ2NmUtMTYsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDE5ODE2Mjg3MTc4ODc3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDQ0ODUzNjMwNjc1MzI3NCwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwNjA5MzM3MDI3ODk4MDQsIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNjA3MzE2NTgzOTIyNDksIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4MDkwNTk1MDQ2MDU2NjMsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MTQ5Mzc3NzI0OTMwNjQ0Niwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjI5NjEzNzE0MzkwMDY1NzQzLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjQ5NTI1ODE3MTAzMzM2NiwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTU1NTA0MjcyNTc5NzcyODQsIm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwicHJvamVjdFBheUdyb3d0aCI6MC4wODg5NDM4NDEyMjQ2MzUxMSwib3RoZXJQYXlHcm93dGgiOjAuMDI0ODQyMTUyOTA2OTQxMzA2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjAyNjI0MDc1MjQ4NTg5MDg5Mywib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODcyMzc2OTIxMzYzMzgsInByb2plY3RTZ2FSYXRlRW5kIjowLjEwMzE1Mjk5NTQzNzQxMzIxLCJvdGhlclNnYVJhdGVFbmQiOjAuMTA5MjI2MTY0NjUxNjM2NTksInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzcxOTIzMTY3OTU4MzQ5LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6MjMsInN1YnNpZHkiOjcuNjYsImxvY2FsQmVuY2htYXJrIjoyM30sImRyaXZlclJhbmdlcyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjpbLTAuMDUsMC4zXSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDEuNjY1MzM0NTM2OTM3NzM0OGUtMTZdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkzMjUzMzA1MDE4NDY5MjcsMC4wMjA3MzU5OTQxODMxODkxNjZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlswLjA0MDc2MDg2OTU2NTIxNzE4NCwwLjA0NDM4NDA1Nzk3MTAxNDUyXSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDAwMTM0NTc1NTY5MzU4MTk3MzddLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MTM5NDU3MDIzNzE3NDQzLDAuMDIwNTUzNDU5OTE0NzYzMDk1XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjAzOTE2NjY2NjY2NjY2NjY4LDAuMDQyNTAwMDAwMDAwMDAwMDldLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbMC4xNSwwLjNdLCJvdGhlclNhbGVzR3Jvd3RoIjpbMC4wNjA3NjA4Njk1NjUyMTcxOSwwLjA2NDM4NDA1Nzk3MTAxNDUzXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMC4wMDUsMC4wMDUxMzQ1NzU1NjkzNTgxOTc1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLjAyNDEzOTQ1NzAyMzcxNzQ0NCwwLjAyNTU1MzQ1OTkxNDc2MzA5Nl0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6WzAuMDQ0MTY2NjY2NjY2NjY2NjgsMC4wNDc1MDAwMDAwMDAwMDAwOV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMC4wODQ5OTk5OTk5OTk5OTk5OSwwLjEzNV0sIm90aGVyU2dhUmF0ZUVuZCI6WzAuMDg5Mjg1NzE0Mjg1NzE0MjcsMC4xMTkyODU3MTQyODU3MTQyN10sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjpbMC4wNDI2MzE1Nzg5NDczNjgzNiwwLjA2NTU1NTU1NTU1NTU1NTU4XSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjAsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6MTMzLjUsIm1heCI6MjUyLjY5LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjoyLCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NjUsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo3Ni40NCwibWF4IjoxMzYuODQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsYWJvclByb2R1Y3Rpdml0eUNhZ3IiOnsidmFsdWUiOjIxLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZEluY3JlYXNlIjp7InZhbHVlIjoxOC43OCwibWF4IjozMy40MywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5Q2FnciI6eyJ2YWx1ZSI6NywibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5SW5jcmVhc2UiOnsidmFsdWUiOjIuODUsIm1heCI6My43NCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjoxNSwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX19LCJmb3JlY2FzdE92ZXJyaWRlcyI6eyIyMDI5Om90aGVyOnNhbGVzIjo4NS4xMywiMjAyOTpwcm9qZWN0OjctOCI6Ny44OX0sImZ1dHVyZUlucHV0QmFzaXMiOiJvdGhlciIsImlucHV0VmFsdWVzIjp7ImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xIjoxMzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTMiOjkyLjc1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6MC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMyLjY1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6MC44MiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEwIjowLjA5LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTIiOjExLjY3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjAuNjIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNCI6Mi40NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1IjowLjY0LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMSI6NzIsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny00IjoyMy4wNCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjYuNzgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny04Ijo1LjE5LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOSI6MC4zNiwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEwIjoxLjgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMyI6OTAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEiOjE0My4yLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMyI6OTcuMzgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi00IjowLjc2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNyI6MzQuNTIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi05IjowLjg2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEyIjoxMi40NywiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEzIjowLjY2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTQiOjIuNTgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNSI6MC42NywiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEiOjc2LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNCI6MjQuMzIsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny02Ijo3LjA0LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctOCI6NS41OSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTkiOjAuMzgsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xMCI6MS45LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTMiOjk1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xIjoxNTAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0zIjoxMDIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi00IjowLjgsImFjdHVhbDpjb21wYW55OjIwMjU6Mi03IjozNi40LCJhY3R1YWw6Y29tcGFueToyMDI1OjItOSI6MC45LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEyIjoxMy4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTMiOjAuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE0IjoyLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNSI6MC43LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMSI6ODAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNS42LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6Ny4zLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTkiOjAuNCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEwIjoyLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTMiOjEwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTE0IjoyLCJiYWxhbmNlLXNoZWV0OjIwMjM6YXNzZXRzIjoxMzIsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NywiYmFsYW5jZS1zaGVldDoyMDIzOmNhc2giOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRBc3NldHMiOjY1LCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzLCJiYWxhbmNlLXNoZWV0OjIwMjM6YnVpbGRpbmdzIjoxOSwiYmFsYW5jZS1zaGVldDoyMDIzOm1hY2hpbmVyeSI6MjQsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmludGFuZ2libGVBc3NldHMiOjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzb2Z0d2FyZSI6NSwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NSwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRMaWFiaWxpdGllcyI6MzksImJhbGFuY2Utc2hlZXQ6MjAyMzpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2LCJiYWxhbmNlLXNoZWV0OjIwMjM6bG9uZ1Rlcm1EZWJ0IjoyOSwiYmFsYW5jZS1zaGVldDoyMDIzOm5ldEFzc2V0cyI6NTcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGV4Ijo1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50QXNzZXRzIjo3MiwiYmFsYW5jZS1zaGVldDoyMDI0OmNhc2giOjI1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6dGFuZ2libGVBc3NldHMiOjU4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YnVpbGRpbmdzIjoyMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmludGFuZ2libGVBc3NldHMiOjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NiwiYmFsYW5jZS1zaGVldDoyMDI0OmxpYWJpbGl0aWVzIjo3OSwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRMaWFiaWxpdGllcyI6NDEsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkTGlhYmlsaXRpZXMiOjM4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bG9uZ1Rlcm1EZWJ0IjozMSwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaGFyZWhvbGRlckVxdWl0eSI6NjEsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4LCJiYWxhbmNlLXNoZWV0OjIwMjU6YXNzZXRzIjoxNTYsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50QXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3LCJiYWxhbmNlLXNoZWV0OjIwMjU6Zml4ZWRBc3NldHMiOjc4LCJiYWxhbmNlLXNoZWV0OjIwMjU6dGFuZ2libGVBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMiwiYmFsYW5jZS1zaGVldDoyMDI1Om1hY2hpbmVyeSI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjksImJhbGFuY2Utc2hlZXQ6MjAyNTpzb2Z0d2FyZSI6NywiYmFsYW5jZS1zaGVldDoyMDI1OmxpYWJpbGl0aWVzIjo4MywiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaG9ydFRlcm1EZWJ0IjoxMSwiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkTGlhYmlsaXRpZXMiOjQwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMiwiYmFsYW5jZS1zaGVldDoyMDI1Om5ldEFzc2V0cyI6NzMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaGFyZWhvbGRlckVxdWl0eSI6NzAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGV4IjoxMCwiZnV0dXJlLWNhcGV4OjIwMjYiOjE1LCJmdXR1cmUtY2FwZXg6MjAyNyI6MTUsImZ1dHVyZS1jYXBleDoyMDI4IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjkiOjAsImZ1dHVyZS1jYXBleDoyMDMwIjowLCJmdXR1cmUtY2FwZXg6MjAzMSI6MCwiZHJpdmVyOnByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDoxIjowLjMsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDcwNzIzNjg0MjEwNTEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjEuMTc0MTg2NDkxMDY0NDY2ZS0xNiwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDE5ODE2Mjg3MTc4ODc3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZTowIjowLjAxOTMyNTMzMDUwMTg0NjkyNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA3MzU5OTQxODMxODkxNjYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDQ0ODUzNjMwNjc1MzI3NCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDYwOTMzNzAyNzg5ODA0LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZToxIjowLjA1NzAxNzU0Mzg1OTY0OTE5LCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI2MDczMTY1ODM5MjI0OSwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODA5MDU5NTA0NjA1NjYzLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkxMzk0NTcwMjM3MTc0NDMsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZToxIjowLjAyMDU1MzQ1OTkxNDc2MzA5NSwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MTQ5Mzc3NzI0OTMwNjQ0NiwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjAiOjAuMDM5MTY2NjY2NjY2NjY2NjgsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZToxIjowLjA0MjUwMDAwMDAwMDAwMDA5LCJkcml2ZXI6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MCwiZHJpdmVyOnByb2plY3RTYWxlc0dyb3d0aCI6MC4yOTYxMzcxNDM5MDA2NTc0MywiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDowIjowLjE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjEiOjAuMywiZHJpdmVyOm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNDk1MjU4MTcxMDMzMzY2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTU1NTA0MjcyNTc5NzcyODQsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDg4OTQzODQxMjI0NjM1MTEsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0MjE1MjkwNjk0MTMwNiwiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjAiOjAuMDI0MTM5NDU3MDIzNzE3NDQ0LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wMjU1NTM0NTk5MTQ3NjMwOTYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjAyNjI0MDc1MjQ4NTg5MDg5MywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTg3MjM3NjkyMTM2MzM4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MCI6MC4wNDQxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjEiOjAuMDQ3NTAwMDAwMDAwMDAwMDksImRyaXZlcjpwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMDMxNTI5OTU0Mzc0MTMyMSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjAiOjAuMDg0OTk5OTk5OTk5OTk5OTksImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDoxIjowLjEzNSwiZHJpdmVyOm90aGVyU2dhUmF0ZUVuZCI6MC4xMDkyMjYxNjQ2NTE2MzY1OSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLjA4OTI4NTcxNDI4NTcxNDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMTE5Mjg1NzE0Mjg1NzE0MjcsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM3MTkyMzE2Nzk1ODM0OSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAuMDQyNjMxNTc4OTQ3MzY4MzYsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjA2NTU1NTU1NTU1NTU1NTU4LCJkcml2ZXI6dXNlZnVsTGlmZSI6MTAsImRyaXZlci1yYW5nZTp1c2VmdWxMaWZlOjAiOjUsImRyaXZlci1yYW5nZTp1c2VmdWxMaWZlOjEiOjIwLCJkcml2ZXI6aW52ZXN0bWVudCI6MjMsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjAiOjE1LCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDoxIjoyMDAsImRyaXZlcjpzdWJzaWR5Ijo3LjY2LCJkcml2ZXItcmFuZ2U6c3Vic2lkeTowIjoxLCJkcml2ZXItcmFuZ2U6c3Vic2lkeToxIjo1MCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoyMCwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjoxMzMuNSwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTp2YWx1ZSI6MiwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTptYXgiOjcsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTp2YWx1ZSI6NjUsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTptYXgiOjk1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2Fncjp2YWx1ZSI6MjIsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTp2YWx1ZSI6NzYuNDQsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6dmFsdWUiOjIxLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOm1heCI6MzUsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6dmFsdWUiOjE4Ljc4LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOnZhbHVlIjo3LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOm1heCI6MTAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOnZhbHVlIjoyLjg1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86dmFsdWUiOjE1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86bWF4Ijo3MCwidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86dmFsdWUiOjIxMywidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86bWF4IjozNTAsInRhcmdldDpsb2NhbEJlbmNobWFyazp2YWx1ZSI6MjMsInRhcmdldDpsb2NhbEJlbmNobWFyazptYXgiOjQwLCJ0YXJnZXQ6b2ZmaWNlclBheUNhZ3I6dmFsdWUiOjYsInRhcmdldDpvZmZpY2VyUGF5Q2FncjptYXgiOjEwLCJ0YXJnZXQ6b2ZmaWNlclBheUluY3JlYXNlOnZhbHVlIjowLCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6bWF4IjoyNTIuNjksInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTptYXgiOjEzNi44NCwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTptYXgiOjMzLjQzLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlJbmNyZWFzZTptYXgiOjMuNzR9LCJtZXRyaWNHcm91cEJhc2VzIjp7ImNvbXBhbnlTYWxlcyI6InJhdGUiLCJwcm9qZWN0U2FsZXMiOiJyYXRlIiwibGFib3JQcm9kdWN0aXZpdHkiOiJyYXRlIiwiZW1wbG95ZWVQYXkiOiJyYXRlIn0sImFwcGxpY2F0aW9uQ2F0ZWdvcnkiOiJnZW5lcmFsIn0=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Separate standard sample inputs from optimized results
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -5850,7 +5850,7 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <v>5.407072368421051</v>
+        <v>5.409356725146197</v>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <v>1.174186491064466e-14</v>
+        <v>5.551115123125783e-15</v>
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
@@ -5892,7 +5892,7 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <v>2.0019816287178878</v>
+        <v>2.0030662342518046</v>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
@@ -5913,7 +5913,7 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <v>5.444853630675327</v>
+        <v>5.409356725146197</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
@@ -5955,7 +5955,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <v>5.40609337027898</v>
+        <v>5.409356725146197</v>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
@@ -5976,7 +5976,7 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <v>4.260731658392249</v>
+        <v>4.257246376811585</v>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
@@ -6018,7 +6018,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>1.9809059504605664</v>
+        <v>1.984645846924027</v>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
@@ -6039,7 +6039,7 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <v>4.149377724930645</v>
+        <v>4.083333333333339</v>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
@@ -6081,7 +6081,7 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <v>29.61371439006574</v>
+        <v>22</v>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
@@ -6102,7 +6102,7 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <v>6.249525817103336</v>
+        <v>6.257246376811586</v>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
         </is>
       </c>
       <c r="B17" s="2">
-        <v>1.5550427257977284</v>
+        <v>1.5</v>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
@@ -6165,7 +6165,7 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <v>8.894384122463512</v>
+        <v>7.000000000000001</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
@@ -6186,7 +6186,7 @@
         </is>
       </c>
       <c r="B20" s="2">
-        <v>2.484215290694131</v>
+        <v>2.484645846924027</v>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
@@ -6207,7 +6207,7 @@
         </is>
       </c>
       <c r="B21" s="2">
-        <v>2.6240752485890892</v>
+        <v>4</v>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
@@ -6228,7 +6228,7 @@
         </is>
       </c>
       <c r="B22" s="2">
-        <v>4.5872376921363385</v>
+        <v>4.583333333333338</v>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
@@ -6249,7 +6249,7 @@
         </is>
       </c>
       <c r="B23" s="2">
-        <v>10.315299543741322</v>
+        <v>11</v>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
@@ -6270,7 +6270,7 @@
         </is>
       </c>
       <c r="B24" s="2">
-        <v>10.92261646516366</v>
+        <v>10.928571428571427</v>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
@@ -6291,7 +6291,7 @@
         </is>
       </c>
       <c r="B25" s="2">
-        <v>5.371923167958349</v>
+        <v>5.380116959064325</v>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
@@ -8970,7 +8970,7 @@
         </is>
       </c>
       <c r="B172" s="2">
-        <v>0.04587237692136338</v>
+        <v>0.045833333333333386</v>
       </c>
       <c r="C172" s="0" t="inlineStr">
         <is>
@@ -8985,7 +8985,7 @@
         </is>
       </c>
       <c r="B173" s="2">
-        <v>0.041493777249306446</v>
+        <v>0.04083333333333339</v>
       </c>
       <c r="C173" s="0" t="inlineStr">
         <is>
@@ -9000,7 +9000,7 @@
         </is>
       </c>
       <c r="B174" s="2">
-        <v>0.024842152906941306</v>
+        <v>0.02484645846924027</v>
       </c>
       <c r="C174" s="0" t="inlineStr">
         <is>
@@ -9015,7 +9015,7 @@
         </is>
       </c>
       <c r="B175" s="2">
-        <v>0.019809059504605663</v>
+        <v>0.01984645846924027</v>
       </c>
       <c r="C175" s="0" t="inlineStr">
         <is>
@@ -9030,7 +9030,7 @@
         </is>
       </c>
       <c r="B176" s="2">
-        <v>0.062495258171033366</v>
+        <v>0.06257246376811586</v>
       </c>
       <c r="C176" s="0" t="inlineStr">
         <is>
@@ -9045,7 +9045,7 @@
         </is>
       </c>
       <c r="B177" s="2">
-        <v>0.04260731658392249</v>
+        <v>0.042572463768115854</v>
       </c>
       <c r="C177" s="0" t="inlineStr">
         <is>
@@ -9075,7 +9075,7 @@
         </is>
       </c>
       <c r="B179" s="2">
-        <v>0.10922616465163659</v>
+        <v>0.10928571428571428</v>
       </c>
       <c r="C179" s="0" t="inlineStr">
         <is>
@@ -9090,7 +9090,7 @@
         </is>
       </c>
       <c r="B180" s="2">
-        <v>0.015550427257977284</v>
+        <v>0.015</v>
       </c>
       <c r="C180" s="0" t="inlineStr">
         <is>
@@ -9105,7 +9105,7 @@
         </is>
       </c>
       <c r="B181" s="2">
-        <v>1.174186491064466e-16</v>
+        <v>5.551115123125783e-17</v>
       </c>
       <c r="C181" s="0" t="inlineStr">
         <is>
@@ -9120,7 +9120,7 @@
         </is>
       </c>
       <c r="B182" s="2">
-        <v>0.026240752485890893</v>
+        <v>0.04</v>
       </c>
       <c r="C182" s="0" t="inlineStr">
         <is>
@@ -9135,7 +9135,7 @@
         </is>
       </c>
       <c r="B183" s="2">
-        <v>0.054448536306753274</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="C183" s="0" t="inlineStr">
         <is>
@@ -9165,7 +9165,7 @@
         </is>
       </c>
       <c r="B185" s="2">
-        <v>0.05371923167958349</v>
+        <v>0.05380116959064325</v>
       </c>
       <c r="C185" s="0" t="inlineStr">
         <is>
@@ -9180,7 +9180,7 @@
         </is>
       </c>
       <c r="B186" s="2">
-        <v>0.054060933702789804</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="C186" s="0" t="inlineStr">
         <is>
@@ -9195,7 +9195,7 @@
         </is>
       </c>
       <c r="B187" s="2">
-        <v>0.08894384122463511</v>
+        <v>0.07</v>
       </c>
       <c r="C187" s="0" t="inlineStr">
         <is>
@@ -9210,7 +9210,7 @@
         </is>
       </c>
       <c r="B188" s="2">
-        <v>0.020019816287178877</v>
+        <v>0.020030662342518046</v>
       </c>
       <c r="C188" s="0" t="inlineStr">
         <is>
@@ -9225,7 +9225,7 @@
         </is>
       </c>
       <c r="B189" s="2">
-        <v>0.29613714390065743</v>
+        <v>0.22</v>
       </c>
       <c r="C189" s="0" t="inlineStr">
         <is>
@@ -9240,7 +9240,7 @@
         </is>
       </c>
       <c r="B190" s="2">
-        <v>0.05407072368421051</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="C190" s="0" t="inlineStr">
         <is>
@@ -9270,7 +9270,7 @@
         </is>
       </c>
       <c r="B192" s="2">
-        <v>0.10315299543741321</v>
+        <v>0.11</v>
       </c>
       <c r="C192" s="0" t="inlineStr">
         <is>
@@ -9855,7 +9855,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4fX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjU5LCJvZmZpY2VyUGF5IjowLjM4LCJkZXByZWNpYXRpb24iOjEuOSwib3RoZXJTZ2EiOjkuNSwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NS4zMSwiZW1wbG95ZWVCb251cyI6MC4yOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNCwib2ZmaWNlckJvbnVzIjowLjA0LCJjb2dzRGVwcmVjaWF0aW9uIjowLjQ3LCJzZ2FEZXByZWNpYXRpb24iOjEuNDMsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMzh9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNTQsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3LjE2LCJlbXBsb3llZUJvbnVzIjowLjM4LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjUyLCJvZmZpY2VyQm9udXMiOjAuMDYsImNvZ3NEZXByZWNpYXRpb24iOjAuMjksInNnYURlcHJlY2lhdGlvbiI6MS4xNSwicmVzZWFyY2hEZXZlbG9wbWVudCI6MC4yOX19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6NiwiZW1wbG95ZWVTYWxhcnkiOjUuNywiZW1wbG95ZWVCb251cyI6MC4zLCJvZmZpY2VyUGF5IjowLjQsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzYsIm9mZmljZXJCb251cyI6MC4wNCwiZGVwcmVjaWF0aW9uIjoyLCJjb2dzRGVwcmVjaWF0aW9uIjowLjUsInNnYURlcHJlY2lhdGlvbiI6MS41LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjQsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsImVtcGxveWVlU2FsYXJ5Ijo3LjYsImVtcGxveWVlQm9udXMiOjAuNCwib2ZmaWNlclBheSI6MC42LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjU0LCJvZmZpY2VyQm9udXMiOjAuMDYsImRlcHJlY2lhdGlvbiI6MS41LCJjb2dzRGVwcmVjaWF0aW9uIjowLjMsInNnYURlcHJlY2lhdGlvbiI6MS4yLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjMsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA3MDcyMzY4NDIxMDUxLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjoxLjE3NDE4NjQ5MTA2NDQ2NmUtMTYsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDE5ODE2Mjg3MTc4ODc3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDQ0ODUzNjMwNjc1MzI3NCwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwNjA5MzM3MDI3ODk4MDQsIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNjA3MzE2NTgzOTIyNDksIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4MDkwNTk1MDQ2MDU2NjMsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MTQ5Mzc3NzI0OTMwNjQ0Niwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjI5NjEzNzE0MzkwMDY1NzQzLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjQ5NTI1ODE3MTAzMzM2NiwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTU1NTA0MjcyNTc5NzcyODQsIm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwicHJvamVjdFBheUdyb3d0aCI6MC4wODg5NDM4NDEyMjQ2MzUxMSwib3RoZXJQYXlHcm93dGgiOjAuMDI0ODQyMTUyOTA2OTQxMzA2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjAyNjI0MDc1MjQ4NTg5MDg5Mywib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODcyMzc2OTIxMzYzMzgsInByb2plY3RTZ2FSYXRlRW5kIjowLjEwMzE1Mjk5NTQzNzQxMzIxLCJvdGhlclNnYVJhdGVFbmQiOjAuMTA5MjI2MTY0NjUxNjM2NTksInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzcxOTIzMTY3OTU4MzQ5LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6MjMsInN1YnNpZHkiOjcuNjYsImxvY2FsQmVuY2htYXJrIjoyM30sImRyaXZlclJhbmdlcyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjpbLTAuMDUsMC4zXSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDEuNjY1MzM0NTM2OTM3NzM0OGUtMTZdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkzMjUzMzA1MDE4NDY5MjcsMC4wMjA3MzU5OTQxODMxODkxNjZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlswLjA0MDc2MDg2OTU2NTIxNzE4NCwwLjA0NDM4NDA1Nzk3MTAxNDUyXSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDAwMTM0NTc1NTY5MzU4MTk3MzddLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MTM5NDU3MDIzNzE3NDQzLDAuMDIwNTUzNDU5OTE0NzYzMDk1XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjAzOTE2NjY2NjY2NjY2NjY4LDAuMDQyNTAwMDAwMDAwMDAwMDldLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbMC4xNSwwLjNdLCJvdGhlclNhbGVzR3Jvd3RoIjpbMC4wNjA3NjA4Njk1NjUyMTcxOSwwLjA2NDM4NDA1Nzk3MTAxNDUzXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMC4wMDUsMC4wMDUxMzQ1NzU1NjkzNTgxOTc1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLjAyNDEzOTQ1NzAyMzcxNzQ0NCwwLjAyNTU1MzQ1OTkxNDc2MzA5Nl0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6WzAuMDQ0MTY2NjY2NjY2NjY2NjgsMC4wNDc1MDAwMDAwMDAwMDAwOV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMC4wODQ5OTk5OTk5OTk5OTk5OSwwLjEzNV0sIm90aGVyU2dhUmF0ZUVuZCI6WzAuMDg5Mjg1NzE0Mjg1NzE0MjcsMC4xMTkyODU3MTQyODU3MTQyN10sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjpbMC4wNDI2MzE1Nzg5NDczNjgzNiwwLjA2NTU1NTU1NTU1NTU1NTU4XSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjAsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6MTMzLjUsIm1heCI6MjUyLjY5LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjoyLCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NjUsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo3Ni40NCwibWF4IjoxMzYuODQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsYWJvclByb2R1Y3Rpdml0eUNhZ3IiOnsidmFsdWUiOjIxLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZEluY3JlYXNlIjp7InZhbHVlIjoxOC43OCwibWF4IjozMy40MywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5Q2FnciI6eyJ2YWx1ZSI6NywibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5SW5jcmVhc2UiOnsidmFsdWUiOjIuODUsIm1heCI6My43NCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjoxNSwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX19LCJmb3JlY2FzdE92ZXJyaWRlcyI6eyIyMDI5Om90aGVyOnNhbGVzIjo4NS4xMywiMjAyOTpwcm9qZWN0OjctOCI6Ny44OX0sImZ1dHVyZUlucHV0QmFzaXMiOiJvdGhlciIsImlucHV0VmFsdWVzIjp7ImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xIjoxMzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTMiOjkyLjc1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6MC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMyLjY1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6MC44MiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEwIjowLjA5LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTIiOjExLjY3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjAuNjIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNCI6Mi40NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1IjowLjY0LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMSI6NzIsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny00IjoyMy4wNCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjYuNzgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny04Ijo1LjE5LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOSI6MC4zNiwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEwIjoxLjgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMyI6OTAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEiOjE0My4yLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMyI6OTcuMzgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi00IjowLjc2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNyI6MzQuNTIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi05IjowLjg2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEyIjoxMi40NywiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEzIjowLjY2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTQiOjIuNTgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNSI6MC42NywiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEiOjc2LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNCI6MjQuMzIsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny02Ijo3LjA0LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctOCI6NS41OSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTkiOjAuMzgsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xMCI6MS45LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTMiOjk1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xIjoxNTAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0zIjoxMDIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi00IjowLjgsImFjdHVhbDpjb21wYW55OjIwMjU6Mi03IjozNi40LCJhY3R1YWw6Y29tcGFueToyMDI1OjItOSI6MC45LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEyIjoxMy4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTMiOjAuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE0IjoyLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNSI6MC43LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMSI6ODAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNS42LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6Ny4zLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTkiOjAuNCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEwIjoyLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTMiOjEwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTE0IjoyLCJiYWxhbmNlLXNoZWV0OjIwMjM6YXNzZXRzIjoxMzIsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NywiYmFsYW5jZS1zaGVldDoyMDIzOmNhc2giOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRBc3NldHMiOjY1LCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzLCJiYWxhbmNlLXNoZWV0OjIwMjM6YnVpbGRpbmdzIjoxOSwiYmFsYW5jZS1zaGVldDoyMDIzOm1hY2hpbmVyeSI6MjQsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmludGFuZ2libGVBc3NldHMiOjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzb2Z0d2FyZSI6NSwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NSwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRMaWFiaWxpdGllcyI6MzksImJhbGFuY2Utc2hlZXQ6MjAyMzpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2LCJiYWxhbmNlLXNoZWV0OjIwMjM6bG9uZ1Rlcm1EZWJ0IjoyOSwiYmFsYW5jZS1zaGVldDoyMDIzOm5ldEFzc2V0cyI6NTcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGV4Ijo1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50QXNzZXRzIjo3MiwiYmFsYW5jZS1zaGVldDoyMDI0OmNhc2giOjI1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6dGFuZ2libGVBc3NldHMiOjU4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YnVpbGRpbmdzIjoyMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmludGFuZ2libGVBc3NldHMiOjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NiwiYmFsYW5jZS1zaGVldDoyMDI0OmxpYWJpbGl0aWVzIjo3OSwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRMaWFiaWxpdGllcyI6NDEsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkTGlhYmlsaXRpZXMiOjM4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bG9uZ1Rlcm1EZWJ0IjozMSwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaGFyZWhvbGRlckVxdWl0eSI6NjEsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4LCJiYWxhbmNlLXNoZWV0OjIwMjU6YXNzZXRzIjoxNTYsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50QXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3LCJiYWxhbmNlLXNoZWV0OjIwMjU6Zml4ZWRBc3NldHMiOjc4LCJiYWxhbmNlLXNoZWV0OjIwMjU6dGFuZ2libGVBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMiwiYmFsYW5jZS1zaGVldDoyMDI1Om1hY2hpbmVyeSI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjksImJhbGFuY2Utc2hlZXQ6MjAyNTpzb2Z0d2FyZSI6NywiYmFsYW5jZS1zaGVldDoyMDI1OmxpYWJpbGl0aWVzIjo4MywiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaG9ydFRlcm1EZWJ0IjoxMSwiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkTGlhYmlsaXRpZXMiOjQwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMiwiYmFsYW5jZS1zaGVldDoyMDI1Om5ldEFzc2V0cyI6NzMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaGFyZWhvbGRlckVxdWl0eSI6NzAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGV4IjoxMCwiZnV0dXJlLWNhcGV4OjIwMjYiOjE1LCJmdXR1cmUtY2FwZXg6MjAyNyI6MTUsImZ1dHVyZS1jYXBleDoyMDI4IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjkiOjAsImZ1dHVyZS1jYXBleDoyMDMwIjowLCJmdXR1cmUtY2FwZXg6MjAzMSI6MCwiZHJpdmVyOnByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDoxIjowLjMsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDcwNzIzNjg0MjEwNTEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjEuMTc0MTg2NDkxMDY0NDY2ZS0xNiwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDE5ODE2Mjg3MTc4ODc3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZTowIjowLjAxOTMyNTMzMDUwMTg0NjkyNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA3MzU5OTQxODMxODkxNjYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDQ0ODUzNjMwNjc1MzI3NCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDYwOTMzNzAyNzg5ODA0LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZToxIjowLjA1NzAxNzU0Mzg1OTY0OTE5LCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI2MDczMTY1ODM5MjI0OSwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODA5MDU5NTA0NjA1NjYzLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkxMzk0NTcwMjM3MTc0NDMsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZToxIjowLjAyMDU1MzQ1OTkxNDc2MzA5NSwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MTQ5Mzc3NzI0OTMwNjQ0NiwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjAiOjAuMDM5MTY2NjY2NjY2NjY2NjgsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZToxIjowLjA0MjUwMDAwMDAwMDAwMDA5LCJkcml2ZXI6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MCwiZHJpdmVyOnByb2plY3RTYWxlc0dyb3d0aCI6MC4yOTYxMzcxNDM5MDA2NTc0MywiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDowIjowLjE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjEiOjAuMywiZHJpdmVyOm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNDk1MjU4MTcxMDMzMzY2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTU1NTA0MjcyNTc5NzcyODQsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDg4OTQzODQxMjI0NjM1MTEsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0MjE1MjkwNjk0MTMwNiwiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjAiOjAuMDI0MTM5NDU3MDIzNzE3NDQ0LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wMjU1NTM0NTk5MTQ3NjMwOTYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjAyNjI0MDc1MjQ4NTg5MDg5MywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTg3MjM3NjkyMTM2MzM4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MCI6MC4wNDQxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjEiOjAuMDQ3NTAwMDAwMDAwMDAwMDksImRyaXZlcjpwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMDMxNTI5OTU0Mzc0MTMyMSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjAiOjAuMDg0OTk5OTk5OTk5OTk5OTksImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDoxIjowLjEzNSwiZHJpdmVyOm90aGVyU2dhUmF0ZUVuZCI6MC4xMDkyMjYxNjQ2NTE2MzY1OSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLjA4OTI4NTcxNDI4NTcxNDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMTE5Mjg1NzE0Mjg1NzE0MjcsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM3MTkyMzE2Nzk1ODM0OSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAuMDQyNjMxNTc4OTQ3MzY4MzYsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjA2NTU1NTU1NTU1NTU1NTU4LCJkcml2ZXI6dXNlZnVsTGlmZSI6MTAsImRyaXZlci1yYW5nZTp1c2VmdWxMaWZlOjAiOjUsImRyaXZlci1yYW5nZTp1c2VmdWxMaWZlOjEiOjIwLCJkcml2ZXI6aW52ZXN0bWVudCI6MjMsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjAiOjE1LCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDoxIjoyMDAsImRyaXZlcjpzdWJzaWR5Ijo3LjY2LCJkcml2ZXItcmFuZ2U6c3Vic2lkeTowIjoxLCJkcml2ZXItcmFuZ2U6c3Vic2lkeToxIjo1MCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoyMCwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjoxMzMuNSwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTp2YWx1ZSI6MiwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTptYXgiOjcsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTp2YWx1ZSI6NjUsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTptYXgiOjk1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2Fncjp2YWx1ZSI6MjIsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTp2YWx1ZSI6NzYuNDQsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6dmFsdWUiOjIxLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOm1heCI6MzUsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6dmFsdWUiOjE4Ljc4LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOnZhbHVlIjo3LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOm1heCI6MTAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOnZhbHVlIjoyLjg1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86dmFsdWUiOjE1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86bWF4Ijo3MCwidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86dmFsdWUiOjIxMywidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86bWF4IjozNTAsInRhcmdldDpsb2NhbEJlbmNobWFyazp2YWx1ZSI6MjMsInRhcmdldDpsb2NhbEJlbmNobWFyazptYXgiOjQwLCJ0YXJnZXQ6b2ZmaWNlclBheUNhZ3I6dmFsdWUiOjYsInRhcmdldDpvZmZpY2VyUGF5Q2FncjptYXgiOjEwLCJ0YXJnZXQ6b2ZmaWNlclBheUluY3JlYXNlOnZhbHVlIjowLCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6bWF4IjoyNTIuNjksInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTptYXgiOjEzNi44NCwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTptYXgiOjMzLjQzLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlJbmNyZWFzZTptYXgiOjMuNzR9LCJtZXRyaWNHcm91cEJhc2VzIjp7ImNvbXBhbnlTYWxlcyI6InJhdGUiLCJwcm9qZWN0U2FsZXMiOiJyYXRlIiwibGFib3JQcm9kdWN0aXZpdHkiOiJyYXRlIiwiZW1wbG95ZWVQYXkiOiJyYXRlIn0sImFwcGxpY2F0aW9uQ2F0ZWdvcnkiOiJnZW5lcmFsIn0=</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4fX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjU5LCJvZmZpY2VyUGF5IjowLjM4LCJkZXByZWNpYXRpb24iOjEuOSwib3RoZXJTZ2EiOjkuNSwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NS4zMSwiZW1wbG95ZWVCb251cyI6MC4yOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNCwib2ZmaWNlckJvbnVzIjowLjA0LCJjb2dzRGVwcmVjaWF0aW9uIjowLjQ3LCJzZ2FEZXByZWNpYXRpb24iOjEuNDMsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMzh9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNTQsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3LjE2LCJlbXBsb3llZUJvbnVzIjowLjM4LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjUyLCJvZmZpY2VyQm9udXMiOjAuMDYsImNvZ3NEZXByZWNpYXRpb24iOjAuMjksInNnYURlcHJlY2lhdGlvbiI6MS4xNSwicmVzZWFyY2hEZXZlbG9wbWVudCI6MC4yOX19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6NiwiZW1wbG95ZWVTYWxhcnkiOjUuNywiZW1wbG95ZWVCb251cyI6MC4zLCJvZmZpY2VyUGF5IjowLjQsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzYsIm9mZmljZXJCb251cyI6MC4wNCwiZGVwcmVjaWF0aW9uIjoyLCJjb2dzRGVwcmVjaWF0aW9uIjowLjUsInNnYURlcHJlY2lhdGlvbiI6MS41LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjQsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsImVtcGxveWVlU2FsYXJ5Ijo3LjYsImVtcGxveWVlQm9udXMiOjAuNCwib2ZmaWNlclBheSI6MC42LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjU0LCJvZmZpY2VyQm9udXMiOjAuMDYsImRlcHJlY2lhdGlvbiI6MS41LCJjb2dzRGVwcmVjaWF0aW9uIjowLjMsInNnYURlcHJlY2lhdGlvbiI6MS4yLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjMsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMSwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI4NTcxNDI4NTcxNDI4LCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwidXNlZnVsTGlmZSI6MTAsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwxLjY2NTMzNDUzNjkzNzczNDhlLTE2XSwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MzI1MzMwNTAxODQ2OTI3LDAuMDIwNzM1OTk0MTgzMTg5MTY2XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDBdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNDA3NjA4Njk1NjUyMTcxODQsMC4wNDQzODQwNTc5NzEwMTQ1Ml0sIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAwMDEzNDU3NTU2OTM1ODE5NzM3XSwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOlswLjAxOTEzOTQ1NzAyMzcxNzQ0MywwLjAyMDU1MzQ1OTkxNDc2MzA5NV0sIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wMzkxNjY2NjY2NjY2NjY2OCwwLjA0MjUwMDAwMDAwMDAwMDA5XSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RTYWxlc0dyb3d0aCI6WzAuMTUsMC4zXSwib3RoZXJTYWxlc0dyb3d0aCI6WzAuMDYwNzYwODY5NTY1MjE3MTksMC4wNjQzODQwNTc5NzEwMTQ1M10sInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOlswLDAuMDNdLCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6WzAuMDA1LDAuMDA1MTM0NTc1NTY5MzU4MTk3NV0sInByb2plY3RQYXlHcm93dGgiOlswLjA1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMC4wMjQxMzk0NTcwMjM3MTc0NDQsMC4wMjU1NTM0NTk5MTQ3NjMwOTZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGgiOlswLjA0NDE2NjY2NjY2NjY2NjY4LDAuMDQ3NTAwMDAwMDAwMDAwMDldLCJwcm9qZWN0U2dhUmF0ZUVuZCI6WzAuMDg0OTk5OTk5OTk5OTk5OTksMC4xMzVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA4OTI4NTcxNDI4NTcxNDI3LDAuMTE5Mjg1NzE0Mjg1NzE0MjddLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAuMDQyNjMxNTc4OTQ3MzY4MzYsMC4wNjU1NTU1NTU1NTU1NTU1OF0sInVzZWZ1bExpZmUiOls1LDIwXSwiaW52ZXN0bWVudCI6WzE1LDIwMF0sInN1YnNpZHkiOlsxLDUwXSwibG9jYWxCZW5jaG1hcmsiOlswLDEwMF19LCJ0YXJnZXRzIjp7ImNvbXBhbnlTYWxlc0NhZ3IiOnsidmFsdWUiOjIwLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjEzMy41LCJtYXgiOjI1Mi42OSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlQYXlTY2hlZHVsZSI6eyJ2YWx1ZSI6MiwibWF4Ijo3LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzU2hhcmUiOnsidmFsdWUiOjY1LCJtYXgiOjk1LCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjIsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6NzYuNDQsIm1heCI6MTM2Ljg0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MTguNzgsIm1heCI6MzMuNDMsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUNhZ3IiOnsidmFsdWUiOjcsIm1heCI6MTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUluY3JlYXNlIjp7InZhbHVlIjoyLjg1LCJtYXgiOjMuNzQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJpbnZlc3RtZW50U2FsZXNSYXRpbyI6eyJ2YWx1ZSI6MTUsIm1heCI6NzAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvIjp7InZhbHVlIjoyMTMsIm1heCI6MzUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibG9jYWxCZW5jaG1hcmsiOnsidmFsdWUiOjIzLCJtYXgiOjQwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUNhZ3IiOnsidmFsdWUiOjYsIm1heCI6MTAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnsiMjAyOTpvdGhlcjpzYWxlcyI6ODUuMTMsIjIwMjk6cHJvamVjdDo3LTgiOjcuODl9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2LjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mi43NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTQiOjAuNzMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi03IjozMi42NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTkiOjAuODIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMCI6MC4wOSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEyIjoxMS42NywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEzIjowLjYyLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTQiOjIuNDUsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNSI6MC42NCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEiOjcyLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNCI6MjMuMDQsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny02Ijo2Ljc4LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOCI6NS4xOSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTkiOjAuMzYsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMCI6MS44LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTMiOjkwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xIjoxNDMuMiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTMiOjk3LjM4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNCI6MC43NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTciOjM0LjUyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItOSI6MC44NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMiI6MTIuNDcsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMyI6MC42NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjoyLjU4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTUiOjAuNjcsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xIjo3NiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0LjMyLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNiI6Ny4wNCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTgiOjUuNTksImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTAiOjEuOSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6MC44LCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTkiOjAuOSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjowLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6Mi43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTUiOjAuNywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNCI6MjUuNiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTYiOjcuMywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTgiOjYsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny05IjowLjQsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xMCI6MiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudEFzc2V0cyI6NjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXNoIjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NSwiYmFsYW5jZS1zaGVldDoyMDIzOnRhbmdpYmxlQXNzZXRzIjo1MywiYmFsYW5jZS1zaGVldDoyMDIzOmJ1aWxkaW5ncyI6MTksImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzppbnRhbmdpYmxlQXNzZXRzIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUsImJhbGFuY2Utc2hlZXQ6MjAyMzpsaWFiaWxpdGllcyI6NzUsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50TGlhYmlsaXRpZXMiOjM5LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZExpYWJpbGl0aWVzIjozNiwiYmFsYW5jZS1zaGVldDoyMDIzOmxvbmdUZXJtRGVidCI6MjksImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hhcmVob2xkZXJFcXVpdHkiOjU0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NSwiYmFsYW5jZS1zaGVldDoyMDI0OmFzc2V0cyI6MTQzLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudEFzc2V0cyI6NzIsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNSwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkQXNzZXRzIjo3MSwiYmFsYW5jZS1zaGVldDoyMDI0OnRhbmdpYmxlQXNzZXRzIjo1OCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAsImJhbGFuY2Utc2hlZXQ6MjAyNDptYWNoaW5lcnkiOjI4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c29mdHdhcmUiOjYsImJhbGFuY2Utc2hlZXQ6MjAyNDpsaWFiaWxpdGllcyI6NzksImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZExpYWJpbGl0aWVzIjozOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEsImJhbGFuY2Utc2hlZXQ6MjAyNDpuZXRBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hhcmVob2xkZXJFcXVpdHkiOjYxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBleCI6OCwiYmFsYW5jZS1zaGVldDoyMDI1OmFzc2V0cyI6MTU2LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXNoIjoyNywiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkQXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI1OmJ1aWxkaW5ncyI6MjIsImJhbGFuY2Utc2hlZXQ6MjAyNTptYWNoaW5lcnkiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTppbnRhbmdpYmxlQXNzZXRzIjo5LCJiYWxhbmNlLXNoZWV0OjIwMjU6c29mdHdhcmUiOjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hvcnRUZXJtRGVidCI6MTEsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MCwiYmFsYW5jZS1zaGVldDoyMDI1OmxvbmdUZXJtRGVidCI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpuZXRBc3NldHMiOjczLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBleCI6MTAsImZ1dHVyZS1jYXBleDoyMDI2IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjciOjE1LCJmdXR1cmUtY2FwZXg6MjAyOCI6MTUsImZ1dHVyZS1jYXBleDoyMDI5IjowLCJmdXR1cmUtY2FwZXg6MjAzMCI6MCwiZnV0dXJlLWNhcGV4OjIwMzEiOjAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjEuNjY1MzM0NTM2OTM3NzM0OGUtMTYsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkzMjUzMzA1MDE4NDY5MjcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNzM1OTk0MTgzMTg5MTY2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLjAxOTEzOTQ1NzAyMzcxNzQ0MywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNTUzNDU5OTE0NzYzMDk1LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjAzOTE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNDI1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MCI6MC4xNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjMsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MCI6MC4wMjQxMzk0NTcwMjM3MTc0NDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDoxIjowLjAyNTU1MzQ1OTkxNDc2MzA5NiwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjowLjA0NDE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MSI6MC4wNDc1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjExLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MCI6MC4wODQ5OTk5OTk5OTk5OTk5OSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjEiOjAuMTM1LCJkcml2ZXI6b3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI4NTcxNDI4NTcxNDI4LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjAiOjAuMDg5Mjg1NzE0Mjg1NzE0MjcsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MSI6MC4xMTkyODU3MTQyODU3MTQyNywiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MCI6MC4wNDI2MzE1Nzg5NDczNjgzNiwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjEiOjAuMDY1NTU1NTU1NTU1NTU1NTgsImRyaXZlcjp1c2VmdWxMaWZlIjoxMCwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MCI6NSwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MSI6MjAsImRyaXZlcjppbnZlc3RtZW50IjoyMywiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjEiOjIwMCwiZHJpdmVyOnN1YnNpZHkiOjcuNjYsImRyaXZlci1yYW5nZTpzdWJzaWR5OjAiOjEsImRyaXZlci1yYW5nZTpzdWJzaWR5OjEiOjUwLCJkcml2ZXI6bG9jYWxCZW5jaG1hcmsiOjIzLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MCI6MCwiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjEiOjEwMCwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6dmFsdWUiOjIwLCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6dmFsdWUiOjEzMy41LCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjoyLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOm1heCI6NywidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOnZhbHVlIjo2NSwidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOm1heCI6OTUsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOnZhbHVlIjoyMiwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOnZhbHVlIjo3Ni40NCwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2Fncjp2YWx1ZSI6MjEsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6bWF4IjozNSwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTp2YWx1ZSI6MTguNzgsInRhcmdldDplbXBsb3llZVBheUNhZ3I6dmFsdWUiOjcsInRhcmdldDplbXBsb3llZVBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6dmFsdWUiOjIuODUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MTUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTptYXgiOjI1Mi42OSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOm1heCI6MTM2Ljg0LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOm1heCI6MzMuNDMsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOm1heCI6My43NH0sIm1ldHJpY0dyb3VwQmFzZXMiOnsiY29tcGFueVNhbGVzIjoicmF0ZSIsInByb2plY3RTYWxlcyI6InJhdGUiLCJsYWJvclByb2R1Y3Rpdml0eSI6InJhdGUiLCJlbXBsb3llZVBheSI6InJhdGUifSwiYXBwbGljYXRpb25DYXRlZ29yeSI6ImdlbmVyYWwiLCJhZGp1c3RlZERyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA3MDcyMzY4NDIxMDUxLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjoxLjE3NDE4NjQ5MTA2NDQ2NmUtMTYsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDE5ODE2Mjg3MTc4ODc3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDQ0ODUzNjMwNjc1MzI3NCwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwNjA5MzM3MDI3ODk4MDQsIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNjA3MzE2NTgzOTIyNDksIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4MDkwNTk1MDQ2MDU2NjMsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MTQ5Mzc3NzI0OTMwNjQ0Niwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjI5NjEzNzE0MzkwMDY1NzQzLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjQ5NTI1ODE3MTAzMzM2NiwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTU1NTA0MjcyNTc5NzcyODQsIm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwicHJvamVjdFBheUdyb3d0aCI6MC4wODg5NDM4NDEyMjQ2MzUxMSwib3RoZXJQYXlHcm93dGgiOjAuMDI0ODQyMTUyOTA2OTQxMzA2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjAyNjI0MDc1MjQ4NTg5MDg5Mywib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODcyMzc2OTIxMzYzMzgsInByb2plY3RTZ2FSYXRlRW5kIjowLjEwMzE1Mjk5NTQzNzQxMzIxLCJvdGhlclNnYVJhdGVFbmQiOjAuMTA5MjI2MTY0NjUxNjM2NTksInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzcxOTIzMTY3OTU4MzQ5LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6MjMsInN1YnNpZHkiOjcuNjYsImxvY2FsQmVuY2htYXJrIjoyM319</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make standard sample optimization reproducible
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -204,7 +204,7 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <v>20.152518023637867</v>
+        <v>20.01053154331047</v>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
@@ -234,7 +234,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <v>127.10000000000002</v>
+        <v>126.03000000000003</v>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
@@ -294,7 +294,7 @@
         </is>
       </c>
       <c r="B11" s="2">
-        <v>67.97614287618285</v>
+        <v>67.86048689138576</v>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
@@ -324,7 +324,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>29.614246350044503</v>
+        <v>29.38972537778437</v>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
@@ -354,7 +354,7 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <v>110.32</v>
+        <v>109.25</v>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
@@ -384,7 +384,7 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <v>32.737848619973995</v>
+        <v>32.53247290200707</v>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
@@ -414,7 +414,7 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <v>28.59999999999998</v>
+        <v>28.37999999999999</v>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <v>373.36814621409894</v>
+        <v>370.4960835509137</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
@@ -1259,22 +1259,22 @@
         <v>150</v>
       </c>
       <c r="E3" s="4">
-        <v>157.31</v>
+        <v>157.3</v>
       </c>
       <c r="F3" s="4">
-        <v>164.98000000000002</v>
+        <v>164.97</v>
       </c>
       <c r="G3" s="4">
-        <v>173.01999999999998</v>
+        <v>173.01</v>
       </c>
       <c r="H3" s="4">
-        <v>206.57</v>
+        <v>206.33999999999997</v>
       </c>
       <c r="I3" s="4">
-        <v>247.85000000000002</v>
+        <v>247.28000000000003</v>
       </c>
       <c r="J3" s="4">
-        <v>300.12</v>
+        <v>299.04</v>
       </c>
     </row>
     <row r="4">
@@ -1295,22 +1295,22 @@
         <v>4.748603351955305</v>
       </c>
       <c r="E4" s="2">
-        <v>4.8733333333333295</v>
+        <v>4.866666666666664</v>
       </c>
       <c r="F4" s="2">
-        <v>4.875723094526752</v>
+        <v>4.876033057851226</v>
       </c>
       <c r="G4" s="2">
-        <v>4.873317977936686</v>
+        <v>4.873613384251674</v>
       </c>
       <c r="H4" s="2">
-        <v>19.39082187030401</v>
+        <v>19.26478238252123</v>
       </c>
       <c r="I4" s="2">
-        <v>19.983540688386526</v>
+        <v>19.841039061742794</v>
       </c>
       <c r="J4" s="2">
-        <v>21.089368569699406</v>
+        <v>20.931737301844056</v>
       </c>
     </row>
     <row r="5">
@@ -1335,16 +1335,16 @@
         <v>112.18</v>
       </c>
       <c r="G5" s="2">
-        <v>117.66</v>
+        <v>117.65</v>
       </c>
       <c r="H5" s="2">
-        <v>139.13</v>
+        <v>138.97</v>
       </c>
       <c r="I5" s="2">
-        <v>166</v>
+        <v>165.63</v>
       </c>
       <c r="J5" s="2">
-        <v>199.78000000000003</v>
+        <v>199.07</v>
       </c>
     </row>
     <row r="6">
@@ -1397,22 +1397,22 @@
         <v>48</v>
       </c>
       <c r="E7" s="4">
-        <v>50.34</v>
+        <v>50.33000000000001</v>
       </c>
       <c r="F7" s="4">
-        <v>52.80000000000001</v>
+        <v>52.78999999999999</v>
       </c>
       <c r="G7" s="4">
         <v>55.359999999999985</v>
       </c>
       <c r="H7" s="4">
-        <v>67.44</v>
+        <v>67.36999999999998</v>
       </c>
       <c r="I7" s="4">
-        <v>81.85000000000002</v>
+        <v>81.65000000000003</v>
       </c>
       <c r="J7" s="4">
-        <v>100.33999999999997</v>
+        <v>99.97000000000003</v>
       </c>
     </row>
     <row r="8">
@@ -1431,22 +1431,22 @@
         <v>32</v>
       </c>
       <c r="E8" s="2">
-        <v>32.00050854999682</v>
+        <v>31.996185632549274</v>
       </c>
       <c r="F8" s="2">
-        <v>32.00387925809189</v>
+        <v>31.99975753167242</v>
       </c>
       <c r="G8" s="2">
-        <v>31.99630100566408</v>
+        <v>31.998150395930864</v>
       </c>
       <c r="H8" s="2">
-        <v>32.64752868277097</v>
+        <v>32.64999515362992</v>
       </c>
       <c r="I8" s="2">
-        <v>33.02400645551746</v>
+        <v>33.019249433840194</v>
       </c>
       <c r="J8" s="2">
-        <v>33.433293349326924</v>
+        <v>33.43031032637775</v>
       </c>
     </row>
     <row r="9">
@@ -1474,13 +1474,13 @@
         <v>44.19</v>
       </c>
       <c r="H9" s="2">
-        <v>48.489999999999995</v>
+        <v>48.459999999999994</v>
       </c>
       <c r="I9" s="2">
-        <v>53.92999999999999</v>
+        <v>53.86</v>
       </c>
       <c r="J9" s="2">
-        <v>60.18</v>
+        <v>60.05</v>
       </c>
     </row>
     <row r="10">
@@ -1771,22 +1771,22 @@
         <v>11.600000000000001</v>
       </c>
       <c r="E18" s="4">
-        <v>11.469999999999999</v>
+        <v>11.460000000000008</v>
       </c>
       <c r="F18" s="4">
-        <v>11.350000000000009</v>
+        <v>11.33999999999999</v>
       </c>
       <c r="G18" s="4">
         <v>11.169999999999984</v>
       </c>
       <c r="H18" s="4">
-        <v>18.950000000000003</v>
+        <v>18.909999999999982</v>
       </c>
       <c r="I18" s="4">
-        <v>27.920000000000027</v>
+        <v>27.790000000000035</v>
       </c>
       <c r="J18" s="4">
-        <v>40.159999999999975</v>
+        <v>39.92000000000003</v>
       </c>
     </row>
     <row r="19">
@@ -1805,22 +1805,22 @@
         <v>7.733333333333333</v>
       </c>
       <c r="E19" s="2">
-        <v>7.291335579429152</v>
+        <v>7.285441830896381</v>
       </c>
       <c r="F19" s="2">
-        <v>6.879621772336045</v>
+        <v>6.8739770867430385</v>
       </c>
       <c r="G19" s="2">
-        <v>6.455901051901505</v>
+        <v>6.456274203803239</v>
       </c>
       <c r="H19" s="2">
-        <v>9.173645737522392</v>
+        <v>9.16448580013569</v>
       </c>
       <c r="I19" s="2">
-        <v>11.26487795037322</v>
+        <v>11.238272403752843</v>
       </c>
       <c r="J19" s="2">
-        <v>13.381314141010254</v>
+        <v>13.349384697699312</v>
       </c>
     </row>
     <row r="20">
@@ -1839,22 +1839,22 @@
         <v>11.600000000000001</v>
       </c>
       <c r="E20" s="4">
-        <v>11.469999999999999</v>
+        <v>11.460000000000008</v>
       </c>
       <c r="F20" s="4">
-        <v>11.350000000000009</v>
+        <v>11.33999999999999</v>
       </c>
       <c r="G20" s="4">
         <v>11.169999999999984</v>
       </c>
       <c r="H20" s="4">
-        <v>18.950000000000003</v>
+        <v>18.909999999999982</v>
       </c>
       <c r="I20" s="4">
-        <v>27.920000000000027</v>
+        <v>27.790000000000035</v>
       </c>
       <c r="J20" s="4">
-        <v>40.159999999999975</v>
+        <v>39.92000000000003</v>
       </c>
     </row>
     <row r="21">
@@ -2079,22 +2079,22 @@
         <v>30.1</v>
       </c>
       <c r="E26" s="4">
-        <v>31.72</v>
+        <v>31.710000000000008</v>
       </c>
       <c r="F26" s="4">
-        <v>33.400000000000006</v>
+        <v>33.389999999999986</v>
       </c>
       <c r="G26" s="4">
         <v>35.13999999999998</v>
       </c>
       <c r="H26" s="4">
-        <v>44.059999999999995</v>
+        <v>44.019999999999975</v>
       </c>
       <c r="I26" s="4">
-        <v>54.74000000000002</v>
+        <v>54.61000000000003</v>
       </c>
       <c r="J26" s="4">
-        <v>68.84999999999998</v>
+        <v>68.61000000000003</v>
       </c>
     </row>
     <row r="27">
@@ -2115,22 +2115,22 @@
         <v>4.768534632788035</v>
       </c>
       <c r="E27" s="2">
-        <v>5.3820598006644405</v>
+        <v>5.348837209302348</v>
       </c>
       <c r="F27" s="2">
-        <v>5.29634300126105</v>
+        <v>5.298013245033051</v>
       </c>
       <c r="G27" s="2">
-        <v>5.20958083832328</v>
+        <v>5.2410901467505155</v>
       </c>
       <c r="H27" s="2">
-        <v>25.384177575412693</v>
+        <v>25.270347182697783</v>
       </c>
       <c r="I27" s="2">
-        <v>24.23967317294604</v>
+        <v>24.057246706042832</v>
       </c>
       <c r="J27" s="2">
-        <v>25.776397515527872</v>
+        <v>25.636330342428117</v>
       </c>
     </row>
     <row r="28">
@@ -2149,22 +2149,22 @@
         <v>20.06666666666667</v>
       </c>
       <c r="E28" s="2">
-        <v>20.164007373974954</v>
+        <v>20.1589319771138</v>
       </c>
       <c r="F28" s="2">
-        <v>20.244878167050555</v>
+        <v>20.240043644298954</v>
       </c>
       <c r="G28" s="2">
-        <v>20.309790775632866</v>
+        <v>20.310964684122293</v>
       </c>
       <c r="H28" s="2">
-        <v>21.32933146149005</v>
+        <v>21.33372104293883</v>
       </c>
       <c r="I28" s="2">
-        <v>22.085939076054075</v>
+        <v>22.08427693303139</v>
       </c>
       <c r="J28" s="2">
-        <v>22.940823670531778</v>
+        <v>22.94341894060996</v>
       </c>
     </row>
     <row r="29">
@@ -2391,22 +2391,22 @@
         <v>0.12808510638297874</v>
       </c>
       <c r="E35" s="2">
-        <v>0.12946938775510203</v>
+        <v>0.12942857142857145</v>
       </c>
       <c r="F35" s="2">
-        <v>0.12996108949416343</v>
+        <v>0.1299221789883268</v>
       </c>
       <c r="G35" s="2">
         <v>0.13063197026022297</v>
       </c>
       <c r="H35" s="2">
-        <v>0.157921146953405</v>
+        <v>0.15777777777777768</v>
       </c>
       <c r="I35" s="2">
-        <v>0.18941176470588245</v>
+        <v>0.18896193771626307</v>
       </c>
       <c r="J35" s="2">
-        <v>0.23026755852842803</v>
+        <v>0.2294648829431439</v>
       </c>
     </row>
     <row r="36">
@@ -2425,22 +2425,22 @@
         <v>15.100000000000001</v>
       </c>
       <c r="E36" s="4">
-        <v>15.739999999999998</v>
+        <v>15.730000000000008</v>
       </c>
       <c r="F36" s="4">
-        <v>16.38000000000001</v>
+        <v>16.36999999999999</v>
       </c>
       <c r="G36" s="4">
         <v>16.969999999999985</v>
       </c>
       <c r="H36" s="4">
-        <v>24.750000000000004</v>
+        <v>24.709999999999983</v>
       </c>
       <c r="I36" s="4">
-        <v>33.72000000000003</v>
+        <v>33.59000000000003</v>
       </c>
       <c r="J36" s="4">
-        <v>45.95999999999997</v>
+        <v>45.72000000000003</v>
       </c>
     </row>
     <row r="37">
@@ -2459,22 +2459,22 @@
         <v>10.066666666666668</v>
       </c>
       <c r="E37" s="2">
-        <v>10.005721187464243</v>
+        <v>10.000000000000005</v>
       </c>
       <c r="F37" s="2">
-        <v>9.928476178930785</v>
+        <v>9.923016305995024</v>
       </c>
       <c r="G37" s="2">
-        <v>9.808114668824405</v>
+        <v>9.808681579099465</v>
       </c>
       <c r="H37" s="2">
-        <v>11.981410659824759</v>
+        <v>11.975380440050396</v>
       </c>
       <c r="I37" s="2">
-        <v>13.605003026023816</v>
+        <v>13.583791653186683</v>
       </c>
       <c r="J37" s="2">
-        <v>15.313874450219902</v>
+        <v>15.288924558587489</v>
       </c>
     </row>
     <row r="38">
@@ -2495,22 +2495,22 @@
         <v>3.1420765027322606</v>
       </c>
       <c r="E38" s="2">
-        <v>4.238410596026476</v>
+        <v>4.172185430463626</v>
       </c>
       <c r="F38" s="2">
-        <v>4.066073697585848</v>
+        <v>4.068658614113052</v>
       </c>
       <c r="G38" s="2">
-        <v>3.601953601953456</v>
+        <v>3.665241295051902</v>
       </c>
       <c r="H38" s="2">
-        <v>45.84560989982338</v>
+        <v>45.60989982321748</v>
       </c>
       <c r="I38" s="2">
-        <v>36.24242424242434</v>
+        <v>35.93686766491322</v>
       </c>
       <c r="J38" s="2">
-        <v>36.298932384341455</v>
+        <v>36.11193807680853</v>
       </c>
     </row>
   </sheetData>
@@ -2663,22 +2663,22 @@
         <v>80</v>
       </c>
       <c r="E3" s="4">
-        <v>84.33</v>
+        <v>84.32</v>
       </c>
       <c r="F3" s="4">
-        <v>88.89</v>
+        <v>88.88</v>
       </c>
       <c r="G3" s="4">
-        <v>93.69</v>
+        <v>93.68</v>
       </c>
       <c r="H3" s="4">
-        <v>121.44</v>
+        <v>121.21</v>
       </c>
       <c r="I3" s="4">
-        <v>157.4</v>
+        <v>156.83</v>
       </c>
       <c r="J3" s="4">
-        <v>204.01</v>
+        <v>202.93</v>
       </c>
     </row>
     <row r="4">
@@ -2699,22 +2699,22 @@
         <v>5.263157894736836</v>
       </c>
       <c r="E4" s="2">
-        <v>5.412499999999998</v>
+        <v>5.399999999999983</v>
       </c>
       <c r="F4" s="2">
-        <v>5.407328352899321</v>
+        <v>5.407969639468702</v>
       </c>
       <c r="G4" s="2">
-        <v>5.39993250084374</v>
+        <v>5.400540054005409</v>
       </c>
       <c r="H4" s="2">
-        <v>29.618956131924424</v>
+        <v>29.387275832621683</v>
       </c>
       <c r="I4" s="2">
-        <v>29.61133069828723</v>
+        <v>29.387014272749788</v>
       </c>
       <c r="J4" s="2">
-        <v>29.61245235069885</v>
+        <v>29.3948861824906</v>
       </c>
     </row>
     <row r="5">
@@ -2733,22 +2733,22 @@
         <v>53.333333333333336</v>
       </c>
       <c r="E5" s="2">
-        <v>53.60752653995296</v>
+        <v>53.60457724094086</v>
       </c>
       <c r="F5" s="2">
-        <v>53.87925809188992</v>
+        <v>53.87646238710069</v>
       </c>
       <c r="G5" s="2">
-        <v>54.14980927060456</v>
+        <v>54.14715912375008</v>
       </c>
       <c r="H5" s="2">
-        <v>58.788788304206804</v>
+        <v>58.74285160414849</v>
       </c>
       <c r="I5" s="2">
-        <v>63.50615291506959</v>
+        <v>63.42203170494985</v>
       </c>
       <c r="J5" s="2">
-        <v>67.97614287618285</v>
+        <v>67.86048689138576</v>
       </c>
     </row>
     <row r="6">
@@ -2767,22 +2767,22 @@
         <v>25.6</v>
       </c>
       <c r="E6" s="4">
-        <v>26.989999999999995</v>
+        <v>26.97999999999999</v>
       </c>
       <c r="F6" s="4">
-        <v>28.450000000000003</v>
+        <v>28.439999999999998</v>
       </c>
       <c r="G6" s="4">
-        <v>29.979999999999997</v>
+        <v>29.980000000000004</v>
       </c>
       <c r="H6" s="4">
-        <v>39.489999999999995</v>
+        <v>39.41999999999999</v>
       </c>
       <c r="I6" s="4">
-        <v>52</v>
+        <v>51.81000000000002</v>
       </c>
       <c r="J6" s="4">
-        <v>68.45999999999998</v>
+        <v>68.1</v>
       </c>
     </row>
     <row r="7">
@@ -2801,22 +2801,22 @@
         <v>32</v>
       </c>
       <c r="E7" s="2">
-        <v>32.005217597533495</v>
+        <v>31.997153700189745</v>
       </c>
       <c r="F7" s="2">
-        <v>32.00584992687592</v>
+        <v>31.998199819982</v>
       </c>
       <c r="G7" s="2">
-        <v>31.999146120183582</v>
+        <v>32.00256191289496</v>
       </c>
       <c r="H7" s="2">
-        <v>32.51811594202898</v>
+        <v>32.52206913620987</v>
       </c>
       <c r="I7" s="2">
-        <v>33.03684879288437</v>
+        <v>33.0357712172416</v>
       </c>
       <c r="J7" s="2">
-        <v>33.557178569677944</v>
+        <v>33.55836988123983</v>
       </c>
     </row>
     <row r="8">
@@ -2835,22 +2835,22 @@
         <v>7.300000000000004</v>
       </c>
       <c r="E8" s="4">
-        <v>7.079999999999991</v>
+        <v>7.069999999999986</v>
       </c>
       <c r="F8" s="4">
-        <v>6.870000000000001</v>
+        <v>6.859999999999996</v>
       </c>
       <c r="G8" s="4">
-        <v>6.629999999999999</v>
+        <v>6.630000000000006</v>
       </c>
       <c r="H8" s="4">
-        <v>12.969999999999995</v>
+        <v>12.929999999999987</v>
       </c>
       <c r="I8" s="4">
-        <v>21.26</v>
+        <v>21.150000000000016</v>
       </c>
       <c r="J8" s="4">
-        <v>32.759999999999984</v>
+        <v>32.54</v>
       </c>
     </row>
     <row r="9">
@@ -2869,22 +2869,22 @@
         <v>9.125000000000005</v>
       </c>
       <c r="E9" s="2">
-        <v>8.395588758448941</v>
+        <v>8.384724857684994</v>
       </c>
       <c r="F9" s="2">
-        <v>7.728653391832603</v>
+        <v>7.718271827182714</v>
       </c>
       <c r="G9" s="2">
-        <v>7.076528978546269</v>
+        <v>7.077284372331347</v>
       </c>
       <c r="H9" s="2">
-        <v>10.68017127799736</v>
+        <v>10.667436680141892</v>
       </c>
       <c r="I9" s="2">
-        <v>13.506988564167727</v>
+        <v>13.485940190014675</v>
       </c>
       <c r="J9" s="2">
-        <v>16.058036370766132</v>
+        <v>16.03508599024294</v>
       </c>
     </row>
     <row r="10">
@@ -3005,22 +3005,22 @@
         <v>15.700000000000005</v>
       </c>
       <c r="E13" s="4">
-        <v>16.71999999999999</v>
+        <v>16.709999999999987</v>
       </c>
       <c r="F13" s="4">
-        <v>17.78</v>
+        <v>17.769999999999996</v>
       </c>
       <c r="G13" s="4">
-        <v>18.869999999999997</v>
+        <v>18.870000000000005</v>
       </c>
       <c r="H13" s="4">
-        <v>25.659999999999997</v>
+        <v>25.619999999999987</v>
       </c>
       <c r="I13" s="4">
-        <v>34.9</v>
+        <v>34.79000000000001</v>
       </c>
       <c r="J13" s="4">
-        <v>47.46999999999998</v>
+        <v>47.24999999999999</v>
       </c>
     </row>
     <row r="14">
@@ -3041,22 +3041,22 @@
         <v>5.2984574111334615</v>
       </c>
       <c r="E14" s="2">
-        <v>6.496815286624114</v>
+        <v>6.433121019108157</v>
       </c>
       <c r="F14" s="2">
-        <v>6.339712918660356</v>
+        <v>6.3435068821065865</v>
       </c>
       <c r="G14" s="2">
-        <v>6.13048368953879</v>
+        <v>6.190208216094595</v>
       </c>
       <c r="H14" s="2">
-        <v>35.9830418653948</v>
+        <v>35.77106518282977</v>
       </c>
       <c r="I14" s="2">
-        <v>36.00935307872175</v>
+        <v>35.792349726776074</v>
       </c>
       <c r="J14" s="2">
-        <v>36.01719197707731</v>
+        <v>35.81488933601602</v>
       </c>
     </row>
     <row r="15">
@@ -3283,22 +3283,22 @@
         <v>0.15392156862745102</v>
       </c>
       <c r="E21" s="2">
-        <v>0.15626168224299058</v>
+        <v>0.1561682242990653</v>
       </c>
       <c r="F21" s="2">
-        <v>0.15734513274336284</v>
+        <v>0.15725663716814156</v>
       </c>
       <c r="G21" s="2">
-        <v>0.15857142857142856</v>
+        <v>0.1585714285714286</v>
       </c>
       <c r="H21" s="2">
-        <v>0.210327868852459</v>
+        <v>0.20999999999999988</v>
       </c>
       <c r="I21" s="2">
-        <v>0.2792</v>
+        <v>0.2783200000000001</v>
       </c>
       <c r="J21" s="2">
-        <v>0.3708593749999998</v>
+        <v>0.36914062499999994</v>
       </c>
     </row>
     <row r="22">
@@ -3611,7 +3611,7 @@
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.87 % / 補助 5.41 % / 他 4.26 %</t>
+          <t xml:space="preserve">全社 4.87 % / 補助 5.4 % / 他 4.26 %</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
@@ -3626,17 +3626,17 @@
       </c>
       <c r="J4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 19.39 % / 補助 29.62 % / 他 7.31 %</t>
+          <t xml:space="preserve">全社 19.26 % / 補助 29.39 % / 他 7.31 %</t>
         </is>
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 19.98 % / 補助 29.61 % / 他 6.25 %</t>
+          <t xml:space="preserve">全社 19.84 % / 補助 29.39 % / 他 6.25 %</t>
         </is>
       </c>
       <c r="L4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 21.09 % / 補助 29.61 % / 他 6.26 %</t>
+          <t xml:space="preserve">全社 20.93 % / 補助 29.39 % / 他 6.26 %</t>
         </is>
       </c>
     </row>
@@ -3673,12 +3673,12 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 68 % / 補助 67.99 % / 他 68 %</t>
+          <t xml:space="preserve">全社 68 % / 補助 68 % / 他 68 %</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 68 % / 補助 67.99 % / 他 68 %</t>
+          <t xml:space="preserve">全社 68 % / 補助 68 % / 他 68 %</t>
         </is>
       </c>
       <c r="I5" s="0" t="inlineStr">
@@ -3693,12 +3693,12 @@
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 66.98 % / 補助 66.96 % / 他 67 %</t>
+          <t xml:space="preserve">全社 66.98 % / 補助 66.96 % / 他 67.01 %</t>
         </is>
       </c>
       <c r="L5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 66.57 % / 補助 66.44 % / 他 66.83 %</t>
+          <t xml:space="preserve">全社 66.57 % / 補助 66.44 % / 他 66.84 %</t>
         </is>
       </c>
     </row>
@@ -3735,12 +3735,12 @@
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32 % / 補助 32.01 % / 他 32 %</t>
+          <t xml:space="preserve">全社 32 % / 補助 32 % / 他 32 %</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32 % / 補助 32.01 % / 他 32 %</t>
+          <t xml:space="preserve">全社 32 % / 補助 32 % / 他 32 %</t>
         </is>
       </c>
       <c r="I6" s="0" t="inlineStr">
@@ -3755,12 +3755,12 @@
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 33.02 % / 補助 33.04 % / 他 33 %</t>
+          <t xml:space="preserve">全社 33.02 % / 補助 33.04 % / 他 32.99 %</t>
         </is>
       </c>
       <c r="L6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 33.43 % / 補助 33.56 % / 他 33.17 %</t>
+          <t xml:space="preserve">全社 33.43 % / 補助 33.56 % / 他 33.16 %</t>
         </is>
       </c>
     </row>
@@ -3802,27 +3802,27 @@
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 25.12 % / 補助 24.28 % / 他 26.11 %</t>
+          <t xml:space="preserve">全社 25.13 % / 補助 24.28 % / 他 26.11 %</t>
         </is>
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 25.54 % / 補助 24.92 % / 他 26.27 %</t>
+          <t xml:space="preserve">全社 25.54 % / 補助 24.93 % / 他 26.27 %</t>
         </is>
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 23.47 % / 補助 21.84 % / 他 25.81 %</t>
+          <t xml:space="preserve">全社 23.49 % / 補助 21.85 % / 他 25.81 %</t>
         </is>
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 21.76 % / 補助 19.53 % / 他 25.64 %</t>
+          <t xml:space="preserve">全社 21.78 % / 補助 19.55 % / 他 25.65 %</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 20.05 % / 補助 17.5 % / 他 25.47 %</t>
+          <t xml:space="preserve">全社 20.08 % / 補助 17.52 % / 他 25.48 %</t>
         </is>
       </c>
     </row>
@@ -3859,12 +3859,12 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.29 % / 補助 8.4 % / 他 6.02 %</t>
+          <t xml:space="preserve">全社 7.29 % / 補助 8.38 % / 他 6.02 %</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.88 % / 補助 7.73 % / 他 5.89 %</t>
+          <t xml:space="preserve">全社 6.87 % / 補助 7.72 % / 他 5.89 %</t>
         </is>
       </c>
       <c r="I8" s="0" t="inlineStr">
@@ -3874,17 +3874,17 @@
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.17 % / 補助 10.68 % / 他 7.02 %</t>
+          <t xml:space="preserve">全社 9.16 % / 補助 10.67 % / 他 7.02 %</t>
         </is>
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.26 % / 補助 13.51 % / 他 7.36 %</t>
+          <t xml:space="preserve">全社 11.24 % / 補助 13.49 % / 他 7.34 %</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.38 % / 補助 16.06 % / 他 7.7 %</t>
+          <t xml:space="preserve">全社 13.35 % / 補助 16.04 % / 他 7.68 %</t>
         </is>
       </c>
     </row>
@@ -3921,12 +3921,12 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.01 % / 補助 11.68 % / 他 8.07 %</t>
+          <t xml:space="preserve">全社 10 % / 補助 11.67 % / 他 8.07 %</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.93 % / 補助 11.7 % / 他 7.86 %</t>
+          <t xml:space="preserve">全社 9.92 % / 補助 11.69 % / 他 7.86 %</t>
         </is>
       </c>
       <c r="I9" s="0" t="inlineStr">
@@ -3936,17 +3936,17 @@
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.98 % / 補助 14.22 % / 他 8.79 %</t>
+          <t xml:space="preserve">全社 11.98 % / 補助 14.21 % / 他 8.79 %</t>
         </is>
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.61 % / 補助 16.24 % / 他 9.02 %</t>
+          <t xml:space="preserve">全社 13.58 % / 補助 16.23 % / 他 9 %</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.31 % / 補助 18.17 % / 他 9.26 %</t>
+          <t xml:space="preserve">全社 15.29 % / 補助 18.15 % / 他 9.24 %</t>
         </is>
       </c>
     </row>
@@ -3998,17 +3998,17 @@
       </c>
       <c r="J10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.51 % / 補助 11.77 % / 他 11.15 %</t>
+          <t xml:space="preserve">全社 11.51 % / 補助 11.76 % / 他 11.15 %</t>
         </is>
       </c>
       <c r="K10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.02 % / 補助 11.04 % / 他 10.98 %</t>
+          <t xml:space="preserve">全社 11.02 % / 補助 11.03 % / 他 10.99 %</t>
         </is>
       </c>
       <c r="L10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.47 % / 補助 10.31 % / 他 10.81 %</t>
+          <t xml:space="preserve">全社 10.47 % / 補助 10.3 % / 他 10.82 %</t>
         </is>
       </c>
     </row>
@@ -4122,17 +4122,17 @@
       </c>
       <c r="J12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.79 % / 補助 6.5 % / 他 12.06 %</t>
+          <t xml:space="preserve">全社 8.8 % / 補助 6.51 % / 他 12.06 %</t>
         </is>
       </c>
       <c r="K12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8 % / 補助 5.6 % / 他 12.17 %</t>
+          <t xml:space="preserve">全社 8.02 % / 補助 5.62 % / 他 12.17 %</t>
         </is>
       </c>
       <c r="L12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.22 % / 補助 4.83 % / 他 12.28 %</t>
+          <t xml:space="preserve">全社 7.24 % / 補助 4.86 % / 他 12.28 %</t>
         </is>
       </c>
     </row>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.64 % / 補助 0.49 % / 他 0.81 %</t>
+          <t xml:space="preserve">全社 0.64 % / 補助 0.5 % / 他 0.81 %</t>
         </is>
       </c>
       <c r="I13" s="0" t="inlineStr">
@@ -4241,22 +4241,22 @@
       </c>
       <c r="I14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.5 % / 補助 8.47 % / 他 12.9 %</t>
+          <t xml:space="preserve">全社 10.5 % / 補助 8.48 % / 他 12.9 %</t>
         </is>
       </c>
       <c r="J14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.35 % / 補助 6.91 % / 他 12.83 %</t>
+          <t xml:space="preserve">全社 9.36 % / 補助 6.92 % / 他 12.83 %</t>
         </is>
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.48 % / 補助 5.93 % / 他 12.91 %</t>
+          <t xml:space="preserve">全社 8.5 % / 補助 5.96 % / 他 12.91 %</t>
         </is>
       </c>
       <c r="L14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.63 % / 補助 5.1 % / 他 12.99 %</t>
+          <t xml:space="preserve">全社 7.65 % / 補助 5.13 % / 他 12.99 %</t>
         </is>
       </c>
     </row>
@@ -4479,12 +4479,12 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 50.38 % / 補助 41.09 % / 他 60.73 %</t>
+          <t xml:space="preserve">全社 50.39 % / 補助 41.11 % / 他 60.73 %</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 50.96 % / 補助 41.51 % / 他 61.72 %</t>
+          <t xml:space="preserve">全社 50.97 % / 補助 41.53 % / 他 61.72 %</t>
         </is>
       </c>
       <c r="I18" s="0" t="inlineStr">
@@ -4494,17 +4494,17 @@
       </c>
       <c r="J18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 43.83 % / 補助 32.7 % / 他 59.35 %</t>
+          <t xml:space="preserve">全社 43.87 % / 補助 32.75 % / 他 59.35 %</t>
         </is>
       </c>
       <c r="K18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 38.4 % / 補助 26.76 % / 他 58.87 %</t>
+          <t xml:space="preserve">全社 38.49 % / 補助 26.85 % / 他 58.93 %</t>
         </is>
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 33.25 % / 補助 21.93 % / 他 58.37 %</t>
+          <t xml:space="preserve">全社 33.36 % / 補助 22.03 % / 他 58.43 %</t>
         </is>
       </c>
     </row>
@@ -4618,17 +4618,17 @@
       </c>
       <c r="J20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.754 億円/人 / 補助 1.012 億円/人 / 他 0.553 億円/人</t>
+          <t xml:space="preserve">全社 0.753 億円/人 / 補助 1.01 億円/人 / 他 0.553 億円/人</t>
         </is>
       </c>
       <c r="K20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.873 億円/人 / 補助 1.28 億円/人 / 他 0.562 億円/人</t>
+          <t xml:space="preserve">全社 0.871 億円/人 / 補助 1.275 億円/人 / 他 0.562 億円/人</t>
         </is>
       </c>
       <c r="L20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.021 億円/人 / 補助 1.619 億円/人 / 他 0.572 億円/人</t>
+          <t xml:space="preserve">全社 1.017 億円/人 / 補助 1.611 億円/人 / 他 0.572 億円/人</t>
         </is>
       </c>
     </row>
@@ -4685,12 +4685,12 @@
       </c>
       <c r="K21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.098 億円/人 / 補助 0.173 億円/人 / 他 0.041 億円/人</t>
+          <t xml:space="preserve">全社 0.098 億円/人 / 補助 0.172 億円/人 / 他 0.041 億円/人</t>
         </is>
       </c>
       <c r="L21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.137 億円/人 / 補助 0.26 億円/人 / 他 0.044 億円/人</t>
+          <t xml:space="preserve">全社 0.136 億円/人 / 補助 0.258 億円/人 / 他 0.044 億円/人</t>
         </is>
       </c>
     </row>
@@ -4747,12 +4747,12 @@
       </c>
       <c r="K22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.189 億円/人 / 補助 0.279 億円/人 / 他 0.121 億円/人</t>
+          <t xml:space="preserve">全社 0.189 億円/人 / 補助 0.278 億円/人 / 他 0.121 億円/人</t>
         </is>
       </c>
       <c r="L22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.23 億円/人 / 補助 0.371 億円/人 / 他 0.125 億円/人</t>
+          <t xml:space="preserve">全社 0.229 億円/人 / 補助 0.369 億円/人 / 他 0.125 億円/人</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.53 pt / 補助 0.41 pt / 他 0.41 pt</t>
+          <t xml:space="preserve">全社 0.52 pt / 補助 0.4 pt / 他 0.41 pt</t>
         </is>
       </c>
       <c r="H24" s="0" t="inlineStr">
@@ -4861,22 +4861,22 @@
       </c>
       <c r="I24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.11 pt / 補助 -0.01 pt / 他 0 pt</t>
+          <t xml:space="preserve">全社 0.11 pt / 補助 -0 pt / 他 0 pt</t>
         </is>
       </c>
       <c r="J24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.6 pt / 補助 27.05 pt / 他 2.55 pt</t>
+          <t xml:space="preserve">全社 15.48 pt / 補助 26.82 pt / 他 2.55 pt</t>
         </is>
       </c>
       <c r="K24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 16.33 pt / 補助 27.11 pt / 他 1.7 pt</t>
+          <t xml:space="preserve">全社 16.19 pt / 補助 26.89 pt / 他 1.7 pt</t>
         </is>
       </c>
       <c r="L24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 17.57 pt / 補助 27.17 pt / 他 1.91 pt</t>
+          <t xml:space="preserve">全社 17.41 pt / 補助 26.96 pt / 他 1.91 pt</t>
         </is>
       </c>
     </row>
@@ -4975,7 +4975,7 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.71 % / 補助 3.28 % / 他 2.06 %</t>
+          <t xml:space="preserve">全社 2.71 % / 補助 3.29 % / 他 2.06 %</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
@@ -4990,17 +4990,17 @@
       </c>
       <c r="J26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.81 % / 補助 3.54 % / 他 1.76 %</t>
+          <t xml:space="preserve">全社 2.81 % / 補助 3.55 % / 他 1.76 %</t>
         </is>
       </c>
       <c r="K26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.34 % / 補助 2.73 % / 他 1.66 %</t>
+          <t xml:space="preserve">全社 2.35 % / 補助 2.74 % / 他 1.66 %</t>
         </is>
       </c>
       <c r="L26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.93 % / 補助 2.11 % / 他 1.56 %</t>
+          <t xml:space="preserve">全社 1.94 % / 補助 2.12 % / 他 1.56 %</t>
         </is>
       </c>
     </row>
@@ -5161,12 +5161,12 @@
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.69 倍 / 補助 3.56 倍 / 他 3.93 倍</t>
+          <t xml:space="preserve">全社 3.68 倍 / 補助 3.55 倍 / 他 3.93 倍</t>
         </is>
       </c>
       <c r="H29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.26 倍 / 補助 2.95 倍 / 他 3.99 倍</t>
+          <t xml:space="preserve">全社 3.25 倍 / 補助 2.94 倍 / 他 3.99 倍</t>
         </is>
       </c>
       <c r="I29" s="0" t="inlineStr">
@@ -5176,17 +5176,17 @@
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.27 倍 / 補助 4.02 倍 / 他 4.99 倍</t>
+          <t xml:space="preserve">全社 4.26 倍 / 補助 4.01 倍 / 他 4.99 倍</t>
         </is>
       </c>
       <c r="K29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5.81 倍 / 補助 5.94 倍 / 他 5.44 倍</t>
+          <t xml:space="preserve">全社 5.79 倍 / 補助 5.92 倍 / 他 5.43 倍</t>
         </is>
       </c>
       <c r="L29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.92 倍 / 補助 8.62 倍 / 他 5.93 倍</t>
+          <t xml:space="preserve">全社 7.88 倍 / 補助 8.57 倍 / 他 5.92 倍</t>
         </is>
       </c>
     </row>
@@ -5347,7 +5347,7 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 53.61 %</t>
+          <t xml:space="preserve">構成比 53.6 %</t>
         </is>
       </c>
       <c r="H32" s="0" t="inlineStr">
@@ -5362,17 +5362,17 @@
       </c>
       <c r="J32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 58.79 %</t>
+          <t xml:space="preserve">構成比 58.74 %</t>
         </is>
       </c>
       <c r="K32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 63.51 %</t>
+          <t xml:space="preserve">構成比 63.42 %</t>
         </is>
       </c>
       <c r="L32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 67.98 %</t>
+          <t xml:space="preserve">構成比 67.86 %</t>
         </is>
       </c>
     </row>
@@ -5409,14 +5409,14 @@
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">補助 5.4 % / 他 4.26 %</t>
+        </is>
+      </c>
+      <c r="H33" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">補助 5.41 % / 他 4.26 %</t>
         </is>
       </c>
-      <c r="H33" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">補助 5.41 % / 他 4.26 %</t>
-        </is>
-      </c>
       <c r="I33" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">補助 5.4 % / 他 4.26 %</t>
@@ -5424,17 +5424,17 @@
       </c>
       <c r="J33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 29.62 % / 他 7.31 %</t>
+          <t xml:space="preserve">補助 29.39 % / 他 7.31 %</t>
         </is>
       </c>
       <c r="K33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 29.61 % / 他 6.25 %</t>
+          <t xml:space="preserve">補助 29.39 % / 他 6.25 %</t>
         </is>
       </c>
       <c r="L33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 29.61 % / 他 6.26 %</t>
+          <t xml:space="preserve">補助 29.39 % / 他 6.26 %</t>
         </is>
       </c>
     </row>
@@ -5471,19 +5471,19 @@
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">差 -0 pt</t>
+        </is>
+      </c>
+      <c r="H34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">差 0 pt</t>
+        </is>
+      </c>
+      <c r="I34" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">差 -0.01 pt</t>
         </is>
       </c>
-      <c r="H34" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">差 -0 pt</t>
-        </is>
-      </c>
-      <c r="I34" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">差 -0.01 pt</t>
-        </is>
-      </c>
       <c r="J34" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">差 0.31 pt</t>
@@ -5491,12 +5491,12 @@
       </c>
       <c r="K34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -0.04 pt</t>
+          <t xml:space="preserve">差 -0.05 pt</t>
         </is>
       </c>
       <c r="L34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -0.39 pt</t>
+          <t xml:space="preserve">差 -0.4 pt</t>
         </is>
       </c>
     </row>
@@ -5533,12 +5533,12 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 2.38 pt</t>
+          <t xml:space="preserve">差 2.37 pt</t>
         </is>
       </c>
       <c r="H35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 1.84 pt</t>
+          <t xml:space="preserve">差 1.83 pt</t>
         </is>
       </c>
       <c r="I35" s="0" t="inlineStr">
@@ -5548,7 +5548,7 @@
       </c>
       <c r="J35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 3.66 pt</t>
+          <t xml:space="preserve">差 3.64 pt</t>
         </is>
       </c>
       <c r="K35" s="0" t="inlineStr">
@@ -5610,17 +5610,17 @@
       </c>
       <c r="J36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.012 億円/人 / 他 0.553 億円/人</t>
+          <t xml:space="preserve">補助 1.01 億円/人 / 他 0.553 億円/人</t>
         </is>
       </c>
       <c r="K36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.28 億円/人 / 他 0.562 億円/人</t>
+          <t xml:space="preserve">補助 1.275 億円/人 / 他 0.562 億円/人</t>
         </is>
       </c>
       <c r="L36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.619 億円/人 / 他 0.572 億円/人</t>
+          <t xml:space="preserve">補助 1.611 億円/人 / 他 0.572 億円/人</t>
         </is>
       </c>
     </row>
@@ -5719,7 +5719,7 @@
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 169.23 %</t>
+          <t xml:space="preserve">寄与率 164.29 %</t>
         </is>
       </c>
       <c r="H38" s="0" t="inlineStr">
@@ -5729,22 +5729,22 @@
       </c>
       <c r="I38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 133.33 %</t>
+          <t xml:space="preserve">寄与率 135.29 %</t>
         </is>
       </c>
       <c r="J38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 81.49 %</t>
+          <t xml:space="preserve">寄与率 81.4 %</t>
         </is>
       </c>
       <c r="K38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 92.42 %</t>
+          <t xml:space="preserve">寄与率 92.57 %</t>
         </is>
       </c>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 93.95 %</t>
+          <t xml:space="preserve">寄与率 93.9 %</t>
         </is>
       </c>
     </row>
@@ -9855,7 +9855,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4fX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjU5LCJvZmZpY2VyUGF5IjowLjM4LCJkZXByZWNpYXRpb24iOjEuOSwib3RoZXJTZ2EiOjkuNSwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NS4zMSwiZW1wbG95ZWVCb251cyI6MC4yOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNCwib2ZmaWNlckJvbnVzIjowLjA0LCJjb2dzRGVwcmVjaWF0aW9uIjowLjQ3LCJzZ2FEZXByZWNpYXRpb24iOjEuNDMsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMzh9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNTQsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3LjE2LCJlbXBsb3llZUJvbnVzIjowLjM4LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjUyLCJvZmZpY2VyQm9udXMiOjAuMDYsImNvZ3NEZXByZWNpYXRpb24iOjAuMjksInNnYURlcHJlY2lhdGlvbiI6MS4xNSwicmVzZWFyY2hEZXZlbG9wbWVudCI6MC4yOX19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6NiwiZW1wbG95ZWVTYWxhcnkiOjUuNywiZW1wbG95ZWVCb251cyI6MC4zLCJvZmZpY2VyUGF5IjowLjQsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzYsIm9mZmljZXJCb251cyI6MC4wNCwiZGVwcmVjaWF0aW9uIjoyLCJjb2dzRGVwcmVjaWF0aW9uIjowLjUsInNnYURlcHJlY2lhdGlvbiI6MS41LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjQsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsImVtcGxveWVlU2FsYXJ5Ijo3LjYsImVtcGxveWVlQm9udXMiOjAuNCwib2ZmaWNlclBheSI6MC42LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjU0LCJvZmZpY2VyQm9udXMiOjAuMDYsImRlcHJlY2lhdGlvbiI6MS41LCJjb2dzRGVwcmVjaWF0aW9uIjowLjMsInNnYURlcHJlY2lhdGlvbiI6MS4yLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjMsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMSwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI4NTcxNDI4NTcxNDI4LCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwidXNlZnVsTGlmZSI6MTAsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwxLjY2NTMzNDUzNjkzNzczNDhlLTE2XSwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MzI1MzMwNTAxODQ2OTI3LDAuMDIwNzM1OTk0MTgzMTg5MTY2XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDBdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNDA3NjA4Njk1NjUyMTcxODQsMC4wNDQzODQwNTc5NzEwMTQ1Ml0sIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAwMDEzNDU3NTU2OTM1ODE5NzM3XSwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOlswLjAxOTEzOTQ1NzAyMzcxNzQ0MywwLjAyMDU1MzQ1OTkxNDc2MzA5NV0sIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wMzkxNjY2NjY2NjY2NjY2OCwwLjA0MjUwMDAwMDAwMDAwMDA5XSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RTYWxlc0dyb3d0aCI6WzAuMTUsMC4zXSwib3RoZXJTYWxlc0dyb3d0aCI6WzAuMDYwNzYwODY5NTY1MjE3MTksMC4wNjQzODQwNTc5NzEwMTQ1M10sInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOlswLDAuMDNdLCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6WzAuMDA1LDAuMDA1MTM0NTc1NTY5MzU4MTk3NV0sInByb2plY3RQYXlHcm93dGgiOlswLjA1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMC4wMjQxMzk0NTcwMjM3MTc0NDQsMC4wMjU1NTM0NTk5MTQ3NjMwOTZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGgiOlswLjA0NDE2NjY2NjY2NjY2NjY4LDAuMDQ3NTAwMDAwMDAwMDAwMDldLCJwcm9qZWN0U2dhUmF0ZUVuZCI6WzAuMDg0OTk5OTk5OTk5OTk5OTksMC4xMzVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA4OTI4NTcxNDI4NTcxNDI3LDAuMTE5Mjg1NzE0Mjg1NzE0MjddLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAuMDQyNjMxNTc4OTQ3MzY4MzYsMC4wNjU1NTU1NTU1NTU1NTU1OF0sInVzZWZ1bExpZmUiOls1LDIwXSwiaW52ZXN0bWVudCI6WzE1LDIwMF0sInN1YnNpZHkiOlsxLDUwXSwibG9jYWxCZW5jaG1hcmsiOlswLDEwMF19LCJ0YXJnZXRzIjp7ImNvbXBhbnlTYWxlc0NhZ3IiOnsidmFsdWUiOjIwLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjEzMy41LCJtYXgiOjI1Mi42OSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlQYXlTY2hlZHVsZSI6eyJ2YWx1ZSI6MiwibWF4Ijo3LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzU2hhcmUiOnsidmFsdWUiOjY1LCJtYXgiOjk1LCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjIsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6NzYuNDQsIm1heCI6MTM2Ljg0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MTguNzgsIm1heCI6MzMuNDMsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUNhZ3IiOnsidmFsdWUiOjcsIm1heCI6MTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUluY3JlYXNlIjp7InZhbHVlIjoyLjg1LCJtYXgiOjMuNzQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJpbnZlc3RtZW50U2FsZXNSYXRpbyI6eyJ2YWx1ZSI6MTUsIm1heCI6NzAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvIjp7InZhbHVlIjoyMTMsIm1heCI6MzUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibG9jYWxCZW5jaG1hcmsiOnsidmFsdWUiOjIzLCJtYXgiOjQwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUNhZ3IiOnsidmFsdWUiOjYsIm1heCI6MTAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnsiMjAyOTpvdGhlcjpzYWxlcyI6ODUuMTMsIjIwMjk6cHJvamVjdDo3LTgiOjcuODl9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2LjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mi43NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTQiOjAuNzMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi03IjozMi42NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTkiOjAuODIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMCI6MC4wOSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEyIjoxMS42NywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEzIjowLjYyLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTQiOjIuNDUsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNSI6MC42NCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEiOjcyLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNCI6MjMuMDQsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny02Ijo2Ljc4LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOCI6NS4xOSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTkiOjAuMzYsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMCI6MS44LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTMiOjkwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xIjoxNDMuMiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTMiOjk3LjM4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNCI6MC43NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTciOjM0LjUyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItOSI6MC44NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMiI6MTIuNDcsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMyI6MC42NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjoyLjU4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTUiOjAuNjcsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xIjo3NiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0LjMyLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNiI6Ny4wNCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTgiOjUuNTksImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTAiOjEuOSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6MC44LCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTkiOjAuOSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjowLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6Mi43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTUiOjAuNywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNCI6MjUuNiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTYiOjcuMywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTgiOjYsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny05IjowLjQsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xMCI6MiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudEFzc2V0cyI6NjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXNoIjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NSwiYmFsYW5jZS1zaGVldDoyMDIzOnRhbmdpYmxlQXNzZXRzIjo1MywiYmFsYW5jZS1zaGVldDoyMDIzOmJ1aWxkaW5ncyI6MTksImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzppbnRhbmdpYmxlQXNzZXRzIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUsImJhbGFuY2Utc2hlZXQ6MjAyMzpsaWFiaWxpdGllcyI6NzUsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50TGlhYmlsaXRpZXMiOjM5LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZExpYWJpbGl0aWVzIjozNiwiYmFsYW5jZS1zaGVldDoyMDIzOmxvbmdUZXJtRGVidCI6MjksImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hhcmVob2xkZXJFcXVpdHkiOjU0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NSwiYmFsYW5jZS1zaGVldDoyMDI0OmFzc2V0cyI6MTQzLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudEFzc2V0cyI6NzIsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNSwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkQXNzZXRzIjo3MSwiYmFsYW5jZS1zaGVldDoyMDI0OnRhbmdpYmxlQXNzZXRzIjo1OCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAsImJhbGFuY2Utc2hlZXQ6MjAyNDptYWNoaW5lcnkiOjI4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c29mdHdhcmUiOjYsImJhbGFuY2Utc2hlZXQ6MjAyNDpsaWFiaWxpdGllcyI6NzksImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZExpYWJpbGl0aWVzIjozOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEsImJhbGFuY2Utc2hlZXQ6MjAyNDpuZXRBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hhcmVob2xkZXJFcXVpdHkiOjYxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBleCI6OCwiYmFsYW5jZS1zaGVldDoyMDI1OmFzc2V0cyI6MTU2LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXNoIjoyNywiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkQXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI1OmJ1aWxkaW5ncyI6MjIsImJhbGFuY2Utc2hlZXQ6MjAyNTptYWNoaW5lcnkiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTppbnRhbmdpYmxlQXNzZXRzIjo5LCJiYWxhbmNlLXNoZWV0OjIwMjU6c29mdHdhcmUiOjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hvcnRUZXJtRGVidCI6MTEsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MCwiYmFsYW5jZS1zaGVldDoyMDI1OmxvbmdUZXJtRGVidCI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpuZXRBc3NldHMiOjczLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBleCI6MTAsImZ1dHVyZS1jYXBleDoyMDI2IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjciOjE1LCJmdXR1cmUtY2FwZXg6MjAyOCI6MTUsImZ1dHVyZS1jYXBleDoyMDI5IjowLCJmdXR1cmUtY2FwZXg6MjAzMCI6MCwiZnV0dXJlLWNhcGV4OjIwMzEiOjAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjEuNjY1MzM0NTM2OTM3NzM0OGUtMTYsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkzMjUzMzA1MDE4NDY5MjcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNzM1OTk0MTgzMTg5MTY2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLjAxOTEzOTQ1NzAyMzcxNzQ0MywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNTUzNDU5OTE0NzYzMDk1LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjAzOTE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNDI1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MCI6MC4xNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjMsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MCI6MC4wMjQxMzk0NTcwMjM3MTc0NDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDoxIjowLjAyNTU1MzQ1OTkxNDc2MzA5NiwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjowLjA0NDE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MSI6MC4wNDc1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjExLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MCI6MC4wODQ5OTk5OTk5OTk5OTk5OSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjEiOjAuMTM1LCJkcml2ZXI6b3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI4NTcxNDI4NTcxNDI4LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjAiOjAuMDg5Mjg1NzE0Mjg1NzE0MjcsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MSI6MC4xMTkyODU3MTQyODU3MTQyNywiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MCI6MC4wNDI2MzE1Nzg5NDczNjgzNiwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjEiOjAuMDY1NTU1NTU1NTU1NTU1NTgsImRyaXZlcjp1c2VmdWxMaWZlIjoxMCwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MCI6NSwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MSI6MjAsImRyaXZlcjppbnZlc3RtZW50IjoyMywiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjEiOjIwMCwiZHJpdmVyOnN1YnNpZHkiOjcuNjYsImRyaXZlci1yYW5nZTpzdWJzaWR5OjAiOjEsImRyaXZlci1yYW5nZTpzdWJzaWR5OjEiOjUwLCJkcml2ZXI6bG9jYWxCZW5jaG1hcmsiOjIzLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MCI6MCwiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjEiOjEwMCwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6dmFsdWUiOjIwLCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6dmFsdWUiOjEzMy41LCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjoyLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOm1heCI6NywidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOnZhbHVlIjo2NSwidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOm1heCI6OTUsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOnZhbHVlIjoyMiwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOnZhbHVlIjo3Ni40NCwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2Fncjp2YWx1ZSI6MjEsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6bWF4IjozNSwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTp2YWx1ZSI6MTguNzgsInRhcmdldDplbXBsb3llZVBheUNhZ3I6dmFsdWUiOjcsInRhcmdldDplbXBsb3llZVBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6dmFsdWUiOjIuODUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MTUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTptYXgiOjI1Mi42OSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOm1heCI6MTM2Ljg0LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOm1heCI6MzMuNDMsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOm1heCI6My43NH0sIm1ldHJpY0dyb3VwQmFzZXMiOnsiY29tcGFueVNhbGVzIjoicmF0ZSIsInByb2plY3RTYWxlcyI6InJhdGUiLCJsYWJvclByb2R1Y3Rpdml0eSI6InJhdGUiLCJlbXBsb3llZVBheSI6InJhdGUifSwiYXBwbGljYXRpb25DYXRlZ29yeSI6ImdlbmVyYWwiLCJhZGp1c3RlZERyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA3MDcyMzY4NDIxMDUxLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjoxLjE3NDE4NjQ5MTA2NDQ2NmUtMTYsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDE5ODE2Mjg3MTc4ODc3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDQ0ODUzNjMwNjc1MzI3NCwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwNjA5MzM3MDI3ODk4MDQsIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNjA3MzE2NTgzOTIyNDksIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4MDkwNTk1MDQ2MDU2NjMsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MTQ5Mzc3NzI0OTMwNjQ0Niwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjI5NjEzNzE0MzkwMDY1NzQzLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjQ5NTI1ODE3MTAzMzM2NiwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTU1NTA0MjcyNTc5NzcyODQsIm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwicHJvamVjdFBheUdyb3d0aCI6MC4wODg5NDM4NDEyMjQ2MzUxMSwib3RoZXJQYXlHcm93dGgiOjAuMDI0ODQyMTUyOTA2OTQxMzA2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjAyNjI0MDc1MjQ4NTg5MDg5Mywib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODcyMzc2OTIxMzYzMzgsInByb2plY3RTZ2FSYXRlRW5kIjowLjEwMzE1Mjk5NTQzNzQxMzIxLCJvdGhlclNnYVJhdGVFbmQiOjAuMTA5MjI2MTY0NjUxNjM2NTksInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzcxOTIzMTY3OTU4MzQ5LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6MjMsInN1YnNpZHkiOjcuNjYsImxvY2FsQmVuY2htYXJrIjoyM319</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4fX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjU5LCJvZmZpY2VyUGF5IjowLjM4LCJkZXByZWNpYXRpb24iOjEuOSwib3RoZXJTZ2EiOjkuNSwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NS4zMSwiZW1wbG95ZWVCb251cyI6MC4yOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNCwib2ZmaWNlckJvbnVzIjowLjA0LCJjb2dzRGVwcmVjaWF0aW9uIjowLjQ3LCJzZ2FEZXByZWNpYXRpb24iOjEuNDMsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMzh9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNTQsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3LjE2LCJlbXBsb3llZUJvbnVzIjowLjM4LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjUyLCJvZmZpY2VyQm9udXMiOjAuMDYsImNvZ3NEZXByZWNpYXRpb24iOjAuMjksInNnYURlcHJlY2lhdGlvbiI6MS4xNSwicmVzZWFyY2hEZXZlbG9wbWVudCI6MC4yOX19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6NiwiZW1wbG95ZWVTYWxhcnkiOjUuNywiZW1wbG95ZWVCb251cyI6MC4zLCJvZmZpY2VyUGF5IjowLjQsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzYsIm9mZmljZXJCb251cyI6MC4wNCwiZGVwcmVjaWF0aW9uIjoyLCJjb2dzRGVwcmVjaWF0aW9uIjowLjUsInNnYURlcHJlY2lhdGlvbiI6MS41LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjQsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsImVtcGxveWVlU2FsYXJ5Ijo3LjYsImVtcGxveWVlQm9udXMiOjAuNCwib2ZmaWNlclBheSI6MC42LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjU0LCJvZmZpY2VyQm9udXMiOjAuMDYsImRlcHJlY2lhdGlvbiI6MS41LCJjb2dzRGVwcmVjaWF0aW9uIjowLjMsInNnYURlcHJlY2lhdGlvbiI6MS4yLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjMsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMSwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI4NTcxNDI4NTcxNDI4LCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwidXNlZnVsTGlmZSI6MTAsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwxLjY2NTMzNDUzNjkzNzczNDhlLTE2XSwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MzI1MzMwNTAxODQ2OTI3LDAuMDIwNzM1OTk0MTgzMTg5MTY2XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDBdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNDA3NjA4Njk1NjUyMTcxODQsMC4wNDQzODQwNTc5NzEwMTQ1Ml0sIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAwMDEzNDU3NTU2OTM1ODE5NzM3XSwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOlswLjAxOTEzOTQ1NzAyMzcxNzQ0MywwLjAyMDU1MzQ1OTkxNDc2MzA5NV0sIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wMzkxNjY2NjY2NjY2NjY2OCwwLjA0MjUwMDAwMDAwMDAwMDA5XSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RTYWxlc0dyb3d0aCI6WzAuMTUsMC4zXSwib3RoZXJTYWxlc0dyb3d0aCI6WzAuMDYwNzYwODY5NTY1MjE3MTksMC4wNjQzODQwNTc5NzEwMTQ1M10sInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOlswLDAuMDNdLCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6WzAuMDA1LDAuMDA1MTM0NTc1NTY5MzU4MTk3NV0sInByb2plY3RQYXlHcm93dGgiOlswLjA1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMC4wMjQxMzk0NTcwMjM3MTc0NDQsMC4wMjU1NTM0NTk5MTQ3NjMwOTZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGgiOlswLjA0NDE2NjY2NjY2NjY2NjY4LDAuMDQ3NTAwMDAwMDAwMDAwMDldLCJwcm9qZWN0U2dhUmF0ZUVuZCI6WzAuMDg0OTk5OTk5OTk5OTk5OTksMC4xMzVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA4OTI4NTcxNDI4NTcxNDI3LDAuMTE5Mjg1NzE0Mjg1NzE0MjddLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAuMDQyNjMxNTc4OTQ3MzY4MzYsMC4wNjU1NTU1NTU1NTU1NTU1OF0sInVzZWZ1bExpZmUiOls1LDIwXSwiaW52ZXN0bWVudCI6WzE1LDIwMF0sInN1YnNpZHkiOlsxLDUwXSwibG9jYWxCZW5jaG1hcmsiOlswLDEwMF19LCJ0YXJnZXRzIjp7ImNvbXBhbnlTYWxlc0NhZ3IiOnsidmFsdWUiOjIwLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjEzMy41LCJtYXgiOjI1Mi42OSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlQYXlTY2hlZHVsZSI6eyJ2YWx1ZSI6MiwibWF4Ijo3LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzU2hhcmUiOnsidmFsdWUiOjY1LCJtYXgiOjk1LCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjIsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6NzYuNDQsIm1heCI6MTM2Ljg0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MTguNzgsIm1heCI6MzMuNDMsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUNhZ3IiOnsidmFsdWUiOjcsIm1heCI6MTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUluY3JlYXNlIjp7InZhbHVlIjoyLjg1LCJtYXgiOjMuNzQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJpbnZlc3RtZW50U2FsZXNSYXRpbyI6eyJ2YWx1ZSI6MTUsIm1heCI6NzAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvIjp7InZhbHVlIjoyMTMsIm1heCI6MzUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibG9jYWxCZW5jaG1hcmsiOnsidmFsdWUiOjIzLCJtYXgiOjQwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUNhZ3IiOnsidmFsdWUiOjYsIm1heCI6MTAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnsiMjAyOTpvdGhlcjpzYWxlcyI6ODUuMTMsIjIwMjk6cHJvamVjdDo3LTgiOjcuODl9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2LjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mi43NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTQiOjAuNzMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi03IjozMi42NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTkiOjAuODIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMCI6MC4wOSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEyIjoxMS42NywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEzIjowLjYyLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTQiOjIuNDUsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNSI6MC42NCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEiOjcyLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNCI6MjMuMDQsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny02Ijo2Ljc4LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOCI6NS4xOSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTkiOjAuMzYsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMCI6MS44LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTMiOjkwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xIjoxNDMuMiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTMiOjk3LjM4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNCI6MC43NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTciOjM0LjUyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItOSI6MC44NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMiI6MTIuNDcsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMyI6MC42NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjoyLjU4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTUiOjAuNjcsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xIjo3NiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0LjMyLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNiI6Ny4wNCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTgiOjUuNTksImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTAiOjEuOSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6MC44LCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTkiOjAuOSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjowLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6Mi43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTUiOjAuNywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNCI6MjUuNiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTYiOjcuMywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTgiOjYsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny05IjowLjQsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xMCI6MiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudEFzc2V0cyI6NjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXNoIjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NSwiYmFsYW5jZS1zaGVldDoyMDIzOnRhbmdpYmxlQXNzZXRzIjo1MywiYmFsYW5jZS1zaGVldDoyMDIzOmJ1aWxkaW5ncyI6MTksImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzppbnRhbmdpYmxlQXNzZXRzIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUsImJhbGFuY2Utc2hlZXQ6MjAyMzpsaWFiaWxpdGllcyI6NzUsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50TGlhYmlsaXRpZXMiOjM5LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZExpYWJpbGl0aWVzIjozNiwiYmFsYW5jZS1zaGVldDoyMDIzOmxvbmdUZXJtRGVidCI6MjksImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hhcmVob2xkZXJFcXVpdHkiOjU0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NSwiYmFsYW5jZS1zaGVldDoyMDI0OmFzc2V0cyI6MTQzLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudEFzc2V0cyI6NzIsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNSwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkQXNzZXRzIjo3MSwiYmFsYW5jZS1zaGVldDoyMDI0OnRhbmdpYmxlQXNzZXRzIjo1OCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAsImJhbGFuY2Utc2hlZXQ6MjAyNDptYWNoaW5lcnkiOjI4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c29mdHdhcmUiOjYsImJhbGFuY2Utc2hlZXQ6MjAyNDpsaWFiaWxpdGllcyI6NzksImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZExpYWJpbGl0aWVzIjozOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEsImJhbGFuY2Utc2hlZXQ6MjAyNDpuZXRBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hhcmVob2xkZXJFcXVpdHkiOjYxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBleCI6OCwiYmFsYW5jZS1zaGVldDoyMDI1OmFzc2V0cyI6MTU2LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXNoIjoyNywiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkQXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI1OmJ1aWxkaW5ncyI6MjIsImJhbGFuY2Utc2hlZXQ6MjAyNTptYWNoaW5lcnkiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTppbnRhbmdpYmxlQXNzZXRzIjo5LCJiYWxhbmNlLXNoZWV0OjIwMjU6c29mdHdhcmUiOjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hvcnRUZXJtRGVidCI6MTEsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MCwiYmFsYW5jZS1zaGVldDoyMDI1OmxvbmdUZXJtRGVidCI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpuZXRBc3NldHMiOjczLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBleCI6MTAsImZ1dHVyZS1jYXBleDoyMDI2IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjciOjE1LCJmdXR1cmUtY2FwZXg6MjAyOCI6MTUsImZ1dHVyZS1jYXBleDoyMDI5IjowLCJmdXR1cmUtY2FwZXg6MjAzMCI6MCwiZnV0dXJlLWNhcGV4OjIwMzEiOjAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjEuNjY1MzM0NTM2OTM3NzM0OGUtMTYsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkzMjUzMzA1MDE4NDY5MjcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNzM1OTk0MTgzMTg5MTY2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLjAxOTEzOTQ1NzAyMzcxNzQ0MywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNTUzNDU5OTE0NzYzMDk1LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjAzOTE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNDI1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MCI6MC4xNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjMsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MCI6MC4wMjQxMzk0NTcwMjM3MTc0NDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDoxIjowLjAyNTU1MzQ1OTkxNDc2MzA5NiwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjowLjA0NDE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MSI6MC4wNDc1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjExLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MCI6MC4wODQ5OTk5OTk5OTk5OTk5OSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjEiOjAuMTM1LCJkcml2ZXI6b3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI4NTcxNDI4NTcxNDI4LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjAiOjAuMDg5Mjg1NzE0Mjg1NzE0MjcsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MSI6MC4xMTkyODU3MTQyODU3MTQyNywiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MCI6MC4wNDI2MzE1Nzg5NDczNjgzNiwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjEiOjAuMDY1NTU1NTU1NTU1NTU1NTgsImRyaXZlcjp1c2VmdWxMaWZlIjoxMCwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MCI6NSwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MSI6MjAsImRyaXZlcjppbnZlc3RtZW50IjoyMywiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjEiOjIwMCwiZHJpdmVyOnN1YnNpZHkiOjcuNjYsImRyaXZlci1yYW5nZTpzdWJzaWR5OjAiOjEsImRyaXZlci1yYW5nZTpzdWJzaWR5OjEiOjUwLCJkcml2ZXI6bG9jYWxCZW5jaG1hcmsiOjIzLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MCI6MCwiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjEiOjEwMCwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6dmFsdWUiOjIwLCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6dmFsdWUiOjEzMy41LCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjoyLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOm1heCI6NywidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOnZhbHVlIjo2NSwidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOm1heCI6OTUsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOnZhbHVlIjoyMiwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOnZhbHVlIjo3Ni40NCwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2Fncjp2YWx1ZSI6MjEsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6bWF4IjozNSwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTp2YWx1ZSI6MTguNzgsInRhcmdldDplbXBsb3llZVBheUNhZ3I6dmFsdWUiOjcsInRhcmdldDplbXBsb3llZVBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6dmFsdWUiOjIuODUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MTUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTptYXgiOjI1Mi42OSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOm1heCI6MTM2Ljg0LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOm1heCI6MzMuNDMsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOm1heCI6My43NH0sIm1ldHJpY0dyb3VwQmFzZXMiOnsiY29tcGFueVNhbGVzIjoicmF0ZSIsInByb2plY3RTYWxlcyI6InJhdGUiLCJsYWJvclByb2R1Y3Rpdml0eSI6InJhdGUiLCJlbXBsb3llZVBheSI6InJhdGUifSwiYXBwbGljYXRpb25DYXRlZ29yeSI6ImdlbmVyYWwiLCJhZGp1c3RlZERyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDAzNjgwNTU1NTU1NTU0LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjoxLjE3NDE4NjQ5MTA2NDQ2NmUtMTYsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDE5ODE2Mjg3MTc4ODc3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDQ0ODUzNjMwNjc1MzI3NCwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwNjA5MzM3MDI3ODk4MDQsIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNjA3MzE2NTgzOTIyNDksIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4MDkwNTk1MDQ2MDU2NjMsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MTQ5Mzc3NzI0OTMwNjQ0Niwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjI5Mzg4NzE0MzkwMDY1NzQsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTQwMTg1NzA3MjY1MjYsInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1NTUwNDI3MjU3OTc3Mjg0LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDg4OTQzODQxMjI0NjM1MTEsIm90aGVyUGF5R3Jvd3RoIjowLjAyNDgxMTgzMzI1Mzg2Njc4NywicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wMjYyNDA3NTI0ODU4OTA4OTMsIm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTg3MjM3NjkyMTM2MzM4LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMDMwMDI5OTU0Mzc0MTMyMiwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTMyNjE2NDY1MTYzNjYsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgxOTIzMTY3OTU4MzQ5NiwidXNlZnVsTGlmZSI6MTAsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9fQ==</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebalance proposal samples toward benchmark medians
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -204,7 +204,7 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <v>20.01053154331047</v>
+        <v>15.448906650814621</v>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
@@ -234,7 +234,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <v>126.03000000000003</v>
+        <v>93.21000000000004</v>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
@@ -294,7 +294,7 @@
         </is>
       </c>
       <c r="B11" s="2">
-        <v>67.86048689138576</v>
+        <v>63.89827961836075</v>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
@@ -324,7 +324,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>29.38972537778437</v>
+        <v>22.000324971691864</v>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
@@ -354,7 +354,7 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <v>109.25</v>
+        <v>76.43</v>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
@@ -384,7 +384,7 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <v>32.53247290200707</v>
+        <v>22.016675856213674</v>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
@@ -414,7 +414,7 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <v>28.37999999999999</v>
+        <v>19.73000000000001</v>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
@@ -444,7 +444,7 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <v>7.018093513861001</v>
+        <v>7.019737997987985</v>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B17" s="2">
-        <v>2.3899999999999997</v>
+        <v>2.8600000000000003</v>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <v>370.4960835509137</v>
+        <v>257.5718015665798</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
@@ -1268,13 +1268,13 @@
         <v>173.01</v>
       </c>
       <c r="H3" s="4">
-        <v>206.33999999999997</v>
+        <v>199.42000000000002</v>
       </c>
       <c r="I3" s="4">
-        <v>247.28000000000003</v>
+        <v>229.88</v>
       </c>
       <c r="J3" s="4">
-        <v>299.04</v>
+        <v>266.22</v>
       </c>
     </row>
     <row r="4">
@@ -1304,13 +1304,13 @@
         <v>4.873613384251674</v>
       </c>
       <c r="H4" s="2">
-        <v>19.26478238252123</v>
+        <v>15.265013583029896</v>
       </c>
       <c r="I4" s="2">
-        <v>19.841039061742794</v>
+        <v>15.27429545682477</v>
       </c>
       <c r="J4" s="2">
-        <v>20.931737301844056</v>
+        <v>15.8082477814512</v>
       </c>
     </row>
     <row r="5">
@@ -1338,13 +1338,13 @@
         <v>117.65</v>
       </c>
       <c r="H5" s="2">
-        <v>138.97</v>
+        <v>134.3</v>
       </c>
       <c r="I5" s="2">
-        <v>165.63</v>
+        <v>153.98000000000002</v>
       </c>
       <c r="J5" s="2">
-        <v>199.07</v>
+        <v>177.26</v>
       </c>
     </row>
     <row r="6">
@@ -1406,13 +1406,13 @@
         <v>55.359999999999985</v>
       </c>
       <c r="H7" s="4">
-        <v>67.36999999999998</v>
+        <v>65.12</v>
       </c>
       <c r="I7" s="4">
-        <v>81.65000000000003</v>
+        <v>75.89999999999998</v>
       </c>
       <c r="J7" s="4">
-        <v>99.97000000000003</v>
+        <v>88.96000000000004</v>
       </c>
     </row>
     <row r="8">
@@ -1440,13 +1440,13 @@
         <v>31.998150395930864</v>
       </c>
       <c r="H8" s="2">
-        <v>32.64999515362992</v>
+        <v>32.654698626015445</v>
       </c>
       <c r="I8" s="2">
-        <v>33.019249433840194</v>
+        <v>33.01722637898033</v>
       </c>
       <c r="J8" s="2">
-        <v>33.43031032637775</v>
+        <v>33.415971752685756</v>
       </c>
     </row>
     <row r="9">
@@ -1474,13 +1474,13 @@
         <v>44.19</v>
       </c>
       <c r="H9" s="2">
-        <v>48.459999999999994</v>
+        <v>47.89</v>
       </c>
       <c r="I9" s="2">
-        <v>53.86</v>
+        <v>52.74</v>
       </c>
       <c r="J9" s="2">
-        <v>60.05</v>
+        <v>58.2</v>
       </c>
     </row>
     <row r="10">
@@ -1514,7 +1514,7 @@
         <v>1.19</v>
       </c>
       <c r="J10" s="2">
-        <v>1.23</v>
+        <v>1.24</v>
       </c>
     </row>
     <row r="11">
@@ -1548,7 +1548,7 @@
         <v>1.06</v>
       </c>
       <c r="J11" s="2">
-        <v>1.1</v>
+        <v>1.1099999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -1610,13 +1610,13 @@
         <v>17.06</v>
       </c>
       <c r="H13" s="2">
-        <v>18.16</v>
+        <v>18.18</v>
       </c>
       <c r="I13" s="2">
-        <v>19.83</v>
+        <v>20.07</v>
       </c>
       <c r="J13" s="2">
-        <v>21.66</v>
+        <v>22.16</v>
       </c>
     </row>
     <row r="14">
@@ -1644,13 +1644,13 @@
         <v>16.21</v>
       </c>
       <c r="H14" s="2">
-        <v>17.7</v>
+        <v>17.9</v>
       </c>
       <c r="I14" s="2">
-        <v>19.33</v>
+        <v>19.78</v>
       </c>
       <c r="J14" s="2">
-        <v>21.12</v>
+        <v>21.87</v>
       </c>
     </row>
     <row r="15">
@@ -1678,13 +1678,13 @@
         <v>0.85</v>
       </c>
       <c r="H15" s="2">
-        <v>0.9199999999999999</v>
+        <v>0.9299999999999999</v>
       </c>
       <c r="I15" s="2">
-        <v>1.01</v>
+        <v>1.03</v>
       </c>
       <c r="J15" s="2">
-        <v>1.1099999999999999</v>
+        <v>1.1400000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -1746,13 +1746,13 @@
         <v>0.81</v>
       </c>
       <c r="H17" s="2">
-        <v>0.97</v>
+        <v>0.9299999999999999</v>
       </c>
       <c r="I17" s="2">
-        <v>1.17</v>
+        <v>1.08</v>
       </c>
       <c r="J17" s="2">
-        <v>1.43</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="18">
@@ -1780,13 +1780,13 @@
         <v>11.169999999999984</v>
       </c>
       <c r="H18" s="4">
-        <v>18.909999999999982</v>
+        <v>17.230000000000004</v>
       </c>
       <c r="I18" s="4">
-        <v>27.790000000000035</v>
+        <v>23.159999999999982</v>
       </c>
       <c r="J18" s="4">
-        <v>39.92000000000003</v>
+        <v>30.760000000000048</v>
       </c>
     </row>
     <row r="19">
@@ -1814,13 +1814,13 @@
         <v>6.456274203803239</v>
       </c>
       <c r="H19" s="2">
-        <v>9.16448580013569</v>
+        <v>8.64005616287233</v>
       </c>
       <c r="I19" s="2">
-        <v>11.238272403752843</v>
+        <v>10.074821646076208</v>
       </c>
       <c r="J19" s="2">
-        <v>13.349384697699312</v>
+        <v>11.554353542183174</v>
       </c>
     </row>
     <row r="20">
@@ -1848,13 +1848,13 @@
         <v>11.169999999999984</v>
       </c>
       <c r="H20" s="4">
-        <v>18.909999999999982</v>
+        <v>17.230000000000004</v>
       </c>
       <c r="I20" s="4">
-        <v>27.790000000000035</v>
+        <v>23.159999999999982</v>
       </c>
       <c r="J20" s="4">
-        <v>39.92000000000003</v>
+        <v>30.760000000000048</v>
       </c>
     </row>
     <row r="21">
@@ -1986,13 +1986,13 @@
         <v>17.06</v>
       </c>
       <c r="H23" s="2">
-        <v>18.16</v>
+        <v>18.18</v>
       </c>
       <c r="I23" s="2">
-        <v>19.83</v>
+        <v>20.07</v>
       </c>
       <c r="J23" s="2">
-        <v>21.66</v>
+        <v>22.16</v>
       </c>
     </row>
     <row r="24">
@@ -2026,7 +2026,7 @@
         <v>1.19</v>
       </c>
       <c r="J24" s="2">
-        <v>1.23</v>
+        <v>1.24</v>
       </c>
     </row>
     <row r="25">
@@ -2088,13 +2088,13 @@
         <v>35.13999999999998</v>
       </c>
       <c r="H26" s="4">
-        <v>44.019999999999975</v>
+        <v>42.36</v>
       </c>
       <c r="I26" s="4">
-        <v>54.61000000000003</v>
+        <v>50.21999999999998</v>
       </c>
       <c r="J26" s="4">
-        <v>68.61000000000003</v>
+        <v>59.96000000000004</v>
       </c>
     </row>
     <row r="27">
@@ -2124,13 +2124,13 @@
         <v>5.2410901467505155</v>
       </c>
       <c r="H27" s="2">
-        <v>25.270347182697783</v>
+        <v>20.54638588503137</v>
       </c>
       <c r="I27" s="2">
-        <v>24.057246706042832</v>
+        <v>18.55524079320108</v>
       </c>
       <c r="J27" s="2">
-        <v>25.636330342428117</v>
+        <v>19.394663480685125</v>
       </c>
     </row>
     <row r="28">
@@ -2158,13 +2158,13 @@
         <v>20.310964684122293</v>
       </c>
       <c r="H28" s="2">
-        <v>21.33372104293883</v>
+        <v>21.241600641861396</v>
       </c>
       <c r="I28" s="2">
-        <v>22.08427693303139</v>
+        <v>21.846180615973545</v>
       </c>
       <c r="J28" s="2">
-        <v>22.94341894060996</v>
+        <v>22.522725565321927</v>
       </c>
     </row>
     <row r="29">
@@ -2192,13 +2192,13 @@
         <v>264</v>
       </c>
       <c r="H29" s="2">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="I29" s="2">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="J29" s="2">
-        <v>294</v>
+        <v>300</v>
       </c>
     </row>
     <row r="30">
@@ -2260,13 +2260,13 @@
         <v>0.06462121212121212</v>
       </c>
       <c r="H31" s="2">
-        <v>0.06627737226277372</v>
+        <v>0.0658695652173913</v>
       </c>
       <c r="I31" s="2">
-        <v>0.06982394366197182</v>
+        <v>0.0696875</v>
       </c>
       <c r="J31" s="2">
-        <v>0.0736734693877551</v>
+        <v>0.07386666666666666</v>
       </c>
     </row>
     <row r="32">
@@ -2296,13 +2296,13 @@
         <v>2.0334928229664984</v>
       </c>
       <c r="H32" s="2">
-        <v>2.562873841572455</v>
+        <v>1.9318008053417657</v>
       </c>
       <c r="I32" s="2">
-        <v>5.3511044239002326</v>
+        <v>5.796204620462042</v>
       </c>
       <c r="J32" s="2">
-        <v>5.513188634001254</v>
+        <v>5.997010463378172</v>
       </c>
     </row>
     <row r="33">
@@ -2336,7 +2336,7 @@
         <v>0.238</v>
       </c>
       <c r="J33" s="2">
-        <v>0.246</v>
+        <v>0.248</v>
       </c>
     </row>
     <row r="34">
@@ -2372,7 +2372,7 @@
         <v>3.4782608695652195</v>
       </c>
       <c r="J34" s="2">
-        <v>3.3613445378151363</v>
+        <v>4.201680672268915</v>
       </c>
     </row>
     <row r="35">
@@ -2400,13 +2400,13 @@
         <v>0.13063197026022297</v>
       </c>
       <c r="H35" s="2">
-        <v>0.15777777777777768</v>
+        <v>0.1507473309608541</v>
       </c>
       <c r="I35" s="2">
-        <v>0.18896193771626307</v>
+        <v>0.17139931740614328</v>
       </c>
       <c r="J35" s="2">
-        <v>0.2294648829431439</v>
+        <v>0.19659016393442638</v>
       </c>
     </row>
     <row r="36">
@@ -2434,13 +2434,13 @@
         <v>16.969999999999985</v>
       </c>
       <c r="H36" s="4">
-        <v>24.709999999999983</v>
+        <v>23.030000000000005</v>
       </c>
       <c r="I36" s="4">
-        <v>33.59000000000003</v>
+        <v>28.959999999999983</v>
       </c>
       <c r="J36" s="4">
-        <v>45.72000000000003</v>
+        <v>36.560000000000045</v>
       </c>
     </row>
     <row r="37">
@@ -2468,13 +2468,13 @@
         <v>9.808681579099465</v>
       </c>
       <c r="H37" s="2">
-        <v>11.975380440050396</v>
+        <v>11.548490622806138</v>
       </c>
       <c r="I37" s="2">
-        <v>13.583791653186683</v>
+        <v>12.597877153297365</v>
       </c>
       <c r="J37" s="2">
-        <v>15.288924558587489</v>
+        <v>13.733002779655939</v>
       </c>
     </row>
     <row r="38">
@@ -2504,13 +2504,13 @@
         <v>3.665241295051902</v>
       </c>
       <c r="H38" s="2">
-        <v>45.60989982321748</v>
+        <v>35.71007660577506</v>
       </c>
       <c r="I38" s="2">
-        <v>35.93686766491322</v>
+        <v>25.749023013460604</v>
       </c>
       <c r="J38" s="2">
-        <v>36.11193807680853</v>
+        <v>26.24309392265216</v>
       </c>
     </row>
   </sheetData>
@@ -2672,13 +2672,13 @@
         <v>93.68</v>
       </c>
       <c r="H3" s="4">
-        <v>121.21</v>
+        <v>114.29</v>
       </c>
       <c r="I3" s="4">
-        <v>156.83</v>
+        <v>139.43</v>
       </c>
       <c r="J3" s="4">
-        <v>202.93</v>
+        <v>170.11</v>
       </c>
     </row>
     <row r="4">
@@ -2708,13 +2708,13 @@
         <v>5.400540054005409</v>
       </c>
       <c r="H4" s="2">
-        <v>29.387275832621683</v>
+        <v>22.000426985482502</v>
       </c>
       <c r="I4" s="2">
-        <v>29.387014272749788</v>
+        <v>21.996675124682817</v>
       </c>
       <c r="J4" s="2">
-        <v>29.3948861824906</v>
+        <v>22.00387291113821</v>
       </c>
     </row>
     <row r="5">
@@ -2742,13 +2742,13 @@
         <v>54.14715912375008</v>
       </c>
       <c r="H5" s="2">
-        <v>58.74285160414849</v>
+        <v>57.31120248721292</v>
       </c>
       <c r="I5" s="2">
-        <v>63.42203170494985</v>
+        <v>60.653384374456245</v>
       </c>
       <c r="J5" s="2">
-        <v>67.86048689138576</v>
+        <v>63.89827961836075</v>
       </c>
     </row>
     <row r="6">
@@ -2776,13 +2776,13 @@
         <v>29.980000000000004</v>
       </c>
       <c r="H6" s="4">
-        <v>39.41999999999999</v>
+        <v>37.17</v>
       </c>
       <c r="I6" s="4">
-        <v>51.81000000000002</v>
+        <v>46.06</v>
       </c>
       <c r="J6" s="4">
-        <v>68.1</v>
+        <v>57.09000000000002</v>
       </c>
     </row>
     <row r="7">
@@ -2810,13 +2810,13 @@
         <v>32.00256191289496</v>
       </c>
       <c r="H7" s="2">
-        <v>32.52206913620987</v>
+        <v>32.522530405109805</v>
       </c>
       <c r="I7" s="2">
-        <v>33.0357712172416</v>
+        <v>33.034497597360684</v>
       </c>
       <c r="J7" s="2">
-        <v>33.55836988123983</v>
+        <v>33.56063723473048</v>
       </c>
     </row>
     <row r="8">
@@ -2844,13 +2844,13 @@
         <v>6.630000000000006</v>
       </c>
       <c r="H8" s="4">
-        <v>12.929999999999987</v>
+        <v>11.260000000000002</v>
       </c>
       <c r="I8" s="4">
-        <v>21.150000000000016</v>
+        <v>16.54</v>
       </c>
       <c r="J8" s="4">
-        <v>32.54</v>
+        <v>23.420000000000023</v>
       </c>
     </row>
     <row r="9">
@@ -2878,13 +2878,13 @@
         <v>7.077284372331347</v>
       </c>
       <c r="H9" s="2">
-        <v>10.667436680141892</v>
+        <v>9.85213054510456</v>
       </c>
       <c r="I9" s="2">
-        <v>13.485940190014675</v>
+        <v>11.862583375170335</v>
       </c>
       <c r="J9" s="2">
-        <v>16.03508599024294</v>
+        <v>13.767562165657528</v>
       </c>
     </row>
     <row r="10">
@@ -2912,13 +2912,13 @@
         <v>7.47</v>
       </c>
       <c r="H10" s="2">
-        <v>7.89</v>
+        <v>7.9</v>
       </c>
       <c r="I10" s="2">
-        <v>8.82</v>
+        <v>9.04</v>
       </c>
       <c r="J10" s="2">
-        <v>9.86</v>
+        <v>10.33</v>
       </c>
     </row>
     <row r="11">
@@ -3014,13 +3014,13 @@
         <v>18.870000000000005</v>
       </c>
       <c r="H13" s="4">
-        <v>25.619999999999987</v>
+        <v>23.960000000000004</v>
       </c>
       <c r="I13" s="4">
-        <v>34.79000000000001</v>
+        <v>30.4</v>
       </c>
       <c r="J13" s="4">
-        <v>47.24999999999999</v>
+        <v>38.600000000000016</v>
       </c>
     </row>
     <row r="14">
@@ -3050,13 +3050,13 @@
         <v>6.190208216094595</v>
       </c>
       <c r="H14" s="2">
-        <v>35.77106518282977</v>
+        <v>26.974032856385797</v>
       </c>
       <c r="I14" s="2">
-        <v>35.792349726776074</v>
+        <v>26.878130217028364</v>
       </c>
       <c r="J14" s="2">
-        <v>35.81488933601602</v>
+        <v>26.973684210526372</v>
       </c>
     </row>
     <row r="15">
@@ -3084,13 +3084,13 @@
         <v>117</v>
       </c>
       <c r="H15" s="2">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I15" s="2">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="J15" s="2">
-        <v>126</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16">
@@ -3152,13 +3152,13 @@
         <v>0.06384615384615384</v>
       </c>
       <c r="H17" s="2">
-        <v>0.06575</v>
+        <v>0.06475409836065574</v>
       </c>
       <c r="I17" s="2">
-        <v>0.07170731707317074</v>
+        <v>0.07118110236220472</v>
       </c>
       <c r="J17" s="2">
-        <v>0.07825396825396826</v>
+        <v>0.07825757575757576</v>
       </c>
     </row>
     <row r="18">
@@ -3188,13 +3188,13 @@
         <v>2.1170472179117716</v>
       </c>
       <c r="H18" s="2">
-        <v>2.9819277108433795</v>
+        <v>1.4220817697017551</v>
       </c>
       <c r="I18" s="2">
-        <v>9.060558286191235</v>
+        <v>9.925246685936395</v>
       </c>
       <c r="J18" s="2">
-        <v>9.129683619479522</v>
+        <v>9.941505765620828</v>
       </c>
     </row>
     <row r="19">
@@ -3292,13 +3292,13 @@
         <v>0.1585714285714286</v>
       </c>
       <c r="H21" s="2">
-        <v>0.20999999999999988</v>
+        <v>0.19322580645161294</v>
       </c>
       <c r="I21" s="2">
-        <v>0.2783200000000001</v>
+        <v>0.23565891472868217</v>
       </c>
       <c r="J21" s="2">
-        <v>0.36914062499999994</v>
+        <v>0.28805970149253746</v>
       </c>
     </row>
     <row r="22">
@@ -3626,17 +3626,17 @@
       </c>
       <c r="J4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 19.26 % / 補助 29.39 % / 他 7.31 %</t>
+          <t xml:space="preserve">全社 15.27 % / 補助 22 % / 他 7.31 %</t>
         </is>
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 19.84 % / 補助 29.39 % / 他 6.25 %</t>
+          <t xml:space="preserve">全社 15.27 % / 補助 22 % / 他 6.25 %</t>
         </is>
       </c>
       <c r="L4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 20.93 % / 補助 29.39 % / 他 6.26 %</t>
+          <t xml:space="preserve">全社 15.81 % / 補助 22 % / 他 6.26 %</t>
         </is>
       </c>
     </row>
@@ -3693,12 +3693,12 @@
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 66.98 % / 補助 66.96 % / 他 67.01 %</t>
+          <t xml:space="preserve">全社 66.98 % / 補助 66.97 % / 他 67.01 %</t>
         </is>
       </c>
       <c r="L5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 66.57 % / 補助 66.44 % / 他 66.84 %</t>
+          <t xml:space="preserve">全社 66.58 % / 補助 66.44 % / 他 66.84 %</t>
         </is>
       </c>
     </row>
@@ -3755,12 +3755,12 @@
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 33.02 % / 補助 33.04 % / 他 32.99 %</t>
+          <t xml:space="preserve">全社 33.02 % / 補助 33.03 % / 他 32.99 %</t>
         </is>
       </c>
       <c r="L6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 33.43 % / 補助 33.56 % / 他 33.16 %</t>
+          <t xml:space="preserve">全社 33.42 % / 補助 33.56 % / 他 33.16 %</t>
         </is>
       </c>
     </row>
@@ -3812,17 +3812,17 @@
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 23.49 % / 補助 21.85 % / 他 25.81 %</t>
+          <t xml:space="preserve">全社 24.01 % / 補助 22.67 % / 他 25.82 %</t>
         </is>
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 21.78 % / 補助 19.55 % / 他 25.65 %</t>
+          <t xml:space="preserve">全社 22.94 % / 補助 21.17 % / 他 25.67 %</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 20.08 % / 補助 17.52 % / 他 25.48 %</t>
+          <t xml:space="preserve">全社 21.86 % / 補助 19.79 % / 他 25.52 %</t>
         </is>
       </c>
     </row>
@@ -3874,17 +3874,17 @@
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.16 % / 補助 10.67 % / 他 7.02 %</t>
+          <t xml:space="preserve">全社 8.64 % / 補助 9.85 % / 他 7.01 %</t>
         </is>
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.24 % / 補助 13.49 % / 他 7.34 %</t>
+          <t xml:space="preserve">全社 10.07 % / 補助 11.86 % / 他 7.32 %</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.35 % / 補助 16.04 % / 他 7.68 %</t>
+          <t xml:space="preserve">全社 11.55 % / 補助 13.77 % / 他 7.64 %</t>
         </is>
       </c>
     </row>
@@ -3936,17 +3936,17 @@
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.98 % / 補助 14.21 % / 他 8.79 %</t>
+          <t xml:space="preserve">全社 11.55 % / 補助 13.61 % / 他 8.77 %</t>
         </is>
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.58 % / 補助 16.23 % / 他 9 %</t>
+          <t xml:space="preserve">全社 12.6 % / 補助 14.95 % / 他 8.98 %</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.29 % / 補助 18.15 % / 他 9.24 %</t>
+          <t xml:space="preserve">全社 13.73 % / 補助 16.3 % / 他 9.2 %</t>
         </is>
       </c>
     </row>
@@ -3998,17 +3998,17 @@
       </c>
       <c r="J10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.51 % / 補助 11.76 % / 他 11.15 %</t>
+          <t xml:space="preserve">全社 11.63 % / 補助 12 % / 他 11.15 %</t>
         </is>
       </c>
       <c r="K10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.02 % / 補助 11.03 % / 他 10.99 %</t>
+          <t xml:space="preserve">全社 11.3 % / 補助 11.5 % / 他 10.99 %</t>
         </is>
       </c>
       <c r="L10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.47 % / 補助 10.3 % / 他 10.82 %</t>
+          <t xml:space="preserve">全社 10.93 % / 補助 11 % / 他 10.82 %</t>
         </is>
       </c>
     </row>
@@ -4122,17 +4122,17 @@
       </c>
       <c r="J12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.8 % / 補助 6.51 % / 他 12.06 %</t>
+          <t xml:space="preserve">全社 9.12 % / 補助 6.91 % / 他 12.08 %</t>
         </is>
       </c>
       <c r="K12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.02 % / 補助 5.62 % / 他 12.17 %</t>
+          <t xml:space="preserve">全社 8.73 % / 補助 6.48 % / 他 12.19 %</t>
         </is>
       </c>
       <c r="L12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.24 % / 補助 4.86 % / 他 12.28 %</t>
+          <t xml:space="preserve">全社 8.32 % / 補助 6.07 % / 他 12.31 %</t>
         </is>
       </c>
     </row>
@@ -4184,17 +4184,17 @@
       </c>
       <c r="J13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.56 % / 補助 0.41 % / 他 0.76 %</t>
+          <t xml:space="preserve">全社 0.58 % / 補助 0.44 % / 他 0.76 %</t>
         </is>
       </c>
       <c r="K13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.48 % / 補助 0.33 % / 他 0.74 %</t>
+          <t xml:space="preserve">全社 0.52 % / 補助 0.37 % / 他 0.74 %</t>
         </is>
       </c>
       <c r="L13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.41 % / 補助 0.27 % / 他 0.71 %</t>
+          <t xml:space="preserve">全社 0.47 % / 補助 0.32 % / 他 0.72 %</t>
         </is>
       </c>
     </row>
@@ -4246,17 +4246,17 @@
       </c>
       <c r="J14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.36 % / 補助 6.92 % / 他 12.83 %</t>
+          <t xml:space="preserve">全社 9.69 % / 補助 7.35 % / 他 12.84 %</t>
         </is>
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.5 % / 補助 5.96 % / 他 12.91 %</t>
+          <t xml:space="preserve">全社 9.25 % / 補助 6.86 % / 他 12.94 %</t>
         </is>
       </c>
       <c r="L14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.65 % / 補助 5.13 % / 他 12.99 %</t>
+          <t xml:space="preserve">全社 8.79 % / 補助 6.4 % / 他 13.03 %</t>
         </is>
       </c>
     </row>
@@ -4308,12 +4308,12 @@
       </c>
       <c r="J15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.066 億円/人 / 補助 0.066 億円/人 / 他 0.067 億円/人</t>
+          <t xml:space="preserve">全社 0.066 億円/人 / 補助 0.065 億円/人 / 他 0.067 億円/人</t>
         </is>
       </c>
       <c r="K15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.07 億円/人 / 補助 0.072 億円/人 / 他 0.068 億円/人</t>
+          <t xml:space="preserve">全社 0.07 億円/人 / 補助 0.071 億円/人 / 他 0.069 億円/人</t>
         </is>
       </c>
       <c r="L15" s="0" t="inlineStr">
@@ -4380,7 +4380,7 @@
       </c>
       <c r="L16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.246 億円/人 / 補助 0.275 億円/人 / 他 0.227 億円/人</t>
+          <t xml:space="preserve">全社 0.248 億円/人 / 補助 0.275 億円/人 / 他 0.23 億円/人</t>
         </is>
       </c>
     </row>
@@ -4432,17 +4432,17 @@
       </c>
       <c r="J17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.56 % / 補助 2.98 % / 他 2.22 %</t>
+          <t xml:space="preserve">全社 1.93 % / 補助 1.42 % / 他 2.32 %</t>
         </is>
       </c>
       <c r="K17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5.35 % / 補助 9.06 % / 他 2.54 %</t>
+          <t xml:space="preserve">全社 5.8 % / 補助 9.93 % / 他 2.63 %</t>
         </is>
       </c>
       <c r="L17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5.51 % / 補助 9.13 % / 他 2.71 %</t>
+          <t xml:space="preserve">全社 6 % / 補助 9.94 % / 他 2.78 %</t>
         </is>
       </c>
     </row>
@@ -4494,17 +4494,17 @@
       </c>
       <c r="J18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 43.87 % / 補助 32.75 % / 他 59.35 %</t>
+          <t xml:space="preserve">全社 45.63 % / 補助 35.06 % / 他 59.4 %</t>
         </is>
       </c>
       <c r="K18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 38.49 % / 補助 26.85 % / 他 58.93 %</t>
+          <t xml:space="preserve">全社 42.33 % / 補助 31.45 % / 他 59.03 %</t>
         </is>
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 33.36 % / 補助 22.03 % / 他 58.43 %</t>
+          <t xml:space="preserve">全社 39.03 % / 補助 28.19 % / 他 58.61 %</t>
         </is>
       </c>
     </row>
@@ -4618,17 +4618,17 @@
       </c>
       <c r="J20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.753 億円/人 / 補助 1.01 億円/人 / 他 0.553 億円/人</t>
+          <t xml:space="preserve">全社 0.723 億円/人 / 補助 0.937 億円/人 / 他 0.553 億円/人</t>
         </is>
       </c>
       <c r="K20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.871 億円/人 / 補助 1.275 億円/人 / 他 0.562 億円/人</t>
+          <t xml:space="preserve">全社 0.798 億円/人 / 補助 1.098 億円/人 / 他 0.562 億円/人</t>
         </is>
       </c>
       <c r="L20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.017 億円/人 / 補助 1.611 億円/人 / 他 0.572 億円/人</t>
+          <t xml:space="preserve">全社 0.887 億円/人 / 補助 1.289 億円/人 / 他 0.572 億円/人</t>
         </is>
       </c>
     </row>
@@ -4680,17 +4680,17 @@
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.069 億円/人 / 補助 0.108 億円/人 / 他 0.039 億円/人</t>
+          <t xml:space="preserve">全社 0.062 億円/人 / 補助 0.092 億円/人 / 他 0.039 億円/人</t>
         </is>
       </c>
       <c r="K21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.098 億円/人 / 補助 0.172 億円/人 / 他 0.041 億円/人</t>
+          <t xml:space="preserve">全社 0.08 億円/人 / 補助 0.13 億円/人 / 他 0.041 億円/人</t>
         </is>
       </c>
       <c r="L21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.136 億円/人 / 補助 0.258 億円/人 / 他 0.044 億円/人</t>
+          <t xml:space="preserve">全社 0.103 億円/人 / 補助 0.177 億円/人 / 他 0.044 億円/人</t>
         </is>
       </c>
     </row>
@@ -4742,17 +4742,17 @@
       </c>
       <c r="J22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.158 億円/人 / 補助 0.21 億円/人 / 他 0.117 億円/人</t>
+          <t xml:space="preserve">全社 0.151 億円/人 / 補助 0.193 億円/人 / 他 0.117 億円/人</t>
         </is>
       </c>
       <c r="K22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.189 億円/人 / 補助 0.278 億円/人 / 他 0.121 億円/人</t>
+          <t xml:space="preserve">全社 0.171 億円/人 / 補助 0.236 億円/人 / 他 0.121 億円/人</t>
         </is>
       </c>
       <c r="L22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.229 億円/人 / 補助 0.369 億円/人 / 他 0.125 億円/人</t>
+          <t xml:space="preserve">全社 0.197 億円/人 / 補助 0.288 億円/人 / 他 0.125 億円/人</t>
         </is>
       </c>
     </row>
@@ -4804,17 +4804,17 @@
       </c>
       <c r="J23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.79 % / 補助 2.56 % / 他 4.76 %</t>
+          <t xml:space="preserve">全社 4.55 % / 補助 4.27 % / 他 4.76 %</t>
         </is>
       </c>
       <c r="K23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.65 % / 補助 2.5 % / 他 4.55 %</t>
+          <t xml:space="preserve">全社 4.35 % / 補助 4.1 % / 他 4.55 %</t>
         </is>
       </c>
       <c r="L23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.52 % / 補助 2.44 % / 他 4.35 %</t>
+          <t xml:space="preserve">全社 4.17 % / 補助 3.94 % / 他 4.35 %</t>
         </is>
       </c>
     </row>
@@ -4866,17 +4866,17 @@
       </c>
       <c r="J24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.48 pt / 補助 26.82 pt / 他 2.55 pt</t>
+          <t xml:space="preserve">全社 10.72 pt / 補助 17.73 pt / 他 2.55 pt</t>
         </is>
       </c>
       <c r="K24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 16.19 pt / 補助 26.89 pt / 他 1.7 pt</t>
+          <t xml:space="preserve">全社 10.93 pt / 補助 17.9 pt / 他 1.7 pt</t>
         </is>
       </c>
       <c r="L24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 17.41 pt / 補助 26.96 pt / 他 1.91 pt</t>
+          <t xml:space="preserve">全社 11.64 pt / 補助 18.07 pt / 他 1.91 pt</t>
         </is>
       </c>
     </row>
@@ -4990,17 +4990,17 @@
       </c>
       <c r="J26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.81 % / 補助 3.55 % / 他 1.76 %</t>
+          <t xml:space="preserve">全社 2.91 % / 補助 3.76 % / 他 1.76 %</t>
         </is>
       </c>
       <c r="K26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.35 % / 補助 2.74 % / 他 1.66 %</t>
+          <t xml:space="preserve">全社 2.52 % / 補助 3.08 % / 他 1.66 %</t>
         </is>
       </c>
       <c r="L26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.94 % / 補助 2.12 % / 他 1.56 %</t>
+          <t xml:space="preserve">全社 2.18 % / 補助 2.53 % / 他 1.56 %</t>
         </is>
       </c>
     </row>
@@ -5176,17 +5176,17 @@
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.26 倍 / 補助 4.01 倍 / 他 4.99 倍</t>
+          <t xml:space="preserve">全社 3.97 倍 / 補助 3.62 倍 / 他 4.98 倍</t>
         </is>
       </c>
       <c r="K29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5.79 倍 / 補助 5.92 倍 / 他 5.43 倍</t>
+          <t xml:space="preserve">全社 4.99 倍 / 補助 4.85 倍 / 他 5.41 倍</t>
         </is>
       </c>
       <c r="L29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.88 倍 / 補助 8.57 倍 / 他 5.92 倍</t>
+          <t xml:space="preserve">全社 6.3 倍 / 補助 6.45 倍 / 他 5.89 倍</t>
         </is>
       </c>
     </row>
@@ -5362,17 +5362,17 @@
       </c>
       <c r="J32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 58.74 %</t>
+          <t xml:space="preserve">構成比 57.31 %</t>
         </is>
       </c>
       <c r="K32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 63.42 %</t>
+          <t xml:space="preserve">構成比 60.65 %</t>
         </is>
       </c>
       <c r="L32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 67.86 %</t>
+          <t xml:space="preserve">構成比 63.9 %</t>
         </is>
       </c>
     </row>
@@ -5424,17 +5424,17 @@
       </c>
       <c r="J33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 29.39 % / 他 7.31 %</t>
+          <t xml:space="preserve">補助 22 % / 他 7.31 %</t>
         </is>
       </c>
       <c r="K33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 29.39 % / 他 6.25 %</t>
+          <t xml:space="preserve">補助 22 % / 他 6.25 %</t>
         </is>
       </c>
       <c r="L33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 29.39 % / 他 6.26 %</t>
+          <t xml:space="preserve">補助 22 % / 他 6.26 %</t>
         </is>
       </c>
     </row>
@@ -5491,7 +5491,7 @@
       </c>
       <c r="K34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -0.05 pt</t>
+          <t xml:space="preserve">差 -0.04 pt</t>
         </is>
       </c>
       <c r="L34" s="0" t="inlineStr">
@@ -5548,17 +5548,17 @@
       </c>
       <c r="J35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 3.64 pt</t>
+          <t xml:space="preserve">差 2.84 pt</t>
         </is>
       </c>
       <c r="K35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 6.14 pt</t>
+          <t xml:space="preserve">差 4.54 pt</t>
         </is>
       </c>
       <c r="L35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 8.36 pt</t>
+          <t xml:space="preserve">差 6.13 pt</t>
         </is>
       </c>
     </row>
@@ -5610,17 +5610,17 @@
       </c>
       <c r="J36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.01 億円/人 / 他 0.553 億円/人</t>
+          <t xml:space="preserve">補助 0.937 億円/人 / 他 0.553 億円/人</t>
         </is>
       </c>
       <c r="K36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.275 億円/人 / 他 0.562 億円/人</t>
+          <t xml:space="preserve">補助 1.098 億円/人 / 他 0.562 億円/人</t>
         </is>
       </c>
       <c r="L36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.611 億円/人 / 他 0.572 億円/人</t>
+          <t xml:space="preserve">補助 1.289 億円/人 / 他 0.572 億円/人</t>
         </is>
       </c>
     </row>
@@ -5672,12 +5672,12 @@
       </c>
       <c r="J37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.066 億円/人 / 他 0.067 億円/人</t>
+          <t xml:space="preserve">補助 0.065 億円/人 / 他 0.067 億円/人</t>
         </is>
       </c>
       <c r="K37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.072 億円/人 / 他 0.068 億円/人</t>
+          <t xml:space="preserve">補助 0.071 億円/人 / 他 0.069 億円/人</t>
         </is>
       </c>
       <c r="L37" s="0" t="inlineStr">
@@ -5734,17 +5734,17 @@
       </c>
       <c r="J38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 81.4 %</t>
+          <t xml:space="preserve">寄与率 76.4 %</t>
         </is>
       </c>
       <c r="K38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 92.57 %</t>
+          <t xml:space="preserve">寄与率 89.04 %</t>
         </is>
       </c>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 93.9 %</t>
+          <t xml:space="preserve">寄与率 90.53 %</t>
         </is>
       </c>
     </row>
@@ -9450,7 +9450,7 @@
         </is>
       </c>
       <c r="B204" s="2">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C204" s="0" t="inlineStr">
         <is>
@@ -9480,7 +9480,7 @@
         </is>
       </c>
       <c r="B206" s="2">
-        <v>133.5</v>
+        <v>82.4</v>
       </c>
       <c r="C206" s="0" t="inlineStr">
         <is>
@@ -9735,7 +9735,7 @@
         </is>
       </c>
       <c r="B223" s="2">
-        <v>76.44</v>
+        <v>74.8</v>
       </c>
       <c r="C223" s="0" t="inlineStr">
         <is>
@@ -9765,7 +9765,7 @@
         </is>
       </c>
       <c r="B225" s="2">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C225" s="0" t="inlineStr">
         <is>
@@ -9855,7 +9855,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4fX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjU5LCJvZmZpY2VyUGF5IjowLjM4LCJkZXByZWNpYXRpb24iOjEuOSwib3RoZXJTZ2EiOjkuNSwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NS4zMSwiZW1wbG95ZWVCb251cyI6MC4yOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNCwib2ZmaWNlckJvbnVzIjowLjA0LCJjb2dzRGVwcmVjaWF0aW9uIjowLjQ3LCJzZ2FEZXByZWNpYXRpb24iOjEuNDMsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMzh9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNTQsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3LjE2LCJlbXBsb3llZUJvbnVzIjowLjM4LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjUyLCJvZmZpY2VyQm9udXMiOjAuMDYsImNvZ3NEZXByZWNpYXRpb24iOjAuMjksInNnYURlcHJlY2lhdGlvbiI6MS4xNSwicmVzZWFyY2hEZXZlbG9wbWVudCI6MC4yOX19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6NiwiZW1wbG95ZWVTYWxhcnkiOjUuNywiZW1wbG95ZWVCb251cyI6MC4zLCJvZmZpY2VyUGF5IjowLjQsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzYsIm9mZmljZXJCb251cyI6MC4wNCwiZGVwcmVjaWF0aW9uIjoyLCJjb2dzRGVwcmVjaWF0aW9uIjowLjUsInNnYURlcHJlY2lhdGlvbiI6MS41LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjQsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsImVtcGxveWVlU2FsYXJ5Ijo3LjYsImVtcGxveWVlQm9udXMiOjAuNCwib2ZmaWNlclBheSI6MC42LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjU0LCJvZmZpY2VyQm9udXMiOjAuMDYsImRlcHJlY2lhdGlvbiI6MS41LCJjb2dzRGVwcmVjaWF0aW9uIjowLjMsInNnYURlcHJlY2lhdGlvbiI6MS4yLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjMsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMSwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI4NTcxNDI4NTcxNDI4LCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwidXNlZnVsTGlmZSI6MTAsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwxLjY2NTMzNDUzNjkzNzczNDhlLTE2XSwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MzI1MzMwNTAxODQ2OTI3LDAuMDIwNzM1OTk0MTgzMTg5MTY2XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDBdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNDA3NjA4Njk1NjUyMTcxODQsMC4wNDQzODQwNTc5NzEwMTQ1Ml0sIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAwMDEzNDU3NTU2OTM1ODE5NzM3XSwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOlswLjAxOTEzOTQ1NzAyMzcxNzQ0MywwLjAyMDU1MzQ1OTkxNDc2MzA5NV0sIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wMzkxNjY2NjY2NjY2NjY2OCwwLjA0MjUwMDAwMDAwMDAwMDA5XSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RTYWxlc0dyb3d0aCI6WzAuMTUsMC4zXSwib3RoZXJTYWxlc0dyb3d0aCI6WzAuMDYwNzYwODY5NTY1MjE3MTksMC4wNjQzODQwNTc5NzEwMTQ1M10sInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOlswLDAuMDNdLCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6WzAuMDA1LDAuMDA1MTM0NTc1NTY5MzU4MTk3NV0sInByb2plY3RQYXlHcm93dGgiOlswLjA1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMC4wMjQxMzk0NTcwMjM3MTc0NDQsMC4wMjU1NTM0NTk5MTQ3NjMwOTZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGgiOlswLjA0NDE2NjY2NjY2NjY2NjY4LDAuMDQ3NTAwMDAwMDAwMDAwMDldLCJwcm9qZWN0U2dhUmF0ZUVuZCI6WzAuMDg0OTk5OTk5OTk5OTk5OTksMC4xMzVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA4OTI4NTcxNDI4NTcxNDI3LDAuMTE5Mjg1NzE0Mjg1NzE0MjddLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAuMDQyNjMxNTc4OTQ3MzY4MzYsMC4wNjU1NTU1NTU1NTU1NTU1OF0sInVzZWZ1bExpZmUiOls1LDIwXSwiaW52ZXN0bWVudCI6WzE1LDIwMF0sInN1YnNpZHkiOlsxLDUwXSwibG9jYWxCZW5jaG1hcmsiOlswLDEwMF19LCJ0YXJnZXRzIjp7ImNvbXBhbnlTYWxlc0NhZ3IiOnsidmFsdWUiOjIwLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjEzMy41LCJtYXgiOjI1Mi42OSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlQYXlTY2hlZHVsZSI6eyJ2YWx1ZSI6MiwibWF4Ijo3LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzU2hhcmUiOnsidmFsdWUiOjY1LCJtYXgiOjk1LCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjIsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6NzYuNDQsIm1heCI6MTM2Ljg0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MTguNzgsIm1heCI6MzMuNDMsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUNhZ3IiOnsidmFsdWUiOjcsIm1heCI6MTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUluY3JlYXNlIjp7InZhbHVlIjoyLjg1LCJtYXgiOjMuNzQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJpbnZlc3RtZW50U2FsZXNSYXRpbyI6eyJ2YWx1ZSI6MTUsIm1heCI6NzAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvIjp7InZhbHVlIjoyMTMsIm1heCI6MzUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibG9jYWxCZW5jaG1hcmsiOnsidmFsdWUiOjIzLCJtYXgiOjQwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUNhZ3IiOnsidmFsdWUiOjYsIm1heCI6MTAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnsiMjAyOTpvdGhlcjpzYWxlcyI6ODUuMTMsIjIwMjk6cHJvamVjdDo3LTgiOjcuODl9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2LjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mi43NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTQiOjAuNzMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi03IjozMi42NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTkiOjAuODIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMCI6MC4wOSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEyIjoxMS42NywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEzIjowLjYyLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTQiOjIuNDUsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNSI6MC42NCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEiOjcyLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNCI6MjMuMDQsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny02Ijo2Ljc4LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOCI6NS4xOSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTkiOjAuMzYsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMCI6MS44LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTMiOjkwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xIjoxNDMuMiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTMiOjk3LjM4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNCI6MC43NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTciOjM0LjUyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItOSI6MC44NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMiI6MTIuNDcsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMyI6MC42NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjoyLjU4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTUiOjAuNjcsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xIjo3NiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0LjMyLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNiI6Ny4wNCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTgiOjUuNTksImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTAiOjEuOSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6MC44LCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTkiOjAuOSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjowLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6Mi43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTUiOjAuNywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNCI6MjUuNiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTYiOjcuMywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTgiOjYsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny05IjowLjQsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xMCI6MiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudEFzc2V0cyI6NjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXNoIjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NSwiYmFsYW5jZS1zaGVldDoyMDIzOnRhbmdpYmxlQXNzZXRzIjo1MywiYmFsYW5jZS1zaGVldDoyMDIzOmJ1aWxkaW5ncyI6MTksImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzppbnRhbmdpYmxlQXNzZXRzIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUsImJhbGFuY2Utc2hlZXQ6MjAyMzpsaWFiaWxpdGllcyI6NzUsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50TGlhYmlsaXRpZXMiOjM5LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZExpYWJpbGl0aWVzIjozNiwiYmFsYW5jZS1zaGVldDoyMDIzOmxvbmdUZXJtRGVidCI6MjksImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hhcmVob2xkZXJFcXVpdHkiOjU0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NSwiYmFsYW5jZS1zaGVldDoyMDI0OmFzc2V0cyI6MTQzLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudEFzc2V0cyI6NzIsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNSwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkQXNzZXRzIjo3MSwiYmFsYW5jZS1zaGVldDoyMDI0OnRhbmdpYmxlQXNzZXRzIjo1OCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAsImJhbGFuY2Utc2hlZXQ6MjAyNDptYWNoaW5lcnkiOjI4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c29mdHdhcmUiOjYsImJhbGFuY2Utc2hlZXQ6MjAyNDpsaWFiaWxpdGllcyI6NzksImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZExpYWJpbGl0aWVzIjozOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEsImJhbGFuY2Utc2hlZXQ6MjAyNDpuZXRBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hhcmVob2xkZXJFcXVpdHkiOjYxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBleCI6OCwiYmFsYW5jZS1zaGVldDoyMDI1OmFzc2V0cyI6MTU2LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXNoIjoyNywiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkQXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI1OmJ1aWxkaW5ncyI6MjIsImJhbGFuY2Utc2hlZXQ6MjAyNTptYWNoaW5lcnkiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTppbnRhbmdpYmxlQXNzZXRzIjo5LCJiYWxhbmNlLXNoZWV0OjIwMjU6c29mdHdhcmUiOjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hvcnRUZXJtRGVidCI6MTEsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MCwiYmFsYW5jZS1zaGVldDoyMDI1OmxvbmdUZXJtRGVidCI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpuZXRBc3NldHMiOjczLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBleCI6MTAsImZ1dHVyZS1jYXBleDoyMDI2IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjciOjE1LCJmdXR1cmUtY2FwZXg6MjAyOCI6MTUsImZ1dHVyZS1jYXBleDoyMDI5IjowLCJmdXR1cmUtY2FwZXg6MjAzMCI6MCwiZnV0dXJlLWNhcGV4OjIwMzEiOjAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjEuNjY1MzM0NTM2OTM3NzM0OGUtMTYsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkzMjUzMzA1MDE4NDY5MjcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNzM1OTk0MTgzMTg5MTY2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLjAxOTEzOTQ1NzAyMzcxNzQ0MywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNTUzNDU5OTE0NzYzMDk1LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjAzOTE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNDI1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MCI6MC4xNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjMsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MCI6MC4wMjQxMzk0NTcwMjM3MTc0NDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDoxIjowLjAyNTU1MzQ1OTkxNDc2MzA5NiwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjowLjA0NDE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MSI6MC4wNDc1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjExLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MCI6MC4wODQ5OTk5OTk5OTk5OTk5OSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjEiOjAuMTM1LCJkcml2ZXI6b3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI4NTcxNDI4NTcxNDI4LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjAiOjAuMDg5Mjg1NzE0Mjg1NzE0MjcsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MSI6MC4xMTkyODU3MTQyODU3MTQyNywiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MCI6MC4wNDI2MzE1Nzg5NDczNjgzNiwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjEiOjAuMDY1NTU1NTU1NTU1NTU1NTgsImRyaXZlcjp1c2VmdWxMaWZlIjoxMCwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MCI6NSwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MSI6MjAsImRyaXZlcjppbnZlc3RtZW50IjoyMywiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjEiOjIwMCwiZHJpdmVyOnN1YnNpZHkiOjcuNjYsImRyaXZlci1yYW5nZTpzdWJzaWR5OjAiOjEsImRyaXZlci1yYW5nZTpzdWJzaWR5OjEiOjUwLCJkcml2ZXI6bG9jYWxCZW5jaG1hcmsiOjIzLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MCI6MCwiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjEiOjEwMCwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6dmFsdWUiOjIwLCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6dmFsdWUiOjEzMy41LCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjoyLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOm1heCI6NywidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOnZhbHVlIjo2NSwidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOm1heCI6OTUsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOnZhbHVlIjoyMiwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOnZhbHVlIjo3Ni40NCwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2Fncjp2YWx1ZSI6MjEsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6bWF4IjozNSwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTp2YWx1ZSI6MTguNzgsInRhcmdldDplbXBsb3llZVBheUNhZ3I6dmFsdWUiOjcsInRhcmdldDplbXBsb3llZVBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6dmFsdWUiOjIuODUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MTUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTptYXgiOjI1Mi42OSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOm1heCI6MTM2Ljg0LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOm1heCI6MzMuNDMsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOm1heCI6My43NH0sIm1ldHJpY0dyb3VwQmFzZXMiOnsiY29tcGFueVNhbGVzIjoicmF0ZSIsInByb2plY3RTYWxlcyI6InJhdGUiLCJsYWJvclByb2R1Y3Rpdml0eSI6InJhdGUiLCJlbXBsb3llZVBheSI6InJhdGUifSwiYXBwbGljYXRpb25DYXRlZ29yeSI6ImdlbmVyYWwiLCJhZGp1c3RlZERyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDAzNjgwNTU1NTU1NTU0LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjoxLjE3NDE4NjQ5MTA2NDQ2NmUtMTYsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDE5ODE2Mjg3MTc4ODc3LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDQ0ODUzNjMwNjc1MzI3NCwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwNjA5MzM3MDI3ODk4MDQsIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNjA3MzE2NTgzOTIyNDksIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4MDkwNTk1MDQ2MDU2NjMsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MTQ5Mzc3NzI0OTMwNjQ0Niwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjI5Mzg4NzE0MzkwMDY1NzQsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTQwMTg1NzA3MjY1MjYsInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1NTUwNDI3MjU3OTc3Mjg0LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDg4OTQzODQxMjI0NjM1MTEsIm90aGVyUGF5R3Jvd3RoIjowLjAyNDgxMTgzMzI1Mzg2Njc4NywicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wMjYyNDA3NTI0ODU4OTA4OTMsIm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTg3MjM3NjkyMTM2MzM4LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMDMwMDI5OTU0Mzc0MTMyMiwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTMyNjE2NDY1MTYzNjYsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgxOTIzMTY3OTU4MzQ5NiwidXNlZnVsTGlmZSI6MTAsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9fQ==</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4fX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjU5LCJvZmZpY2VyUGF5IjowLjM4LCJkZXByZWNpYXRpb24iOjEuOSwib3RoZXJTZ2EiOjkuNSwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NS4zMSwiZW1wbG95ZWVCb251cyI6MC4yOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNCwib2ZmaWNlckJvbnVzIjowLjA0LCJjb2dzRGVwcmVjaWF0aW9uIjowLjQ3LCJzZ2FEZXByZWNpYXRpb24iOjEuNDMsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMzh9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNTQsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3LjE2LCJlbXBsb3llZUJvbnVzIjowLjM4LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjUyLCJvZmZpY2VyQm9udXMiOjAuMDYsImNvZ3NEZXByZWNpYXRpb24iOjAuMjksInNnYURlcHJlY2lhdGlvbiI6MS4xNSwicmVzZWFyY2hEZXZlbG9wbWVudCI6MC4yOX19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6NiwiZW1wbG95ZWVTYWxhcnkiOjUuNywiZW1wbG95ZWVCb251cyI6MC4zLCJvZmZpY2VyUGF5IjowLjQsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzYsIm9mZmljZXJCb251cyI6MC4wNCwiZGVwcmVjaWF0aW9uIjoyLCJjb2dzRGVwcmVjaWF0aW9uIjowLjUsInNnYURlcHJlY2lhdGlvbiI6MS41LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjQsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsImVtcGxveWVlU2FsYXJ5Ijo3LjYsImVtcGxveWVlQm9udXMiOjAuNCwib2ZmaWNlclBheSI6MC42LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjU0LCJvZmZpY2VyQm9udXMiOjAuMDYsImRlcHJlY2lhdGlvbiI6MS41LCJjb2dzRGVwcmVjaWF0aW9uIjowLjMsInNnYURlcHJlY2lhdGlvbiI6MS4yLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjMsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMSwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI4NTcxNDI4NTcxNDI4LCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwidXNlZnVsTGlmZSI6MTAsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwxLjY2NTMzNDUzNjkzNzczNDhlLTE2XSwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MzI1MzMwNTAxODQ2OTI3LDAuMDIwNzM1OTk0MTgzMTg5MTY2XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDBdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNDA3NjA4Njk1NjUyMTcxODQsMC4wNDQzODQwNTc5NzEwMTQ1Ml0sIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAwMDEzNDU3NTU2OTM1ODE5NzM3XSwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOlswLjAxOTEzOTQ1NzAyMzcxNzQ0MywwLjAyMDU1MzQ1OTkxNDc2MzA5NV0sIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wMzkxNjY2NjY2NjY2NjY2OCwwLjA0MjUwMDAwMDAwMDAwMDA5XSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RTYWxlc0dyb3d0aCI6WzAuMTUsMC4zXSwib3RoZXJTYWxlc0dyb3d0aCI6WzAuMDYwNzYwODY5NTY1MjE3MTksMC4wNjQzODQwNTc5NzEwMTQ1M10sInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOlswLDAuMDNdLCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6WzAuMDA1LDAuMDA1MTM0NTc1NTY5MzU4MTk3NV0sInByb2plY3RQYXlHcm93dGgiOlswLjA1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMC4wMjQxMzk0NTcwMjM3MTc0NDQsMC4wMjU1NTM0NTk5MTQ3NjMwOTZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGgiOlswLjA0NDE2NjY2NjY2NjY2NjY4LDAuMDQ3NTAwMDAwMDAwMDAwMDldLCJwcm9qZWN0U2dhUmF0ZUVuZCI6WzAuMDg0OTk5OTk5OTk5OTk5OTksMC4xMzVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA4OTI4NTcxNDI4NTcxNDI3LDAuMTE5Mjg1NzE0Mjg1NzE0MjddLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAuMDQyNjMxNTc4OTQ3MzY4MzYsMC4wNjU1NTU1NTU1NTU1NTU1OF0sInVzZWZ1bExpZmUiOls1LDIwXSwiaW52ZXN0bWVudCI6WzE1LDIwMF0sInN1YnNpZHkiOlsxLDUwXSwibG9jYWxCZW5jaG1hcmsiOlswLDEwMF19LCJ0YXJnZXRzIjp7ImNvbXBhbnlTYWxlc0NhZ3IiOnsidmFsdWUiOjE1LCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjgyLjQsIm1heCI6MjUyLjY5LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjoyLCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NjAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo3NC44LCJtYXgiOjEzNi44NCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImxhYm9yUHJvZHVjdGl2aXR5Q2FnciI6eyJ2YWx1ZSI6MjEsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkSW5jcmVhc2UiOnsidmFsdWUiOjE4Ljc4LCJtYXgiOjMzLjQzLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6Mi44NSwibWF4IjozLjc0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiaW52ZXN0bWVudFNhbGVzUmF0aW8iOnsidmFsdWUiOjE1LCJtYXgiOjcwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZFN1YnNpZHlSYXRpbyI6eyJ2YWx1ZSI6MjEzLCJtYXgiOjM1MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImxvY2FsQmVuY2htYXJrIjp7InZhbHVlIjoyMywibWF4Ijo0MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlDYWdyIjp7InZhbHVlIjo2LCJtYXgiOjEwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUluY3JlYXNlIjp7InZhbHVlIjowLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfX0sImZvcmVjYXN0T3ZlcnJpZGVzIjp7IjIwMjk6b3RoZXI6c2FsZXMiOjg1LjEzLCIyMDI5OnByb2plY3Q6Ny04Ijo3Ljl9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2LjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mi43NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTQiOjAuNzMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi03IjozMi42NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTkiOjAuODIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMCI6MC4wOSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEyIjoxMS42NywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEzIjowLjYyLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTQiOjIuNDUsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNSI6MC42NCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEiOjcyLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNCI6MjMuMDQsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny02Ijo2Ljc4LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOCI6NS4xOSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTkiOjAuMzYsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMCI6MS44LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTMiOjkwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xIjoxNDMuMiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTMiOjk3LjM4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNCI6MC43NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTciOjM0LjUyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItOSI6MC44NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMiI6MTIuNDcsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMyI6MC42NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjoyLjU4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTUiOjAuNjcsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xIjo3NiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0LjMyLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNiI6Ny4wNCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTgiOjUuNTksImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTAiOjEuOSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6MC44LCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTkiOjAuOSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjowLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6Mi43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTUiOjAuNywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNCI6MjUuNiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTYiOjcuMywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTgiOjYsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny05IjowLjQsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xMCI6MiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudEFzc2V0cyI6NjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXNoIjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NSwiYmFsYW5jZS1zaGVldDoyMDIzOnRhbmdpYmxlQXNzZXRzIjo1MywiYmFsYW5jZS1zaGVldDoyMDIzOmJ1aWxkaW5ncyI6MTksImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzppbnRhbmdpYmxlQXNzZXRzIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUsImJhbGFuY2Utc2hlZXQ6MjAyMzpsaWFiaWxpdGllcyI6NzUsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50TGlhYmlsaXRpZXMiOjM5LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZExpYWJpbGl0aWVzIjozNiwiYmFsYW5jZS1zaGVldDoyMDIzOmxvbmdUZXJtRGVidCI6MjksImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hhcmVob2xkZXJFcXVpdHkiOjU0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NSwiYmFsYW5jZS1zaGVldDoyMDI0OmFzc2V0cyI6MTQzLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudEFzc2V0cyI6NzIsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNSwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkQXNzZXRzIjo3MSwiYmFsYW5jZS1zaGVldDoyMDI0OnRhbmdpYmxlQXNzZXRzIjo1OCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAsImJhbGFuY2Utc2hlZXQ6MjAyNDptYWNoaW5lcnkiOjI4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c29mdHdhcmUiOjYsImJhbGFuY2Utc2hlZXQ6MjAyNDpsaWFiaWxpdGllcyI6NzksImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZExpYWJpbGl0aWVzIjozOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEsImJhbGFuY2Utc2hlZXQ6MjAyNDpuZXRBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hhcmVob2xkZXJFcXVpdHkiOjYxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBleCI6OCwiYmFsYW5jZS1zaGVldDoyMDI1OmFzc2V0cyI6MTU2LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXNoIjoyNywiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkQXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI1OmJ1aWxkaW5ncyI6MjIsImJhbGFuY2Utc2hlZXQ6MjAyNTptYWNoaW5lcnkiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTppbnRhbmdpYmxlQXNzZXRzIjo5LCJiYWxhbmNlLXNoZWV0OjIwMjU6c29mdHdhcmUiOjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hvcnRUZXJtRGVidCI6MTEsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MCwiYmFsYW5jZS1zaGVldDoyMDI1OmxvbmdUZXJtRGVidCI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpuZXRBc3NldHMiOjczLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBleCI6MTAsImZ1dHVyZS1jYXBleDoyMDI2IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjciOjE1LCJmdXR1cmUtY2FwZXg6MjAyOCI6MTUsImZ1dHVyZS1jYXBleDoyMDI5IjowLCJmdXR1cmUtY2FwZXg6MjAzMCI6MCwiZnV0dXJlLWNhcGV4OjIwMzEiOjAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjEuNjY1MzM0NTM2OTM3NzM0OGUtMTYsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkzMjUzMzA1MDE4NDY5MjcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNzM1OTk0MTgzMTg5MTY2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLjAxOTEzOTQ1NzAyMzcxNzQ0MywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNTUzNDU5OTE0NzYzMDk1LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjAzOTE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNDI1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MCI6MC4xNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjMsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MCI6MC4wMjQxMzk0NTcwMjM3MTc0NDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDoxIjowLjAyNTU1MzQ1OTkxNDc2MzA5NiwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjowLjA0NDE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MSI6MC4wNDc1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjExLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MCI6MC4wODQ5OTk5OTk5OTk5OTk5OSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjEiOjAuMTM1LCJkcml2ZXI6b3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI4NTcxNDI4NTcxNDI4LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjAiOjAuMDg5Mjg1NzE0Mjg1NzE0MjcsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MSI6MC4xMTkyODU3MTQyODU3MTQyNywiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MCI6MC4wNDI2MzE1Nzg5NDczNjgzNiwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjEiOjAuMDY1NTU1NTU1NTU1NTU1NTgsImRyaXZlcjp1c2VmdWxMaWZlIjoxMCwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MCI6NSwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MSI6MjAsImRyaXZlcjppbnZlc3RtZW50IjoyMywiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjEiOjIwMCwiZHJpdmVyOnN1YnNpZHkiOjcuNjYsImRyaXZlci1yYW5nZTpzdWJzaWR5OjAiOjEsImRyaXZlci1yYW5nZTpzdWJzaWR5OjEiOjUwLCJkcml2ZXI6bG9jYWxCZW5jaG1hcmsiOjIzLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MCI6MCwiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjEiOjEwMCwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6dmFsdWUiOjE1LCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6dmFsdWUiOjgyLjQsInRhcmdldDpjb21wYW55UGF5U2NoZWR1bGU6dmFsdWUiOjIsInRhcmdldDpjb21wYW55UGF5U2NoZWR1bGU6bWF4Ijo3LCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6dmFsdWUiOjYwLCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6bWF4Ijo5NSwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6dmFsdWUiOjIyLCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6dmFsdWUiOjc0LjgsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6dmFsdWUiOjIxLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOm1heCI6MzUsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6dmFsdWUiOjE4Ljc4LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOnZhbHVlIjo3LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOm1heCI6MTAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOnZhbHVlIjoyLjg1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86dmFsdWUiOjE1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86bWF4Ijo3MCwidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86dmFsdWUiOjIxMywidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86bWF4IjozNTAsInRhcmdldDpsb2NhbEJlbmNobWFyazp2YWx1ZSI6MjMsInRhcmdldDpsb2NhbEJlbmNobWFyazptYXgiOjQwLCJ0YXJnZXQ6b2ZmaWNlclBheUNhZ3I6dmFsdWUiOjYsInRhcmdldDpvZmZpY2VyUGF5Q2FncjptYXgiOjEwLCJ0YXJnZXQ6b2ZmaWNlclBheUluY3JlYXNlOnZhbHVlIjowLCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6bWF4IjoyNTIuNjksInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTptYXgiOjEzNi44NCwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTptYXgiOjMzLjQzLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlJbmNyZWFzZTptYXgiOjMuNzR9LCJtZXRyaWNHcm91cEJhc2VzIjp7ImNvbXBhbnlTYWxlcyI6InJhdGUiLCJwcm9qZWN0U2FsZXMiOiJyYXRlIiwibGFib3JQcm9kdWN0aXZpdHkiOiJyYXRlIiwiZW1wbG95ZWVQYXkiOiJyYXRlIn0sImFwcGxpY2F0aW9uQ2F0ZWdvcnkiOiJnZW5lcmFsIiwiYWRqdXN0ZWREcml2ZXJzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQwMzY4MDU1NTU1NTU1NCwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MS4xNzQxODY0OTEwNjQ0NjZlLTE2LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAxOTgxNjI4NzE3ODg3NywicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQ0NDg1MzYzMDY3NTMyNzQsInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDYwOTMzNzAyNzg5ODA0LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjYwNzMxNjU4MzkyMjQ5LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODA5MDU5NTA0NjA1NjYzLCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDE0OTM3NzcyNDkzMDY0NDYsIm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMiwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NDAxODU3MDcyNjUyNiwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTU1NTA0MjcyNTc5NzcyODQsIm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwicHJvamVjdFBheUdyb3d0aCI6MC4xLCJvdGhlclBheUdyb3d0aCI6MC4wMjU1NTM0NTk5MTQ3NjMwOTYsInByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTg3MjM3NjkyMTM2MzM4LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMSwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTMyNjE2NDY1MTYzNjYsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgxOTIzMTY3OTU4MzQ5NiwidXNlZnVsTGlmZSI6MTAsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9fQ==</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make saved sample optimization results stable
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -204,7 +204,7 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <v>15.448906650814621</v>
+        <v>15.464691482957393</v>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
@@ -234,7 +234,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <v>93.21000000000004</v>
+        <v>93.33000000000001</v>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
@@ -264,7 +264,7 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <v>2.0136531491304233</v>
+        <v>2.0628917862888008</v>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
@@ -294,7 +294,7 @@
         </is>
       </c>
       <c r="B11" s="2">
-        <v>63.89827961836075</v>
+        <v>63.91350052560445</v>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
@@ -324,7 +324,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>22.000324971691864</v>
+        <v>22.02271203454029</v>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
@@ -354,7 +354,7 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <v>76.43</v>
+        <v>76.54</v>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
@@ -384,7 +384,7 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <v>22.016675856213674</v>
+        <v>23.49843476135365</v>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
@@ -414,7 +414,7 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <v>19.73000000000001</v>
+        <v>19.660000000000004</v>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
@@ -444,7 +444,7 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <v>7.019737997987985</v>
+        <v>7.000299957045453</v>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B17" s="2">
-        <v>2.8600000000000003</v>
+        <v>2.46</v>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <v>257.5718015665798</v>
+        <v>256.6579634464752</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
@@ -1259,22 +1259,22 @@
         <v>150</v>
       </c>
       <c r="E3" s="4">
-        <v>157.3</v>
+        <v>157.31</v>
       </c>
       <c r="F3" s="4">
-        <v>164.97</v>
+        <v>164.98000000000002</v>
       </c>
       <c r="G3" s="4">
-        <v>173.01</v>
+        <v>173.03</v>
       </c>
       <c r="H3" s="4">
-        <v>199.42000000000002</v>
+        <v>199.47</v>
       </c>
       <c r="I3" s="4">
-        <v>229.88</v>
+        <v>229.95999999999998</v>
       </c>
       <c r="J3" s="4">
-        <v>266.22</v>
+        <v>266.36</v>
       </c>
     </row>
     <row r="4">
@@ -1295,22 +1295,22 @@
         <v>4.748603351955305</v>
       </c>
       <c r="E4" s="2">
-        <v>4.866666666666664</v>
+        <v>4.8733333333333295</v>
       </c>
       <c r="F4" s="2">
-        <v>4.876033057851226</v>
+        <v>4.875723094526752</v>
       </c>
       <c r="G4" s="2">
-        <v>4.873613384251674</v>
+        <v>4.879379318705279</v>
       </c>
       <c r="H4" s="2">
-        <v>15.265013583029896</v>
+        <v>15.28058718141363</v>
       </c>
       <c r="I4" s="2">
-        <v>15.27429545682477</v>
+        <v>15.285506592470032</v>
       </c>
       <c r="J4" s="2">
-        <v>15.8082477814512</v>
+        <v>15.828839798225802</v>
       </c>
     </row>
     <row r="5">
@@ -1332,19 +1332,19 @@
         <v>106.97</v>
       </c>
       <c r="F5" s="2">
-        <v>112.18</v>
+        <v>112.19</v>
       </c>
       <c r="G5" s="2">
-        <v>117.65</v>
+        <v>117.67</v>
       </c>
       <c r="H5" s="2">
-        <v>134.3</v>
+        <v>134.36</v>
       </c>
       <c r="I5" s="2">
-        <v>153.98000000000002</v>
+        <v>154.09</v>
       </c>
       <c r="J5" s="2">
-        <v>177.26</v>
+        <v>177.45999999999998</v>
       </c>
     </row>
     <row r="6">
@@ -1397,22 +1397,22 @@
         <v>48</v>
       </c>
       <c r="E7" s="4">
-        <v>50.33000000000001</v>
+        <v>50.34</v>
       </c>
       <c r="F7" s="4">
-        <v>52.78999999999999</v>
+        <v>52.79000000000002</v>
       </c>
       <c r="G7" s="4">
-        <v>55.359999999999985</v>
+        <v>55.36</v>
       </c>
       <c r="H7" s="4">
-        <v>65.12</v>
+        <v>65.10999999999999</v>
       </c>
       <c r="I7" s="4">
-        <v>75.89999999999998</v>
+        <v>75.86999999999998</v>
       </c>
       <c r="J7" s="4">
-        <v>88.96000000000004</v>
+        <v>88.90000000000003</v>
       </c>
     </row>
     <row r="8">
@@ -1431,22 +1431,22 @@
         <v>32</v>
       </c>
       <c r="E8" s="2">
-        <v>31.996185632549274</v>
+        <v>32.00050854999682</v>
       </c>
       <c r="F8" s="2">
-        <v>31.99975753167242</v>
+        <v>31.997817917323324</v>
       </c>
       <c r="G8" s="2">
-        <v>31.998150395930864</v>
+        <v>31.994451829162575</v>
       </c>
       <c r="H8" s="2">
-        <v>32.654698626015445</v>
+        <v>32.641499974933566</v>
       </c>
       <c r="I8" s="2">
-        <v>33.01722637898033</v>
+        <v>32.99269438163158</v>
       </c>
       <c r="J8" s="2">
-        <v>33.415971752685756</v>
+        <v>33.37588226460431</v>
       </c>
     </row>
     <row r="9">
@@ -1465,22 +1465,22 @@
         <v>36.4</v>
       </c>
       <c r="E9" s="2">
-        <v>38.87</v>
+        <v>38.86</v>
       </c>
       <c r="F9" s="2">
-        <v>41.449999999999996</v>
+        <v>41.44</v>
       </c>
       <c r="G9" s="2">
-        <v>44.19</v>
+        <v>44.15</v>
       </c>
       <c r="H9" s="2">
-        <v>47.89</v>
+        <v>47.87</v>
       </c>
       <c r="I9" s="2">
-        <v>52.74</v>
+        <v>52.519999999999996</v>
       </c>
       <c r="J9" s="2">
-        <v>58.2</v>
+        <v>57.73</v>
       </c>
     </row>
     <row r="10">
@@ -1601,22 +1601,22 @@
         <v>14</v>
       </c>
       <c r="E13" s="2">
-        <v>14.95</v>
+        <v>14.940000000000001</v>
       </c>
       <c r="F13" s="2">
-        <v>15.96</v>
+        <v>15.95</v>
       </c>
       <c r="G13" s="2">
-        <v>17.06</v>
+        <v>17.02</v>
       </c>
       <c r="H13" s="2">
-        <v>18.18</v>
+        <v>18.15</v>
       </c>
       <c r="I13" s="2">
-        <v>20.07</v>
+        <v>19.84</v>
       </c>
       <c r="J13" s="2">
-        <v>22.16</v>
+        <v>21.689999999999998</v>
       </c>
     </row>
     <row r="14">
@@ -1638,19 +1638,19 @@
         <v>14.2</v>
       </c>
       <c r="F14" s="2">
-        <v>15.16</v>
+        <v>15.15</v>
       </c>
       <c r="G14" s="2">
-        <v>16.21</v>
+        <v>16.17</v>
       </c>
       <c r="H14" s="2">
-        <v>17.9</v>
+        <v>17.69</v>
       </c>
       <c r="I14" s="2">
-        <v>19.78</v>
+        <v>19.35</v>
       </c>
       <c r="J14" s="2">
-        <v>21.87</v>
+        <v>21.16</v>
       </c>
     </row>
     <row r="15">
@@ -1669,7 +1669,7 @@
         <v>0.7</v>
       </c>
       <c r="E15" s="2">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="F15" s="2">
         <v>0.8</v>
@@ -1678,13 +1678,13 @@
         <v>0.85</v>
       </c>
       <c r="H15" s="2">
-        <v>0.9299999999999999</v>
+        <v>0.9199999999999999</v>
       </c>
       <c r="I15" s="2">
-        <v>1.03</v>
+        <v>1.01</v>
       </c>
       <c r="J15" s="2">
-        <v>1.1400000000000001</v>
+        <v>1.1099999999999999</v>
       </c>
     </row>
     <row r="16">
@@ -1771,22 +1771,22 @@
         <v>11.600000000000001</v>
       </c>
       <c r="E18" s="4">
-        <v>11.460000000000008</v>
+        <v>11.480000000000004</v>
       </c>
       <c r="F18" s="4">
-        <v>11.33999999999999</v>
+        <v>11.350000000000016</v>
       </c>
       <c r="G18" s="4">
-        <v>11.169999999999984</v>
+        <v>11.210000000000004</v>
       </c>
       <c r="H18" s="4">
-        <v>17.230000000000004</v>
+        <v>17.239999999999988</v>
       </c>
       <c r="I18" s="4">
-        <v>23.159999999999982</v>
+        <v>23.34999999999998</v>
       </c>
       <c r="J18" s="4">
-        <v>30.760000000000048</v>
+        <v>31.170000000000044</v>
       </c>
     </row>
     <row r="19">
@@ -1805,22 +1805,22 @@
         <v>7.733333333333333</v>
       </c>
       <c r="E19" s="2">
-        <v>7.285441830896381</v>
+        <v>7.297692454389424</v>
       </c>
       <c r="F19" s="2">
-        <v>6.8739770867430385</v>
+        <v>6.879621772336049</v>
       </c>
       <c r="G19" s="2">
-        <v>6.456274203803239</v>
+        <v>6.478645321620531</v>
       </c>
       <c r="H19" s="2">
-        <v>8.64005616287233</v>
+        <v>8.64290369479119</v>
       </c>
       <c r="I19" s="2">
-        <v>10.074821646076208</v>
+        <v>10.1539398156201</v>
       </c>
       <c r="J19" s="2">
-        <v>11.554353542183174</v>
+        <v>11.702207538669485</v>
       </c>
     </row>
     <row r="20">
@@ -1839,22 +1839,22 @@
         <v>11.600000000000001</v>
       </c>
       <c r="E20" s="4">
-        <v>11.460000000000008</v>
+        <v>11.480000000000004</v>
       </c>
       <c r="F20" s="4">
-        <v>11.33999999999999</v>
+        <v>11.350000000000016</v>
       </c>
       <c r="G20" s="4">
-        <v>11.169999999999984</v>
+        <v>11.210000000000004</v>
       </c>
       <c r="H20" s="4">
-        <v>17.230000000000004</v>
+        <v>17.239999999999988</v>
       </c>
       <c r="I20" s="4">
-        <v>23.159999999999982</v>
+        <v>23.34999999999998</v>
       </c>
       <c r="J20" s="4">
-        <v>30.760000000000048</v>
+        <v>31.170000000000044</v>
       </c>
     </row>
     <row r="21">
@@ -1977,22 +1977,22 @@
         <v>14</v>
       </c>
       <c r="E23" s="2">
-        <v>14.95</v>
+        <v>14.940000000000001</v>
       </c>
       <c r="F23" s="2">
-        <v>15.96</v>
+        <v>15.95</v>
       </c>
       <c r="G23" s="2">
-        <v>17.06</v>
+        <v>17.02</v>
       </c>
       <c r="H23" s="2">
-        <v>18.18</v>
+        <v>18.15</v>
       </c>
       <c r="I23" s="2">
-        <v>20.07</v>
+        <v>19.84</v>
       </c>
       <c r="J23" s="2">
-        <v>22.16</v>
+        <v>21.689999999999998</v>
       </c>
     </row>
     <row r="24">
@@ -2079,22 +2079,22 @@
         <v>30.1</v>
       </c>
       <c r="E26" s="4">
-        <v>31.710000000000008</v>
+        <v>31.720000000000006</v>
       </c>
       <c r="F26" s="4">
-        <v>33.389999999999986</v>
+        <v>33.390000000000015</v>
       </c>
       <c r="G26" s="4">
-        <v>35.13999999999998</v>
+        <v>35.14</v>
       </c>
       <c r="H26" s="4">
-        <v>42.36</v>
+        <v>42.33999999999998</v>
       </c>
       <c r="I26" s="4">
-        <v>50.21999999999998</v>
+        <v>50.17999999999998</v>
       </c>
       <c r="J26" s="4">
-        <v>59.96000000000004</v>
+        <v>59.90000000000004</v>
       </c>
     </row>
     <row r="27">
@@ -2115,22 +2115,22 @@
         <v>4.768534632788035</v>
       </c>
       <c r="E27" s="2">
-        <v>5.348837209302348</v>
+        <v>5.382059800664463</v>
       </c>
       <c r="F27" s="2">
-        <v>5.298013245033051</v>
+        <v>5.264817150063084</v>
       </c>
       <c r="G27" s="2">
-        <v>5.2410901467505155</v>
+        <v>5.241090146750471</v>
       </c>
       <c r="H27" s="2">
-        <v>20.54638588503137</v>
+        <v>20.489470688673816</v>
       </c>
       <c r="I27" s="2">
-        <v>18.55524079320108</v>
+        <v>18.516769012753898</v>
       </c>
       <c r="J27" s="2">
-        <v>19.394663480685125</v>
+        <v>19.37026703866096</v>
       </c>
     </row>
     <row r="28">
@@ -2149,22 +2149,22 @@
         <v>20.06666666666667</v>
       </c>
       <c r="E28" s="2">
-        <v>20.1589319771138</v>
+        <v>20.164007373974957</v>
       </c>
       <c r="F28" s="2">
-        <v>20.240043644298954</v>
+        <v>20.23881682628198</v>
       </c>
       <c r="G28" s="2">
-        <v>20.310964684122293</v>
+        <v>20.30861700283188</v>
       </c>
       <c r="H28" s="2">
-        <v>21.241600641861396</v>
+        <v>21.226249561337536</v>
       </c>
       <c r="I28" s="2">
-        <v>21.846180615973545</v>
+        <v>21.821186293268386</v>
       </c>
       <c r="J28" s="2">
-        <v>22.522725565321927</v>
+        <v>22.488361615858253</v>
       </c>
     </row>
     <row r="29">
@@ -2189,16 +2189,16 @@
         <v>252</v>
       </c>
       <c r="G29" s="2">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="H29" s="2">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="I29" s="2">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="J29" s="2">
-        <v>300</v>
+        <v>295</v>
       </c>
     </row>
     <row r="30">
@@ -2251,22 +2251,22 @@
         <v>0.06086956521739131</v>
       </c>
       <c r="E31" s="2">
-        <v>0.06229166666666666</v>
+        <v>0.06225000000000001</v>
       </c>
       <c r="F31" s="2">
-        <v>0.06333333333333334</v>
+        <v>0.06329365079365079</v>
       </c>
       <c r="G31" s="2">
-        <v>0.06462121212121212</v>
+        <v>0.0647148288973384</v>
       </c>
       <c r="H31" s="2">
-        <v>0.0658695652173913</v>
+        <v>0.06648351648351648</v>
       </c>
       <c r="I31" s="2">
-        <v>0.0696875</v>
+        <v>0.06985915492957746</v>
       </c>
       <c r="J31" s="2">
-        <v>0.07386666666666666</v>
+        <v>0.07352542372881356</v>
       </c>
     </row>
     <row r="32">
@@ -2287,22 +2287,22 @@
         <v>1.9901321235802572</v>
       </c>
       <c r="E32" s="2">
-        <v>2.336309523809521</v>
+        <v>2.267857142857155</v>
       </c>
       <c r="F32" s="2">
-        <v>1.6722408026756064</v>
+        <v>1.6765474596799779</v>
       </c>
       <c r="G32" s="2">
-        <v>2.0334928229664984</v>
+        <v>2.2453723017509475</v>
       </c>
       <c r="H32" s="2">
-        <v>1.9318008053417657</v>
+        <v>2.733048385222303</v>
       </c>
       <c r="I32" s="2">
-        <v>5.796204620462042</v>
+        <v>5.077406588290079</v>
       </c>
       <c r="J32" s="2">
-        <v>5.997010463378172</v>
+        <v>5.24808638600327</v>
       </c>
     </row>
     <row r="33">
@@ -2391,22 +2391,22 @@
         <v>0.12808510638297874</v>
       </c>
       <c r="E35" s="2">
-        <v>0.12942857142857145</v>
+        <v>0.12946938775510206</v>
       </c>
       <c r="F35" s="2">
-        <v>0.1299221789883268</v>
+        <v>0.12992217898832692</v>
       </c>
       <c r="G35" s="2">
-        <v>0.13063197026022297</v>
+        <v>0.13111940298507463</v>
       </c>
       <c r="H35" s="2">
-        <v>0.1507473309608541</v>
+        <v>0.15230215827338123</v>
       </c>
       <c r="I35" s="2">
-        <v>0.17139931740614328</v>
+        <v>0.1736332179930795</v>
       </c>
       <c r="J35" s="2">
-        <v>0.19659016393442638</v>
+        <v>0.1996666666666668</v>
       </c>
     </row>
     <row r="36">
@@ -2425,22 +2425,22 @@
         <v>15.100000000000001</v>
       </c>
       <c r="E36" s="4">
-        <v>15.730000000000008</v>
+        <v>15.750000000000004</v>
       </c>
       <c r="F36" s="4">
-        <v>16.36999999999999</v>
+        <v>16.380000000000017</v>
       </c>
       <c r="G36" s="4">
-        <v>16.969999999999985</v>
+        <v>17.010000000000005</v>
       </c>
       <c r="H36" s="4">
-        <v>23.030000000000005</v>
+        <v>23.03999999999999</v>
       </c>
       <c r="I36" s="4">
-        <v>28.959999999999983</v>
+        <v>29.14999999999998</v>
       </c>
       <c r="J36" s="4">
-        <v>36.560000000000045</v>
+        <v>36.97000000000004</v>
       </c>
     </row>
     <row r="37">
@@ -2459,22 +2459,22 @@
         <v>10.066666666666668</v>
       </c>
       <c r="E37" s="2">
-        <v>10.000000000000005</v>
+        <v>10.012078062424514</v>
       </c>
       <c r="F37" s="2">
-        <v>9.923016305995024</v>
+        <v>9.928476178930788</v>
       </c>
       <c r="G37" s="2">
-        <v>9.808681579099465</v>
+        <v>9.830665202566031</v>
       </c>
       <c r="H37" s="2">
-        <v>11.548490622806138</v>
+        <v>11.550609114152497</v>
       </c>
       <c r="I37" s="2">
-        <v>12.597877153297365</v>
+        <v>12.676117585667065</v>
       </c>
       <c r="J37" s="2">
-        <v>13.733002779655939</v>
+        <v>13.879711668418695</v>
       </c>
     </row>
     <row r="38">
@@ -2495,22 +2495,22 @@
         <v>3.1420765027322606</v>
       </c>
       <c r="E38" s="2">
-        <v>4.172185430463626</v>
+        <v>4.304635761589415</v>
       </c>
       <c r="F38" s="2">
-        <v>4.068658614113052</v>
+        <v>4.000000000000092</v>
       </c>
       <c r="G38" s="2">
-        <v>3.665241295051902</v>
+        <v>3.846153846153766</v>
       </c>
       <c r="H38" s="2">
-        <v>35.71007660577506</v>
+        <v>35.44973544973533</v>
       </c>
       <c r="I38" s="2">
-        <v>25.749023013460604</v>
+        <v>26.51909722222221</v>
       </c>
       <c r="J38" s="2">
-        <v>26.24309392265216</v>
+        <v>26.826758147513097</v>
       </c>
     </row>
   </sheetData>
@@ -2663,22 +2663,22 @@
         <v>80</v>
       </c>
       <c r="E3" s="4">
-        <v>84.32</v>
+        <v>84.33</v>
       </c>
       <c r="F3" s="4">
-        <v>88.88</v>
+        <v>88.89</v>
       </c>
       <c r="G3" s="4">
-        <v>93.68</v>
+        <v>93.7</v>
       </c>
       <c r="H3" s="4">
-        <v>114.29</v>
+        <v>114.34</v>
       </c>
       <c r="I3" s="4">
-        <v>139.43</v>
+        <v>139.51</v>
       </c>
       <c r="J3" s="4">
-        <v>170.11</v>
+        <v>170.24</v>
       </c>
     </row>
     <row r="4">
@@ -2699,22 +2699,22 @@
         <v>5.263157894736836</v>
       </c>
       <c r="E4" s="2">
-        <v>5.399999999999983</v>
+        <v>5.412499999999998</v>
       </c>
       <c r="F4" s="2">
-        <v>5.407969639468702</v>
+        <v>5.407328352899321</v>
       </c>
       <c r="G4" s="2">
-        <v>5.400540054005409</v>
+        <v>5.41118236022049</v>
       </c>
       <c r="H4" s="2">
-        <v>22.000426985482502</v>
+        <v>22.027748132337255</v>
       </c>
       <c r="I4" s="2">
-        <v>21.996675124682817</v>
+        <v>22.01329368549938</v>
       </c>
       <c r="J4" s="2">
-        <v>22.00387291113821</v>
+        <v>22.027094831911697</v>
       </c>
     </row>
     <row r="5">
@@ -2733,22 +2733,22 @@
         <v>53.333333333333336</v>
       </c>
       <c r="E5" s="2">
-        <v>53.60457724094086</v>
+        <v>53.60752653995296</v>
       </c>
       <c r="F5" s="2">
-        <v>53.87646238710069</v>
+        <v>53.87925809188992</v>
       </c>
       <c r="G5" s="2">
-        <v>54.14715912375008</v>
+        <v>54.1524591111368</v>
       </c>
       <c r="H5" s="2">
-        <v>57.31120248721292</v>
+        <v>57.321903043064125</v>
       </c>
       <c r="I5" s="2">
-        <v>60.653384374456245</v>
+        <v>60.66707253435381</v>
       </c>
       <c r="J5" s="2">
-        <v>63.89827961836075</v>
+        <v>63.91350052560445</v>
       </c>
     </row>
     <row r="6">
@@ -2767,7 +2767,7 @@
         <v>25.6</v>
       </c>
       <c r="E6" s="4">
-        <v>26.97999999999999</v>
+        <v>26.989999999999995</v>
       </c>
       <c r="F6" s="4">
         <v>28.439999999999998</v>
@@ -2776,13 +2776,13 @@
         <v>29.980000000000004</v>
       </c>
       <c r="H6" s="4">
-        <v>37.17</v>
+        <v>37.16</v>
       </c>
       <c r="I6" s="4">
-        <v>46.06</v>
+        <v>46.02999999999999</v>
       </c>
       <c r="J6" s="4">
-        <v>57.09000000000002</v>
+        <v>57.02000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -2801,22 +2801,22 @@
         <v>32</v>
       </c>
       <c r="E7" s="2">
-        <v>31.997153700189745</v>
+        <v>32.005217597533495</v>
       </c>
       <c r="F7" s="2">
-        <v>31.998199819982</v>
+        <v>31.994600067499153</v>
       </c>
       <c r="G7" s="2">
-        <v>32.00256191289496</v>
+        <v>31.995731056563503</v>
       </c>
       <c r="H7" s="2">
-        <v>32.522530405109805</v>
+        <v>32.49956270771383</v>
       </c>
       <c r="I7" s="2">
-        <v>33.034497597360684</v>
+        <v>32.99405060569134</v>
       </c>
       <c r="J7" s="2">
-        <v>33.56063723473048</v>
+        <v>33.49389097744361</v>
       </c>
     </row>
     <row r="8">
@@ -2835,22 +2835,22 @@
         <v>7.300000000000004</v>
       </c>
       <c r="E8" s="4">
-        <v>7.069999999999986</v>
+        <v>7.079999999999991</v>
       </c>
       <c r="F8" s="4">
         <v>6.859999999999996</v>
       </c>
       <c r="G8" s="4">
-        <v>6.630000000000006</v>
+        <v>6.640000000000004</v>
       </c>
       <c r="H8" s="4">
-        <v>11.260000000000002</v>
+        <v>11.239999999999997</v>
       </c>
       <c r="I8" s="4">
-        <v>16.54</v>
+        <v>16.689999999999984</v>
       </c>
       <c r="J8" s="4">
-        <v>23.420000000000023</v>
+        <v>23.760000000000012</v>
       </c>
     </row>
     <row r="9">
@@ -2869,22 +2869,22 @@
         <v>9.125000000000005</v>
       </c>
       <c r="E9" s="2">
-        <v>8.384724857684994</v>
+        <v>8.395588758448941</v>
       </c>
       <c r="F9" s="2">
-        <v>7.718271827182714</v>
+        <v>7.717403532455839</v>
       </c>
       <c r="G9" s="2">
-        <v>7.077284372331347</v>
+        <v>7.086446104589118</v>
       </c>
       <c r="H9" s="2">
-        <v>9.85213054510456</v>
+        <v>9.830330592968336</v>
       </c>
       <c r="I9" s="2">
-        <v>11.862583375170335</v>
+        <v>11.963300121855053</v>
       </c>
       <c r="J9" s="2">
-        <v>13.767562165657528</v>
+        <v>13.95676691729324</v>
       </c>
     </row>
     <row r="10">
@@ -2909,16 +2909,16 @@
         <v>6.94</v>
       </c>
       <c r="G10" s="2">
-        <v>7.47</v>
+        <v>7.46</v>
       </c>
       <c r="H10" s="2">
         <v>7.9</v>
       </c>
       <c r="I10" s="2">
-        <v>9.04</v>
+        <v>8.85</v>
       </c>
       <c r="J10" s="2">
-        <v>10.33</v>
+        <v>9.92</v>
       </c>
     </row>
     <row r="11">
@@ -3005,7 +3005,7 @@
         <v>15.700000000000005</v>
       </c>
       <c r="E13" s="4">
-        <v>16.709999999999987</v>
+        <v>16.71999999999999</v>
       </c>
       <c r="F13" s="4">
         <v>17.769999999999996</v>
@@ -3014,13 +3014,13 @@
         <v>18.870000000000005</v>
       </c>
       <c r="H13" s="4">
-        <v>23.960000000000004</v>
+        <v>23.939999999999998</v>
       </c>
       <c r="I13" s="4">
-        <v>30.4</v>
+        <v>30.359999999999985</v>
       </c>
       <c r="J13" s="4">
-        <v>38.600000000000016</v>
+        <v>38.53000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -3041,22 +3041,22 @@
         <v>5.2984574111334615</v>
       </c>
       <c r="E14" s="2">
-        <v>6.433121019108157</v>
+        <v>6.496815286624114</v>
       </c>
       <c r="F14" s="2">
-        <v>6.3435068821065865</v>
+        <v>6.279904306220119</v>
       </c>
       <c r="G14" s="2">
         <v>6.190208216094595</v>
       </c>
       <c r="H14" s="2">
-        <v>26.974032856385797</v>
+        <v>26.868044515103296</v>
       </c>
       <c r="I14" s="2">
-        <v>26.878130217028364</v>
+        <v>26.81704260651625</v>
       </c>
       <c r="J14" s="2">
-        <v>26.973684210526372</v>
+        <v>26.910408432147648</v>
       </c>
     </row>
     <row r="15">
@@ -3084,13 +3084,13 @@
         <v>117</v>
       </c>
       <c r="H15" s="2">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I15" s="2">
+        <v>124</v>
+      </c>
+      <c r="J15" s="2">
         <v>127</v>
-      </c>
-      <c r="J15" s="2">
-        <v>132</v>
       </c>
     </row>
     <row r="16">
@@ -3149,16 +3149,16 @@
         <v>0.06252252252252252</v>
       </c>
       <c r="G17" s="2">
-        <v>0.06384615384615384</v>
+        <v>0.06376068376068376</v>
       </c>
       <c r="H17" s="2">
-        <v>0.06475409836065574</v>
+        <v>0.06583333333333334</v>
       </c>
       <c r="I17" s="2">
-        <v>0.07118110236220472</v>
+        <v>0.07137096774193548</v>
       </c>
       <c r="J17" s="2">
-        <v>0.07825757575757576</v>
+        <v>0.07811023622047245</v>
       </c>
     </row>
     <row r="18">
@@ -3185,16 +3185,16 @@
         <v>1.780850618059926</v>
       </c>
       <c r="G18" s="2">
-        <v>2.1170472179117716</v>
+        <v>1.9803443434567525</v>
       </c>
       <c r="H18" s="2">
-        <v>1.4220817697017551</v>
+        <v>3.250670241286868</v>
       </c>
       <c r="I18" s="2">
-        <v>9.925246685936395</v>
+        <v>8.411596570028568</v>
       </c>
       <c r="J18" s="2">
-        <v>9.941505765620828</v>
+        <v>9.442590862582879</v>
       </c>
     </row>
     <row r="19">
@@ -3283,7 +3283,7 @@
         <v>0.15392156862745102</v>
       </c>
       <c r="E21" s="2">
-        <v>0.1561682242990653</v>
+        <v>0.15626168224299058</v>
       </c>
       <c r="F21" s="2">
         <v>0.15725663716814156</v>
@@ -3292,13 +3292,13 @@
         <v>0.1585714285714286</v>
       </c>
       <c r="H21" s="2">
-        <v>0.19322580645161294</v>
+        <v>0.1962295081967213</v>
       </c>
       <c r="I21" s="2">
-        <v>0.23565891472868217</v>
+        <v>0.24095238095238083</v>
       </c>
       <c r="J21" s="2">
-        <v>0.28805970149253746</v>
+        <v>0.29868217054263574</v>
       </c>
     </row>
     <row r="22">
@@ -3611,7 +3611,7 @@
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.87 % / 補助 5.4 % / 他 4.26 %</t>
+          <t xml:space="preserve">全社 4.87 % / 補助 5.41 % / 他 4.26 %</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
@@ -3621,22 +3621,22 @@
       </c>
       <c r="I4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.87 % / 補助 5.4 % / 他 4.26 %</t>
+          <t xml:space="preserve">全社 4.88 % / 補助 5.41 % / 他 4.26 %</t>
         </is>
       </c>
       <c r="J4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.27 % / 補助 22 % / 他 7.31 %</t>
+          <t xml:space="preserve">全社 15.28 % / 補助 22.03 % / 他 7.31 %</t>
         </is>
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.27 % / 補助 22 % / 他 6.25 %</t>
+          <t xml:space="preserve">全社 15.29 % / 補助 22.01 % / 他 6.25 %</t>
         </is>
       </c>
       <c r="L4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.81 % / 補助 22 % / 他 6.26 %</t>
+          <t xml:space="preserve">全社 15.83 % / 補助 22.03 % / 他 6.27 %</t>
         </is>
       </c>
     </row>
@@ -3673,32 +3673,32 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 68 % / 補助 68 % / 他 68 %</t>
+          <t xml:space="preserve">全社 68 % / 補助 67.99 % / 他 68 %</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 68 % / 補助 68 % / 他 68 %</t>
+          <t xml:space="preserve">全社 68 % / 補助 68.01 % / 他 68 %</t>
         </is>
       </c>
       <c r="I5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 68 % / 補助 68 % / 他 68.01 %</t>
+          <t xml:space="preserve">全社 68.01 % / 補助 68 % / 他 68.01 %</t>
         </is>
       </c>
       <c r="J5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 67.35 % / 補助 67.48 % / 他 67.17 %</t>
+          <t xml:space="preserve">全社 67.36 % / 補助 67.5 % / 他 67.17 %</t>
         </is>
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 66.98 % / 補助 66.97 % / 他 67.01 %</t>
+          <t xml:space="preserve">全社 67.01 % / 補助 67.01 % / 他 67.01 %</t>
         </is>
       </c>
       <c r="L5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 66.58 % / 補助 66.44 % / 他 66.84 %</t>
+          <t xml:space="preserve">全社 66.62 % / 補助 66.51 % / 他 66.83 %</t>
         </is>
       </c>
     </row>
@@ -3735,32 +3735,32 @@
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32 % / 補助 32 % / 他 32 %</t>
+          <t xml:space="preserve">全社 32 % / 補助 32.01 % / 他 32 %</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32 % / 補助 32 % / 他 32 %</t>
+          <t xml:space="preserve">全社 32 % / 補助 31.99 % / 他 32 %</t>
         </is>
       </c>
       <c r="I6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32 % / 補助 32 % / 他 31.99 %</t>
+          <t xml:space="preserve">全社 31.99 % / 補助 32 % / 他 31.99 %</t>
         </is>
       </c>
       <c r="J6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32.65 % / 補助 32.52 % / 他 32.83 %</t>
+          <t xml:space="preserve">全社 32.64 % / 補助 32.5 % / 他 32.83 %</t>
         </is>
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 33.02 % / 補助 33.03 % / 他 32.99 %</t>
+          <t xml:space="preserve">全社 32.99 % / 補助 32.99 % / 他 32.99 %</t>
         </is>
       </c>
       <c r="L6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 33.42 % / 補助 33.56 % / 他 33.16 %</t>
+          <t xml:space="preserve">全社 33.38 % / 補助 33.49 % / 他 33.17 %</t>
         </is>
       </c>
     </row>
@@ -3797,32 +3797,32 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.71 % / 補助 23.61 % / 他 25.98 %</t>
+          <t xml:space="preserve">全社 24.7 % / 補助 23.61 % / 他 25.97 %</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 25.13 % / 補助 24.28 % / 他 26.11 %</t>
+          <t xml:space="preserve">全社 25.12 % / 補助 24.28 % / 他 26.1 %</t>
         </is>
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 25.54 % / 補助 24.93 % / 他 26.27 %</t>
+          <t xml:space="preserve">全社 25.52 % / 補助 24.91 % / 他 26.23 %</t>
         </is>
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.01 % / 補助 22.67 % / 他 25.82 %</t>
+          <t xml:space="preserve">全社 24 % / 補助 22.67 % / 他 25.78 %</t>
         </is>
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 22.94 % / 補助 21.17 % / 他 25.67 %</t>
+          <t xml:space="preserve">全社 22.84 % / 補助 21.03 % / 他 25.63 %</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 21.86 % / 補助 19.79 % / 他 25.52 %</t>
+          <t xml:space="preserve">全社 21.67 % / 補助 19.54 % / 他 25.46 %</t>
         </is>
       </c>
     </row>
@@ -3859,32 +3859,32 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.29 % / 補助 8.38 % / 他 6.02 %</t>
+          <t xml:space="preserve">全社 7.3 % / 補助 8.4 % / 他 6.03 %</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.87 % / 補助 7.72 % / 他 5.89 %</t>
+          <t xml:space="preserve">全社 6.88 % / 補助 7.72 % / 他 5.9 %</t>
         </is>
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.46 % / 補助 7.08 % / 他 5.72 %</t>
+          <t xml:space="preserve">全社 6.48 % / 補助 7.09 % / 他 5.76 %</t>
         </is>
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.64 % / 補助 9.85 % / 他 7.01 %</t>
+          <t xml:space="preserve">全社 8.64 % / 補助 9.83 % / 他 7.05 %</t>
         </is>
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.07 % / 補助 11.86 % / 他 7.32 %</t>
+          <t xml:space="preserve">全社 10.15 % / 補助 11.96 % / 他 7.36 %</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.55 % / 補助 13.77 % / 他 7.64 %</t>
+          <t xml:space="preserve">全社 11.7 % / 補助 13.96 % / 他 7.71 %</t>
         </is>
       </c>
     </row>
@@ -3921,32 +3921,32 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10 % / 補助 11.67 % / 他 8.07 %</t>
+          <t xml:space="preserve">全社 10.01 % / 補助 11.68 % / 他 8.08 %</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.92 % / 補助 11.69 % / 他 7.86 %</t>
+          <t xml:space="preserve">全社 9.93 % / 補助 11.69 % / 他 7.87 %</t>
         </is>
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.81 % / 補助 11.67 % / 他 7.61 %</t>
+          <t xml:space="preserve">全社 9.83 % / 補助 11.68 % / 他 7.65 %</t>
         </is>
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.55 % / 補助 13.61 % / 他 8.77 %</t>
+          <t xml:space="preserve">全社 11.55 % / 補助 13.59 % / 他 8.81 %</t>
         </is>
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.6 % / 補助 14.95 % / 他 8.98 %</t>
+          <t xml:space="preserve">全社 12.68 % / 補助 15.05 % / 他 9.02 %</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.73 % / 補助 16.3 % / 他 9.2 %</t>
+          <t xml:space="preserve">全社 13.88 % / 補助 16.48 % / 他 9.27 %</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
       </c>
       <c r="J10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.63 % / 補助 12 % / 他 11.15 %</t>
+          <t xml:space="preserve">全社 11.64 % / 補助 12 % / 他 11.15 %</t>
         </is>
       </c>
       <c r="K10" s="0" t="inlineStr">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="L10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.93 % / 補助 11 % / 他 10.82 %</t>
+          <t xml:space="preserve">全社 10.93 % / 補助 10.99 % / 他 10.82 %</t>
         </is>
       </c>
     </row>
@@ -4107,32 +4107,32 @@
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.5 % / 補助 7.65 % / 他 11.65 %</t>
+          <t xml:space="preserve">全社 9.5 % / 補助 7.65 % / 他 11.63 %</t>
         </is>
       </c>
       <c r="H12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.67 % / 補助 7.81 % / 他 11.85 %</t>
+          <t xml:space="preserve">全社 9.67 % / 補助 7.81 % / 他 11.84 %</t>
         </is>
       </c>
       <c r="I12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.86 % / 補助 7.97 % / 他 12.09 %</t>
+          <t xml:space="preserve">全社 9.84 % / 補助 7.96 % / 他 12.05 %</t>
         </is>
       </c>
       <c r="J12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.12 % / 補助 6.91 % / 他 12.08 %</t>
+          <t xml:space="preserve">全社 9.1 % / 補助 6.91 % / 他 12.04 %</t>
         </is>
       </c>
       <c r="K12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.73 % / 補助 6.48 % / 他 12.19 %</t>
+          <t xml:space="preserve">全社 8.63 % / 補助 6.34 % / 他 12.15 %</t>
         </is>
       </c>
       <c r="L12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.32 % / 補助 6.07 % / 他 12.31 %</t>
+          <t xml:space="preserve">全社 8.14 % / 補助 5.83 % / 他 12.25 %</t>
         </is>
       </c>
     </row>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.64 % / 補助 0.5 % / 他 0.81 %</t>
+          <t xml:space="preserve">全社 0.64 % / 補助 0.49 % / 他 0.81 %</t>
         </is>
       </c>
       <c r="I13" s="0" t="inlineStr">
@@ -4231,32 +4231,32 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.16 % / 補助 8.15 % / 他 12.48 %</t>
+          <t xml:space="preserve">全社 10.15 % / 補助 8.15 % / 他 12.47 %</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.32 % / 補助 8.3 % / 他 12.67 %</t>
+          <t xml:space="preserve">全社 10.31 % / 補助 8.3 % / 他 12.66 %</t>
         </is>
       </c>
       <c r="I14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.5 % / 補助 8.48 % / 他 12.9 %</t>
+          <t xml:space="preserve">全社 10.48 % / 補助 8.46 % / 他 12.86 %</t>
         </is>
       </c>
       <c r="J14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.69 % / 補助 7.35 % / 他 12.84 %</t>
+          <t xml:space="preserve">全社 9.68 % / 補助 7.35 % / 他 12.8 %</t>
         </is>
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.25 % / 補助 6.86 % / 他 12.94 %</t>
+          <t xml:space="preserve">全社 9.15 % / 補助 6.72 % / 他 12.89 %</t>
         </is>
       </c>
       <c r="L14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.79 % / 補助 6.4 % / 他 13.03 %</t>
+          <t xml:space="preserve">全社 8.61 % / 補助 6.15 % / 他 12.96 %</t>
         </is>
       </c>
     </row>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="J15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.066 億円/人 / 補助 0.065 億円/人 / 他 0.067 億円/人</t>
+          <t xml:space="preserve">全社 0.066 億円/人 / 補助 0.066 億円/人 / 他 0.067 億円/人</t>
         </is>
       </c>
       <c r="K15" s="0" t="inlineStr">
@@ -4417,32 +4417,32 @@
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.34 % / 補助 2.38 % / 他 2.31 %</t>
+          <t xml:space="preserve">全社 2.27 % / 補助 2.38 % / 他 2.19 %</t>
         </is>
       </c>
       <c r="H17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.67 % / 補助 1.78 % / 他 1.6 %</t>
+          <t xml:space="preserve">全社 1.68 % / 補助 1.78 % / 他 1.61 %</t>
         </is>
       </c>
       <c r="I17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.03 % / 補助 2.12 % / 他 1.98 %</t>
+          <t xml:space="preserve">全社 2.25 % / 補助 1.98 % / 他 2.47 %</t>
         </is>
       </c>
       <c r="J17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.93 % / 補助 1.42 % / 他 2.32 %</t>
+          <t xml:space="preserve">全社 2.73 % / 補助 3.25 % / 他 2.31 %</t>
         </is>
       </c>
       <c r="K17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5.8 % / 補助 9.93 % / 他 2.63 %</t>
+          <t xml:space="preserve">全社 5.08 % / 補助 8.41 % / 他 2.53 %</t>
         </is>
       </c>
       <c r="L17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6 % / 補助 9.94 % / 他 2.78 %</t>
+          <t xml:space="preserve">全社 5.25 % / 補助 9.44 % / 他 2 %</t>
         </is>
       </c>
     </row>
@@ -4479,32 +4479,32 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 50.39 % / 補助 41.11 % / 他 60.73 %</t>
+          <t xml:space="preserve">全社 50.35 % / 補助 41.09 % / 他 60.67 %</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 50.97 % / 補助 41.53 % / 他 61.72 %</t>
+          <t xml:space="preserve">全社 50.94 % / 補助 41.53 % / 他 61.65 %</t>
         </is>
       </c>
       <c r="I18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 51.71 % / 補助 42.08 % / 他 62.88 %</t>
+          <t xml:space="preserve">全社 51.59 % / 補助 42.02 % / 他 62.69 %</t>
         </is>
       </c>
       <c r="J18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 45.63 % / 補助 35.06 % / 他 59.4 %</t>
+          <t xml:space="preserve">全社 45.58 % / 補助 35.09 % / 他 59.24 %</t>
         </is>
       </c>
       <c r="K18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 42.33 % / 補助 31.45 % / 他 59.03 %</t>
+          <t xml:space="preserve">全社 41.91 % / 補助 30.86 % / 他 58.83 %</t>
         </is>
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 39.03 % / 補助 28.19 % / 他 58.61 %</t>
+          <t xml:space="preserve">全社 38.28 % / 補助 27.17 % / 他 58.31 %</t>
         </is>
       </c>
     </row>
@@ -4613,22 +4613,22 @@
       </c>
       <c r="I20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.655 億円/人 / 補助 0.801 億円/人 / 他 0.54 億円/人</t>
+          <t xml:space="preserve">全社 0.658 億円/人 / 補助 0.801 億円/人 / 他 0.543 億円/人</t>
         </is>
       </c>
       <c r="J20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.723 億円/人 / 補助 0.937 億円/人 / 他 0.553 億円/人</t>
+          <t xml:space="preserve">全社 0.731 億円/人 / 補助 0.953 億円/人 / 他 0.556 億円/人</t>
         </is>
       </c>
       <c r="K20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.798 億円/人 / 補助 1.098 億円/人 / 他 0.562 億円/人</t>
+          <t xml:space="preserve">全社 0.81 億円/人 / 補助 1.125 億円/人 / 他 0.565 億円/人</t>
         </is>
       </c>
       <c r="L20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.887 億円/人 / 補助 1.289 億円/人 / 他 0.572 億円/人</t>
+          <t xml:space="preserve">全社 0.903 億円/人 / 補助 1.34 億円/人 / 他 0.572 億円/人</t>
         </is>
       </c>
     </row>
@@ -4675,22 +4675,22 @@
       </c>
       <c r="I21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.042 億円/人 / 補助 0.057 億円/人 / 他 0.031 億円/人</t>
+          <t xml:space="preserve">全社 0.043 億円/人 / 補助 0.057 億円/人 / 他 0.031 億円/人</t>
         </is>
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.062 億円/人 / 補助 0.092 億円/人 / 他 0.039 億円/人</t>
+          <t xml:space="preserve">全社 0.063 億円/人 / 補助 0.094 億円/人 / 他 0.039 億円/人</t>
         </is>
       </c>
       <c r="K21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.08 億円/人 / 補助 0.13 億円/人 / 他 0.041 億円/人</t>
+          <t xml:space="preserve">全社 0.082 億円/人 / 補助 0.135 億円/人 / 他 0.042 億円/人</t>
         </is>
       </c>
       <c r="L21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.103 億円/人 / 補助 0.177 億円/人 / 他 0.044 億円/人</t>
+          <t xml:space="preserve">全社 0.106 億円/人 / 補助 0.187 億円/人 / 他 0.044 億円/人</t>
         </is>
       </c>
     </row>
@@ -4737,22 +4737,22 @@
       </c>
       <c r="I22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.131 億円/人 / 補助 0.159 億円/人 / 他 0.108 億円/人</t>
+          <t xml:space="preserve">全社 0.131 億円/人 / 補助 0.159 億円/人 / 他 0.109 億円/人</t>
         </is>
       </c>
       <c r="J22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.151 億円/人 / 補助 0.193 億円/人 / 他 0.117 億円/人</t>
+          <t xml:space="preserve">全社 0.152 億円/人 / 補助 0.196 億円/人 / 他 0.118 億円/人</t>
         </is>
       </c>
       <c r="K22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.171 億円/人 / 補助 0.236 億円/人 / 他 0.121 億円/人</t>
+          <t xml:space="preserve">全社 0.174 億円/人 / 補助 0.241 億円/人 / 他 0.122 億円/人</t>
         </is>
       </c>
       <c r="L22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.197 億円/人 / 補助 0.288 億円/人 / 他 0.125 億円/人</t>
+          <t xml:space="preserve">全社 0.2 億円/人 / 補助 0.299 億円/人 / 他 0.125 億円/人</t>
         </is>
       </c>
     </row>
@@ -4799,22 +4799,22 @@
       </c>
       <c r="I23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.76 % / 補助 5.41 % / 他 4.26 %</t>
+          <t xml:space="preserve">全社 4.37 % / 補助 5.41 % / 他 3.55 %</t>
         </is>
       </c>
       <c r="J23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.55 % / 補助 4.27 % / 他 4.76 %</t>
+          <t xml:space="preserve">全社 3.8 % / 補助 2.56 % / 他 4.79 %</t>
         </is>
       </c>
       <c r="K23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.35 % / 補助 4.1 % / 他 4.55 %</t>
+          <t xml:space="preserve">全社 4.03 % / 補助 3.33 % / 他 4.58 %</t>
         </is>
       </c>
       <c r="L23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.17 % / 補助 3.94 % / 他 4.35 %</t>
+          <t xml:space="preserve">全社 3.87 % / 補助 2.42 % / 他 5 %</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.52 pt / 補助 0.4 pt / 他 0.41 pt</t>
+          <t xml:space="preserve">全社 0.53 pt / 補助 0.41 pt / 他 0.41 pt</t>
         </is>
       </c>
       <c r="H24" s="0" t="inlineStr">
@@ -4861,22 +4861,22 @@
       </c>
       <c r="I24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.11 pt / 補助 -0 pt / 他 0 pt</t>
+          <t xml:space="preserve">全社 0.51 pt / 補助 0.01 pt / 他 0.71 pt</t>
         </is>
       </c>
       <c r="J24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.72 pt / 補助 17.73 pt / 他 2.55 pt</t>
+          <t xml:space="preserve">全社 11.48 pt / 補助 19.46 pt / 他 2.52 pt</t>
         </is>
       </c>
       <c r="K24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.93 pt / 補助 17.9 pt / 他 1.7 pt</t>
+          <t xml:space="preserve">全社 11.26 pt / 補助 18.68 pt / 他 1.67 pt</t>
         </is>
       </c>
       <c r="L24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.64 pt / 補助 18.07 pt / 他 1.91 pt</t>
+          <t xml:space="preserve">全社 11.96 pt / 補助 19.61 pt / 他 1.27 pt</t>
         </is>
       </c>
     </row>
@@ -4975,7 +4975,7 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.71 % / 補助 3.29 % / 他 2.06 %</t>
+          <t xml:space="preserve">全社 2.71 % / 補助 3.28 % / 他 2.06 %</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
@@ -5161,32 +5161,32 @@
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.68 倍 / 補助 3.55 倍 / 他 3.93 倍</t>
+          <t xml:space="preserve">全社 3.69 倍 / 補助 3.56 倍 / 他 3.93 倍</t>
         </is>
       </c>
       <c r="H29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.25 倍 / 補助 2.94 倍 / 他 3.99 倍</t>
+          <t xml:space="preserve">全社 3.26 倍 / 補助 2.94 倍 / 他 3.99 倍</t>
         </is>
       </c>
       <c r="I29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.93 倍 / 補助 2.54 倍 / 他 4.03 倍</t>
+          <t xml:space="preserve">全社 2.93 倍 / 補助 2.54 倍 / 他 4.05 倍</t>
         </is>
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.97 倍 / 補助 3.62 倍 / 他 4.98 倍</t>
+          <t xml:space="preserve">全社 3.97 倍 / 補助 3.61 倍 / 他 5 倍</t>
         </is>
       </c>
       <c r="K29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.99 倍 / 補助 4.85 倍 / 他 5.41 倍</t>
+          <t xml:space="preserve">全社 5.03 倍 / 補助 4.88 倍 / 他 5.44 倍</t>
         </is>
       </c>
       <c r="L29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.3 倍 / 補助 6.45 倍 / 他 5.89 倍</t>
+          <t xml:space="preserve">全社 6.37 倍 / 補助 6.53 倍 / 他 5.94 倍</t>
         </is>
       </c>
     </row>
@@ -5347,7 +5347,7 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 53.6 %</t>
+          <t xml:space="preserve">構成比 53.61 %</t>
         </is>
       </c>
       <c r="H32" s="0" t="inlineStr">
@@ -5362,17 +5362,17 @@
       </c>
       <c r="J32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 57.31 %</t>
+          <t xml:space="preserve">構成比 57.32 %</t>
         </is>
       </c>
       <c r="K32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 60.65 %</t>
+          <t xml:space="preserve">構成比 60.67 %</t>
         </is>
       </c>
       <c r="L32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 63.9 %</t>
+          <t xml:space="preserve">構成比 63.91 %</t>
         </is>
       </c>
     </row>
@@ -5409,7 +5409,7 @@
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 5.4 % / 他 4.26 %</t>
+          <t xml:space="preserve">補助 5.41 % / 他 4.26 %</t>
         </is>
       </c>
       <c r="H33" s="0" t="inlineStr">
@@ -5419,22 +5419,22 @@
       </c>
       <c r="I33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 5.4 % / 他 4.26 %</t>
+          <t xml:space="preserve">補助 5.41 % / 他 4.26 %</t>
         </is>
       </c>
       <c r="J33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 22 % / 他 7.31 %</t>
+          <t xml:space="preserve">補助 22.03 % / 他 7.31 %</t>
         </is>
       </c>
       <c r="K33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 22 % / 他 6.25 %</t>
+          <t xml:space="preserve">補助 22.01 % / 他 6.25 %</t>
         </is>
       </c>
       <c r="L33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 22 % / 他 6.26 %</t>
+          <t xml:space="preserve">補助 22.03 % / 他 6.27 %</t>
         </is>
       </c>
     </row>
@@ -5471,32 +5471,32 @@
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">差 -0.01 pt</t>
+        </is>
+      </c>
+      <c r="H34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">差 0.01 pt</t>
+        </is>
+      </c>
+      <c r="I34" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">差 -0 pt</t>
         </is>
       </c>
-      <c r="H34" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">差 0 pt</t>
-        </is>
-      </c>
-      <c r="I34" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">差 -0.01 pt</t>
-        </is>
-      </c>
       <c r="J34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 0.31 pt</t>
+          <t xml:space="preserve">差 0.33 pt</t>
         </is>
       </c>
       <c r="K34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -0.04 pt</t>
+          <t xml:space="preserve">差 -0 pt</t>
         </is>
       </c>
       <c r="L34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -0.4 pt</t>
+          <t xml:space="preserve">差 -0.33 pt</t>
         </is>
       </c>
     </row>
@@ -5538,27 +5538,27 @@
       </c>
       <c r="H35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 1.83 pt</t>
+          <t xml:space="preserve">差 1.82 pt</t>
         </is>
       </c>
       <c r="I35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 1.35 pt</t>
+          <t xml:space="preserve">差 1.33 pt</t>
         </is>
       </c>
       <c r="J35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 2.84 pt</t>
+          <t xml:space="preserve">差 2.78 pt</t>
         </is>
       </c>
       <c r="K35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 4.54 pt</t>
+          <t xml:space="preserve">差 4.6 pt</t>
         </is>
       </c>
       <c r="L35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 6.13 pt</t>
+          <t xml:space="preserve">差 6.25 pt</t>
         </is>
       </c>
     </row>
@@ -5605,22 +5605,22 @@
       </c>
       <c r="I36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.801 億円/人 / 他 0.54 億円/人</t>
+          <t xml:space="preserve">補助 0.801 億円/人 / 他 0.543 億円/人</t>
         </is>
       </c>
       <c r="J36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.937 億円/人 / 他 0.553 億円/人</t>
+          <t xml:space="preserve">補助 0.953 億円/人 / 他 0.556 億円/人</t>
         </is>
       </c>
       <c r="K36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.098 億円/人 / 他 0.562 億円/人</t>
+          <t xml:space="preserve">補助 1.125 億円/人 / 他 0.565 億円/人</t>
         </is>
       </c>
       <c r="L36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.289 億円/人 / 他 0.572 億円/人</t>
+          <t xml:space="preserve">補助 1.34 億円/人 / 他 0.572 億円/人</t>
         </is>
       </c>
     </row>
@@ -5672,7 +5672,7 @@
       </c>
       <c r="J37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.065 億円/人 / 他 0.067 億円/人</t>
+          <t xml:space="preserve">補助 0.066 億円/人 / 他 0.067 億円/人</t>
         </is>
       </c>
       <c r="K37" s="0" t="inlineStr">
@@ -5719,32 +5719,32 @@
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 164.29 %</t>
+          <t xml:space="preserve">寄与率 183.33 %</t>
         </is>
       </c>
       <c r="H38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 175 %</t>
+          <t xml:space="preserve">寄与率 169.23 %</t>
         </is>
       </c>
       <c r="I38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 135.29 %</t>
+          <t xml:space="preserve">寄与率 157.14 %</t>
         </is>
       </c>
       <c r="J38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 76.4 %</t>
+          <t xml:space="preserve">寄与率 76.29 %</t>
         </is>
       </c>
       <c r="K38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 89.04 %</t>
+          <t xml:space="preserve">寄与率 89.2 %</t>
         </is>
       </c>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 90.53 %</t>
+          <t xml:space="preserve">寄与率 90.41 %</t>
         </is>
       </c>
     </row>
@@ -9855,7 +9855,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4fX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjU5LCJvZmZpY2VyUGF5IjowLjM4LCJkZXByZWNpYXRpb24iOjEuOSwib3RoZXJTZ2EiOjkuNSwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NS4zMSwiZW1wbG95ZWVCb251cyI6MC4yOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNCwib2ZmaWNlckJvbnVzIjowLjA0LCJjb2dzRGVwcmVjaWF0aW9uIjowLjQ3LCJzZ2FEZXByZWNpYXRpb24iOjEuNDMsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMzh9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNTQsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3LjE2LCJlbXBsb3llZUJvbnVzIjowLjM4LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjUyLCJvZmZpY2VyQm9udXMiOjAuMDYsImNvZ3NEZXByZWNpYXRpb24iOjAuMjksInNnYURlcHJlY2lhdGlvbiI6MS4xNSwicmVzZWFyY2hEZXZlbG9wbWVudCI6MC4yOX19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6NiwiZW1wbG95ZWVTYWxhcnkiOjUuNywiZW1wbG95ZWVCb251cyI6MC4zLCJvZmZpY2VyUGF5IjowLjQsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzYsIm9mZmljZXJCb251cyI6MC4wNCwiZGVwcmVjaWF0aW9uIjoyLCJjb2dzRGVwcmVjaWF0aW9uIjowLjUsInNnYURlcHJlY2lhdGlvbiI6MS41LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjQsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsImVtcGxveWVlU2FsYXJ5Ijo3LjYsImVtcGxveWVlQm9udXMiOjAuNCwib2ZmaWNlclBheSI6MC42LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjU0LCJvZmZpY2VyQm9udXMiOjAuMDYsImRlcHJlY2lhdGlvbiI6MS41LCJjb2dzRGVwcmVjaWF0aW9uIjowLjMsInNnYURlcHJlY2lhdGlvbiI6MS4yLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjMsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMSwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI4NTcxNDI4NTcxNDI4LCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwidXNlZnVsTGlmZSI6MTAsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwxLjY2NTMzNDUzNjkzNzczNDhlLTE2XSwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MzI1MzMwNTAxODQ2OTI3LDAuMDIwNzM1OTk0MTgzMTg5MTY2XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDBdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNDA3NjA4Njk1NjUyMTcxODQsMC4wNDQzODQwNTc5NzEwMTQ1Ml0sIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAwMDEzNDU3NTU2OTM1ODE5NzM3XSwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOlswLjAxOTEzOTQ1NzAyMzcxNzQ0MywwLjAyMDU1MzQ1OTkxNDc2MzA5NV0sIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wMzkxNjY2NjY2NjY2NjY2OCwwLjA0MjUwMDAwMDAwMDAwMDA5XSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RTYWxlc0dyb3d0aCI6WzAuMTUsMC4zXSwib3RoZXJTYWxlc0dyb3d0aCI6WzAuMDYwNzYwODY5NTY1MjE3MTksMC4wNjQzODQwNTc5NzEwMTQ1M10sInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOlswLDAuMDNdLCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6WzAuMDA1LDAuMDA1MTM0NTc1NTY5MzU4MTk3NV0sInByb2plY3RQYXlHcm93dGgiOlswLjA1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMC4wMjQxMzk0NTcwMjM3MTc0NDQsMC4wMjU1NTM0NTk5MTQ3NjMwOTZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGgiOlswLjA0NDE2NjY2NjY2NjY2NjY4LDAuMDQ3NTAwMDAwMDAwMDAwMDldLCJwcm9qZWN0U2dhUmF0ZUVuZCI6WzAuMDg0OTk5OTk5OTk5OTk5OTksMC4xMzVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA4OTI4NTcxNDI4NTcxNDI3LDAuMTE5Mjg1NzE0Mjg1NzE0MjddLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAuMDQyNjMxNTc4OTQ3MzY4MzYsMC4wNjU1NTU1NTU1NTU1NTU1OF0sInVzZWZ1bExpZmUiOls1LDIwXSwiaW52ZXN0bWVudCI6WzE1LDIwMF0sInN1YnNpZHkiOlsxLDUwXSwibG9jYWxCZW5jaG1hcmsiOlswLDEwMF19LCJ0YXJnZXRzIjp7ImNvbXBhbnlTYWxlc0NhZ3IiOnsidmFsdWUiOjE1LCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjgyLjQsIm1heCI6MjUyLjY5LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjoyLCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NjAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo3NC44LCJtYXgiOjEzNi44NCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImxhYm9yUHJvZHVjdGl2aXR5Q2FnciI6eyJ2YWx1ZSI6MjEsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkSW5jcmVhc2UiOnsidmFsdWUiOjE4Ljc4LCJtYXgiOjMzLjQzLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6Mi44NSwibWF4IjozLjc0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiaW52ZXN0bWVudFNhbGVzUmF0aW8iOnsidmFsdWUiOjE1LCJtYXgiOjcwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZFN1YnNpZHlSYXRpbyI6eyJ2YWx1ZSI6MjEzLCJtYXgiOjM1MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImxvY2FsQmVuY2htYXJrIjp7InZhbHVlIjoyMywibWF4Ijo0MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlDYWdyIjp7InZhbHVlIjo2LCJtYXgiOjEwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUluY3JlYXNlIjp7InZhbHVlIjowLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfX0sImZvcmVjYXN0T3ZlcnJpZGVzIjp7IjIwMjk6b3RoZXI6c2FsZXMiOjg1LjEzLCIyMDI5OnByb2plY3Q6Ny04Ijo3Ljl9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2LjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mi43NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTQiOjAuNzMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi03IjozMi42NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTkiOjAuODIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMCI6MC4wOSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEyIjoxMS42NywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEzIjowLjYyLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTQiOjIuNDUsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNSI6MC42NCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEiOjcyLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNCI6MjMuMDQsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny02Ijo2Ljc4LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOCI6NS4xOSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTkiOjAuMzYsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMCI6MS44LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTMiOjkwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xIjoxNDMuMiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTMiOjk3LjM4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNCI6MC43NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTciOjM0LjUyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItOSI6MC44NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMiI6MTIuNDcsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMyI6MC42NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjoyLjU4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTUiOjAuNjcsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xIjo3NiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0LjMyLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNiI6Ny4wNCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTgiOjUuNTksImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTAiOjEuOSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6MC44LCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTkiOjAuOSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjowLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6Mi43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTUiOjAuNywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNCI6MjUuNiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTYiOjcuMywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTgiOjYsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny05IjowLjQsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xMCI6MiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudEFzc2V0cyI6NjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXNoIjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NSwiYmFsYW5jZS1zaGVldDoyMDIzOnRhbmdpYmxlQXNzZXRzIjo1MywiYmFsYW5jZS1zaGVldDoyMDIzOmJ1aWxkaW5ncyI6MTksImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzppbnRhbmdpYmxlQXNzZXRzIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUsImJhbGFuY2Utc2hlZXQ6MjAyMzpsaWFiaWxpdGllcyI6NzUsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50TGlhYmlsaXRpZXMiOjM5LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZExpYWJpbGl0aWVzIjozNiwiYmFsYW5jZS1zaGVldDoyMDIzOmxvbmdUZXJtRGVidCI6MjksImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hhcmVob2xkZXJFcXVpdHkiOjU0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NSwiYmFsYW5jZS1zaGVldDoyMDI0OmFzc2V0cyI6MTQzLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudEFzc2V0cyI6NzIsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNSwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkQXNzZXRzIjo3MSwiYmFsYW5jZS1zaGVldDoyMDI0OnRhbmdpYmxlQXNzZXRzIjo1OCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAsImJhbGFuY2Utc2hlZXQ6MjAyNDptYWNoaW5lcnkiOjI4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c29mdHdhcmUiOjYsImJhbGFuY2Utc2hlZXQ6MjAyNDpsaWFiaWxpdGllcyI6NzksImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZExpYWJpbGl0aWVzIjozOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEsImJhbGFuY2Utc2hlZXQ6MjAyNDpuZXRBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hhcmVob2xkZXJFcXVpdHkiOjYxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBleCI6OCwiYmFsYW5jZS1zaGVldDoyMDI1OmFzc2V0cyI6MTU2LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXNoIjoyNywiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkQXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI1OmJ1aWxkaW5ncyI6MjIsImJhbGFuY2Utc2hlZXQ6MjAyNTptYWNoaW5lcnkiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTppbnRhbmdpYmxlQXNzZXRzIjo5LCJiYWxhbmNlLXNoZWV0OjIwMjU6c29mdHdhcmUiOjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hvcnRUZXJtRGVidCI6MTEsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MCwiYmFsYW5jZS1zaGVldDoyMDI1OmxvbmdUZXJtRGVidCI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpuZXRBc3NldHMiOjczLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBleCI6MTAsImZ1dHVyZS1jYXBleDoyMDI2IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjciOjE1LCJmdXR1cmUtY2FwZXg6MjAyOCI6MTUsImZ1dHVyZS1jYXBleDoyMDI5IjowLCJmdXR1cmUtY2FwZXg6MjAzMCI6MCwiZnV0dXJlLWNhcGV4OjIwMzEiOjAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjEuNjY1MzM0NTM2OTM3NzM0OGUtMTYsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkzMjUzMzA1MDE4NDY5MjcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNzM1OTk0MTgzMTg5MTY2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLjAxOTEzOTQ1NzAyMzcxNzQ0MywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNTUzNDU5OTE0NzYzMDk1LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjAzOTE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNDI1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MCI6MC4xNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjMsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MCI6MC4wMjQxMzk0NTcwMjM3MTc0NDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDoxIjowLjAyNTU1MzQ1OTkxNDc2MzA5NiwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjowLjA0NDE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MSI6MC4wNDc1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjExLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MCI6MC4wODQ5OTk5OTk5OTk5OTk5OSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjEiOjAuMTM1LCJkcml2ZXI6b3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI4NTcxNDI4NTcxNDI4LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjAiOjAuMDg5Mjg1NzE0Mjg1NzE0MjcsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MSI6MC4xMTkyODU3MTQyODU3MTQyNywiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MCI6MC4wNDI2MzE1Nzg5NDczNjgzNiwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjEiOjAuMDY1NTU1NTU1NTU1NTU1NTgsImRyaXZlcjp1c2VmdWxMaWZlIjoxMCwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MCI6NSwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MSI6MjAsImRyaXZlcjppbnZlc3RtZW50IjoyMywiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjEiOjIwMCwiZHJpdmVyOnN1YnNpZHkiOjcuNjYsImRyaXZlci1yYW5nZTpzdWJzaWR5OjAiOjEsImRyaXZlci1yYW5nZTpzdWJzaWR5OjEiOjUwLCJkcml2ZXI6bG9jYWxCZW5jaG1hcmsiOjIzLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MCI6MCwiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjEiOjEwMCwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6dmFsdWUiOjE1LCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6dmFsdWUiOjgyLjQsInRhcmdldDpjb21wYW55UGF5U2NoZWR1bGU6dmFsdWUiOjIsInRhcmdldDpjb21wYW55UGF5U2NoZWR1bGU6bWF4Ijo3LCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6dmFsdWUiOjYwLCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6bWF4Ijo5NSwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6dmFsdWUiOjIyLCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6dmFsdWUiOjc0LjgsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6dmFsdWUiOjIxLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOm1heCI6MzUsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6dmFsdWUiOjE4Ljc4LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOnZhbHVlIjo3LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOm1heCI6MTAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOnZhbHVlIjoyLjg1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86dmFsdWUiOjE1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86bWF4Ijo3MCwidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86dmFsdWUiOjIxMywidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86bWF4IjozNTAsInRhcmdldDpsb2NhbEJlbmNobWFyazp2YWx1ZSI6MjMsInRhcmdldDpsb2NhbEJlbmNobWFyazptYXgiOjQwLCJ0YXJnZXQ6b2ZmaWNlclBheUNhZ3I6dmFsdWUiOjYsInRhcmdldDpvZmZpY2VyUGF5Q2FncjptYXgiOjEwLCJ0YXJnZXQ6b2ZmaWNlclBheUluY3JlYXNlOnZhbHVlIjowLCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6bWF4IjoyNTIuNjksInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTptYXgiOjEzNi44NCwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTptYXgiOjMzLjQzLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlJbmNyZWFzZTptYXgiOjMuNzR9LCJtZXRyaWNHcm91cEJhc2VzIjp7ImNvbXBhbnlTYWxlcyI6InJhdGUiLCJwcm9qZWN0U2FsZXMiOiJyYXRlIiwibGFib3JQcm9kdWN0aXZpdHkiOiJyYXRlIiwiZW1wbG95ZWVQYXkiOiJyYXRlIn0sImFwcGxpY2F0aW9uQ2F0ZWdvcnkiOiJnZW5lcmFsIiwiYWRqdXN0ZWREcml2ZXJzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQwMzY4MDU1NTU1NTU1NCwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MS4xNzQxODY0OTEwNjQ0NjZlLTE2LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAxOTgxNjI4NzE3ODg3NywicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQ0NDg1MzYzMDY3NTMyNzQsInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDYwOTMzNzAyNzg5ODA0LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjYwNzMxNjU4MzkyMjQ5LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODA5MDU5NTA0NjA1NjYzLCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDE0OTM3NzcyNDkzMDY0NDYsIm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMiwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NDAxODU3MDcyNjUyNiwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTU1NTA0MjcyNTc5NzcyODQsIm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwicHJvamVjdFBheUdyb3d0aCI6MC4xLCJvdGhlclBheUdyb3d0aCI6MC4wMjU1NTM0NTk5MTQ3NjMwOTYsInByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTg3MjM3NjkyMTM2MzM4LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMSwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTMyNjE2NDY1MTYzNjYsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgxOTIzMTY3OTU4MzQ5NiwidXNlZnVsTGlmZSI6MTAsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9fQ==</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4fX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjU5LCJvZmZpY2VyUGF5IjowLjM4LCJkZXByZWNpYXRpb24iOjEuOSwib3RoZXJTZ2EiOjkuNSwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NS4zMSwiZW1wbG95ZWVCb251cyI6MC4yOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNCwib2ZmaWNlckJvbnVzIjowLjA0LCJjb2dzRGVwcmVjaWF0aW9uIjowLjQ3LCJzZ2FEZXByZWNpYXRpb24iOjEuNDMsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMzh9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNTQsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3LjE2LCJlbXBsb3llZUJvbnVzIjowLjM4LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjUyLCJvZmZpY2VyQm9udXMiOjAuMDYsImNvZ3NEZXByZWNpYXRpb24iOjAuMjksInNnYURlcHJlY2lhdGlvbiI6MS4xNSwicmVzZWFyY2hEZXZlbG9wbWVudCI6MC4yOX19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6NiwiZW1wbG95ZWVTYWxhcnkiOjUuNywiZW1wbG95ZWVCb251cyI6MC4zLCJvZmZpY2VyUGF5IjowLjQsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzYsIm9mZmljZXJCb251cyI6MC4wNCwiZGVwcmVjaWF0aW9uIjoyLCJjb2dzRGVwcmVjaWF0aW9uIjowLjUsInNnYURlcHJlY2lhdGlvbiI6MS41LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjQsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsImVtcGxveWVlU2FsYXJ5Ijo3LjYsImVtcGxveWVlQm9udXMiOjAuNCwib2ZmaWNlclBheSI6MC42LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjU0LCJvZmZpY2VyQm9udXMiOjAuMDYsImRlcHJlY2lhdGlvbiI6MS41LCJjb2dzRGVwcmVjaWF0aW9uIjowLjMsInNnYURlcHJlY2lhdGlvbiI6MS4yLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjMsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMSwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI4NTcxNDI4NTcxNDI4LCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwidXNlZnVsTGlmZSI6MTAsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwxLjY2NTMzNDUzNjkzNzczNDhlLTE2XSwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MzI1MzMwNTAxODQ2OTI3LDAuMDIwNzM1OTk0MTgzMTg5MTY2XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDBdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNDA3NjA4Njk1NjUyMTcxODQsMC4wNDQzODQwNTc5NzEwMTQ1Ml0sIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAwMDEzNDU3NTU2OTM1ODE5NzM3XSwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOlswLjAxOTEzOTQ1NzAyMzcxNzQ0MywwLjAyMDU1MzQ1OTkxNDc2MzA5NV0sIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wMzkxNjY2NjY2NjY2NjY2OCwwLjA0MjUwMDAwMDAwMDAwMDA5XSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RTYWxlc0dyb3d0aCI6WzAuMTUsMC4zXSwib3RoZXJTYWxlc0dyb3d0aCI6WzAuMDYwNzYwODY5NTY1MjE3MTksMC4wNjQzODQwNTc5NzEwMTQ1M10sInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOlswLDAuMDNdLCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6WzAuMDA1LDAuMDA1MTM0NTc1NTY5MzU4MTk3NV0sInByb2plY3RQYXlHcm93dGgiOlswLjA1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMC4wMjQxMzk0NTcwMjM3MTc0NDQsMC4wMjU1NTM0NTk5MTQ3NjMwOTZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGgiOlswLjA0NDE2NjY2NjY2NjY2NjY4LDAuMDQ3NTAwMDAwMDAwMDAwMDldLCJwcm9qZWN0U2dhUmF0ZUVuZCI6WzAuMDg0OTk5OTk5OTk5OTk5OTksMC4xMzVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA4OTI4NTcxNDI4NTcxNDI3LDAuMTE5Mjg1NzE0Mjg1NzE0MjddLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAuMDQyNjMxNTc4OTQ3MzY4MzYsMC4wNjU1NTU1NTU1NTU1NTU1OF0sInVzZWZ1bExpZmUiOls1LDIwXSwiaW52ZXN0bWVudCI6WzE1LDIwMF0sInN1YnNpZHkiOlsxLDUwXSwibG9jYWxCZW5jaG1hcmsiOlswLDEwMF19LCJ0YXJnZXRzIjp7ImNvbXBhbnlTYWxlc0NhZ3IiOnsidmFsdWUiOjE1LCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjgyLjQsIm1heCI6MjUyLjY5LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjoyLCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NjAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo3NC44LCJtYXgiOjEzNi44NCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImxhYm9yUHJvZHVjdGl2aXR5Q2FnciI6eyJ2YWx1ZSI6MjEsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkSW5jcmVhc2UiOnsidmFsdWUiOjE4Ljc4LCJtYXgiOjMzLjQzLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6Mi44NSwibWF4IjozLjc0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiaW52ZXN0bWVudFNhbGVzUmF0aW8iOnsidmFsdWUiOjE1LCJtYXgiOjcwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZFN1YnNpZHlSYXRpbyI6eyJ2YWx1ZSI6MjEzLCJtYXgiOjM1MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImxvY2FsQmVuY2htYXJrIjp7InZhbHVlIjoyMywibWF4Ijo0MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlDYWdyIjp7InZhbHVlIjo2LCJtYXgiOjEwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUluY3JlYXNlIjp7InZhbHVlIjowLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfX0sImZvcmVjYXN0T3ZlcnJpZGVzIjp7IjIwMjk6b3RoZXI6c2FsZXMiOjg1LjEzLCIyMDI5OnByb2plY3Q6Ny04Ijo3Ljl9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2LjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mi43NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTQiOjAuNzMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi03IjozMi42NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTkiOjAuODIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMCI6MC4wOSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEyIjoxMS42NywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEzIjowLjYyLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTQiOjIuNDUsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNSI6MC42NCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEiOjcyLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNCI6MjMuMDQsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny02Ijo2Ljc4LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOCI6NS4xOSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTkiOjAuMzYsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMCI6MS44LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTMiOjkwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xIjoxNDMuMiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTMiOjk3LjM4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNCI6MC43NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTciOjM0LjUyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItOSI6MC44NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMiI6MTIuNDcsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMyI6MC42NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjoyLjU4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTUiOjAuNjcsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xIjo3NiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0LjMyLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNiI6Ny4wNCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTgiOjUuNTksImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTAiOjEuOSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6MC44LCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTkiOjAuOSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjowLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6Mi43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTUiOjAuNywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNCI6MjUuNiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTYiOjcuMywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTgiOjYsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny05IjowLjQsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xMCI6MiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudEFzc2V0cyI6NjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXNoIjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NSwiYmFsYW5jZS1zaGVldDoyMDIzOnRhbmdpYmxlQXNzZXRzIjo1MywiYmFsYW5jZS1zaGVldDoyMDIzOmJ1aWxkaW5ncyI6MTksImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzppbnRhbmdpYmxlQXNzZXRzIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUsImJhbGFuY2Utc2hlZXQ6MjAyMzpsaWFiaWxpdGllcyI6NzUsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50TGlhYmlsaXRpZXMiOjM5LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZExpYWJpbGl0aWVzIjozNiwiYmFsYW5jZS1zaGVldDoyMDIzOmxvbmdUZXJtRGVidCI6MjksImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hhcmVob2xkZXJFcXVpdHkiOjU0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NSwiYmFsYW5jZS1zaGVldDoyMDI0OmFzc2V0cyI6MTQzLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudEFzc2V0cyI6NzIsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNSwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkQXNzZXRzIjo3MSwiYmFsYW5jZS1zaGVldDoyMDI0OnRhbmdpYmxlQXNzZXRzIjo1OCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAsImJhbGFuY2Utc2hlZXQ6MjAyNDptYWNoaW5lcnkiOjI4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c29mdHdhcmUiOjYsImJhbGFuY2Utc2hlZXQ6MjAyNDpsaWFiaWxpdGllcyI6NzksImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZExpYWJpbGl0aWVzIjozOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEsImJhbGFuY2Utc2hlZXQ6MjAyNDpuZXRBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hhcmVob2xkZXJFcXVpdHkiOjYxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBleCI6OCwiYmFsYW5jZS1zaGVldDoyMDI1OmFzc2V0cyI6MTU2LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXNoIjoyNywiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkQXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI1OmJ1aWxkaW5ncyI6MjIsImJhbGFuY2Utc2hlZXQ6MjAyNTptYWNoaW5lcnkiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTppbnRhbmdpYmxlQXNzZXRzIjo5LCJiYWxhbmNlLXNoZWV0OjIwMjU6c29mdHdhcmUiOjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hvcnRUZXJtRGVidCI6MTEsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MCwiYmFsYW5jZS1zaGVldDoyMDI1OmxvbmdUZXJtRGVidCI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpuZXRBc3NldHMiOjczLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBleCI6MTAsImZ1dHVyZS1jYXBleDoyMDI2IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjciOjE1LCJmdXR1cmUtY2FwZXg6MjAyOCI6MTUsImZ1dHVyZS1jYXBleDoyMDI5IjowLCJmdXR1cmUtY2FwZXg6MjAzMCI6MCwiZnV0dXJlLWNhcGV4OjIwMzEiOjAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjEuNjY1MzM0NTM2OTM3NzM0OGUtMTYsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkzMjUzMzA1MDE4NDY5MjcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNzM1OTk0MTgzMTg5MTY2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLjAxOTEzOTQ1NzAyMzcxNzQ0MywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNTUzNDU5OTE0NzYzMDk1LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjAzOTE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNDI1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MCI6MC4xNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjMsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MCI6MC4wMjQxMzk0NTcwMjM3MTc0NDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDoxIjowLjAyNTU1MzQ1OTkxNDc2MzA5NiwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjowLjA0NDE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MSI6MC4wNDc1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjExLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MCI6MC4wODQ5OTk5OTk5OTk5OTk5OSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjEiOjAuMTM1LCJkcml2ZXI6b3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI4NTcxNDI4NTcxNDI4LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjAiOjAuMDg5Mjg1NzE0Mjg1NzE0MjcsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MSI6MC4xMTkyODU3MTQyODU3MTQyNywiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MCI6MC4wNDI2MzE1Nzg5NDczNjgzNiwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjEiOjAuMDY1NTU1NTU1NTU1NTU1NTgsImRyaXZlcjp1c2VmdWxMaWZlIjoxMCwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MCI6NSwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MSI6MjAsImRyaXZlcjppbnZlc3RtZW50IjoyMywiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjEiOjIwMCwiZHJpdmVyOnN1YnNpZHkiOjcuNjYsImRyaXZlci1yYW5nZTpzdWJzaWR5OjAiOjEsImRyaXZlci1yYW5nZTpzdWJzaWR5OjEiOjUwLCJkcml2ZXI6bG9jYWxCZW5jaG1hcmsiOjIzLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MCI6MCwiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjEiOjEwMCwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6dmFsdWUiOjE1LCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6dmFsdWUiOjgyLjQsInRhcmdldDpjb21wYW55UGF5U2NoZWR1bGU6dmFsdWUiOjIsInRhcmdldDpjb21wYW55UGF5U2NoZWR1bGU6bWF4Ijo3LCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6dmFsdWUiOjYwLCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6bWF4Ijo5NSwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6dmFsdWUiOjIyLCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6dmFsdWUiOjc0LjgsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6dmFsdWUiOjIxLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOm1heCI6MzUsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6dmFsdWUiOjE4Ljc4LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOnZhbHVlIjo3LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOm1heCI6MTAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOnZhbHVlIjoyLjg1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86dmFsdWUiOjE1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86bWF4Ijo3MCwidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86dmFsdWUiOjIxMywidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86bWF4IjozNTAsInRhcmdldDpsb2NhbEJlbmNobWFyazp2YWx1ZSI6MjMsInRhcmdldDpsb2NhbEJlbmNobWFyazptYXgiOjQwLCJ0YXJnZXQ6b2ZmaWNlclBheUNhZ3I6dmFsdWUiOjYsInRhcmdldDpvZmZpY2VyUGF5Q2FncjptYXgiOjEwLCJ0YXJnZXQ6b2ZmaWNlclBheUluY3JlYXNlOnZhbHVlIjowLCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6bWF4IjoyNTIuNjksInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTptYXgiOjEzNi44NCwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTptYXgiOjMzLjQzLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlJbmNyZWFzZTptYXgiOjMuNzR9LCJtZXRyaWNHcm91cEJhc2VzIjp7ImNvbXBhbnlTYWxlcyI6InJhdGUiLCJwcm9qZWN0U2FsZXMiOiJyYXRlIiwibGFib3JQcm9kdWN0aXZpdHkiOiJyYXRlIiwiZW1wbG95ZWVQYXkiOiJyYXRlIn0sImFwcGxpY2F0aW9uQ2F0ZWdvcnkiOiJnZW5lcmFsIiwiYWRqdXN0ZWREcml2ZXJzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQxMDU5NTc2MDIzMzkxNiwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MS4xNzQxODY0OTEwNjQ0NjZlLTE2LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAxOTk4MjEzNTUxMTg3OTg3MywicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwNjM5MDEyNDk3MjI5MzQsInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MTIwNDUxMzMzMTU3NjMsIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNjA1NTE2MjczMDA1MjcsIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4ODEzNjc1MDA5MTcxMTcsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDYwOTM1Mzk0MzcxNzg1NSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyMDIyNDg3MjE2OTQ2NjczLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU2NTE3ODU5NDUyMTc5LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNDk5MDQ4MTM0MTI2NTU1LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDg5MDA2MjI5OTc1MDgwMSwib3RoZXJQYXlHcm93dGgiOjAuMDI0ODg3NzYxNzEwMzMzMDMsInByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDI5MDQ1NDgyMzk3MjA1MDU1LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU3ODQ4MTQ3MzIzMDg2NjUsInByb2plY3RTZ2FSYXRlRW5kIjowLjEwOTkzMTgwOTE2NDg0ODI0LCJvdGhlclNnYVJhdGVFbmQiOjAuMTA5MjcyNTg5ODcyMTI4MjMsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1Mzc3ODA1NzYyODcxNjMyLCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6MjMsInN1YnNpZHkiOjcuNjYsImxvY2FsQmVuY2htYXJrIjoyM319</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Align company profit and headcount inputs with round six
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -1830,135 +1830,99 @@
         </is>
       </c>
       <c r="B20" s="4">
-        <v>11.000000000000007</v>
+        <v>10.73</v>
       </c>
       <c r="C20" s="4">
-        <v>11.299999999999997</v>
+        <v>11.01</v>
       </c>
       <c r="D20" s="4">
-        <v>11.600000000000001</v>
+        <v>11.3</v>
       </c>
       <c r="E20" s="4">
-        <v>11.480000000000004</v>
+        <v>11.17</v>
       </c>
       <c r="F20" s="4">
-        <v>11.350000000000016</v>
+        <v>11.02</v>
       </c>
       <c r="G20" s="4">
-        <v>11.210000000000004</v>
+        <v>10.86</v>
       </c>
       <c r="H20" s="4">
-        <v>17.239999999999988</v>
+        <v>15.55</v>
       </c>
       <c r="I20" s="4">
-        <v>23.34999999999998</v>
+        <v>21.49</v>
       </c>
       <c r="J20" s="4">
-        <v>31.170000000000044</v>
+        <v>29.12</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2-19 税引前当期純利益（モデル未対応）（億円）</t>
-        </is>
-      </c>
-      <c r="B21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="C21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">2-19 税引前当期純利益（億円）</t>
+        </is>
+      </c>
+      <c r="B21" s="2">
+        <v>10.73</v>
+      </c>
+      <c r="C21" s="2">
+        <v>11.01</v>
+      </c>
+      <c r="D21" s="2">
+        <v>11.3</v>
+      </c>
+      <c r="E21" s="2">
+        <v>11.17</v>
+      </c>
+      <c r="F21" s="2">
+        <v>11.02</v>
+      </c>
+      <c r="G21" s="2">
+        <v>10.86</v>
+      </c>
+      <c r="H21" s="2">
+        <v>15.55</v>
+      </c>
+      <c r="I21" s="2">
+        <v>21.49</v>
+      </c>
+      <c r="J21" s="2">
+        <v>29.12</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2-20 当期純利益（モデル未対応）（億円）</t>
-        </is>
-      </c>
-      <c r="B22" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="C22" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D22" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E22" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F22" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G22" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H22" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I22" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J22" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">2-20 当期純利益（億円）</t>
+        </is>
+      </c>
+      <c r="B22" s="2">
+        <v>7.51</v>
+      </c>
+      <c r="C22" s="2">
+        <v>7.71</v>
+      </c>
+      <c r="D22" s="2">
+        <v>7.91</v>
+      </c>
+      <c r="E22" s="2">
+        <v>7.82</v>
+      </c>
+      <c r="F22" s="2">
+        <v>7.71</v>
+      </c>
+      <c r="G22" s="2">
+        <v>7.6</v>
+      </c>
+      <c r="H22" s="2">
+        <v>10.88</v>
+      </c>
+      <c r="I22" s="2">
+        <v>15.04</v>
+      </c>
+      <c r="J22" s="2">
+        <v>20.38</v>
       </c>
     </row>
     <row r="23">
@@ -6386,7 +6350,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C229"/>
+  <dimension ref="A1:C244"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="72" customWidth="1"/>
@@ -6521,11 +6485,11 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2023:2-3</t>
+          <t xml:space="preserve">actual:company:2023:2-18</t>
         </is>
       </c>
       <c r="B9" s="2">
-        <v>92.75</v>
+        <v>10.73</v>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
@@ -6536,11 +6500,11 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2023:2-4</t>
+          <t xml:space="preserve">actual:company:2023:2-19</t>
         </is>
       </c>
       <c r="B10" s="2">
-        <v>0.73</v>
+        <v>10.73</v>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
@@ -6551,11 +6515,11 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2023:2-7</t>
+          <t xml:space="preserve">actual:company:2023:2-20</t>
         </is>
       </c>
       <c r="B11" s="2">
-        <v>32.65</v>
+        <v>7.51</v>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
@@ -6566,11 +6530,11 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2023:2-9</t>
+          <t xml:space="preserve">actual:company:2023:2-27</t>
         </is>
       </c>
       <c r="B12" s="2">
-        <v>0.82</v>
+        <v>210</v>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
@@ -6581,11 +6545,11 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-1</t>
+          <t xml:space="preserve">actual:company:2023:2-28</t>
         </is>
       </c>
       <c r="B13" s="2">
-        <v>143.2</v>
+        <v>5</v>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
@@ -6596,11 +6560,11 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-10</t>
+          <t xml:space="preserve">actual:company:2023:2-3</t>
         </is>
       </c>
       <c r="B14" s="2">
-        <v>0.1</v>
+        <v>92.75</v>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
@@ -6611,11 +6575,11 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-12</t>
+          <t xml:space="preserve">actual:company:2023:2-4</t>
         </is>
       </c>
       <c r="B15" s="2">
-        <v>12.47</v>
+        <v>0.73</v>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
@@ -6626,11 +6590,11 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-13</t>
+          <t xml:space="preserve">actual:company:2023:2-7</t>
         </is>
       </c>
       <c r="B16" s="2">
-        <v>0.66</v>
+        <v>32.65</v>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
@@ -6641,11 +6605,11 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-14</t>
+          <t xml:space="preserve">actual:company:2023:2-9</t>
         </is>
       </c>
       <c r="B17" s="2">
-        <v>2.58</v>
+        <v>0.82</v>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
@@ -6656,11 +6620,11 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-15</t>
+          <t xml:space="preserve">actual:company:2024:2-1</t>
         </is>
       </c>
       <c r="B18" s="2">
-        <v>0.67</v>
+        <v>143.2</v>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
@@ -6671,11 +6635,11 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-3</t>
+          <t xml:space="preserve">actual:company:2024:2-10</t>
         </is>
       </c>
       <c r="B19" s="2">
-        <v>97.38</v>
+        <v>0.1</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
@@ -6686,11 +6650,11 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-4</t>
+          <t xml:space="preserve">actual:company:2024:2-12</t>
         </is>
       </c>
       <c r="B20" s="2">
-        <v>0.76</v>
+        <v>12.47</v>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
@@ -6701,11 +6665,11 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-7</t>
+          <t xml:space="preserve">actual:company:2024:2-13</t>
         </is>
       </c>
       <c r="B21" s="2">
-        <v>34.52</v>
+        <v>0.66</v>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
@@ -6716,11 +6680,11 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-9</t>
+          <t xml:space="preserve">actual:company:2024:2-14</t>
         </is>
       </c>
       <c r="B22" s="2">
-        <v>0.86</v>
+        <v>2.58</v>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
@@ -6731,11 +6695,11 @@
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-1</t>
+          <t xml:space="preserve">actual:company:2024:2-15</t>
         </is>
       </c>
       <c r="B23" s="2">
-        <v>150</v>
+        <v>0.67</v>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
@@ -6746,11 +6710,11 @@
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-10</t>
+          <t xml:space="preserve">actual:company:2024:2-18</t>
         </is>
       </c>
       <c r="B24" s="2">
-        <v>0.1</v>
+        <v>11.01</v>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
@@ -6761,11 +6725,11 @@
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-12</t>
+          <t xml:space="preserve">actual:company:2024:2-19</t>
         </is>
       </c>
       <c r="B25" s="2">
-        <v>13.3</v>
+        <v>11.01</v>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
@@ -6776,11 +6740,11 @@
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-13</t>
+          <t xml:space="preserve">actual:company:2024:2-20</t>
         </is>
       </c>
       <c r="B26" s="2">
-        <v>0.7</v>
+        <v>7.71</v>
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
@@ -6791,11 +6755,11 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-14</t>
+          <t xml:space="preserve">actual:company:2024:2-27</t>
         </is>
       </c>
       <c r="B27" s="2">
-        <v>2.7</v>
+        <v>220</v>
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
@@ -6806,11 +6770,11 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-15</t>
+          <t xml:space="preserve">actual:company:2024:2-28</t>
         </is>
       </c>
       <c r="B28" s="2">
-        <v>0.7</v>
+        <v>5</v>
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
@@ -6821,11 +6785,11 @@
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-3</t>
+          <t xml:space="preserve">actual:company:2024:2-3</t>
         </is>
       </c>
       <c r="B29" s="2">
-        <v>102</v>
+        <v>97.38</v>
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
@@ -6836,11 +6800,11 @@
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-4</t>
+          <t xml:space="preserve">actual:company:2024:2-4</t>
         </is>
       </c>
       <c r="B30" s="2">
-        <v>0.8</v>
+        <v>0.76</v>
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
@@ -6851,11 +6815,11 @@
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-7</t>
+          <t xml:space="preserve">actual:company:2024:2-7</t>
         </is>
       </c>
       <c r="B31" s="2">
-        <v>36.4</v>
+        <v>34.52</v>
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
@@ -6866,11 +6830,11 @@
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-9</t>
+          <t xml:space="preserve">actual:company:2024:2-9</t>
         </is>
       </c>
       <c r="B32" s="2">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
@@ -6881,11 +6845,11 @@
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2023:7-1</t>
+          <t xml:space="preserve">actual:company:2025:2-1</t>
         </is>
       </c>
       <c r="B33" s="2">
-        <v>72</v>
+        <v>150</v>
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
@@ -6896,11 +6860,11 @@
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2023:7-10</t>
+          <t xml:space="preserve">actual:company:2025:2-10</t>
         </is>
       </c>
       <c r="B34" s="2">
-        <v>1.8</v>
+        <v>0.1</v>
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
@@ -6911,11 +6875,11 @@
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2023:7-13</t>
+          <t xml:space="preserve">actual:company:2025:2-12</t>
         </is>
       </c>
       <c r="B35" s="2">
-        <v>90</v>
+        <v>13.3</v>
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
@@ -6926,11 +6890,11 @@
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2023:7-14</t>
+          <t xml:space="preserve">actual:company:2025:2-13</t>
         </is>
       </c>
       <c r="B36" s="2">
-        <v>2</v>
+        <v>0.7</v>
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
@@ -6941,11 +6905,11 @@
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2023:7-4</t>
+          <t xml:space="preserve">actual:company:2025:2-14</t>
         </is>
       </c>
       <c r="B37" s="2">
-        <v>23.04</v>
+        <v>2.7</v>
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
@@ -6956,11 +6920,11 @@
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2023:7-6</t>
+          <t xml:space="preserve">actual:company:2025:2-15</t>
         </is>
       </c>
       <c r="B38" s="2">
-        <v>6.78</v>
+        <v>0.7</v>
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
@@ -6971,11 +6935,11 @@
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2023:7-8</t>
+          <t xml:space="preserve">actual:company:2025:2-18</t>
         </is>
       </c>
       <c r="B39" s="2">
-        <v>5.19</v>
+        <v>11.3</v>
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
@@ -6986,11 +6950,11 @@
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2023:7-9</t>
+          <t xml:space="preserve">actual:company:2025:2-19</t>
         </is>
       </c>
       <c r="B40" s="2">
-        <v>0.36</v>
+        <v>11.3</v>
       </c>
       <c r="C40" s="0" t="inlineStr">
         <is>
@@ -7001,11 +6965,11 @@
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2024:7-1</t>
+          <t xml:space="preserve">actual:company:2025:2-20</t>
         </is>
       </c>
       <c r="B41" s="2">
-        <v>76</v>
+        <v>7.91</v>
       </c>
       <c r="C41" s="0" t="inlineStr">
         <is>
@@ -7016,11 +6980,11 @@
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2024:7-10</t>
+          <t xml:space="preserve">actual:company:2025:2-27</t>
         </is>
       </c>
       <c r="B42" s="2">
-        <v>1.9</v>
+        <v>230</v>
       </c>
       <c r="C42" s="0" t="inlineStr">
         <is>
@@ -7031,11 +6995,11 @@
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2024:7-13</t>
+          <t xml:space="preserve">actual:company:2025:2-28</t>
         </is>
       </c>
       <c r="B43" s="2">
-        <v>95</v>
+        <v>5</v>
       </c>
       <c r="C43" s="0" t="inlineStr">
         <is>
@@ -7046,11 +7010,11 @@
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2024:7-14</t>
+          <t xml:space="preserve">actual:company:2025:2-3</t>
         </is>
       </c>
       <c r="B44" s="2">
-        <v>2</v>
+        <v>102</v>
       </c>
       <c r="C44" s="0" t="inlineStr">
         <is>
@@ -7061,11 +7025,11 @@
     <row r="45">
       <c r="A45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2024:7-4</t>
+          <t xml:space="preserve">actual:company:2025:2-4</t>
         </is>
       </c>
       <c r="B45" s="2">
-        <v>24.32</v>
+        <v>0.8</v>
       </c>
       <c r="C45" s="0" t="inlineStr">
         <is>
@@ -7076,11 +7040,11 @@
     <row r="46">
       <c r="A46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2024:7-6</t>
+          <t xml:space="preserve">actual:company:2025:2-7</t>
         </is>
       </c>
       <c r="B46" s="2">
-        <v>7.04</v>
+        <v>36.4</v>
       </c>
       <c r="C46" s="0" t="inlineStr">
         <is>
@@ -7091,11 +7055,11 @@
     <row r="47">
       <c r="A47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2024:7-8</t>
+          <t xml:space="preserve">actual:company:2025:2-9</t>
         </is>
       </c>
       <c r="B47" s="2">
-        <v>5.59</v>
+        <v>0.9</v>
       </c>
       <c r="C47" s="0" t="inlineStr">
         <is>
@@ -7106,11 +7070,11 @@
     <row r="48">
       <c r="A48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2024:7-9</t>
+          <t xml:space="preserve">actual:project:2023:7-1</t>
         </is>
       </c>
       <c r="B48" s="2">
-        <v>0.38</v>
+        <v>72</v>
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
@@ -7121,11 +7085,11 @@
     <row r="49">
       <c r="A49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2025:7-1</t>
+          <t xml:space="preserve">actual:project:2023:7-10</t>
         </is>
       </c>
       <c r="B49" s="2">
-        <v>80</v>
+        <v>1.8</v>
       </c>
       <c r="C49" s="0" t="inlineStr">
         <is>
@@ -7136,11 +7100,11 @@
     <row r="50">
       <c r="A50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2025:7-10</t>
+          <t xml:space="preserve">actual:project:2023:7-13</t>
         </is>
       </c>
       <c r="B50" s="2">
-        <v>2</v>
+        <v>90</v>
       </c>
       <c r="C50" s="0" t="inlineStr">
         <is>
@@ -7151,11 +7115,11 @@
     <row r="51">
       <c r="A51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2025:7-13</t>
+          <t xml:space="preserve">actual:project:2023:7-14</t>
         </is>
       </c>
       <c r="B51" s="2">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="C51" s="0" t="inlineStr">
         <is>
@@ -7166,11 +7130,11 @@
     <row r="52">
       <c r="A52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2025:7-14</t>
+          <t xml:space="preserve">actual:project:2023:7-4</t>
         </is>
       </c>
       <c r="B52" s="2">
-        <v>2</v>
+        <v>23.04</v>
       </c>
       <c r="C52" s="0" t="inlineStr">
         <is>
@@ -7181,11 +7145,11 @@
     <row r="53">
       <c r="A53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2025:7-4</t>
+          <t xml:space="preserve">actual:project:2023:7-6</t>
         </is>
       </c>
       <c r="B53" s="2">
-        <v>25.6</v>
+        <v>6.78</v>
       </c>
       <c r="C53" s="0" t="inlineStr">
         <is>
@@ -7196,11 +7160,11 @@
     <row r="54">
       <c r="A54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2025:7-6</t>
+          <t xml:space="preserve">actual:project:2023:7-8</t>
         </is>
       </c>
       <c r="B54" s="2">
-        <v>7.3</v>
+        <v>5.19</v>
       </c>
       <c r="C54" s="0" t="inlineStr">
         <is>
@@ -7211,11 +7175,11 @@
     <row r="55">
       <c r="A55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2025:7-8</t>
+          <t xml:space="preserve">actual:project:2023:7-9</t>
         </is>
       </c>
       <c r="B55" s="2">
-        <v>6</v>
+        <v>0.36</v>
       </c>
       <c r="C55" s="0" t="inlineStr">
         <is>
@@ -7226,11 +7190,11 @@
     <row r="56">
       <c r="A56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2025:7-9</t>
+          <t xml:space="preserve">actual:project:2024:7-1</t>
         </is>
       </c>
       <c r="B56" s="2">
-        <v>0.4</v>
+        <v>76</v>
       </c>
       <c r="C56" s="0" t="inlineStr">
         <is>
@@ -7241,11 +7205,11 @@
     <row r="57">
       <c r="A57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:assets</t>
+          <t xml:space="preserve">actual:project:2024:7-10</t>
         </is>
       </c>
       <c r="B57" s="2">
-        <v>132</v>
+        <v>1.9</v>
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
@@ -7256,11 +7220,11 @@
     <row r="58">
       <c r="A58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:buildings</t>
+          <t xml:space="preserve">actual:project:2024:7-13</t>
         </is>
       </c>
       <c r="B58" s="2">
-        <v>19</v>
+        <v>95</v>
       </c>
       <c r="C58" s="0" t="inlineStr">
         <is>
@@ -7271,11 +7235,11 @@
     <row r="59">
       <c r="A59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:capex</t>
+          <t xml:space="preserve">actual:project:2024:7-14</t>
         </is>
       </c>
       <c r="B59" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C59" s="0" t="inlineStr">
         <is>
@@ -7286,11 +7250,11 @@
     <row r="60">
       <c r="A60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:capital</t>
+          <t xml:space="preserve">actual:project:2024:7-4</t>
         </is>
       </c>
       <c r="B60" s="2">
-        <v>10</v>
+        <v>24.32</v>
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
@@ -7301,11 +7265,11 @@
     <row r="61">
       <c r="A61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:cash</t>
+          <t xml:space="preserve">actual:project:2024:7-6</t>
         </is>
       </c>
       <c r="B61" s="2">
-        <v>24</v>
+        <v>7.04</v>
       </c>
       <c r="C61" s="0" t="inlineStr">
         <is>
@@ -7316,11 +7280,11 @@
     <row r="62">
       <c r="A62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:currentAssets</t>
+          <t xml:space="preserve">actual:project:2024:7-8</t>
         </is>
       </c>
       <c r="B62" s="2">
-        <v>67</v>
+        <v>5.59</v>
       </c>
       <c r="C62" s="0" t="inlineStr">
         <is>
@@ -7331,11 +7295,11 @@
     <row r="63">
       <c r="A63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:currentLiabilities</t>
+          <t xml:space="preserve">actual:project:2024:7-9</t>
         </is>
       </c>
       <c r="B63" s="2">
-        <v>39</v>
+        <v>0.38</v>
       </c>
       <c r="C63" s="0" t="inlineStr">
         <is>
@@ -7346,11 +7310,11 @@
     <row r="64">
       <c r="A64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:fixedAssets</t>
+          <t xml:space="preserve">actual:project:2025:7-1</t>
         </is>
       </c>
       <c r="B64" s="2">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="C64" s="0" t="inlineStr">
         <is>
@@ -7361,11 +7325,11 @@
     <row r="65">
       <c r="A65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:fixedLiabilities</t>
+          <t xml:space="preserve">actual:project:2025:7-10</t>
         </is>
       </c>
       <c r="B65" s="2">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="C65" s="0" t="inlineStr">
         <is>
@@ -7376,11 +7340,11 @@
     <row r="66">
       <c r="A66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:intangibleAssets</t>
+          <t xml:space="preserve">actual:project:2025:7-13</t>
         </is>
       </c>
       <c r="B66" s="2">
-        <v>7</v>
+        <v>100</v>
       </c>
       <c r="C66" s="0" t="inlineStr">
         <is>
@@ -7391,11 +7355,11 @@
     <row r="67">
       <c r="A67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:land</t>
+          <t xml:space="preserve">actual:project:2025:7-14</t>
         </is>
       </c>
       <c r="B67" s="2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C67" s="0" t="inlineStr">
         <is>
@@ -7406,11 +7370,11 @@
     <row r="68">
       <c r="A68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:liabilities</t>
+          <t xml:space="preserve">actual:project:2025:7-4</t>
         </is>
       </c>
       <c r="B68" s="2">
-        <v>75</v>
+        <v>25.6</v>
       </c>
       <c r="C68" s="0" t="inlineStr">
         <is>
@@ -7421,11 +7385,11 @@
     <row r="69">
       <c r="A69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:longTermDebt</t>
+          <t xml:space="preserve">actual:project:2025:7-6</t>
         </is>
       </c>
       <c r="B69" s="2">
-        <v>29</v>
+        <v>7.3</v>
       </c>
       <c r="C69" s="0" t="inlineStr">
         <is>
@@ -7436,11 +7400,11 @@
     <row r="70">
       <c r="A70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:machinery</t>
+          <t xml:space="preserve">actual:project:2025:7-8</t>
         </is>
       </c>
       <c r="B70" s="2">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="C70" s="0" t="inlineStr">
         <is>
@@ -7451,11 +7415,11 @@
     <row r="71">
       <c r="A71" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:netAssets</t>
+          <t xml:space="preserve">actual:project:2025:7-9</t>
         </is>
       </c>
       <c r="B71" s="2">
-        <v>57</v>
+        <v>0.4</v>
       </c>
       <c r="C71" s="0" t="inlineStr">
         <is>
@@ -7466,11 +7430,11 @@
     <row r="72">
       <c r="A72" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:shareholderEquity</t>
+          <t xml:space="preserve">balance-sheet:2023:assets</t>
         </is>
       </c>
       <c r="B72" s="2">
-        <v>54</v>
+        <v>132</v>
       </c>
       <c r="C72" s="0" t="inlineStr">
         <is>
@@ -7481,11 +7445,11 @@
     <row r="73">
       <c r="A73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:shortTermDebt</t>
+          <t xml:space="preserve">balance-sheet:2023:buildings</t>
         </is>
       </c>
       <c r="B73" s="2">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="C73" s="0" t="inlineStr">
         <is>
@@ -7496,7 +7460,7 @@
     <row r="74">
       <c r="A74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:software</t>
+          <t xml:space="preserve">balance-sheet:2023:capex</t>
         </is>
       </c>
       <c r="B74" s="2">
@@ -7511,11 +7475,11 @@
     <row r="75">
       <c r="A75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2023:tangibleAssets</t>
+          <t xml:space="preserve">balance-sheet:2023:capital</t>
         </is>
       </c>
       <c r="B75" s="2">
-        <v>53</v>
+        <v>10</v>
       </c>
       <c r="C75" s="0" t="inlineStr">
         <is>
@@ -7526,11 +7490,11 @@
     <row r="76">
       <c r="A76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:assets</t>
+          <t xml:space="preserve">balance-sheet:2023:cash</t>
         </is>
       </c>
       <c r="B76" s="2">
-        <v>143</v>
+        <v>24</v>
       </c>
       <c r="C76" s="0" t="inlineStr">
         <is>
@@ -7541,11 +7505,11 @@
     <row r="77">
       <c r="A77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:buildings</t>
+          <t xml:space="preserve">balance-sheet:2023:currentAssets</t>
         </is>
       </c>
       <c r="B77" s="2">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="C77" s="0" t="inlineStr">
         <is>
@@ -7556,11 +7520,11 @@
     <row r="78">
       <c r="A78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:capex</t>
+          <t xml:space="preserve">balance-sheet:2023:currentLiabilities</t>
         </is>
       </c>
       <c r="B78" s="2">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="C78" s="0" t="inlineStr">
         <is>
@@ -7571,11 +7535,11 @@
     <row r="79">
       <c r="A79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:capital</t>
+          <t xml:space="preserve">balance-sheet:2023:fixedAssets</t>
         </is>
       </c>
       <c r="B79" s="2">
-        <v>10</v>
+        <v>65</v>
       </c>
       <c r="C79" s="0" t="inlineStr">
         <is>
@@ -7586,11 +7550,11 @@
     <row r="80">
       <c r="A80" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:cash</t>
+          <t xml:space="preserve">balance-sheet:2023:fixedLiabilities</t>
         </is>
       </c>
       <c r="B80" s="2">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="C80" s="0" t="inlineStr">
         <is>
@@ -7601,11 +7565,11 @@
     <row r="81">
       <c r="A81" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:currentAssets</t>
+          <t xml:space="preserve">balance-sheet:2023:intangibleAssets</t>
         </is>
       </c>
       <c r="B81" s="2">
-        <v>72</v>
+        <v>7</v>
       </c>
       <c r="C81" s="0" t="inlineStr">
         <is>
@@ -7616,11 +7580,11 @@
     <row r="82">
       <c r="A82" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:currentLiabilities</t>
+          <t xml:space="preserve">balance-sheet:2023:land</t>
         </is>
       </c>
       <c r="B82" s="2">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="C82" s="0" t="inlineStr">
         <is>
@@ -7631,11 +7595,11 @@
     <row r="83">
       <c r="A83" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:fixedAssets</t>
+          <t xml:space="preserve">balance-sheet:2023:liabilities</t>
         </is>
       </c>
       <c r="B83" s="2">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C83" s="0" t="inlineStr">
         <is>
@@ -7646,11 +7610,11 @@
     <row r="84">
       <c r="A84" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:fixedLiabilities</t>
+          <t xml:space="preserve">balance-sheet:2023:longTermDebt</t>
         </is>
       </c>
       <c r="B84" s="2">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="C84" s="0" t="inlineStr">
         <is>
@@ -7661,11 +7625,11 @@
     <row r="85">
       <c r="A85" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:intangibleAssets</t>
+          <t xml:space="preserve">balance-sheet:2023:machinery</t>
         </is>
       </c>
       <c r="B85" s="2">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="C85" s="0" t="inlineStr">
         <is>
@@ -7676,11 +7640,11 @@
     <row r="86">
       <c r="A86" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:land</t>
+          <t xml:space="preserve">balance-sheet:2023:netAssets</t>
         </is>
       </c>
       <c r="B86" s="2">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="C86" s="0" t="inlineStr">
         <is>
@@ -7691,11 +7655,11 @@
     <row r="87">
       <c r="A87" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:liabilities</t>
+          <t xml:space="preserve">balance-sheet:2023:shareholderEquity</t>
         </is>
       </c>
       <c r="B87" s="2">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="C87" s="0" t="inlineStr">
         <is>
@@ -7706,11 +7670,11 @@
     <row r="88">
       <c r="A88" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:longTermDebt</t>
+          <t xml:space="preserve">balance-sheet:2023:shortTermDebt</t>
         </is>
       </c>
       <c r="B88" s="2">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="C88" s="0" t="inlineStr">
         <is>
@@ -7721,11 +7685,11 @@
     <row r="89">
       <c r="A89" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:machinery</t>
+          <t xml:space="preserve">balance-sheet:2023:software</t>
         </is>
       </c>
       <c r="B89" s="2">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="C89" s="0" t="inlineStr">
         <is>
@@ -7736,11 +7700,11 @@
     <row r="90">
       <c r="A90" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:netAssets</t>
+          <t xml:space="preserve">balance-sheet:2023:tangibleAssets</t>
         </is>
       </c>
       <c r="B90" s="2">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="C90" s="0" t="inlineStr">
         <is>
@@ -7751,11 +7715,11 @@
     <row r="91">
       <c r="A91" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:shareholderEquity</t>
+          <t xml:space="preserve">balance-sheet:2024:assets</t>
         </is>
       </c>
       <c r="B91" s="2">
-        <v>61</v>
+        <v>143</v>
       </c>
       <c r="C91" s="0" t="inlineStr">
         <is>
@@ -7766,11 +7730,11 @@
     <row r="92">
       <c r="A92" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:shortTermDebt</t>
+          <t xml:space="preserve">balance-sheet:2024:buildings</t>
         </is>
       </c>
       <c r="B92" s="2">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C92" s="0" t="inlineStr">
         <is>
@@ -7781,11 +7745,11 @@
     <row r="93">
       <c r="A93" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:software</t>
+          <t xml:space="preserve">balance-sheet:2024:capex</t>
         </is>
       </c>
       <c r="B93" s="2">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C93" s="0" t="inlineStr">
         <is>
@@ -7796,11 +7760,11 @@
     <row r="94">
       <c r="A94" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2024:tangibleAssets</t>
+          <t xml:space="preserve">balance-sheet:2024:capital</t>
         </is>
       </c>
       <c r="B94" s="2">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="C94" s="0" t="inlineStr">
         <is>
@@ -7811,11 +7775,11 @@
     <row r="95">
       <c r="A95" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:assets</t>
+          <t xml:space="preserve">balance-sheet:2024:cash</t>
         </is>
       </c>
       <c r="B95" s="2">
-        <v>156</v>
+        <v>25</v>
       </c>
       <c r="C95" s="0" t="inlineStr">
         <is>
@@ -7826,11 +7790,11 @@
     <row r="96">
       <c r="A96" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:buildings</t>
+          <t xml:space="preserve">balance-sheet:2024:currentAssets</t>
         </is>
       </c>
       <c r="B96" s="2">
-        <v>22</v>
+        <v>72</v>
       </c>
       <c r="C96" s="0" t="inlineStr">
         <is>
@@ -7841,11 +7805,11 @@
     <row r="97">
       <c r="A97" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:capex</t>
+          <t xml:space="preserve">balance-sheet:2024:currentLiabilities</t>
         </is>
       </c>
       <c r="B97" s="2">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="C97" s="0" t="inlineStr">
         <is>
@@ -7856,11 +7820,11 @@
     <row r="98">
       <c r="A98" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:capital</t>
+          <t xml:space="preserve">balance-sheet:2024:fixedAssets</t>
         </is>
       </c>
       <c r="B98" s="2">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="C98" s="0" t="inlineStr">
         <is>
@@ -7871,11 +7835,11 @@
     <row r="99">
       <c r="A99" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:cash</t>
+          <t xml:space="preserve">balance-sheet:2024:fixedLiabilities</t>
         </is>
       </c>
       <c r="B99" s="2">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="C99" s="0" t="inlineStr">
         <is>
@@ -7886,11 +7850,11 @@
     <row r="100">
       <c r="A100" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:currentAssets</t>
+          <t xml:space="preserve">balance-sheet:2024:intangibleAssets</t>
         </is>
       </c>
       <c r="B100" s="2">
-        <v>78</v>
+        <v>8</v>
       </c>
       <c r="C100" s="0" t="inlineStr">
         <is>
@@ -7901,11 +7865,11 @@
     <row r="101">
       <c r="A101" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:currentLiabilities</t>
+          <t xml:space="preserve">balance-sheet:2024:land</t>
         </is>
       </c>
       <c r="B101" s="2">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="C101" s="0" t="inlineStr">
         <is>
@@ -7916,11 +7880,11 @@
     <row r="102">
       <c r="A102" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:fixedAssets</t>
+          <t xml:space="preserve">balance-sheet:2024:liabilities</t>
         </is>
       </c>
       <c r="B102" s="2">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C102" s="0" t="inlineStr">
         <is>
@@ -7931,11 +7895,11 @@
     <row r="103">
       <c r="A103" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:fixedLiabilities</t>
+          <t xml:space="preserve">balance-sheet:2024:longTermDebt</t>
         </is>
       </c>
       <c r="B103" s="2">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C103" s="0" t="inlineStr">
         <is>
@@ -7946,11 +7910,11 @@
     <row r="104">
       <c r="A104" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:intangibleAssets</t>
+          <t xml:space="preserve">balance-sheet:2024:machinery</t>
         </is>
       </c>
       <c r="B104" s="2">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="C104" s="0" t="inlineStr">
         <is>
@@ -7961,11 +7925,11 @@
     <row r="105">
       <c r="A105" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:land</t>
+          <t xml:space="preserve">balance-sheet:2024:netAssets</t>
         </is>
       </c>
       <c r="B105" s="2">
-        <v>10</v>
+        <v>64</v>
       </c>
       <c r="C105" s="0" t="inlineStr">
         <is>
@@ -7976,11 +7940,11 @@
     <row r="106">
       <c r="A106" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:liabilities</t>
+          <t xml:space="preserve">balance-sheet:2024:shareholderEquity</t>
         </is>
       </c>
       <c r="B106" s="2">
-        <v>83</v>
+        <v>61</v>
       </c>
       <c r="C106" s="0" t="inlineStr">
         <is>
@@ -7991,11 +7955,11 @@
     <row r="107">
       <c r="A107" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:longTermDebt</t>
+          <t xml:space="preserve">balance-sheet:2024:shortTermDebt</t>
         </is>
       </c>
       <c r="B107" s="2">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="C107" s="0" t="inlineStr">
         <is>
@@ -8006,11 +7970,11 @@
     <row r="108">
       <c r="A108" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:machinery</t>
+          <t xml:space="preserve">balance-sheet:2024:software</t>
         </is>
       </c>
       <c r="B108" s="2">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="C108" s="0" t="inlineStr">
         <is>
@@ -8021,11 +7985,11 @@
     <row r="109">
       <c r="A109" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:netAssets</t>
+          <t xml:space="preserve">balance-sheet:2024:tangibleAssets</t>
         </is>
       </c>
       <c r="B109" s="2">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="C109" s="0" t="inlineStr">
         <is>
@@ -8036,11 +8000,11 @@
     <row r="110">
       <c r="A110" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:shareholderEquity</t>
+          <t xml:space="preserve">balance-sheet:2025:assets</t>
         </is>
       </c>
       <c r="B110" s="2">
-        <v>70</v>
+        <v>156</v>
       </c>
       <c r="C110" s="0" t="inlineStr">
         <is>
@@ -8051,11 +8015,11 @@
     <row r="111">
       <c r="A111" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:shortTermDebt</t>
+          <t xml:space="preserve">balance-sheet:2025:buildings</t>
         </is>
       </c>
       <c r="B111" s="2">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C111" s="0" t="inlineStr">
         <is>
@@ -8066,11 +8030,11 @@
     <row r="112">
       <c r="A112" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:software</t>
+          <t xml:space="preserve">balance-sheet:2025:capex</t>
         </is>
       </c>
       <c r="B112" s="2">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C112" s="0" t="inlineStr">
         <is>
@@ -8081,11 +8045,11 @@
     <row r="113">
       <c r="A113" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">balance-sheet:2025:tangibleAssets</t>
+          <t xml:space="preserve">balance-sheet:2025:capital</t>
         </is>
       </c>
       <c r="B113" s="2">
-        <v>64</v>
+        <v>10</v>
       </c>
       <c r="C113" s="0" t="inlineStr">
         <is>
@@ -8096,11 +8060,11 @@
     <row r="114">
       <c r="A114" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:investment:0</t>
+          <t xml:space="preserve">balance-sheet:2025:cash</t>
         </is>
       </c>
       <c r="B114" s="2">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="C114" s="0" t="inlineStr">
         <is>
@@ -8111,11 +8075,11 @@
     <row r="115">
       <c r="A115" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:investment:1</t>
+          <t xml:space="preserve">balance-sheet:2025:currentAssets</t>
         </is>
       </c>
       <c r="B115" s="2">
-        <v>200</v>
+        <v>78</v>
       </c>
       <c r="C115" s="0" t="inlineStr">
         <is>
@@ -8126,26 +8090,26 @@
     <row r="116">
       <c r="A116" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:localBenchmark:0</t>
+          <t xml:space="preserve">balance-sheet:2025:currentLiabilities</t>
         </is>
       </c>
       <c r="B116" s="2">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="C116" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:localBenchmark:1</t>
+          <t xml:space="preserve">balance-sheet:2025:fixedAssets</t>
         </is>
       </c>
       <c r="B117" s="2">
-        <v>100</v>
+        <v>78</v>
       </c>
       <c r="C117" s="0" t="inlineStr">
         <is>
@@ -8156,11 +8120,11 @@
     <row r="118">
       <c r="A118" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherCogsImprovement:0</t>
+          <t xml:space="preserve">balance-sheet:2025:fixedLiabilities</t>
         </is>
       </c>
       <c r="B118" s="2">
-        <v>0.005</v>
+        <v>40</v>
       </c>
       <c r="C118" s="0" t="inlineStr">
         <is>
@@ -8171,11 +8135,11 @@
     <row r="119">
       <c r="A119" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherCogsImprovement:1</t>
+          <t xml:space="preserve">balance-sheet:2025:intangibleAssets</t>
         </is>
       </c>
       <c r="B119" s="2">
-        <v>0.0051345755693581975</v>
+        <v>9</v>
       </c>
       <c r="C119" s="0" t="inlineStr">
         <is>
@@ -8186,26 +8150,26 @@
     <row r="120">
       <c r="A120" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherCogsImprovementToBase:0</t>
+          <t xml:space="preserve">balance-sheet:2025:land</t>
         </is>
       </c>
       <c r="B120" s="2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C120" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherCogsImprovementToBase:1</t>
+          <t xml:space="preserve">balance-sheet:2025:liabilities</t>
         </is>
       </c>
       <c r="B121" s="2">
-        <v>0.00013457556935819737</v>
+        <v>83</v>
       </c>
       <c r="C121" s="0" t="inlineStr">
         <is>
@@ -8216,11 +8180,11 @@
     <row r="122">
       <c r="A122" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherHeadcountGrowth:0</t>
+          <t xml:space="preserve">balance-sheet:2025:longTermDebt</t>
         </is>
       </c>
       <c r="B122" s="2">
-        <v>0.04416666666666668</v>
+        <v>32</v>
       </c>
       <c r="C122" s="0" t="inlineStr">
         <is>
@@ -8231,11 +8195,11 @@
     <row r="123">
       <c r="A123" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherHeadcountGrowth:1</t>
+          <t xml:space="preserve">balance-sheet:2025:machinery</t>
         </is>
       </c>
       <c r="B123" s="2">
-        <v>0.04750000000000009</v>
+        <v>32</v>
       </c>
       <c r="C123" s="0" t="inlineStr">
         <is>
@@ -8246,11 +8210,11 @@
     <row r="124">
       <c r="A124" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherHeadcountGrowthToBase:0</t>
+          <t xml:space="preserve">balance-sheet:2025:netAssets</t>
         </is>
       </c>
       <c r="B124" s="2">
-        <v>0.03916666666666668</v>
+        <v>73</v>
       </c>
       <c r="C124" s="0" t="inlineStr">
         <is>
@@ -8261,11 +8225,11 @@
     <row r="125">
       <c r="A125" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherHeadcountGrowthToBase:1</t>
+          <t xml:space="preserve">balance-sheet:2025:shareholderEquity</t>
         </is>
       </c>
       <c r="B125" s="2">
-        <v>0.04250000000000009</v>
+        <v>70</v>
       </c>
       <c r="C125" s="0" t="inlineStr">
         <is>
@@ -8276,11 +8240,11 @@
     <row r="126">
       <c r="A126" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherPayGrowth:0</t>
+          <t xml:space="preserve">balance-sheet:2025:shortTermDebt</t>
         </is>
       </c>
       <c r="B126" s="2">
-        <v>0.024139457023717444</v>
+        <v>11</v>
       </c>
       <c r="C126" s="0" t="inlineStr">
         <is>
@@ -8291,11 +8255,11 @@
     <row r="127">
       <c r="A127" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherPayGrowth:1</t>
+          <t xml:space="preserve">balance-sheet:2025:software</t>
         </is>
       </c>
       <c r="B127" s="2">
-        <v>0.025553459914763096</v>
+        <v>7</v>
       </c>
       <c r="C127" s="0" t="inlineStr">
         <is>
@@ -8306,11 +8270,11 @@
     <row r="128">
       <c r="A128" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherPayGrowthToBase:0</t>
+          <t xml:space="preserve">balance-sheet:2025:tangibleAssets</t>
         </is>
       </c>
       <c r="B128" s="2">
-        <v>0.019139457023717443</v>
+        <v>64</v>
       </c>
       <c r="C128" s="0" t="inlineStr">
         <is>
@@ -8321,11 +8285,11 @@
     <row r="129">
       <c r="A129" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherPayGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:investment:0</t>
         </is>
       </c>
       <c r="B129" s="2">
-        <v>0.020553459914763095</v>
+        <v>15</v>
       </c>
       <c r="C129" s="0" t="inlineStr">
         <is>
@@ -8336,11 +8300,11 @@
     <row r="130">
       <c r="A130" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSalesGrowth:0</t>
+          <t xml:space="preserve">driver-range:investment:1</t>
         </is>
       </c>
       <c r="B130" s="2">
-        <v>0.06076086956521719</v>
+        <v>200</v>
       </c>
       <c r="C130" s="0" t="inlineStr">
         <is>
@@ -8351,26 +8315,26 @@
     <row r="131">
       <c r="A131" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSalesGrowth:1</t>
+          <t xml:space="preserve">driver-range:localBenchmark:0</t>
         </is>
       </c>
       <c r="B131" s="2">
-        <v>0.06438405797101453</v>
+        <v>0</v>
       </c>
       <c r="C131" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSalesGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:localBenchmark:1</t>
         </is>
       </c>
       <c r="B132" s="2">
-        <v>0.040760869565217184</v>
+        <v>100</v>
       </c>
       <c r="C132" s="0" t="inlineStr">
         <is>
@@ -8381,11 +8345,11 @@
     <row r="133">
       <c r="A133" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSalesGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:otherCogsImprovement:0</t>
         </is>
       </c>
       <c r="B133" s="2">
-        <v>0.04438405797101452</v>
+        <v>0.005</v>
       </c>
       <c r="C133" s="0" t="inlineStr">
         <is>
@@ -8396,22 +8360,22 @@
     <row r="134">
       <c r="A134" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSgaImprovementToBase:0</t>
+          <t xml:space="preserve">driver-range:otherCogsImprovement:1</t>
         </is>
       </c>
       <c r="B134" s="2">
-        <v>0</v>
+        <v>0.0051345755693581975</v>
       </c>
       <c r="C134" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSgaImprovementToBase:1</t>
+          <t xml:space="preserve">driver-range:otherCogsImprovementToBase:0</t>
         </is>
       </c>
       <c r="B135" s="2">
@@ -8426,11 +8390,11 @@
     <row r="136">
       <c r="A136" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSgaRateEnd:0</t>
+          <t xml:space="preserve">driver-range:otherCogsImprovementToBase:1</t>
         </is>
       </c>
       <c r="B136" s="2">
-        <v>0.08928571428571427</v>
+        <v>0.00013457556935819737</v>
       </c>
       <c r="C136" s="0" t="inlineStr">
         <is>
@@ -8441,11 +8405,11 @@
     <row r="137">
       <c r="A137" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSgaRateEnd:1</t>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowth:0</t>
         </is>
       </c>
       <c r="B137" s="2">
-        <v>0.11928571428571427</v>
+        <v>0.04416666666666668</v>
       </c>
       <c r="C137" s="0" t="inlineStr">
         <is>
@@ -8456,26 +8420,26 @@
     <row r="138">
       <c r="A138" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsImprovementAfterBase:0</t>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowth:1</t>
         </is>
       </c>
       <c r="B138" s="2">
-        <v>0</v>
+        <v>0.04750000000000009</v>
       </c>
       <c r="C138" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsImprovementAfterBase:1</t>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowthToBase:0</t>
         </is>
       </c>
       <c r="B139" s="2">
-        <v>0.03</v>
+        <v>0.03916666666666668</v>
       </c>
       <c r="C139" s="0" t="inlineStr">
         <is>
@@ -8486,26 +8450,26 @@
     <row r="140">
       <c r="A140" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsImprovementToBase:0</t>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowthToBase:1</t>
         </is>
       </c>
       <c r="B140" s="2">
-        <v>0</v>
+        <v>0.04250000000000009</v>
       </c>
       <c r="C140" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsImprovementToBase:1</t>
+          <t xml:space="preserve">driver-range:otherPayGrowth:0</t>
         </is>
       </c>
       <c r="B141" s="2">
-        <v>1.6653345369377348e-16</v>
+        <v>0.024139457023717444</v>
       </c>
       <c r="C141" s="0" t="inlineStr">
         <is>
@@ -8516,26 +8480,26 @@
     <row r="142">
       <c r="A142" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectHeadcountGrowth:0</t>
+          <t xml:space="preserve">driver-range:otherPayGrowth:1</t>
         </is>
       </c>
       <c r="B142" s="2">
-        <v>0</v>
+        <v>0.025553459914763096</v>
       </c>
       <c r="C142" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectHeadcountGrowth:1</t>
+          <t xml:space="preserve">driver-range:otherPayGrowthToBase:0</t>
         </is>
       </c>
       <c r="B143" s="2">
-        <v>0.08</v>
+        <v>0.019139457023717443</v>
       </c>
       <c r="C143" s="0" t="inlineStr">
         <is>
@@ -8546,11 +8510,11 @@
     <row r="144">
       <c r="A144" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectHeadcountGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:otherPayGrowthToBase:1</t>
         </is>
       </c>
       <c r="B144" s="2">
-        <v>0.051169590643274754</v>
+        <v>0.020553459914763095</v>
       </c>
       <c r="C144" s="0" t="inlineStr">
         <is>
@@ -8561,11 +8525,11 @@
     <row r="145">
       <c r="A145" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectHeadcountGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:otherSalesGrowth:0</t>
         </is>
       </c>
       <c r="B145" s="2">
-        <v>0.05701754385964919</v>
+        <v>0.06076086956521719</v>
       </c>
       <c r="C145" s="0" t="inlineStr">
         <is>
@@ -8576,11 +8540,11 @@
     <row r="146">
       <c r="A146" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectMarketGrowth:0</t>
+          <t xml:space="preserve">driver-range:otherSalesGrowth:1</t>
         </is>
       </c>
       <c r="B146" s="2">
-        <v>-0.05</v>
+        <v>0.06438405797101453</v>
       </c>
       <c r="C146" s="0" t="inlineStr">
         <is>
@@ -8591,11 +8555,11 @@
     <row r="147">
       <c r="A147" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectMarketGrowth:1</t>
+          <t xml:space="preserve">driver-range:otherSalesGrowthToBase:0</t>
         </is>
       </c>
       <c r="B147" s="2">
-        <v>0.3</v>
+        <v>0.040760869565217184</v>
       </c>
       <c r="C147" s="0" t="inlineStr">
         <is>
@@ -8606,11 +8570,11 @@
     <row r="148">
       <c r="A148" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectOfficerPayGrowth:0</t>
+          <t xml:space="preserve">driver-range:otherSalesGrowthToBase:1</t>
         </is>
       </c>
       <c r="B148" s="2">
-        <v>0.04263157894736836</v>
+        <v>0.04438405797101452</v>
       </c>
       <c r="C148" s="0" t="inlineStr">
         <is>
@@ -8621,41 +8585,41 @@
     <row r="149">
       <c r="A149" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectOfficerPayGrowth:1</t>
+          <t xml:space="preserve">driver-range:otherSgaImprovementToBase:0</t>
         </is>
       </c>
       <c r="B149" s="2">
-        <v>0.06555555555555558</v>
+        <v>0</v>
       </c>
       <c r="C149" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectOfficerPayGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:otherSgaImprovementToBase:1</t>
         </is>
       </c>
       <c r="B150" s="2">
-        <v>0.051169590643274754</v>
+        <v>0</v>
       </c>
       <c r="C150" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectOfficerPayGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:otherSgaRateEnd:0</t>
         </is>
       </c>
       <c r="B151" s="2">
-        <v>0.05701754385964919</v>
+        <v>0.08928571428571427</v>
       </c>
       <c r="C151" s="0" t="inlineStr">
         <is>
@@ -8666,11 +8630,11 @@
     <row r="152">
       <c r="A152" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectPayGrowth:0</t>
+          <t xml:space="preserve">driver-range:otherSgaRateEnd:1</t>
         </is>
       </c>
       <c r="B152" s="2">
-        <v>0.05</v>
+        <v>0.11928571428571427</v>
       </c>
       <c r="C152" s="0" t="inlineStr">
         <is>
@@ -8681,26 +8645,26 @@
     <row r="153">
       <c r="A153" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectPayGrowth:1</t>
+          <t xml:space="preserve">driver-range:projectCogsImprovementAfterBase:0</t>
         </is>
       </c>
       <c r="B153" s="2">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="C153" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectPayGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:projectCogsImprovementAfterBase:1</t>
         </is>
       </c>
       <c r="B154" s="2">
-        <v>0.019325330501846927</v>
+        <v>0.03</v>
       </c>
       <c r="C154" s="0" t="inlineStr">
         <is>
@@ -8711,26 +8675,26 @@
     <row r="155">
       <c r="A155" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectPayGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:projectCogsImprovementToBase:0</t>
         </is>
       </c>
       <c r="B155" s="2">
-        <v>0.020735994183189166</v>
+        <v>0</v>
       </c>
       <c r="C155" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSalesGrowth:0</t>
+          <t xml:space="preserve">driver-range:projectCogsImprovementToBase:1</t>
         </is>
       </c>
       <c r="B156" s="2">
-        <v>0.15</v>
+        <v>1.6653345369377348e-16</v>
       </c>
       <c r="C156" s="0" t="inlineStr">
         <is>
@@ -8741,26 +8705,26 @@
     <row r="157">
       <c r="A157" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSalesGrowth:1</t>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowth:0</t>
         </is>
       </c>
       <c r="B157" s="2">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="C157" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSalesGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowth:1</t>
         </is>
       </c>
       <c r="B158" s="2">
-        <v>0.051169590643274754</v>
+        <v>0.08</v>
       </c>
       <c r="C158" s="0" t="inlineStr">
         <is>
@@ -8771,11 +8735,11 @@
     <row r="159">
       <c r="A159" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSalesGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowthToBase:0</t>
         </is>
       </c>
       <c r="B159" s="2">
-        <v>0.05701754385964919</v>
+        <v>0.051169590643274754</v>
       </c>
       <c r="C159" s="0" t="inlineStr">
         <is>
@@ -8786,41 +8750,41 @@
     <row r="160">
       <c r="A160" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSgaImprovementToBase:0</t>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowthToBase:1</t>
         </is>
       </c>
       <c r="B160" s="2">
-        <v>0</v>
+        <v>0.05701754385964919</v>
       </c>
       <c r="C160" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSgaImprovementToBase:1</t>
+          <t xml:space="preserve">driver-range:projectMarketGrowth:0</t>
         </is>
       </c>
       <c r="B161" s="2">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
       <c r="C161" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSgaRateEnd:0</t>
+          <t xml:space="preserve">driver-range:projectMarketGrowth:1</t>
         </is>
       </c>
       <c r="B162" s="2">
-        <v>0.08499999999999999</v>
+        <v>0.3</v>
       </c>
       <c r="C162" s="0" t="inlineStr">
         <is>
@@ -8831,11 +8795,11 @@
     <row r="163">
       <c r="A163" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSgaRateEnd:1</t>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowth:0</t>
         </is>
       </c>
       <c r="B163" s="2">
-        <v>0.135</v>
+        <v>0.04263157894736836</v>
       </c>
       <c r="C163" s="0" t="inlineStr">
         <is>
@@ -8846,11 +8810,11 @@
     <row r="164">
       <c r="A164" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:subsidy:0</t>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowth:1</t>
         </is>
       </c>
       <c r="B164" s="2">
-        <v>1</v>
+        <v>0.06555555555555558</v>
       </c>
       <c r="C164" s="0" t="inlineStr">
         <is>
@@ -8861,11 +8825,11 @@
     <row r="165">
       <c r="A165" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:subsidy:1</t>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowthToBase:0</t>
         </is>
       </c>
       <c r="B165" s="2">
-        <v>50</v>
+        <v>0.051169590643274754</v>
       </c>
       <c r="C165" s="0" t="inlineStr">
         <is>
@@ -8876,11 +8840,11 @@
     <row r="166">
       <c r="A166" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:usefulLife:0</t>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowthToBase:1</t>
         </is>
       </c>
       <c r="B166" s="2">
-        <v>5</v>
+        <v>0.05701754385964919</v>
       </c>
       <c r="C166" s="0" t="inlineStr">
         <is>
@@ -8891,11 +8855,11 @@
     <row r="167">
       <c r="A167" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:usefulLife:1</t>
+          <t xml:space="preserve">driver-range:projectPayGrowth:0</t>
         </is>
       </c>
       <c r="B167" s="2">
-        <v>20</v>
+        <v>0.05</v>
       </c>
       <c r="C167" s="0" t="inlineStr">
         <is>
@@ -8906,11 +8870,11 @@
     <row r="168">
       <c r="A168" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:investment</t>
+          <t xml:space="preserve">driver-range:projectPayGrowth:1</t>
         </is>
       </c>
       <c r="B168" s="2">
-        <v>23</v>
+        <v>0.1</v>
       </c>
       <c r="C168" s="0" t="inlineStr">
         <is>
@@ -8921,11 +8885,11 @@
     <row r="169">
       <c r="A169" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:localBenchmark</t>
+          <t xml:space="preserve">driver-range:projectPayGrowthToBase:0</t>
         </is>
       </c>
       <c r="B169" s="2">
-        <v>23</v>
+        <v>0.019325330501846927</v>
       </c>
       <c r="C169" s="0" t="inlineStr">
         <is>
@@ -8936,11 +8900,11 @@
     <row r="170">
       <c r="A170" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherCogsImprovement</t>
+          <t xml:space="preserve">driver-range:projectPayGrowthToBase:1</t>
         </is>
       </c>
       <c r="B170" s="2">
-        <v>0.005</v>
+        <v>0.020735994183189166</v>
       </c>
       <c r="C170" s="0" t="inlineStr">
         <is>
@@ -8951,26 +8915,26 @@
     <row r="171">
       <c r="A171" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherCogsImprovementToBase</t>
+          <t xml:space="preserve">driver-range:projectSalesGrowth:0</t>
         </is>
       </c>
       <c r="B171" s="2">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="C171" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherHeadcountGrowth</t>
+          <t xml:space="preserve">driver-range:projectSalesGrowth:1</t>
         </is>
       </c>
       <c r="B172" s="2">
-        <v>0.045833333333333386</v>
+        <v>0.3</v>
       </c>
       <c r="C172" s="0" t="inlineStr">
         <is>
@@ -8981,11 +8945,11 @@
     <row r="173">
       <c r="A173" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherHeadcountGrowthToBase</t>
+          <t xml:space="preserve">driver-range:projectSalesGrowthToBase:0</t>
         </is>
       </c>
       <c r="B173" s="2">
-        <v>0.04083333333333339</v>
+        <v>0.051169590643274754</v>
       </c>
       <c r="C173" s="0" t="inlineStr">
         <is>
@@ -8996,11 +8960,11 @@
     <row r="174">
       <c r="A174" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherPayGrowth</t>
+          <t xml:space="preserve">driver-range:projectSalesGrowthToBase:1</t>
         </is>
       </c>
       <c r="B174" s="2">
-        <v>0.02484645846924027</v>
+        <v>0.05701754385964919</v>
       </c>
       <c r="C174" s="0" t="inlineStr">
         <is>
@@ -9011,41 +8975,41 @@
     <row r="175">
       <c r="A175" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherPayGrowthToBase</t>
+          <t xml:space="preserve">driver-range:projectSgaImprovementToBase:0</t>
         </is>
       </c>
       <c r="B175" s="2">
-        <v>0.01984645846924027</v>
+        <v>0</v>
       </c>
       <c r="C175" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSalesGrowth</t>
+          <t xml:space="preserve">driver-range:projectSgaImprovementToBase:1</t>
         </is>
       </c>
       <c r="B176" s="2">
-        <v>0.06257246376811586</v>
+        <v>0</v>
       </c>
       <c r="C176" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSalesGrowthToBase</t>
+          <t xml:space="preserve">driver-range:projectSgaRateEnd:0</t>
         </is>
       </c>
       <c r="B177" s="2">
-        <v>0.042572463768115854</v>
+        <v>0.08499999999999999</v>
       </c>
       <c r="C177" s="0" t="inlineStr">
         <is>
@@ -9056,26 +9020,26 @@
     <row r="178">
       <c r="A178" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSgaImprovementToBase</t>
+          <t xml:space="preserve">driver-range:projectSgaRateEnd:1</t>
         </is>
       </c>
       <c r="B178" s="2">
-        <v>0</v>
+        <v>0.135</v>
       </c>
       <c r="C178" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSgaRateEnd</t>
+          <t xml:space="preserve">driver-range:subsidy:0</t>
         </is>
       </c>
       <c r="B179" s="2">
-        <v>0.10928571428571428</v>
+        <v>1</v>
       </c>
       <c r="C179" s="0" t="inlineStr">
         <is>
@@ -9086,11 +9050,11 @@
     <row r="180">
       <c r="A180" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectCogsImprovementAfterBase</t>
+          <t xml:space="preserve">driver-range:subsidy:1</t>
         </is>
       </c>
       <c r="B180" s="2">
-        <v>0.015</v>
+        <v>50</v>
       </c>
       <c r="C180" s="0" t="inlineStr">
         <is>
@@ -9101,11 +9065,11 @@
     <row r="181">
       <c r="A181" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectCogsImprovementToBase</t>
+          <t xml:space="preserve">driver-range:usefulLife:0</t>
         </is>
       </c>
       <c r="B181" s="2">
-        <v>5.551115123125783e-17</v>
+        <v>5</v>
       </c>
       <c r="C181" s="0" t="inlineStr">
         <is>
@@ -9116,11 +9080,11 @@
     <row r="182">
       <c r="A182" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectHeadcountGrowth</t>
+          <t xml:space="preserve">driver-range:usefulLife:1</t>
         </is>
       </c>
       <c r="B182" s="2">
-        <v>0.04</v>
+        <v>20</v>
       </c>
       <c r="C182" s="0" t="inlineStr">
         <is>
@@ -9131,11 +9095,11 @@
     <row r="183">
       <c r="A183" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectHeadcountGrowthToBase</t>
+          <t xml:space="preserve">driver:investment</t>
         </is>
       </c>
       <c r="B183" s="2">
-        <v>0.05409356725146197</v>
+        <v>23</v>
       </c>
       <c r="C183" s="0" t="inlineStr">
         <is>
@@ -9146,11 +9110,11 @@
     <row r="184">
       <c r="A184" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectMarketGrowth</t>
+          <t xml:space="preserve">driver:localBenchmark</t>
         </is>
       </c>
       <c r="B184" s="2">
-        <v>0.05</v>
+        <v>23</v>
       </c>
       <c r="C184" s="0" t="inlineStr">
         <is>
@@ -9161,11 +9125,11 @@
     <row r="185">
       <c r="A185" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectOfficerPayGrowth</t>
+          <t xml:space="preserve">driver:otherCogsImprovement</t>
         </is>
       </c>
       <c r="B185" s="2">
-        <v>0.05380116959064325</v>
+        <v>0.005</v>
       </c>
       <c r="C185" s="0" t="inlineStr">
         <is>
@@ -9176,26 +9140,26 @@
     <row r="186">
       <c r="A186" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectOfficerPayGrowthToBase</t>
+          <t xml:space="preserve">driver:otherCogsImprovementToBase</t>
         </is>
       </c>
       <c r="B186" s="2">
-        <v>0.05409356725146197</v>
+        <v>0</v>
       </c>
       <c r="C186" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectPayGrowth</t>
+          <t xml:space="preserve">driver:otherHeadcountGrowth</t>
         </is>
       </c>
       <c r="B187" s="2">
-        <v>0.07</v>
+        <v>0.045833333333333386</v>
       </c>
       <c r="C187" s="0" t="inlineStr">
         <is>
@@ -9206,11 +9170,11 @@
     <row r="188">
       <c r="A188" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectPayGrowthToBase</t>
+          <t xml:space="preserve">driver:otherHeadcountGrowthToBase</t>
         </is>
       </c>
       <c r="B188" s="2">
-        <v>0.020030662342518046</v>
+        <v>0.04083333333333339</v>
       </c>
       <c r="C188" s="0" t="inlineStr">
         <is>
@@ -9221,11 +9185,11 @@
     <row r="189">
       <c r="A189" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSalesGrowth</t>
+          <t xml:space="preserve">driver:otherPayGrowth</t>
         </is>
       </c>
       <c r="B189" s="2">
-        <v>0.22</v>
+        <v>0.02484645846924027</v>
       </c>
       <c r="C189" s="0" t="inlineStr">
         <is>
@@ -9236,11 +9200,11 @@
     <row r="190">
       <c r="A190" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSalesGrowthToBase</t>
+          <t xml:space="preserve">driver:otherPayGrowthToBase</t>
         </is>
       </c>
       <c r="B190" s="2">
-        <v>0.05409356725146197</v>
+        <v>0.01984645846924027</v>
       </c>
       <c r="C190" s="0" t="inlineStr">
         <is>
@@ -9251,26 +9215,26 @@
     <row r="191">
       <c r="A191" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSgaImprovementToBase</t>
+          <t xml:space="preserve">driver:otherSalesGrowth</t>
         </is>
       </c>
       <c r="B191" s="2">
-        <v>0</v>
+        <v>0.06257246376811586</v>
       </c>
       <c r="C191" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSgaRateEnd</t>
+          <t xml:space="preserve">driver:otherSalesGrowthToBase</t>
         </is>
       </c>
       <c r="B192" s="2">
-        <v>0.11</v>
+        <v>0.042572463768115854</v>
       </c>
       <c r="C192" s="0" t="inlineStr">
         <is>
@@ -9281,26 +9245,26 @@
     <row r="193">
       <c r="A193" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:subsidy</t>
+          <t xml:space="preserve">driver:otherSgaImprovementToBase</t>
         </is>
       </c>
       <c r="B193" s="2">
-        <v>7.66</v>
+        <v>0</v>
       </c>
       <c r="C193" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:usefulLife</t>
+          <t xml:space="preserve">driver:otherSgaRateEnd</t>
         </is>
       </c>
       <c r="B194" s="2">
-        <v>10</v>
+        <v>0.10928571428571428</v>
       </c>
       <c r="C194" s="0" t="inlineStr">
         <is>
@@ -9311,11 +9275,11 @@
     <row r="195">
       <c r="A195" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2026</t>
+          <t xml:space="preserve">driver:projectCogsImprovementAfterBase</t>
         </is>
       </c>
       <c r="B195" s="2">
-        <v>15</v>
+        <v>0.015</v>
       </c>
       <c r="C195" s="0" t="inlineStr">
         <is>
@@ -9326,11 +9290,11 @@
     <row r="196">
       <c r="A196" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2027</t>
+          <t xml:space="preserve">driver:projectCogsImprovementToBase</t>
         </is>
       </c>
       <c r="B196" s="2">
-        <v>15</v>
+        <v>5.551115123125783e-17</v>
       </c>
       <c r="C196" s="0" t="inlineStr">
         <is>
@@ -9341,11 +9305,11 @@
     <row r="197">
       <c r="A197" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2028</t>
+          <t xml:space="preserve">driver:projectHeadcountGrowth</t>
         </is>
       </c>
       <c r="B197" s="2">
-        <v>15</v>
+        <v>0.04</v>
       </c>
       <c r="C197" s="0" t="inlineStr">
         <is>
@@ -9356,56 +9320,56 @@
     <row r="198">
       <c r="A198" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2029</t>
+          <t xml:space="preserve">driver:projectHeadcountGrowthToBase</t>
         </is>
       </c>
       <c r="B198" s="2">
-        <v>0</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="C198" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2030</t>
+          <t xml:space="preserve">driver:projectMarketGrowth</t>
         </is>
       </c>
       <c r="B199" s="2">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="C199" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2031</t>
+          <t xml:space="preserve">driver:projectOfficerPayGrowth</t>
         </is>
       </c>
       <c r="B200" s="2">
-        <v>0</v>
+        <v>0.05380116959064325</v>
       </c>
       <c r="C200" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companyPaySchedule:max</t>
+          <t xml:space="preserve">driver:projectOfficerPayGrowthToBase</t>
         </is>
       </c>
       <c r="B201" s="2">
-        <v>7</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="C201" s="0" t="inlineStr">
         <is>
@@ -9416,11 +9380,11 @@
     <row r="202">
       <c r="A202" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companyPaySchedule:value</t>
+          <t xml:space="preserve">driver:projectPayGrowth</t>
         </is>
       </c>
       <c r="B202" s="2">
-        <v>2</v>
+        <v>0.07</v>
       </c>
       <c r="C202" s="0" t="inlineStr">
         <is>
@@ -9431,11 +9395,11 @@
     <row r="203">
       <c r="A203" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesCagr:max</t>
+          <t xml:space="preserve">driver:projectPayGrowthToBase</t>
         </is>
       </c>
       <c r="B203" s="2">
-        <v>35</v>
+        <v>0.020030662342518046</v>
       </c>
       <c r="C203" s="0" t="inlineStr">
         <is>
@@ -9446,11 +9410,11 @@
     <row r="204">
       <c r="A204" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesCagr:value</t>
+          <t xml:space="preserve">driver:projectSalesGrowth</t>
         </is>
       </c>
       <c r="B204" s="2">
-        <v>15</v>
+        <v>0.22</v>
       </c>
       <c r="C204" s="0" t="inlineStr">
         <is>
@@ -9461,11 +9425,11 @@
     <row r="205">
       <c r="A205" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesIncrease:max</t>
+          <t xml:space="preserve">driver:projectSalesGrowthToBase</t>
         </is>
       </c>
       <c r="B205" s="2">
-        <v>252.69</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="C205" s="0" t="inlineStr">
         <is>
@@ -9476,26 +9440,26 @@
     <row r="206">
       <c r="A206" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesIncrease:value</t>
+          <t xml:space="preserve">driver:projectSgaImprovementToBase</t>
         </is>
       </c>
       <c r="B206" s="2">
-        <v>82.4</v>
+        <v>0</v>
       </c>
       <c r="C206" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayCagr:max</t>
+          <t xml:space="preserve">driver:projectSgaRateEnd</t>
         </is>
       </c>
       <c r="B207" s="2">
-        <v>10</v>
+        <v>0.11</v>
       </c>
       <c r="C207" s="0" t="inlineStr">
         <is>
@@ -9506,11 +9470,11 @@
     <row r="208">
       <c r="A208" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayCagr:value</t>
+          <t xml:space="preserve">driver:subsidy</t>
         </is>
       </c>
       <c r="B208" s="2">
-        <v>7</v>
+        <v>7.66</v>
       </c>
       <c r="C208" s="0" t="inlineStr">
         <is>
@@ -9521,11 +9485,11 @@
     <row r="209">
       <c r="A209" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayIncrease:max</t>
+          <t xml:space="preserve">driver:usefulLife</t>
         </is>
       </c>
       <c r="B209" s="2">
-        <v>3.74</v>
+        <v>10</v>
       </c>
       <c r="C209" s="0" t="inlineStr">
         <is>
@@ -9536,11 +9500,11 @@
     <row r="210">
       <c r="A210" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayIncrease:value</t>
+          <t xml:space="preserve">future-capex:2026</t>
         </is>
       </c>
       <c r="B210" s="2">
-        <v>2.85</v>
+        <v>15</v>
       </c>
       <c r="C210" s="0" t="inlineStr">
         <is>
@@ -9551,11 +9515,11 @@
     <row r="211">
       <c r="A211" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:investmentSalesRatio:max</t>
+          <t xml:space="preserve">future-capex:2027</t>
         </is>
       </c>
       <c r="B211" s="2">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="C211" s="0" t="inlineStr">
         <is>
@@ -9566,7 +9530,7 @@
     <row r="212">
       <c r="A212" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:investmentSalesRatio:value</t>
+          <t xml:space="preserve">future-capex:2028</t>
         </is>
       </c>
       <c r="B212" s="2">
@@ -9581,56 +9545,56 @@
     <row r="213">
       <c r="A213" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:laborProductivityCagr:max</t>
+          <t xml:space="preserve">future-capex:2029</t>
         </is>
       </c>
       <c r="B213" s="2">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="C213" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:laborProductivityCagr:value</t>
+          <t xml:space="preserve">future-capex:2030</t>
         </is>
       </c>
       <c r="B214" s="2">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="C214" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:localBenchmark:max</t>
+          <t xml:space="preserve">future-capex:2031</t>
         </is>
       </c>
       <c r="B215" s="2">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="C215" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:localBenchmark:value</t>
+          <t xml:space="preserve">target:companyPaySchedule:max</t>
         </is>
       </c>
       <c r="B216" s="2">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="C216" s="0" t="inlineStr">
         <is>
@@ -9641,11 +9605,11 @@
     <row r="217">
       <c r="A217" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayCagr:max</t>
+          <t xml:space="preserve">target:companyPaySchedule:value</t>
         </is>
       </c>
       <c r="B217" s="2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C217" s="0" t="inlineStr">
         <is>
@@ -9656,11 +9620,11 @@
     <row r="218">
       <c r="A218" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayCagr:value</t>
+          <t xml:space="preserve">target:companySalesCagr:max</t>
         </is>
       </c>
       <c r="B218" s="2">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="C218" s="0" t="inlineStr">
         <is>
@@ -9671,26 +9635,26 @@
     <row r="219">
       <c r="A219" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayIncrease:value</t>
+          <t xml:space="preserve">target:companySalesCagr:value</t>
         </is>
       </c>
       <c r="B219" s="2">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="C219" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesCagr:max</t>
+          <t xml:space="preserve">target:companySalesIncrease:max</t>
         </is>
       </c>
       <c r="B220" s="2">
-        <v>35</v>
+        <v>252.69</v>
       </c>
       <c r="C220" s="0" t="inlineStr">
         <is>
@@ -9701,11 +9665,11 @@
     <row r="221">
       <c r="A221" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesCagr:value</t>
+          <t xml:space="preserve">target:companySalesIncrease:value</t>
         </is>
       </c>
       <c r="B221" s="2">
-        <v>22</v>
+        <v>82.4</v>
       </c>
       <c r="C221" s="0" t="inlineStr">
         <is>
@@ -9716,11 +9680,11 @@
     <row r="222">
       <c r="A222" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesIncrease:max</t>
+          <t xml:space="preserve">target:employeePayCagr:max</t>
         </is>
       </c>
       <c r="B222" s="2">
-        <v>136.84</v>
+        <v>10</v>
       </c>
       <c r="C222" s="0" t="inlineStr">
         <is>
@@ -9731,11 +9695,11 @@
     <row r="223">
       <c r="A223" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesIncrease:value</t>
+          <t xml:space="preserve">target:employeePayCagr:value</t>
         </is>
       </c>
       <c r="B223" s="2">
-        <v>74.8</v>
+        <v>7</v>
       </c>
       <c r="C223" s="0" t="inlineStr">
         <is>
@@ -9746,11 +9710,11 @@
     <row r="224">
       <c r="A224" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesShare:max</t>
+          <t xml:space="preserve">target:employeePayIncrease:max</t>
         </is>
       </c>
       <c r="B224" s="2">
-        <v>95</v>
+        <v>3.74</v>
       </c>
       <c r="C224" s="0" t="inlineStr">
         <is>
@@ -9761,11 +9725,11 @@
     <row r="225">
       <c r="A225" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesShare:value</t>
+          <t xml:space="preserve">target:employeePayIncrease:value</t>
         </is>
       </c>
       <c r="B225" s="2">
-        <v>60</v>
+        <v>2.85</v>
       </c>
       <c r="C225" s="0" t="inlineStr">
         <is>
@@ -9776,11 +9740,11 @@
     <row r="226">
       <c r="A226" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:valueAddedIncrease:max</t>
+          <t xml:space="preserve">target:investmentSalesRatio:max</t>
         </is>
       </c>
       <c r="B226" s="2">
-        <v>33.43</v>
+        <v>70</v>
       </c>
       <c r="C226" s="0" t="inlineStr">
         <is>
@@ -9791,11 +9755,11 @@
     <row r="227">
       <c r="A227" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:valueAddedIncrease:value</t>
+          <t xml:space="preserve">target:investmentSalesRatio:value</t>
         </is>
       </c>
       <c r="B227" s="2">
-        <v>18.78</v>
+        <v>15</v>
       </c>
       <c r="C227" s="0" t="inlineStr">
         <is>
@@ -9806,11 +9770,11 @@
     <row r="228">
       <c r="A228" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:valueAddedSubsidyRatio:max</t>
+          <t xml:space="preserve">target:laborProductivityCagr:max</t>
         </is>
       </c>
       <c r="B228" s="2">
-        <v>350</v>
+        <v>35</v>
       </c>
       <c r="C228" s="0" t="inlineStr">
         <is>
@@ -9821,13 +9785,238 @@
     <row r="229">
       <c r="A229" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">target:laborProductivityCagr:value</t>
+        </is>
+      </c>
+      <c r="B229" s="2">
+        <v>21</v>
+      </c>
+      <c r="C229" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:localBenchmark:max</t>
+        </is>
+      </c>
+      <c r="B230" s="2">
+        <v>40</v>
+      </c>
+      <c r="C230" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:localBenchmark:value</t>
+        </is>
+      </c>
+      <c r="B231" s="2">
+        <v>23</v>
+      </c>
+      <c r="C231" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:officerPayCagr:max</t>
+        </is>
+      </c>
+      <c r="B232" s="2">
+        <v>10</v>
+      </c>
+      <c r="C232" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:officerPayCagr:value</t>
+        </is>
+      </c>
+      <c r="B233" s="2">
+        <v>6</v>
+      </c>
+      <c r="C233" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:officerPayIncrease:value</t>
+        </is>
+      </c>
+      <c r="B234" s="2">
+        <v>0</v>
+      </c>
+      <c r="C234" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesCagr:max</t>
+        </is>
+      </c>
+      <c r="B235" s="2">
+        <v>35</v>
+      </c>
+      <c r="C235" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesCagr:value</t>
+        </is>
+      </c>
+      <c r="B236" s="2">
+        <v>22</v>
+      </c>
+      <c r="C236" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesIncrease:max</t>
+        </is>
+      </c>
+      <c r="B237" s="2">
+        <v>136.84</v>
+      </c>
+      <c r="C237" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesIncrease:value</t>
+        </is>
+      </c>
+      <c r="B238" s="2">
+        <v>74.8</v>
+      </c>
+      <c r="C238" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesShare:max</t>
+        </is>
+      </c>
+      <c r="B239" s="2">
+        <v>95</v>
+      </c>
+      <c r="C239" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesShare:value</t>
+        </is>
+      </c>
+      <c r="B240" s="2">
+        <v>60</v>
+      </c>
+      <c r="C240" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:valueAddedIncrease:max</t>
+        </is>
+      </c>
+      <c r="B241" s="2">
+        <v>33.43</v>
+      </c>
+      <c r="C241" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:valueAddedIncrease:value</t>
+        </is>
+      </c>
+      <c r="B242" s="2">
+        <v>18.78</v>
+      </c>
+      <c r="C242" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:valueAddedSubsidyRatio:max</t>
+        </is>
+      </c>
+      <c r="B243" s="2">
+        <v>350</v>
+      </c>
+      <c r="C243" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">target:valueAddedSubsidyRatio:value</t>
         </is>
       </c>
-      <c r="B229" s="2">
+      <c r="B244" s="2">
         <v>213</v>
       </c>
-      <c r="C229" s="0" t="inlineStr">
+      <c r="C244" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">入力済み</t>
         </is>
@@ -9855,7 +10044,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4fX0seyJ5ZWFyIjoyMDI0LCJyb2xlIjoicHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3NiwiY29ncyI6NTEuNjgsImVtcGxveWVlUGF5Ijo1LjU5LCJvZmZpY2VyUGF5IjowLjM4LCJkZXByZWNpYXRpb24iOjEuOSwib3RoZXJTZ2EiOjkuNSwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NS4zMSwiZW1wbG95ZWVCb251cyI6MC4yOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNCwib2ZmaWNlckJvbnVzIjowLjA0LCJjb2dzRGVwcmVjaWF0aW9uIjowLjQ3LCJzZ2FEZXByZWNpYXRpb24iOjEuNDMsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMzh9LCJvdGhlciI6eyJzYWxlcyI6NjcuMiwiY29ncyI6NDUuNywiZW1wbG95ZWVQYXkiOjcuNTQsIm9mZmljZXJQYXkiOjAuNTgsImRlcHJlY2lhdGlvbiI6MS40NCwib3RoZXJTZ2EiOjcuNjgsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3LjE2LCJlbXBsb3llZUJvbnVzIjowLjM4LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjUyLCJvZmZpY2VyQm9udXMiOjAuMDYsImNvZ3NEZXByZWNpYXRpb24iOjAuMjksInNnYURlcHJlY2lhdGlvbiI6MS4xNSwicmVzZWFyY2hEZXZlbG9wbWVudCI6MC4yOX19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwLCJjb2dzIjo1NC40LCJlbXBsb3llZVBheSI6NiwiZW1wbG95ZWVTYWxhcnkiOjUuNywiZW1wbG95ZWVCb251cyI6MC4zLCJvZmZpY2VyUGF5IjowLjQsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzYsIm9mZmljZXJCb251cyI6MC4wNCwiZGVwcmVjaWF0aW9uIjoyLCJjb2dzRGVwcmVjaWF0aW9uIjowLjUsInNnYURlcHJlY2lhdGlvbiI6MS41LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjQsIm90aGVyU2dhIjoxMCwiaGVhZGNvdW50IjoxMDAsIm9mZmljZXJDb3VudCI6Mn0sIm90aGVyIjp7InNhbGVzIjo3MCwiY29ncyI6NDcuNiwiZW1wbG95ZWVQYXkiOjgsImVtcGxveWVlU2FsYXJ5Ijo3LjYsImVtcGxveWVlQm9udXMiOjAuNCwib2ZmaWNlclBheSI6MC42LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjU0LCJvZmZpY2VyQm9udXMiOjAuMDYsImRlcHJlY2lhdGlvbiI6MS41LCJjb2dzRGVwcmVjaWF0aW9uIjowLjMsInNnYURlcHJlY2lhdGlvbiI6MS4yLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjMsIm90aGVyU2dhIjo4LCJoZWFkY291bnQiOjEzMCwib2ZmaWNlckNvdW50IjozfX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMSwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI4NTcxNDI4NTcxNDI4LCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwidXNlZnVsTGlmZSI6MTAsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwxLjY2NTMzNDUzNjkzNzczNDhlLTE2XSwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MzI1MzMwNTAxODQ2OTI3LDAuMDIwNzM1OTk0MTgzMTg5MTY2XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDBdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNDA3NjA4Njk1NjUyMTcxODQsMC4wNDQzODQwNTc5NzEwMTQ1Ml0sIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAwMDEzNDU3NTU2OTM1ODE5NzM3XSwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOlswLjAxOTEzOTQ1NzAyMzcxNzQ0MywwLjAyMDU1MzQ1OTkxNDc2MzA5NV0sIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wMzkxNjY2NjY2NjY2NjY2OCwwLjA0MjUwMDAwMDAwMDAwMDA5XSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RTYWxlc0dyb3d0aCI6WzAuMTUsMC4zXSwib3RoZXJTYWxlc0dyb3d0aCI6WzAuMDYwNzYwODY5NTY1MjE3MTksMC4wNjQzODQwNTc5NzEwMTQ1M10sInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOlswLDAuMDNdLCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6WzAuMDA1LDAuMDA1MTM0NTc1NTY5MzU4MTk3NV0sInByb2plY3RQYXlHcm93dGgiOlswLjA1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMC4wMjQxMzk0NTcwMjM3MTc0NDQsMC4wMjU1NTM0NTk5MTQ3NjMwOTZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGgiOlswLjA0NDE2NjY2NjY2NjY2NjY4LDAuMDQ3NTAwMDAwMDAwMDAwMDldLCJwcm9qZWN0U2dhUmF0ZUVuZCI6WzAuMDg0OTk5OTk5OTk5OTk5OTksMC4xMzVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA4OTI4NTcxNDI4NTcxNDI3LDAuMTE5Mjg1NzE0Mjg1NzE0MjddLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAuMDQyNjMxNTc4OTQ3MzY4MzYsMC4wNjU1NTU1NTU1NTU1NTU1OF0sInVzZWZ1bExpZmUiOls1LDIwXSwiaW52ZXN0bWVudCI6WzE1LDIwMF0sInN1YnNpZHkiOlsxLDUwXSwibG9jYWxCZW5jaG1hcmsiOlswLDEwMF19LCJ0YXJnZXRzIjp7ImNvbXBhbnlTYWxlc0NhZ3IiOnsidmFsdWUiOjE1LCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjgyLjQsIm1heCI6MjUyLjY5LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjoyLCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NjAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo3NC44LCJtYXgiOjEzNi44NCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImxhYm9yUHJvZHVjdGl2aXR5Q2FnciI6eyJ2YWx1ZSI6MjEsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkSW5jcmVhc2UiOnsidmFsdWUiOjE4Ljc4LCJtYXgiOjMzLjQzLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6Mi44NSwibWF4IjozLjc0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiaW52ZXN0bWVudFNhbGVzUmF0aW8iOnsidmFsdWUiOjE1LCJtYXgiOjcwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZFN1YnNpZHlSYXRpbyI6eyJ2YWx1ZSI6MjEzLCJtYXgiOjM1MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImxvY2FsQmVuY2htYXJrIjp7InZhbHVlIjoyMywibWF4Ijo0MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlDYWdyIjp7InZhbHVlIjo2LCJtYXgiOjEwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUluY3JlYXNlIjp7InZhbHVlIjowLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfX0sImZvcmVjYXN0T3ZlcnJpZGVzIjp7IjIwMjk6b3RoZXI6c2FsZXMiOjg1LjEzLCIyMDI5OnByb2plY3Q6Ny04Ijo3Ljl9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2LjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mi43NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTQiOjAuNzMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi03IjozMi42NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTkiOjAuODIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMCI6MC4wOSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEyIjoxMS42NywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEzIjowLjYyLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTQiOjIuNDUsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNSI6MC42NCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEiOjcyLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNCI6MjMuMDQsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny02Ijo2Ljc4LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOCI6NS4xOSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTkiOjAuMzYsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMCI6MS44LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTMiOjkwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xIjoxNDMuMiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTMiOjk3LjM4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNCI6MC43NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTciOjM0LjUyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItOSI6MC44NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMiI6MTIuNDcsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMyI6MC42NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjoyLjU4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTUiOjAuNjcsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xIjo3NiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0LjMyLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNiI6Ny4wNCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTgiOjUuNTksImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTAiOjEuOSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6MC44LCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTkiOjAuOSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjowLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6Mi43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTUiOjAuNywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNCI6MjUuNiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTYiOjcuMywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTgiOjYsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny05IjowLjQsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xMCI6MiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudEFzc2V0cyI6NjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXNoIjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NSwiYmFsYW5jZS1zaGVldDoyMDIzOnRhbmdpYmxlQXNzZXRzIjo1MywiYmFsYW5jZS1zaGVldDoyMDIzOmJ1aWxkaW5ncyI6MTksImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzppbnRhbmdpYmxlQXNzZXRzIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUsImJhbGFuY2Utc2hlZXQ6MjAyMzpsaWFiaWxpdGllcyI6NzUsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50TGlhYmlsaXRpZXMiOjM5LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZExpYWJpbGl0aWVzIjozNiwiYmFsYW5jZS1zaGVldDoyMDIzOmxvbmdUZXJtRGVidCI6MjksImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hhcmVob2xkZXJFcXVpdHkiOjU0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NSwiYmFsYW5jZS1zaGVldDoyMDI0OmFzc2V0cyI6MTQzLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudEFzc2V0cyI6NzIsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNSwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkQXNzZXRzIjo3MSwiYmFsYW5jZS1zaGVldDoyMDI0OnRhbmdpYmxlQXNzZXRzIjo1OCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAsImJhbGFuY2Utc2hlZXQ6MjAyNDptYWNoaW5lcnkiOjI4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c29mdHdhcmUiOjYsImJhbGFuY2Utc2hlZXQ6MjAyNDpsaWFiaWxpdGllcyI6NzksImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZExpYWJpbGl0aWVzIjozOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEsImJhbGFuY2Utc2hlZXQ6MjAyNDpuZXRBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hhcmVob2xkZXJFcXVpdHkiOjYxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBleCI6OCwiYmFsYW5jZS1zaGVldDoyMDI1OmFzc2V0cyI6MTU2LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXNoIjoyNywiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkQXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI1OmJ1aWxkaW5ncyI6MjIsImJhbGFuY2Utc2hlZXQ6MjAyNTptYWNoaW5lcnkiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTppbnRhbmdpYmxlQXNzZXRzIjo5LCJiYWxhbmNlLXNoZWV0OjIwMjU6c29mdHdhcmUiOjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hvcnRUZXJtRGVidCI6MTEsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MCwiYmFsYW5jZS1zaGVldDoyMDI1OmxvbmdUZXJtRGVidCI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpuZXRBc3NldHMiOjczLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBleCI6MTAsImZ1dHVyZS1jYXBleDoyMDI2IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjciOjE1LCJmdXR1cmUtY2FwZXg6MjAyOCI6MTUsImZ1dHVyZS1jYXBleDoyMDI5IjowLCJmdXR1cmUtY2FwZXg6MjAzMCI6MCwiZnV0dXJlLWNhcGV4OjIwMzEiOjAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjEuNjY1MzM0NTM2OTM3NzM0OGUtMTYsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkzMjUzMzA1MDE4NDY5MjcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNzM1OTk0MTgzMTg5MTY2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLjAxOTEzOTQ1NzAyMzcxNzQ0MywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNTUzNDU5OTE0NzYzMDk1LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjAzOTE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNDI1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MCI6MC4xNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjMsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MCI6MC4wMjQxMzk0NTcwMjM3MTc0NDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDoxIjowLjAyNTU1MzQ1OTkxNDc2MzA5NiwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjowLjA0NDE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MSI6MC4wNDc1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjExLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MCI6MC4wODQ5OTk5OTk5OTk5OTk5OSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjEiOjAuMTM1LCJkcml2ZXI6b3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI4NTcxNDI4NTcxNDI4LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjAiOjAuMDg5Mjg1NzE0Mjg1NzE0MjcsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MSI6MC4xMTkyODU3MTQyODU3MTQyNywiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MCI6MC4wNDI2MzE1Nzg5NDczNjgzNiwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjEiOjAuMDY1NTU1NTU1NTU1NTU1NTgsImRyaXZlcjp1c2VmdWxMaWZlIjoxMCwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MCI6NSwiZHJpdmVyLXJhbmdlOnVzZWZ1bExpZmU6MSI6MjAsImRyaXZlcjppbnZlc3RtZW50IjoyMywiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjEiOjIwMCwiZHJpdmVyOnN1YnNpZHkiOjcuNjYsImRyaXZlci1yYW5nZTpzdWJzaWR5OjAiOjEsImRyaXZlci1yYW5nZTpzdWJzaWR5OjEiOjUwLCJkcml2ZXI6bG9jYWxCZW5jaG1hcmsiOjIzLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MCI6MCwiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjEiOjEwMCwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6dmFsdWUiOjE1LCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6dmFsdWUiOjgyLjQsInRhcmdldDpjb21wYW55UGF5U2NoZWR1bGU6dmFsdWUiOjIsInRhcmdldDpjb21wYW55UGF5U2NoZWR1bGU6bWF4Ijo3LCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6dmFsdWUiOjYwLCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6bWF4Ijo5NSwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6dmFsdWUiOjIyLCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6dmFsdWUiOjc0LjgsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6dmFsdWUiOjIxLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOm1heCI6MzUsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6dmFsdWUiOjE4Ljc4LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOnZhbHVlIjo3LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOm1heCI6MTAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOnZhbHVlIjoyLjg1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86dmFsdWUiOjE1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86bWF4Ijo3MCwidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86dmFsdWUiOjIxMywidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86bWF4IjozNTAsInRhcmdldDpsb2NhbEJlbmNobWFyazp2YWx1ZSI6MjMsInRhcmdldDpsb2NhbEJlbmNobWFyazptYXgiOjQwLCJ0YXJnZXQ6b2ZmaWNlclBheUNhZ3I6dmFsdWUiOjYsInRhcmdldDpvZmZpY2VyUGF5Q2FncjptYXgiOjEwLCJ0YXJnZXQ6b2ZmaWNlclBheUluY3JlYXNlOnZhbHVlIjowLCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6bWF4IjoyNTIuNjksInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTptYXgiOjEzNi44NCwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTptYXgiOjMzLjQzLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlJbmNyZWFzZTptYXgiOjMuNzR9LCJtZXRyaWNHcm91cEJhc2VzIjp7ImNvbXBhbnlTYWxlcyI6InJhdGUiLCJwcm9qZWN0U2FsZXMiOiJyYXRlIiwibGFib3JQcm9kdWN0aXZpdHkiOiJyYXRlIiwiZW1wbG95ZWVQYXkiOiJyYXRlIn0sImFwcGxpY2F0aW9uQ2F0ZWdvcnkiOiJnZW5lcmFsIiwiYWRqdXN0ZWREcml2ZXJzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQxMDU5NTc2MDIzMzkxNiwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MS4xNzQxODY0OTEwNjQ0NjZlLTE2LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAxOTk4MjEzNTUxMTg3OTg3MywicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwNjM5MDEyNDk3MjI5MzQsInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MTIwNDUxMzMzMTU3NjMsIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNjA1NTE2MjczMDA1MjcsIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4ODEzNjc1MDA5MTcxMTcsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDYwOTM1Mzk0MzcxNzg1NSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyMDIyNDg3MjE2OTQ2NjczLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU2NTE3ODU5NDUyMTc5LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNDk5MDQ4MTM0MTI2NTU1LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDg5MDA2MjI5OTc1MDgwMSwib3RoZXJQYXlHcm93dGgiOjAuMDI0ODg3NzYxNzEwMzMzMDMsInByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDI5MDQ1NDgyMzk3MjA1MDU1LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU3ODQ4MTQ3MzIzMDg2NjUsInByb2plY3RTZ2FSYXRlRW5kIjowLjEwOTkzMTgwOTE2NDg0ODI0LCJvdGhlclNnYVJhdGVFbmQiOjAuMTA5MjcyNTg5ODcyMTI4MjMsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1Mzc3ODA1NzYyODcxNjMyLCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6MjMsInN1YnNpZHkiOjcuNjYsImxvY2FsQmVuY2htYXJrIjoyM319</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4LCJvcmRpbmFyeUluY29tZSI6MTAuNzMsInByZVRheEluY29tZSI6MTAuNzMsIm5ldEluY29tZSI6Ny41MX19LHsieWVhciI6MjAyNCwicm9sZSI6InByZXZpb3VzIiwicHJvamVjdCI6eyJzYWxlcyI6NzYsImNvZ3MiOjUxLjY4LCJlbXBsb3llZVBheSI6NS41OSwib2ZmaWNlclBheSI6MC4zOCwiZGVwcmVjaWF0aW9uIjoxLjksIm90aGVyU2dhIjo5LjUsImhlYWRjb3VudCI6OTUsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjUuMzEsImVtcGxveWVlQm9udXMiOjAuMjgsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzQsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40Nywic2dhRGVwcmVjaWF0aW9uIjoxLjQzLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM4fSwib3RoZXIiOnsic2FsZXMiOjY3LjIsImNvZ3MiOjQ1LjcsImVtcGxveWVlUGF5Ijo3LjU0LCJvZmZpY2VyUGF5IjowLjU4LCJkZXByZWNpYXRpb24iOjEuNDQsIm90aGVyU2dhIjo3LjY4LCJoZWFkY291bnQiOjEyNSwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ny4xNiwiZW1wbG95ZWVCb251cyI6MC4zOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41Miwib2ZmaWNlckJvbnVzIjowLjA2LCJjb2dzRGVwcmVjaWF0aW9uIjowLjI5LCJzZ2FEZXByZWNpYXRpb24iOjEuMTUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMjksIm9yZGluYXJ5SW5jb21lIjoxMS4wMSwicHJlVGF4SW5jb21lIjoxMS4wMSwibmV0SW5jb21lIjo3LjcxfX0seyJ5ZWFyIjoyMDI1LCJyb2xlIjoibGF0ZXN0IiwicHJvamVjdCI6eyJzYWxlcyI6ODAsImNvZ3MiOjU0LjQsImVtcGxveWVlUGF5Ijo2LCJlbXBsb3llZVNhbGFyeSI6NS43LCJlbXBsb3llZUJvbnVzIjowLjMsIm9mZmljZXJQYXkiOjAuNCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNiwib2ZmaWNlckJvbnVzIjowLjA0LCJkZXByZWNpYXRpb24iOjIsImNvZ3NEZXByZWNpYXRpb24iOjAuNSwic2dhRGVwcmVjaWF0aW9uIjoxLjUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuNCwib3RoZXJTZ2EiOjEwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwLCJjb2dzIjo0Ny42LCJlbXBsb3llZVBheSI6OCwiZW1wbG95ZWVTYWxhcnkiOjcuNiwiZW1wbG95ZWVCb251cyI6MC40LCJvZmZpY2VyUGF5IjowLjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTQsIm9mZmljZXJCb251cyI6MC4wNiwiZGVwcmVjaWF0aW9uIjoxLjUsImNvZ3NEZXByZWNpYXRpb24iOjAuMywic2dhRGVwcmVjaWF0aW9uIjoxLjIsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMywib3RoZXJTZ2EiOjgsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjoxMS4zLCJwcmVUYXhJbmNvbWUiOjExLjMsIm5ldEluY29tZSI6Ny45MX19XSwiYmFsYW5jZVNoZWV0cyI6W3sieWVhciI6MjAyMywiYXNzZXRzIjoxMzIsImN1cnJlbnRBc3NldHMiOjY3LCJjYXNoIjoyNCwiZml4ZWRBc3NldHMiOjY1LCJ0YW5naWJsZUFzc2V0cyI6NTMsImJ1aWxkaW5ncyI6MTksIm1hY2hpbmVyeSI6MjQsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo3LCJzb2Z0d2FyZSI6NSwibGlhYmlsaXRpZXMiOjc1LCJjdXJyZW50TGlhYmlsaXRpZXMiOjM5LCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzYsImxvbmdUZXJtRGVidCI6MjksIm5ldEFzc2V0cyI6NTcsInNoYXJlaG9sZGVyRXF1aXR5Ijo1NCwiY2FwaXRhbCI6MTAsImNhcGV4Ijo1fSx7InllYXIiOjIwMjQsImFzc2V0cyI6MTQzLCJjdXJyZW50QXNzZXRzIjo3MiwiY2FzaCI6MjUsImZpeGVkQXNzZXRzIjo3MSwidGFuZ2libGVBc3NldHMiOjU4LCJidWlsZGluZ3MiOjIwLCJtYWNoaW5lcnkiOjI4LCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OCwic29mdHdhcmUiOjYsImxpYWJpbGl0aWVzIjo3OSwiY3VycmVudExpYWJpbGl0aWVzIjo0MSwic2hvcnRUZXJtRGVidCI6MTIsImZpeGVkTGlhYmlsaXRpZXMiOjM4LCJsb25nVGVybURlYnQiOjMxLCJuZXRBc3NldHMiOjY0LCJzaGFyZWhvbGRlckVxdWl0eSI6NjEsImNhcGl0YWwiOjEwLCJjYXBleCI6OH0seyJ5ZWFyIjoyMDI1LCJhc3NldHMiOjE1NiwiY3VycmVudEFzc2V0cyI6NzgsImNhc2giOjI3LCJmaXhlZEFzc2V0cyI6NzgsInRhbmdpYmxlQXNzZXRzIjo2NCwiYnVpbGRpbmdzIjoyMiwibWFjaGluZXJ5IjozMiwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjksInNvZnR3YXJlIjo3LCJsaWFiaWxpdGllcyI6ODMsImN1cnJlbnRMaWFiaWxpdGllcyI6NDMsInNob3J0VGVybURlYnQiOjExLCJmaXhlZExpYWJpbGl0aWVzIjo0MCwibG9uZ1Rlcm1EZWJ0IjozMiwibmV0QXNzZXRzIjo3Mywic2hhcmVob2xkZXJFcXVpdHkiOjcwLCJjYXBpdGFsIjoxMCwiY2FwZXgiOjEwfV0sImZ1dHVyZUNhcGV4IjpbeyJ5ZWFyIjoyMDI2LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyNywidmFsdWUiOjE1fSx7InllYXIiOjIwMjgsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI5LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMwLCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMxLCJ2YWx1ZSI6MH1dLCJkcml2ZXJzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6NS41NTExMTUxMjMxMjU3ODNlLTE3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5Nywib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI1NzI0NjM3NjgxMTU4NTQsIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksIm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMiwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NzI0NjM3NjgxMTU4NiwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsIm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwicHJvamVjdFBheUdyb3d0aCI6MC4wNywib3RoZXJQYXlHcm93dGgiOjAuMDI0ODQ2NDU4NDY5MjQwMjcsInByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTgzMzMzMzMzMzMzMzM4NiwicHJvamVjdFNnYVJhdGVFbmQiOjAuMTEsIm90aGVyU2dhUmF0ZUVuZCI6MC4xMDkyODU3MTQyODU3MTQyOCwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzODAxMTY5NTkwNjQzMjUsInVzZWZ1bExpZmUiOjEwLCJpbnZlc3RtZW50IjoyMywic3Vic2lkeSI6Ny42NiwibG9jYWxCZW5jaG1hcmsiOjIzfSwiZHJpdmVyUmFuZ2VzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOlstMC4wNSwwLjNdLCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6WzAsMS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNl0sInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOlswLjAxOTMyNTMzMDUwMTg0NjkyNywwLjAyMDczNTk5NDE4MzE4OTE2Nl0sInByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6WzAuMDQwNzYwODY5NTY1MjE3MTg0LDAuMDQ0Mzg0MDU3OTcxMDE0NTJdLCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6WzAsMC4wMDAxMzQ1NzU1NjkzNTgxOTczN10sIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkxMzk0NTcwMjM3MTc0NDMsMC4wMjA1NTM0NTk5MTQ3NjMwOTVdLCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6WzAuMDM5MTY2NjY2NjY2NjY2NjgsMC4wNDI1MDAwMDAwMDAwMDAwOV0sIm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDBdLCJwcm9qZWN0U2FsZXNHcm93dGgiOlswLjE1LDAuM10sIm90aGVyU2FsZXNHcm93dGgiOlswLjA2MDc2MDg2OTU2NTIxNzE5LDAuMDY0Mzg0MDU3OTcxMDE0NTNdLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjpbMCwwLjAzXSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOlswLjAwNSwwLjAwNTEzNDU3NTU2OTM1ODE5NzVdLCJwcm9qZWN0UGF5R3Jvd3RoIjpbMC4wNSwwLjFdLCJvdGhlclBheUdyb3d0aCI6WzAuMDI0MTM5NDU3MDIzNzE3NDQ0LDAuMDI1NTUzNDU5OTE0NzYzMDk2XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6WzAsMC4wOF0sIm90aGVySGVhZGNvdW50R3Jvd3RoIjpbMC4wNDQxNjY2NjY2NjY2NjY2OCwwLjA0NzUwMDAwMDAwMDAwMDA5XSwicHJvamVjdFNnYVJhdGVFbmQiOlswLjA4NDk5OTk5OTk5OTk5OTk5LDAuMTM1XSwib3RoZXJTZ2FSYXRlRW5kIjpbMC4wODkyODU3MTQyODU3MTQyNywwLjExOTI4NTcxNDI4NTcxNDI3XSwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOlswLjA0MjYzMTU3ODk0NzM2ODM2LDAuMDY1NTU1NTU1NTU1NTU1NThdLCJ1c2VmdWxMaWZlIjpbNSwyMF0sImludmVzdG1lbnQiOlsxNSwyMDBdLCJzdWJzaWR5IjpbMSw1MF0sImxvY2FsQmVuY2htYXJrIjpbMCwxMDBdfSwidGFyZ2V0cyI6eyJjb21wYW55U2FsZXNDYWdyIjp7InZhbHVlIjoxNSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo4Mi40LCJtYXgiOjI1Mi42OSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlQYXlTY2hlZHVsZSI6eyJ2YWx1ZSI6MiwibWF4Ijo3LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzU2hhcmUiOnsidmFsdWUiOjYwLCJtYXgiOjk1LCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjIsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6NzQuOCwibWF4IjoxMzYuODQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsYWJvclByb2R1Y3Rpdml0eUNhZ3IiOnsidmFsdWUiOjIxLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZEluY3JlYXNlIjp7InZhbHVlIjoxOC43OCwibWF4IjozMy40MywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5Q2FnciI6eyJ2YWx1ZSI6NywibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5SW5jcmVhc2UiOnsidmFsdWUiOjIuODUsIm1heCI6My43NCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjoxNSwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX19LCJmb3JlY2FzdE92ZXJyaWRlcyI6eyIyMDI5Om90aGVyOnNhbGVzIjo4NS4xMywiMjAyOTpwcm9qZWN0OjctOCI6Ny45fSwiZnV0dXJlSW5wdXRCYXNpcyI6Im90aGVyIiwiaW5wdXRWYWx1ZXMiOnsiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEiOjEzNi40LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMyI6OTIuNzUsImFjdHVhbDpjb21wYW55OjIwMjM6Mi00IjowLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItNyI6MzIuNjUsImFjdHVhbDpjb21wYW55OjIwMjM6Mi05IjowLjgyLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTAiOjAuMDksImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMiI6MTEuNjcsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMyI6MC42MiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE0IjoyLjQ1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTUiOjAuNjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xOCI6MTAuNzMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xOSI6MTAuNzMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yMCI6Ny41MSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTI3IjoyMTAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEiOjcyLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNCI6MjMuMDQsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny02Ijo2Ljc4LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOCI6NS4xOSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTkiOjAuMzYsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMCI6MS44LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTMiOjkwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xIjoxNDMuMiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTMiOjk3LjM4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNCI6MC43NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTciOjM0LjUyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItOSI6MC44NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMiI6MTIuNDcsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMyI6MC42NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjoyLjU4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTUiOjAuNjcsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xOCI6MTEuMDEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xOSI6MTEuMDEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0yMCI6Ny43MSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTI3IjoyMjAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEiOjc2LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNCI6MjQuMzIsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny02Ijo3LjA0LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctOCI6NS41OSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTkiOjAuMzgsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xMCI6MS45LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTMiOjk1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xIjoxNTAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0zIjoxMDIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi00IjowLjgsImFjdHVhbDpjb21wYW55OjIwMjU6Mi03IjozNi40LCJhY3R1YWw6Y29tcGFueToyMDI1OjItOSI6MC45LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEyIjoxMy4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTMiOjAuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE0IjoyLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNSI6MC43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTgiOjExLjMsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xOSI6MTEuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTIwIjo3LjkxLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjciOjIzMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMSI6ODAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNS42LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6Ny4zLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTkiOjAuNCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEwIjoyLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTMiOjEwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTE0IjoyLCJiYWxhbmNlLXNoZWV0OjIwMjM6YXNzZXRzIjoxMzIsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NywiYmFsYW5jZS1zaGVldDoyMDIzOmNhc2giOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRBc3NldHMiOjY1LCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzLCJiYWxhbmNlLXNoZWV0OjIwMjM6YnVpbGRpbmdzIjoxOSwiYmFsYW5jZS1zaGVldDoyMDIzOm1hY2hpbmVyeSI6MjQsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmludGFuZ2libGVBc3NldHMiOjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzb2Z0d2FyZSI6NSwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NSwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRMaWFiaWxpdGllcyI6MzksImJhbGFuY2Utc2hlZXQ6MjAyMzpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2LCJiYWxhbmNlLXNoZWV0OjIwMjM6bG9uZ1Rlcm1EZWJ0IjoyOSwiYmFsYW5jZS1zaGVldDoyMDIzOm5ldEFzc2V0cyI6NTcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGV4Ijo1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50QXNzZXRzIjo3MiwiYmFsYW5jZS1zaGVldDoyMDI0OmNhc2giOjI1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6dGFuZ2libGVBc3NldHMiOjU4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YnVpbGRpbmdzIjoyMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmludGFuZ2libGVBc3NldHMiOjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NiwiYmFsYW5jZS1zaGVldDoyMDI0OmxpYWJpbGl0aWVzIjo3OSwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRMaWFiaWxpdGllcyI6NDEsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkTGlhYmlsaXRpZXMiOjM4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bG9uZ1Rlcm1EZWJ0IjozMSwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaGFyZWhvbGRlckVxdWl0eSI6NjEsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4LCJiYWxhbmNlLXNoZWV0OjIwMjU6YXNzZXRzIjoxNTYsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50QXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3LCJiYWxhbmNlLXNoZWV0OjIwMjU6Zml4ZWRBc3NldHMiOjc4LCJiYWxhbmNlLXNoZWV0OjIwMjU6dGFuZ2libGVBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMiwiYmFsYW5jZS1zaGVldDoyMDI1Om1hY2hpbmVyeSI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjksImJhbGFuY2Utc2hlZXQ6MjAyNTpzb2Z0d2FyZSI6NywiYmFsYW5jZS1zaGVldDoyMDI1OmxpYWJpbGl0aWVzIjo4MywiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaG9ydFRlcm1EZWJ0IjoxMSwiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkTGlhYmlsaXRpZXMiOjQwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMiwiYmFsYW5jZS1zaGVldDoyMDI1Om5ldEFzc2V0cyI6NzMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaGFyZWhvbGRlckVxdWl0eSI6NzAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGV4IjoxMCwiZnV0dXJlLWNhcGV4OjIwMjYiOjE1LCJmdXR1cmUtY2FwZXg6MjAyNyI6MTUsImZ1dHVyZS1jYXBleDoyMDI4IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjkiOjAsImZ1dHVyZS1jYXBleDoyMDMwIjowLCJmdXR1cmUtY2FwZXg6MjAzMSI6MCwiZHJpdmVyOnByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDoxIjowLjMsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjUuNTUxMTE1MTIzMTI1NzgzZS0xNywiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZTowIjowLjAxOTMyNTMzMDUwMTg0NjkyNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA3MzU5OTQxODMxODkxNjYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNTcyNDYzNzY4MTE1ODU0LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZTowIjowLjA0MDc2MDg2OTU2NTIxNzE4NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNDQzODQwNTc5NzEwMTQ1MiwiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjAuMDAwMTM0NTc1NTY5MzU4MTk3MzcsImRyaXZlcjpvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDE5MTM5NDU3MDIzNzE3NDQzLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA1NTM0NTk5MTQ3NjMwOTUsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjAiOjAuMDM5MTY2NjY2NjY2NjY2NjgsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZToxIjowLjA0MjUwMDAwMDAwMDAwMDA5LCJkcml2ZXI6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MCwiZHJpdmVyOnByb2plY3RTYWxlc0dyb3d0aCI6MC4yMiwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDowIjowLjE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjEiOjAuMywiZHJpdmVyOm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTcyNDYzNzY4MTE1ODYsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoOjAiOjAuMDYwNzYwODY5NTY1MjE3MTksImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoOjEiOjAuMDY0Mzg0MDU3OTcxMDE0NTMsImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2U6MSI6MC4wMywiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjAiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MSI6MC4wMDUxMzQ1NzU1NjkzNTgxOTc1LCJkcml2ZXI6cHJvamVjdFBheUdyb3d0aCI6MC4wNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGg6MCI6MC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGg6MSI6MC4xLCJkcml2ZXI6b3RoZXJQYXlHcm93dGgiOjAuMDI0ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDowIjowLjAyNDEzOTQ1NzAyMzcxNzQ0NCwiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjEiOjAuMDI1NTUzNDU5OTE0NzYzMDk2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTgzMzMzMzMzMzMzMzM4NiwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjAiOjAuMDQ0MTY2NjY2NjY2NjY2NjgsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDoxIjowLjA0NzUwMDAwMDAwMDAwMDA5LCJkcml2ZXI6cHJvamVjdFNnYVJhdGVFbmQiOjAuMTEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDowIjowLjA4NDk5OTk5OTk5OTk5OTk5LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MSI6MC4xMzUsImRyaXZlcjpvdGhlclNnYVJhdGVFbmQiOjAuMTA5Mjg1NzE0Mjg1NzE0MjgsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MCI6MC4wODkyODU3MTQyODU3MTQyNywiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDoxIjowLjExOTI4NTcxNDI4NTcxNDI3LCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzODAxMTY5NTkwNjQzMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDowIjowLjA0MjYzMTU3ODk0NzM2ODM2LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MSI6MC4wNjU1NTU1NTU1NTU1NTU1OCwiZHJpdmVyOnVzZWZ1bExpZmUiOjEwLCJkcml2ZXItcmFuZ2U6dXNlZnVsTGlmZTowIjo1LCJkcml2ZXItcmFuZ2U6dXNlZnVsTGlmZToxIjoyMCwiZHJpdmVyOmludmVzdG1lbnQiOjIzLCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDowIjoxNSwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MSI6MjAwLCJkcml2ZXI6c3Vic2lkeSI6Ny42NiwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MCI6MSwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MSI6NTAsImRyaXZlcjpsb2NhbEJlbmNobWFyayI6MjMsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazowIjowLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MSI6MTAwLCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2Fncjp2YWx1ZSI6MTUsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTp2YWx1ZSI6ODIuNCwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTp2YWx1ZSI6MiwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTptYXgiOjcsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTp2YWx1ZSI6NjAsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTptYXgiOjk1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2Fncjp2YWx1ZSI6MjIsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTp2YWx1ZSI6NzQuOCwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2Fncjp2YWx1ZSI6MjEsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6bWF4IjozNSwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTp2YWx1ZSI6MTguNzgsInRhcmdldDplbXBsb3llZVBheUNhZ3I6dmFsdWUiOjcsInRhcmdldDplbXBsb3llZVBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6dmFsdWUiOjIuODUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MTUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTptYXgiOjI1Mi42OSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOm1heCI6MTM2Ljg0LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOm1heCI6MzMuNDMsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOm1heCI6My43NH0sIm1ldHJpY0dyb3VwQmFzZXMiOnsiY29tcGFueVNhbGVzIjoicmF0ZSIsInByb2plY3RTYWxlcyI6InJhdGUiLCJsYWJvclByb2R1Y3Rpdml0eSI6InJhdGUiLCJlbXBsb3llZVBheSI6InJhdGUifSwiYXBwbGljYXRpb25DYXRlZ29yeSI6ImdlbmVyYWwiLCJhZGp1c3RlZERyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDEwNTk1NzYwMjMzOTE2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjoxLjE3NDE4NjQ5MTA2NDQ2NmUtMTYsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDE5OTgyMTM1NTExODc5ODczLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA2MzkwMTI0OTcyMjkzNCwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQxMjA0NTEzMzMxNTc2Mywib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI2MDU1MTYyNzMwMDUyNywib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg4MTM2NzUwMDkxNzExNywib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwNjA5MzUzOTQzNzE3ODU1LCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIwMjI0ODcyMTY5NDY2NzMsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTY1MTc4NTk0NTIxNzksInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE0OTkwNDgxMzQxMjY1NTUsIm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwicHJvamVjdFBheUdyb3d0aCI6MC4wODkwMDYyMjk5NzUwODAxLCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4ODc3NjE3MTAzMzMwMywicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wMjkwNDU0ODIzOTcyMDUwNTUsIm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTc4NDgxNDczMjMwODY2NSwicHJvamVjdFNnYVJhdGVFbmQiOjAuMTA5OTMxODA5MTY0ODQ4MjQsIm90aGVyU2dhUmF0ZUVuZCI6MC4xMDkyNzI1ODk4NzIxMjgyMywicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzNzc4MDU3NjI4NzE2MzIsInVzZWZ1bExpZmUiOjEwLCJpbnZlc3RtZW50IjoyMywic3Vic2lkeSI6Ny42NiwibG9jYWxCZW5jaG1hcmsiOjIzfX0=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Expand other-business PL inputs
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -1839,22 +1839,22 @@
         <v>11.3</v>
       </c>
       <c r="E20" s="4">
-        <v>11.17</v>
+        <v>11.169999999999991</v>
       </c>
       <c r="F20" s="4">
-        <v>11.02</v>
+        <v>11.019999999999996</v>
       </c>
       <c r="G20" s="4">
-        <v>10.86</v>
+        <v>10.860000000000003</v>
       </c>
       <c r="H20" s="4">
-        <v>15.55</v>
+        <v>16.009999999999998</v>
       </c>
       <c r="I20" s="4">
-        <v>21.49</v>
+        <v>22.009999999999984</v>
       </c>
       <c r="J20" s="4">
-        <v>29.12</v>
+        <v>29.700000000000014</v>
       </c>
     </row>
     <row r="21">
@@ -1873,22 +1873,22 @@
         <v>11.3</v>
       </c>
       <c r="E21" s="2">
-        <v>11.17</v>
+        <v>11.169999999999991</v>
       </c>
       <c r="F21" s="2">
-        <v>11.02</v>
+        <v>11.019999999999996</v>
       </c>
       <c r="G21" s="2">
-        <v>10.86</v>
+        <v>10.860000000000003</v>
       </c>
       <c r="H21" s="2">
-        <v>15.55</v>
+        <v>16.009999999999998</v>
       </c>
       <c r="I21" s="2">
-        <v>21.49</v>
+        <v>22.009999999999984</v>
       </c>
       <c r="J21" s="2">
-        <v>29.12</v>
+        <v>29.700000000000014</v>
       </c>
     </row>
     <row r="22">
@@ -1907,22 +1907,22 @@
         <v>7.91</v>
       </c>
       <c r="E22" s="2">
-        <v>7.82</v>
+        <v>7.815999999999994</v>
       </c>
       <c r="F22" s="2">
-        <v>7.71</v>
+        <v>7.711999999999997</v>
       </c>
       <c r="G22" s="2">
-        <v>7.6</v>
+        <v>7.5980000000000025</v>
       </c>
       <c r="H22" s="2">
-        <v>10.88</v>
+        <v>11.197999999999997</v>
       </c>
       <c r="I22" s="2">
-        <v>15.04</v>
+        <v>15.402999999999988</v>
       </c>
       <c r="J22" s="2">
-        <v>20.38</v>
+        <v>20.78200000000001</v>
       </c>
     </row>
     <row r="23">
@@ -10044,7 +10044,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4LCJvcmRpbmFyeUluY29tZSI6MTAuNzMsInByZVRheEluY29tZSI6MTAuNzMsIm5ldEluY29tZSI6Ny41MX19LHsieWVhciI6MjAyNCwicm9sZSI6InByZXZpb3VzIiwicHJvamVjdCI6eyJzYWxlcyI6NzYsImNvZ3MiOjUxLjY4LCJlbXBsb3llZVBheSI6NS41OSwib2ZmaWNlclBheSI6MC4zOCwiZGVwcmVjaWF0aW9uIjoxLjksIm90aGVyU2dhIjo5LjUsImhlYWRjb3VudCI6OTUsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjUuMzEsImVtcGxveWVlQm9udXMiOjAuMjgsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzQsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40Nywic2dhRGVwcmVjaWF0aW9uIjoxLjQzLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM4fSwib3RoZXIiOnsic2FsZXMiOjY3LjIsImNvZ3MiOjQ1LjcsImVtcGxveWVlUGF5Ijo3LjU0LCJvZmZpY2VyUGF5IjowLjU4LCJkZXByZWNpYXRpb24iOjEuNDQsIm90aGVyU2dhIjo3LjY4LCJoZWFkY291bnQiOjEyNSwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ny4xNiwiZW1wbG95ZWVCb251cyI6MC4zOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41Miwib2ZmaWNlckJvbnVzIjowLjA2LCJjb2dzRGVwcmVjaWF0aW9uIjowLjI5LCJzZ2FEZXByZWNpYXRpb24iOjEuMTUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMjksIm9yZGluYXJ5SW5jb21lIjoxMS4wMSwicHJlVGF4SW5jb21lIjoxMS4wMSwibmV0SW5jb21lIjo3LjcxfX0seyJ5ZWFyIjoyMDI1LCJyb2xlIjoibGF0ZXN0IiwicHJvamVjdCI6eyJzYWxlcyI6ODAsImNvZ3MiOjU0LjQsImVtcGxveWVlUGF5Ijo2LCJlbXBsb3llZVNhbGFyeSI6NS43LCJlbXBsb3llZUJvbnVzIjowLjMsIm9mZmljZXJQYXkiOjAuNCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNiwib2ZmaWNlckJvbnVzIjowLjA0LCJkZXByZWNpYXRpb24iOjIsImNvZ3NEZXByZWNpYXRpb24iOjAuNSwic2dhRGVwcmVjaWF0aW9uIjoxLjUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuNCwib3RoZXJTZ2EiOjEwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwLCJjb2dzIjo0Ny42LCJlbXBsb3llZVBheSI6OCwiZW1wbG95ZWVTYWxhcnkiOjcuNiwiZW1wbG95ZWVCb251cyI6MC40LCJvZmZpY2VyUGF5IjowLjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTQsIm9mZmljZXJCb251cyI6MC4wNiwiZGVwcmVjaWF0aW9uIjoxLjUsImNvZ3NEZXByZWNpYXRpb24iOjAuMywic2dhRGVwcmVjaWF0aW9uIjoxLjIsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMywib3RoZXJTZ2EiOjgsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjoxMS4zLCJwcmVUYXhJbmNvbWUiOjExLjMsIm5ldEluY29tZSI6Ny45MX19XSwiYmFsYW5jZVNoZWV0cyI6W3sieWVhciI6MjAyMywiYXNzZXRzIjoxMzIsImN1cnJlbnRBc3NldHMiOjY3LCJjYXNoIjoyNCwiZml4ZWRBc3NldHMiOjY1LCJ0YW5naWJsZUFzc2V0cyI6NTMsImJ1aWxkaW5ncyI6MTksIm1hY2hpbmVyeSI6MjQsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo3LCJzb2Z0d2FyZSI6NSwibGlhYmlsaXRpZXMiOjc1LCJjdXJyZW50TGlhYmlsaXRpZXMiOjM5LCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzYsImxvbmdUZXJtRGVidCI6MjksIm5ldEFzc2V0cyI6NTcsInNoYXJlaG9sZGVyRXF1aXR5Ijo1NCwiY2FwaXRhbCI6MTAsImNhcGV4Ijo1fSx7InllYXIiOjIwMjQsImFzc2V0cyI6MTQzLCJjdXJyZW50QXNzZXRzIjo3MiwiY2FzaCI6MjUsImZpeGVkQXNzZXRzIjo3MSwidGFuZ2libGVBc3NldHMiOjU4LCJidWlsZGluZ3MiOjIwLCJtYWNoaW5lcnkiOjI4LCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OCwic29mdHdhcmUiOjYsImxpYWJpbGl0aWVzIjo3OSwiY3VycmVudExpYWJpbGl0aWVzIjo0MSwic2hvcnRUZXJtRGVidCI6MTIsImZpeGVkTGlhYmlsaXRpZXMiOjM4LCJsb25nVGVybURlYnQiOjMxLCJuZXRBc3NldHMiOjY0LCJzaGFyZWhvbGRlckVxdWl0eSI6NjEsImNhcGl0YWwiOjEwLCJjYXBleCI6OH0seyJ5ZWFyIjoyMDI1LCJhc3NldHMiOjE1NiwiY3VycmVudEFzc2V0cyI6NzgsImNhc2giOjI3LCJmaXhlZEFzc2V0cyI6NzgsInRhbmdpYmxlQXNzZXRzIjo2NCwiYnVpbGRpbmdzIjoyMiwibWFjaGluZXJ5IjozMiwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjksInNvZnR3YXJlIjo3LCJsaWFiaWxpdGllcyI6ODMsImN1cnJlbnRMaWFiaWxpdGllcyI6NDMsInNob3J0VGVybURlYnQiOjExLCJmaXhlZExpYWJpbGl0aWVzIjo0MCwibG9uZ1Rlcm1EZWJ0IjozMiwibmV0QXNzZXRzIjo3Mywic2hhcmVob2xkZXJFcXVpdHkiOjcwLCJjYXBpdGFsIjoxMCwiY2FwZXgiOjEwfV0sImZ1dHVyZUNhcGV4IjpbeyJ5ZWFyIjoyMDI2LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyNywidmFsdWUiOjE1fSx7InllYXIiOjIwMjgsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI5LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMwLCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMxLCJ2YWx1ZSI6MH1dLCJkcml2ZXJzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6NS41NTExMTUxMjMxMjU3ODNlLTE3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5Nywib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI1NzI0NjM3NjgxMTU4NTQsIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksIm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMiwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NzI0NjM3NjgxMTU4NiwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsIm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwicHJvamVjdFBheUdyb3d0aCI6MC4wNywib3RoZXJQYXlHcm93dGgiOjAuMDI0ODQ2NDU4NDY5MjQwMjcsInByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTgzMzMzMzMzMzMzMzM4NiwicHJvamVjdFNnYVJhdGVFbmQiOjAuMTEsIm90aGVyU2dhUmF0ZUVuZCI6MC4xMDkyODU3MTQyODU3MTQyOCwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzODAxMTY5NTkwNjQzMjUsInVzZWZ1bExpZmUiOjEwLCJpbnZlc3RtZW50IjoyMywic3Vic2lkeSI6Ny42NiwibG9jYWxCZW5jaG1hcmsiOjIzfSwiZHJpdmVyUmFuZ2VzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOlstMC4wNSwwLjNdLCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6WzAsMS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNl0sInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOlswLjAxOTMyNTMzMDUwMTg0NjkyNywwLjAyMDczNTk5NDE4MzE4OTE2Nl0sInByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6WzAuMDQwNzYwODY5NTY1MjE3MTg0LDAuMDQ0Mzg0MDU3OTcxMDE0NTJdLCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6WzAsMC4wMDAxMzQ1NzU1NjkzNTgxOTczN10sIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkxMzk0NTcwMjM3MTc0NDMsMC4wMjA1NTM0NTk5MTQ3NjMwOTVdLCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6WzAuMDM5MTY2NjY2NjY2NjY2NjgsMC4wNDI1MDAwMDAwMDAwMDAwOV0sIm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDBdLCJwcm9qZWN0U2FsZXNHcm93dGgiOlswLjE1LDAuM10sIm90aGVyU2FsZXNHcm93dGgiOlswLjA2MDc2MDg2OTU2NTIxNzE5LDAuMDY0Mzg0MDU3OTcxMDE0NTNdLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjpbMCwwLjAzXSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOlswLjAwNSwwLjAwNTEzNDU3NTU2OTM1ODE5NzVdLCJwcm9qZWN0UGF5R3Jvd3RoIjpbMC4wNSwwLjFdLCJvdGhlclBheUdyb3d0aCI6WzAuMDI0MTM5NDU3MDIzNzE3NDQ0LDAuMDI1NTUzNDU5OTE0NzYzMDk2XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6WzAsMC4wOF0sIm90aGVySGVhZGNvdW50R3Jvd3RoIjpbMC4wNDQxNjY2NjY2NjY2NjY2OCwwLjA0NzUwMDAwMDAwMDAwMDA5XSwicHJvamVjdFNnYVJhdGVFbmQiOlswLjA4NDk5OTk5OTk5OTk5OTk5LDAuMTM1XSwib3RoZXJTZ2FSYXRlRW5kIjpbMC4wODkyODU3MTQyODU3MTQyNywwLjExOTI4NTcxNDI4NTcxNDI3XSwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOlswLjA0MjYzMTU3ODk0NzM2ODM2LDAuMDY1NTU1NTU1NTU1NTU1NThdLCJ1c2VmdWxMaWZlIjpbNSwyMF0sImludmVzdG1lbnQiOlsxNSwyMDBdLCJzdWJzaWR5IjpbMSw1MF0sImxvY2FsQmVuY2htYXJrIjpbMCwxMDBdfSwidGFyZ2V0cyI6eyJjb21wYW55U2FsZXNDYWdyIjp7InZhbHVlIjoxNSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo4Mi40LCJtYXgiOjI1Mi42OSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlQYXlTY2hlZHVsZSI6eyJ2YWx1ZSI6MiwibWF4Ijo3LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzU2hhcmUiOnsidmFsdWUiOjYwLCJtYXgiOjk1LCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjIsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6NzQuOCwibWF4IjoxMzYuODQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsYWJvclByb2R1Y3Rpdml0eUNhZ3IiOnsidmFsdWUiOjIxLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZEluY3JlYXNlIjp7InZhbHVlIjoxOC43OCwibWF4IjozMy40MywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5Q2FnciI6eyJ2YWx1ZSI6NywibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5SW5jcmVhc2UiOnsidmFsdWUiOjIuODUsIm1heCI6My43NCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjoxNSwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX19LCJmb3JlY2FzdE92ZXJyaWRlcyI6eyIyMDI5Om90aGVyOnNhbGVzIjo4NS4xMywiMjAyOTpwcm9qZWN0OjctOCI6Ny45fSwiZnV0dXJlSW5wdXRCYXNpcyI6Im90aGVyIiwiaW5wdXRWYWx1ZXMiOnsiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEiOjEzNi40LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMyI6OTIuNzUsImFjdHVhbDpjb21wYW55OjIwMjM6Mi00IjowLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItNyI6MzIuNjUsImFjdHVhbDpjb21wYW55OjIwMjM6Mi05IjowLjgyLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTAiOjAuMDksImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMiI6MTEuNjcsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMyI6MC42MiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE0IjoyLjQ1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTUiOjAuNjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xOCI6MTAuNzMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xOSI6MTAuNzMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yMCI6Ny41MSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTI3IjoyMTAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEiOjcyLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNCI6MjMuMDQsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny02Ijo2Ljc4LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOCI6NS4xOSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTkiOjAuMzYsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMCI6MS44LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTMiOjkwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xIjoxNDMuMiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTMiOjk3LjM4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNCI6MC43NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTciOjM0LjUyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItOSI6MC44NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMiI6MTIuNDcsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMyI6MC42NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjoyLjU4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTUiOjAuNjcsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xOCI6MTEuMDEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xOSI6MTEuMDEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0yMCI6Ny43MSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTI3IjoyMjAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEiOjc2LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNCI6MjQuMzIsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny02Ijo3LjA0LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctOCI6NS41OSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTkiOjAuMzgsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xMCI6MS45LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTMiOjk1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xIjoxNTAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0zIjoxMDIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi00IjowLjgsImFjdHVhbDpjb21wYW55OjIwMjU6Mi03IjozNi40LCJhY3R1YWw6Y29tcGFueToyMDI1OjItOSI6MC45LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEyIjoxMy4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTMiOjAuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE0IjoyLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNSI6MC43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTgiOjExLjMsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xOSI6MTEuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTIwIjo3LjkxLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjciOjIzMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMSI6ODAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNS42LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6Ny4zLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTkiOjAuNCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEwIjoyLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTMiOjEwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTE0IjoyLCJiYWxhbmNlLXNoZWV0OjIwMjM6YXNzZXRzIjoxMzIsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NywiYmFsYW5jZS1zaGVldDoyMDIzOmNhc2giOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRBc3NldHMiOjY1LCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzLCJiYWxhbmNlLXNoZWV0OjIwMjM6YnVpbGRpbmdzIjoxOSwiYmFsYW5jZS1zaGVldDoyMDIzOm1hY2hpbmVyeSI6MjQsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmludGFuZ2libGVBc3NldHMiOjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzb2Z0d2FyZSI6NSwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NSwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRMaWFiaWxpdGllcyI6MzksImJhbGFuY2Utc2hlZXQ6MjAyMzpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2LCJiYWxhbmNlLXNoZWV0OjIwMjM6bG9uZ1Rlcm1EZWJ0IjoyOSwiYmFsYW5jZS1zaGVldDoyMDIzOm5ldEFzc2V0cyI6NTcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGV4Ijo1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50QXNzZXRzIjo3MiwiYmFsYW5jZS1zaGVldDoyMDI0OmNhc2giOjI1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6dGFuZ2libGVBc3NldHMiOjU4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YnVpbGRpbmdzIjoyMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmludGFuZ2libGVBc3NldHMiOjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NiwiYmFsYW5jZS1zaGVldDoyMDI0OmxpYWJpbGl0aWVzIjo3OSwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRMaWFiaWxpdGllcyI6NDEsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkTGlhYmlsaXRpZXMiOjM4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bG9uZ1Rlcm1EZWJ0IjozMSwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaGFyZWhvbGRlckVxdWl0eSI6NjEsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4LCJiYWxhbmNlLXNoZWV0OjIwMjU6YXNzZXRzIjoxNTYsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50QXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3LCJiYWxhbmNlLXNoZWV0OjIwMjU6Zml4ZWRBc3NldHMiOjc4LCJiYWxhbmNlLXNoZWV0OjIwMjU6dGFuZ2libGVBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMiwiYmFsYW5jZS1zaGVldDoyMDI1Om1hY2hpbmVyeSI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjksImJhbGFuY2Utc2hlZXQ6MjAyNTpzb2Z0d2FyZSI6NywiYmFsYW5jZS1zaGVldDoyMDI1OmxpYWJpbGl0aWVzIjo4MywiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaG9ydFRlcm1EZWJ0IjoxMSwiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkTGlhYmlsaXRpZXMiOjQwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMiwiYmFsYW5jZS1zaGVldDoyMDI1Om5ldEFzc2V0cyI6NzMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaGFyZWhvbGRlckVxdWl0eSI6NzAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGV4IjoxMCwiZnV0dXJlLWNhcGV4OjIwMjYiOjE1LCJmdXR1cmUtY2FwZXg6MjAyNyI6MTUsImZ1dHVyZS1jYXBleDoyMDI4IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjkiOjAsImZ1dHVyZS1jYXBleDoyMDMwIjowLCJmdXR1cmUtY2FwZXg6MjAzMSI6MCwiZHJpdmVyOnByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDoxIjowLjMsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjUuNTUxMTE1MTIzMTI1NzgzZS0xNywiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZTowIjowLjAxOTMyNTMzMDUwMTg0NjkyNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA3MzU5OTQxODMxODkxNjYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNTcyNDYzNzY4MTE1ODU0LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZTowIjowLjA0MDc2MDg2OTU2NTIxNzE4NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNDQzODQwNTc5NzEwMTQ1MiwiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjAuMDAwMTM0NTc1NTY5MzU4MTk3MzcsImRyaXZlcjpvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDE5MTM5NDU3MDIzNzE3NDQzLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA1NTM0NTk5MTQ3NjMwOTUsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjAiOjAuMDM5MTY2NjY2NjY2NjY2NjgsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZToxIjowLjA0MjUwMDAwMDAwMDAwMDA5LCJkcml2ZXI6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MCwiZHJpdmVyOnByb2plY3RTYWxlc0dyb3d0aCI6MC4yMiwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDowIjowLjE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjEiOjAuMywiZHJpdmVyOm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTcyNDYzNzY4MTE1ODYsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoOjAiOjAuMDYwNzYwODY5NTY1MjE3MTksImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoOjEiOjAuMDY0Mzg0MDU3OTcxMDE0NTMsImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2U6MSI6MC4wMywiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjAiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MSI6MC4wMDUxMzQ1NzU1NjkzNTgxOTc1LCJkcml2ZXI6cHJvamVjdFBheUdyb3d0aCI6MC4wNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGg6MCI6MC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGg6MSI6MC4xLCJkcml2ZXI6b3RoZXJQYXlHcm93dGgiOjAuMDI0ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDowIjowLjAyNDEzOTQ1NzAyMzcxNzQ0NCwiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjEiOjAuMDI1NTUzNDU5OTE0NzYzMDk2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTgzMzMzMzMzMzMzMzM4NiwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjAiOjAuMDQ0MTY2NjY2NjY2NjY2NjgsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDoxIjowLjA0NzUwMDAwMDAwMDAwMDA5LCJkcml2ZXI6cHJvamVjdFNnYVJhdGVFbmQiOjAuMTEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDowIjowLjA4NDk5OTk5OTk5OTk5OTk5LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MSI6MC4xMzUsImRyaXZlcjpvdGhlclNnYVJhdGVFbmQiOjAuMTA5Mjg1NzE0Mjg1NzE0MjgsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MCI6MC4wODkyODU3MTQyODU3MTQyNywiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDoxIjowLjExOTI4NTcxNDI4NTcxNDI3LCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzODAxMTY5NTkwNjQzMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDowIjowLjA0MjYzMTU3ODk0NzM2ODM2LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MSI6MC4wNjU1NTU1NTU1NTU1NTU1OCwiZHJpdmVyOnVzZWZ1bExpZmUiOjEwLCJkcml2ZXItcmFuZ2U6dXNlZnVsTGlmZTowIjo1LCJkcml2ZXItcmFuZ2U6dXNlZnVsTGlmZToxIjoyMCwiZHJpdmVyOmludmVzdG1lbnQiOjIzLCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDowIjoxNSwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MSI6MjAwLCJkcml2ZXI6c3Vic2lkeSI6Ny42NiwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MCI6MSwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MSI6NTAsImRyaXZlcjpsb2NhbEJlbmNobWFyayI6MjMsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazowIjowLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MSI6MTAwLCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2Fncjp2YWx1ZSI6MTUsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTp2YWx1ZSI6ODIuNCwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTp2YWx1ZSI6MiwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTptYXgiOjcsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTp2YWx1ZSI6NjAsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTptYXgiOjk1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2Fncjp2YWx1ZSI6MjIsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTp2YWx1ZSI6NzQuOCwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2Fncjp2YWx1ZSI6MjEsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6bWF4IjozNSwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTp2YWx1ZSI6MTguNzgsInRhcmdldDplbXBsb3llZVBheUNhZ3I6dmFsdWUiOjcsInRhcmdldDplbXBsb3llZVBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6dmFsdWUiOjIuODUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MTUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTptYXgiOjI1Mi42OSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOm1heCI6MTM2Ljg0LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOm1heCI6MzMuNDMsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOm1heCI6My43NH0sIm1ldHJpY0dyb3VwQmFzZXMiOnsiY29tcGFueVNhbGVzIjoicmF0ZSIsInByb2plY3RTYWxlcyI6InJhdGUiLCJsYWJvclByb2R1Y3Rpdml0eSI6InJhdGUiLCJlbXBsb3llZVBheSI6InJhdGUifSwiYXBwbGljYXRpb25DYXRlZ29yeSI6ImdlbmVyYWwiLCJhZGp1c3RlZERyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDEwNTk1NzYwMjMzOTE2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjoxLjE3NDE4NjQ5MTA2NDQ2NmUtMTYsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDE5OTgyMTM1NTExODc5ODczLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA2MzkwMTI0OTcyMjkzNCwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQxMjA0NTEzMzMxNTc2Mywib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI2MDU1MTYyNzMwMDUyNywib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg4MTM2NzUwMDkxNzExNywib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwNjA5MzUzOTQzNzE3ODU1LCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIwMjI0ODcyMTY5NDY2NzMsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTY1MTc4NTk0NTIxNzksInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE0OTkwNDgxMzQxMjY1NTUsIm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwicHJvamVjdFBheUdyb3d0aCI6MC4wODkwMDYyMjk5NzUwODAxLCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4ODc3NjE3MTAzMzMwMywicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wMjkwNDU0ODIzOTcyMDUwNTUsIm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTc4NDgxNDczMjMwODY2NSwicHJvamVjdFNnYVJhdGVFbmQiOjAuMTA5OTMxODA5MTY0ODQ4MjQsIm90aGVyU2dhUmF0ZUVuZCI6MC4xMDkyNzI1ODk4NzIxMjgyMywicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzNzc4MDU3NjI4NzE2MzIsInVzZWZ1bExpZmUiOjEwLCJpbnZlc3RtZW50IjoyMywic3Vic2lkeSI6Ny42NiwibG9jYWxCZW5jaG1hcmsiOjIzfX0=</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4LCJvcmRpbmFyeUluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsInByZVRheEluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsIm5ldEluY29tZSI6Mi43NjQwMDAwMDAwMDAwMDJ9fSx7InllYXIiOjIwMjQsInJvbGUiOiJwcmV2aW91cyIsInByb2plY3QiOnsic2FsZXMiOjc2LCJjb2dzIjo1MS42OCwiZW1wbG95ZWVQYXkiOjUuNTksIm9mZmljZXJQYXkiOjAuMzgsImRlcHJlY2lhdGlvbiI6MS45LCJvdGhlclNnYSI6OS41LCJoZWFkY291bnQiOjk1LCJvZmZpY2VyQ291bnQiOjIsImVtcGxveWVlU2FsYXJ5Ijo1LjMxLCJlbXBsb3llZUJvbnVzIjowLjI4LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjM0LCJvZmZpY2VyQm9udXMiOjAuMDQsImNvZ3NEZXByZWNpYXRpb24iOjAuNDcsInNnYURlcHJlY2lhdGlvbiI6MS40MywicmVzZWFyY2hEZXZlbG9wbWVudCI6MC4zOH0sIm90aGVyIjp7InNhbGVzIjo2Ny4yLCJjb2dzIjo0NS43LCJlbXBsb3llZVBheSI6Ny41NCwib2ZmaWNlclBheSI6MC41OCwiZGVwcmVjaWF0aW9uIjoxLjQ0LCJvdGhlclNnYSI6Ny42OCwiaGVhZGNvdW50IjoxMjUsIm9mZmljZXJDb3VudCI6MywiZW1wbG95ZWVTYWxhcnkiOjcuMTYsImVtcGxveWVlQm9udXMiOjAuMzgsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTIsIm9mZmljZXJCb251cyI6MC4wNiwiY29nc0RlcHJlY2lhdGlvbiI6MC4yOSwic2dhRGVwcmVjaWF0aW9uIjoxLjE1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI5LCJvcmRpbmFyeUluY29tZSI6My45Njk5OTk5OTk5OTk5OTcsInByZVRheEluY29tZSI6My45Njk5OTk5OTk5OTk5OTcsIm5ldEluY29tZSI6Mi43ODE5OTk5OTk5OTk5OTgzfX0seyJ5ZWFyIjoyMDI1LCJyb2xlIjoibGF0ZXN0IiwicHJvamVjdCI6eyJzYWxlcyI6ODAsImNvZ3MiOjU0LjQsImVtcGxveWVlUGF5Ijo2LCJlbXBsb3llZVNhbGFyeSI6NS43LCJlbXBsb3llZUJvbnVzIjowLjMsIm9mZmljZXJQYXkiOjAuNCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNiwib2ZmaWNlckJvbnVzIjowLjA0LCJkZXByZWNpYXRpb24iOjIsImNvZ3NEZXByZWNpYXRpb24iOjAuNSwic2dhRGVwcmVjaWF0aW9uIjoxLjUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuNCwib3RoZXJTZ2EiOjEwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwLCJjb2dzIjo0Ny42LCJlbXBsb3llZVBheSI6OCwiZW1wbG95ZWVTYWxhcnkiOjcuNiwiZW1wbG95ZWVCb251cyI6MC40LCJvZmZpY2VyUGF5IjowLjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTQsIm9mZmljZXJCb251cyI6MC4wNiwiZGVwcmVjaWF0aW9uIjoxLjUsImNvZ3NEZXByZWNpYXRpb24iOjAuMywic2dhRGVwcmVjaWF0aW9uIjoxLjIsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMywib3RoZXJTZ2EiOjgsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjozLjk5OTk5OTk5OTk5OTk5NjQsInByZVRheEluY29tZSI6My45OTk5OTk5OTk5OTk5OTY0LCJuZXRJbmNvbWUiOjIuNzk5OTk5OTk5OTk5OTk3fX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMSwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI4NTcxNDI4NTcxNDI4LCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwidXNlZnVsTGlmZSI6MTAsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwxLjY2NTMzNDUzNjkzNzczNDhlLTE2XSwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MzI1MzMwNTAxODQ2OTI3LDAuMDIwNzM1OTk0MTgzMTg5MTY2XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDBdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNDA3NjA4Njk1NjUyMTcxODQsMC4wNDQzODQwNTc5NzEwMTQ1Ml0sIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAwMDEzNDU3NTU2OTM1ODE5NzM3XSwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOlswLjAxOTEzOTQ1NzAyMzcxNzQ0MywwLjAyMDU1MzQ1OTkxNDc2MzA5NV0sIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wMzkxNjY2NjY2NjY2NjY2OCwwLjA0MjUwMDAwMDAwMDAwMDA5XSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RTYWxlc0dyb3d0aCI6WzAuMTUsMC4zXSwib3RoZXJTYWxlc0dyb3d0aCI6WzAuMDYwNzYwODY5NTY1MjE3MTksMC4wNjQzODQwNTc5NzEwMTQ1M10sInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOlswLDAuMDNdLCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6WzAuMDA1LDAuMDA1MTM0NTc1NTY5MzU4MTk3NV0sInByb2plY3RQYXlHcm93dGgiOlswLjA1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMC4wMjQxMzk0NTcwMjM3MTc0NDQsMC4wMjU1NTM0NTk5MTQ3NjMwOTZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGgiOlswLjA0NDE2NjY2NjY2NjY2NjY4LDAuMDQ3NTAwMDAwMDAwMDAwMDldLCJwcm9qZWN0U2dhUmF0ZUVuZCI6WzAuMDg0OTk5OTk5OTk5OTk5OTksMC4xMzVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA4OTI4NTcxNDI4NTcxNDI3LDAuMTE5Mjg1NzE0Mjg1NzE0MjddLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAuMDQyNjMxNTc4OTQ3MzY4MzYsMC4wNjU1NTU1NTU1NTU1NTU1OF0sInVzZWZ1bExpZmUiOls1LDIwXSwiaW52ZXN0bWVudCI6WzE1LDIwMF0sInN1YnNpZHkiOlsxLDUwXSwibG9jYWxCZW5jaG1hcmsiOlswLDEwMF19LCJ0YXJnZXRzIjp7ImNvbXBhbnlTYWxlc0NhZ3IiOnsidmFsdWUiOjE1LCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjgyLjQsIm1heCI6MjUyLjY5LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjoyLCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NjAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo3NC44LCJtYXgiOjEzNi44NCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImxhYm9yUHJvZHVjdGl2aXR5Q2FnciI6eyJ2YWx1ZSI6MjEsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkSW5jcmVhc2UiOnsidmFsdWUiOjE4Ljc4LCJtYXgiOjMzLjQzLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6Mi44NSwibWF4IjozLjc0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiaW52ZXN0bWVudFNhbGVzUmF0aW8iOnsidmFsdWUiOjE1LCJtYXgiOjcwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZFN1YnNpZHlSYXRpbyI6eyJ2YWx1ZSI6MjEzLCJtYXgiOjM1MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImxvY2FsQmVuY2htYXJrIjp7InZhbHVlIjoyMywibWF4Ijo0MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlDYWdyIjp7InZhbHVlIjo2LCJtYXgiOjEwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUluY3JlYXNlIjp7InZhbHVlIjowLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfX0sImZvcmVjYXN0T3ZlcnJpZGVzIjp7IjIwMjk6b3RoZXI6c2FsZXMiOjg1LjEzLCIyMDI5OnByb2plY3Q6Ny04Ijo3Ljl9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2LjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mi43NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTQiOjAuNzMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi03IjozMi42NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTkiOjAuODIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMCI6MC4wOSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEyIjoxMS42NywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEzIjowLjYyLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTQiOjIuNDUsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNSI6MC42NCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE4IjoxMC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE5IjoxMC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTIwIjo3LjUxLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjciOjIxMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMSI6NzIsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny00IjoyMy4wNCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjYuNzgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny04Ijo1LjE5LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOSI6MC4zNiwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEwIjoxLjgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMyI6OTAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEiOjE0My4yLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMyI6OTcuMzgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi00IjowLjc2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNyI6MzQuNTIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi05IjowLjg2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEyIjoxMi40NywiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEzIjowLjY2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTQiOjIuNTgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNSI6MC42NywiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE4IjoxMS4wMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE5IjoxMS4wMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTIwIjo3LjcxLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjciOjIyMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMSI6NzYsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny00IjoyNC4zMiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTYiOjcuMDQsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny04Ijo1LjU5LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctOSI6MC4zOCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEwIjoxLjksImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xMyI6OTUsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEiOjE1MCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTMiOjEwMiwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTQiOjAuOCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTciOjM2LjQsImFjdHVhbDpjb21wYW55OjIwMjU6Mi05IjowLjksImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMCI6MC4xLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTIiOjEzLjMsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMyI6MC43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTQiOjIuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE1IjowLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xOCI6MTEuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE5IjoxMS4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjAiOjcuOTEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yNyI6MjMwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xIjo4MCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTQiOjI1LjYsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny02Ijo3LjMsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny04Ijo2LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOSI6MC40LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTAiOjIsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xMyI6MTAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTQiOjIsImJhbGFuY2Utc2hlZXQ6MjAyMzphc3NldHMiOjEzMiwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRBc3NldHMiOjY3LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FzaCI6MjQsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZEFzc2V0cyI6NjUsImJhbGFuY2Utc2hlZXQ6MjAyMzp0YW5naWJsZUFzc2V0cyI6NTMsImJhbGFuY2Utc2hlZXQ6MjAyMzpidWlsZGluZ3MiOjE5LCJiYWxhbmNlLXNoZWV0OjIwMjM6bWFjaGluZXJ5IjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmxhbmQiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjM6aW50YW5naWJsZUFzc2V0cyI6NywiYmFsYW5jZS1zaGVldDoyMDIzOnNvZnR3YXJlIjo1LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGlhYmlsaXRpZXMiOjc1LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudExpYWJpbGl0aWVzIjozOSwiYmFsYW5jZS1zaGVldDoyMDIzOnNob3J0VGVybURlYnQiOjEyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRMaWFiaWxpdGllcyI6MzYsImJhbGFuY2Utc2hlZXQ6MjAyMzpsb25nVGVybURlYnQiOjI5LCJiYWxhbmNlLXNoZWV0OjIwMjM6bmV0QXNzZXRzIjo1NywiYmFsYW5jZS1zaGVldDoyMDIzOnNoYXJlaG9sZGVyRXF1aXR5Ijo1NCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGl0YWwiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwZXgiOjUsImJhbGFuY2Utc2hlZXQ6MjAyNDphc3NldHMiOjE0MywiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRBc3NldHMiOjcyLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FzaCI6MjUsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZEFzc2V0cyI6NzEsImJhbGFuY2Utc2hlZXQ6MjAyNDp0YW5naWJsZUFzc2V0cyI6NTgsImJhbGFuY2Utc2hlZXQ6MjAyNDpidWlsZGluZ3MiOjIwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bWFjaGluZXJ5IjoyOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxhbmQiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6aW50YW5naWJsZUFzc2V0cyI6OCwiYmFsYW5jZS1zaGVldDoyMDI0OnNvZnR3YXJlIjo2LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGlhYmlsaXRpZXMiOjc5LCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudExpYWJpbGl0aWVzIjo0MSwiYmFsYW5jZS1zaGVldDoyMDI0OnNob3J0VGVybURlYnQiOjEyLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRMaWFiaWxpdGllcyI6MzgsImJhbGFuY2Utc2hlZXQ6MjAyNDpsb25nVGVybURlYnQiOjMxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bmV0QXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI0OnNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGl0YWwiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwZXgiOjgsImJhbGFuY2Utc2hlZXQ6MjAyNTphc3NldHMiOjE1NiwiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRBc3NldHMiOjc4LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FzaCI6MjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTp0YW5naWJsZUFzc2V0cyI6NjQsImJhbGFuY2Utc2hlZXQ6MjAyNTpidWlsZGluZ3MiOjIyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bWFjaGluZXJ5IjozMiwiYmFsYW5jZS1zaGVldDoyMDI1OmxhbmQiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjU6aW50YW5naWJsZUFzc2V0cyI6OSwiYmFsYW5jZS1zaGVldDoyMDI1OnNvZnR3YXJlIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjU6bGlhYmlsaXRpZXMiOjgzLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudExpYWJpbGl0aWVzIjo0MywiYmFsYW5jZS1zaGVldDoyMDI1OnNob3J0VGVybURlYnQiOjExLCJiYWxhbmNlLXNoZWV0OjIwMjU6Zml4ZWRMaWFiaWxpdGllcyI6NDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpsb25nVGVybURlYnQiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bmV0QXNzZXRzIjo3MywiYmFsYW5jZS1zaGVldDoyMDI1OnNoYXJlaG9sZGVyRXF1aXR5Ijo3MCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGl0YWwiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwZXgiOjEwLCJmdXR1cmUtY2FwZXg6MjAyNiI6MTUsImZ1dHVyZS1jYXBleDoyMDI3IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjgiOjE1LCJmdXR1cmUtY2FwZXg6MjAyOSI6MCwiZnV0dXJlLWNhcGV4OjIwMzAiOjAsImZ1dHVyZS1jYXBleDoyMDMxIjowLCJkcml2ZXI6cHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MCI6LTAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjEiOjAuMywiZHJpdmVyOnByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aFRvQmFzZToxIjowLjA1NzAxNzU0Mzg1OTY0OTE5LCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6NS41NTExMTUxMjMxMjU3ODNlLTE3LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjoxLjY2NTMzNDUzNjkzNzczNDhlLTE2LCJkcml2ZXI6cHJvamVjdFBheUdyb3d0aFRvQmFzZSI6MC4wMjAwMzA2NjIzNDI1MTgwNDYsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDE5MzI1MzMwNTAxODQ2OTI3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZToxIjowLjAyMDczNTk5NDE4MzE4OTE2NiwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZToxIjowLjA1NzAxNzU0Mzg1OTY0OTE5LCJkcml2ZXI6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MCwiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZToxIjowLjA1NzAxNzU0Mzg1OTY0OTE5LCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI1NzI0NjM3NjgxMTU4NTQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjAiOjAuMDQwNzYwODY5NTY1MjE3MTg0LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZToxIjowLjA0NDM4NDA1Nzk3MTAxNDUyLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMDAxMzQ1NzU1NjkzNTgxOTczNywiZHJpdmVyOm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkxMzk0NTcwMjM3MTc0NDMsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZToxIjowLjAyMDU1MzQ1OTkxNDc2MzA5NSwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wMzkxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDQyNTAwMDAwMDAwMDAwMDksImRyaXZlcjpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjAiOjAuMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MSI6MC4zLCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NzI0NjM3NjgxMTU4NiwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MCI6MC4wNjA3NjA4Njk1NjUyMTcxOSwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MSI6MC4wNjQzODQwNTc5NzEwMTQ1MywiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZToxIjowLjAzLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDoxIjowLjAwNTEzNDU3NTU2OTM1ODE5NzUsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDowIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDoxIjowLjEsImRyaXZlcjpvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjAiOjAuMDI0MTM5NDU3MDIzNzE3NDQ0LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wMjU1NTM0NTk5MTQ3NjMwOTYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjA0LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aDowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aDoxIjowLjA4LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MCI6MC4wNDQxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjEiOjAuMDQ3NTAwMDAwMDAwMDAwMDksImRyaXZlcjpwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjAiOjAuMDg0OTk5OTk5OTk5OTk5OTksImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDoxIjowLjEzNSwiZHJpdmVyOm90aGVyU2dhUmF0ZUVuZCI6MC4xMDkyODU3MTQyODU3MTQyOCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLjA4OTI4NTcxNDI4NTcxNDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMTE5Mjg1NzE0Mjg1NzE0MjcsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAuMDQyNjMxNTc4OTQ3MzY4MzYsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjA2NTU1NTU1NTU1NTU1NTU4LCJkcml2ZXI6dXNlZnVsTGlmZSI6MTAsImRyaXZlci1yYW5nZTp1c2VmdWxMaWZlOjAiOjUsImRyaXZlci1yYW5nZTp1c2VmdWxMaWZlOjEiOjIwLCJkcml2ZXI6aW52ZXN0bWVudCI6MjMsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjAiOjE1LCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDoxIjoyMDAsImRyaXZlcjpzdWJzaWR5Ijo3LjY2LCJkcml2ZXItcmFuZ2U6c3Vic2lkeTowIjoxLCJkcml2ZXItcmFuZ2U6c3Vic2lkeToxIjo1MCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoxNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjo4Mi40LCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjoyLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOm1heCI6NywidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOnZhbHVlIjo2MCwidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOm1heCI6OTUsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOnZhbHVlIjoyMiwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOnZhbHVlIjo3NC44LCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOnZhbHVlIjoyMSwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2FncjptYXgiOjM1LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOnZhbHVlIjoxOC43OCwidGFyZ2V0OmVtcGxveWVlUGF5Q2Fncjp2YWx1ZSI6NywidGFyZ2V0OmVtcGxveWVlUGF5Q2FncjptYXgiOjEwLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlJbmNyZWFzZTp2YWx1ZSI6Mi44NSwidGFyZ2V0OmludmVzdG1lbnRTYWxlc1JhdGlvOnZhbHVlIjoxNSwidGFyZ2V0OmludmVzdG1lbnRTYWxlc1JhdGlvOm1heCI6NzAsInRhcmdldDp2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvOnZhbHVlIjoyMTMsInRhcmdldDp2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvOm1heCI6MzUwLCJ0YXJnZXQ6bG9jYWxCZW5jaG1hcms6dmFsdWUiOjIzLCJ0YXJnZXQ6bG9jYWxCZW5jaG1hcms6bWF4Ijo0MCwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOnZhbHVlIjo2LCJ0YXJnZXQ6b2ZmaWNlclBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0Om9mZmljZXJQYXlJbmNyZWFzZTp2YWx1ZSI6MCwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOm1heCI6MjUyLjY5LCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6bWF4IjoxMzYuODQsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6bWF4IjozMy40MywidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6bWF4IjozLjc0fSwibWV0cmljR3JvdXBCYXNlcyI6eyJjb21wYW55U2FsZXMiOiJyYXRlIiwicHJvamVjdFNhbGVzIjoicmF0ZSIsImxhYm9yUHJvZHVjdGl2aXR5IjoicmF0ZSIsImVtcGxveWVlUGF5IjoicmF0ZSJ9LCJhcHBsaWNhdGlvbkNhdGVnb3J5IjoiZ2VuZXJhbCIsImFkanVzdGVkRHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MTA1OTU3NjAyMzM5MTYsInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjEuMTc0MTg2NDkxMDY0NDY2ZS0xNiwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6MC4wMTk5ODIxMzU1MTE4Nzk4NzMsInByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDU0MDYzOTAxMjQ5NzIyOTM0LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDEyMDQ1MTMzMzE1NzYzLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjYwNTUxNjI3MzAwNTI3LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODgxMzY3NTAwOTE3MTE3LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA2MDkzNTM5NDM3MTc4NTUsIm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMjAyMjQ4NzIxNjk0NjY3Mywib3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NjUxNzg1OTQ1MjE3OSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTQ5OTA0ODEzNDEyNjU1NSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA4OTAwNjIyOTk3NTA4MDEsIm90aGVyUGF5R3Jvd3RoIjowLjAyNDg4Nzc2MTcxMDMzMzAzLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjAyOTA0NTQ4MjM5NzIwNTA1NSwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1Nzg0ODE0NzMyMzA4NjY1LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMDk5MzE4MDkxNjQ4NDgyNCwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI3MjU4OTg3MjEyODIzLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM3NzgwNTc2Mjg3MTYzMiwidXNlZnVsTGlmZSI6MTAsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9fQ==</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename other business to base business
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -3560,47 +3560,47 @@
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 — / 補助 — / 他 —</t>
+          <t xml:space="preserve">全社 — / 補助 — / ベース —</t>
         </is>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.99 % / 補助 5.56 % / 他 4.35 %</t>
+          <t xml:space="preserve">全社 4.99 % / 補助 5.56 % / ベース 4.35 %</t>
         </is>
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.75 % / 補助 5.26 % / 他 4.17 %</t>
+          <t xml:space="preserve">全社 4.75 % / 補助 5.26 % / ベース 4.17 %</t>
         </is>
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.87 % / 補助 5.41 % / 他 4.26 %</t>
+          <t xml:space="preserve">全社 4.87 % / 補助 5.41 % / ベース 4.26 %</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.88 % / 補助 5.41 % / 他 4.26 %</t>
+          <t xml:space="preserve">全社 4.88 % / 補助 5.41 % / ベース 4.26 %</t>
         </is>
       </c>
       <c r="I4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.88 % / 補助 5.41 % / 他 4.26 %</t>
+          <t xml:space="preserve">全社 4.88 % / 補助 5.41 % / ベース 4.26 %</t>
         </is>
       </c>
       <c r="J4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.28 % / 補助 22.03 % / 他 7.31 %</t>
+          <t xml:space="preserve">全社 15.28 % / 補助 22.03 % / ベース 7.31 %</t>
         </is>
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.29 % / 補助 22.01 % / 他 6.25 %</t>
+          <t xml:space="preserve">全社 15.29 % / 補助 22.01 % / ベース 6.25 %</t>
         </is>
       </c>
       <c r="L4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.83 % / 補助 22.03 % / 他 6.27 %</t>
+          <t xml:space="preserve">全社 15.83 % / 補助 22.03 % / ベース 6.27 %</t>
         </is>
       </c>
     </row>
@@ -3622,47 +3622,47 @@
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 68 % / 補助 68 % / 他 68 %</t>
+          <t xml:space="preserve">全社 68 % / 補助 68 % / ベース 68 %</t>
         </is>
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 68 % / 補助 68 % / 他 68.01 %</t>
+          <t xml:space="preserve">全社 68 % / 補助 68 % / ベース 68.01 %</t>
         </is>
       </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 68 % / 補助 68 % / 他 68 %</t>
+          <t xml:space="preserve">全社 68 % / 補助 68 % / ベース 68 %</t>
         </is>
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 68 % / 補助 67.99 % / 他 68 %</t>
+          <t xml:space="preserve">全社 68 % / 補助 67.99 % / ベース 68 %</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 68 % / 補助 68.01 % / 他 68 %</t>
+          <t xml:space="preserve">全社 68 % / 補助 68.01 % / ベース 68 %</t>
         </is>
       </c>
       <c r="I5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 68.01 % / 補助 68 % / 他 68.01 %</t>
+          <t xml:space="preserve">全社 68.01 % / 補助 68 % / ベース 68.01 %</t>
         </is>
       </c>
       <c r="J5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 67.36 % / 補助 67.5 % / 他 67.17 %</t>
+          <t xml:space="preserve">全社 67.36 % / 補助 67.5 % / ベース 67.17 %</t>
         </is>
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 67.01 % / 補助 67.01 % / 他 67.01 %</t>
+          <t xml:space="preserve">全社 67.01 % / 補助 67.01 % / ベース 67.01 %</t>
         </is>
       </c>
       <c r="L5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 66.62 % / 補助 66.51 % / 他 66.83 %</t>
+          <t xml:space="preserve">全社 66.62 % / 補助 66.51 % / ベース 66.83 %</t>
         </is>
       </c>
     </row>
@@ -3684,47 +3684,47 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32 % / 補助 32 % / 他 32 %</t>
+          <t xml:space="preserve">全社 32 % / 補助 32 % / ベース 32 %</t>
         </is>
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32 % / 補助 32 % / 他 31.99 %</t>
+          <t xml:space="preserve">全社 32 % / 補助 32 % / ベース 31.99 %</t>
         </is>
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32 % / 補助 32 % / 他 32 %</t>
+          <t xml:space="preserve">全社 32 % / 補助 32 % / ベース 32 %</t>
         </is>
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32 % / 補助 32.01 % / 他 32 %</t>
+          <t xml:space="preserve">全社 32 % / 補助 32.01 % / ベース 32 %</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32 % / 補助 31.99 % / 他 32 %</t>
+          <t xml:space="preserve">全社 32 % / 補助 31.99 % / ベース 32 %</t>
         </is>
       </c>
       <c r="I6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 31.99 % / 補助 32 % / 他 31.99 %</t>
+          <t xml:space="preserve">全社 31.99 % / 補助 32 % / ベース 31.99 %</t>
         </is>
       </c>
       <c r="J6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32.64 % / 補助 32.5 % / 他 32.83 %</t>
+          <t xml:space="preserve">全社 32.64 % / 補助 32.5 % / ベース 32.83 %</t>
         </is>
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32.99 % / 補助 32.99 % / 他 32.99 %</t>
+          <t xml:space="preserve">全社 32.99 % / 補助 32.99 % / ベース 32.99 %</t>
         </is>
       </c>
       <c r="L6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 33.38 % / 補助 33.49 % / 他 33.17 %</t>
+          <t xml:space="preserve">全社 33.38 % / 補助 33.49 % / ベース 33.17 %</t>
         </is>
       </c>
     </row>
@@ -3746,47 +3746,47 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 23.94 % / 補助 22.58 % / 他 25.45 %</t>
+          <t xml:space="preserve">全社 23.94 % / 補助 22.58 % / ベース 25.45 %</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.11 % / 補助 22.74 % / 他 25.65 %</t>
+          <t xml:space="preserve">全社 24.11 % / 補助 22.74 % / ベース 25.65 %</t>
         </is>
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.27 % / 補助 22.88 % / 他 25.86 %</t>
+          <t xml:space="preserve">全社 24.27 % / 補助 22.88 % / ベース 25.86 %</t>
         </is>
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.7 % / 補助 23.61 % / 他 25.97 %</t>
+          <t xml:space="preserve">全社 24.7 % / 補助 23.61 % / ベース 25.97 %</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 25.12 % / 補助 24.28 % / 他 26.1 %</t>
+          <t xml:space="preserve">全社 25.12 % / 補助 24.28 % / ベース 26.1 %</t>
         </is>
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 25.52 % / 補助 24.91 % / 他 26.23 %</t>
+          <t xml:space="preserve">全社 25.52 % / 補助 24.91 % / ベース 26.23 %</t>
         </is>
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24 % / 補助 22.67 % / 他 25.78 %</t>
+          <t xml:space="preserve">全社 24 % / 補助 22.67 % / ベース 25.78 %</t>
         </is>
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 22.84 % / 補助 21.03 % / 他 25.63 %</t>
+          <t xml:space="preserve">全社 22.84 % / 補助 21.03 % / ベース 25.63 %</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 21.67 % / 補助 19.54 % / 他 25.46 %</t>
+          <t xml:space="preserve">全社 21.67 % / 補助 19.54 % / ベース 25.46 %</t>
         </is>
       </c>
     </row>
@@ -3808,47 +3808,47 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.06 % / 補助 9.42 % / 他 6.55 %</t>
+          <t xml:space="preserve">全社 8.06 % / 補助 9.42 % / ベース 6.55 %</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.89 % / 補助 9.26 % / 他 6.34 %</t>
+          <t xml:space="preserve">全社 7.89 % / 補助 9.26 % / ベース 6.34 %</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.73 % / 補助 9.13 % / 他 6.14 %</t>
+          <t xml:space="preserve">全社 7.73 % / 補助 9.13 % / ベース 6.14 %</t>
         </is>
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.3 % / 補助 8.4 % / 他 6.03 %</t>
+          <t xml:space="preserve">全社 7.3 % / 補助 8.4 % / ベース 6.03 %</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.88 % / 補助 7.72 % / 他 5.9 %</t>
+          <t xml:space="preserve">全社 6.88 % / 補助 7.72 % / ベース 5.9 %</t>
         </is>
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.48 % / 補助 7.09 % / 他 5.76 %</t>
+          <t xml:space="preserve">全社 6.48 % / 補助 7.09 % / ベース 5.76 %</t>
         </is>
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.64 % / 補助 9.83 % / 他 7.05 %</t>
+          <t xml:space="preserve">全社 8.64 % / 補助 9.83 % / ベース 7.05 %</t>
         </is>
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.15 % / 補助 11.96 % / 他 7.36 %</t>
+          <t xml:space="preserve">全社 10.15 % / 補助 11.96 % / ベース 7.36 %</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.7 % / 補助 13.96 % / 他 7.71 %</t>
+          <t xml:space="preserve">全社 11.7 % / 補助 13.96 % / ベース 7.71 %</t>
         </is>
       </c>
     </row>
@@ -3870,47 +3870,47 @@
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.4 % / 補助 11.92 % / 他 8.7 %</t>
+          <t xml:space="preserve">全社 10.4 % / 補助 11.92 % / ベース 8.7 %</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.22 % / 補助 11.76 % / 他 8.48 %</t>
+          <t xml:space="preserve">全社 10.22 % / 補助 11.76 % / ベース 8.48 %</t>
         </is>
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.07 % / 補助 11.63 % / 他 8.29 %</t>
+          <t xml:space="preserve">全社 10.07 % / 補助 11.63 % / ベース 8.29 %</t>
         </is>
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.01 % / 補助 11.68 % / 他 8.08 %</t>
+          <t xml:space="preserve">全社 10.01 % / 補助 11.68 % / ベース 8.08 %</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.93 % / 補助 11.69 % / 他 7.87 %</t>
+          <t xml:space="preserve">全社 9.93 % / 補助 11.69 % / ベース 7.87 %</t>
         </is>
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.83 % / 補助 11.68 % / 他 7.65 %</t>
+          <t xml:space="preserve">全社 9.83 % / 補助 11.68 % / ベース 7.65 %</t>
         </is>
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.55 % / 補助 13.59 % / 他 8.81 %</t>
+          <t xml:space="preserve">全社 11.55 % / 補助 13.59 % / ベース 8.81 %</t>
         </is>
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.68 % / 補助 15.05 % / 他 9.02 %</t>
+          <t xml:space="preserve">全社 12.68 % / 補助 15.05 % / ベース 9.02 %</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.88 % / 補助 16.48 % / 他 9.27 %</t>
+          <t xml:space="preserve">全社 13.88 % / 補助 16.48 % / ベース 9.27 %</t>
         </is>
       </c>
     </row>
@@ -3932,47 +3932,47 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.99 % / 補助 12.5 % / 他 11.43 %</t>
+          <t xml:space="preserve">全社 11.99 % / 補助 12.5 % / ベース 11.43 %</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12 % / 補助 12.5 % / 他 11.43 %</t>
+          <t xml:space="preserve">全社 12 % / 補助 12.5 % / ベース 11.43 %</t>
         </is>
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12 % / 補助 12.5 % / 他 11.43 %</t>
+          <t xml:space="preserve">全社 12 % / 補助 12.5 % / ベース 11.43 %</t>
         </is>
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12 % / 補助 12.5 % / 他 11.43 %</t>
+          <t xml:space="preserve">全社 12 % / 補助 12.5 % / ベース 11.43 %</t>
         </is>
       </c>
       <c r="H10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.01 % / 補助 12.5 % / 他 11.43 %</t>
+          <t xml:space="preserve">全社 12.01 % / 補助 12.5 % / ベース 11.43 %</t>
         </is>
       </c>
       <c r="I10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.01 % / 補助 12.5 % / 他 11.43 %</t>
+          <t xml:space="preserve">全社 12.01 % / 補助 12.5 % / ベース 11.43 %</t>
         </is>
       </c>
       <c r="J10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.64 % / 補助 12 % / 他 11.15 %</t>
+          <t xml:space="preserve">全社 11.64 % / 補助 12 % / ベース 11.15 %</t>
         </is>
       </c>
       <c r="K10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.3 % / 補助 11.5 % / 他 10.99 %</t>
+          <t xml:space="preserve">全社 11.3 % / 補助 11.5 % / ベース 10.99 %</t>
         </is>
       </c>
       <c r="L10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.93 % / 補助 10.99 % / 他 10.82 %</t>
+          <t xml:space="preserve">全社 10.93 % / 補助 10.99 % / ベース 10.82 %</t>
         </is>
       </c>
     </row>
@@ -4056,47 +4056,47 @@
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.01 % / 補助 7.21 % / 他 11.02 %</t>
+          <t xml:space="preserve">全社 9.01 % / 補助 7.21 % / ベース 11.02 %</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.17 % / 補助 7.36 % / 他 11.22 %</t>
+          <t xml:space="preserve">全社 9.17 % / 補助 7.36 % / ベース 11.22 %</t>
         </is>
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.33 % / 補助 7.5 % / 他 11.43 %</t>
+          <t xml:space="preserve">全社 9.33 % / 補助 7.5 % / ベース 11.43 %</t>
         </is>
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.5 % / 補助 7.65 % / 他 11.63 %</t>
+          <t xml:space="preserve">全社 9.5 % / 補助 7.65 % / ベース 11.63 %</t>
         </is>
       </c>
       <c r="H12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.67 % / 補助 7.81 % / 他 11.84 %</t>
+          <t xml:space="preserve">全社 9.67 % / 補助 7.81 % / ベース 11.84 %</t>
         </is>
       </c>
       <c r="I12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.84 % / 補助 7.96 % / 他 12.05 %</t>
+          <t xml:space="preserve">全社 9.84 % / 補助 7.96 % / ベース 12.05 %</t>
         </is>
       </c>
       <c r="J12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.1 % / 補助 6.91 % / 他 12.04 %</t>
+          <t xml:space="preserve">全社 9.1 % / 補助 6.91 % / ベース 12.04 %</t>
         </is>
       </c>
       <c r="K12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.63 % / 補助 6.34 % / 他 12.15 %</t>
+          <t xml:space="preserve">全社 8.63 % / 補助 6.34 % / ベース 12.15 %</t>
         </is>
       </c>
       <c r="L12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.14 % / 補助 5.83 % / 他 12.25 %</t>
+          <t xml:space="preserve">全社 8.14 % / 補助 5.83 % / ベース 12.25 %</t>
         </is>
       </c>
     </row>
@@ -4118,47 +4118,47 @@
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.67 % / 補助 0.5 % / 他 0.85 %</t>
+          <t xml:space="preserve">全社 0.67 % / 補助 0.5 % / ベース 0.85 %</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.67 % / 補助 0.5 % / 他 0.86 %</t>
+          <t xml:space="preserve">全社 0.67 % / 補助 0.5 % / ベース 0.86 %</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.67 % / 補助 0.5 % / 他 0.86 %</t>
+          <t xml:space="preserve">全社 0.67 % / 補助 0.5 % / ベース 0.86 %</t>
         </is>
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.65 % / 補助 0.5 % / 他 0.84 %</t>
+          <t xml:space="preserve">全社 0.65 % / 補助 0.5 % / ベース 0.84 %</t>
         </is>
       </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.64 % / 補助 0.49 % / 他 0.81 %</t>
+          <t xml:space="preserve">全社 0.64 % / 補助 0.49 % / ベース 0.81 %</t>
         </is>
       </c>
       <c r="I13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.64 % / 補助 0.5 % / 他 0.81 %</t>
+          <t xml:space="preserve">全社 0.64 % / 補助 0.5 % / ベース 0.81 %</t>
         </is>
       </c>
       <c r="J13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.58 % / 補助 0.44 % / 他 0.76 %</t>
+          <t xml:space="preserve">全社 0.58 % / 補助 0.44 % / ベース 0.76 %</t>
         </is>
       </c>
       <c r="K13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.52 % / 補助 0.37 % / 他 0.74 %</t>
+          <t xml:space="preserve">全社 0.52 % / 補助 0.37 % / ベース 0.74 %</t>
         </is>
       </c>
       <c r="L13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.47 % / 補助 0.32 % / 他 0.72 %</t>
+          <t xml:space="preserve">全社 0.47 % / 補助 0.32 % / ベース 0.72 %</t>
         </is>
       </c>
     </row>
@@ -4180,47 +4180,47 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.68 % / 補助 7.71 % / 他 11.88 %</t>
+          <t xml:space="preserve">全社 9.68 % / 補助 7.71 % / ベース 11.88 %</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.84 % / 補助 7.86 % / 他 12.08 %</t>
+          <t xml:space="preserve">全社 9.84 % / 補助 7.86 % / ベース 12.08 %</t>
         </is>
       </c>
       <c r="F14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10 % / 補助 8 % / 他 12.29 %</t>
+          <t xml:space="preserve">全社 10 % / 補助 8 % / ベース 12.29 %</t>
         </is>
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.15 % / 補助 8.15 % / 他 12.47 %</t>
+          <t xml:space="preserve">全社 10.15 % / 補助 8.15 % / ベース 12.47 %</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.31 % / 補助 8.3 % / 他 12.66 %</t>
+          <t xml:space="preserve">全社 10.31 % / 補助 8.3 % / ベース 12.66 %</t>
         </is>
       </c>
       <c r="I14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.48 % / 補助 8.46 % / 他 12.86 %</t>
+          <t xml:space="preserve">全社 10.48 % / 補助 8.46 % / ベース 12.86 %</t>
         </is>
       </c>
       <c r="J14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.68 % / 補助 7.35 % / 他 12.8 %</t>
+          <t xml:space="preserve">全社 9.68 % / 補助 7.35 % / ベース 12.8 %</t>
         </is>
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.15 % / 補助 6.72 % / 他 12.89 %</t>
+          <t xml:space="preserve">全社 9.15 % / 補助 6.72 % / ベース 12.89 %</t>
         </is>
       </c>
       <c r="L14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.61 % / 補助 6.15 % / 他 12.96 %</t>
+          <t xml:space="preserve">全社 8.61 % / 補助 6.15 % / ベース 12.96 %</t>
         </is>
       </c>
     </row>
@@ -4242,47 +4242,47 @@
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.059 億円/人 / 補助 0.058 億円/人 / 他 0.059 億円/人</t>
+          <t xml:space="preserve">全社 0.059 億円/人 / 補助 0.058 億円/人 / ベース 0.059 億円/人</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.06 億円/人 / 補助 0.059 億円/人 / 他 0.06 億円/人</t>
+          <t xml:space="preserve">全社 0.06 億円/人 / 補助 0.059 億円/人 / ベース 0.06 億円/人</t>
         </is>
       </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.061 億円/人 / 補助 0.06 億円/人 / 他 0.062 億円/人</t>
+          <t xml:space="preserve">全社 0.061 億円/人 / 補助 0.06 億円/人 / ベース 0.062 億円/人</t>
         </is>
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.062 億円/人 / 補助 0.061 億円/人 / 他 0.063 億円/人</t>
+          <t xml:space="preserve">全社 0.062 億円/人 / 補助 0.061 億円/人 / ベース 0.063 億円/人</t>
         </is>
       </c>
       <c r="H15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.063 億円/人 / 補助 0.063 億円/人 / 他 0.064 億円/人</t>
+          <t xml:space="preserve">全社 0.063 億円/人 / 補助 0.063 億円/人 / ベース 0.064 億円/人</t>
         </is>
       </c>
       <c r="I15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.065 億円/人 / 補助 0.064 億円/人 / 他 0.065 億円/人</t>
+          <t xml:space="preserve">全社 0.065 億円/人 / 補助 0.064 億円/人 / ベース 0.065 億円/人</t>
         </is>
       </c>
       <c r="J15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.066 億円/人 / 補助 0.066 億円/人 / 他 0.067 億円/人</t>
+          <t xml:space="preserve">全社 0.066 億円/人 / 補助 0.066 億円/人 / ベース 0.067 億円/人</t>
         </is>
       </c>
       <c r="K15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.07 億円/人 / 補助 0.071 億円/人 / 他 0.069 億円/人</t>
+          <t xml:space="preserve">全社 0.07 億円/人 / 補助 0.071 億円/人 / ベース 0.069 億円/人</t>
         </is>
       </c>
       <c r="L15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.074 億円/人 / 補助 0.078 億円/人 / 他 0.07 億円/人</t>
+          <t xml:space="preserve">全社 0.074 億円/人 / 補助 0.078 億円/人 / ベース 0.07 億円/人</t>
         </is>
       </c>
     </row>
@@ -4304,47 +4304,47 @@
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.182 億円/人 / 補助 0.18 億円/人 / 他 0.183 億円/人</t>
+          <t xml:space="preserve">全社 0.182 億円/人 / 補助 0.18 億円/人 / ベース 0.183 億円/人</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.192 億円/人 / 補助 0.19 億円/人 / 他 0.193 億円/人</t>
+          <t xml:space="preserve">全社 0.192 億円/人 / 補助 0.19 億円/人 / ベース 0.193 億円/人</t>
         </is>
       </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.2 億円/人 / 補助 0.2 億円/人 / 他 0.2 億円/人</t>
+          <t xml:space="preserve">全社 0.2 億円/人 / 補助 0.2 億円/人 / ベース 0.2 億円/人</t>
         </is>
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.206 億円/人 / 補助 0.21 億円/人 / 他 0.203 億円/人</t>
+          <t xml:space="preserve">全社 0.206 億円/人 / 補助 0.21 億円/人 / ベース 0.203 億円/人</t>
         </is>
       </c>
       <c r="H16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.212 億円/人 / 補助 0.22 億円/人 / 他 0.207 億円/人</t>
+          <t xml:space="preserve">全社 0.212 億円/人 / 補助 0.22 億円/人 / ベース 0.207 億円/人</t>
         </is>
       </c>
       <c r="I16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.222 億円/人 / 補助 0.235 億円/人 / 他 0.213 億円/人</t>
+          <t xml:space="preserve">全社 0.222 億円/人 / 補助 0.235 億円/人 / ベース 0.213 億円/人</t>
         </is>
       </c>
       <c r="J16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.23 億円/人 / 補助 0.25 億円/人 / 他 0.217 億円/人</t>
+          <t xml:space="preserve">全社 0.23 億円/人 / 補助 0.25 億円/人 / ベース 0.217 億円/人</t>
         </is>
       </c>
       <c r="K16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.238 億円/人 / 補助 0.26 億円/人 / 他 0.223 億円/人</t>
+          <t xml:space="preserve">全社 0.238 億円/人 / 補助 0.26 億円/人 / ベース 0.223 億円/人</t>
         </is>
       </c>
       <c r="L16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.248 億円/人 / 補助 0.275 億円/人 / 他 0.23 億円/人</t>
+          <t xml:space="preserve">全社 0.248 億円/人 / 補助 0.275 億円/人 / ベース 0.23 億円/人</t>
         </is>
       </c>
     </row>
@@ -4366,47 +4366,47 @@
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 — / 補助 — / 他 —</t>
+          <t xml:space="preserve">全社 — / 補助 — / ベース —</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.98 % / 補助 2.04 % / 他 1.95 %</t>
+          <t xml:space="preserve">全社 1.98 % / 補助 2.04 % / ベース 1.95 %</t>
         </is>
       </c>
       <c r="F17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.99 % / 補助 1.97 % / 他 2.02 %</t>
+          <t xml:space="preserve">全社 1.99 % / 補助 1.97 % / ベース 2.02 %</t>
         </is>
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.27 % / 補助 2.38 % / 他 2.19 %</t>
+          <t xml:space="preserve">全社 2.27 % / 補助 2.38 % / ベース 2.19 %</t>
         </is>
       </c>
       <c r="H17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.68 % / 補助 1.78 % / 他 1.61 %</t>
+          <t xml:space="preserve">全社 1.68 % / 補助 1.78 % / ベース 1.61 %</t>
         </is>
       </c>
       <c r="I17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.25 % / 補助 1.98 % / 他 2.47 %</t>
+          <t xml:space="preserve">全社 2.25 % / 補助 1.98 % / ベース 2.47 %</t>
         </is>
       </c>
       <c r="J17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.73 % / 補助 3.25 % / 他 2.31 %</t>
+          <t xml:space="preserve">全社 2.73 % / 補助 3.25 % / ベース 2.31 %</t>
         </is>
       </c>
       <c r="K17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5.08 % / 補助 8.41 % / 他 2.53 %</t>
+          <t xml:space="preserve">全社 5.08 % / 補助 8.41 % / ベース 2.53 %</t>
         </is>
       </c>
       <c r="L17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5.25 % / 補助 9.44 % / 他 2 %</t>
+          <t xml:space="preserve">全社 5.25 % / 補助 9.44 % / ベース 2 %</t>
         </is>
       </c>
     </row>
@@ -4428,47 +4428,47 @@
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 48.21 % / 補助 39.28 % / 他 57.74 %</t>
+          <t xml:space="preserve">全社 48.21 % / 補助 39.28 % / ベース 57.74 %</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 49.04 % / 補助 40.04 % / 他 58.76 %</t>
+          <t xml:space="preserve">全社 49.04 % / 補助 40.04 % / ベース 58.76 %</t>
         </is>
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 49.83 % / 補助 40.76 % / 他 59.72 %</t>
+          <t xml:space="preserve">全社 49.83 % / 補助 40.76 % / ベース 59.72 %</t>
         </is>
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 50.35 % / 補助 41.09 % / 他 60.67 %</t>
+          <t xml:space="preserve">全社 50.35 % / 補助 41.09 % / ベース 60.67 %</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 50.94 % / 補助 41.53 % / 他 61.65 %</t>
+          <t xml:space="preserve">全社 50.94 % / 補助 41.53 % / ベース 61.65 %</t>
         </is>
       </c>
       <c r="I18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 51.59 % / 補助 42.02 % / 他 62.69 %</t>
+          <t xml:space="preserve">全社 51.59 % / 補助 42.02 % / ベース 62.69 %</t>
         </is>
       </c>
       <c r="J18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 45.58 % / 補助 35.09 % / 他 59.24 %</t>
+          <t xml:space="preserve">全社 45.58 % / 補助 35.09 % / ベース 59.24 %</t>
         </is>
       </c>
       <c r="K18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 41.91 % / 補助 30.86 % / 他 58.83 %</t>
+          <t xml:space="preserve">全社 41.91 % / 補助 30.86 % / ベース 58.83 %</t>
         </is>
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 38.28 % / 補助 27.17 % / 他 58.31 %</t>
+          <t xml:space="preserve">全社 38.28 % / 補助 27.17 % / ベース 58.31 %</t>
         </is>
       </c>
     </row>
@@ -4552,47 +4552,47 @@
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.65 億円/人 / 補助 0.8 億円/人 / 他 0.537 億円/人</t>
+          <t xml:space="preserve">全社 0.65 億円/人 / 補助 0.8 億円/人 / ベース 0.537 億円/人</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.651 億円/人 / 補助 0.8 億円/人 / 他 0.538 億円/人</t>
+          <t xml:space="preserve">全社 0.651 億円/人 / 補助 0.8 億円/人 / ベース 0.538 億円/人</t>
         </is>
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.652 億円/人 / 補助 0.8 億円/人 / 他 0.538 億円/人</t>
+          <t xml:space="preserve">全社 0.652 億円/人 / 補助 0.8 億円/人 / ベース 0.538 億円/人</t>
         </is>
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.655 億円/人 / 補助 0.803 億円/人 / 他 0.541 億円/人</t>
+          <t xml:space="preserve">全社 0.655 億円/人 / 補助 0.803 億円/人 / ベース 0.541 億円/人</t>
         </is>
       </c>
       <c r="H20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.655 億円/人 / 補助 0.801 億円/人 / 他 0.54 億円/人</t>
+          <t xml:space="preserve">全社 0.655 億円/人 / 補助 0.801 億円/人 / ベース 0.54 億円/人</t>
         </is>
       </c>
       <c r="I20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.658 億円/人 / 補助 0.801 億円/人 / 他 0.543 億円/人</t>
+          <t xml:space="preserve">全社 0.658 億円/人 / 補助 0.801 億円/人 / ベース 0.543 億円/人</t>
         </is>
       </c>
       <c r="J20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.731 億円/人 / 補助 0.953 億円/人 / 他 0.556 億円/人</t>
+          <t xml:space="preserve">全社 0.731 億円/人 / 補助 0.953 億円/人 / ベース 0.556 億円/人</t>
         </is>
       </c>
       <c r="K20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.81 億円/人 / 補助 1.125 億円/人 / 他 0.565 億円/人</t>
+          <t xml:space="preserve">全社 0.81 億円/人 / 補助 1.125 億円/人 / ベース 0.565 億円/人</t>
         </is>
       </c>
       <c r="L20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.903 億円/人 / 補助 1.34 億円/人 / 他 0.572 億円/人</t>
+          <t xml:space="preserve">全社 0.903 億円/人 / 補助 1.34 億円/人 / ベース 0.572 億円/人</t>
         </is>
       </c>
     </row>
@@ -4614,47 +4614,47 @@
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.052 億円/人 / 補助 0.075 億円/人 / 他 0.035 億円/人</t>
+          <t xml:space="preserve">全社 0.052 億円/人 / 補助 0.075 億円/人 / ベース 0.035 億円/人</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.051 億円/人 / 補助 0.074 億円/人 / 他 0.034 億円/人</t>
+          <t xml:space="preserve">全社 0.051 億円/人 / 補助 0.074 億円/人 / ベース 0.034 億円/人</t>
         </is>
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.05 億円/人 / 補助 0.073 億円/人 / 他 0.033 億円/人</t>
+          <t xml:space="preserve">全社 0.05 億円/人 / 補助 0.073 億円/人 / ベース 0.033 億円/人</t>
         </is>
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.048 億円/人 / 補助 0.067 億円/人 / 他 0.033 億円/人</t>
+          <t xml:space="preserve">全社 0.048 億円/人 / 補助 0.067 億円/人 / ベース 0.033 億円/人</t>
         </is>
       </c>
       <c r="H21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.045 億円/人 / 補助 0.062 億円/人 / 他 0.032 億円/人</t>
+          <t xml:space="preserve">全社 0.045 億円/人 / 補助 0.062 億円/人 / ベース 0.032 億円/人</t>
         </is>
       </c>
       <c r="I21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.043 億円/人 / 補助 0.057 億円/人 / 他 0.031 億円/人</t>
+          <t xml:space="preserve">全社 0.043 億円/人 / 補助 0.057 億円/人 / ベース 0.031 億円/人</t>
         </is>
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.063 億円/人 / 補助 0.094 億円/人 / 他 0.039 億円/人</t>
+          <t xml:space="preserve">全社 0.063 億円/人 / 補助 0.094 億円/人 / ベース 0.039 億円/人</t>
         </is>
       </c>
       <c r="K21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.082 億円/人 / 補助 0.135 億円/人 / 他 0.042 億円/人</t>
+          <t xml:space="preserve">全社 0.082 億円/人 / 補助 0.135 億円/人 / ベース 0.042 億円/人</t>
         </is>
       </c>
       <c r="L21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.106 億円/人 / 補助 0.187 億円/人 / 他 0.044 億円/人</t>
+          <t xml:space="preserve">全社 0.106 億円/人 / 補助 0.187 億円/人 / ベース 0.044 億円/人</t>
         </is>
       </c>
     </row>
@@ -4676,47 +4676,47 @@
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.127 億円/人 / 補助 0.154 億円/人 / 他 0.108 億円/人</t>
+          <t xml:space="preserve">全社 0.127 億円/人 / 補助 0.154 億円/人 / ベース 0.108 億円/人</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.128 億円/人 / 補助 0.154 億円/人 / 他 0.108 億円/人</t>
+          <t xml:space="preserve">全社 0.128 億円/人 / 補助 0.154 億円/人 / ベース 0.108 億円/人</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.128 億円/人 / 補助 0.154 億円/人 / 他 0.108 億円/人</t>
+          <t xml:space="preserve">全社 0.128 億円/人 / 補助 0.154 億円/人 / ベース 0.108 億円/人</t>
         </is>
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.129 億円/人 / 補助 0.156 億円/人 / 他 0.109 億円/人</t>
+          <t xml:space="preserve">全社 0.129 億円/人 / 補助 0.156 億円/人 / ベース 0.109 億円/人</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.13 億円/人 / 補助 0.157 億円/人 / 他 0.108 億円/人</t>
+          <t xml:space="preserve">全社 0.13 億円/人 / 補助 0.157 億円/人 / ベース 0.108 億円/人</t>
         </is>
       </c>
       <c r="I22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.131 億円/人 / 補助 0.159 億円/人 / 他 0.109 億円/人</t>
+          <t xml:space="preserve">全社 0.131 億円/人 / 補助 0.159 億円/人 / ベース 0.109 億円/人</t>
         </is>
       </c>
       <c r="J22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.152 億円/人 / 補助 0.196 億円/人 / 他 0.118 億円/人</t>
+          <t xml:space="preserve">全社 0.152 億円/人 / 補助 0.196 億円/人 / ベース 0.118 億円/人</t>
         </is>
       </c>
       <c r="K22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.174 億円/人 / 補助 0.241 億円/人 / 他 0.122 億円/人</t>
+          <t xml:space="preserve">全社 0.174 億円/人 / 補助 0.241 億円/人 / ベース 0.122 億円/人</t>
         </is>
       </c>
       <c r="L22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.2 億円/人 / 補助 0.299 億円/人 / 他 0.125 億円/人</t>
+          <t xml:space="preserve">全社 0.2 億円/人 / 補助 0.299 億円/人 / ベース 0.125 億円/人</t>
         </is>
       </c>
     </row>
@@ -4738,47 +4738,47 @@
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 — / 補助 — / 他 —</t>
+          <t xml:space="preserve">全社 — / 補助 — / ベース —</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.76 % / 補助 5.56 % / 他 4.17 %</t>
+          <t xml:space="preserve">全社 4.76 % / 補助 5.56 % / ベース 4.17 %</t>
         </is>
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.55 % / 補助 5.26 % / 他 4 %</t>
+          <t xml:space="preserve">全社 4.55 % / 補助 5.26 % / ベース 4 %</t>
         </is>
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.35 % / 補助 5 % / 他 3.85 %</t>
+          <t xml:space="preserve">全社 4.35 % / 補助 5 % / ベース 3.85 %</t>
         </is>
       </c>
       <c r="H23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5 % / 補助 5.71 % / 他 4.44 %</t>
+          <t xml:space="preserve">全社 5 % / 補助 5.71 % / ベース 4.44 %</t>
         </is>
       </c>
       <c r="I23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.37 % / 補助 5.41 % / 他 3.55 %</t>
+          <t xml:space="preserve">全社 4.37 % / 補助 5.41 % / ベース 3.55 %</t>
         </is>
       </c>
       <c r="J23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.8 % / 補助 2.56 % / 他 4.79 %</t>
+          <t xml:space="preserve">全社 3.8 % / 補助 2.56 % / ベース 4.79 %</t>
         </is>
       </c>
       <c r="K23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.03 % / 補助 3.33 % / 他 4.58 %</t>
+          <t xml:space="preserve">全社 4.03 % / 補助 3.33 % / ベース 4.58 %</t>
         </is>
       </c>
       <c r="L23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.87 % / 補助 2.42 % / 他 5 %</t>
+          <t xml:space="preserve">全社 3.87 % / 補助 2.42 % / ベース 5 %</t>
         </is>
       </c>
     </row>
@@ -4800,47 +4800,47 @@
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 — / 補助 — / 他 —</t>
+          <t xml:space="preserve">全社 — / 補助 — / ベース —</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.22 pt / 補助 0 pt / 他 0.18 pt</t>
+          <t xml:space="preserve">全社 0.22 pt / 補助 0 pt / ベース 0.18 pt</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.2 pt / 補助 0 pt / 他 0.17 pt</t>
+          <t xml:space="preserve">全社 0.2 pt / 補助 0 pt / ベース 0.17 pt</t>
         </is>
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.53 pt / 補助 0.41 pt / 他 0.41 pt</t>
+          <t xml:space="preserve">全社 0.53 pt / 補助 0.41 pt / ベース 0.41 pt</t>
         </is>
       </c>
       <c r="H24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 -0.12 pt / 補助 -0.31 pt / 他 -0.18 pt</t>
+          <t xml:space="preserve">全社 -0.12 pt / 補助 -0.31 pt / ベース -0.18 pt</t>
         </is>
       </c>
       <c r="I24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.51 pt / 補助 0.01 pt / 他 0.71 pt</t>
+          <t xml:space="preserve">全社 0.51 pt / 補助 0.01 pt / ベース 0.71 pt</t>
         </is>
       </c>
       <c r="J24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.48 pt / 補助 19.46 pt / 他 2.52 pt</t>
+          <t xml:space="preserve">全社 11.48 pt / 補助 19.46 pt / ベース 2.52 pt</t>
         </is>
       </c>
       <c r="K24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.26 pt / 補助 18.68 pt / 他 1.67 pt</t>
+          <t xml:space="preserve">全社 11.26 pt / 補助 18.68 pt / ベース 1.67 pt</t>
         </is>
       </c>
       <c r="L24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.96 pt / 補助 19.61 pt / 他 1.27 pt</t>
+          <t xml:space="preserve">全社 11.96 pt / 補助 19.61 pt / ベース 1.27 pt</t>
         </is>
       </c>
     </row>
@@ -4924,47 +4924,47 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.33 % / 補助 2.5 % / 他 2.14 %</t>
+          <t xml:space="preserve">全社 2.33 % / 補助 2.5 % / ベース 2.14 %</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.33 % / 補助 2.5 % / 他 2.14 %</t>
+          <t xml:space="preserve">全社 2.33 % / 補助 2.5 % / ベース 2.14 %</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.33 % / 補助 2.5 % / 他 2.14 %</t>
+          <t xml:space="preserve">全社 2.33 % / 補助 2.5 % / ベース 2.14 %</t>
         </is>
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.71 % / 補助 3.28 % / 他 2.06 %</t>
+          <t xml:space="preserve">全社 2.71 % / 補助 3.28 % / ベース 2.06 %</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.05 % / 補助 3.97 % / 他 1.97 %</t>
+          <t xml:space="preserve">全社 3.05 % / 補助 3.97 % / ベース 1.97 %</t>
         </is>
       </c>
       <c r="I26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.35 % / 補助 4.59 % / 他 1.89 %</t>
+          <t xml:space="preserve">全社 3.35 % / 補助 4.59 % / ベース 1.89 %</t>
         </is>
       </c>
       <c r="J26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.91 % / 補助 3.76 % / 他 1.76 %</t>
+          <t xml:space="preserve">全社 2.91 % / 補助 3.76 % / ベース 1.76 %</t>
         </is>
       </c>
       <c r="K26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.52 % / 補助 3.08 % / 他 1.66 %</t>
+          <t xml:space="preserve">全社 2.52 % / 補助 3.08 % / ベース 1.66 %</t>
         </is>
       </c>
       <c r="L26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.18 % / 補助 2.53 % / 他 1.56 %</t>
+          <t xml:space="preserve">全社 2.18 % / 補助 2.53 % / ベース 1.56 %</t>
         </is>
       </c>
     </row>
@@ -5110,47 +5110,47 @@
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.46 倍 / 補助 4.77 倍 / 他 4.06 倍</t>
+          <t xml:space="preserve">全社 4.46 倍 / 補助 4.77 倍 / ベース 4.06 倍</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.38 倍 / 補助 4.71 倍 / 他 3.96 倍</t>
+          <t xml:space="preserve">全社 4.38 倍 / 補助 4.71 倍 / ベース 3.96 倍</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.31 倍 / 補助 4.65 倍 / 他 3.87 倍</t>
+          <t xml:space="preserve">全社 4.31 倍 / 補助 4.65 倍 / ベース 3.87 倍</t>
         </is>
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.69 倍 / 補助 3.56 倍 / 他 3.93 倍</t>
+          <t xml:space="preserve">全社 3.69 倍 / 補助 3.56 倍 / ベース 3.93 倍</t>
         </is>
       </c>
       <c r="H29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.26 倍 / 補助 2.94 倍 / 他 3.99 倍</t>
+          <t xml:space="preserve">全社 3.26 倍 / 補助 2.94 倍 / ベース 3.99 倍</t>
         </is>
       </c>
       <c r="I29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.93 倍 / 補助 2.54 倍 / 他 4.05 倍</t>
+          <t xml:space="preserve">全社 2.93 倍 / 補助 2.54 倍 / ベース 4.05 倍</t>
         </is>
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.97 倍 / 補助 3.61 倍 / 他 5 倍</t>
+          <t xml:space="preserve">全社 3.97 倍 / 補助 3.61 倍 / ベース 5 倍</t>
         </is>
       </c>
       <c r="K29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5.03 倍 / 補助 4.88 倍 / 他 5.44 倍</t>
+          <t xml:space="preserve">全社 5.03 倍 / 補助 4.88 倍 / ベース 5.44 倍</t>
         </is>
       </c>
       <c r="L29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.37 倍 / 補助 6.53 倍 / 他 5.94 倍</t>
+          <t xml:space="preserve">全社 6.37 倍 / 補助 6.53 倍 / ベース 5.94 倍</t>
         </is>
       </c>
     </row>
@@ -5219,7 +5219,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">5. 補助事業とその他事業の比較</t>
+          <t xml:space="preserve">5. 補助事業とベース事業の比較</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -5358,47 +5358,47 @@
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 — / 他 —</t>
+          <t xml:space="preserve">補助 — / ベース —</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 5.56 % / 他 4.35 %</t>
+          <t xml:space="preserve">補助 5.56 % / ベース 4.35 %</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 5.26 % / 他 4.17 %</t>
+          <t xml:space="preserve">補助 5.26 % / ベース 4.17 %</t>
         </is>
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 5.41 % / 他 4.26 %</t>
+          <t xml:space="preserve">補助 5.41 % / ベース 4.26 %</t>
         </is>
       </c>
       <c r="H33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 5.41 % / 他 4.26 %</t>
+          <t xml:space="preserve">補助 5.41 % / ベース 4.26 %</t>
         </is>
       </c>
       <c r="I33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 5.41 % / 他 4.26 %</t>
+          <t xml:space="preserve">補助 5.41 % / ベース 4.26 %</t>
         </is>
       </c>
       <c r="J33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 22.03 % / 他 7.31 %</t>
+          <t xml:space="preserve">補助 22.03 % / ベース 7.31 %</t>
         </is>
       </c>
       <c r="K33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 22.01 % / 他 6.25 %</t>
+          <t xml:space="preserve">補助 22.01 % / ベース 6.25 %</t>
         </is>
       </c>
       <c r="L33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 22.03 % / 他 6.27 %</t>
+          <t xml:space="preserve">補助 22.03 % / ベース 6.27 %</t>
         </is>
       </c>
     </row>
@@ -5410,7 +5410,7 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業原価率－その他事業原価率</t>
+          <t xml:space="preserve">補助事業原価率－ベース事業原価率</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -5472,7 +5472,7 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業営業利益率－その他事業営業利益率</t>
+          <t xml:space="preserve">補助事業営業利益率－ベース事業営業利益率</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -5544,47 +5544,47 @@
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.8 億円/人 / 他 0.537 億円/人</t>
+          <t xml:space="preserve">補助 0.8 億円/人 / ベース 0.537 億円/人</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.8 億円/人 / 他 0.538 億円/人</t>
+          <t xml:space="preserve">補助 0.8 億円/人 / ベース 0.538 億円/人</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.8 億円/人 / 他 0.538 億円/人</t>
+          <t xml:space="preserve">補助 0.8 億円/人 / ベース 0.538 億円/人</t>
         </is>
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.803 億円/人 / 他 0.541 億円/人</t>
+          <t xml:space="preserve">補助 0.803 億円/人 / ベース 0.541 億円/人</t>
         </is>
       </c>
       <c r="H36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.801 億円/人 / 他 0.54 億円/人</t>
+          <t xml:space="preserve">補助 0.801 億円/人 / ベース 0.54 億円/人</t>
         </is>
       </c>
       <c r="I36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.801 億円/人 / 他 0.543 億円/人</t>
+          <t xml:space="preserve">補助 0.801 億円/人 / ベース 0.543 億円/人</t>
         </is>
       </c>
       <c r="J36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.953 億円/人 / 他 0.556 億円/人</t>
+          <t xml:space="preserve">補助 0.953 億円/人 / ベース 0.556 億円/人</t>
         </is>
       </c>
       <c r="K36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.125 億円/人 / 他 0.565 億円/人</t>
+          <t xml:space="preserve">補助 1.125 億円/人 / ベース 0.565 億円/人</t>
         </is>
       </c>
       <c r="L36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.34 億円/人 / 他 0.572 億円/人</t>
+          <t xml:space="preserve">補助 1.34 億円/人 / ベース 0.572 億円/人</t>
         </is>
       </c>
     </row>
@@ -5606,47 +5606,47 @@
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.058 億円/人 / 他 0.059 億円/人</t>
+          <t xml:space="preserve">補助 0.058 億円/人 / ベース 0.059 億円/人</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.059 億円/人 / 他 0.06 億円/人</t>
+          <t xml:space="preserve">補助 0.059 億円/人 / ベース 0.06 億円/人</t>
         </is>
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.06 億円/人 / 他 0.062 億円/人</t>
+          <t xml:space="preserve">補助 0.06 億円/人 / ベース 0.062 億円/人</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.061 億円/人 / 他 0.063 億円/人</t>
+          <t xml:space="preserve">補助 0.061 億円/人 / ベース 0.063 億円/人</t>
         </is>
       </c>
       <c r="H37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.063 億円/人 / 他 0.064 億円/人</t>
+          <t xml:space="preserve">補助 0.063 億円/人 / ベース 0.064 億円/人</t>
         </is>
       </c>
       <c r="I37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.064 億円/人 / 他 0.065 億円/人</t>
+          <t xml:space="preserve">補助 0.064 億円/人 / ベース 0.065 億円/人</t>
         </is>
       </c>
       <c r="J37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.066 億円/人 / 他 0.067 億円/人</t>
+          <t xml:space="preserve">補助 0.066 億円/人 / ベース 0.067 億円/人</t>
         </is>
       </c>
       <c r="K37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.071 億円/人 / 他 0.069 億円/人</t>
+          <t xml:space="preserve">補助 0.071 億円/人 / ベース 0.069 億円/人</t>
         </is>
       </c>
       <c r="L37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.078 億円/人 / 他 0.07 億円/人</t>
+          <t xml:space="preserve">補助 0.078 億円/人 / ベース 0.07 億円/人</t>
         </is>
       </c>
     </row>
@@ -5936,7 +5936,7 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">その他事業 売上成長率（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 売上成長率（設備導入期間）</t>
         </is>
       </c>
       <c r="B10" s="2">
@@ -5957,7 +5957,7 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">その他事業 原価率改善ポイント（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 原価率改善ポイント（設備導入期間）</t>
         </is>
       </c>
       <c r="B11" s="2">
@@ -5978,7 +5978,7 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">その他事業1人当たり給与支給総額の年平均上昇率（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業1人当たり給与支給総額の年平均上昇率（設備導入期間）</t>
         </is>
       </c>
       <c r="B12" s="2">
@@ -5999,7 +5999,7 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">その他事業 常時使用する従業員数の成長率（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 常時使用する従業員数の成長率（設備導入期間）</t>
         </is>
       </c>
       <c r="B13" s="2">
@@ -6020,7 +6020,7 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">その他事業 その他販管費率改善ポイント（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 その他販管費率改善ポイント（設備導入期間）</t>
         </is>
       </c>
       <c r="B14" s="2">
@@ -6062,7 +6062,7 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">その他事業 売上成長率（基準年度後）</t>
+          <t xml:space="preserve">ベース事業 売上成長率（基準年度後）</t>
         </is>
       </c>
       <c r="B16" s="2">
@@ -6104,7 +6104,7 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">その他事業 原価率改善ポイント（基準年度後）</t>
+          <t xml:space="preserve">ベース事業 原価率改善ポイント（基準年度後）</t>
         </is>
       </c>
       <c r="B18" s="2">
@@ -6146,7 +6146,7 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">その他事業1人当たり給与支給総額の年平均上昇率（基準年度後）</t>
+          <t xml:space="preserve">ベース事業1人当たり給与支給総額の年平均上昇率（基準年度後）</t>
         </is>
       </c>
       <c r="B20" s="2">
@@ -6188,7 +6188,7 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">その他事業 常時使用する従業員数の成長率（基準年度後）</t>
+          <t xml:space="preserve">ベース事業 常時使用する従業員数の成長率（基準年度後）</t>
         </is>
       </c>
       <c r="B22" s="2">
@@ -6230,7 +6230,7 @@
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">その他事業 その他販管費率（事業化報告3年目）</t>
+          <t xml:space="preserve">ベース事業 その他販管費率（事業化報告3年目）</t>
         </is>
       </c>
       <c r="B24" s="2">

</xml_diff>

<commit_message>
Expose PL assumptions and align sample capex
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -1465,22 +1465,22 @@
         <v>36.4</v>
       </c>
       <c r="E9" s="2">
-        <v>38.86</v>
+        <v>38.870000000000005</v>
       </c>
       <c r="F9" s="2">
-        <v>41.44</v>
+        <v>41.47</v>
       </c>
       <c r="G9" s="2">
-        <v>44.15</v>
+        <v>44.18</v>
       </c>
       <c r="H9" s="2">
-        <v>47.87</v>
+        <v>47.93</v>
       </c>
       <c r="I9" s="2">
-        <v>52.519999999999996</v>
+        <v>52.589999999999996</v>
       </c>
       <c r="J9" s="2">
-        <v>57.73</v>
+        <v>57.81</v>
       </c>
     </row>
     <row r="10">
@@ -1499,22 +1499,22 @@
         <v>1</v>
       </c>
       <c r="E10" s="2">
-        <v>1.03</v>
+        <v>1.04</v>
       </c>
       <c r="F10" s="2">
-        <v>1.06</v>
+        <v>1.09</v>
       </c>
       <c r="G10" s="2">
-        <v>1.1099999999999999</v>
+        <v>1.1400000000000001</v>
       </c>
       <c r="H10" s="2">
-        <v>1.15</v>
+        <v>1.21</v>
       </c>
       <c r="I10" s="2">
-        <v>1.19</v>
+        <v>1.26</v>
       </c>
       <c r="J10" s="2">
-        <v>1.24</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="11">
@@ -1533,22 +1533,22 @@
         <v>0.9</v>
       </c>
       <c r="E11" s="2">
-        <v>0.93</v>
+        <v>0.9400000000000001</v>
       </c>
       <c r="F11" s="2">
-        <v>0.9600000000000001</v>
+        <v>0.99</v>
       </c>
       <c r="G11" s="2">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="H11" s="2">
-        <v>1.04</v>
+        <v>1.09</v>
       </c>
       <c r="I11" s="2">
-        <v>1.06</v>
+        <v>1.1300000000000001</v>
       </c>
       <c r="J11" s="2">
-        <v>1.1099999999999999</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="12">
@@ -1573,16 +1573,16 @@
         <v>0.1</v>
       </c>
       <c r="G12" s="2">
-        <v>0.11</v>
+        <v>0.12000000000000001</v>
       </c>
       <c r="H12" s="2">
-        <v>0.11</v>
+        <v>0.12000000000000001</v>
       </c>
       <c r="I12" s="2">
         <v>0.13</v>
       </c>
       <c r="J12" s="2">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="13">
@@ -1771,22 +1771,22 @@
         <v>11.600000000000001</v>
       </c>
       <c r="E18" s="4">
-        <v>11.480000000000004</v>
+        <v>11.470000000000006</v>
       </c>
       <c r="F18" s="4">
-        <v>11.350000000000016</v>
+        <v>11.320000000000014</v>
       </c>
       <c r="G18" s="4">
-        <v>11.210000000000004</v>
+        <v>11.180000000000003</v>
       </c>
       <c r="H18" s="4">
-        <v>17.239999999999988</v>
+        <v>17.179999999999986</v>
       </c>
       <c r="I18" s="4">
-        <v>23.34999999999998</v>
+        <v>23.27999999999998</v>
       </c>
       <c r="J18" s="4">
-        <v>31.170000000000044</v>
+        <v>31.090000000000046</v>
       </c>
     </row>
     <row r="19">
@@ -1805,22 +1805,22 @@
         <v>7.733333333333333</v>
       </c>
       <c r="E19" s="2">
-        <v>7.297692454389424</v>
+        <v>7.291335579429156</v>
       </c>
       <c r="F19" s="2">
-        <v>6.879621772336049</v>
+        <v>6.861437750030315</v>
       </c>
       <c r="G19" s="2">
-        <v>6.478645321620531</v>
+        <v>6.46130728775357</v>
       </c>
       <c r="H19" s="2">
-        <v>8.64290369479119</v>
+        <v>8.612823983556417</v>
       </c>
       <c r="I19" s="2">
-        <v>10.1539398156201</v>
+        <v>10.12349973908505</v>
       </c>
       <c r="J19" s="2">
-        <v>11.702207538669485</v>
+        <v>11.672172998948808</v>
       </c>
     </row>
     <row r="20">
@@ -1839,22 +1839,22 @@
         <v>11.3</v>
       </c>
       <c r="E20" s="4">
-        <v>11.169999999999991</v>
+        <v>11.159999999999991</v>
       </c>
       <c r="F20" s="4">
-        <v>11.019999999999996</v>
+        <v>10.989999999999995</v>
       </c>
       <c r="G20" s="4">
-        <v>10.860000000000003</v>
+        <v>10.830000000000005</v>
       </c>
       <c r="H20" s="4">
-        <v>16.009999999999998</v>
+        <v>15.949999999999996</v>
       </c>
       <c r="I20" s="4">
-        <v>22.009999999999984</v>
+        <v>21.939999999999984</v>
       </c>
       <c r="J20" s="4">
-        <v>29.700000000000014</v>
+        <v>29.62000000000001</v>
       </c>
     </row>
     <row r="21">
@@ -1873,22 +1873,22 @@
         <v>11.3</v>
       </c>
       <c r="E21" s="2">
-        <v>11.169999999999991</v>
+        <v>11.159999999999991</v>
       </c>
       <c r="F21" s="2">
-        <v>11.019999999999996</v>
+        <v>10.989999999999995</v>
       </c>
       <c r="G21" s="2">
-        <v>10.860000000000003</v>
+        <v>10.830000000000005</v>
       </c>
       <c r="H21" s="2">
-        <v>16.009999999999998</v>
+        <v>15.949999999999996</v>
       </c>
       <c r="I21" s="2">
-        <v>22.009999999999984</v>
+        <v>21.939999999999984</v>
       </c>
       <c r="J21" s="2">
-        <v>29.700000000000014</v>
+        <v>29.62000000000001</v>
       </c>
     </row>
     <row r="22">
@@ -1907,22 +1907,22 @@
         <v>7.91</v>
       </c>
       <c r="E22" s="2">
-        <v>7.815999999999994</v>
+        <v>7.805999999999994</v>
       </c>
       <c r="F22" s="2">
-        <v>7.711999999999997</v>
+        <v>7.691999999999997</v>
       </c>
       <c r="G22" s="2">
-        <v>7.5980000000000025</v>
+        <v>7.578000000000003</v>
       </c>
       <c r="H22" s="2">
-        <v>11.197999999999997</v>
+        <v>11.157999999999998</v>
       </c>
       <c r="I22" s="2">
-        <v>15.402999999999988</v>
+        <v>15.352999999999987</v>
       </c>
       <c r="J22" s="2">
-        <v>20.78200000000001</v>
+        <v>20.732000000000006</v>
       </c>
     </row>
     <row r="23">
@@ -1975,22 +1975,22 @@
         <v>1</v>
       </c>
       <c r="E24" s="2">
-        <v>1.03</v>
+        <v>1.04</v>
       </c>
       <c r="F24" s="2">
-        <v>1.06</v>
+        <v>1.09</v>
       </c>
       <c r="G24" s="2">
-        <v>1.1099999999999999</v>
+        <v>1.1400000000000001</v>
       </c>
       <c r="H24" s="2">
-        <v>1.15</v>
+        <v>1.21</v>
       </c>
       <c r="I24" s="2">
-        <v>1.19</v>
+        <v>1.26</v>
       </c>
       <c r="J24" s="2">
-        <v>1.24</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="25">
@@ -2055,7 +2055,7 @@
         <v>42.33999999999998</v>
       </c>
       <c r="I26" s="4">
-        <v>50.17999999999998</v>
+        <v>50.17999999999997</v>
       </c>
       <c r="J26" s="4">
         <v>59.90000000000004</v>
@@ -2091,10 +2091,10 @@
         <v>20.489470688673816</v>
       </c>
       <c r="I27" s="2">
-        <v>18.516769012753898</v>
+        <v>18.516769012753876</v>
       </c>
       <c r="J27" s="2">
-        <v>19.37026703866096</v>
+        <v>19.370267038660984</v>
       </c>
     </row>
     <row r="28">
@@ -2285,22 +2285,22 @@
         <v>0.2</v>
       </c>
       <c r="E33" s="2">
-        <v>0.20600000000000002</v>
+        <v>0.20800000000000002</v>
       </c>
       <c r="F33" s="2">
-        <v>0.21200000000000002</v>
+        <v>0.21800000000000003</v>
       </c>
       <c r="G33" s="2">
-        <v>0.22199999999999998</v>
+        <v>0.22800000000000004</v>
       </c>
       <c r="H33" s="2">
-        <v>0.22999999999999998</v>
+        <v>0.242</v>
       </c>
       <c r="I33" s="2">
-        <v>0.238</v>
+        <v>0.252</v>
       </c>
       <c r="J33" s="2">
-        <v>0.248</v>
+        <v>0.264</v>
       </c>
     </row>
     <row r="34">
@@ -2321,22 +2321,22 @@
         <v>4.166666666666674</v>
       </c>
       <c r="E34" s="2">
-        <v>3.0000000000000027</v>
+        <v>4.0000000000000036</v>
       </c>
       <c r="F34" s="2">
-        <v>2.9126213592232997</v>
+        <v>4.807692307692313</v>
       </c>
       <c r="G34" s="2">
-        <v>4.7169811320754595</v>
+        <v>4.587155963302747</v>
       </c>
       <c r="H34" s="2">
-        <v>3.603603603603611</v>
+        <v>6.140350877192957</v>
       </c>
       <c r="I34" s="2">
-        <v>3.4782608695652195</v>
+        <v>4.132231404958686</v>
       </c>
       <c r="J34" s="2">
-        <v>4.201680672268915</v>
+        <v>4.761904761904767</v>
       </c>
     </row>
     <row r="35">
@@ -2367,7 +2367,7 @@
         <v>0.15230215827338123</v>
       </c>
       <c r="I35" s="2">
-        <v>0.1736332179930795</v>
+        <v>0.17363321799307949</v>
       </c>
       <c r="J35" s="2">
         <v>0.1996666666666668</v>
@@ -2389,22 +2389,22 @@
         <v>15.100000000000001</v>
       </c>
       <c r="E36" s="4">
-        <v>15.750000000000004</v>
+        <v>15.740000000000006</v>
       </c>
       <c r="F36" s="4">
-        <v>16.380000000000017</v>
+        <v>16.350000000000016</v>
       </c>
       <c r="G36" s="4">
-        <v>17.010000000000005</v>
+        <v>16.980000000000004</v>
       </c>
       <c r="H36" s="4">
-        <v>23.03999999999999</v>
+        <v>22.979999999999986</v>
       </c>
       <c r="I36" s="4">
-        <v>29.14999999999998</v>
+        <v>29.07999999999998</v>
       </c>
       <c r="J36" s="4">
-        <v>36.97000000000004</v>
+        <v>36.89000000000004</v>
       </c>
     </row>
     <row r="37">
@@ -2423,22 +2423,22 @@
         <v>10.066666666666668</v>
       </c>
       <c r="E37" s="2">
-        <v>10.012078062424514</v>
+        <v>10.005721187464246</v>
       </c>
       <c r="F37" s="2">
-        <v>9.928476178930788</v>
+        <v>9.910292156625054</v>
       </c>
       <c r="G37" s="2">
-        <v>9.830665202566031</v>
+        <v>9.813327168699072</v>
       </c>
       <c r="H37" s="2">
-        <v>11.550609114152497</v>
+        <v>11.520529402917726</v>
       </c>
       <c r="I37" s="2">
-        <v>12.676117585667065</v>
+        <v>12.645677509132017</v>
       </c>
       <c r="J37" s="2">
-        <v>13.879711668418695</v>
+        <v>13.849677128698017</v>
       </c>
     </row>
     <row r="38">
@@ -2459,22 +2459,22 @@
         <v>3.1420765027322606</v>
       </c>
       <c r="E38" s="2">
-        <v>4.304635761589415</v>
+        <v>4.238410596026521</v>
       </c>
       <c r="F38" s="2">
-        <v>4.000000000000092</v>
+        <v>3.875476493011498</v>
       </c>
       <c r="G38" s="2">
-        <v>3.846153846153766</v>
+        <v>3.85321100917424</v>
       </c>
       <c r="H38" s="2">
-        <v>35.44973544973533</v>
+        <v>35.33568904593629</v>
       </c>
       <c r="I38" s="2">
-        <v>26.51909722222221</v>
+        <v>26.544821583986057</v>
       </c>
       <c r="J38" s="2">
-        <v>26.826758147513097</v>
+        <v>26.856946354883316</v>
       </c>
     </row>
   </sheetData>
@@ -3761,32 +3761,32 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.7 % / 補助 23.61 % / ベース 25.97 %</t>
+          <t xml:space="preserve">全社 24.71 % / 補助 23.61 % / ベース 25.98 %</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 25.12 % / 補助 24.28 % / ベース 26.1 %</t>
+          <t xml:space="preserve">全社 25.14 % / 補助 24.28 % / ベース 26.14 %</t>
         </is>
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 25.52 % / 補助 24.91 % / ベース 26.23 %</t>
+          <t xml:space="preserve">全社 25.53 % / 補助 24.91 % / ベース 26.27 %</t>
         </is>
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24 % / 補助 22.67 % / ベース 25.78 %</t>
+          <t xml:space="preserve">全社 24.03 % / 補助 22.67 % / ベース 25.85 %</t>
         </is>
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 22.84 % / 補助 21.03 % / ベース 25.63 %</t>
+          <t xml:space="preserve">全社 22.87 % / 補助 21.03 % / ベース 25.7 %</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 21.67 % / 補助 19.54 % / ベース 25.46 %</t>
+          <t xml:space="preserve">全社 21.7 % / 補助 19.54 % / ベース 25.54 %</t>
         </is>
       </c>
     </row>
@@ -3823,32 +3823,32 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.3 % / 補助 8.4 % / ベース 6.03 %</t>
+          <t xml:space="preserve">全社 7.29 % / 補助 8.4 % / ベース 6.02 %</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.88 % / 補助 7.72 % / ベース 5.9 %</t>
+          <t xml:space="preserve">全社 6.86 % / 補助 7.72 % / ベース 5.86 %</t>
         </is>
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.48 % / 補助 7.09 % / ベース 5.76 %</t>
+          <t xml:space="preserve">全社 6.46 % / 補助 7.09 % / ベース 5.72 %</t>
         </is>
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.64 % / 補助 9.83 % / ベース 7.05 %</t>
+          <t xml:space="preserve">全社 8.61 % / 補助 9.83 % / ベース 6.98 %</t>
         </is>
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.15 % / 補助 11.96 % / ベース 7.36 %</t>
+          <t xml:space="preserve">全社 10.12 % / 補助 11.96 % / ベース 7.29 %</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.7 % / 補助 13.96 % / ベース 7.71 %</t>
+          <t xml:space="preserve">全社 11.67 % / 補助 13.96 % / ベース 7.63 %</t>
         </is>
       </c>
     </row>
@@ -3885,32 +3885,32 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.01 % / 補助 11.68 % / ベース 8.08 %</t>
+          <t xml:space="preserve">全社 10.01 % / 補助 11.68 % / ベース 8.07 %</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.93 % / 補助 11.69 % / ベース 7.87 %</t>
+          <t xml:space="preserve">全社 9.91 % / 補助 11.69 % / ベース 7.83 %</t>
         </is>
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.83 % / 補助 11.68 % / ベース 7.65 %</t>
+          <t xml:space="preserve">全社 9.81 % / 補助 11.68 % / ベース 7.61 %</t>
         </is>
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.55 % / 補助 13.59 % / ベース 8.81 %</t>
+          <t xml:space="preserve">全社 11.52 % / 補助 13.59 % / ベース 8.74 %</t>
         </is>
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.68 % / 補助 15.05 % / ベース 9.02 %</t>
+          <t xml:space="preserve">全社 12.65 % / 補助 15.05 % / ベース 8.94 %</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.88 % / 補助 16.48 % / ベース 9.27 %</t>
+          <t xml:space="preserve">全社 13.85 % / 補助 16.48 % / ベース 9.19 %</t>
         </is>
       </c>
     </row>
@@ -4133,32 +4133,32 @@
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.65 % / 補助 0.5 % / ベース 0.84 %</t>
+          <t xml:space="preserve">全社 0.66 % / 補助 0.5 % / ベース 0.85 %</t>
         </is>
       </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.64 % / 補助 0.49 % / ベース 0.81 %</t>
+          <t xml:space="preserve">全社 0.66 % / 補助 0.49 % / ベース 0.85 %</t>
         </is>
       </c>
       <c r="I13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.64 % / 補助 0.5 % / ベース 0.81 %</t>
+          <t xml:space="preserve">全社 0.66 % / 補助 0.5 % / ベース 0.84 %</t>
         </is>
       </c>
       <c r="J13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.58 % / 補助 0.44 % / ベース 0.76 %</t>
+          <t xml:space="preserve">全社 0.61 % / 補助 0.44 % / ベース 0.83 %</t>
         </is>
       </c>
       <c r="K13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.52 % / 補助 0.37 % / ベース 0.74 %</t>
+          <t xml:space="preserve">全社 0.55 % / 補助 0.37 % / ベース 0.82 %</t>
         </is>
       </c>
       <c r="L13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.47 % / 補助 0.32 % / ベース 0.72 %</t>
+          <t xml:space="preserve">全社 0.5 % / 補助 0.32 % / ベース 0.8 %</t>
         </is>
       </c>
     </row>
@@ -4195,32 +4195,32 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.15 % / 補助 8.15 % / ベース 12.47 %</t>
+          <t xml:space="preserve">全社 10.16 % / 補助 8.15 % / ベース 12.48 %</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.31 % / 補助 8.3 % / ベース 12.66 %</t>
+          <t xml:space="preserve">全社 10.33 % / 補助 8.3 % / ベース 12.7 %</t>
         </is>
       </c>
       <c r="I14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.48 % / 補助 8.46 % / ベース 12.86 %</t>
+          <t xml:space="preserve">全社 10.5 % / 補助 8.46 % / ベース 12.9 %</t>
         </is>
       </c>
       <c r="J14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.68 % / 補助 7.35 % / ベース 12.8 %</t>
+          <t xml:space="preserve">全社 9.71 % / 補助 7.35 % / ベース 12.87 %</t>
         </is>
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.15 % / 補助 6.72 % / ベース 12.89 %</t>
+          <t xml:space="preserve">全社 9.18 % / 補助 6.72 % / ベース 12.97 %</t>
         </is>
       </c>
       <c r="L14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.61 % / 補助 6.15 % / ベース 12.96 %</t>
+          <t xml:space="preserve">全社 8.64 % / 補助 6.15 % / ベース 13.05 %</t>
         </is>
       </c>
     </row>
@@ -4319,32 +4319,32 @@
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.206 億円/人 / 補助 0.21 億円/人 / ベース 0.203 億円/人</t>
+          <t xml:space="preserve">全社 0.208 億円/人 / 補助 0.21 億円/人 / ベース 0.207 億円/人</t>
         </is>
       </c>
       <c r="H16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.212 億円/人 / 補助 0.22 億円/人 / ベース 0.207 億円/人</t>
+          <t xml:space="preserve">全社 0.218 億円/人 / 補助 0.22 億円/人 / ベース 0.217 億円/人</t>
         </is>
       </c>
       <c r="I16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.222 億円/人 / 補助 0.235 億円/人 / ベース 0.213 億円/人</t>
+          <t xml:space="preserve">全社 0.228 億円/人 / 補助 0.235 億円/人 / ベース 0.223 億円/人</t>
         </is>
       </c>
       <c r="J16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.23 億円/人 / 補助 0.25 億円/人 / ベース 0.217 億円/人</t>
+          <t xml:space="preserve">全社 0.242 億円/人 / 補助 0.25 億円/人 / ベース 0.237 億円/人</t>
         </is>
       </c>
       <c r="K16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.238 億円/人 / 補助 0.26 億円/人 / ベース 0.223 億円/人</t>
+          <t xml:space="preserve">全社 0.252 億円/人 / 補助 0.26 億円/人 / ベース 0.247 億円/人</t>
         </is>
       </c>
       <c r="L16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.248 億円/人 / 補助 0.275 億円/人 / ベース 0.23 億円/人</t>
+          <t xml:space="preserve">全社 0.264 億円/人 / 補助 0.275 億円/人 / ベース 0.257 億円/人</t>
         </is>
       </c>
     </row>
@@ -4443,32 +4443,32 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 50.35 % / 補助 41.09 % / ベース 60.67 %</t>
+          <t xml:space="preserve">全社 50.38 % / 補助 41.09 % / ベース 60.73 %</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 50.94 % / 補助 41.53 % / ベース 61.65 %</t>
+          <t xml:space="preserve">全社 51.03 % / 補助 41.53 % / ベース 61.84 %</t>
         </is>
       </c>
       <c r="I18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 51.59 % / 補助 42.02 % / ベース 62.69 %</t>
+          <t xml:space="preserve">全社 51.68 % / 補助 42.02 % / ベース 62.88 %</t>
         </is>
       </c>
       <c r="J18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 45.58 % / 補助 35.09 % / ベース 59.24 %</t>
+          <t xml:space="preserve">全社 45.73 % / 補助 35.09 % / ベース 59.57 %</t>
         </is>
       </c>
       <c r="K18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 41.91 % / 補助 30.86 % / ベース 58.83 %</t>
+          <t xml:space="preserve">全社 42.05 % / 補助 30.86 % / ベース 59.18 %</t>
         </is>
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 38.28 % / 補助 27.17 % / ベース 58.31 %</t>
+          <t xml:space="preserve">全社 38.41 % / 補助 27.17 % / ベース 58.68 %</t>
         </is>
       </c>
     </row>
@@ -4649,12 +4649,12 @@
       </c>
       <c r="K21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.082 億円/人 / 補助 0.135 億円/人 / ベース 0.042 億円/人</t>
+          <t xml:space="preserve">全社 0.082 億円/人 / 補助 0.135 億円/人 / ベース 0.041 億円/人</t>
         </is>
       </c>
       <c r="L21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.106 億円/人 / 補助 0.187 億円/人 / ベース 0.044 億円/人</t>
+          <t xml:space="preserve">全社 0.105 億円/人 / 補助 0.187 億円/人 / ベース 0.044 億円/人</t>
         </is>
       </c>
     </row>
@@ -5001,17 +5001,17 @@
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.54 %</t>
+          <t xml:space="preserve">全社 4.88 %</t>
         </is>
       </c>
       <c r="H27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.09 %</t>
+          <t xml:space="preserve">全社 4.65 %</t>
         </is>
       </c>
       <c r="I27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.67 %</t>
+          <t xml:space="preserve">全社 4.43 %</t>
         </is>
       </c>
       <c r="J27" s="0" t="inlineStr">
@@ -5063,17 +5063,17 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.95 倍</t>
+          <t xml:space="preserve">全社 0.49 倍</t>
         </is>
       </c>
       <c r="H28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.92 倍</t>
+          <t xml:space="preserve">全社 0.47 倍</t>
         </is>
       </c>
       <c r="I28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.88 倍</t>
+          <t xml:space="preserve">全社 0.45 倍</t>
         </is>
       </c>
       <c r="J28" s="0" t="inlineStr">
@@ -5130,27 +5130,27 @@
       </c>
       <c r="H29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.26 倍 / 補助 2.94 倍 / ベース 3.99 倍</t>
+          <t xml:space="preserve">全社 3.25 倍 / 補助 2.94 倍 / ベース 3.97 倍</t>
         </is>
       </c>
       <c r="I29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.93 倍 / 補助 2.54 倍 / ベース 4.05 倍</t>
+          <t xml:space="preserve">全社 2.93 倍 / 補助 2.54 倍 / ベース 4.03 倍</t>
         </is>
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.97 倍 / 補助 3.61 倍 / ベース 5 倍</t>
+          <t xml:space="preserve">全社 3.96 倍 / 補助 3.61 倍 / ベース 4.96 倍</t>
         </is>
       </c>
       <c r="K29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5.03 倍 / 補助 4.88 倍 / ベース 5.44 倍</t>
+          <t xml:space="preserve">全社 5.01 倍 / 補助 4.88 倍 / ベース 5.39 倍</t>
         </is>
       </c>
       <c r="L29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.37 倍 / 補助 6.53 倍 / ベース 5.94 倍</t>
+          <t xml:space="preserve">全社 6.36 倍 / 補助 6.53 倍 / ベース 5.89 倍</t>
         </is>
       </c>
     </row>
@@ -5187,17 +5187,17 @@
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.49 倍</t>
+          <t xml:space="preserve">全社 0.95 倍</t>
         </is>
       </c>
       <c r="H30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.51 倍</t>
+          <t xml:space="preserve">全社 1 倍</t>
         </is>
       </c>
       <c r="I30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.54 倍</t>
+          <t xml:space="preserve">全社 1.05 倍</t>
         </is>
       </c>
       <c r="J30" s="0" t="inlineStr">
@@ -5497,32 +5497,32 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 2.37 pt</t>
+          <t xml:space="preserve">差 2.38 pt</t>
         </is>
       </c>
       <c r="H35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 1.82 pt</t>
+          <t xml:space="preserve">差 1.86 pt</t>
         </is>
       </c>
       <c r="I35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 1.33 pt</t>
+          <t xml:space="preserve">差 1.36 pt</t>
         </is>
       </c>
       <c r="J35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 2.78 pt</t>
+          <t xml:space="preserve">差 2.85 pt</t>
         </is>
       </c>
       <c r="K35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 4.6 pt</t>
+          <t xml:space="preserve">差 4.68 pt</t>
         </is>
       </c>
       <c r="L35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 6.25 pt</t>
+          <t xml:space="preserve">差 6.33 pt</t>
         </is>
       </c>
     </row>
@@ -5683,12 +5683,12 @@
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 183.33 %</t>
+          <t xml:space="preserve">寄与率 169.23 %</t>
         </is>
       </c>
       <c r="H38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 169.23 %</t>
+          <t xml:space="preserve">寄与率 146.67 %</t>
         </is>
       </c>
       <c r="I38" s="0" t="inlineStr">
@@ -5698,17 +5698,17 @@
       </c>
       <c r="J38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 76.29 %</t>
+          <t xml:space="preserve">寄与率 76.67 %</t>
         </is>
       </c>
       <c r="K38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 89.2 %</t>
+          <t xml:space="preserve">寄与率 89.34 %</t>
         </is>
       </c>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 90.41 %</t>
+          <t xml:space="preserve">寄与率 90.52 %</t>
         </is>
       </c>
     </row>
@@ -5718,7 +5718,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="68" customWidth="1"/>
@@ -5810,11 +5810,11 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 売上成長率（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 原価率（売上実績が0の場合の開始水準）</t>
         </is>
       </c>
       <c r="B4" s="2">
-        <v>5.409356725146197</v>
+        <v>68</v>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
@@ -5822,20 +5822,20 @@
         </is>
       </c>
       <c r="D4" s="2">
-        <v>5.116959064327475</v>
+        <v>0</v>
       </c>
       <c r="E4" s="2">
-        <v>5.701754385964919</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 原価率改善ポイント（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 原価率（売上実績が0の場合の開始水準）</t>
         </is>
       </c>
       <c r="B5" s="2">
-        <v>5.551115123125783e-15</v>
+        <v>68</v>
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
@@ -5846,34 +5846,34 @@
         <v>0</v>
       </c>
       <c r="E5" s="2">
-        <v>1.6653345369377348e-14</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 1人当たり給与支給総額上昇率（設備導入期間）</t>
+          <t xml:space="preserve">実効税率</t>
         </is>
       </c>
       <c r="B6" s="2">
-        <v>2.0030662342518046</v>
+        <v>30</v>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">基準年度額が最新決算期額以上（成長率0%以上）</t>
+          <t xml:space="preserve">—</t>
         </is>
       </c>
       <c r="D6" s="2">
-        <v>1.9325330501846927</v>
+        <v>0</v>
       </c>
       <c r="E6" s="2">
-        <v>2.0735994183189166</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 常時使用する従業員数の成長率（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 売上成長率（設備導入期間）</t>
         </is>
       </c>
       <c r="B7" s="2">
@@ -5894,11 +5894,11 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 その他販管費率改善ポイント（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 原価率改善ポイント（設備導入期間）</t>
         </is>
       </c>
       <c r="B8" s="2">
-        <v>0</v>
+        <v>5.551115123125783e-15</v>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
@@ -5909,38 +5909,38 @@
         <v>0</v>
       </c>
       <c r="E8" s="2">
-        <v>0</v>
+        <v>1.6653345369377348e-14</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">役員1人当たり給与支給総額上昇率（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 1人当たり給与支給総額上昇率（設備導入期間）</t>
         </is>
       </c>
       <c r="B9" s="2">
-        <v>5.409356725146197</v>
+        <v>2.0030662342518046</v>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">—</t>
+          <t xml:space="preserve">基準年度額が最新決算期額以上（成長率0%以上）</t>
         </is>
       </c>
       <c r="D9" s="2">
-        <v>5.116959064327475</v>
+        <v>1.9325330501846927</v>
       </c>
       <c r="E9" s="2">
-        <v>5.701754385964919</v>
+        <v>2.0735994183189166</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 売上成長率（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 常時使用する従業員数の成長率（設備導入期間）</t>
         </is>
       </c>
       <c r="B10" s="2">
-        <v>4.257246376811585</v>
+        <v>5.409356725146197</v>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
@@ -5948,16 +5948,16 @@
         </is>
       </c>
       <c r="D10" s="2">
-        <v>4.076086956521719</v>
+        <v>5.116959064327475</v>
       </c>
       <c r="E10" s="2">
-        <v>4.438405797101453</v>
+        <v>5.701754385964919</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 原価率改善ポイント（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 その他販管費率改善ポイント（設備導入期間）</t>
         </is>
       </c>
       <c r="B11" s="2">
@@ -5972,17 +5972,17 @@
         <v>0</v>
       </c>
       <c r="E11" s="2">
-        <v>0.013457556935819737</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業1人当たり給与支給総額の年平均上昇率（設備導入期間）</t>
+          <t xml:space="preserve">役員1人当たり給与支給総額上昇率（設備導入期間）</t>
         </is>
       </c>
       <c r="B12" s="2">
-        <v>1.984645846924027</v>
+        <v>5.409356725146197</v>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
@@ -5990,20 +5990,20 @@
         </is>
       </c>
       <c r="D12" s="2">
-        <v>1.9139457023717443</v>
+        <v>5.116959064327475</v>
       </c>
       <c r="E12" s="2">
-        <v>2.0553459914763095</v>
+        <v>5.701754385964919</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 常時使用する従業員数の成長率（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 売上成長率（設備導入期間）</t>
         </is>
       </c>
       <c r="B13" s="2">
-        <v>4.083333333333339</v>
+        <v>4.257246376811585</v>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
@@ -6011,16 +6011,16 @@
         </is>
       </c>
       <c r="D13" s="2">
-        <v>3.9166666666666683</v>
+        <v>4.076086956521719</v>
       </c>
       <c r="E13" s="2">
-        <v>4.250000000000009</v>
+        <v>4.438405797101453</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 その他販管費率改善ポイント（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 原価率改善ポイント（設備導入期間）</t>
         </is>
       </c>
       <c r="B14" s="2">
@@ -6035,17 +6035,17 @@
         <v>0</v>
       </c>
       <c r="E14" s="2">
-        <v>0</v>
+        <v>0.013457556935819737</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 売上成長率（基準年度後）</t>
+          <t xml:space="preserve">ベース事業1人当たり給与支給総額の年平均上昇率（設備導入期間）</t>
         </is>
       </c>
       <c r="B15" s="2">
-        <v>22</v>
+        <v>1.984645846924027</v>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
@@ -6053,20 +6053,20 @@
         </is>
       </c>
       <c r="D15" s="2">
-        <v>15</v>
+        <v>1.9139457023717443</v>
       </c>
       <c r="E15" s="2">
-        <v>30</v>
+        <v>2.0553459914763095</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 売上成長率（基準年度後）</t>
+          <t xml:space="preserve">ベース事業 役員1人当たり給与支給総額上昇率（設備導入期間）</t>
         </is>
       </c>
       <c r="B16" s="2">
-        <v>6.257246376811586</v>
+        <v>4</v>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
@@ -6074,20 +6074,20 @@
         </is>
       </c>
       <c r="D16" s="2">
-        <v>6.076086956521719</v>
+        <v>0</v>
       </c>
       <c r="E16" s="2">
-        <v>6.438405797101453</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 原価率改善ポイント（基準年度後）</t>
+          <t xml:space="preserve">ベース事業 常時使用する従業員数の成長率（設備導入期間）</t>
         </is>
       </c>
       <c r="B17" s="2">
-        <v>1.5</v>
+        <v>4.083333333333339</v>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
@@ -6095,20 +6095,20 @@
         </is>
       </c>
       <c r="D17" s="2">
-        <v>0</v>
+        <v>3.9166666666666683</v>
       </c>
       <c r="E17" s="2">
-        <v>3</v>
+        <v>4.250000000000009</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 原価率改善ポイント（基準年度後）</t>
+          <t xml:space="preserve">ベース事業 その他販管費率改善ポイント（設備導入期間）</t>
         </is>
       </c>
       <c r="B18" s="2">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
@@ -6116,20 +6116,20 @@
         </is>
       </c>
       <c r="D18" s="2">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E18" s="2">
-        <v>0.5134575569358197</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業1人当たり給与支給総額の年平均上昇率</t>
+          <t xml:space="preserve">補助事業 売上成長率（基準年度後）</t>
         </is>
       </c>
       <c r="B19" s="2">
-        <v>7.000000000000001</v>
+        <v>22</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
@@ -6137,20 +6137,20 @@
         </is>
       </c>
       <c r="D19" s="2">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E19" s="2">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業1人当たり給与支給総額の年平均上昇率（基準年度後）</t>
+          <t xml:space="preserve">ベース事業 売上成長率（基準年度後）</t>
         </is>
       </c>
       <c r="B20" s="2">
-        <v>2.484645846924027</v>
+        <v>6.257246376811586</v>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
@@ -6158,20 +6158,20 @@
         </is>
       </c>
       <c r="D20" s="2">
-        <v>2.4139457023717443</v>
+        <v>6.076086956521719</v>
       </c>
       <c r="E20" s="2">
-        <v>2.5553459914763095</v>
+        <v>6.438405797101453</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 常時使用する従業員数の成長率</t>
+          <t xml:space="preserve">補助事業 原価率改善ポイント（基準年度後）</t>
         </is>
       </c>
       <c r="B21" s="2">
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
@@ -6182,17 +6182,17 @@
         <v>0</v>
       </c>
       <c r="E21" s="2">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 常時使用する従業員数の成長率（基準年度後）</t>
+          <t xml:space="preserve">ベース事業 原価率改善ポイント（基準年度後）</t>
         </is>
       </c>
       <c r="B22" s="2">
-        <v>4.583333333333338</v>
+        <v>0.5</v>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
@@ -6200,20 +6200,20 @@
         </is>
       </c>
       <c r="D22" s="2">
-        <v>4.416666666666668</v>
+        <v>0.5</v>
       </c>
       <c r="E22" s="2">
-        <v>4.750000000000009</v>
+        <v>0.5134575569358197</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 その他販管費率（事業化報告3年目）</t>
+          <t xml:space="preserve">補助事業1人当たり給与支給総額の年平均上昇率</t>
         </is>
       </c>
       <c r="B23" s="2">
-        <v>11</v>
+        <v>7.000000000000001</v>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
@@ -6221,20 +6221,20 @@
         </is>
       </c>
       <c r="D23" s="2">
-        <v>8.5</v>
+        <v>5</v>
       </c>
       <c r="E23" s="2">
-        <v>13.5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 その他販管費率（事業化報告3年目）</t>
+          <t xml:space="preserve">ベース事業1人当たり給与支給総額の年平均上昇率（基準年度後）</t>
         </is>
       </c>
       <c r="B24" s="2">
-        <v>10.928571428571427</v>
+        <v>2.484645846924027</v>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
@@ -6242,20 +6242,20 @@
         </is>
       </c>
       <c r="D24" s="2">
-        <v>8.928571428571427</v>
+        <v>2.4139457023717443</v>
       </c>
       <c r="E24" s="2">
-        <v>11.928571428571427</v>
+        <v>2.5553459914763095</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">役員1人当たり給与支給総額の年平均上昇率</t>
+          <t xml:space="preserve">ベース事業 役員1人当たり給与支給総額上昇率（基準年度後）</t>
         </is>
       </c>
       <c r="B25" s="2">
-        <v>5.380116959064325</v>
+        <v>4.5</v>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
@@ -6263,82 +6263,187 @@
         </is>
       </c>
       <c r="D25" s="2">
-        <v>4.263157894736836</v>
+        <v>0</v>
       </c>
       <c r="E25" s="2">
-        <v>6.555555555555557</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">新規投資の耐用年数</t>
+          <t xml:space="preserve">補助事業 常時使用する従業員数の成長率</t>
         </is>
       </c>
       <c r="B26" s="2">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D26" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E26" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="D26" s="2">
+        <v>0</v>
+      </c>
+      <c r="E26" s="2">
+        <v>8</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業投資額</t>
+          <t xml:space="preserve">ベース事業 常時使用する従業員数の成長率（基準年度後）</t>
         </is>
       </c>
       <c r="B27" s="2">
-        <v>23</v>
+        <v>4.583333333333338</v>
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">20億円以上（専門家経費・外注費を除く補助対象経費）</t>
-        </is>
-      </c>
-      <c r="D27" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E27" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D27" s="2">
+        <v>4.416666666666668</v>
+      </c>
+      <c r="E27" s="2">
+        <v>4.750000000000009</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">補助事業 その他販管費率（事業化報告3年目）</t>
+        </is>
+      </c>
+      <c r="B28" s="2">
+        <v>11</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D28" s="2">
+        <v>8.5</v>
+      </c>
+      <c r="E28" s="2">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ベース事業 その他販管費率（事業化報告3年目）</t>
+        </is>
+      </c>
+      <c r="B29" s="2">
+        <v>10.928571428571427</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D29" s="2">
+        <v>8.928571428571427</v>
+      </c>
+      <c r="E29" s="2">
+        <v>11.928571428571427</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">役員1人当たり給与支給総額の年平均上昇率</t>
+        </is>
+      </c>
+      <c r="B30" s="2">
+        <v>5.380116959064325</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D30" s="2">
+        <v>4.263157894736836</v>
+      </c>
+      <c r="E30" s="2">
+        <v>6.555555555555557</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">新規投資の耐用年数</t>
+        </is>
+      </c>
+      <c r="B31" s="2">
+        <v>10</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">補助事業投資額</t>
+        </is>
+      </c>
+      <c r="B32" s="2">
+        <v>23</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20億円以上（専門家経費・外注費を除く補助対象経費）</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E32" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">申請補助金額</t>
         </is>
       </c>
-      <c r="B28" s="2">
+      <c r="B33" s="2">
         <v>7.66</v>
       </c>
-      <c r="C28" s="0" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">50億円以下、かつ投資額の1/3以下（現在上限7.66億円）</t>
         </is>
       </c>
-      <c r="D28" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E28" s="0" t="inlineStr">
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E33" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6350,7 +6455,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C244"/>
+  <dimension ref="A1:C259"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="72" customWidth="1"/>
@@ -8285,26 +8390,26 @@
     <row r="129">
       <c r="A129" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:investment:0</t>
+          <t xml:space="preserve">driver-range:effectiveTaxRate:0</t>
         </is>
       </c>
       <c r="B129" s="2">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="C129" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:investment:1</t>
+          <t xml:space="preserve">driver-range:effectiveTaxRate:1</t>
         </is>
       </c>
       <c r="B130" s="2">
-        <v>200</v>
+        <v>0.6</v>
       </c>
       <c r="C130" s="0" t="inlineStr">
         <is>
@@ -8315,26 +8420,26 @@
     <row r="131">
       <c r="A131" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:localBenchmark:0</t>
+          <t xml:space="preserve">driver-range:investment:0</t>
         </is>
       </c>
       <c r="B131" s="2">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="C131" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:localBenchmark:1</t>
+          <t xml:space="preserve">driver-range:investment:1</t>
         </is>
       </c>
       <c r="B132" s="2">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="C132" s="0" t="inlineStr">
         <is>
@@ -8345,26 +8450,26 @@
     <row r="133">
       <c r="A133" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherCogsImprovement:0</t>
+          <t xml:space="preserve">driver-range:localBenchmark:0</t>
         </is>
       </c>
       <c r="B133" s="2">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="C133" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherCogsImprovement:1</t>
+          <t xml:space="preserve">driver-range:localBenchmark:1</t>
         </is>
       </c>
       <c r="B134" s="2">
-        <v>0.0051345755693581975</v>
+        <v>100</v>
       </c>
       <c r="C134" s="0" t="inlineStr">
         <is>
@@ -8375,26 +8480,26 @@
     <row r="135">
       <c r="A135" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherCogsImprovementToBase:0</t>
+          <t xml:space="preserve">driver-range:otherCogsImprovement:0</t>
         </is>
       </c>
       <c r="B135" s="2">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="C135" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherCogsImprovementToBase:1</t>
+          <t xml:space="preserve">driver-range:otherCogsImprovement:1</t>
         </is>
       </c>
       <c r="B136" s="2">
-        <v>0.00013457556935819737</v>
+        <v>0.0051345755693581975</v>
       </c>
       <c r="C136" s="0" t="inlineStr">
         <is>
@@ -8405,26 +8510,26 @@
     <row r="137">
       <c r="A137" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherHeadcountGrowth:0</t>
+          <t xml:space="preserve">driver-range:otherCogsImprovementToBase:0</t>
         </is>
       </c>
       <c r="B137" s="2">
-        <v>0.04416666666666668</v>
+        <v>0</v>
       </c>
       <c r="C137" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherHeadcountGrowth:1</t>
+          <t xml:space="preserve">driver-range:otherCogsImprovementToBase:1</t>
         </is>
       </c>
       <c r="B138" s="2">
-        <v>0.04750000000000009</v>
+        <v>0.00013457556935819737</v>
       </c>
       <c r="C138" s="0" t="inlineStr">
         <is>
@@ -8435,26 +8540,26 @@
     <row r="139">
       <c r="A139" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherHeadcountGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:otherCogsRateWhenSalesZero:0</t>
         </is>
       </c>
       <c r="B139" s="2">
-        <v>0.03916666666666668</v>
+        <v>0</v>
       </c>
       <c r="C139" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherHeadcountGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:otherCogsRateWhenSalesZero:1</t>
         </is>
       </c>
       <c r="B140" s="2">
-        <v>0.04250000000000009</v>
+        <v>0.99</v>
       </c>
       <c r="C140" s="0" t="inlineStr">
         <is>
@@ -8465,11 +8570,11 @@
     <row r="141">
       <c r="A141" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherPayGrowth:0</t>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowth:0</t>
         </is>
       </c>
       <c r="B141" s="2">
-        <v>0.024139457023717444</v>
+        <v>0.04416666666666668</v>
       </c>
       <c r="C141" s="0" t="inlineStr">
         <is>
@@ -8480,11 +8585,11 @@
     <row r="142">
       <c r="A142" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherPayGrowth:1</t>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowth:1</t>
         </is>
       </c>
       <c r="B142" s="2">
-        <v>0.025553459914763096</v>
+        <v>0.04750000000000009</v>
       </c>
       <c r="C142" s="0" t="inlineStr">
         <is>
@@ -8495,11 +8600,11 @@
     <row r="143">
       <c r="A143" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherPayGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowthToBase:0</t>
         </is>
       </c>
       <c r="B143" s="2">
-        <v>0.019139457023717443</v>
+        <v>0.03916666666666668</v>
       </c>
       <c r="C143" s="0" t="inlineStr">
         <is>
@@ -8510,11 +8615,11 @@
     <row r="144">
       <c r="A144" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherPayGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowthToBase:1</t>
         </is>
       </c>
       <c r="B144" s="2">
-        <v>0.020553459914763095</v>
+        <v>0.04250000000000009</v>
       </c>
       <c r="C144" s="0" t="inlineStr">
         <is>
@@ -8525,26 +8630,26 @@
     <row r="145">
       <c r="A145" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSalesGrowth:0</t>
+          <t xml:space="preserve">driver-range:otherOfficerPayGrowth:0</t>
         </is>
       </c>
       <c r="B145" s="2">
-        <v>0.06076086956521719</v>
+        <v>0</v>
       </c>
       <c r="C145" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSalesGrowth:1</t>
+          <t xml:space="preserve">driver-range:otherOfficerPayGrowth:1</t>
         </is>
       </c>
       <c r="B146" s="2">
-        <v>0.06438405797101453</v>
+        <v>0.08</v>
       </c>
       <c r="C146" s="0" t="inlineStr">
         <is>
@@ -8555,26 +8660,26 @@
     <row r="147">
       <c r="A147" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSalesGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:otherOfficerPayGrowthToBase:0</t>
         </is>
       </c>
       <c r="B147" s="2">
-        <v>0.040760869565217184</v>
+        <v>0</v>
       </c>
       <c r="C147" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSalesGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:otherOfficerPayGrowthToBase:1</t>
         </is>
       </c>
       <c r="B148" s="2">
-        <v>0.04438405797101452</v>
+        <v>0.08</v>
       </c>
       <c r="C148" s="0" t="inlineStr">
         <is>
@@ -8585,41 +8690,41 @@
     <row r="149">
       <c r="A149" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSgaImprovementToBase:0</t>
+          <t xml:space="preserve">driver-range:otherPayGrowth:0</t>
         </is>
       </c>
       <c r="B149" s="2">
-        <v>0</v>
+        <v>0.024139457023717444</v>
       </c>
       <c r="C149" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSgaImprovementToBase:1</t>
+          <t xml:space="preserve">driver-range:otherPayGrowth:1</t>
         </is>
       </c>
       <c r="B150" s="2">
-        <v>0</v>
+        <v>0.025553459914763096</v>
       </c>
       <c r="C150" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSgaRateEnd:0</t>
+          <t xml:space="preserve">driver-range:otherPayGrowthToBase:0</t>
         </is>
       </c>
       <c r="B151" s="2">
-        <v>0.08928571428571427</v>
+        <v>0.019139457023717443</v>
       </c>
       <c r="C151" s="0" t="inlineStr">
         <is>
@@ -8630,11 +8735,11 @@
     <row r="152">
       <c r="A152" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSgaRateEnd:1</t>
+          <t xml:space="preserve">driver-range:otherPayGrowthToBase:1</t>
         </is>
       </c>
       <c r="B152" s="2">
-        <v>0.11928571428571427</v>
+        <v>0.020553459914763095</v>
       </c>
       <c r="C152" s="0" t="inlineStr">
         <is>
@@ -8645,26 +8750,26 @@
     <row r="153">
       <c r="A153" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsImprovementAfterBase:0</t>
+          <t xml:space="preserve">driver-range:otherSalesGrowth:0</t>
         </is>
       </c>
       <c r="B153" s="2">
-        <v>0</v>
+        <v>0.06076086956521719</v>
       </c>
       <c r="C153" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsImprovementAfterBase:1</t>
+          <t xml:space="preserve">driver-range:otherSalesGrowth:1</t>
         </is>
       </c>
       <c r="B154" s="2">
-        <v>0.03</v>
+        <v>0.06438405797101453</v>
       </c>
       <c r="C154" s="0" t="inlineStr">
         <is>
@@ -8675,26 +8780,26 @@
     <row r="155">
       <c r="A155" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsImprovementToBase:0</t>
+          <t xml:space="preserve">driver-range:otherSalesGrowthToBase:0</t>
         </is>
       </c>
       <c r="B155" s="2">
-        <v>0</v>
+        <v>0.040760869565217184</v>
       </c>
       <c r="C155" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsImprovementToBase:1</t>
+          <t xml:space="preserve">driver-range:otherSalesGrowthToBase:1</t>
         </is>
       </c>
       <c r="B156" s="2">
-        <v>1.6653345369377348e-16</v>
+        <v>0.04438405797101452</v>
       </c>
       <c r="C156" s="0" t="inlineStr">
         <is>
@@ -8705,7 +8810,7 @@
     <row r="157">
       <c r="A157" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectHeadcountGrowth:0</t>
+          <t xml:space="preserve">driver-range:otherSgaImprovementToBase:0</t>
         </is>
       </c>
       <c r="B157" s="2">
@@ -8720,26 +8825,26 @@
     <row r="158">
       <c r="A158" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectHeadcountGrowth:1</t>
+          <t xml:space="preserve">driver-range:otherSgaImprovementToBase:1</t>
         </is>
       </c>
       <c r="B158" s="2">
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="C158" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectHeadcountGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:otherSgaRateEnd:0</t>
         </is>
       </c>
       <c r="B159" s="2">
-        <v>0.051169590643274754</v>
+        <v>0.08928571428571427</v>
       </c>
       <c r="C159" s="0" t="inlineStr">
         <is>
@@ -8750,11 +8855,11 @@
     <row r="160">
       <c r="A160" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectHeadcountGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:otherSgaRateEnd:1</t>
         </is>
       </c>
       <c r="B160" s="2">
-        <v>0.05701754385964919</v>
+        <v>0.11928571428571427</v>
       </c>
       <c r="C160" s="0" t="inlineStr">
         <is>
@@ -8765,26 +8870,26 @@
     <row r="161">
       <c r="A161" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectMarketGrowth:0</t>
+          <t xml:space="preserve">driver-range:projectCogsImprovementAfterBase:0</t>
         </is>
       </c>
       <c r="B161" s="2">
-        <v>-0.05</v>
+        <v>0</v>
       </c>
       <c r="C161" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectMarketGrowth:1</t>
+          <t xml:space="preserve">driver-range:projectCogsImprovementAfterBase:1</t>
         </is>
       </c>
       <c r="B162" s="2">
-        <v>0.3</v>
+        <v>0.03</v>
       </c>
       <c r="C162" s="0" t="inlineStr">
         <is>
@@ -8795,26 +8900,26 @@
     <row r="163">
       <c r="A163" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectOfficerPayGrowth:0</t>
+          <t xml:space="preserve">driver-range:projectCogsImprovementToBase:0</t>
         </is>
       </c>
       <c r="B163" s="2">
-        <v>0.04263157894736836</v>
+        <v>0</v>
       </c>
       <c r="C163" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectOfficerPayGrowth:1</t>
+          <t xml:space="preserve">driver-range:projectCogsImprovementToBase:1</t>
         </is>
       </c>
       <c r="B164" s="2">
-        <v>0.06555555555555558</v>
+        <v>1.6653345369377348e-16</v>
       </c>
       <c r="C164" s="0" t="inlineStr">
         <is>
@@ -8825,26 +8930,26 @@
     <row r="165">
       <c r="A165" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectOfficerPayGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:projectCogsRateWhenSalesZero:0</t>
         </is>
       </c>
       <c r="B165" s="2">
-        <v>0.051169590643274754</v>
+        <v>0</v>
       </c>
       <c r="C165" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectOfficerPayGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:projectCogsRateWhenSalesZero:1</t>
         </is>
       </c>
       <c r="B166" s="2">
-        <v>0.05701754385964919</v>
+        <v>0.99</v>
       </c>
       <c r="C166" s="0" t="inlineStr">
         <is>
@@ -8855,26 +8960,26 @@
     <row r="167">
       <c r="A167" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectPayGrowth:0</t>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowth:0</t>
         </is>
       </c>
       <c r="B167" s="2">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="C167" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectPayGrowth:1</t>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowth:1</t>
         </is>
       </c>
       <c r="B168" s="2">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="C168" s="0" t="inlineStr">
         <is>
@@ -8885,11 +8990,11 @@
     <row r="169">
       <c r="A169" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectPayGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowthToBase:0</t>
         </is>
       </c>
       <c r="B169" s="2">
-        <v>0.019325330501846927</v>
+        <v>0.051169590643274754</v>
       </c>
       <c r="C169" s="0" t="inlineStr">
         <is>
@@ -8900,11 +9005,11 @@
     <row r="170">
       <c r="A170" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectPayGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowthToBase:1</t>
         </is>
       </c>
       <c r="B170" s="2">
-        <v>0.020735994183189166</v>
+        <v>0.05701754385964919</v>
       </c>
       <c r="C170" s="0" t="inlineStr">
         <is>
@@ -8915,11 +9020,11 @@
     <row r="171">
       <c r="A171" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSalesGrowth:0</t>
+          <t xml:space="preserve">driver-range:projectMarketGrowth:0</t>
         </is>
       </c>
       <c r="B171" s="2">
-        <v>0.15</v>
+        <v>-0.05</v>
       </c>
       <c r="C171" s="0" t="inlineStr">
         <is>
@@ -8930,7 +9035,7 @@
     <row r="172">
       <c r="A172" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSalesGrowth:1</t>
+          <t xml:space="preserve">driver-range:projectMarketGrowth:1</t>
         </is>
       </c>
       <c r="B172" s="2">
@@ -8945,11 +9050,11 @@
     <row r="173">
       <c r="A173" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSalesGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowth:0</t>
         </is>
       </c>
       <c r="B173" s="2">
-        <v>0.051169590643274754</v>
+        <v>0.04263157894736836</v>
       </c>
       <c r="C173" s="0" t="inlineStr">
         <is>
@@ -8960,11 +9065,11 @@
     <row r="174">
       <c r="A174" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSalesGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowth:1</t>
         </is>
       </c>
       <c r="B174" s="2">
-        <v>0.05701754385964919</v>
+        <v>0.06555555555555558</v>
       </c>
       <c r="C174" s="0" t="inlineStr">
         <is>
@@ -8975,41 +9080,41 @@
     <row r="175">
       <c r="A175" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSgaImprovementToBase:0</t>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowthToBase:0</t>
         </is>
       </c>
       <c r="B175" s="2">
-        <v>0</v>
+        <v>0.051169590643274754</v>
       </c>
       <c r="C175" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSgaImprovementToBase:1</t>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowthToBase:1</t>
         </is>
       </c>
       <c r="B176" s="2">
-        <v>0</v>
+        <v>0.05701754385964919</v>
       </c>
       <c r="C176" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSgaRateEnd:0</t>
+          <t xml:space="preserve">driver-range:projectPayGrowth:0</t>
         </is>
       </c>
       <c r="B177" s="2">
-        <v>0.08499999999999999</v>
+        <v>0.05</v>
       </c>
       <c r="C177" s="0" t="inlineStr">
         <is>
@@ -9020,11 +9125,11 @@
     <row r="178">
       <c r="A178" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSgaRateEnd:1</t>
+          <t xml:space="preserve">driver-range:projectPayGrowth:1</t>
         </is>
       </c>
       <c r="B178" s="2">
-        <v>0.135</v>
+        <v>0.1</v>
       </c>
       <c r="C178" s="0" t="inlineStr">
         <is>
@@ -9035,11 +9140,11 @@
     <row r="179">
       <c r="A179" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:subsidy:0</t>
+          <t xml:space="preserve">driver-range:projectPayGrowthToBase:0</t>
         </is>
       </c>
       <c r="B179" s="2">
-        <v>1</v>
+        <v>0.019325330501846927</v>
       </c>
       <c r="C179" s="0" t="inlineStr">
         <is>
@@ -9050,11 +9155,11 @@
     <row r="180">
       <c r="A180" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:subsidy:1</t>
+          <t xml:space="preserve">driver-range:projectPayGrowthToBase:1</t>
         </is>
       </c>
       <c r="B180" s="2">
-        <v>50</v>
+        <v>0.020735994183189166</v>
       </c>
       <c r="C180" s="0" t="inlineStr">
         <is>
@@ -9065,11 +9170,11 @@
     <row r="181">
       <c r="A181" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:usefulLife:0</t>
+          <t xml:space="preserve">driver-range:projectSalesGrowth:0</t>
         </is>
       </c>
       <c r="B181" s="2">
-        <v>5</v>
+        <v>0.15</v>
       </c>
       <c r="C181" s="0" t="inlineStr">
         <is>
@@ -9080,11 +9185,11 @@
     <row r="182">
       <c r="A182" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:usefulLife:1</t>
+          <t xml:space="preserve">driver-range:projectSalesGrowth:1</t>
         </is>
       </c>
       <c r="B182" s="2">
-        <v>20</v>
+        <v>0.3</v>
       </c>
       <c r="C182" s="0" t="inlineStr">
         <is>
@@ -9095,11 +9200,11 @@
     <row r="183">
       <c r="A183" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:investment</t>
+          <t xml:space="preserve">driver-range:projectSalesGrowthToBase:0</t>
         </is>
       </c>
       <c r="B183" s="2">
-        <v>23</v>
+        <v>0.051169590643274754</v>
       </c>
       <c r="C183" s="0" t="inlineStr">
         <is>
@@ -9110,11 +9215,11 @@
     <row r="184">
       <c r="A184" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:localBenchmark</t>
+          <t xml:space="preserve">driver-range:projectSalesGrowthToBase:1</t>
         </is>
       </c>
       <c r="B184" s="2">
-        <v>23</v>
+        <v>0.05701754385964919</v>
       </c>
       <c r="C184" s="0" t="inlineStr">
         <is>
@@ -9125,22 +9230,22 @@
     <row r="185">
       <c r="A185" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherCogsImprovement</t>
+          <t xml:space="preserve">driver-range:projectSgaImprovementToBase:0</t>
         </is>
       </c>
       <c r="B185" s="2">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="C185" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherCogsImprovementToBase</t>
+          <t xml:space="preserve">driver-range:projectSgaImprovementToBase:1</t>
         </is>
       </c>
       <c r="B186" s="2">
@@ -9155,11 +9260,11 @@
     <row r="187">
       <c r="A187" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherHeadcountGrowth</t>
+          <t xml:space="preserve">driver-range:projectSgaRateEnd:0</t>
         </is>
       </c>
       <c r="B187" s="2">
-        <v>0.045833333333333386</v>
+        <v>0.08499999999999999</v>
       </c>
       <c r="C187" s="0" t="inlineStr">
         <is>
@@ -9170,11 +9275,11 @@
     <row r="188">
       <c r="A188" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherHeadcountGrowthToBase</t>
+          <t xml:space="preserve">driver-range:projectSgaRateEnd:1</t>
         </is>
       </c>
       <c r="B188" s="2">
-        <v>0.04083333333333339</v>
+        <v>0.135</v>
       </c>
       <c r="C188" s="0" t="inlineStr">
         <is>
@@ -9185,11 +9290,11 @@
     <row r="189">
       <c r="A189" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherPayGrowth</t>
+          <t xml:space="preserve">driver-range:subsidy:0</t>
         </is>
       </c>
       <c r="B189" s="2">
-        <v>0.02484645846924027</v>
+        <v>1</v>
       </c>
       <c r="C189" s="0" t="inlineStr">
         <is>
@@ -9200,11 +9305,11 @@
     <row r="190">
       <c r="A190" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherPayGrowthToBase</t>
+          <t xml:space="preserve">driver-range:subsidy:1</t>
         </is>
       </c>
       <c r="B190" s="2">
-        <v>0.01984645846924027</v>
+        <v>50</v>
       </c>
       <c r="C190" s="0" t="inlineStr">
         <is>
@@ -9215,11 +9320,11 @@
     <row r="191">
       <c r="A191" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSalesGrowth</t>
+          <t xml:space="preserve">driver-range:usefulLife:0</t>
         </is>
       </c>
       <c r="B191" s="2">
-        <v>0.06257246376811586</v>
+        <v>5</v>
       </c>
       <c r="C191" s="0" t="inlineStr">
         <is>
@@ -9230,11 +9335,11 @@
     <row r="192">
       <c r="A192" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSalesGrowthToBase</t>
+          <t xml:space="preserve">driver-range:usefulLife:1</t>
         </is>
       </c>
       <c r="B192" s="2">
-        <v>0.042572463768115854</v>
+        <v>20</v>
       </c>
       <c r="C192" s="0" t="inlineStr">
         <is>
@@ -9245,26 +9350,26 @@
     <row r="193">
       <c r="A193" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSgaImprovementToBase</t>
+          <t xml:space="preserve">driver:effectiveTaxRate</t>
         </is>
       </c>
       <c r="B193" s="2">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="C193" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSgaRateEnd</t>
+          <t xml:space="preserve">driver:investment</t>
         </is>
       </c>
       <c r="B194" s="2">
-        <v>0.10928571428571428</v>
+        <v>23</v>
       </c>
       <c r="C194" s="0" t="inlineStr">
         <is>
@@ -9275,11 +9380,11 @@
     <row r="195">
       <c r="A195" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectCogsImprovementAfterBase</t>
+          <t xml:space="preserve">driver:localBenchmark</t>
         </is>
       </c>
       <c r="B195" s="2">
-        <v>0.015</v>
+        <v>23</v>
       </c>
       <c r="C195" s="0" t="inlineStr">
         <is>
@@ -9290,11 +9395,11 @@
     <row r="196">
       <c r="A196" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectCogsImprovementToBase</t>
+          <t xml:space="preserve">driver:otherCogsImprovement</t>
         </is>
       </c>
       <c r="B196" s="2">
-        <v>5.551115123125783e-17</v>
+        <v>0.005</v>
       </c>
       <c r="C196" s="0" t="inlineStr">
         <is>
@@ -9305,26 +9410,26 @@
     <row r="197">
       <c r="A197" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectHeadcountGrowth</t>
+          <t xml:space="preserve">driver:otherCogsImprovementToBase</t>
         </is>
       </c>
       <c r="B197" s="2">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="C197" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectHeadcountGrowthToBase</t>
+          <t xml:space="preserve">driver:otherCogsRateWhenSalesZero</t>
         </is>
       </c>
       <c r="B198" s="2">
-        <v>0.05409356725146197</v>
+        <v>0.68</v>
       </c>
       <c r="C198" s="0" t="inlineStr">
         <is>
@@ -9335,11 +9440,11 @@
     <row r="199">
       <c r="A199" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectMarketGrowth</t>
+          <t xml:space="preserve">driver:otherHeadcountGrowth</t>
         </is>
       </c>
       <c r="B199" s="2">
-        <v>0.05</v>
+        <v>0.045833333333333386</v>
       </c>
       <c r="C199" s="0" t="inlineStr">
         <is>
@@ -9350,11 +9455,11 @@
     <row r="200">
       <c r="A200" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectOfficerPayGrowth</t>
+          <t xml:space="preserve">driver:otherHeadcountGrowthToBase</t>
         </is>
       </c>
       <c r="B200" s="2">
-        <v>0.05380116959064325</v>
+        <v>0.04083333333333339</v>
       </c>
       <c r="C200" s="0" t="inlineStr">
         <is>
@@ -9365,11 +9470,11 @@
     <row r="201">
       <c r="A201" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectOfficerPayGrowthToBase</t>
+          <t xml:space="preserve">driver:otherOfficerPayGrowth</t>
         </is>
       </c>
       <c r="B201" s="2">
-        <v>0.05409356725146197</v>
+        <v>0.045</v>
       </c>
       <c r="C201" s="0" t="inlineStr">
         <is>
@@ -9380,11 +9485,11 @@
     <row r="202">
       <c r="A202" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectPayGrowth</t>
+          <t xml:space="preserve">driver:otherOfficerPayGrowthToBase</t>
         </is>
       </c>
       <c r="B202" s="2">
-        <v>0.07</v>
+        <v>0.04</v>
       </c>
       <c r="C202" s="0" t="inlineStr">
         <is>
@@ -9395,11 +9500,11 @@
     <row r="203">
       <c r="A203" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectPayGrowthToBase</t>
+          <t xml:space="preserve">driver:otherPayGrowth</t>
         </is>
       </c>
       <c r="B203" s="2">
-        <v>0.020030662342518046</v>
+        <v>0.02484645846924027</v>
       </c>
       <c r="C203" s="0" t="inlineStr">
         <is>
@@ -9410,11 +9515,11 @@
     <row r="204">
       <c r="A204" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSalesGrowth</t>
+          <t xml:space="preserve">driver:otherPayGrowthToBase</t>
         </is>
       </c>
       <c r="B204" s="2">
-        <v>0.22</v>
+        <v>0.01984645846924027</v>
       </c>
       <c r="C204" s="0" t="inlineStr">
         <is>
@@ -9425,11 +9530,11 @@
     <row r="205">
       <c r="A205" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSalesGrowthToBase</t>
+          <t xml:space="preserve">driver:otherSalesGrowth</t>
         </is>
       </c>
       <c r="B205" s="2">
-        <v>0.05409356725146197</v>
+        <v>0.06257246376811586</v>
       </c>
       <c r="C205" s="0" t="inlineStr">
         <is>
@@ -9440,41 +9545,41 @@
     <row r="206">
       <c r="A206" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSgaImprovementToBase</t>
+          <t xml:space="preserve">driver:otherSalesGrowthToBase</t>
         </is>
       </c>
       <c r="B206" s="2">
-        <v>0</v>
+        <v>0.042572463768115854</v>
       </c>
       <c r="C206" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSgaRateEnd</t>
+          <t xml:space="preserve">driver:otherSgaImprovementToBase</t>
         </is>
       </c>
       <c r="B207" s="2">
-        <v>0.11</v>
+        <v>0</v>
       </c>
       <c r="C207" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:subsidy</t>
+          <t xml:space="preserve">driver:otherSgaRateEnd</t>
         </is>
       </c>
       <c r="B208" s="2">
-        <v>7.66</v>
+        <v>0.10928571428571428</v>
       </c>
       <c r="C208" s="0" t="inlineStr">
         <is>
@@ -9485,11 +9590,11 @@
     <row r="209">
       <c r="A209" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:usefulLife</t>
+          <t xml:space="preserve">driver:projectCogsImprovementAfterBase</t>
         </is>
       </c>
       <c r="B209" s="2">
-        <v>10</v>
+        <v>0.015</v>
       </c>
       <c r="C209" s="0" t="inlineStr">
         <is>
@@ -9500,11 +9605,11 @@
     <row r="210">
       <c r="A210" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2026</t>
+          <t xml:space="preserve">driver:projectCogsImprovementToBase</t>
         </is>
       </c>
       <c r="B210" s="2">
-        <v>15</v>
+        <v>5.551115123125783e-17</v>
       </c>
       <c r="C210" s="0" t="inlineStr">
         <is>
@@ -9515,11 +9620,11 @@
     <row r="211">
       <c r="A211" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2027</t>
+          <t xml:space="preserve">driver:projectCogsRateWhenSalesZero</t>
         </is>
       </c>
       <c r="B211" s="2">
-        <v>15</v>
+        <v>0.68</v>
       </c>
       <c r="C211" s="0" t="inlineStr">
         <is>
@@ -9530,11 +9635,11 @@
     <row r="212">
       <c r="A212" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2028</t>
+          <t xml:space="preserve">driver:projectHeadcountGrowth</t>
         </is>
       </c>
       <c r="B212" s="2">
-        <v>15</v>
+        <v>0.04</v>
       </c>
       <c r="C212" s="0" t="inlineStr">
         <is>
@@ -9545,56 +9650,56 @@
     <row r="213">
       <c r="A213" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2029</t>
+          <t xml:space="preserve">driver:projectHeadcountGrowthToBase</t>
         </is>
       </c>
       <c r="B213" s="2">
-        <v>0</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="C213" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2030</t>
+          <t xml:space="preserve">driver:projectMarketGrowth</t>
         </is>
       </c>
       <c r="B214" s="2">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="C214" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2031</t>
+          <t xml:space="preserve">driver:projectOfficerPayGrowth</t>
         </is>
       </c>
       <c r="B215" s="2">
-        <v>0</v>
+        <v>0.05380116959064325</v>
       </c>
       <c r="C215" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companyPaySchedule:max</t>
+          <t xml:space="preserve">driver:projectOfficerPayGrowthToBase</t>
         </is>
       </c>
       <c r="B216" s="2">
-        <v>7</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="C216" s="0" t="inlineStr">
         <is>
@@ -9605,11 +9710,11 @@
     <row r="217">
       <c r="A217" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companyPaySchedule:value</t>
+          <t xml:space="preserve">driver:projectPayGrowth</t>
         </is>
       </c>
       <c r="B217" s="2">
-        <v>2</v>
+        <v>0.07</v>
       </c>
       <c r="C217" s="0" t="inlineStr">
         <is>
@@ -9620,11 +9725,11 @@
     <row r="218">
       <c r="A218" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesCagr:max</t>
+          <t xml:space="preserve">driver:projectPayGrowthToBase</t>
         </is>
       </c>
       <c r="B218" s="2">
-        <v>35</v>
+        <v>0.020030662342518046</v>
       </c>
       <c r="C218" s="0" t="inlineStr">
         <is>
@@ -9635,11 +9740,11 @@
     <row r="219">
       <c r="A219" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesCagr:value</t>
+          <t xml:space="preserve">driver:projectSalesGrowth</t>
         </is>
       </c>
       <c r="B219" s="2">
-        <v>15</v>
+        <v>0.22</v>
       </c>
       <c r="C219" s="0" t="inlineStr">
         <is>
@@ -9650,11 +9755,11 @@
     <row r="220">
       <c r="A220" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesIncrease:max</t>
+          <t xml:space="preserve">driver:projectSalesGrowthToBase</t>
         </is>
       </c>
       <c r="B220" s="2">
-        <v>252.69</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="C220" s="0" t="inlineStr">
         <is>
@@ -9665,26 +9770,26 @@
     <row r="221">
       <c r="A221" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesIncrease:value</t>
+          <t xml:space="preserve">driver:projectSgaImprovementToBase</t>
         </is>
       </c>
       <c r="B221" s="2">
-        <v>82.4</v>
+        <v>0</v>
       </c>
       <c r="C221" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayCagr:max</t>
+          <t xml:space="preserve">driver:projectSgaRateEnd</t>
         </is>
       </c>
       <c r="B222" s="2">
-        <v>10</v>
+        <v>0.11</v>
       </c>
       <c r="C222" s="0" t="inlineStr">
         <is>
@@ -9695,11 +9800,11 @@
     <row r="223">
       <c r="A223" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayCagr:value</t>
+          <t xml:space="preserve">driver:subsidy</t>
         </is>
       </c>
       <c r="B223" s="2">
-        <v>7</v>
+        <v>7.66</v>
       </c>
       <c r="C223" s="0" t="inlineStr">
         <is>
@@ -9710,11 +9815,11 @@
     <row r="224">
       <c r="A224" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayIncrease:max</t>
+          <t xml:space="preserve">driver:usefulLife</t>
         </is>
       </c>
       <c r="B224" s="2">
-        <v>3.74</v>
+        <v>10</v>
       </c>
       <c r="C224" s="0" t="inlineStr">
         <is>
@@ -9725,11 +9830,11 @@
     <row r="225">
       <c r="A225" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayIncrease:value</t>
+          <t xml:space="preserve">future-capex:2026</t>
         </is>
       </c>
       <c r="B225" s="2">
-        <v>2.85</v>
+        <v>7.67</v>
       </c>
       <c r="C225" s="0" t="inlineStr">
         <is>
@@ -9740,11 +9845,11 @@
     <row r="226">
       <c r="A226" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:investmentSalesRatio:max</t>
+          <t xml:space="preserve">future-capex:2027</t>
         </is>
       </c>
       <c r="B226" s="2">
-        <v>70</v>
+        <v>7.67</v>
       </c>
       <c r="C226" s="0" t="inlineStr">
         <is>
@@ -9755,11 +9860,11 @@
     <row r="227">
       <c r="A227" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:investmentSalesRatio:value</t>
+          <t xml:space="preserve">future-capex:2028</t>
         </is>
       </c>
       <c r="B227" s="2">
-        <v>15</v>
+        <v>7.66</v>
       </c>
       <c r="C227" s="0" t="inlineStr">
         <is>
@@ -9770,56 +9875,56 @@
     <row r="228">
       <c r="A228" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:laborProductivityCagr:max</t>
+          <t xml:space="preserve">future-capex:2029</t>
         </is>
       </c>
       <c r="B228" s="2">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="C228" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:laborProductivityCagr:value</t>
+          <t xml:space="preserve">future-capex:2030</t>
         </is>
       </c>
       <c r="B229" s="2">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="C229" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:localBenchmark:max</t>
+          <t xml:space="preserve">future-capex:2031</t>
         </is>
       </c>
       <c r="B230" s="2">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="C230" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:localBenchmark:value</t>
+          <t xml:space="preserve">target:companyPaySchedule:max</t>
         </is>
       </c>
       <c r="B231" s="2">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="C231" s="0" t="inlineStr">
         <is>
@@ -9830,11 +9935,11 @@
     <row r="232">
       <c r="A232" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayCagr:max</t>
+          <t xml:space="preserve">target:companyPaySchedule:value</t>
         </is>
       </c>
       <c r="B232" s="2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C232" s="0" t="inlineStr">
         <is>
@@ -9845,11 +9950,11 @@
     <row r="233">
       <c r="A233" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayCagr:value</t>
+          <t xml:space="preserve">target:companySalesCagr:max</t>
         </is>
       </c>
       <c r="B233" s="2">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="C233" s="0" t="inlineStr">
         <is>
@@ -9860,26 +9965,26 @@
     <row r="234">
       <c r="A234" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayIncrease:value</t>
+          <t xml:space="preserve">target:companySalesCagr:value</t>
         </is>
       </c>
       <c r="B234" s="2">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="C234" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesCagr:max</t>
+          <t xml:space="preserve">target:companySalesIncrease:max</t>
         </is>
       </c>
       <c r="B235" s="2">
-        <v>35</v>
+        <v>252.69</v>
       </c>
       <c r="C235" s="0" t="inlineStr">
         <is>
@@ -9890,11 +9995,11 @@
     <row r="236">
       <c r="A236" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesCagr:value</t>
+          <t xml:space="preserve">target:companySalesIncrease:value</t>
         </is>
       </c>
       <c r="B236" s="2">
-        <v>22</v>
+        <v>82.4</v>
       </c>
       <c r="C236" s="0" t="inlineStr">
         <is>
@@ -9905,11 +10010,11 @@
     <row r="237">
       <c r="A237" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesIncrease:max</t>
+          <t xml:space="preserve">target:employeePayCagr:max</t>
         </is>
       </c>
       <c r="B237" s="2">
-        <v>136.84</v>
+        <v>10</v>
       </c>
       <c r="C237" s="0" t="inlineStr">
         <is>
@@ -9920,11 +10025,11 @@
     <row r="238">
       <c r="A238" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesIncrease:value</t>
+          <t xml:space="preserve">target:employeePayCagr:value</t>
         </is>
       </c>
       <c r="B238" s="2">
-        <v>74.8</v>
+        <v>7</v>
       </c>
       <c r="C238" s="0" t="inlineStr">
         <is>
@@ -9935,11 +10040,11 @@
     <row r="239">
       <c r="A239" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesShare:max</t>
+          <t xml:space="preserve">target:employeePayIncrease:max</t>
         </is>
       </c>
       <c r="B239" s="2">
-        <v>95</v>
+        <v>3.74</v>
       </c>
       <c r="C239" s="0" t="inlineStr">
         <is>
@@ -9950,11 +10055,11 @@
     <row r="240">
       <c r="A240" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesShare:value</t>
+          <t xml:space="preserve">target:employeePayIncrease:value</t>
         </is>
       </c>
       <c r="B240" s="2">
-        <v>60</v>
+        <v>2.85</v>
       </c>
       <c r="C240" s="0" t="inlineStr">
         <is>
@@ -9965,11 +10070,11 @@
     <row r="241">
       <c r="A241" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:valueAddedIncrease:max</t>
+          <t xml:space="preserve">target:investmentSalesRatio:max</t>
         </is>
       </c>
       <c r="B241" s="2">
-        <v>33.43</v>
+        <v>70</v>
       </c>
       <c r="C241" s="0" t="inlineStr">
         <is>
@@ -9980,11 +10085,11 @@
     <row r="242">
       <c r="A242" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:valueAddedIncrease:value</t>
+          <t xml:space="preserve">target:investmentSalesRatio:value</t>
         </is>
       </c>
       <c r="B242" s="2">
-        <v>18.78</v>
+        <v>15</v>
       </c>
       <c r="C242" s="0" t="inlineStr">
         <is>
@@ -9995,11 +10100,11 @@
     <row r="243">
       <c r="A243" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:valueAddedSubsidyRatio:max</t>
+          <t xml:space="preserve">target:laborProductivityCagr:max</t>
         </is>
       </c>
       <c r="B243" s="2">
-        <v>350</v>
+        <v>35</v>
       </c>
       <c r="C243" s="0" t="inlineStr">
         <is>
@@ -10010,13 +10115,238 @@
     <row r="244">
       <c r="A244" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">target:laborProductivityCagr:value</t>
+        </is>
+      </c>
+      <c r="B244" s="2">
+        <v>21</v>
+      </c>
+      <c r="C244" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:localBenchmark:max</t>
+        </is>
+      </c>
+      <c r="B245" s="2">
+        <v>40</v>
+      </c>
+      <c r="C245" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:localBenchmark:value</t>
+        </is>
+      </c>
+      <c r="B246" s="2">
+        <v>23</v>
+      </c>
+      <c r="C246" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:officerPayCagr:max</t>
+        </is>
+      </c>
+      <c r="B247" s="2">
+        <v>10</v>
+      </c>
+      <c r="C247" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:officerPayCagr:value</t>
+        </is>
+      </c>
+      <c r="B248" s="2">
+        <v>6</v>
+      </c>
+      <c r="C248" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:officerPayIncrease:value</t>
+        </is>
+      </c>
+      <c r="B249" s="2">
+        <v>0</v>
+      </c>
+      <c r="C249" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesCagr:max</t>
+        </is>
+      </c>
+      <c r="B250" s="2">
+        <v>35</v>
+      </c>
+      <c r="C250" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesCagr:value</t>
+        </is>
+      </c>
+      <c r="B251" s="2">
+        <v>22</v>
+      </c>
+      <c r="C251" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesIncrease:max</t>
+        </is>
+      </c>
+      <c r="B252" s="2">
+        <v>136.84</v>
+      </c>
+      <c r="C252" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesIncrease:value</t>
+        </is>
+      </c>
+      <c r="B253" s="2">
+        <v>74.8</v>
+      </c>
+      <c r="C253" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesShare:max</t>
+        </is>
+      </c>
+      <c r="B254" s="2">
+        <v>95</v>
+      </c>
+      <c r="C254" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesShare:value</t>
+        </is>
+      </c>
+      <c r="B255" s="2">
+        <v>60</v>
+      </c>
+      <c r="C255" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:valueAddedIncrease:max</t>
+        </is>
+      </c>
+      <c r="B256" s="2">
+        <v>33.43</v>
+      </c>
+      <c r="C256" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:valueAddedIncrease:value</t>
+        </is>
+      </c>
+      <c r="B257" s="2">
+        <v>18.78</v>
+      </c>
+      <c r="C257" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:valueAddedSubsidyRatio:max</t>
+        </is>
+      </c>
+      <c r="B258" s="2">
+        <v>350</v>
+      </c>
+      <c r="C258" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">target:valueAddedSubsidyRatio:value</t>
         </is>
       </c>
-      <c r="B244" s="2">
+      <c r="B259" s="2">
         <v>213</v>
       </c>
-      <c r="C244" s="0" t="inlineStr">
+      <c r="C259" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">入力済み</t>
         </is>
@@ -10044,7 +10374,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4LCJvcmRpbmFyeUluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsInByZVRheEluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsIm5ldEluY29tZSI6Mi43NjQwMDAwMDAwMDAwMDJ9fSx7InllYXIiOjIwMjQsInJvbGUiOiJwcmV2aW91cyIsInByb2plY3QiOnsic2FsZXMiOjc2LCJjb2dzIjo1MS42OCwiZW1wbG95ZWVQYXkiOjUuNTksIm9mZmljZXJQYXkiOjAuMzgsImRlcHJlY2lhdGlvbiI6MS45LCJvdGhlclNnYSI6OS41LCJoZWFkY291bnQiOjk1LCJvZmZpY2VyQ291bnQiOjIsImVtcGxveWVlU2FsYXJ5Ijo1LjMxLCJlbXBsb3llZUJvbnVzIjowLjI4LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjM0LCJvZmZpY2VyQm9udXMiOjAuMDQsImNvZ3NEZXByZWNpYXRpb24iOjAuNDcsInNnYURlcHJlY2lhdGlvbiI6MS40MywicmVzZWFyY2hEZXZlbG9wbWVudCI6MC4zOH0sIm90aGVyIjp7InNhbGVzIjo2Ny4yLCJjb2dzIjo0NS43LCJlbXBsb3llZVBheSI6Ny41NCwib2ZmaWNlclBheSI6MC41OCwiZGVwcmVjaWF0aW9uIjoxLjQ0LCJvdGhlclNnYSI6Ny42OCwiaGVhZGNvdW50IjoxMjUsIm9mZmljZXJDb3VudCI6MywiZW1wbG95ZWVTYWxhcnkiOjcuMTYsImVtcGxveWVlQm9udXMiOjAuMzgsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTIsIm9mZmljZXJCb251cyI6MC4wNiwiY29nc0RlcHJlY2lhdGlvbiI6MC4yOSwic2dhRGVwcmVjaWF0aW9uIjoxLjE1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI5LCJvcmRpbmFyeUluY29tZSI6My45Njk5OTk5OTk5OTk5OTcsInByZVRheEluY29tZSI6My45Njk5OTk5OTk5OTk5OTcsIm5ldEluY29tZSI6Mi43ODE5OTk5OTk5OTk5OTgzfX0seyJ5ZWFyIjoyMDI1LCJyb2xlIjoibGF0ZXN0IiwicHJvamVjdCI6eyJzYWxlcyI6ODAsImNvZ3MiOjU0LjQsImVtcGxveWVlUGF5Ijo2LCJlbXBsb3llZVNhbGFyeSI6NS43LCJlbXBsb3llZUJvbnVzIjowLjMsIm9mZmljZXJQYXkiOjAuNCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNiwib2ZmaWNlckJvbnVzIjowLjA0LCJkZXByZWNpYXRpb24iOjIsImNvZ3NEZXByZWNpYXRpb24iOjAuNSwic2dhRGVwcmVjaWF0aW9uIjoxLjUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuNCwib3RoZXJTZ2EiOjEwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwLCJjb2dzIjo0Ny42LCJlbXBsb3llZVBheSI6OCwiZW1wbG95ZWVTYWxhcnkiOjcuNiwiZW1wbG95ZWVCb251cyI6MC40LCJvZmZpY2VyUGF5IjowLjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTQsIm9mZmljZXJCb251cyI6MC4wNiwiZGVwcmVjaWF0aW9uIjoxLjUsImNvZ3NEZXByZWNpYXRpb24iOjAuMywic2dhRGVwcmVjaWF0aW9uIjoxLjIsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMywib3RoZXJTZ2EiOjgsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjozLjk5OTk5OTk5OTk5OTk5NjQsInByZVRheEluY29tZSI6My45OTk5OTk5OTk5OTk5OTY0LCJuZXRJbmNvbWUiOjIuNzk5OTk5OTk5OTk5OTk3fX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjoxNX0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MTV9LHsieWVhciI6MjAyOCwidmFsdWUiOjE1fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMSwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI4NTcxNDI4NTcxNDI4LCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwidXNlZnVsTGlmZSI6MTAsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwxLjY2NTMzNDUzNjkzNzczNDhlLTE2XSwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MzI1MzMwNTAxODQ2OTI3LDAuMDIwNzM1OTk0MTgzMTg5MTY2XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDBdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNDA3NjA4Njk1NjUyMTcxODQsMC4wNDQzODQwNTc5NzEwMTQ1Ml0sIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAwMDEzNDU3NTU2OTM1ODE5NzM3XSwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOlswLjAxOTEzOTQ1NzAyMzcxNzQ0MywwLjAyMDU1MzQ1OTkxNDc2MzA5NV0sIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wMzkxNjY2NjY2NjY2NjY2OCwwLjA0MjUwMDAwMDAwMDAwMDA5XSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RTYWxlc0dyb3d0aCI6WzAuMTUsMC4zXSwib3RoZXJTYWxlc0dyb3d0aCI6WzAuMDYwNzYwODY5NTY1MjE3MTksMC4wNjQzODQwNTc5NzEwMTQ1M10sInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOlswLDAuMDNdLCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6WzAuMDA1LDAuMDA1MTM0NTc1NTY5MzU4MTk3NV0sInByb2plY3RQYXlHcm93dGgiOlswLjA1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMC4wMjQxMzk0NTcwMjM3MTc0NDQsMC4wMjU1NTM0NTk5MTQ3NjMwOTZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGgiOlswLjA0NDE2NjY2NjY2NjY2NjY4LDAuMDQ3NTAwMDAwMDAwMDAwMDldLCJwcm9qZWN0U2dhUmF0ZUVuZCI6WzAuMDg0OTk5OTk5OTk5OTk5OTksMC4xMzVdLCJvdGhlclNnYVJhdGVFbmQiOlswLjA4OTI4NTcxNDI4NTcxNDI3LDAuMTE5Mjg1NzE0Mjg1NzE0MjddLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAuMDQyNjMxNTc4OTQ3MzY4MzYsMC4wNjU1NTU1NTU1NTU1NTU1OF0sInVzZWZ1bExpZmUiOls1LDIwXSwiaW52ZXN0bWVudCI6WzE1LDIwMF0sInN1YnNpZHkiOlsxLDUwXSwibG9jYWxCZW5jaG1hcmsiOlswLDEwMF19LCJ0YXJnZXRzIjp7ImNvbXBhbnlTYWxlc0NhZ3IiOnsidmFsdWUiOjE1LCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjgyLjQsIm1heCI6MjUyLjY5LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjoyLCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NjAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo3NC44LCJtYXgiOjEzNi44NCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImxhYm9yUHJvZHVjdGl2aXR5Q2FnciI6eyJ2YWx1ZSI6MjEsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkSW5jcmVhc2UiOnsidmFsdWUiOjE4Ljc4LCJtYXgiOjMzLjQzLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6Mi44NSwibWF4IjozLjc0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiaW52ZXN0bWVudFNhbGVzUmF0aW8iOnsidmFsdWUiOjE1LCJtYXgiOjcwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZFN1YnNpZHlSYXRpbyI6eyJ2YWx1ZSI6MjEzLCJtYXgiOjM1MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImxvY2FsQmVuY2htYXJrIjp7InZhbHVlIjoyMywibWF4Ijo0MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlDYWdyIjp7InZhbHVlIjo2LCJtYXgiOjEwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUluY3JlYXNlIjp7InZhbHVlIjowLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfX0sImZvcmVjYXN0T3ZlcnJpZGVzIjp7IjIwMjk6b3RoZXI6c2FsZXMiOjg1LjEzLCIyMDI5OnByb2plY3Q6Ny04Ijo3Ljl9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2LjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mi43NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTQiOjAuNzMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi03IjozMi42NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTkiOjAuODIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMCI6MC4wOSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEyIjoxMS42NywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEzIjowLjYyLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTQiOjIuNDUsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNSI6MC42NCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE4IjoxMC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE5IjoxMC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTIwIjo3LjUxLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjciOjIxMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMSI6NzIsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny00IjoyMy4wNCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjYuNzgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny04Ijo1LjE5LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOSI6MC4zNiwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEwIjoxLjgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMyI6OTAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEiOjE0My4yLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMyI6OTcuMzgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi00IjowLjc2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNyI6MzQuNTIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi05IjowLjg2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEyIjoxMi40NywiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEzIjowLjY2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTQiOjIuNTgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNSI6MC42NywiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE4IjoxMS4wMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE5IjoxMS4wMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTIwIjo3LjcxLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjciOjIyMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMSI6NzYsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny00IjoyNC4zMiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTYiOjcuMDQsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny04Ijo1LjU5LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctOSI6MC4zOCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEwIjoxLjksImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xMyI6OTUsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEiOjE1MCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTMiOjEwMiwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTQiOjAuOCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTciOjM2LjQsImFjdHVhbDpjb21wYW55OjIwMjU6Mi05IjowLjksImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMCI6MC4xLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTIiOjEzLjMsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMyI6MC43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTQiOjIuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE1IjowLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xOCI6MTEuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE5IjoxMS4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjAiOjcuOTEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yNyI6MjMwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xIjo4MCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTQiOjI1LjYsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny02Ijo3LjMsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny04Ijo2LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOSI6MC40LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTAiOjIsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xMyI6MTAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTQiOjIsImJhbGFuY2Utc2hlZXQ6MjAyMzphc3NldHMiOjEzMiwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRBc3NldHMiOjY3LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FzaCI6MjQsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZEFzc2V0cyI6NjUsImJhbGFuY2Utc2hlZXQ6MjAyMzp0YW5naWJsZUFzc2V0cyI6NTMsImJhbGFuY2Utc2hlZXQ6MjAyMzpidWlsZGluZ3MiOjE5LCJiYWxhbmNlLXNoZWV0OjIwMjM6bWFjaGluZXJ5IjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmxhbmQiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjM6aW50YW5naWJsZUFzc2V0cyI6NywiYmFsYW5jZS1zaGVldDoyMDIzOnNvZnR3YXJlIjo1LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGlhYmlsaXRpZXMiOjc1LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudExpYWJpbGl0aWVzIjozOSwiYmFsYW5jZS1zaGVldDoyMDIzOnNob3J0VGVybURlYnQiOjEyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRMaWFiaWxpdGllcyI6MzYsImJhbGFuY2Utc2hlZXQ6MjAyMzpsb25nVGVybURlYnQiOjI5LCJiYWxhbmNlLXNoZWV0OjIwMjM6bmV0QXNzZXRzIjo1NywiYmFsYW5jZS1zaGVldDoyMDIzOnNoYXJlaG9sZGVyRXF1aXR5Ijo1NCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGl0YWwiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwZXgiOjUsImJhbGFuY2Utc2hlZXQ6MjAyNDphc3NldHMiOjE0MywiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRBc3NldHMiOjcyLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FzaCI6MjUsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZEFzc2V0cyI6NzEsImJhbGFuY2Utc2hlZXQ6MjAyNDp0YW5naWJsZUFzc2V0cyI6NTgsImJhbGFuY2Utc2hlZXQ6MjAyNDpidWlsZGluZ3MiOjIwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bWFjaGluZXJ5IjoyOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxhbmQiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6aW50YW5naWJsZUFzc2V0cyI6OCwiYmFsYW5jZS1zaGVldDoyMDI0OnNvZnR3YXJlIjo2LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGlhYmlsaXRpZXMiOjc5LCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudExpYWJpbGl0aWVzIjo0MSwiYmFsYW5jZS1zaGVldDoyMDI0OnNob3J0VGVybURlYnQiOjEyLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRMaWFiaWxpdGllcyI6MzgsImJhbGFuY2Utc2hlZXQ6MjAyNDpsb25nVGVybURlYnQiOjMxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bmV0QXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI0OnNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGl0YWwiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwZXgiOjgsImJhbGFuY2Utc2hlZXQ6MjAyNTphc3NldHMiOjE1NiwiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRBc3NldHMiOjc4LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FzaCI6MjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTp0YW5naWJsZUFzc2V0cyI6NjQsImJhbGFuY2Utc2hlZXQ6MjAyNTpidWlsZGluZ3MiOjIyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bWFjaGluZXJ5IjozMiwiYmFsYW5jZS1zaGVldDoyMDI1OmxhbmQiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjU6aW50YW5naWJsZUFzc2V0cyI6OSwiYmFsYW5jZS1zaGVldDoyMDI1OnNvZnR3YXJlIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjU6bGlhYmlsaXRpZXMiOjgzLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudExpYWJpbGl0aWVzIjo0MywiYmFsYW5jZS1zaGVldDoyMDI1OnNob3J0VGVybURlYnQiOjExLCJiYWxhbmNlLXNoZWV0OjIwMjU6Zml4ZWRMaWFiaWxpdGllcyI6NDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpsb25nVGVybURlYnQiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bmV0QXNzZXRzIjo3MywiYmFsYW5jZS1zaGVldDoyMDI1OnNoYXJlaG9sZGVyRXF1aXR5Ijo3MCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGl0YWwiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwZXgiOjEwLCJmdXR1cmUtY2FwZXg6MjAyNiI6MTUsImZ1dHVyZS1jYXBleDoyMDI3IjoxNSwiZnV0dXJlLWNhcGV4OjIwMjgiOjE1LCJmdXR1cmUtY2FwZXg6MjAyOSI6MCwiZnV0dXJlLWNhcGV4OjIwMzAiOjAsImZ1dHVyZS1jYXBleDoyMDMxIjowLCJkcml2ZXI6cHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MCI6LTAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjEiOjAuMywiZHJpdmVyOnByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aFRvQmFzZToxIjowLjA1NzAxNzU0Mzg1OTY0OTE5LCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6NS41NTExMTUxMjMxMjU3ODNlLTE3LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjoxLjY2NTMzNDUzNjkzNzczNDhlLTE2LCJkcml2ZXI6cHJvamVjdFBheUdyb3d0aFRvQmFzZSI6MC4wMjAwMzA2NjIzNDI1MTgwNDYsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDE5MzI1MzMwNTAxODQ2OTI3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZToxIjowLjAyMDczNTk5NDE4MzE4OTE2NiwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZToxIjowLjA1NzAxNzU0Mzg1OTY0OTE5LCJkcml2ZXI6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MCwiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZToxIjowLjA1NzAxNzU0Mzg1OTY0OTE5LCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI1NzI0NjM3NjgxMTU4NTQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjAiOjAuMDQwNzYwODY5NTY1MjE3MTg0LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZToxIjowLjA0NDM4NDA1Nzk3MTAxNDUyLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMDAxMzQ1NzU1NjkzNTgxOTczNywiZHJpdmVyOm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkxMzk0NTcwMjM3MTc0NDMsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZToxIjowLjAyMDU1MzQ1OTkxNDc2MzA5NSwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wMzkxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDQyNTAwMDAwMDAwMDAwMDksImRyaXZlcjpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjAiOjAuMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MSI6MC4zLCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NzI0NjM3NjgxMTU4NiwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MCI6MC4wNjA3NjA4Njk1NjUyMTcxOSwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MSI6MC4wNjQzODQwNTc5NzEwMTQ1MywiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZToxIjowLjAzLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDoxIjowLjAwNTEzNDU3NTU2OTM1ODE5NzUsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDowIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDoxIjowLjEsImRyaXZlcjpvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjAiOjAuMDI0MTM5NDU3MDIzNzE3NDQ0LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wMjU1NTM0NTk5MTQ3NjMwOTYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjA0LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aDowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aDoxIjowLjA4LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MCI6MC4wNDQxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjEiOjAuMDQ3NTAwMDAwMDAwMDAwMDksImRyaXZlcjpwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjAiOjAuMDg0OTk5OTk5OTk5OTk5OTksImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDoxIjowLjEzNSwiZHJpdmVyOm90aGVyU2dhUmF0ZUVuZCI6MC4xMDkyODU3MTQyODU3MTQyOCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLjA4OTI4NTcxNDI4NTcxNDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMTE5Mjg1NzE0Mjg1NzE0MjcsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAuMDQyNjMxNTc4OTQ3MzY4MzYsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjA2NTU1NTU1NTU1NTU1NTU4LCJkcml2ZXI6dXNlZnVsTGlmZSI6MTAsImRyaXZlci1yYW5nZTp1c2VmdWxMaWZlOjAiOjUsImRyaXZlci1yYW5nZTp1c2VmdWxMaWZlOjEiOjIwLCJkcml2ZXI6aW52ZXN0bWVudCI6MjMsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjAiOjE1LCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDoxIjoyMDAsImRyaXZlcjpzdWJzaWR5Ijo3LjY2LCJkcml2ZXItcmFuZ2U6c3Vic2lkeTowIjoxLCJkcml2ZXItcmFuZ2U6c3Vic2lkeToxIjo1MCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoxNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjo4Mi40LCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjoyLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOm1heCI6NywidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOnZhbHVlIjo2MCwidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOm1heCI6OTUsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOnZhbHVlIjoyMiwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOnZhbHVlIjo3NC44LCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOnZhbHVlIjoyMSwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2FncjptYXgiOjM1LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOnZhbHVlIjoxOC43OCwidGFyZ2V0OmVtcGxveWVlUGF5Q2Fncjp2YWx1ZSI6NywidGFyZ2V0OmVtcGxveWVlUGF5Q2FncjptYXgiOjEwLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlJbmNyZWFzZTp2YWx1ZSI6Mi44NSwidGFyZ2V0OmludmVzdG1lbnRTYWxlc1JhdGlvOnZhbHVlIjoxNSwidGFyZ2V0OmludmVzdG1lbnRTYWxlc1JhdGlvOm1heCI6NzAsInRhcmdldDp2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvOnZhbHVlIjoyMTMsInRhcmdldDp2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvOm1heCI6MzUwLCJ0YXJnZXQ6bG9jYWxCZW5jaG1hcms6dmFsdWUiOjIzLCJ0YXJnZXQ6bG9jYWxCZW5jaG1hcms6bWF4Ijo0MCwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOnZhbHVlIjo2LCJ0YXJnZXQ6b2ZmaWNlclBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0Om9mZmljZXJQYXlJbmNyZWFzZTp2YWx1ZSI6MCwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOm1heCI6MjUyLjY5LCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6bWF4IjoxMzYuODQsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6bWF4IjozMy40MywidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6bWF4IjozLjc0fSwibWV0cmljR3JvdXBCYXNlcyI6eyJjb21wYW55U2FsZXMiOiJyYXRlIiwicHJvamVjdFNhbGVzIjoicmF0ZSIsImxhYm9yUHJvZHVjdGl2aXR5IjoicmF0ZSIsImVtcGxveWVlUGF5IjoicmF0ZSJ9LCJhcHBsaWNhdGlvbkNhdGVnb3J5IjoiZ2VuZXJhbCIsImFkanVzdGVkRHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MTA1OTU3NjAyMzM5MTYsInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjEuMTc0MTg2NDkxMDY0NDY2ZS0xNiwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6MC4wMTk5ODIxMzU1MTE4Nzk4NzMsInByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDU0MDYzOTAxMjQ5NzIyOTM0LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDEyMDQ1MTMzMzE1NzYzLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjYwNTUxNjI3MzAwNTI3LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODgxMzY3NTAwOTE3MTE3LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA2MDkzNTM5NDM3MTc4NTUsIm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMjAyMjQ4NzIxNjk0NjY3Mywib3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NjUxNzg1OTQ1MjE3OSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTQ5OTA0ODEzNDEyNjU1NSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA4OTAwNjIyOTk3NTA4MDEsIm90aGVyUGF5R3Jvd3RoIjowLjAyNDg4Nzc2MTcxMDMzMzAzLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjAyOTA0NTQ4MjM5NzIwNTA1NSwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1Nzg0ODE0NzMyMzA4NjY1LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMDk5MzE4MDkxNjQ4NDgyNCwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTI3MjU4OTg3MjEyODIzLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM3NzgwNTc2Mjg3MTYzMiwidXNlZnVsTGlmZSI6MTAsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9fQ==</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4LCJvcmRpbmFyeUluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsInByZVRheEluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsIm5ldEluY29tZSI6Mi43NjQwMDAwMDAwMDAwMDJ9fSx7InllYXIiOjIwMjQsInJvbGUiOiJwcmV2aW91cyIsInByb2plY3QiOnsic2FsZXMiOjc2LCJjb2dzIjo1MS42OCwiZW1wbG95ZWVQYXkiOjUuNTksIm9mZmljZXJQYXkiOjAuMzgsImRlcHJlY2lhdGlvbiI6MS45LCJvdGhlclNnYSI6OS41LCJoZWFkY291bnQiOjk1LCJvZmZpY2VyQ291bnQiOjIsImVtcGxveWVlU2FsYXJ5Ijo1LjMxLCJlbXBsb3llZUJvbnVzIjowLjI4LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjM0LCJvZmZpY2VyQm9udXMiOjAuMDQsImNvZ3NEZXByZWNpYXRpb24iOjAuNDcsInNnYURlcHJlY2lhdGlvbiI6MS40MywicmVzZWFyY2hEZXZlbG9wbWVudCI6MC4zOH0sIm90aGVyIjp7InNhbGVzIjo2Ny4yLCJjb2dzIjo0NS43LCJlbXBsb3llZVBheSI6Ny41NCwib2ZmaWNlclBheSI6MC41OCwiZGVwcmVjaWF0aW9uIjoxLjQ0LCJvdGhlclNnYSI6Ny42OCwiaGVhZGNvdW50IjoxMjUsIm9mZmljZXJDb3VudCI6MywiZW1wbG95ZWVTYWxhcnkiOjcuMTYsImVtcGxveWVlQm9udXMiOjAuMzgsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTIsIm9mZmljZXJCb251cyI6MC4wNiwiY29nc0RlcHJlY2lhdGlvbiI6MC4yOSwic2dhRGVwcmVjaWF0aW9uIjoxLjE1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI5LCJvcmRpbmFyeUluY29tZSI6My45Njk5OTk5OTk5OTk5OTcsInByZVRheEluY29tZSI6My45Njk5OTk5OTk5OTk5OTcsIm5ldEluY29tZSI6Mi43ODE5OTk5OTk5OTk5OTgzfX0seyJ5ZWFyIjoyMDI1LCJyb2xlIjoibGF0ZXN0IiwicHJvamVjdCI6eyJzYWxlcyI6ODAsImNvZ3MiOjU0LjQsImVtcGxveWVlUGF5Ijo2LCJlbXBsb3llZVNhbGFyeSI6NS43LCJlbXBsb3llZUJvbnVzIjowLjMsIm9mZmljZXJQYXkiOjAuNCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNiwib2ZmaWNlckJvbnVzIjowLjA0LCJkZXByZWNpYXRpb24iOjIsImNvZ3NEZXByZWNpYXRpb24iOjAuNSwic2dhRGVwcmVjaWF0aW9uIjoxLjUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuNCwib3RoZXJTZ2EiOjEwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwLCJjb2dzIjo0Ny42LCJlbXBsb3llZVBheSI6OCwiZW1wbG95ZWVTYWxhcnkiOjcuNiwiZW1wbG95ZWVCb251cyI6MC40LCJvZmZpY2VyUGF5IjowLjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTQsIm9mZmljZXJCb251cyI6MC4wNiwiZGVwcmVjaWF0aW9uIjoxLjUsImNvZ3NEZXByZWNpYXRpb24iOjAuMywic2dhRGVwcmVjaWF0aW9uIjoxLjIsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMywib3RoZXJTZ2EiOjgsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjozLjk5OTk5OTk5OTk5OTk5NjQsInByZVRheEluY29tZSI6My45OTk5OTk5OTk5OTk5OTY0LCJuZXRJbmNvbWUiOjIuNzk5OTk5OTk5OTk5OTk3fX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjo3LjY3fSx7InllYXIiOjIwMjcsInZhbHVlIjo3LjY3fSx7InllYXIiOjIwMjgsInZhbHVlIjo3LjY2fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTcyNDYzNzY4MTE1ODYsInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsInByb2plY3RTZ2FSYXRlRW5kIjowLjExLCJvdGhlclNnYVJhdGVFbmQiOjAuMTA5Mjg1NzE0Mjg1NzE0MjgsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6MjMsInN1YnNpZHkiOjcuNjYsImxvY2FsQmVuY2htYXJrIjoyM30sImRyaXZlclJhbmdlcyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjpbLTAuMDUsMC4zXSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6WzAsMC45OV0sIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjpbMCwwLjk5XSwiZWZmZWN0aXZlVGF4UmF0ZSI6WzAsMC42XSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDEuNjY1MzM0NTM2OTM3NzM0OGUtMTZdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkzMjUzMzA1MDE4NDY5MjcsMC4wMjA3MzU5OTQxODMxODkxNjZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlswLjA0MDc2MDg2OTU2NTIxNzE4NCwwLjA0NDM4NDA1Nzk3MTAxNDUyXSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDAwMTM0NTc1NTY5MzU4MTk3MzddLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MTM5NDU3MDIzNzE3NDQzLDAuMDIwNTUzNDU5OTE0NzYzMDk1XSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjAzOTE2NjY2NjY2NjY2NjY4LDAuMDQyNTAwMDAwMDAwMDAwMDldLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbMC4xNSwwLjNdLCJvdGhlclNhbGVzR3Jvd3RoIjpbMC4wNjA3NjA4Njk1NjUyMTcxOSwwLjA2NDM4NDA1Nzk3MTAxNDUzXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMC4wMDUsMC4wMDUxMzQ1NzU1NjkzNTgxOTc1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLjAyNDEzOTQ1NzAyMzcxNzQ0NCwwLjAyNTU1MzQ1OTkxNDc2MzA5Nl0sIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6WzAsMC4wOF0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6WzAuMDQ0MTY2NjY2NjY2NjY2NjgsMC4wNDc1MDAwMDAwMDAwMDAwOV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMC4wODQ5OTk5OTk5OTk5OTk5OSwwLjEzNV0sIm90aGVyU2dhUmF0ZUVuZCI6WzAuMDg5Mjg1NzE0Mjg1NzE0MjcsMC4xMTkyODU3MTQyODU3MTQyN10sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjpbMC4wNDI2MzE1Nzg5NDczNjgzNiwwLjA2NTU1NTU1NTU1NTU1NTU4XSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MTUsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6ODIuNCwibWF4IjoyNTIuNjksInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55UGF5U2NoZWR1bGUiOnsidmFsdWUiOjIsIm1heCI6NywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc1NoYXJlIjp7InZhbHVlIjo2MCwibWF4Ijo5NSwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0NhZ3IiOnsidmFsdWUiOjIyLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjc0LjgsIm1heCI6MTM2Ljg0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MTguNzgsIm1heCI6MzMuNDMsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUNhZ3IiOnsidmFsdWUiOjcsIm1heCI6MTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUluY3JlYXNlIjp7InZhbHVlIjoyLjg1LCJtYXgiOjMuNzQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJpbnZlc3RtZW50U2FsZXNSYXRpbyI6eyJ2YWx1ZSI6MTUsIm1heCI6NzAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvIjp7InZhbHVlIjoyMTMsIm1heCI6MzUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibG9jYWxCZW5jaG1hcmsiOnsidmFsdWUiOjIzLCJtYXgiOjQwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUNhZ3IiOnsidmFsdWUiOjYsIm1heCI6MTAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnsiMjAyOTpvdGhlcjpzYWxlcyI6ODUuMTMsIjIwMjk6cHJvamVjdDo3LTgiOjcuOX0sImZ1dHVyZUlucHV0QmFzaXMiOiJvdGhlciIsImlucHV0VmFsdWVzIjp7ImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xIjoxMzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTMiOjkyLjc1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6MC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMyLjY1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6MC44MiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEwIjowLjA5LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTIiOjExLjY3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjAuNjIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNCI6Mi40NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1IjowLjY0LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTgiOjEwLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTkiOjEwLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjAiOjcuNTEsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yNyI6MjEwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xIjo3MiwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTQiOjIzLjA0LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNiI6Ni43OCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTgiOjUuMTksImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny05IjowLjM2LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTAiOjEuOCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEzIjo5MCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMSI6MTQzLjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0zIjo5Ny4zOCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTQiOjAuNzYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi03IjozNC41MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTkiOjAuODYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMCI6MC4xLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTIiOjEyLjQ3LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTMiOjAuNjYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNCI6Mi41OCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE1IjowLjY3LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTgiOjExLjAxLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTkiOjExLjAxLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjAiOjcuNzEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0yNyI6MjIwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xIjo3NiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0LjMyLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNiI6Ny4wNCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTgiOjUuNTksImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTAiOjEuOSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6MC44LCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTkiOjAuOSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjowLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6Mi43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTUiOjAuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE4IjoxMS4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTkiOjExLjMsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yMCI6Ny45MSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI3IjoyMzAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNCI6MjUuNiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTYiOjcuMywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTgiOjYsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny05IjowLjQsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xMCI6MiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudEFzc2V0cyI6NjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXNoIjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NSwiYmFsYW5jZS1zaGVldDoyMDIzOnRhbmdpYmxlQXNzZXRzIjo1MywiYmFsYW5jZS1zaGVldDoyMDIzOmJ1aWxkaW5ncyI6MTksImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzppbnRhbmdpYmxlQXNzZXRzIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUsImJhbGFuY2Utc2hlZXQ6MjAyMzpsaWFiaWxpdGllcyI6NzUsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50TGlhYmlsaXRpZXMiOjM5LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZExpYWJpbGl0aWVzIjozNiwiYmFsYW5jZS1zaGVldDoyMDIzOmxvbmdUZXJtRGVidCI6MjksImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hhcmVob2xkZXJFcXVpdHkiOjU0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NSwiYmFsYW5jZS1zaGVldDoyMDI0OmFzc2V0cyI6MTQzLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudEFzc2V0cyI6NzIsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNSwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkQXNzZXRzIjo3MSwiYmFsYW5jZS1zaGVldDoyMDI0OnRhbmdpYmxlQXNzZXRzIjo1OCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAsImJhbGFuY2Utc2hlZXQ6MjAyNDptYWNoaW5lcnkiOjI4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c29mdHdhcmUiOjYsImJhbGFuY2Utc2hlZXQ6MjAyNDpsaWFiaWxpdGllcyI6NzksImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZExpYWJpbGl0aWVzIjozOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEsImJhbGFuY2Utc2hlZXQ6MjAyNDpuZXRBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hhcmVob2xkZXJFcXVpdHkiOjYxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBleCI6OCwiYmFsYW5jZS1zaGVldDoyMDI1OmFzc2V0cyI6MTU2LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXNoIjoyNywiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkQXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI1OmJ1aWxkaW5ncyI6MjIsImJhbGFuY2Utc2hlZXQ6MjAyNTptYWNoaW5lcnkiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTppbnRhbmdpYmxlQXNzZXRzIjo5LCJiYWxhbmNlLXNoZWV0OjIwMjU6c29mdHdhcmUiOjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hvcnRUZXJtRGVidCI6MTEsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MCwiYmFsYW5jZS1zaGVldDoyMDI1OmxvbmdUZXJtRGVidCI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpuZXRBc3NldHMiOjczLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBleCI6MTAsImZ1dHVyZS1jYXBleDoyMDI2Ijo3LjY3LCJmdXR1cmUtY2FwZXg6MjAyNyI6Ny42NywiZnV0dXJlLWNhcGV4OjIwMjgiOjcuNjYsImZ1dHVyZS1jYXBleDoyMDI5IjowLCJmdXR1cmUtY2FwZXg6MjAzMCI6MCwiZnV0dXJlLWNhcGV4OjIwMzEiOjAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC45OSwiZHJpdmVyOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvOjEiOjAuOTksImRyaXZlcjplZmZlY3RpdmVUYXhSYXRlIjowLjMsImRyaXZlci1yYW5nZTplZmZlY3RpdmVUYXhSYXRlOjAiOjAsImRyaXZlci1yYW5nZTplZmZlY3RpdmVUYXhSYXRlOjEiOjAuNiwiZHJpdmVyOnByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aFRvQmFzZToxIjowLjA1NzAxNzU0Mzg1OTY0OTE5LCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6NS41NTExMTUxMjMxMjU3ODNlLTE3LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjoxLjY2NTMzNDUzNjkzNzczNDhlLTE2LCJkcml2ZXI6cHJvamVjdFBheUdyb3d0aFRvQmFzZSI6MC4wMjAwMzA2NjIzNDI1MTgwNDYsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDE5MzI1MzMwNTAxODQ2OTI3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZToxIjowLjAyMDczNTk5NDE4MzE4OTE2NiwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZToxIjowLjA1NzAxNzU0Mzg1OTY0OTE5LCJkcml2ZXI6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MCwiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZToxIjowLjA1NzAxNzU0Mzg1OTY0OTE5LCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI1NzI0NjM3NjgxMTU4NTQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjAiOjAuMDQwNzYwODY5NTY1MjE3MTg0LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZToxIjowLjA0NDM4NDA1Nzk3MTAxNDUyLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMDAxMzQ1NzU1NjkzNTgxOTczNywiZHJpdmVyOm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkxMzk0NTcwMjM3MTc0NDMsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZToxIjowLjAyMDU1MzQ1OTkxNDc2MzA5NSwiZHJpdmVyOm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjAiOjAuMDM5MTY2NjY2NjY2NjY2NjgsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZToxIjowLjA0MjUwMDAwMDAwMDAwMDA5LCJkcml2ZXI6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MCwiZHJpdmVyOnByb2plY3RTYWxlc0dyb3d0aCI6MC4yMiwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDowIjowLjE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjEiOjAuMywiZHJpdmVyOm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTcyNDYzNzY4MTE1ODYsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoOjAiOjAuMDYwNzYwODY5NTY1MjE3MTksImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoOjEiOjAuMDY0Mzg0MDU3OTcxMDE0NTMsImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2U6MSI6MC4wMywiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjAiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MSI6MC4wMDUxMzQ1NzU1NjkzNTgxOTc1LCJkcml2ZXI6cHJvamVjdFBheUdyb3d0aCI6MC4wNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGg6MCI6MC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGg6MSI6MC4xLCJkcml2ZXI6b3RoZXJQYXlHcm93dGgiOjAuMDI0ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDowIjowLjAyNDEzOTQ1NzAyMzcxNzQ0NCwiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjEiOjAuMDI1NTUzNDU5OTE0NzYzMDk2LCJkcml2ZXI6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjowLjA0NSwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjA0LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aDowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aDoxIjowLjA4LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MCI6MC4wNDQxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjEiOjAuMDQ3NTAwMDAwMDAwMDAwMDksImRyaXZlcjpwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjAiOjAuMDg0OTk5OTk5OTk5OTk5OTksImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDoxIjowLjEzNSwiZHJpdmVyOm90aGVyU2dhUmF0ZUVuZCI6MC4xMDkyODU3MTQyODU3MTQyOCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLjA4OTI4NTcxNDI4NTcxNDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMTE5Mjg1NzE0Mjg1NzE0MjcsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAuMDQyNjMxNTc4OTQ3MzY4MzYsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjA2NTU1NTU1NTU1NTU1NTU4LCJkcml2ZXI6dXNlZnVsTGlmZSI6MTAsImRyaXZlci1yYW5nZTp1c2VmdWxMaWZlOjAiOjUsImRyaXZlci1yYW5nZTp1c2VmdWxMaWZlOjEiOjIwLCJkcml2ZXI6aW52ZXN0bWVudCI6MjMsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjAiOjE1LCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDoxIjoyMDAsImRyaXZlcjpzdWJzaWR5Ijo3LjY2LCJkcml2ZXItcmFuZ2U6c3Vic2lkeTowIjoxLCJkcml2ZXItcmFuZ2U6c3Vic2lkeToxIjo1MCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoxNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjo4Mi40LCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjoyLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOm1heCI6NywidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOnZhbHVlIjo2MCwidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOm1heCI6OTUsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOnZhbHVlIjoyMiwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOnZhbHVlIjo3NC44LCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOnZhbHVlIjoyMSwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2FncjptYXgiOjM1LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOnZhbHVlIjoxOC43OCwidGFyZ2V0OmVtcGxveWVlUGF5Q2Fncjp2YWx1ZSI6NywidGFyZ2V0OmVtcGxveWVlUGF5Q2FncjptYXgiOjEwLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlJbmNyZWFzZTp2YWx1ZSI6Mi44NSwidGFyZ2V0OmludmVzdG1lbnRTYWxlc1JhdGlvOnZhbHVlIjoxNSwidGFyZ2V0OmludmVzdG1lbnRTYWxlc1JhdGlvOm1heCI6NzAsInRhcmdldDp2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvOnZhbHVlIjoyMTMsInRhcmdldDp2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvOm1heCI6MzUwLCJ0YXJnZXQ6bG9jYWxCZW5jaG1hcms6dmFsdWUiOjIzLCJ0YXJnZXQ6bG9jYWxCZW5jaG1hcms6bWF4Ijo0MCwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOnZhbHVlIjo2LCJ0YXJnZXQ6b2ZmaWNlclBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0Om9mZmljZXJQYXlJbmNyZWFzZTp2YWx1ZSI6MCwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOm1heCI6MjUyLjY5LCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6bWF4IjoxMzYuODQsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6bWF4IjozMy40MywidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6bWF4IjozLjc0fSwibWV0cmljR3JvdXBCYXNlcyI6eyJjb21wYW55U2FsZXMiOiJyYXRlIiwicHJvamVjdFNhbGVzIjoicmF0ZSIsImxhYm9yUHJvZHVjdGl2aXR5IjoicmF0ZSIsImVtcGxveWVlUGF5IjoicmF0ZSJ9LCJhcHBsaWNhdGlvbkNhdGVnb3J5IjoiZ2VuZXJhbCIsImFkanVzdGVkRHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZWZmZWN0aXZlVGF4UmF0ZSI6MC4zLCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MTA1OTU3NjAyMzM5MTYsInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjEuMTc0MTg2NDkxMDY0NDY2ZS0xNiwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6MC4wMTk5ODIxMzU1MTE4Nzk4NzMsInByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDU0MDYzOTAxMjQ5NzIyOTM0LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDEyMDQ1MTMzMzE1NzYzLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjYwNTUxNjI3MzAwNTI3LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODgxMzY3NTAwOTE3MTE3LCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDYwOTM1Mzk0MzcxNzg1NSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyMDIyNDg3MjE2OTQ2NjczLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU2NTE3ODU5NDUyMTc5LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNDk5MDQ4MTM0MTI2NTU1LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDg5MDA2MjI5OTc1MDgwMSwib3RoZXJQYXlHcm93dGgiOjAuMDI0ODg3NzYxNzEwMzMzMDMsIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6MC4wNDUsInByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDI5MDQ1NDgyMzk3MjA1MDU1LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU3ODQ4MTQ3MzIzMDg2NjUsInByb2plY3RTZ2FSYXRlRW5kIjowLjEwOTkzMTgwOTE2NDg0ODI0LCJvdGhlclNnYVJhdGVFbmQiOjAuMTA5MjcyNTg5ODcyMTI4MjMsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1Mzc3ODA1NzYyODcxNjMyLCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6MjMsInN1YnNpZHkiOjcuNjYsImxvY2FsQmVuY2htYXJrIjoyM319</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Expose detailed accounting assumptions as forecast drivers
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -384,7 +384,7 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <v>23.49843476135365</v>
+        <v>23.487308177598077</v>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
@@ -414,7 +414,7 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <v>19.660000000000004</v>
+        <v>19.66</v>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <v>256.6579634464752</v>
+        <v>256.65796344647515</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
@@ -1465,22 +1465,22 @@
         <v>36.4</v>
       </c>
       <c r="E9" s="2">
-        <v>38.870000000000005</v>
+        <v>38.85</v>
       </c>
       <c r="F9" s="2">
-        <v>41.47</v>
+        <v>41.44</v>
       </c>
       <c r="G9" s="2">
-        <v>44.18</v>
+        <v>44.15</v>
       </c>
       <c r="H9" s="2">
-        <v>47.93</v>
+        <v>47.900000000000006</v>
       </c>
       <c r="I9" s="2">
-        <v>52.589999999999996</v>
+        <v>52.56</v>
       </c>
       <c r="J9" s="2">
-        <v>57.81</v>
+        <v>57.769999999999996</v>
       </c>
     </row>
     <row r="10">
@@ -1545,10 +1545,10 @@
         <v>1.09</v>
       </c>
       <c r="I11" s="2">
-        <v>1.1300000000000001</v>
+        <v>1.1400000000000001</v>
       </c>
       <c r="J11" s="2">
-        <v>1.18</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="12">
@@ -1579,10 +1579,10 @@
         <v>0.12000000000000001</v>
       </c>
       <c r="I12" s="2">
+        <v>0.12000000000000001</v>
+      </c>
+      <c r="J12" s="2">
         <v>0.13</v>
-      </c>
-      <c r="J12" s="2">
-        <v>0.14</v>
       </c>
     </row>
     <row r="13">
@@ -1644,13 +1644,13 @@
         <v>16.17</v>
       </c>
       <c r="H14" s="2">
-        <v>17.69</v>
+        <v>17.68</v>
       </c>
       <c r="I14" s="2">
-        <v>19.35</v>
+        <v>19.34</v>
       </c>
       <c r="J14" s="2">
-        <v>21.16</v>
+        <v>21.15</v>
       </c>
     </row>
     <row r="15">
@@ -1678,13 +1678,13 @@
         <v>0.85</v>
       </c>
       <c r="H15" s="2">
-        <v>0.9199999999999999</v>
+        <v>0.9299999999999999</v>
       </c>
       <c r="I15" s="2">
-        <v>1.01</v>
+        <v>1.02</v>
       </c>
       <c r="J15" s="2">
-        <v>1.1099999999999999</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="16">
@@ -1709,16 +1709,16 @@
         <v>3.8499999999999996</v>
       </c>
       <c r="G16" s="2">
-        <v>4.43</v>
+        <v>4.42</v>
       </c>
       <c r="H16" s="2">
-        <v>4.43</v>
+        <v>4.42</v>
       </c>
       <c r="I16" s="2">
-        <v>4.43</v>
+        <v>4.42</v>
       </c>
       <c r="J16" s="2">
-        <v>4.43</v>
+        <v>4.42</v>
       </c>
     </row>
     <row r="17">
@@ -1737,22 +1737,22 @@
         <v>0.7</v>
       </c>
       <c r="E17" s="2">
-        <v>0.73</v>
+        <v>0.71</v>
       </c>
       <c r="F17" s="2">
-        <v>0.77</v>
+        <v>0.74</v>
       </c>
       <c r="G17" s="2">
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H17" s="2">
-        <v>0.9299999999999999</v>
+        <v>0.9099999999999999</v>
       </c>
       <c r="I17" s="2">
-        <v>1.08</v>
+        <v>1.06</v>
       </c>
       <c r="J17" s="2">
-        <v>1.26</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="18">
@@ -1771,22 +1771,22 @@
         <v>11.600000000000001</v>
       </c>
       <c r="E18" s="4">
-        <v>11.470000000000006</v>
+        <v>11.490000000000006</v>
       </c>
       <c r="F18" s="4">
-        <v>11.320000000000014</v>
+        <v>11.350000000000016</v>
       </c>
       <c r="G18" s="4">
-        <v>11.180000000000003</v>
+        <v>11.21</v>
       </c>
       <c r="H18" s="4">
-        <v>17.179999999999986</v>
+        <v>17.209999999999987</v>
       </c>
       <c r="I18" s="4">
-        <v>23.27999999999998</v>
+        <v>23.309999999999974</v>
       </c>
       <c r="J18" s="4">
-        <v>31.090000000000046</v>
+        <v>31.130000000000045</v>
       </c>
     </row>
     <row r="19">
@@ -1805,22 +1805,22 @@
         <v>7.733333333333333</v>
       </c>
       <c r="E19" s="2">
-        <v>7.291335579429156</v>
+        <v>7.304049329349695</v>
       </c>
       <c r="F19" s="2">
-        <v>6.861437750030315</v>
+        <v>6.879621772336049</v>
       </c>
       <c r="G19" s="2">
-        <v>6.46130728775357</v>
+        <v>6.478645321620529</v>
       </c>
       <c r="H19" s="2">
-        <v>8.612823983556417</v>
+        <v>8.627863839173804</v>
       </c>
       <c r="I19" s="2">
-        <v>10.12349973908505</v>
+        <v>10.136545486171498</v>
       </c>
       <c r="J19" s="2">
-        <v>11.672172998948808</v>
+        <v>11.687190268809147</v>
       </c>
     </row>
     <row r="20">
@@ -1839,22 +1839,22 @@
         <v>11.3</v>
       </c>
       <c r="E20" s="4">
-        <v>11.159999999999991</v>
+        <v>11.129999999999999</v>
       </c>
       <c r="F20" s="4">
-        <v>10.989999999999995</v>
+        <v>10.97</v>
       </c>
       <c r="G20" s="4">
-        <v>10.830000000000005</v>
+        <v>10.81</v>
       </c>
       <c r="H20" s="4">
-        <v>15.949999999999996</v>
+        <v>15.5</v>
       </c>
       <c r="I20" s="4">
-        <v>21.939999999999984</v>
+        <v>21.46</v>
       </c>
       <c r="J20" s="4">
-        <v>29.62000000000001</v>
+        <v>29.130000000000003</v>
       </c>
     </row>
     <row r="21">
@@ -1873,22 +1873,22 @@
         <v>11.3</v>
       </c>
       <c r="E21" s="2">
-        <v>11.159999999999991</v>
+        <v>11.129999999999999</v>
       </c>
       <c r="F21" s="2">
-        <v>10.989999999999995</v>
+        <v>10.97</v>
       </c>
       <c r="G21" s="2">
-        <v>10.830000000000005</v>
+        <v>10.81</v>
       </c>
       <c r="H21" s="2">
-        <v>15.949999999999996</v>
+        <v>15.5</v>
       </c>
       <c r="I21" s="2">
-        <v>21.939999999999984</v>
+        <v>21.46</v>
       </c>
       <c r="J21" s="2">
-        <v>29.62000000000001</v>
+        <v>29.130000000000003</v>
       </c>
     </row>
     <row r="22">
@@ -1907,22 +1907,22 @@
         <v>7.91</v>
       </c>
       <c r="E22" s="2">
-        <v>7.805999999999994</v>
+        <v>7.79</v>
       </c>
       <c r="F22" s="2">
-        <v>7.691999999999997</v>
+        <v>7.68</v>
       </c>
       <c r="G22" s="2">
-        <v>7.578000000000003</v>
+        <v>7.57</v>
       </c>
       <c r="H22" s="2">
-        <v>11.157999999999998</v>
+        <v>10.85</v>
       </c>
       <c r="I22" s="2">
-        <v>15.352999999999987</v>
+        <v>15.030000000000001</v>
       </c>
       <c r="J22" s="2">
-        <v>20.732000000000006</v>
+        <v>20.39</v>
       </c>
     </row>
     <row r="23">
@@ -2043,22 +2043,22 @@
         <v>30.1</v>
       </c>
       <c r="E26" s="4">
-        <v>31.720000000000006</v>
+        <v>31.740000000000006</v>
       </c>
       <c r="F26" s="4">
-        <v>33.390000000000015</v>
+        <v>33.420000000000016</v>
       </c>
       <c r="G26" s="4">
-        <v>35.14</v>
+        <v>35.17</v>
       </c>
       <c r="H26" s="4">
-        <v>42.33999999999998</v>
+        <v>42.36999999999998</v>
       </c>
       <c r="I26" s="4">
-        <v>50.17999999999997</v>
+        <v>50.20999999999997</v>
       </c>
       <c r="J26" s="4">
-        <v>59.90000000000004</v>
+        <v>59.94000000000004</v>
       </c>
     </row>
     <row r="27">
@@ -2079,22 +2079,22 @@
         <v>4.768534632788035</v>
       </c>
       <c r="E27" s="2">
-        <v>5.382059800664463</v>
+        <v>5.448504983388713</v>
       </c>
       <c r="F27" s="2">
-        <v>5.264817150063084</v>
+        <v>5.293005671077533</v>
       </c>
       <c r="G27" s="2">
-        <v>5.241090146750471</v>
+        <v>5.236385397965249</v>
       </c>
       <c r="H27" s="2">
-        <v>20.489470688673816</v>
+        <v>20.47199317600221</v>
       </c>
       <c r="I27" s="2">
-        <v>18.516769012753876</v>
+        <v>18.5036582487609</v>
       </c>
       <c r="J27" s="2">
-        <v>19.370267038660984</v>
+        <v>19.378609838677697</v>
       </c>
     </row>
     <row r="28">
@@ -2113,22 +2113,22 @@
         <v>20.06666666666667</v>
       </c>
       <c r="E28" s="2">
-        <v>20.164007373974957</v>
+        <v>20.176721123895497</v>
       </c>
       <c r="F28" s="2">
-        <v>20.23881682628198</v>
+        <v>20.257000848587715</v>
       </c>
       <c r="G28" s="2">
-        <v>20.30861700283188</v>
+        <v>20.32595503669884</v>
       </c>
       <c r="H28" s="2">
-        <v>21.226249561337536</v>
+        <v>21.241289416954924</v>
       </c>
       <c r="I28" s="2">
-        <v>21.821186293268386</v>
+        <v>21.834232040354834</v>
       </c>
       <c r="J28" s="2">
-        <v>22.488361615858253</v>
+        <v>22.50337888571859</v>
       </c>
     </row>
     <row r="29">
@@ -2355,22 +2355,22 @@
         <v>0.12808510638297874</v>
       </c>
       <c r="E35" s="2">
-        <v>0.12946938775510206</v>
+        <v>0.1295510204081633</v>
       </c>
       <c r="F35" s="2">
-        <v>0.12992217898832692</v>
+        <v>0.13003891050583663</v>
       </c>
       <c r="G35" s="2">
-        <v>0.13111940298507463</v>
+        <v>0.1312313432835821</v>
       </c>
       <c r="H35" s="2">
-        <v>0.15230215827338123</v>
+        <v>0.152410071942446</v>
       </c>
       <c r="I35" s="2">
-        <v>0.17363321799307949</v>
+        <v>0.17373702422145318</v>
       </c>
       <c r="J35" s="2">
-        <v>0.1996666666666668</v>
+        <v>0.19980000000000014</v>
       </c>
     </row>
     <row r="36">
@@ -2389,22 +2389,22 @@
         <v>15.100000000000001</v>
       </c>
       <c r="E36" s="4">
-        <v>15.740000000000006</v>
+        <v>15.760000000000005</v>
       </c>
       <c r="F36" s="4">
-        <v>16.350000000000016</v>
+        <v>16.380000000000017</v>
       </c>
       <c r="G36" s="4">
-        <v>16.980000000000004</v>
+        <v>17.01</v>
       </c>
       <c r="H36" s="4">
-        <v>22.979999999999986</v>
+        <v>23.009999999999987</v>
       </c>
       <c r="I36" s="4">
-        <v>29.07999999999998</v>
+        <v>29.109999999999975</v>
       </c>
       <c r="J36" s="4">
-        <v>36.89000000000004</v>
+        <v>36.93000000000004</v>
       </c>
     </row>
     <row r="37">
@@ -2423,22 +2423,22 @@
         <v>10.066666666666668</v>
       </c>
       <c r="E37" s="2">
-        <v>10.005721187464246</v>
+        <v>10.018434937384784</v>
       </c>
       <c r="F37" s="2">
-        <v>9.910292156625054</v>
+        <v>9.928476178930788</v>
       </c>
       <c r="G37" s="2">
-        <v>9.813327168699072</v>
+        <v>9.83066520256603</v>
       </c>
       <c r="H37" s="2">
-        <v>11.520529402917726</v>
+        <v>11.535569258535112</v>
       </c>
       <c r="I37" s="2">
-        <v>12.645677509132017</v>
+        <v>12.658723256218462</v>
       </c>
       <c r="J37" s="2">
-        <v>13.849677128698017</v>
+        <v>13.864694398558358</v>
       </c>
     </row>
     <row r="38">
@@ -2459,22 +2459,22 @@
         <v>3.1420765027322606</v>
       </c>
       <c r="E38" s="2">
-        <v>4.238410596026521</v>
+        <v>4.370860927152331</v>
       </c>
       <c r="F38" s="2">
-        <v>3.875476493011498</v>
+        <v>3.9340101522843396</v>
       </c>
       <c r="G38" s="2">
-        <v>3.85321100917424</v>
+        <v>3.8461538461537437</v>
       </c>
       <c r="H38" s="2">
-        <v>35.33568904593629</v>
+        <v>35.27336860670185</v>
       </c>
       <c r="I38" s="2">
-        <v>26.544821583986057</v>
+        <v>26.510212950890867</v>
       </c>
       <c r="J38" s="2">
-        <v>26.856946354883316</v>
+        <v>26.863620748883797</v>
       </c>
     </row>
   </sheetData>
@@ -2805,16 +2805,16 @@
         <v>6.859999999999996</v>
       </c>
       <c r="G8" s="4">
-        <v>6.640000000000004</v>
+        <v>6.650000000000006</v>
       </c>
       <c r="H8" s="4">
-        <v>11.239999999999997</v>
+        <v>11.249999999999998</v>
       </c>
       <c r="I8" s="4">
-        <v>16.689999999999984</v>
+        <v>16.69999999999998</v>
       </c>
       <c r="J8" s="4">
-        <v>23.760000000000012</v>
+        <v>23.77000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -2839,16 +2839,16 @@
         <v>7.717403532455839</v>
       </c>
       <c r="G9" s="2">
-        <v>7.086446104589118</v>
+        <v>7.097118463180369</v>
       </c>
       <c r="H9" s="2">
-        <v>9.830330592968336</v>
+        <v>9.83907643869162</v>
       </c>
       <c r="I9" s="2">
-        <v>11.963300121855053</v>
+        <v>11.970468066805234</v>
       </c>
       <c r="J9" s="2">
-        <v>13.95676691729324</v>
+        <v>13.962640977443613</v>
       </c>
     </row>
     <row r="10">
@@ -2975,16 +2975,16 @@
         <v>17.769999999999996</v>
       </c>
       <c r="G13" s="4">
-        <v>18.870000000000005</v>
+        <v>18.880000000000006</v>
       </c>
       <c r="H13" s="4">
-        <v>23.939999999999998</v>
+        <v>23.95</v>
       </c>
       <c r="I13" s="4">
-        <v>30.359999999999985</v>
+        <v>30.369999999999983</v>
       </c>
       <c r="J13" s="4">
-        <v>38.53000000000001</v>
+        <v>38.540000000000006</v>
       </c>
     </row>
     <row r="14">
@@ -3011,16 +3011,16 @@
         <v>6.279904306220119</v>
       </c>
       <c r="G14" s="2">
-        <v>6.190208216094595</v>
+        <v>6.246482836240919</v>
       </c>
       <c r="H14" s="2">
-        <v>26.868044515103296</v>
+        <v>26.853813559321992</v>
       </c>
       <c r="I14" s="2">
-        <v>26.81704260651625</v>
+        <v>26.805845511482197</v>
       </c>
       <c r="J14" s="2">
-        <v>26.910408432147648</v>
+        <v>26.901547579848618</v>
       </c>
     </row>
     <row r="15">
@@ -3253,16 +3253,16 @@
         <v>0.15725663716814156</v>
       </c>
       <c r="G21" s="2">
-        <v>0.1585714285714286</v>
+        <v>0.158655462184874</v>
       </c>
       <c r="H21" s="2">
-        <v>0.1962295081967213</v>
+        <v>0.19631147540983607</v>
       </c>
       <c r="I21" s="2">
-        <v>0.24095238095238083</v>
+        <v>0.2410317460317459</v>
       </c>
       <c r="J21" s="2">
-        <v>0.29868217054263574</v>
+        <v>0.29875968992248064</v>
       </c>
     </row>
     <row r="22">
@@ -3761,32 +3761,32 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.71 % / 補助 23.61 % / ベース 25.98 %</t>
+          <t xml:space="preserve">全社 24.7 % / 補助 23.61 % / ベース 25.95 %</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 25.14 % / 補助 24.28 % / ベース 26.14 %</t>
+          <t xml:space="preserve">全社 25.12 % / 補助 24.28 % / ベース 26.1 %</t>
         </is>
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 25.53 % / 補助 24.91 % / ベース 26.27 %</t>
+          <t xml:space="preserve">全社 25.52 % / 補助 24.9 % / ベース 26.24 %</t>
         </is>
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.03 % / 補助 22.67 % / ベース 25.85 %</t>
+          <t xml:space="preserve">全社 24.01 % / 補助 22.66 % / ベース 25.83 %</t>
         </is>
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 22.87 % / 補助 21.03 % / ベース 25.7 %</t>
+          <t xml:space="preserve">全社 22.86 % / 補助 21.02 % / ベース 25.68 %</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 21.7 % / 補助 19.54 % / ベース 25.54 %</t>
+          <t xml:space="preserve">全社 21.69 % / 補助 19.53 % / ベース 25.51 %</t>
         </is>
       </c>
     </row>
@@ -3823,32 +3823,32 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.29 % / 補助 8.4 % / ベース 6.02 %</t>
+          <t xml:space="preserve">全社 7.3 % / 補助 8.4 % / ベース 6.04 %</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.86 % / 補助 7.72 % / ベース 5.86 %</t>
+          <t xml:space="preserve">全社 6.88 % / 補助 7.72 % / ベース 5.9 %</t>
         </is>
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.46 % / 補助 7.09 % / ベース 5.72 %</t>
+          <t xml:space="preserve">全社 6.48 % / 補助 7.1 % / ベース 5.75 %</t>
         </is>
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.61 % / 補助 9.83 % / ベース 6.98 %</t>
+          <t xml:space="preserve">全社 8.63 % / 補助 9.84 % / ベース 7 %</t>
         </is>
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.12 % / 補助 11.96 % / ベース 7.29 %</t>
+          <t xml:space="preserve">全社 10.14 % / 補助 11.97 % / ベース 7.31 %</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.67 % / 補助 13.96 % / ベース 7.63 %</t>
+          <t xml:space="preserve">全社 11.69 % / 補助 13.96 % / ベース 7.66 %</t>
         </is>
       </c>
     </row>
@@ -3885,32 +3885,32 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.01 % / 補助 11.68 % / ベース 8.07 %</t>
+          <t xml:space="preserve">全社 10.02 % / 補助 11.68 % / ベース 8.1 %</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.91 % / 補助 11.69 % / ベース 7.83 %</t>
+          <t xml:space="preserve">全社 9.93 % / 補助 11.69 % / ベース 7.87 %</t>
         </is>
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.81 % / 補助 11.68 % / ベース 7.61 %</t>
+          <t xml:space="preserve">全社 9.83 % / 補助 11.69 % / ベース 7.64 %</t>
         </is>
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.52 % / 補助 13.59 % / ベース 8.74 %</t>
+          <t xml:space="preserve">全社 11.54 % / 補助 13.6 % / ベース 8.76 %</t>
         </is>
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.65 % / 補助 15.05 % / ベース 8.94 %</t>
+          <t xml:space="preserve">全社 12.66 % / 補助 15.05 % / ベース 8.97 %</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.85 % / 補助 16.48 % / ベース 9.19 %</t>
+          <t xml:space="preserve">全社 13.86 % / 補助 16.49 % / ベース 9.22 %</t>
         </is>
       </c>
     </row>
@@ -4443,32 +4443,32 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 50.38 % / 補助 41.09 % / ベース 60.73 %</t>
+          <t xml:space="preserve">全社 50.35 % / 補助 41.09 % / ベース 60.65 %</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 51.03 % / 補助 41.53 % / ベース 61.84 %</t>
+          <t xml:space="preserve">全社 50.99 % / 補助 41.53 % / ベース 61.73 %</t>
         </is>
       </c>
       <c r="I18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 51.68 % / 補助 42.02 % / ベース 62.88 %</t>
+          <t xml:space="preserve">全社 51.63 % / 補助 42 % / ベース 62.8 %</t>
         </is>
       </c>
       <c r="J18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 45.73 % / 補助 35.09 % / ベース 59.57 %</t>
+          <t xml:space="preserve">全社 45.69 % / 補助 35.07 % / ベース 59.5 %</t>
         </is>
       </c>
       <c r="K18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 42.05 % / 補助 30.86 % / ベース 59.18 %</t>
+          <t xml:space="preserve">全社 42.02 % / 補助 30.85 % / ベース 59.12 %</t>
         </is>
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 38.41 % / 補助 27.17 % / ベース 58.68 %</t>
+          <t xml:space="preserve">全社 38.39 % / 補助 27.17 % / ベース 58.6 %</t>
         </is>
       </c>
     </row>
@@ -4654,7 +4654,7 @@
       </c>
       <c r="L21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.105 億円/人 / 補助 0.187 億円/人 / ベース 0.044 億円/人</t>
+          <t xml:space="preserve">全社 0.106 億円/人 / 補助 0.187 億円/人 / ベース 0.044 億円/人</t>
         </is>
       </c>
     </row>
@@ -4691,12 +4691,12 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.129 億円/人 / 補助 0.156 億円/人 / ベース 0.109 億円/人</t>
+          <t xml:space="preserve">全社 0.13 億円/人 / 補助 0.156 億円/人 / ベース 0.109 億円/人</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.13 億円/人 / 補助 0.157 億円/人 / ベース 0.108 億円/人</t>
+          <t xml:space="preserve">全社 0.13 億円/人 / 補助 0.157 億円/人 / ベース 0.109 億円/人</t>
         </is>
       </c>
       <c r="I22" s="0" t="inlineStr">
@@ -5125,32 +5125,32 @@
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.69 倍 / 補助 3.56 倍 / ベース 3.93 倍</t>
+          <t xml:space="preserve">全社 3.69 倍 / 補助 3.56 倍 / ベース 3.94 倍</t>
         </is>
       </c>
       <c r="H29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.25 倍 / 補助 2.94 倍 / ベース 3.97 倍</t>
+          <t xml:space="preserve">全社 3.26 倍 / 補助 2.94 倍 / ベース 3.99 倍</t>
         </is>
       </c>
       <c r="I29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.93 倍 / 補助 2.54 倍 / ベース 4.03 倍</t>
+          <t xml:space="preserve">全社 2.93 倍 / 補助 2.55 倍 / ベース 4.04 倍</t>
         </is>
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.96 倍 / 補助 3.61 倍 / ベース 4.96 倍</t>
+          <t xml:space="preserve">全社 3.97 倍 / 補助 3.62 倍 / ベース 4.97 倍</t>
         </is>
       </c>
       <c r="K29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5.01 倍 / 補助 4.88 倍 / ベース 5.39 倍</t>
+          <t xml:space="preserve">全社 5.02 倍 / 補助 4.88 倍 / ベース 5.41 倍</t>
         </is>
       </c>
       <c r="L29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.36 倍 / 補助 6.53 倍 / ベース 5.89 倍</t>
+          <t xml:space="preserve">全社 6.37 倍 / 補助 6.53 倍 / ベース 5.91 倍</t>
         </is>
       </c>
     </row>
@@ -5497,32 +5497,32 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 2.38 pt</t>
+          <t xml:space="preserve">差 2.35 pt</t>
         </is>
       </c>
       <c r="H35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 1.86 pt</t>
+          <t xml:space="preserve">差 1.82 pt</t>
         </is>
       </c>
       <c r="I35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 1.36 pt</t>
+          <t xml:space="preserve">差 1.35 pt</t>
         </is>
       </c>
       <c r="J35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 2.85 pt</t>
+          <t xml:space="preserve">差 2.84 pt</t>
         </is>
       </c>
       <c r="K35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 4.68 pt</t>
+          <t xml:space="preserve">差 4.66 pt</t>
         </is>
       </c>
       <c r="L35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 6.33 pt</t>
+          <t xml:space="preserve">差 6.31 pt</t>
         </is>
       </c>
     </row>
@@ -5683,17 +5683,17 @@
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 169.23 %</t>
+          <t xml:space="preserve">寄与率 200 %</t>
         </is>
       </c>
       <c r="H38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 146.67 %</t>
+          <t xml:space="preserve">寄与率 157.14 %</t>
         </is>
       </c>
       <c r="I38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 157.14 %</t>
+          <t xml:space="preserve">寄与率 150 %</t>
         </is>
       </c>
       <c r="J38" s="0" t="inlineStr">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 90.52 %</t>
+          <t xml:space="preserve">寄与率 90.41 %</t>
         </is>
       </c>
     </row>
@@ -5718,7 +5718,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="68" customWidth="1"/>
@@ -5821,11 +5821,15 @@
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D4" s="2">
-        <v>0</v>
-      </c>
-      <c r="E4" s="2">
-        <v>99</v>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -5842,185 +5846,221 @@
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D5" s="2">
-        <v>0</v>
-      </c>
-      <c r="E5" s="2">
-        <v>99</v>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">実効税率</t>
+          <t xml:space="preserve">補助事業 従業員給与総額に占める給与の割合</t>
         </is>
       </c>
       <c r="B6" s="2">
-        <v>30</v>
+        <v>95</v>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D6" s="2">
-        <v>0</v>
-      </c>
-      <c r="E6" s="2">
-        <v>60</v>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 売上成長率（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 従業員給与総額に占める給与の割合</t>
         </is>
       </c>
       <c r="B7" s="2">
-        <v>5.409356725146197</v>
+        <v>95</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D7" s="2">
-        <v>5.116959064327475</v>
-      </c>
-      <c r="E7" s="2">
-        <v>5.701754385964919</v>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 原価率改善ポイント（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 役員給与総額に占める役員報酬の割合</t>
         </is>
       </c>
       <c r="B8" s="2">
-        <v>5.551115123125783e-15</v>
+        <v>90</v>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D8" s="2">
-        <v>0</v>
-      </c>
-      <c r="E8" s="2">
-        <v>1.6653345369377348e-14</v>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 1人当たり給与支給総額上昇率（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 役員給与総額に占める役員報酬の割合</t>
         </is>
       </c>
       <c r="B9" s="2">
-        <v>2.0030662342518046</v>
+        <v>90</v>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">基準年度額が最新決算期額以上（成長率0%以上）</t>
-        </is>
-      </c>
-      <c r="D9" s="2">
-        <v>1.9325330501846927</v>
-      </c>
-      <c r="E9" s="2">
-        <v>2.0735994183189166</v>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 常時使用する従業員数の成長率（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 減価償却費のうち売上原価に含める割合</t>
         </is>
       </c>
       <c r="B10" s="2">
-        <v>5.409356725146197</v>
+        <v>25</v>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D10" s="2">
-        <v>5.116959064327475</v>
-      </c>
-      <c r="E10" s="2">
-        <v>5.701754385964919</v>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 その他販管費率改善ポイント（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 減価償却費のうち売上原価に含める割合</t>
         </is>
       </c>
       <c r="B11" s="2">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D11" s="2">
-        <v>0</v>
-      </c>
-      <c r="E11" s="2">
-        <v>0</v>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">役員1人当たり給与支給総額上昇率（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 研究開発費の売上高比率</t>
         </is>
       </c>
       <c r="B12" s="2">
-        <v>5.409356725146197</v>
+        <v>0.5</v>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D12" s="2">
-        <v>5.116959064327475</v>
-      </c>
-      <c r="E12" s="2">
-        <v>5.701754385964919</v>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 売上成長率（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 研究開発費の売上高比率</t>
         </is>
       </c>
       <c r="B13" s="2">
-        <v>4.257246376811585</v>
+        <v>0.4</v>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D13" s="2">
-        <v>4.076086956521719</v>
-      </c>
-      <c r="E13" s="2">
-        <v>4.438405797101453</v>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 原価率改善ポイント（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 営業外損益の売上高比率</t>
         </is>
       </c>
       <c r="B14" s="2">
@@ -6031,105 +6071,125 @@
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D14" s="2">
-        <v>0</v>
-      </c>
-      <c r="E14" s="2">
-        <v>0.013457556935819737</v>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E14" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業1人当たり給与支給総額の年平均上昇率（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 営業外損益の売上高比率</t>
         </is>
       </c>
       <c r="B15" s="2">
-        <v>1.984645846924027</v>
+        <v>-0.5</v>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D15" s="2">
-        <v>1.9139457023717443</v>
-      </c>
-      <c r="E15" s="2">
-        <v>2.0553459914763095</v>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 役員1人当たり給与支給総額上昇率（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 特別損益の売上高比率</t>
         </is>
       </c>
       <c r="B16" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D16" s="2">
-        <v>0</v>
-      </c>
-      <c r="E16" s="2">
-        <v>8</v>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 常時使用する従業員数の成長率（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 特別損益の売上高比率</t>
         </is>
       </c>
       <c r="B17" s="2">
-        <v>4.083333333333339</v>
+        <v>0</v>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D17" s="2">
-        <v>3.9166666666666683</v>
-      </c>
-      <c r="E17" s="2">
-        <v>4.250000000000009</v>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 その他販管費率改善ポイント（設備導入期間）</t>
+          <t xml:space="preserve">実効税率（当期純利益割合＝100%－実効税率）</t>
         </is>
       </c>
       <c r="B18" s="2">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D18" s="2">
-        <v>0</v>
-      </c>
-      <c r="E18" s="2">
-        <v>0</v>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 売上成長率（基準年度後）</t>
+          <t xml:space="preserve">補助事業 売上成長率（設備導入期間）</t>
         </is>
       </c>
       <c r="B19" s="2">
-        <v>22</v>
+        <v>5.409356725146197</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
@@ -6137,20 +6197,20 @@
         </is>
       </c>
       <c r="D19" s="2">
-        <v>15</v>
+        <v>5.116959064327475</v>
       </c>
       <c r="E19" s="2">
-        <v>30</v>
+        <v>5.701754385964919</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 売上成長率（基準年度後）</t>
+          <t xml:space="preserve">補助事業 原価率改善ポイント（設備導入期間）</t>
         </is>
       </c>
       <c r="B20" s="2">
-        <v>6.257246376811586</v>
+        <v>5.551115123125783e-15</v>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
@@ -6158,41 +6218,41 @@
         </is>
       </c>
       <c r="D20" s="2">
-        <v>6.076086956521719</v>
+        <v>0</v>
       </c>
       <c r="E20" s="2">
-        <v>6.438405797101453</v>
+        <v>1.6653345369377348e-14</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 原価率改善ポイント（基準年度後）</t>
+          <t xml:space="preserve">補助事業 1人当たり給与支給総額上昇率（設備導入期間）</t>
         </is>
       </c>
       <c r="B21" s="2">
-        <v>1.5</v>
+        <v>2.0030662342518046</v>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">—</t>
+          <t xml:space="preserve">基準年度額が最新決算期額以上（成長率0%以上）</t>
         </is>
       </c>
       <c r="D21" s="2">
-        <v>0</v>
+        <v>1.9325330501846927</v>
       </c>
       <c r="E21" s="2">
-        <v>3</v>
+        <v>2.0735994183189166</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 原価率改善ポイント（基準年度後）</t>
+          <t xml:space="preserve">補助事業 常時使用する従業員数の成長率（設備導入期間）</t>
         </is>
       </c>
       <c r="B22" s="2">
-        <v>0.5</v>
+        <v>5.409356725146197</v>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
@@ -6200,20 +6260,20 @@
         </is>
       </c>
       <c r="D22" s="2">
-        <v>0.5</v>
+        <v>5.116959064327475</v>
       </c>
       <c r="E22" s="2">
-        <v>0.5134575569358197</v>
+        <v>5.701754385964919</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業1人当たり給与支給総額の年平均上昇率</t>
+          <t xml:space="preserve">補助事業 その他販管費率改善ポイント（設備導入期間）</t>
         </is>
       </c>
       <c r="B23" s="2">
-        <v>7.000000000000001</v>
+        <v>0</v>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
@@ -6221,20 +6281,20 @@
         </is>
       </c>
       <c r="D23" s="2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E23" s="2">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業1人当たり給与支給総額の年平均上昇率（基準年度後）</t>
+          <t xml:space="preserve">役員1人当たり給与支給総額上昇率（設備導入期間）</t>
         </is>
       </c>
       <c r="B24" s="2">
-        <v>2.484645846924027</v>
+        <v>5.409356725146197</v>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
@@ -6242,20 +6302,20 @@
         </is>
       </c>
       <c r="D24" s="2">
-        <v>2.4139457023717443</v>
+        <v>5.116959064327475</v>
       </c>
       <c r="E24" s="2">
-        <v>2.5553459914763095</v>
+        <v>5.701754385964919</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 役員1人当たり給与支給総額上昇率（基準年度後）</t>
+          <t xml:space="preserve">ベース事業 売上成長率（設備導入期間）</t>
         </is>
       </c>
       <c r="B25" s="2">
-        <v>4.5</v>
+        <v>4.257246376811585</v>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
@@ -6263,20 +6323,20 @@
         </is>
       </c>
       <c r="D25" s="2">
-        <v>0</v>
+        <v>4.076086956521719</v>
       </c>
       <c r="E25" s="2">
-        <v>8</v>
+        <v>4.438405797101453</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 常時使用する従業員数の成長率</t>
+          <t xml:space="preserve">ベース事業 原価率改善ポイント（設備導入期間）</t>
         </is>
       </c>
       <c r="B26" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
@@ -6287,17 +6347,17 @@
         <v>0</v>
       </c>
       <c r="E26" s="2">
-        <v>8</v>
+        <v>0.013457556935819737</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 常時使用する従業員数の成長率（基準年度後）</t>
+          <t xml:space="preserve">ベース事業1人当たり給与支給総額の年平均上昇率（設備導入期間）</t>
         </is>
       </c>
       <c r="B27" s="2">
-        <v>4.583333333333338</v>
+        <v>1.984645846924027</v>
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
@@ -6305,41 +6365,45 @@
         </is>
       </c>
       <c r="D27" s="2">
-        <v>4.416666666666668</v>
+        <v>1.9139457023717443</v>
       </c>
       <c r="E27" s="2">
-        <v>4.750000000000009</v>
+        <v>2.0553459914763095</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 その他販管費率（事業化報告3年目）</t>
+          <t xml:space="preserve">ベース事業 役員1人当たり給与支給総額上昇率（設備導入期間）</t>
         </is>
       </c>
       <c r="B28" s="2">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D28" s="2">
-        <v>8.5</v>
-      </c>
-      <c r="E28" s="2">
-        <v>13.5</v>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 その他販管費率（事業化報告3年目）</t>
+          <t xml:space="preserve">ベース事業 常時使用する従業員数の成長率（設備導入期間）</t>
         </is>
       </c>
       <c r="B29" s="2">
-        <v>10.928571428571427</v>
+        <v>4.083333333333339</v>
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
@@ -6347,20 +6411,20 @@
         </is>
       </c>
       <c r="D29" s="2">
-        <v>8.928571428571427</v>
+        <v>3.9166666666666683</v>
       </c>
       <c r="E29" s="2">
-        <v>11.928571428571427</v>
+        <v>4.250000000000009</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">役員1人当たり給与支給総額の年平均上昇率</t>
+          <t xml:space="preserve">ベース事業 その他販管費率改善ポイント（設備導入期間）</t>
         </is>
       </c>
       <c r="B30" s="2">
-        <v>5.380116959064325</v>
+        <v>0</v>
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
@@ -6368,82 +6432,338 @@
         </is>
       </c>
       <c r="D30" s="2">
-        <v>4.263157894736836</v>
+        <v>0</v>
       </c>
       <c r="E30" s="2">
-        <v>6.555555555555557</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">新規投資の耐用年数</t>
+          <t xml:space="preserve">補助事業 売上成長率（基準年度後）</t>
         </is>
       </c>
       <c r="B31" s="2">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D31" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E31" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="D31" s="2">
+        <v>15</v>
+      </c>
+      <c r="E31" s="2">
+        <v>30</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業投資額</t>
+          <t xml:space="preserve">ベース事業 売上成長率（基準年度後）</t>
         </is>
       </c>
       <c r="B32" s="2">
-        <v>23</v>
+        <v>6.257246376811586</v>
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">20億円以上（専門家経費・外注費を除く補助対象経費）</t>
-        </is>
-      </c>
-      <c r="D32" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E32" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D32" s="2">
+        <v>6.076086956521719</v>
+      </c>
+      <c r="E32" s="2">
+        <v>6.438405797101453</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">補助事業 原価率改善ポイント（基準年度後）</t>
+        </is>
+      </c>
+      <c r="B33" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D33" s="2">
+        <v>0</v>
+      </c>
+      <c r="E33" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ベース事業 原価率改善ポイント（基準年度後）</t>
+        </is>
+      </c>
+      <c r="B34" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D34" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E34" s="2">
+        <v>0.5134575569358197</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">補助事業1人当たり給与支給総額の年平均上昇率</t>
+        </is>
+      </c>
+      <c r="B35" s="2">
+        <v>7.000000000000001</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D35" s="2">
+        <v>5</v>
+      </c>
+      <c r="E35" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ベース事業1人当たり給与支給総額の年平均上昇率（基準年度後）</t>
+        </is>
+      </c>
+      <c r="B36" s="2">
+        <v>2.484645846924027</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D36" s="2">
+        <v>2.4139457023717443</v>
+      </c>
+      <c r="E36" s="2">
+        <v>2.5553459914763095</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ベース事業 役員1人当たり給与支給総額上昇率（基準年度後）</t>
+        </is>
+      </c>
+      <c r="B37" s="2">
+        <v>4.5</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">補助事業 常時使用する従業員数の成長率</t>
+        </is>
+      </c>
+      <c r="B38" s="2">
+        <v>4</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D38" s="2">
+        <v>0</v>
+      </c>
+      <c r="E38" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ベース事業 常時使用する従業員数の成長率（基準年度後）</t>
+        </is>
+      </c>
+      <c r="B39" s="2">
+        <v>4.583333333333338</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D39" s="2">
+        <v>4.416666666666668</v>
+      </c>
+      <c r="E39" s="2">
+        <v>4.750000000000009</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">補助事業 その他販管費率（事業化報告3年目）</t>
+        </is>
+      </c>
+      <c r="B40" s="2">
+        <v>11</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D40" s="2">
+        <v>8.5</v>
+      </c>
+      <c r="E40" s="2">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ベース事業 その他販管費率（事業化報告3年目）</t>
+        </is>
+      </c>
+      <c r="B41" s="2">
+        <v>10.928571428571427</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D41" s="2">
+        <v>8.928571428571427</v>
+      </c>
+      <c r="E41" s="2">
+        <v>11.928571428571427</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">役員1人当たり給与支給総額の年平均上昇率</t>
+        </is>
+      </c>
+      <c r="B42" s="2">
+        <v>5.380116959064325</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D42" s="2">
+        <v>4.263157894736836</v>
+      </c>
+      <c r="E42" s="2">
+        <v>6.555555555555557</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">新規投資の耐用年数</t>
+        </is>
+      </c>
+      <c r="B43" s="2">
+        <v>10</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">補助事業投資額</t>
+        </is>
+      </c>
+      <c r="B44" s="2">
+        <v>23</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20億円以上（専門家経費・外注費を除く補助対象経費）</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E44" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">申請補助金額</t>
         </is>
       </c>
-      <c r="B33" s="2">
+      <c r="B45" s="2">
         <v>7.66</v>
       </c>
-      <c r="C33" s="0" t="inlineStr">
+      <c r="C45" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">50億円以下、かつ投資額の1/3以下（現在上限7.66億円）</t>
         </is>
       </c>
-      <c r="D33" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E33" s="0" t="inlineStr">
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E45" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6455,7 +6775,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C259"/>
+  <dimension ref="A1:C295"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="72" customWidth="1"/>
@@ -8480,26 +8800,26 @@
     <row r="135">
       <c r="A135" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherCogsImprovement:0</t>
+          <t xml:space="preserve">driver-range:otherCogsDepreciationShare:0</t>
         </is>
       </c>
       <c r="B135" s="2">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="C135" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherCogsImprovement:1</t>
+          <t xml:space="preserve">driver-range:otherCogsDepreciationShare:1</t>
         </is>
       </c>
       <c r="B136" s="2">
-        <v>0.0051345755693581975</v>
+        <v>1</v>
       </c>
       <c r="C136" s="0" t="inlineStr">
         <is>
@@ -8510,26 +8830,26 @@
     <row r="137">
       <c r="A137" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherCogsImprovementToBase:0</t>
+          <t xml:space="preserve">driver-range:otherCogsImprovement:0</t>
         </is>
       </c>
       <c r="B137" s="2">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="C137" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherCogsImprovementToBase:1</t>
+          <t xml:space="preserve">driver-range:otherCogsImprovement:1</t>
         </is>
       </c>
       <c r="B138" s="2">
-        <v>0.00013457556935819737</v>
+        <v>0.0051345755693581975</v>
       </c>
       <c r="C138" s="0" t="inlineStr">
         <is>
@@ -8540,7 +8860,7 @@
     <row r="139">
       <c r="A139" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherCogsRateWhenSalesZero:0</t>
+          <t xml:space="preserve">driver-range:otherCogsImprovementToBase:0</t>
         </is>
       </c>
       <c r="B139" s="2">
@@ -8555,11 +8875,11 @@
     <row r="140">
       <c r="A140" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherCogsRateWhenSalesZero:1</t>
+          <t xml:space="preserve">driver-range:otherCogsImprovementToBase:1</t>
         </is>
       </c>
       <c r="B140" s="2">
-        <v>0.99</v>
+        <v>0.00013457556935819737</v>
       </c>
       <c r="C140" s="0" t="inlineStr">
         <is>
@@ -8570,26 +8890,26 @@
     <row r="141">
       <c r="A141" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherHeadcountGrowth:0</t>
+          <t xml:space="preserve">driver-range:otherCogsRateWhenSalesZero:0</t>
         </is>
       </c>
       <c r="B141" s="2">
-        <v>0.04416666666666668</v>
+        <v>0</v>
       </c>
       <c r="C141" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherHeadcountGrowth:1</t>
+          <t xml:space="preserve">driver-range:otherCogsRateWhenSalesZero:1</t>
         </is>
       </c>
       <c r="B142" s="2">
-        <v>0.04750000000000009</v>
+        <v>0.99</v>
       </c>
       <c r="C142" s="0" t="inlineStr">
         <is>
@@ -8600,26 +8920,26 @@
     <row r="143">
       <c r="A143" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherHeadcountGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:otherEmployeeSalaryShare:0</t>
         </is>
       </c>
       <c r="B143" s="2">
-        <v>0.03916666666666668</v>
+        <v>0</v>
       </c>
       <c r="C143" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherHeadcountGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:otherEmployeeSalaryShare:1</t>
         </is>
       </c>
       <c r="B144" s="2">
-        <v>0.04250000000000009</v>
+        <v>1</v>
       </c>
       <c r="C144" s="0" t="inlineStr">
         <is>
@@ -8630,26 +8950,26 @@
     <row r="145">
       <c r="A145" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherOfficerPayGrowth:0</t>
+          <t xml:space="preserve">driver-range:otherExtraordinaryRate:0</t>
         </is>
       </c>
       <c r="B145" s="2">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="C145" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherOfficerPayGrowth:1</t>
+          <t xml:space="preserve">driver-range:otherExtraordinaryRate:1</t>
         </is>
       </c>
       <c r="B146" s="2">
-        <v>0.08</v>
+        <v>0.5</v>
       </c>
       <c r="C146" s="0" t="inlineStr">
         <is>
@@ -8660,26 +8980,26 @@
     <row r="147">
       <c r="A147" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherOfficerPayGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowth:0</t>
         </is>
       </c>
       <c r="B147" s="2">
-        <v>0</v>
+        <v>0.04416666666666668</v>
       </c>
       <c r="C147" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherOfficerPayGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowth:1</t>
         </is>
       </c>
       <c r="B148" s="2">
-        <v>0.08</v>
+        <v>0.04750000000000009</v>
       </c>
       <c r="C148" s="0" t="inlineStr">
         <is>
@@ -8690,11 +9010,11 @@
     <row r="149">
       <c r="A149" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherPayGrowth:0</t>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowthToBase:0</t>
         </is>
       </c>
       <c r="B149" s="2">
-        <v>0.024139457023717444</v>
+        <v>0.03916666666666668</v>
       </c>
       <c r="C149" s="0" t="inlineStr">
         <is>
@@ -8705,11 +9025,11 @@
     <row r="150">
       <c r="A150" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherPayGrowth:1</t>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowthToBase:1</t>
         </is>
       </c>
       <c r="B150" s="2">
-        <v>0.025553459914763096</v>
+        <v>0.04250000000000009</v>
       </c>
       <c r="C150" s="0" t="inlineStr">
         <is>
@@ -8720,11 +9040,11 @@
     <row r="151">
       <c r="A151" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherPayGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:otherNonOperatingRate:0</t>
         </is>
       </c>
       <c r="B151" s="2">
-        <v>0.019139457023717443</v>
+        <v>-0.5</v>
       </c>
       <c r="C151" s="0" t="inlineStr">
         <is>
@@ -8735,11 +9055,11 @@
     <row r="152">
       <c r="A152" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherPayGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:otherNonOperatingRate:1</t>
         </is>
       </c>
       <c r="B152" s="2">
-        <v>0.020553459914763095</v>
+        <v>0.5</v>
       </c>
       <c r="C152" s="0" t="inlineStr">
         <is>
@@ -8750,26 +9070,26 @@
     <row r="153">
       <c r="A153" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSalesGrowth:0</t>
+          <t xml:space="preserve">driver-range:otherOfficerCompensationShare:0</t>
         </is>
       </c>
       <c r="B153" s="2">
-        <v>0.06076086956521719</v>
+        <v>0</v>
       </c>
       <c r="C153" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSalesGrowth:1</t>
+          <t xml:space="preserve">driver-range:otherOfficerCompensationShare:1</t>
         </is>
       </c>
       <c r="B154" s="2">
-        <v>0.06438405797101453</v>
+        <v>1</v>
       </c>
       <c r="C154" s="0" t="inlineStr">
         <is>
@@ -8780,26 +9100,26 @@
     <row r="155">
       <c r="A155" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSalesGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:otherOfficerPayGrowth:0</t>
         </is>
       </c>
       <c r="B155" s="2">
-        <v>0.040760869565217184</v>
+        <v>0</v>
       </c>
       <c r="C155" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSalesGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:otherOfficerPayGrowth:1</t>
         </is>
       </c>
       <c r="B156" s="2">
-        <v>0.04438405797101452</v>
+        <v>0.08</v>
       </c>
       <c r="C156" s="0" t="inlineStr">
         <is>
@@ -8810,7 +9130,7 @@
     <row r="157">
       <c r="A157" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSgaImprovementToBase:0</t>
+          <t xml:space="preserve">driver-range:otherOfficerPayGrowthToBase:0</t>
         </is>
       </c>
       <c r="B157" s="2">
@@ -8825,26 +9145,26 @@
     <row r="158">
       <c r="A158" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSgaImprovementToBase:1</t>
+          <t xml:space="preserve">driver-range:otherOfficerPayGrowthToBase:1</t>
         </is>
       </c>
       <c r="B158" s="2">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="C158" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSgaRateEnd:0</t>
+          <t xml:space="preserve">driver-range:otherPayGrowth:0</t>
         </is>
       </c>
       <c r="B159" s="2">
-        <v>0.08928571428571427</v>
+        <v>0.024139457023717444</v>
       </c>
       <c r="C159" s="0" t="inlineStr">
         <is>
@@ -8855,11 +9175,11 @@
     <row r="160">
       <c r="A160" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSgaRateEnd:1</t>
+          <t xml:space="preserve">driver-range:otherPayGrowth:1</t>
         </is>
       </c>
       <c r="B160" s="2">
-        <v>0.11928571428571427</v>
+        <v>0.025553459914763096</v>
       </c>
       <c r="C160" s="0" t="inlineStr">
         <is>
@@ -8870,26 +9190,26 @@
     <row r="161">
       <c r="A161" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsImprovementAfterBase:0</t>
+          <t xml:space="preserve">driver-range:otherPayGrowthToBase:0</t>
         </is>
       </c>
       <c r="B161" s="2">
-        <v>0</v>
+        <v>0.019139457023717443</v>
       </c>
       <c r="C161" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsImprovementAfterBase:1</t>
+          <t xml:space="preserve">driver-range:otherPayGrowthToBase:1</t>
         </is>
       </c>
       <c r="B162" s="2">
-        <v>0.03</v>
+        <v>0.020553459914763095</v>
       </c>
       <c r="C162" s="0" t="inlineStr">
         <is>
@@ -8900,7 +9220,7 @@
     <row r="163">
       <c r="A163" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsImprovementToBase:0</t>
+          <t xml:space="preserve">driver-range:otherResearchDevelopmentRate:0</t>
         </is>
       </c>
       <c r="B163" s="2">
@@ -8915,11 +9235,11 @@
     <row r="164">
       <c r="A164" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsImprovementToBase:1</t>
+          <t xml:space="preserve">driver-range:otherResearchDevelopmentRate:1</t>
         </is>
       </c>
       <c r="B164" s="2">
-        <v>1.6653345369377348e-16</v>
+        <v>0.3</v>
       </c>
       <c r="C164" s="0" t="inlineStr">
         <is>
@@ -8930,26 +9250,26 @@
     <row r="165">
       <c r="A165" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsRateWhenSalesZero:0</t>
+          <t xml:space="preserve">driver-range:otherSalesGrowth:0</t>
         </is>
       </c>
       <c r="B165" s="2">
-        <v>0</v>
+        <v>0.06076086956521719</v>
       </c>
       <c r="C165" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsRateWhenSalesZero:1</t>
+          <t xml:space="preserve">driver-range:otherSalesGrowth:1</t>
         </is>
       </c>
       <c r="B166" s="2">
-        <v>0.99</v>
+        <v>0.06438405797101453</v>
       </c>
       <c r="C166" s="0" t="inlineStr">
         <is>
@@ -8960,26 +9280,26 @@
     <row r="167">
       <c r="A167" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectHeadcountGrowth:0</t>
+          <t xml:space="preserve">driver-range:otherSalesGrowthToBase:0</t>
         </is>
       </c>
       <c r="B167" s="2">
-        <v>0</v>
+        <v>0.040760869565217184</v>
       </c>
       <c r="C167" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectHeadcountGrowth:1</t>
+          <t xml:space="preserve">driver-range:otherSalesGrowthToBase:1</t>
         </is>
       </c>
       <c r="B168" s="2">
-        <v>0.08</v>
+        <v>0.04438405797101452</v>
       </c>
       <c r="C168" s="0" t="inlineStr">
         <is>
@@ -8990,41 +9310,41 @@
     <row r="169">
       <c r="A169" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectHeadcountGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:otherSgaImprovementToBase:0</t>
         </is>
       </c>
       <c r="B169" s="2">
-        <v>0.051169590643274754</v>
+        <v>0</v>
       </c>
       <c r="C169" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectHeadcountGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:otherSgaImprovementToBase:1</t>
         </is>
       </c>
       <c r="B170" s="2">
-        <v>0.05701754385964919</v>
+        <v>0</v>
       </c>
       <c r="C170" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectMarketGrowth:0</t>
+          <t xml:space="preserve">driver-range:otherSgaRateEnd:0</t>
         </is>
       </c>
       <c r="B171" s="2">
-        <v>-0.05</v>
+        <v>0.08928571428571427</v>
       </c>
       <c r="C171" s="0" t="inlineStr">
         <is>
@@ -9035,11 +9355,11 @@
     <row r="172">
       <c r="A172" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectMarketGrowth:1</t>
+          <t xml:space="preserve">driver-range:otherSgaRateEnd:1</t>
         </is>
       </c>
       <c r="B172" s="2">
-        <v>0.3</v>
+        <v>0.11928571428571427</v>
       </c>
       <c r="C172" s="0" t="inlineStr">
         <is>
@@ -9050,26 +9370,26 @@
     <row r="173">
       <c r="A173" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectOfficerPayGrowth:0</t>
+          <t xml:space="preserve">driver-range:projectCogsDepreciationShare:0</t>
         </is>
       </c>
       <c r="B173" s="2">
-        <v>0.04263157894736836</v>
+        <v>0</v>
       </c>
       <c r="C173" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectOfficerPayGrowth:1</t>
+          <t xml:space="preserve">driver-range:projectCogsDepreciationShare:1</t>
         </is>
       </c>
       <c r="B174" s="2">
-        <v>0.06555555555555558</v>
+        <v>1</v>
       </c>
       <c r="C174" s="0" t="inlineStr">
         <is>
@@ -9080,26 +9400,26 @@
     <row r="175">
       <c r="A175" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectOfficerPayGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:projectCogsImprovementAfterBase:0</t>
         </is>
       </c>
       <c r="B175" s="2">
-        <v>0.051169590643274754</v>
+        <v>0</v>
       </c>
       <c r="C175" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectOfficerPayGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:projectCogsImprovementAfterBase:1</t>
         </is>
       </c>
       <c r="B176" s="2">
-        <v>0.05701754385964919</v>
+        <v>0.03</v>
       </c>
       <c r="C176" s="0" t="inlineStr">
         <is>
@@ -9110,26 +9430,26 @@
     <row r="177">
       <c r="A177" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectPayGrowth:0</t>
+          <t xml:space="preserve">driver-range:projectCogsImprovementToBase:0</t>
         </is>
       </c>
       <c r="B177" s="2">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="C177" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectPayGrowth:1</t>
+          <t xml:space="preserve">driver-range:projectCogsImprovementToBase:1</t>
         </is>
       </c>
       <c r="B178" s="2">
-        <v>0.1</v>
+        <v>1.6653345369377348e-16</v>
       </c>
       <c r="C178" s="0" t="inlineStr">
         <is>
@@ -9140,26 +9460,26 @@
     <row r="179">
       <c r="A179" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectPayGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:projectCogsRateWhenSalesZero:0</t>
         </is>
       </c>
       <c r="B179" s="2">
-        <v>0.019325330501846927</v>
+        <v>0</v>
       </c>
       <c r="C179" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectPayGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:projectCogsRateWhenSalesZero:1</t>
         </is>
       </c>
       <c r="B180" s="2">
-        <v>0.020735994183189166</v>
+        <v>0.99</v>
       </c>
       <c r="C180" s="0" t="inlineStr">
         <is>
@@ -9170,26 +9490,26 @@
     <row r="181">
       <c r="A181" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSalesGrowth:0</t>
+          <t xml:space="preserve">driver-range:projectEmployeeSalaryShare:0</t>
         </is>
       </c>
       <c r="B181" s="2">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="C181" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSalesGrowth:1</t>
+          <t xml:space="preserve">driver-range:projectEmployeeSalaryShare:1</t>
         </is>
       </c>
       <c r="B182" s="2">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="C182" s="0" t="inlineStr">
         <is>
@@ -9200,11 +9520,11 @@
     <row r="183">
       <c r="A183" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSalesGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:projectExtraordinaryRate:0</t>
         </is>
       </c>
       <c r="B183" s="2">
-        <v>0.051169590643274754</v>
+        <v>-0.5</v>
       </c>
       <c r="C183" s="0" t="inlineStr">
         <is>
@@ -9215,11 +9535,11 @@
     <row r="184">
       <c r="A184" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSalesGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:projectExtraordinaryRate:1</t>
         </is>
       </c>
       <c r="B184" s="2">
-        <v>0.05701754385964919</v>
+        <v>0.5</v>
       </c>
       <c r="C184" s="0" t="inlineStr">
         <is>
@@ -9230,7 +9550,7 @@
     <row r="185">
       <c r="A185" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSgaImprovementToBase:0</t>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowth:0</t>
         </is>
       </c>
       <c r="B185" s="2">
@@ -9245,26 +9565,26 @@
     <row r="186">
       <c r="A186" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSgaImprovementToBase:1</t>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowth:1</t>
         </is>
       </c>
       <c r="B186" s="2">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="C186" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSgaRateEnd:0</t>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowthToBase:0</t>
         </is>
       </c>
       <c r="B187" s="2">
-        <v>0.08499999999999999</v>
+        <v>0.051169590643274754</v>
       </c>
       <c r="C187" s="0" t="inlineStr">
         <is>
@@ -9275,11 +9595,11 @@
     <row r="188">
       <c r="A188" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSgaRateEnd:1</t>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowthToBase:1</t>
         </is>
       </c>
       <c r="B188" s="2">
-        <v>0.135</v>
+        <v>0.05701754385964919</v>
       </c>
       <c r="C188" s="0" t="inlineStr">
         <is>
@@ -9290,11 +9610,11 @@
     <row r="189">
       <c r="A189" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:subsidy:0</t>
+          <t xml:space="preserve">driver-range:projectMarketGrowth:0</t>
         </is>
       </c>
       <c r="B189" s="2">
-        <v>1</v>
+        <v>-0.05</v>
       </c>
       <c r="C189" s="0" t="inlineStr">
         <is>
@@ -9305,11 +9625,11 @@
     <row r="190">
       <c r="A190" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:subsidy:1</t>
+          <t xml:space="preserve">driver-range:projectMarketGrowth:1</t>
         </is>
       </c>
       <c r="B190" s="2">
-        <v>50</v>
+        <v>0.3</v>
       </c>
       <c r="C190" s="0" t="inlineStr">
         <is>
@@ -9320,11 +9640,11 @@
     <row r="191">
       <c r="A191" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:usefulLife:0</t>
+          <t xml:space="preserve">driver-range:projectNonOperatingRate:0</t>
         </is>
       </c>
       <c r="B191" s="2">
-        <v>5</v>
+        <v>-0.5</v>
       </c>
       <c r="C191" s="0" t="inlineStr">
         <is>
@@ -9335,11 +9655,11 @@
     <row r="192">
       <c r="A192" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:usefulLife:1</t>
+          <t xml:space="preserve">driver-range:projectNonOperatingRate:1</t>
         </is>
       </c>
       <c r="B192" s="2">
-        <v>20</v>
+        <v>0.5</v>
       </c>
       <c r="C192" s="0" t="inlineStr">
         <is>
@@ -9350,26 +9670,26 @@
     <row r="193">
       <c r="A193" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:effectiveTaxRate</t>
+          <t xml:space="preserve">driver-range:projectOfficerCompensationShare:0</t>
         </is>
       </c>
       <c r="B193" s="2">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="C193" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:investment</t>
+          <t xml:space="preserve">driver-range:projectOfficerCompensationShare:1</t>
         </is>
       </c>
       <c r="B194" s="2">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="C194" s="0" t="inlineStr">
         <is>
@@ -9380,11 +9700,11 @@
     <row r="195">
       <c r="A195" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:localBenchmark</t>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowth:0</t>
         </is>
       </c>
       <c r="B195" s="2">
-        <v>23</v>
+        <v>0.04263157894736836</v>
       </c>
       <c r="C195" s="0" t="inlineStr">
         <is>
@@ -9395,11 +9715,11 @@
     <row r="196">
       <c r="A196" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherCogsImprovement</t>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowth:1</t>
         </is>
       </c>
       <c r="B196" s="2">
-        <v>0.005</v>
+        <v>0.06555555555555558</v>
       </c>
       <c r="C196" s="0" t="inlineStr">
         <is>
@@ -9410,26 +9730,26 @@
     <row r="197">
       <c r="A197" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherCogsImprovementToBase</t>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowthToBase:0</t>
         </is>
       </c>
       <c r="B197" s="2">
-        <v>0</v>
+        <v>0.051169590643274754</v>
       </c>
       <c r="C197" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherCogsRateWhenSalesZero</t>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowthToBase:1</t>
         </is>
       </c>
       <c r="B198" s="2">
-        <v>0.68</v>
+        <v>0.05701754385964919</v>
       </c>
       <c r="C198" s="0" t="inlineStr">
         <is>
@@ -9440,11 +9760,11 @@
     <row r="199">
       <c r="A199" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherHeadcountGrowth</t>
+          <t xml:space="preserve">driver-range:projectPayGrowth:0</t>
         </is>
       </c>
       <c r="B199" s="2">
-        <v>0.045833333333333386</v>
+        <v>0.05</v>
       </c>
       <c r="C199" s="0" t="inlineStr">
         <is>
@@ -9455,11 +9775,11 @@
     <row r="200">
       <c r="A200" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherHeadcountGrowthToBase</t>
+          <t xml:space="preserve">driver-range:projectPayGrowth:1</t>
         </is>
       </c>
       <c r="B200" s="2">
-        <v>0.04083333333333339</v>
+        <v>0.1</v>
       </c>
       <c r="C200" s="0" t="inlineStr">
         <is>
@@ -9470,11 +9790,11 @@
     <row r="201">
       <c r="A201" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherOfficerPayGrowth</t>
+          <t xml:space="preserve">driver-range:projectPayGrowthToBase:0</t>
         </is>
       </c>
       <c r="B201" s="2">
-        <v>0.045</v>
+        <v>0.019325330501846927</v>
       </c>
       <c r="C201" s="0" t="inlineStr">
         <is>
@@ -9485,11 +9805,11 @@
     <row r="202">
       <c r="A202" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherOfficerPayGrowthToBase</t>
+          <t xml:space="preserve">driver-range:projectPayGrowthToBase:1</t>
         </is>
       </c>
       <c r="B202" s="2">
-        <v>0.04</v>
+        <v>0.020735994183189166</v>
       </c>
       <c r="C202" s="0" t="inlineStr">
         <is>
@@ -9500,26 +9820,26 @@
     <row r="203">
       <c r="A203" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherPayGrowth</t>
+          <t xml:space="preserve">driver-range:projectResearchDevelopmentRate:0</t>
         </is>
       </c>
       <c r="B203" s="2">
-        <v>0.02484645846924027</v>
+        <v>0</v>
       </c>
       <c r="C203" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherPayGrowthToBase</t>
+          <t xml:space="preserve">driver-range:projectResearchDevelopmentRate:1</t>
         </is>
       </c>
       <c r="B204" s="2">
-        <v>0.01984645846924027</v>
+        <v>0.3</v>
       </c>
       <c r="C204" s="0" t="inlineStr">
         <is>
@@ -9530,11 +9850,11 @@
     <row r="205">
       <c r="A205" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSalesGrowth</t>
+          <t xml:space="preserve">driver-range:projectSalesGrowth:0</t>
         </is>
       </c>
       <c r="B205" s="2">
-        <v>0.06257246376811586</v>
+        <v>0.15</v>
       </c>
       <c r="C205" s="0" t="inlineStr">
         <is>
@@ -9545,11 +9865,11 @@
     <row r="206">
       <c r="A206" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSalesGrowthToBase</t>
+          <t xml:space="preserve">driver-range:projectSalesGrowth:1</t>
         </is>
       </c>
       <c r="B206" s="2">
-        <v>0.042572463768115854</v>
+        <v>0.3</v>
       </c>
       <c r="C206" s="0" t="inlineStr">
         <is>
@@ -9560,26 +9880,26 @@
     <row r="207">
       <c r="A207" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSgaImprovementToBase</t>
+          <t xml:space="preserve">driver-range:projectSalesGrowthToBase:0</t>
         </is>
       </c>
       <c r="B207" s="2">
-        <v>0</v>
+        <v>0.051169590643274754</v>
       </c>
       <c r="C207" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSgaRateEnd</t>
+          <t xml:space="preserve">driver-range:projectSalesGrowthToBase:1</t>
         </is>
       </c>
       <c r="B208" s="2">
-        <v>0.10928571428571428</v>
+        <v>0.05701754385964919</v>
       </c>
       <c r="C208" s="0" t="inlineStr">
         <is>
@@ -9590,41 +9910,41 @@
     <row r="209">
       <c r="A209" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectCogsImprovementAfterBase</t>
+          <t xml:space="preserve">driver-range:projectSgaImprovementToBase:0</t>
         </is>
       </c>
       <c r="B209" s="2">
-        <v>0.015</v>
+        <v>0</v>
       </c>
       <c r="C209" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectCogsImprovementToBase</t>
+          <t xml:space="preserve">driver-range:projectSgaImprovementToBase:1</t>
         </is>
       </c>
       <c r="B210" s="2">
-        <v>5.551115123125783e-17</v>
+        <v>0</v>
       </c>
       <c r="C210" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectCogsRateWhenSalesZero</t>
+          <t xml:space="preserve">driver-range:projectSgaRateEnd:0</t>
         </is>
       </c>
       <c r="B211" s="2">
-        <v>0.68</v>
+        <v>0.08499999999999999</v>
       </c>
       <c r="C211" s="0" t="inlineStr">
         <is>
@@ -9635,11 +9955,11 @@
     <row r="212">
       <c r="A212" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectHeadcountGrowth</t>
+          <t xml:space="preserve">driver-range:projectSgaRateEnd:1</t>
         </is>
       </c>
       <c r="B212" s="2">
-        <v>0.04</v>
+        <v>0.135</v>
       </c>
       <c r="C212" s="0" t="inlineStr">
         <is>
@@ -9650,11 +9970,11 @@
     <row r="213">
       <c r="A213" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectHeadcountGrowthToBase</t>
+          <t xml:space="preserve">driver-range:subsidy:0</t>
         </is>
       </c>
       <c r="B213" s="2">
-        <v>0.05409356725146197</v>
+        <v>1</v>
       </c>
       <c r="C213" s="0" t="inlineStr">
         <is>
@@ -9665,11 +9985,11 @@
     <row r="214">
       <c r="A214" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectMarketGrowth</t>
+          <t xml:space="preserve">driver-range:subsidy:1</t>
         </is>
       </c>
       <c r="B214" s="2">
-        <v>0.05</v>
+        <v>50</v>
       </c>
       <c r="C214" s="0" t="inlineStr">
         <is>
@@ -9680,11 +10000,11 @@
     <row r="215">
       <c r="A215" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectOfficerPayGrowth</t>
+          <t xml:space="preserve">driver-range:usefulLife:0</t>
         </is>
       </c>
       <c r="B215" s="2">
-        <v>0.05380116959064325</v>
+        <v>5</v>
       </c>
       <c r="C215" s="0" t="inlineStr">
         <is>
@@ -9695,11 +10015,11 @@
     <row r="216">
       <c r="A216" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectOfficerPayGrowthToBase</t>
+          <t xml:space="preserve">driver-range:usefulLife:1</t>
         </is>
       </c>
       <c r="B216" s="2">
-        <v>0.05409356725146197</v>
+        <v>20</v>
       </c>
       <c r="C216" s="0" t="inlineStr">
         <is>
@@ -9710,11 +10030,11 @@
     <row r="217">
       <c r="A217" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectPayGrowth</t>
+          <t xml:space="preserve">driver:effectiveTaxRate</t>
         </is>
       </c>
       <c r="B217" s="2">
-        <v>0.07</v>
+        <v>0.3</v>
       </c>
       <c r="C217" s="0" t="inlineStr">
         <is>
@@ -9725,11 +10045,11 @@
     <row r="218">
       <c r="A218" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectPayGrowthToBase</t>
+          <t xml:space="preserve">driver:investment</t>
         </is>
       </c>
       <c r="B218" s="2">
-        <v>0.020030662342518046</v>
+        <v>23</v>
       </c>
       <c r="C218" s="0" t="inlineStr">
         <is>
@@ -9740,11 +10060,11 @@
     <row r="219">
       <c r="A219" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSalesGrowth</t>
+          <t xml:space="preserve">driver:localBenchmark</t>
         </is>
       </c>
       <c r="B219" s="2">
-        <v>0.22</v>
+        <v>23</v>
       </c>
       <c r="C219" s="0" t="inlineStr">
         <is>
@@ -9755,11 +10075,11 @@
     <row r="220">
       <c r="A220" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSalesGrowthToBase</t>
+          <t xml:space="preserve">driver:otherCogsDepreciationShare</t>
         </is>
       </c>
       <c r="B220" s="2">
-        <v>0.05409356725146197</v>
+        <v>0.2</v>
       </c>
       <c r="C220" s="0" t="inlineStr">
         <is>
@@ -9770,41 +10090,41 @@
     <row r="221">
       <c r="A221" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSgaImprovementToBase</t>
+          <t xml:space="preserve">driver:otherCogsImprovement</t>
         </is>
       </c>
       <c r="B221" s="2">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="C221" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSgaRateEnd</t>
+          <t xml:space="preserve">driver:otherCogsImprovementToBase</t>
         </is>
       </c>
       <c r="B222" s="2">
-        <v>0.11</v>
+        <v>0</v>
       </c>
       <c r="C222" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:subsidy</t>
+          <t xml:space="preserve">driver:otherCogsRateWhenSalesZero</t>
         </is>
       </c>
       <c r="B223" s="2">
-        <v>7.66</v>
+        <v>0.68</v>
       </c>
       <c r="C223" s="0" t="inlineStr">
         <is>
@@ -9815,11 +10135,11 @@
     <row r="224">
       <c r="A224" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:usefulLife</t>
+          <t xml:space="preserve">driver:otherEmployeeSalaryShare</t>
         </is>
       </c>
       <c r="B224" s="2">
-        <v>10</v>
+        <v>0.95</v>
       </c>
       <c r="C224" s="0" t="inlineStr">
         <is>
@@ -9830,26 +10150,26 @@
     <row r="225">
       <c r="A225" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2026</t>
+          <t xml:space="preserve">driver:otherExtraordinaryRate</t>
         </is>
       </c>
       <c r="B225" s="2">
-        <v>7.67</v>
+        <v>0</v>
       </c>
       <c r="C225" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2027</t>
+          <t xml:space="preserve">driver:otherHeadcountGrowth</t>
         </is>
       </c>
       <c r="B226" s="2">
-        <v>7.67</v>
+        <v>0.045833333333333386</v>
       </c>
       <c r="C226" s="0" t="inlineStr">
         <is>
@@ -9860,11 +10180,11 @@
     <row r="227">
       <c r="A227" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2028</t>
+          <t xml:space="preserve">driver:otherHeadcountGrowthToBase</t>
         </is>
       </c>
       <c r="B227" s="2">
-        <v>7.66</v>
+        <v>0.04083333333333339</v>
       </c>
       <c r="C227" s="0" t="inlineStr">
         <is>
@@ -9875,56 +10195,56 @@
     <row r="228">
       <c r="A228" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2029</t>
+          <t xml:space="preserve">driver:otherNonOperatingRate</t>
         </is>
       </c>
       <c r="B228" s="2">
-        <v>0</v>
+        <v>-0.005</v>
       </c>
       <c r="C228" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2030</t>
+          <t xml:space="preserve">driver:otherOfficerCompensationShare</t>
         </is>
       </c>
       <c r="B229" s="2">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="C229" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2031</t>
+          <t xml:space="preserve">driver:otherOfficerPayGrowth</t>
         </is>
       </c>
       <c r="B230" s="2">
-        <v>0</v>
+        <v>0.045</v>
       </c>
       <c r="C230" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companyPaySchedule:max</t>
+          <t xml:space="preserve">driver:otherOfficerPayGrowthToBase</t>
         </is>
       </c>
       <c r="B231" s="2">
-        <v>7</v>
+        <v>0.04</v>
       </c>
       <c r="C231" s="0" t="inlineStr">
         <is>
@@ -9935,11 +10255,11 @@
     <row r="232">
       <c r="A232" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companyPaySchedule:value</t>
+          <t xml:space="preserve">driver:otherPayGrowth</t>
         </is>
       </c>
       <c r="B232" s="2">
-        <v>2</v>
+        <v>0.02484645846924027</v>
       </c>
       <c r="C232" s="0" t="inlineStr">
         <is>
@@ -9950,11 +10270,11 @@
     <row r="233">
       <c r="A233" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesCagr:max</t>
+          <t xml:space="preserve">driver:otherPayGrowthToBase</t>
         </is>
       </c>
       <c r="B233" s="2">
-        <v>35</v>
+        <v>0.01984645846924027</v>
       </c>
       <c r="C233" s="0" t="inlineStr">
         <is>
@@ -9965,11 +10285,11 @@
     <row r="234">
       <c r="A234" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesCagr:value</t>
+          <t xml:space="preserve">driver:otherResearchDevelopmentRate</t>
         </is>
       </c>
       <c r="B234" s="2">
-        <v>15</v>
+        <v>0.004</v>
       </c>
       <c r="C234" s="0" t="inlineStr">
         <is>
@@ -9980,11 +10300,11 @@
     <row r="235">
       <c r="A235" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesIncrease:max</t>
+          <t xml:space="preserve">driver:otherSalesGrowth</t>
         </is>
       </c>
       <c r="B235" s="2">
-        <v>252.69</v>
+        <v>0.06257246376811586</v>
       </c>
       <c r="C235" s="0" t="inlineStr">
         <is>
@@ -9995,11 +10315,11 @@
     <row r="236">
       <c r="A236" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesIncrease:value</t>
+          <t xml:space="preserve">driver:otherSalesGrowthToBase</t>
         </is>
       </c>
       <c r="B236" s="2">
-        <v>82.4</v>
+        <v>0.042572463768115854</v>
       </c>
       <c r="C236" s="0" t="inlineStr">
         <is>
@@ -10010,26 +10330,26 @@
     <row r="237">
       <c r="A237" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayCagr:max</t>
+          <t xml:space="preserve">driver:otherSgaImprovementToBase</t>
         </is>
       </c>
       <c r="B237" s="2">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C237" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayCagr:value</t>
+          <t xml:space="preserve">driver:otherSgaRateEnd</t>
         </is>
       </c>
       <c r="B238" s="2">
-        <v>7</v>
+        <v>0.10928571428571428</v>
       </c>
       <c r="C238" s="0" t="inlineStr">
         <is>
@@ -10040,11 +10360,11 @@
     <row r="239">
       <c r="A239" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayIncrease:max</t>
+          <t xml:space="preserve">driver:projectCogsDepreciationShare</t>
         </is>
       </c>
       <c r="B239" s="2">
-        <v>3.74</v>
+        <v>0.25</v>
       </c>
       <c r="C239" s="0" t="inlineStr">
         <is>
@@ -10055,11 +10375,11 @@
     <row r="240">
       <c r="A240" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayIncrease:value</t>
+          <t xml:space="preserve">driver:projectCogsImprovementAfterBase</t>
         </is>
       </c>
       <c r="B240" s="2">
-        <v>2.85</v>
+        <v>0.015</v>
       </c>
       <c r="C240" s="0" t="inlineStr">
         <is>
@@ -10070,11 +10390,11 @@
     <row r="241">
       <c r="A241" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:investmentSalesRatio:max</t>
+          <t xml:space="preserve">driver:projectCogsImprovementToBase</t>
         </is>
       </c>
       <c r="B241" s="2">
-        <v>70</v>
+        <v>5.551115123125783e-17</v>
       </c>
       <c r="C241" s="0" t="inlineStr">
         <is>
@@ -10085,11 +10405,11 @@
     <row r="242">
       <c r="A242" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:investmentSalesRatio:value</t>
+          <t xml:space="preserve">driver:projectCogsRateWhenSalesZero</t>
         </is>
       </c>
       <c r="B242" s="2">
-        <v>15</v>
+        <v>0.68</v>
       </c>
       <c r="C242" s="0" t="inlineStr">
         <is>
@@ -10100,11 +10420,11 @@
     <row r="243">
       <c r="A243" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:laborProductivityCagr:max</t>
+          <t xml:space="preserve">driver:projectEmployeeSalaryShare</t>
         </is>
       </c>
       <c r="B243" s="2">
-        <v>35</v>
+        <v>0.95</v>
       </c>
       <c r="C243" s="0" t="inlineStr">
         <is>
@@ -10115,26 +10435,26 @@
     <row r="244">
       <c r="A244" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:laborProductivityCagr:value</t>
+          <t xml:space="preserve">driver:projectExtraordinaryRate</t>
         </is>
       </c>
       <c r="B244" s="2">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="C244" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:localBenchmark:max</t>
+          <t xml:space="preserve">driver:projectHeadcountGrowth</t>
         </is>
       </c>
       <c r="B245" s="2">
-        <v>40</v>
+        <v>0.04</v>
       </c>
       <c r="C245" s="0" t="inlineStr">
         <is>
@@ -10145,11 +10465,11 @@
     <row r="246">
       <c r="A246" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:localBenchmark:value</t>
+          <t xml:space="preserve">driver:projectHeadcountGrowthToBase</t>
         </is>
       </c>
       <c r="B246" s="2">
-        <v>23</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="C246" s="0" t="inlineStr">
         <is>
@@ -10160,11 +10480,11 @@
     <row r="247">
       <c r="A247" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayCagr:max</t>
+          <t xml:space="preserve">driver:projectMarketGrowth</t>
         </is>
       </c>
       <c r="B247" s="2">
-        <v>10</v>
+        <v>0.05</v>
       </c>
       <c r="C247" s="0" t="inlineStr">
         <is>
@@ -10175,41 +10495,41 @@
     <row r="248">
       <c r="A248" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayCagr:value</t>
+          <t xml:space="preserve">driver:projectNonOperatingRate</t>
         </is>
       </c>
       <c r="B248" s="2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="C248" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayIncrease:value</t>
+          <t xml:space="preserve">driver:projectOfficerCompensationShare</t>
         </is>
       </c>
       <c r="B249" s="2">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="C249" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesCagr:max</t>
+          <t xml:space="preserve">driver:projectOfficerPayGrowth</t>
         </is>
       </c>
       <c r="B250" s="2">
-        <v>35</v>
+        <v>0.05380116959064325</v>
       </c>
       <c r="C250" s="0" t="inlineStr">
         <is>
@@ -10220,11 +10540,11 @@
     <row r="251">
       <c r="A251" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesCagr:value</t>
+          <t xml:space="preserve">driver:projectOfficerPayGrowthToBase</t>
         </is>
       </c>
       <c r="B251" s="2">
-        <v>22</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="C251" s="0" t="inlineStr">
         <is>
@@ -10235,11 +10555,11 @@
     <row r="252">
       <c r="A252" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesIncrease:max</t>
+          <t xml:space="preserve">driver:projectPayGrowth</t>
         </is>
       </c>
       <c r="B252" s="2">
-        <v>136.84</v>
+        <v>0.07</v>
       </c>
       <c r="C252" s="0" t="inlineStr">
         <is>
@@ -10250,11 +10570,11 @@
     <row r="253">
       <c r="A253" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesIncrease:value</t>
+          <t xml:space="preserve">driver:projectPayGrowthToBase</t>
         </is>
       </c>
       <c r="B253" s="2">
-        <v>74.8</v>
+        <v>0.020030662342518046</v>
       </c>
       <c r="C253" s="0" t="inlineStr">
         <is>
@@ -10265,11 +10585,11 @@
     <row r="254">
       <c r="A254" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesShare:max</t>
+          <t xml:space="preserve">driver:projectResearchDevelopmentRate</t>
         </is>
       </c>
       <c r="B254" s="2">
-        <v>95</v>
+        <v>0.005</v>
       </c>
       <c r="C254" s="0" t="inlineStr">
         <is>
@@ -10280,11 +10600,11 @@
     <row r="255">
       <c r="A255" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesShare:value</t>
+          <t xml:space="preserve">driver:projectSalesGrowth</t>
         </is>
       </c>
       <c r="B255" s="2">
-        <v>60</v>
+        <v>0.22</v>
       </c>
       <c r="C255" s="0" t="inlineStr">
         <is>
@@ -10295,11 +10615,11 @@
     <row r="256">
       <c r="A256" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:valueAddedIncrease:max</t>
+          <t xml:space="preserve">driver:projectSalesGrowthToBase</t>
         </is>
       </c>
       <c r="B256" s="2">
-        <v>33.43</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="C256" s="0" t="inlineStr">
         <is>
@@ -10310,26 +10630,26 @@
     <row r="257">
       <c r="A257" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:valueAddedIncrease:value</t>
+          <t xml:space="preserve">driver:projectSgaImprovementToBase</t>
         </is>
       </c>
       <c r="B257" s="2">
-        <v>18.78</v>
+        <v>0</v>
       </c>
       <c r="C257" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:valueAddedSubsidyRatio:max</t>
+          <t xml:space="preserve">driver:projectSgaRateEnd</t>
         </is>
       </c>
       <c r="B258" s="2">
-        <v>350</v>
+        <v>0.11</v>
       </c>
       <c r="C258" s="0" t="inlineStr">
         <is>
@@ -10340,13 +10660,553 @@
     <row r="259">
       <c r="A259" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">driver:subsidy</t>
+        </is>
+      </c>
+      <c r="B259" s="2">
+        <v>7.66</v>
+      </c>
+      <c r="C259" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver:usefulLife</t>
+        </is>
+      </c>
+      <c r="B260" s="2">
+        <v>10</v>
+      </c>
+      <c r="C260" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">future-capex:2026</t>
+        </is>
+      </c>
+      <c r="B261" s="2">
+        <v>7.67</v>
+      </c>
+      <c r="C261" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">future-capex:2027</t>
+        </is>
+      </c>
+      <c r="B262" s="2">
+        <v>7.67</v>
+      </c>
+      <c r="C262" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">future-capex:2028</t>
+        </is>
+      </c>
+      <c r="B263" s="2">
+        <v>7.66</v>
+      </c>
+      <c r="C263" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">future-capex:2029</t>
+        </is>
+      </c>
+      <c r="B264" s="2">
+        <v>0</v>
+      </c>
+      <c r="C264" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">future-capex:2030</t>
+        </is>
+      </c>
+      <c r="B265" s="2">
+        <v>0</v>
+      </c>
+      <c r="C265" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">future-capex:2031</t>
+        </is>
+      </c>
+      <c r="B266" s="2">
+        <v>0</v>
+      </c>
+      <c r="C266" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:companyPaySchedule:max</t>
+        </is>
+      </c>
+      <c r="B267" s="2">
+        <v>7</v>
+      </c>
+      <c r="C267" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:companyPaySchedule:value</t>
+        </is>
+      </c>
+      <c r="B268" s="2">
+        <v>2</v>
+      </c>
+      <c r="C268" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:companySalesCagr:max</t>
+        </is>
+      </c>
+      <c r="B269" s="2">
+        <v>35</v>
+      </c>
+      <c r="C269" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:companySalesCagr:value</t>
+        </is>
+      </c>
+      <c r="B270" s="2">
+        <v>15</v>
+      </c>
+      <c r="C270" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:companySalesIncrease:max</t>
+        </is>
+      </c>
+      <c r="B271" s="2">
+        <v>252.69</v>
+      </c>
+      <c r="C271" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:companySalesIncrease:value</t>
+        </is>
+      </c>
+      <c r="B272" s="2">
+        <v>82.4</v>
+      </c>
+      <c r="C272" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:employeePayCagr:max</t>
+        </is>
+      </c>
+      <c r="B273" s="2">
+        <v>10</v>
+      </c>
+      <c r="C273" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:employeePayCagr:value</t>
+        </is>
+      </c>
+      <c r="B274" s="2">
+        <v>7</v>
+      </c>
+      <c r="C274" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:employeePayIncrease:max</t>
+        </is>
+      </c>
+      <c r="B275" s="2">
+        <v>3.74</v>
+      </c>
+      <c r="C275" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:employeePayIncrease:value</t>
+        </is>
+      </c>
+      <c r="B276" s="2">
+        <v>2.85</v>
+      </c>
+      <c r="C276" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:investmentSalesRatio:max</t>
+        </is>
+      </c>
+      <c r="B277" s="2">
+        <v>70</v>
+      </c>
+      <c r="C277" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:investmentSalesRatio:value</t>
+        </is>
+      </c>
+      <c r="B278" s="2">
+        <v>15</v>
+      </c>
+      <c r="C278" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:laborProductivityCagr:max</t>
+        </is>
+      </c>
+      <c r="B279" s="2">
+        <v>35</v>
+      </c>
+      <c r="C279" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:laborProductivityCagr:value</t>
+        </is>
+      </c>
+      <c r="B280" s="2">
+        <v>21</v>
+      </c>
+      <c r="C280" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:localBenchmark:max</t>
+        </is>
+      </c>
+      <c r="B281" s="2">
+        <v>40</v>
+      </c>
+      <c r="C281" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:localBenchmark:value</t>
+        </is>
+      </c>
+      <c r="B282" s="2">
+        <v>23</v>
+      </c>
+      <c r="C282" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:officerPayCagr:max</t>
+        </is>
+      </c>
+      <c r="B283" s="2">
+        <v>10</v>
+      </c>
+      <c r="C283" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:officerPayCagr:value</t>
+        </is>
+      </c>
+      <c r="B284" s="2">
+        <v>6</v>
+      </c>
+      <c r="C284" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:officerPayIncrease:value</t>
+        </is>
+      </c>
+      <c r="B285" s="2">
+        <v>0</v>
+      </c>
+      <c r="C285" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">明示的な0</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesCagr:max</t>
+        </is>
+      </c>
+      <c r="B286" s="2">
+        <v>35</v>
+      </c>
+      <c r="C286" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesCagr:value</t>
+        </is>
+      </c>
+      <c r="B287" s="2">
+        <v>22</v>
+      </c>
+      <c r="C287" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesIncrease:max</t>
+        </is>
+      </c>
+      <c r="B288" s="2">
+        <v>136.84</v>
+      </c>
+      <c r="C288" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesIncrease:value</t>
+        </is>
+      </c>
+      <c r="B289" s="2">
+        <v>74.8</v>
+      </c>
+      <c r="C289" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesShare:max</t>
+        </is>
+      </c>
+      <c r="B290" s="2">
+        <v>95</v>
+      </c>
+      <c r="C290" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesShare:value</t>
+        </is>
+      </c>
+      <c r="B291" s="2">
+        <v>60</v>
+      </c>
+      <c r="C291" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:valueAddedIncrease:max</t>
+        </is>
+      </c>
+      <c r="B292" s="2">
+        <v>33.43</v>
+      </c>
+      <c r="C292" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:valueAddedIncrease:value</t>
+        </is>
+      </c>
+      <c r="B293" s="2">
+        <v>18.78</v>
+      </c>
+      <c r="C293" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:valueAddedSubsidyRatio:max</t>
+        </is>
+      </c>
+      <c r="B294" s="2">
+        <v>350</v>
+      </c>
+      <c r="C294" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">target:valueAddedSubsidyRatio:value</t>
         </is>
       </c>
-      <c r="B259" s="2">
+      <c r="B295" s="2">
         <v>213</v>
       </c>
-      <c r="C259" s="0" t="inlineStr">
+      <c r="C295" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">入力済み</t>
         </is>
@@ -10374,7 +11234,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4LCJvcmRpbmFyeUluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsInByZVRheEluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsIm5ldEluY29tZSI6Mi43NjQwMDAwMDAwMDAwMDJ9fSx7InllYXIiOjIwMjQsInJvbGUiOiJwcmV2aW91cyIsInByb2plY3QiOnsic2FsZXMiOjc2LCJjb2dzIjo1MS42OCwiZW1wbG95ZWVQYXkiOjUuNTksIm9mZmljZXJQYXkiOjAuMzgsImRlcHJlY2lhdGlvbiI6MS45LCJvdGhlclNnYSI6OS41LCJoZWFkY291bnQiOjk1LCJvZmZpY2VyQ291bnQiOjIsImVtcGxveWVlU2FsYXJ5Ijo1LjMxLCJlbXBsb3llZUJvbnVzIjowLjI4LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjowLjM0LCJvZmZpY2VyQm9udXMiOjAuMDQsImNvZ3NEZXByZWNpYXRpb24iOjAuNDcsInNnYURlcHJlY2lhdGlvbiI6MS40MywicmVzZWFyY2hEZXZlbG9wbWVudCI6MC4zOH0sIm90aGVyIjp7InNhbGVzIjo2Ny4yLCJjb2dzIjo0NS43LCJlbXBsb3llZVBheSI6Ny41NCwib2ZmaWNlclBheSI6MC41OCwiZGVwcmVjaWF0aW9uIjoxLjQ0LCJvdGhlclNnYSI6Ny42OCwiaGVhZGNvdW50IjoxMjUsIm9mZmljZXJDb3VudCI6MywiZW1wbG95ZWVTYWxhcnkiOjcuMTYsImVtcGxveWVlQm9udXMiOjAuMzgsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTIsIm9mZmljZXJCb251cyI6MC4wNiwiY29nc0RlcHJlY2lhdGlvbiI6MC4yOSwic2dhRGVwcmVjaWF0aW9uIjoxLjE1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI5LCJvcmRpbmFyeUluY29tZSI6My45Njk5OTk5OTk5OTk5OTcsInByZVRheEluY29tZSI6My45Njk5OTk5OTk5OTk5OTcsIm5ldEluY29tZSI6Mi43ODE5OTk5OTk5OTk5OTgzfX0seyJ5ZWFyIjoyMDI1LCJyb2xlIjoibGF0ZXN0IiwicHJvamVjdCI6eyJzYWxlcyI6ODAsImNvZ3MiOjU0LjQsImVtcGxveWVlUGF5Ijo2LCJlbXBsb3llZVNhbGFyeSI6NS43LCJlbXBsb3llZUJvbnVzIjowLjMsIm9mZmljZXJQYXkiOjAuNCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNiwib2ZmaWNlckJvbnVzIjowLjA0LCJkZXByZWNpYXRpb24iOjIsImNvZ3NEZXByZWNpYXRpb24iOjAuNSwic2dhRGVwcmVjaWF0aW9uIjoxLjUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuNCwib3RoZXJTZ2EiOjEwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwLCJjb2dzIjo0Ny42LCJlbXBsb3llZVBheSI6OCwiZW1wbG95ZWVTYWxhcnkiOjcuNiwiZW1wbG95ZWVCb251cyI6MC40LCJvZmZpY2VyUGF5IjowLjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTQsIm9mZmljZXJCb251cyI6MC4wNiwiZGVwcmVjaWF0aW9uIjoxLjUsImNvZ3NEZXByZWNpYXRpb24iOjAuMywic2dhRGVwcmVjaWF0aW9uIjoxLjIsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMywib3RoZXJTZ2EiOjgsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjozLjk5OTk5OTk5OTk5OTk5NjQsInByZVRheEluY29tZSI6My45OTk5OTk5OTk5OTk5OTY0LCJuZXRJbmNvbWUiOjIuNzk5OTk5OTk5OTk5OTk3fX1dLCJiYWxhbmNlU2hlZXRzIjpbeyJ5ZWFyIjoyMDIzLCJhc3NldHMiOjEzMiwiY3VycmVudEFzc2V0cyI6NjcsImNhc2giOjI0LCJmaXhlZEFzc2V0cyI6NjUsInRhbmdpYmxlQXNzZXRzIjo1MywiYnVpbGRpbmdzIjoxOSwibWFjaGluZXJ5IjoyNCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjcsInNvZnR3YXJlIjo1LCJsaWFiaWxpdGllcyI6NzUsImN1cnJlbnRMaWFiaWxpdGllcyI6MzksInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozNiwibG9uZ1Rlcm1EZWJ0IjoyOSwibmV0QXNzZXRzIjo1Nywic2hhcmVob2xkZXJFcXVpdHkiOjU0LCJjYXBpdGFsIjoxMCwiY2FwZXgiOjV9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMsImN1cnJlbnRBc3NldHMiOjcyLCJjYXNoIjoyNSwiZml4ZWRBc3NldHMiOjcxLCJ0YW5naWJsZUFzc2V0cyI6NTgsImJ1aWxkaW5ncyI6MjAsIm1hY2hpbmVyeSI6MjgsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo4LCJzb2Z0d2FyZSI6NiwibGlhYmlsaXRpZXMiOjc5LCJjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJzaG9ydFRlcm1EZWJ0IjoxMiwiZml4ZWRMaWFiaWxpdGllcyI6MzgsImxvbmdUZXJtRGVidCI6MzEsIm5ldEFzc2V0cyI6NjQsInNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiY2FwaXRhbCI6MTAsImNhcGV4Ijo4fSx7InllYXIiOjIwMjUsImFzc2V0cyI6MTU2LCJjdXJyZW50QXNzZXRzIjo3OCwiY2FzaCI6MjcsImZpeGVkQXNzZXRzIjo3OCwidGFuZ2libGVBc3NldHMiOjY0LCJidWlsZGluZ3MiOjIyLCJtYWNoaW5lcnkiOjMyLCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6OSwic29mdHdhcmUiOjcsImxpYWJpbGl0aWVzIjo4MywiY3VycmVudExpYWJpbGl0aWVzIjo0Mywic2hvcnRUZXJtRGVidCI6MTEsImZpeGVkTGlhYmlsaXRpZXMiOjQwLCJsb25nVGVybURlYnQiOjMyLCJuZXRBc3NldHMiOjczLCJzaGFyZWhvbGRlckVxdWl0eSI6NzAsImNhcGl0YWwiOjEwLCJjYXBleCI6MTB9XSwiZnV0dXJlQ2FwZXgiOlt7InllYXIiOjIwMjYsInZhbHVlIjo3LjY3fSx7InllYXIiOjIwMjcsInZhbHVlIjo3LjY3fSx7InllYXIiOjIwMjgsInZhbHVlIjo3LjY2fSx7InllYXIiOjIwMjksInZhbHVlIjowfSx7InllYXIiOjIwMzAsInZhbHVlIjowfSx7InllYXIiOjIwMzEsInZhbHVlIjowfV0sImRyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTcyNDYzNzY4MTE1ODYsInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsInByb2plY3RTZ2FSYXRlRW5kIjowLjExLCJvdGhlclNnYVJhdGVFbmQiOjAuMTA5Mjg1NzE0Mjg1NzE0MjgsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6MjMsInN1YnNpZHkiOjcuNjYsImxvY2FsQmVuY2htYXJrIjoyM30sImRyaXZlclJhbmdlcyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjpbLTAuMDUsMC4zXSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6WzAsMC45OV0sIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjpbMCwwLjk5XSwiZWZmZWN0aXZlVGF4UmF0ZSI6WzAsMC42XSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDEuNjY1MzM0NTM2OTM3NzM0OGUtMTZdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkzMjUzMzA1MDE4NDY5MjcsMC4wMjA3MzU5OTQxODMxODkxNjZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlswLjA0MDc2MDg2OTU2NTIxNzE4NCwwLjA0NDM4NDA1Nzk3MTAxNDUyXSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDAwMTM0NTc1NTY5MzU4MTk3MzddLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MTM5NDU3MDIzNzE3NDQzLDAuMDIwNTUzNDU5OTE0NzYzMDk1XSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjAzOTE2NjY2NjY2NjY2NjY4LDAuMDQyNTAwMDAwMDAwMDAwMDldLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbMC4xNSwwLjNdLCJvdGhlclNhbGVzR3Jvd3RoIjpbMC4wNjA3NjA4Njk1NjUyMTcxOSwwLjA2NDM4NDA1Nzk3MTAxNDUzXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMC4wMDUsMC4wMDUxMzQ1NzU1NjkzNTgxOTc1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLjAyNDEzOTQ1NzAyMzcxNzQ0NCwwLjAyNTU1MzQ1OTkxNDc2MzA5Nl0sIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6WzAsMC4wOF0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6WzAuMDQ0MTY2NjY2NjY2NjY2NjgsMC4wNDc1MDAwMDAwMDAwMDAwOV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMC4wODQ5OTk5OTk5OTk5OTk5OSwwLjEzNV0sIm90aGVyU2dhUmF0ZUVuZCI6WzAuMDg5Mjg1NzE0Mjg1NzE0MjcsMC4xMTkyODU3MTQyODU3MTQyN10sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjpbMC4wNDI2MzE1Nzg5NDczNjgzNiwwLjA2NTU1NTU1NTU1NTU1NTU4XSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MTUsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6ODIuNCwibWF4IjoyNTIuNjksInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55UGF5U2NoZWR1bGUiOnsidmFsdWUiOjIsIm1heCI6NywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc1NoYXJlIjp7InZhbHVlIjo2MCwibWF4Ijo5NSwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0NhZ3IiOnsidmFsdWUiOjIyLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjc0LjgsIm1heCI6MTM2Ljg0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MTguNzgsIm1heCI6MzMuNDMsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUNhZ3IiOnsidmFsdWUiOjcsIm1heCI6MTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUluY3JlYXNlIjp7InZhbHVlIjoyLjg1LCJtYXgiOjMuNzQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJpbnZlc3RtZW50U2FsZXNSYXRpbyI6eyJ2YWx1ZSI6MTUsIm1heCI6NzAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvIjp7InZhbHVlIjoyMTMsIm1heCI6MzUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibG9jYWxCZW5jaG1hcmsiOnsidmFsdWUiOjIzLCJtYXgiOjQwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUNhZ3IiOnsidmFsdWUiOjYsIm1heCI6MTAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnsiMjAyOTpvdGhlcjpzYWxlcyI6ODUuMTMsIjIwMjk6cHJvamVjdDo3LTgiOjcuOX0sImZ1dHVyZUlucHV0QmFzaXMiOiJvdGhlciIsImlucHV0VmFsdWVzIjp7ImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xIjoxMzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTMiOjkyLjc1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6MC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMyLjY1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6MC44MiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEwIjowLjA5LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTIiOjExLjY3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjAuNjIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNCI6Mi40NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1IjowLjY0LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTgiOjEwLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTkiOjEwLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjAiOjcuNTEsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yNyI6MjEwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xIjo3MiwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTQiOjIzLjA0LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNiI6Ni43OCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTgiOjUuMTksImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny05IjowLjM2LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTAiOjEuOCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEzIjo5MCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMSI6MTQzLjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0zIjo5Ny4zOCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTQiOjAuNzYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi03IjozNC41MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTkiOjAuODYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMCI6MC4xLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTIiOjEyLjQ3LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTMiOjAuNjYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNCI6Mi41OCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE1IjowLjY3LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTgiOjExLjAxLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTkiOjExLjAxLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjAiOjcuNzEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0yNyI6MjIwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xIjo3NiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0LjMyLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNiI6Ny4wNCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTgiOjUuNTksImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTAiOjEuOSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6MC44LCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTkiOjAuOSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjowLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6Mi43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTUiOjAuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE4IjoxMS4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTkiOjExLjMsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yMCI6Ny45MSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI3IjoyMzAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNCI6MjUuNiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTYiOjcuMywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTgiOjYsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny05IjowLjQsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xMCI6MiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudEFzc2V0cyI6NjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXNoIjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NSwiYmFsYW5jZS1zaGVldDoyMDIzOnRhbmdpYmxlQXNzZXRzIjo1MywiYmFsYW5jZS1zaGVldDoyMDIzOmJ1aWxkaW5ncyI6MTksImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzppbnRhbmdpYmxlQXNzZXRzIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUsImJhbGFuY2Utc2hlZXQ6MjAyMzpsaWFiaWxpdGllcyI6NzUsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50TGlhYmlsaXRpZXMiOjM5LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZExpYWJpbGl0aWVzIjozNiwiYmFsYW5jZS1zaGVldDoyMDIzOmxvbmdUZXJtRGVidCI6MjksImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hhcmVob2xkZXJFcXVpdHkiOjU0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NSwiYmFsYW5jZS1zaGVldDoyMDI0OmFzc2V0cyI6MTQzLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudEFzc2V0cyI6NzIsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNSwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkQXNzZXRzIjo3MSwiYmFsYW5jZS1zaGVldDoyMDI0OnRhbmdpYmxlQXNzZXRzIjo1OCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAsImJhbGFuY2Utc2hlZXQ6MjAyNDptYWNoaW5lcnkiOjI4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c29mdHdhcmUiOjYsImJhbGFuY2Utc2hlZXQ6MjAyNDpsaWFiaWxpdGllcyI6NzksImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZExpYWJpbGl0aWVzIjozOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEsImJhbGFuY2Utc2hlZXQ6MjAyNDpuZXRBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hhcmVob2xkZXJFcXVpdHkiOjYxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBleCI6OCwiYmFsYW5jZS1zaGVldDoyMDI1OmFzc2V0cyI6MTU2LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXNoIjoyNywiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkQXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI1OmJ1aWxkaW5ncyI6MjIsImJhbGFuY2Utc2hlZXQ6MjAyNTptYWNoaW5lcnkiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTppbnRhbmdpYmxlQXNzZXRzIjo5LCJiYWxhbmNlLXNoZWV0OjIwMjU6c29mdHdhcmUiOjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hvcnRUZXJtRGVidCI6MTEsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MCwiYmFsYW5jZS1zaGVldDoyMDI1OmxvbmdUZXJtRGVidCI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpuZXRBc3NldHMiOjczLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBleCI6MTAsImZ1dHVyZS1jYXBleDoyMDI2Ijo3LjY3LCJmdXR1cmUtY2FwZXg6MjAyNyI6Ny42NywiZnV0dXJlLWNhcGV4OjIwMjgiOjcuNjYsImZ1dHVyZS1jYXBleDoyMDI5IjowLCJmdXR1cmUtY2FwZXg6MjAzMCI6MCwiZnV0dXJlLWNhcGV4OjIwMzEiOjAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC45OSwiZHJpdmVyOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvOjEiOjAuOTksImRyaXZlcjplZmZlY3RpdmVUYXhSYXRlIjowLjMsImRyaXZlci1yYW5nZTplZmZlY3RpdmVUYXhSYXRlOjAiOjAsImRyaXZlci1yYW5nZTplZmZlY3RpdmVUYXhSYXRlOjEiOjAuNiwiZHJpdmVyOnByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aFRvQmFzZToxIjowLjA1NzAxNzU0Mzg1OTY0OTE5LCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6NS41NTExMTUxMjMxMjU3ODNlLTE3LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjoxLjY2NTMzNDUzNjkzNzczNDhlLTE2LCJkcml2ZXI6cHJvamVjdFBheUdyb3d0aFRvQmFzZSI6MC4wMjAwMzA2NjIzNDI1MTgwNDYsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDE5MzI1MzMwNTAxODQ2OTI3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZToxIjowLjAyMDczNTk5NDE4MzE4OTE2NiwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZToxIjowLjA1NzAxNzU0Mzg1OTY0OTE5LCJkcml2ZXI6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MCwiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZToxIjowLjA1NzAxNzU0Mzg1OTY0OTE5LCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI1NzI0NjM3NjgxMTU4NTQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjAiOjAuMDQwNzYwODY5NTY1MjE3MTg0LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZToxIjowLjA0NDM4NDA1Nzk3MTAxNDUyLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MC4wMDAxMzQ1NzU1NjkzNTgxOTczNywiZHJpdmVyOm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkxMzk0NTcwMjM3MTc0NDMsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZToxIjowLjAyMDU1MzQ1OTkxNDc2MzA5NSwiZHJpdmVyOm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjAiOjAuMDM5MTY2NjY2NjY2NjY2NjgsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZToxIjowLjA0MjUwMDAwMDAwMDAwMDA5LCJkcml2ZXI6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MCwiZHJpdmVyOnByb2plY3RTYWxlc0dyb3d0aCI6MC4yMiwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDowIjowLjE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjEiOjAuMywiZHJpdmVyOm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTcyNDYzNzY4MTE1ODYsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoOjAiOjAuMDYwNzYwODY5NTY1MjE3MTksImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoOjEiOjAuMDY0Mzg0MDU3OTcxMDE0NTMsImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2U6MSI6MC4wMywiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjAiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MSI6MC4wMDUxMzQ1NzU1NjkzNTgxOTc1LCJkcml2ZXI6cHJvamVjdFBheUdyb3d0aCI6MC4wNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGg6MCI6MC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGg6MSI6MC4xLCJkcml2ZXI6b3RoZXJQYXlHcm93dGgiOjAuMDI0ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDowIjowLjAyNDEzOTQ1NzAyMzcxNzQ0NCwiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjEiOjAuMDI1NTUzNDU5OTE0NzYzMDk2LCJkcml2ZXI6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjowLjA0NSwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjA0LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aDowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aDoxIjowLjA4LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MCI6MC4wNDQxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjEiOjAuMDQ3NTAwMDAwMDAwMDAwMDksImRyaXZlcjpwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjAiOjAuMDg0OTk5OTk5OTk5OTk5OTksImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDoxIjowLjEzNSwiZHJpdmVyOm90aGVyU2dhUmF0ZUVuZCI6MC4xMDkyODU3MTQyODU3MTQyOCwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLjA4OTI4NTcxNDI4NTcxNDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMTE5Mjg1NzE0Mjg1NzE0MjcsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAuMDQyNjMxNTc4OTQ3MzY4MzYsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjA2NTU1NTU1NTU1NTU1NTU4LCJkcml2ZXI6dXNlZnVsTGlmZSI6MTAsImRyaXZlci1yYW5nZTp1c2VmdWxMaWZlOjAiOjUsImRyaXZlci1yYW5nZTp1c2VmdWxMaWZlOjEiOjIwLCJkcml2ZXI6aW52ZXN0bWVudCI6MjMsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjAiOjE1LCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDoxIjoyMDAsImRyaXZlcjpzdWJzaWR5Ijo3LjY2LCJkcml2ZXItcmFuZ2U6c3Vic2lkeTowIjoxLCJkcml2ZXItcmFuZ2U6c3Vic2lkeToxIjo1MCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoxNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjo4Mi40LCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjoyLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOm1heCI6NywidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOnZhbHVlIjo2MCwidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOm1heCI6OTUsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOnZhbHVlIjoyMiwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOnZhbHVlIjo3NC44LCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOnZhbHVlIjoyMSwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2FncjptYXgiOjM1LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOnZhbHVlIjoxOC43OCwidGFyZ2V0OmVtcGxveWVlUGF5Q2Fncjp2YWx1ZSI6NywidGFyZ2V0OmVtcGxveWVlUGF5Q2FncjptYXgiOjEwLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlJbmNyZWFzZTp2YWx1ZSI6Mi44NSwidGFyZ2V0OmludmVzdG1lbnRTYWxlc1JhdGlvOnZhbHVlIjoxNSwidGFyZ2V0OmludmVzdG1lbnRTYWxlc1JhdGlvOm1heCI6NzAsInRhcmdldDp2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvOnZhbHVlIjoyMTMsInRhcmdldDp2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvOm1heCI6MzUwLCJ0YXJnZXQ6bG9jYWxCZW5jaG1hcms6dmFsdWUiOjIzLCJ0YXJnZXQ6bG9jYWxCZW5jaG1hcms6bWF4Ijo0MCwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOnZhbHVlIjo2LCJ0YXJnZXQ6b2ZmaWNlclBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0Om9mZmljZXJQYXlJbmNyZWFzZTp2YWx1ZSI6MCwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOm1heCI6MjUyLjY5LCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6bWF4IjoxMzYuODQsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6bWF4IjozMy40MywidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6bWF4IjozLjc0fSwibWV0cmljR3JvdXBCYXNlcyI6eyJjb21wYW55U2FsZXMiOiJyYXRlIiwicHJvamVjdFNhbGVzIjoicmF0ZSIsImxhYm9yUHJvZHVjdGl2aXR5IjoicmF0ZSIsImVtcGxveWVlUGF5IjoicmF0ZSJ9LCJhcHBsaWNhdGlvbkNhdGVnb3J5IjoiZ2VuZXJhbCIsImFkanVzdGVkRHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZWZmZWN0aXZlVGF4UmF0ZSI6MC4zLCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MTA1OTU3NjAyMzM5MTYsInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjEuMTc0MTg2NDkxMDY0NDY2ZS0xNiwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6MC4wMTk5ODIxMzU1MTE4Nzk4NzMsInByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDU0MDYzOTAxMjQ5NzIyOTM0LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDEyMDQ1MTMzMzE1NzYzLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjYwNTUxNjI3MzAwNTI3LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODgxMzY3NTAwOTE3MTE3LCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDYwOTM1Mzk0MzcxNzg1NSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyMDIyNDg3MjE2OTQ2NjczLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU2NTE3ODU5NDUyMTc5LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNDk5MDQ4MTM0MTI2NTU1LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDg5MDA2MjI5OTc1MDgwMSwib3RoZXJQYXlHcm93dGgiOjAuMDI0ODg3NzYxNzEwMzMzMDMsIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6MC4wNDUsInByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDI5MDQ1NDgyMzk3MjA1MDU1LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU3ODQ4MTQ3MzIzMDg2NjUsInByb2plY3RTZ2FSYXRlRW5kIjowLjEwOTkzMTgwOTE2NDg0ODI0LCJvdGhlclNnYVJhdGVFbmQiOjAuMTA5MjcyNTg5ODcyMTI4MjMsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1Mzc3ODA1NzYyODcxNjMyLCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6MjMsInN1YnNpZHkiOjcuNjYsImxvY2FsQmVuY2htYXJrIjoyM319</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4LCJvcmRpbmFyeUluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsInByZVRheEluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsIm5ldEluY29tZSI6Ny41MX19LHsieWVhciI6MjAyNCwicm9sZSI6InByZXZpb3VzIiwicHJvamVjdCI6eyJzYWxlcyI6NzYsImNvZ3MiOjUxLjY4LCJlbXBsb3llZVBheSI6NS41OSwib2ZmaWNlclBheSI6MC4zOCwiZGVwcmVjaWF0aW9uIjoxLjksIm90aGVyU2dhIjo5LjUsImhlYWRjb3VudCI6OTUsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjUuMzEsImVtcGxveWVlQm9udXMiOjAuMjgsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzQsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40Nywic2dhRGVwcmVjaWF0aW9uIjoxLjQzLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM4fSwib3RoZXIiOnsic2FsZXMiOjY3LjIsImNvZ3MiOjQ1LjcsImVtcGxveWVlUGF5Ijo3LjU0LCJvZmZpY2VyUGF5IjowLjU4LCJkZXByZWNpYXRpb24iOjEuNDQsIm90aGVyU2dhIjo3LjY4LCJoZWFkY291bnQiOjEyNSwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ny4xNiwiZW1wbG95ZWVCb251cyI6MC4zOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41Miwib2ZmaWNlckJvbnVzIjowLjA2LCJjb2dzRGVwcmVjaWF0aW9uIjowLjI5LCJzZ2FEZXByZWNpYXRpb24iOjEuMTUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMjksIm9yZGluYXJ5SW5jb21lIjozLjk2OTk5OTk5OTk5OTk5NywicHJlVGF4SW5jb21lIjozLjk2OTk5OTk5OTk5OTk5NywibmV0SW5jb21lIjo3LjcxfX0seyJ5ZWFyIjoyMDI1LCJyb2xlIjoibGF0ZXN0IiwicHJvamVjdCI6eyJzYWxlcyI6ODAsImNvZ3MiOjU0LjQsImVtcGxveWVlUGF5Ijo2LCJlbXBsb3llZVNhbGFyeSI6NS43LCJlbXBsb3llZUJvbnVzIjowLjMsIm9mZmljZXJQYXkiOjAuNCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNiwib2ZmaWNlckJvbnVzIjowLjA0LCJkZXByZWNpYXRpb24iOjIsImNvZ3NEZXByZWNpYXRpb24iOjAuNSwic2dhRGVwcmVjaWF0aW9uIjoxLjUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuNCwib3RoZXJTZ2EiOjEwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwLCJjb2dzIjo0Ny42LCJlbXBsb3llZVBheSI6OCwiZW1wbG95ZWVTYWxhcnkiOjcuNiwiZW1wbG95ZWVCb251cyI6MC40LCJvZmZpY2VyUGF5IjowLjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTQsIm9mZmljZXJCb251cyI6MC4wNiwiZGVwcmVjaWF0aW9uIjoxLjUsImNvZ3NEZXByZWNpYXRpb24iOjAuMywic2dhRGVwcmVjaWF0aW9uIjoxLjIsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMywib3RoZXJTZ2EiOjgsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjozLjk5OTk5OTk5OTk5OTk5NjQsInByZVRheEluY29tZSI6My45OTk5OTk5OTk5OTk5OTY0LCJuZXRJbmNvbWUiOjcuOTF9fV0sImJhbGFuY2VTaGVldHMiOlt7InllYXIiOjIwMjMsImFzc2V0cyI6MTMyLCJjdXJyZW50QXNzZXRzIjo2NywiY2FzaCI6MjQsImZpeGVkQXNzZXRzIjo2NSwidGFuZ2libGVBc3NldHMiOjUzLCJidWlsZGluZ3MiOjE5LCJtYWNoaW5lcnkiOjI0LCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6Nywic29mdHdhcmUiOjUsImxpYWJpbGl0aWVzIjo3NSwiY3VycmVudExpYWJpbGl0aWVzIjozOSwic2hvcnRUZXJtRGVidCI6MTIsImZpeGVkTGlhYmlsaXRpZXMiOjM2LCJsb25nVGVybURlYnQiOjI5LCJuZXRBc3NldHMiOjU3LCJzaGFyZWhvbGRlckVxdWl0eSI6NTQsImNhcGl0YWwiOjEwLCJjYXBleCI6NX0seyJ5ZWFyIjoyMDI0LCJhc3NldHMiOjE0MywiY3VycmVudEFzc2V0cyI6NzIsImNhc2giOjI1LCJmaXhlZEFzc2V0cyI6NzEsInRhbmdpYmxlQXNzZXRzIjo1OCwiYnVpbGRpbmdzIjoyMCwibWFjaGluZXJ5IjoyOCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjgsInNvZnR3YXJlIjo2LCJsaWFiaWxpdGllcyI6NzksImN1cnJlbnRMaWFiaWxpdGllcyI6NDEsInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozOCwibG9uZ1Rlcm1EZWJ0IjozMSwibmV0QXNzZXRzIjo2NCwic2hhcmVob2xkZXJFcXVpdHkiOjYxLCJjYXBpdGFsIjoxMCwiY2FwZXgiOjh9LHsieWVhciI6MjAyNSwiYXNzZXRzIjoxNTYsImN1cnJlbnRBc3NldHMiOjc4LCJjYXNoIjoyNywiZml4ZWRBc3NldHMiOjc4LCJ0YW5naWJsZUFzc2V0cyI6NjQsImJ1aWxkaW5ncyI6MjIsIm1hY2hpbmVyeSI6MzIsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo5LCJzb2Z0d2FyZSI6NywibGlhYmlsaXRpZXMiOjgzLCJjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJzaG9ydFRlcm1EZWJ0IjoxMSwiZml4ZWRMaWFiaWxpdGllcyI6NDAsImxvbmdUZXJtRGVidCI6MzIsIm5ldEFzc2V0cyI6NzMsInNoYXJlaG9sZGVyRXF1aXR5Ijo3MCwiY2FwaXRhbCI6MTAsImNhcGV4IjoxMH1dLCJmdXR1cmVDYXBleCI6W3sieWVhciI6MjAyNiwidmFsdWUiOjcuNjd9LHsieWVhciI6MjAyNywidmFsdWUiOjcuNjd9LHsieWVhciI6MjAyOCwidmFsdWUiOjcuNjZ9LHsieWVhciI6MjAyOSwidmFsdWUiOjB9LHsieWVhciI6MjAzMCwidmFsdWUiOjB9LHsieWVhciI6MjAzMSwidmFsdWUiOjB9XSwiZHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTcyNDYzNzY4MTE1ODYsInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsInByb2plY3RTZ2FSYXRlRW5kIjowLjExLCJvdGhlclNnYVJhdGVFbmQiOjAuMTA5Mjg1NzE0Mjg1NzE0MjgsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6MjMsInN1YnNpZHkiOjcuNjYsImxvY2FsQmVuY2htYXJrIjoyM30sImRyaXZlclJhbmdlcyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjpbLTAuMDUsMC4zXSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6WzAsMC45OV0sIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjpbMCwwLjk5XSwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOlswLDFdLCJvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOlswLDFdLCJwcm9qZWN0T2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjpbMCwxXSwib3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOlswLDFdLCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjpbMCwxXSwib3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOlswLDFdLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOlswLDAuM10sIm90aGVyUmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOlswLDAuM10sInByb2plY3ROb25PcGVyYXRpbmdSYXRlIjpbLTAuNSwwLjVdLCJvdGhlck5vbk9wZXJhdGluZ1JhdGUiOlstMC41LDAuNV0sInByb2plY3RFeHRyYW9yZGluYXJ5UmF0ZSI6Wy0wLjUsMC41XSwib3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6Wy0wLjUsMC41XSwiZWZmZWN0aXZlVGF4UmF0ZSI6WzAsMC42XSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDEuNjY1MzM0NTM2OTM3NzM0OGUtMTZdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkzMjUzMzA1MDE4NDY5MjcsMC4wMjA3MzU5OTQxODMxODkxNjZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlswLjA0MDc2MDg2OTU2NTIxNzE4NCwwLjA0NDM4NDA1Nzk3MTAxNDUyXSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDAwMTM0NTc1NTY5MzU4MTk3MzddLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MTM5NDU3MDIzNzE3NDQzLDAuMDIwNTUzNDU5OTE0NzYzMDk1XSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjAzOTE2NjY2NjY2NjY2NjY4LDAuMDQyNTAwMDAwMDAwMDAwMDldLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbMC4xNSwwLjNdLCJvdGhlclNhbGVzR3Jvd3RoIjpbMC4wNjA3NjA4Njk1NjUyMTcxOSwwLjA2NDM4NDA1Nzk3MTAxNDUzXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMC4wMDUsMC4wMDUxMzQ1NzU1NjkzNTgxOTc1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLjAyNDEzOTQ1NzAyMzcxNzQ0NCwwLjAyNTU1MzQ1OTkxNDc2MzA5Nl0sIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6WzAsMC4wOF0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6WzAuMDQ0MTY2NjY2NjY2NjY2NjgsMC4wNDc1MDAwMDAwMDAwMDAwOV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMC4wODQ5OTk5OTk5OTk5OTk5OSwwLjEzNV0sIm90aGVyU2dhUmF0ZUVuZCI6WzAuMDg5Mjg1NzE0Mjg1NzE0MjcsMC4xMTkyODU3MTQyODU3MTQyN10sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjpbMC4wNDI2MzE1Nzg5NDczNjgzNiwwLjA2NTU1NTU1NTU1NTU1NTU4XSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MTUsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6ODIuNCwibWF4IjoyNTIuNjksInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55UGF5U2NoZWR1bGUiOnsidmFsdWUiOjIsIm1heCI6NywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc1NoYXJlIjp7InZhbHVlIjo2MCwibWF4Ijo5NSwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0NhZ3IiOnsidmFsdWUiOjIyLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjc0LjgsIm1heCI6MTM2Ljg0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MTguNzgsIm1heCI6MzMuNDMsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUNhZ3IiOnsidmFsdWUiOjcsIm1heCI6MTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUluY3JlYXNlIjp7InZhbHVlIjoyLjg1LCJtYXgiOjMuNzQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJpbnZlc3RtZW50U2FsZXNSYXRpbyI6eyJ2YWx1ZSI6MTUsIm1heCI6NzAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvIjp7InZhbHVlIjoyMTMsIm1heCI6MzUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibG9jYWxCZW5jaG1hcmsiOnsidmFsdWUiOjIzLCJtYXgiOjQwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUNhZ3IiOnsidmFsdWUiOjYsIm1heCI6MTAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnsiMjAyOTpvdGhlcjpzYWxlcyI6ODUuMTMsIjIwMjk6cHJvamVjdDo3LTgiOjcuOX0sImZ1dHVyZUlucHV0QmFzaXMiOiJvdGhlciIsImlucHV0VmFsdWVzIjp7ImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xIjoxMzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTMiOjkyLjc1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6MC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMyLjY1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6MC44MiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEwIjowLjA5LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTIiOjExLjY3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjAuNjIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNCI6Mi40NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1IjowLjY0LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTgiOjEwLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTkiOjEwLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjAiOjcuNTEsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yNyI6MjEwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xIjo3MiwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTQiOjIzLjA0LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNiI6Ni43OCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTgiOjUuMTksImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny05IjowLjM2LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTAiOjEuOCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEzIjo5MCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMSI6MTQzLjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0zIjo5Ny4zOCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTQiOjAuNzYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi03IjozNC41MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTkiOjAuODYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMCI6MC4xLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTIiOjEyLjQ3LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTMiOjAuNjYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNCI6Mi41OCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE1IjowLjY3LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTgiOjExLjAxLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTkiOjExLjAxLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjAiOjcuNzEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0yNyI6MjIwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xIjo3NiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0LjMyLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNiI6Ny4wNCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTgiOjUuNTksImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTAiOjEuOSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6MC44LCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTkiOjAuOSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjowLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6Mi43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTUiOjAuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE4IjoxMS4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTkiOjExLjMsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yMCI6Ny45MSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI3IjoyMzAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNCI6MjUuNiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTYiOjcuMywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTgiOjYsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny05IjowLjQsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xMCI6MiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudEFzc2V0cyI6NjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXNoIjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NSwiYmFsYW5jZS1zaGVldDoyMDIzOnRhbmdpYmxlQXNzZXRzIjo1MywiYmFsYW5jZS1zaGVldDoyMDIzOmJ1aWxkaW5ncyI6MTksImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzppbnRhbmdpYmxlQXNzZXRzIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUsImJhbGFuY2Utc2hlZXQ6MjAyMzpsaWFiaWxpdGllcyI6NzUsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50TGlhYmlsaXRpZXMiOjM5LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZExpYWJpbGl0aWVzIjozNiwiYmFsYW5jZS1zaGVldDoyMDIzOmxvbmdUZXJtRGVidCI6MjksImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hhcmVob2xkZXJFcXVpdHkiOjU0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NSwiYmFsYW5jZS1zaGVldDoyMDI0OmFzc2V0cyI6MTQzLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudEFzc2V0cyI6NzIsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNSwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkQXNzZXRzIjo3MSwiYmFsYW5jZS1zaGVldDoyMDI0OnRhbmdpYmxlQXNzZXRzIjo1OCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAsImJhbGFuY2Utc2hlZXQ6MjAyNDptYWNoaW5lcnkiOjI4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c29mdHdhcmUiOjYsImJhbGFuY2Utc2hlZXQ6MjAyNDpsaWFiaWxpdGllcyI6NzksImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZExpYWJpbGl0aWVzIjozOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEsImJhbGFuY2Utc2hlZXQ6MjAyNDpuZXRBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hhcmVob2xkZXJFcXVpdHkiOjYxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBleCI6OCwiYmFsYW5jZS1zaGVldDoyMDI1OmFzc2V0cyI6MTU2LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXNoIjoyNywiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkQXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI1OmJ1aWxkaW5ncyI6MjIsImJhbGFuY2Utc2hlZXQ6MjAyNTptYWNoaW5lcnkiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTppbnRhbmdpYmxlQXNzZXRzIjo5LCJiYWxhbmNlLXNoZWV0OjIwMjU6c29mdHdhcmUiOjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hvcnRUZXJtRGVidCI6MTEsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MCwiYmFsYW5jZS1zaGVldDoyMDI1OmxvbmdUZXJtRGVidCI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpuZXRBc3NldHMiOjczLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBleCI6MTAsImZ1dHVyZS1jYXBleDoyMDI2Ijo3LjY3LCJmdXR1cmUtY2FwZXg6MjAyNyI6Ny42NywiZnV0dXJlLWNhcGV4OjIwMjgiOjcuNjYsImZ1dHVyZS1jYXBleDoyMDI5IjowLCJmdXR1cmUtY2FwZXg6MjAzMCI6MCwiZnV0dXJlLWNhcGV4OjIwMzEiOjAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC45OSwiZHJpdmVyOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvOjEiOjAuOTksImRyaXZlcjpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwiZHJpdmVyLXJhbmdlOnByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZToxIjoxLCJkcml2ZXI6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJkcml2ZXItcmFuZ2U6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjowLjksImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGU6MSI6MC4zLCJkcml2ZXI6b3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjEiOjAuMywiZHJpdmVyOnByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdE5vbk9wZXJhdGluZ1JhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOnByb2plY3ROb25PcGVyYXRpbmdSYXRlOjEiOjAuNSwiZHJpdmVyOm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJOb25PcGVyYXRpbmdSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpvdGhlck5vbk9wZXJhdGluZ1JhdGU6MSI6MC41LCJkcml2ZXI6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6b3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6ZWZmZWN0aXZlVGF4UmF0ZSI6MC4zLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZTowIjowLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZToxIjowLjYsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjUuNTUxMTE1MTIzMTI1NzgzZS0xNywiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZTowIjowLjAxOTMyNTMzMDUwMTg0NjkyNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA3MzU5OTQxODMxODkxNjYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNTcyNDYzNzY4MTE1ODU0LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZTowIjowLjA0MDc2MDg2OTU2NTIxNzE4NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNDQzODQwNTc5NzEwMTQ1MiwiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjAuMDAwMTM0NTc1NTY5MzU4MTk3MzcsImRyaXZlcjpvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDE5MTM5NDU3MDIzNzE3NDQzLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA1NTM0NTk5MTQ3NjMwOTUsImRyaXZlcjpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZToxIjowLjA4LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjAzOTE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNDI1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MCI6MC4xNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjMsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MCI6MC4wMjQxMzk0NTcwMjM3MTc0NDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDoxIjowLjAyNTU1MzQ1OTkxNDc2MzA5NiwiZHJpdmVyOm90aGVyT2ZmaWNlclBheUdyb3d0aCI6MC4wNDUsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aDoxIjowLjA4LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTgzMzMzMzMzMzMzMzM4NiwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjAiOjAuMDQ0MTY2NjY2NjY2NjY2NjgsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDoxIjowLjA0NzUwMDAwMDAwMDAwMDA5LCJkcml2ZXI6cHJvamVjdFNnYVJhdGVFbmQiOjAuMTEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDowIjowLjA4NDk5OTk5OTk5OTk5OTk5LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MSI6MC4xMzUsImRyaXZlcjpvdGhlclNnYVJhdGVFbmQiOjAuMTA5Mjg1NzE0Mjg1NzE0MjgsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MCI6MC4wODkyODU3MTQyODU3MTQyNywiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDoxIjowLjExOTI4NTcxNDI4NTcxNDI3LCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzODAxMTY5NTkwNjQzMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDowIjowLjA0MjYzMTU3ODk0NzM2ODM2LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MSI6MC4wNjU1NTU1NTU1NTU1NTU1OCwiZHJpdmVyOnVzZWZ1bExpZmUiOjEwLCJkcml2ZXItcmFuZ2U6dXNlZnVsTGlmZTowIjo1LCJkcml2ZXItcmFuZ2U6dXNlZnVsTGlmZToxIjoyMCwiZHJpdmVyOmludmVzdG1lbnQiOjIzLCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDowIjoxNSwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MSI6MjAwLCJkcml2ZXI6c3Vic2lkeSI6Ny42NiwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MCI6MSwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MSI6NTAsImRyaXZlcjpsb2NhbEJlbmNobWFyayI6MjMsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazowIjowLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MSI6MTAwLCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2Fncjp2YWx1ZSI6MTUsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTp2YWx1ZSI6ODIuNCwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTp2YWx1ZSI6MiwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTptYXgiOjcsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTp2YWx1ZSI6NjAsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTptYXgiOjk1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2Fncjp2YWx1ZSI6MjIsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTp2YWx1ZSI6NzQuOCwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2Fncjp2YWx1ZSI6MjEsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6bWF4IjozNSwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTp2YWx1ZSI6MTguNzgsInRhcmdldDplbXBsb3llZVBheUNhZ3I6dmFsdWUiOjcsInRhcmdldDplbXBsb3llZVBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6dmFsdWUiOjIuODUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MTUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTptYXgiOjI1Mi42OSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOm1heCI6MTM2Ljg0LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOm1heCI6MzMuNDMsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOm1heCI6My43NH0sIm1ldHJpY0dyb3VwQmFzZXMiOnsiY29tcGFueVNhbGVzIjoicmF0ZSIsInByb2plY3RTYWxlcyI6InJhdGUiLCJsYWJvclByb2R1Y3Rpdml0eSI6InJhdGUiLCJlbXBsb3llZVBheSI6InJhdGUifSwiYXBwbGljYXRpb25DYXRlZ29yeSI6ImdlbmVyYWwiLCJhZGp1c3RlZERyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsInByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwib3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwicHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yNSwib3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMiwicHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsInByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJvdGhlck5vbk9wZXJhdGluZ1JhdGUiOi0wLjAwNSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjowLCJlZmZlY3RpdmVUYXhSYXRlIjowLjMsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQxMDU5NTc2MDIzMzkxNiwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MS4xNzQxODY0OTEwNjQ0NjZlLTE2LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAxOTk4MjEzNTUxMTg3OTg3MywicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwNjM5MDEyNDk3MjI5MzQsInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MTIwNDUxMzMzMTU3NjMsIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNjA1NTE2MjczMDA1MjcsIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4ODEzNjc1MDA5MTcxMTcsIm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwNjA5MzUzOTQzNzE3ODU1LCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIwMjI0ODcyMTY5NDY2NzMsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTY1MTc4NTk0NTIxNzksInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE0OTkwNDgxMzQxMjY1NTUsIm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwicHJvamVjdFBheUdyb3d0aCI6MC4wODkwMDYyMjk5NzUwODAxLCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4ODc3NjE3MTAzMzMwMywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wMjkwNDU0ODIzOTcyMDUwNTUsIm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTc4NDgxNDczMjMwODY2NSwicHJvamVjdFNnYVJhdGVFbmQiOjAuMTA5OTMxODA5MTY0ODQ4MjQsIm90aGVyU2dhUmF0ZUVuZCI6MC4xMDkyNzI1ODk4NzIxMjgyMywicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzNzc4MDU3NjI4NzE2MzIsInVzZWZ1bExpZmUiOjEwLCJpbnZlc3RtZW50IjoyMywic3Vic2lkeSI6Ny42NiwibG9jYWxCZW5jaG1hcmsiOjIzfX0=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove automatic annual capex allocation
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -5001,17 +5001,17 @@
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.88 %</t>
+          <t xml:space="preserve">全社 0 %</t>
         </is>
       </c>
       <c r="H27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.65 %</t>
+          <t xml:space="preserve">全社 0 %</t>
         </is>
       </c>
       <c r="I27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.43 %</t>
+          <t xml:space="preserve">全社 0 %</t>
         </is>
       </c>
       <c r="J27" s="0" t="inlineStr">
@@ -5063,17 +5063,17 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.49 倍</t>
+          <t xml:space="preserve">全社 0 倍</t>
         </is>
       </c>
       <c r="H28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.47 倍</t>
+          <t xml:space="preserve">全社 0 倍</t>
         </is>
       </c>
       <c r="I28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.45 倍</t>
+          <t xml:space="preserve">全社 0 倍</t>
         </is>
       </c>
       <c r="J28" s="0" t="inlineStr">
@@ -5187,17 +5187,17 @@
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.95 倍</t>
+          <t xml:space="preserve">全社 —</t>
         </is>
       </c>
       <c r="H30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1 倍</t>
+          <t xml:space="preserve">全社 —</t>
         </is>
       </c>
       <c r="I30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.05 倍</t>
+          <t xml:space="preserve">全社 —</t>
         </is>
       </c>
       <c r="J30" s="0" t="inlineStr">
@@ -6697,7 +6697,7 @@
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">新規投資の耐用年数</t>
+          <t xml:space="preserve">新規投資の平均耐用年数（減価償却費の自動予測用・モデル内管理・第6次公式様式外）</t>
         </is>
       </c>
       <c r="B43" s="2">
@@ -6775,7 +6775,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C295"/>
+  <dimension ref="A1:C289"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="72" customWidth="1"/>
@@ -10690,11 +10690,11 @@
     <row r="261">
       <c r="A261" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2026</t>
+          <t xml:space="preserve">target:companyPaySchedule:max</t>
         </is>
       </c>
       <c r="B261" s="2">
-        <v>7.67</v>
+        <v>7</v>
       </c>
       <c r="C261" s="0" t="inlineStr">
         <is>
@@ -10705,11 +10705,11 @@
     <row r="262">
       <c r="A262" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2027</t>
+          <t xml:space="preserve">target:companyPaySchedule:value</t>
         </is>
       </c>
       <c r="B262" s="2">
-        <v>7.67</v>
+        <v>2</v>
       </c>
       <c r="C262" s="0" t="inlineStr">
         <is>
@@ -10720,11 +10720,11 @@
     <row r="263">
       <c r="A263" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2028</t>
+          <t xml:space="preserve">target:companySalesCagr:max</t>
         </is>
       </c>
       <c r="B263" s="2">
-        <v>7.66</v>
+        <v>35</v>
       </c>
       <c r="C263" s="0" t="inlineStr">
         <is>
@@ -10735,56 +10735,56 @@
     <row r="264">
       <c r="A264" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2029</t>
+          <t xml:space="preserve">target:companySalesCagr:value</t>
         </is>
       </c>
       <c r="B264" s="2">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="C264" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2030</t>
+          <t xml:space="preserve">target:companySalesIncrease:max</t>
         </is>
       </c>
       <c r="B265" s="2">
-        <v>0</v>
+        <v>252.69</v>
       </c>
       <c r="C265" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">future-capex:2031</t>
+          <t xml:space="preserve">target:companySalesIncrease:value</t>
         </is>
       </c>
       <c r="B266" s="2">
-        <v>0</v>
+        <v>82.4</v>
       </c>
       <c r="C266" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companyPaySchedule:max</t>
+          <t xml:space="preserve">target:employeePayCagr:max</t>
         </is>
       </c>
       <c r="B267" s="2">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C267" s="0" t="inlineStr">
         <is>
@@ -10795,11 +10795,11 @@
     <row r="268">
       <c r="A268" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companyPaySchedule:value</t>
+          <t xml:space="preserve">target:employeePayCagr:value</t>
         </is>
       </c>
       <c r="B268" s="2">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C268" s="0" t="inlineStr">
         <is>
@@ -10810,11 +10810,11 @@
     <row r="269">
       <c r="A269" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesCagr:max</t>
+          <t xml:space="preserve">target:employeePayIncrease:max</t>
         </is>
       </c>
       <c r="B269" s="2">
-        <v>35</v>
+        <v>3.74</v>
       </c>
       <c r="C269" s="0" t="inlineStr">
         <is>
@@ -10825,11 +10825,11 @@
     <row r="270">
       <c r="A270" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesCagr:value</t>
+          <t xml:space="preserve">target:employeePayIncrease:value</t>
         </is>
       </c>
       <c r="B270" s="2">
-        <v>15</v>
+        <v>2.85</v>
       </c>
       <c r="C270" s="0" t="inlineStr">
         <is>
@@ -10840,11 +10840,11 @@
     <row r="271">
       <c r="A271" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesIncrease:max</t>
+          <t xml:space="preserve">target:investmentSalesRatio:max</t>
         </is>
       </c>
       <c r="B271" s="2">
-        <v>252.69</v>
+        <v>70</v>
       </c>
       <c r="C271" s="0" t="inlineStr">
         <is>
@@ -10855,11 +10855,11 @@
     <row r="272">
       <c r="A272" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesIncrease:value</t>
+          <t xml:space="preserve">target:investmentSalesRatio:value</t>
         </is>
       </c>
       <c r="B272" s="2">
-        <v>82.4</v>
+        <v>15</v>
       </c>
       <c r="C272" s="0" t="inlineStr">
         <is>
@@ -10870,11 +10870,11 @@
     <row r="273">
       <c r="A273" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayCagr:max</t>
+          <t xml:space="preserve">target:laborProductivityCagr:max</t>
         </is>
       </c>
       <c r="B273" s="2">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="C273" s="0" t="inlineStr">
         <is>
@@ -10885,11 +10885,11 @@
     <row r="274">
       <c r="A274" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayCagr:value</t>
+          <t xml:space="preserve">target:laborProductivityCagr:value</t>
         </is>
       </c>
       <c r="B274" s="2">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C274" s="0" t="inlineStr">
         <is>
@@ -10900,11 +10900,11 @@
     <row r="275">
       <c r="A275" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayIncrease:max</t>
+          <t xml:space="preserve">target:localBenchmark:max</t>
         </is>
       </c>
       <c r="B275" s="2">
-        <v>3.74</v>
+        <v>40</v>
       </c>
       <c r="C275" s="0" t="inlineStr">
         <is>
@@ -10915,11 +10915,11 @@
     <row r="276">
       <c r="A276" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayIncrease:value</t>
+          <t xml:space="preserve">target:localBenchmark:value</t>
         </is>
       </c>
       <c r="B276" s="2">
-        <v>2.85</v>
+        <v>23</v>
       </c>
       <c r="C276" s="0" t="inlineStr">
         <is>
@@ -10930,11 +10930,11 @@
     <row r="277">
       <c r="A277" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:investmentSalesRatio:max</t>
+          <t xml:space="preserve">target:officerPayCagr:max</t>
         </is>
       </c>
       <c r="B277" s="2">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="C277" s="0" t="inlineStr">
         <is>
@@ -10945,11 +10945,11 @@
     <row r="278">
       <c r="A278" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:investmentSalesRatio:value</t>
+          <t xml:space="preserve">target:officerPayCagr:value</t>
         </is>
       </c>
       <c r="B278" s="2">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C278" s="0" t="inlineStr">
         <is>
@@ -10960,26 +10960,26 @@
     <row r="279">
       <c r="A279" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:laborProductivityCagr:max</t>
+          <t xml:space="preserve">target:officerPayIncrease:value</t>
         </is>
       </c>
       <c r="B279" s="2">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="C279" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:laborProductivityCagr:value</t>
+          <t xml:space="preserve">target:projectSalesCagr:max</t>
         </is>
       </c>
       <c r="B280" s="2">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="C280" s="0" t="inlineStr">
         <is>
@@ -10990,11 +10990,11 @@
     <row r="281">
       <c r="A281" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:localBenchmark:max</t>
+          <t xml:space="preserve">target:projectSalesCagr:value</t>
         </is>
       </c>
       <c r="B281" s="2">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="C281" s="0" t="inlineStr">
         <is>
@@ -11005,11 +11005,11 @@
     <row r="282">
       <c r="A282" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:localBenchmark:value</t>
+          <t xml:space="preserve">target:projectSalesIncrease:max</t>
         </is>
       </c>
       <c r="B282" s="2">
-        <v>23</v>
+        <v>136.84</v>
       </c>
       <c r="C282" s="0" t="inlineStr">
         <is>
@@ -11020,11 +11020,11 @@
     <row r="283">
       <c r="A283" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayCagr:max</t>
+          <t xml:space="preserve">target:projectSalesIncrease:value</t>
         </is>
       </c>
       <c r="B283" s="2">
-        <v>10</v>
+        <v>74.8</v>
       </c>
       <c r="C283" s="0" t="inlineStr">
         <is>
@@ -11035,11 +11035,11 @@
     <row r="284">
       <c r="A284" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayCagr:value</t>
+          <t xml:space="preserve">target:projectSalesShare:max</t>
         </is>
       </c>
       <c r="B284" s="2">
-        <v>6</v>
+        <v>95</v>
       </c>
       <c r="C284" s="0" t="inlineStr">
         <is>
@@ -11050,26 +11050,26 @@
     <row r="285">
       <c r="A285" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayIncrease:value</t>
+          <t xml:space="preserve">target:projectSalesShare:value</t>
         </is>
       </c>
       <c r="B285" s="2">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="C285" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesCagr:max</t>
+          <t xml:space="preserve">target:valueAddedIncrease:max</t>
         </is>
       </c>
       <c r="B286" s="2">
-        <v>35</v>
+        <v>33.43</v>
       </c>
       <c r="C286" s="0" t="inlineStr">
         <is>
@@ -11080,11 +11080,11 @@
     <row r="287">
       <c r="A287" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesCagr:value</t>
+          <t xml:space="preserve">target:valueAddedIncrease:value</t>
         </is>
       </c>
       <c r="B287" s="2">
-        <v>22</v>
+        <v>18.78</v>
       </c>
       <c r="C287" s="0" t="inlineStr">
         <is>
@@ -11095,11 +11095,11 @@
     <row r="288">
       <c r="A288" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesIncrease:max</t>
+          <t xml:space="preserve">target:valueAddedSubsidyRatio:max</t>
         </is>
       </c>
       <c r="B288" s="2">
-        <v>136.84</v>
+        <v>350</v>
       </c>
       <c r="C288" s="0" t="inlineStr">
         <is>
@@ -11110,103 +11110,13 @@
     <row r="289">
       <c r="A289" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesIncrease:value</t>
+          <t xml:space="preserve">target:valueAddedSubsidyRatio:value</t>
         </is>
       </c>
       <c r="B289" s="2">
-        <v>74.8</v>
+        <v>213</v>
       </c>
       <c r="C289" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">入力済み</t>
-        </is>
-      </c>
-    </row>
-    <row r="290">
-      <c r="A290" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">target:projectSalesShare:max</t>
-        </is>
-      </c>
-      <c r="B290" s="2">
-        <v>95</v>
-      </c>
-      <c r="C290" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">入力済み</t>
-        </is>
-      </c>
-    </row>
-    <row r="291">
-      <c r="A291" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">target:projectSalesShare:value</t>
-        </is>
-      </c>
-      <c r="B291" s="2">
-        <v>60</v>
-      </c>
-      <c r="C291" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">入力済み</t>
-        </is>
-      </c>
-    </row>
-    <row r="292">
-      <c r="A292" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">target:valueAddedIncrease:max</t>
-        </is>
-      </c>
-      <c r="B292" s="2">
-        <v>33.43</v>
-      </c>
-      <c r="C292" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">入力済み</t>
-        </is>
-      </c>
-    </row>
-    <row r="293">
-      <c r="A293" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">target:valueAddedIncrease:value</t>
-        </is>
-      </c>
-      <c r="B293" s="2">
-        <v>18.78</v>
-      </c>
-      <c r="C293" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">入力済み</t>
-        </is>
-      </c>
-    </row>
-    <row r="294">
-      <c r="A294" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">target:valueAddedSubsidyRatio:max</t>
-        </is>
-      </c>
-      <c r="B294" s="2">
-        <v>350</v>
-      </c>
-      <c r="C294" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">入力済み</t>
-        </is>
-      </c>
-    </row>
-    <row r="295">
-      <c r="A295" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">target:valueAddedSubsidyRatio:value</t>
-        </is>
-      </c>
-      <c r="B295" s="2">
-        <v>213</v>
-      </c>
-      <c r="C295" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">入力済み</t>
         </is>
@@ -11234,7 +11144,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4LCJvcmRpbmFyeUluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsInByZVRheEluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsIm5ldEluY29tZSI6Ny41MX19LHsieWVhciI6MjAyNCwicm9sZSI6InByZXZpb3VzIiwicHJvamVjdCI6eyJzYWxlcyI6NzYsImNvZ3MiOjUxLjY4LCJlbXBsb3llZVBheSI6NS41OSwib2ZmaWNlclBheSI6MC4zOCwiZGVwcmVjaWF0aW9uIjoxLjksIm90aGVyU2dhIjo5LjUsImhlYWRjb3VudCI6OTUsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjUuMzEsImVtcGxveWVlQm9udXMiOjAuMjgsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzQsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40Nywic2dhRGVwcmVjaWF0aW9uIjoxLjQzLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM4fSwib3RoZXIiOnsic2FsZXMiOjY3LjIsImNvZ3MiOjQ1LjcsImVtcGxveWVlUGF5Ijo3LjU0LCJvZmZpY2VyUGF5IjowLjU4LCJkZXByZWNpYXRpb24iOjEuNDQsIm90aGVyU2dhIjo3LjY4LCJoZWFkY291bnQiOjEyNSwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ny4xNiwiZW1wbG95ZWVCb251cyI6MC4zOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41Miwib2ZmaWNlckJvbnVzIjowLjA2LCJjb2dzRGVwcmVjaWF0aW9uIjowLjI5LCJzZ2FEZXByZWNpYXRpb24iOjEuMTUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMjksIm9yZGluYXJ5SW5jb21lIjozLjk2OTk5OTk5OTk5OTk5NywicHJlVGF4SW5jb21lIjozLjk2OTk5OTk5OTk5OTk5NywibmV0SW5jb21lIjo3LjcxfX0seyJ5ZWFyIjoyMDI1LCJyb2xlIjoibGF0ZXN0IiwicHJvamVjdCI6eyJzYWxlcyI6ODAsImNvZ3MiOjU0LjQsImVtcGxveWVlUGF5Ijo2LCJlbXBsb3llZVNhbGFyeSI6NS43LCJlbXBsb3llZUJvbnVzIjowLjMsIm9mZmljZXJQYXkiOjAuNCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNiwib2ZmaWNlckJvbnVzIjowLjA0LCJkZXByZWNpYXRpb24iOjIsImNvZ3NEZXByZWNpYXRpb24iOjAuNSwic2dhRGVwcmVjaWF0aW9uIjoxLjUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuNCwib3RoZXJTZ2EiOjEwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwLCJjb2dzIjo0Ny42LCJlbXBsb3llZVBheSI6OCwiZW1wbG95ZWVTYWxhcnkiOjcuNiwiZW1wbG95ZWVCb251cyI6MC40LCJvZmZpY2VyUGF5IjowLjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTQsIm9mZmljZXJCb251cyI6MC4wNiwiZGVwcmVjaWF0aW9uIjoxLjUsImNvZ3NEZXByZWNpYXRpb24iOjAuMywic2dhRGVwcmVjaWF0aW9uIjoxLjIsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMywib3RoZXJTZ2EiOjgsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjozLjk5OTk5OTk5OTk5OTk5NjQsInByZVRheEluY29tZSI6My45OTk5OTk5OTk5OTk5OTY0LCJuZXRJbmNvbWUiOjcuOTF9fV0sImJhbGFuY2VTaGVldHMiOlt7InllYXIiOjIwMjMsImFzc2V0cyI6MTMyLCJjdXJyZW50QXNzZXRzIjo2NywiY2FzaCI6MjQsImZpeGVkQXNzZXRzIjo2NSwidGFuZ2libGVBc3NldHMiOjUzLCJidWlsZGluZ3MiOjE5LCJtYWNoaW5lcnkiOjI0LCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6Nywic29mdHdhcmUiOjUsImxpYWJpbGl0aWVzIjo3NSwiY3VycmVudExpYWJpbGl0aWVzIjozOSwic2hvcnRUZXJtRGVidCI6MTIsImZpeGVkTGlhYmlsaXRpZXMiOjM2LCJsb25nVGVybURlYnQiOjI5LCJuZXRBc3NldHMiOjU3LCJzaGFyZWhvbGRlckVxdWl0eSI6NTQsImNhcGl0YWwiOjEwLCJjYXBleCI6NX0seyJ5ZWFyIjoyMDI0LCJhc3NldHMiOjE0MywiY3VycmVudEFzc2V0cyI6NzIsImNhc2giOjI1LCJmaXhlZEFzc2V0cyI6NzEsInRhbmdpYmxlQXNzZXRzIjo1OCwiYnVpbGRpbmdzIjoyMCwibWFjaGluZXJ5IjoyOCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjgsInNvZnR3YXJlIjo2LCJsaWFiaWxpdGllcyI6NzksImN1cnJlbnRMaWFiaWxpdGllcyI6NDEsInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozOCwibG9uZ1Rlcm1EZWJ0IjozMSwibmV0QXNzZXRzIjo2NCwic2hhcmVob2xkZXJFcXVpdHkiOjYxLCJjYXBpdGFsIjoxMCwiY2FwZXgiOjh9LHsieWVhciI6MjAyNSwiYXNzZXRzIjoxNTYsImN1cnJlbnRBc3NldHMiOjc4LCJjYXNoIjoyNywiZml4ZWRBc3NldHMiOjc4LCJ0YW5naWJsZUFzc2V0cyI6NjQsImJ1aWxkaW5ncyI6MjIsIm1hY2hpbmVyeSI6MzIsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo5LCJzb2Z0d2FyZSI6NywibGlhYmlsaXRpZXMiOjgzLCJjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJzaG9ydFRlcm1EZWJ0IjoxMSwiZml4ZWRMaWFiaWxpdGllcyI6NDAsImxvbmdUZXJtRGVidCI6MzIsIm5ldEFzc2V0cyI6NzMsInNoYXJlaG9sZGVyRXF1aXR5Ijo3MCwiY2FwaXRhbCI6MTAsImNhcGV4IjoxMH1dLCJmdXR1cmVDYXBleCI6W3sieWVhciI6MjAyNiwidmFsdWUiOjcuNjd9LHsieWVhciI6MjAyNywidmFsdWUiOjcuNjd9LHsieWVhciI6MjAyOCwidmFsdWUiOjcuNjZ9LHsieWVhciI6MjAyOSwidmFsdWUiOjB9LHsieWVhciI6MjAzMCwidmFsdWUiOjB9LHsieWVhciI6MjAzMSwidmFsdWUiOjB9XSwiZHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTcyNDYzNzY4MTE1ODYsInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsInByb2plY3RTZ2FSYXRlRW5kIjowLjExLCJvdGhlclNnYVJhdGVFbmQiOjAuMTA5Mjg1NzE0Mjg1NzE0MjgsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6MjMsInN1YnNpZHkiOjcuNjYsImxvY2FsQmVuY2htYXJrIjoyM30sImRyaXZlclJhbmdlcyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjpbLTAuMDUsMC4zXSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6WzAsMC45OV0sIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjpbMCwwLjk5XSwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOlswLDFdLCJvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOlswLDFdLCJwcm9qZWN0T2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjpbMCwxXSwib3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOlswLDFdLCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjpbMCwxXSwib3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOlswLDFdLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOlswLDAuM10sIm90aGVyUmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOlswLDAuM10sInByb2plY3ROb25PcGVyYXRpbmdSYXRlIjpbLTAuNSwwLjVdLCJvdGhlck5vbk9wZXJhdGluZ1JhdGUiOlstMC41LDAuNV0sInByb2plY3RFeHRyYW9yZGluYXJ5UmF0ZSI6Wy0wLjUsMC41XSwib3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6Wy0wLjUsMC41XSwiZWZmZWN0aXZlVGF4UmF0ZSI6WzAsMC42XSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDEuNjY1MzM0NTM2OTM3NzM0OGUtMTZdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkzMjUzMzA1MDE4NDY5MjcsMC4wMjA3MzU5OTQxODMxODkxNjZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlswLjA0MDc2MDg2OTU2NTIxNzE4NCwwLjA0NDM4NDA1Nzk3MTAxNDUyXSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDAwMTM0NTc1NTY5MzU4MTk3MzddLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MTM5NDU3MDIzNzE3NDQzLDAuMDIwNTUzNDU5OTE0NzYzMDk1XSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjAzOTE2NjY2NjY2NjY2NjY4LDAuMDQyNTAwMDAwMDAwMDAwMDldLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbMC4xNSwwLjNdLCJvdGhlclNhbGVzR3Jvd3RoIjpbMC4wNjA3NjA4Njk1NjUyMTcxOSwwLjA2NDM4NDA1Nzk3MTAxNDUzXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMC4wMDUsMC4wMDUxMzQ1NzU1NjkzNTgxOTc1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLjAyNDEzOTQ1NzAyMzcxNzQ0NCwwLjAyNTU1MzQ1OTkxNDc2MzA5Nl0sIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6WzAsMC4wOF0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6WzAuMDQ0MTY2NjY2NjY2NjY2NjgsMC4wNDc1MDAwMDAwMDAwMDAwOV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMC4wODQ5OTk5OTk5OTk5OTk5OSwwLjEzNV0sIm90aGVyU2dhUmF0ZUVuZCI6WzAuMDg5Mjg1NzE0Mjg1NzE0MjcsMC4xMTkyODU3MTQyODU3MTQyN10sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjpbMC4wNDI2MzE1Nzg5NDczNjgzNiwwLjA2NTU1NTU1NTU1NTU1NTU4XSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MTUsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6ODIuNCwibWF4IjoyNTIuNjksInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55UGF5U2NoZWR1bGUiOnsidmFsdWUiOjIsIm1heCI6NywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc1NoYXJlIjp7InZhbHVlIjo2MCwibWF4Ijo5NSwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0NhZ3IiOnsidmFsdWUiOjIyLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjc0LjgsIm1heCI6MTM2Ljg0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MTguNzgsIm1heCI6MzMuNDMsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUNhZ3IiOnsidmFsdWUiOjcsIm1heCI6MTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUluY3JlYXNlIjp7InZhbHVlIjoyLjg1LCJtYXgiOjMuNzQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJpbnZlc3RtZW50U2FsZXNSYXRpbyI6eyJ2YWx1ZSI6MTUsIm1heCI6NzAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvIjp7InZhbHVlIjoyMTMsIm1heCI6MzUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibG9jYWxCZW5jaG1hcmsiOnsidmFsdWUiOjIzLCJtYXgiOjQwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUNhZ3IiOnsidmFsdWUiOjYsIm1heCI6MTAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnsiMjAyOTpvdGhlcjpzYWxlcyI6ODUuMTMsIjIwMjk6cHJvamVjdDo3LTgiOjcuOX0sImZ1dHVyZUlucHV0QmFzaXMiOiJvdGhlciIsImlucHV0VmFsdWVzIjp7ImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xIjoxMzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTMiOjkyLjc1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6MC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMyLjY1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6MC44MiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEwIjowLjA5LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTIiOjExLjY3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjAuNjIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNCI6Mi40NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1IjowLjY0LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTgiOjEwLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTkiOjEwLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjAiOjcuNTEsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yNyI6MjEwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xIjo3MiwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTQiOjIzLjA0LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNiI6Ni43OCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTgiOjUuMTksImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny05IjowLjM2LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTAiOjEuOCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEzIjo5MCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMSI6MTQzLjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0zIjo5Ny4zOCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTQiOjAuNzYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi03IjozNC41MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTkiOjAuODYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMCI6MC4xLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTIiOjEyLjQ3LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTMiOjAuNjYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNCI6Mi41OCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE1IjowLjY3LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTgiOjExLjAxLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTkiOjExLjAxLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjAiOjcuNzEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0yNyI6MjIwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xIjo3NiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0LjMyLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNiI6Ny4wNCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTgiOjUuNTksImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTAiOjEuOSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6MC44LCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTkiOjAuOSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjowLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6Mi43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTUiOjAuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE4IjoxMS4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTkiOjExLjMsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yMCI6Ny45MSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI3IjoyMzAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNCI6MjUuNiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTYiOjcuMywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTgiOjYsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny05IjowLjQsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xMCI6MiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudEFzc2V0cyI6NjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXNoIjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NSwiYmFsYW5jZS1zaGVldDoyMDIzOnRhbmdpYmxlQXNzZXRzIjo1MywiYmFsYW5jZS1zaGVldDoyMDIzOmJ1aWxkaW5ncyI6MTksImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzppbnRhbmdpYmxlQXNzZXRzIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUsImJhbGFuY2Utc2hlZXQ6MjAyMzpsaWFiaWxpdGllcyI6NzUsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50TGlhYmlsaXRpZXMiOjM5LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZExpYWJpbGl0aWVzIjozNiwiYmFsYW5jZS1zaGVldDoyMDIzOmxvbmdUZXJtRGVidCI6MjksImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hhcmVob2xkZXJFcXVpdHkiOjU0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NSwiYmFsYW5jZS1zaGVldDoyMDI0OmFzc2V0cyI6MTQzLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudEFzc2V0cyI6NzIsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNSwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkQXNzZXRzIjo3MSwiYmFsYW5jZS1zaGVldDoyMDI0OnRhbmdpYmxlQXNzZXRzIjo1OCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAsImJhbGFuY2Utc2hlZXQ6MjAyNDptYWNoaW5lcnkiOjI4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c29mdHdhcmUiOjYsImJhbGFuY2Utc2hlZXQ6MjAyNDpsaWFiaWxpdGllcyI6NzksImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZExpYWJpbGl0aWVzIjozOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEsImJhbGFuY2Utc2hlZXQ6MjAyNDpuZXRBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hhcmVob2xkZXJFcXVpdHkiOjYxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBleCI6OCwiYmFsYW5jZS1zaGVldDoyMDI1OmFzc2V0cyI6MTU2LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXNoIjoyNywiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkQXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI1OmJ1aWxkaW5ncyI6MjIsImJhbGFuY2Utc2hlZXQ6MjAyNTptYWNoaW5lcnkiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTppbnRhbmdpYmxlQXNzZXRzIjo5LCJiYWxhbmNlLXNoZWV0OjIwMjU6c29mdHdhcmUiOjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hvcnRUZXJtRGVidCI6MTEsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MCwiYmFsYW5jZS1zaGVldDoyMDI1OmxvbmdUZXJtRGVidCI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpuZXRBc3NldHMiOjczLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBleCI6MTAsImZ1dHVyZS1jYXBleDoyMDI2Ijo3LjY3LCJmdXR1cmUtY2FwZXg6MjAyNyI6Ny42NywiZnV0dXJlLWNhcGV4OjIwMjgiOjcuNjYsImZ1dHVyZS1jYXBleDoyMDI5IjowLCJmdXR1cmUtY2FwZXg6MjAzMCI6MCwiZnV0dXJlLWNhcGV4OjIwMzEiOjAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC45OSwiZHJpdmVyOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvOjEiOjAuOTksImRyaXZlcjpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwiZHJpdmVyLXJhbmdlOnByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZToxIjoxLCJkcml2ZXI6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJkcml2ZXItcmFuZ2U6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjowLjksImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGU6MSI6MC4zLCJkcml2ZXI6b3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjEiOjAuMywiZHJpdmVyOnByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdE5vbk9wZXJhdGluZ1JhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOnByb2plY3ROb25PcGVyYXRpbmdSYXRlOjEiOjAuNSwiZHJpdmVyOm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJOb25PcGVyYXRpbmdSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpvdGhlck5vbk9wZXJhdGluZ1JhdGU6MSI6MC41LCJkcml2ZXI6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6b3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6ZWZmZWN0aXZlVGF4UmF0ZSI6MC4zLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZTowIjowLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZToxIjowLjYsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjUuNTUxMTE1MTIzMTI1NzgzZS0xNywiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZTowIjowLjAxOTMyNTMzMDUwMTg0NjkyNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA3MzU5OTQxODMxODkxNjYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNTcyNDYzNzY4MTE1ODU0LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZTowIjowLjA0MDc2MDg2OTU2NTIxNzE4NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNDQzODQwNTc5NzEwMTQ1MiwiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjAuMDAwMTM0NTc1NTY5MzU4MTk3MzcsImRyaXZlcjpvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDE5MTM5NDU3MDIzNzE3NDQzLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA1NTM0NTk5MTQ3NjMwOTUsImRyaXZlcjpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZToxIjowLjA4LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjAzOTE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNDI1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MCI6MC4xNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjMsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MCI6MC4wMjQxMzk0NTcwMjM3MTc0NDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDoxIjowLjAyNTU1MzQ1OTkxNDc2MzA5NiwiZHJpdmVyOm90aGVyT2ZmaWNlclBheUdyb3d0aCI6MC4wNDUsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aDoxIjowLjA4LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTgzMzMzMzMzMzMzMzM4NiwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjAiOjAuMDQ0MTY2NjY2NjY2NjY2NjgsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDoxIjowLjA0NzUwMDAwMDAwMDAwMDA5LCJkcml2ZXI6cHJvamVjdFNnYVJhdGVFbmQiOjAuMTEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDowIjowLjA4NDk5OTk5OTk5OTk5OTk5LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MSI6MC4xMzUsImRyaXZlcjpvdGhlclNnYVJhdGVFbmQiOjAuMTA5Mjg1NzE0Mjg1NzE0MjgsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MCI6MC4wODkyODU3MTQyODU3MTQyNywiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDoxIjowLjExOTI4NTcxNDI4NTcxNDI3LCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzODAxMTY5NTkwNjQzMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDowIjowLjA0MjYzMTU3ODk0NzM2ODM2LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MSI6MC4wNjU1NTU1NTU1NTU1NTU1OCwiZHJpdmVyOnVzZWZ1bExpZmUiOjEwLCJkcml2ZXItcmFuZ2U6dXNlZnVsTGlmZTowIjo1LCJkcml2ZXItcmFuZ2U6dXNlZnVsTGlmZToxIjoyMCwiZHJpdmVyOmludmVzdG1lbnQiOjIzLCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDowIjoxNSwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MSI6MjAwLCJkcml2ZXI6c3Vic2lkeSI6Ny42NiwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MCI6MSwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MSI6NTAsImRyaXZlcjpsb2NhbEJlbmNobWFyayI6MjMsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazowIjowLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MSI6MTAwLCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2Fncjp2YWx1ZSI6MTUsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTp2YWx1ZSI6ODIuNCwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTp2YWx1ZSI6MiwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTptYXgiOjcsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTp2YWx1ZSI6NjAsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTptYXgiOjk1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2Fncjp2YWx1ZSI6MjIsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTp2YWx1ZSI6NzQuOCwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2Fncjp2YWx1ZSI6MjEsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6bWF4IjozNSwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTp2YWx1ZSI6MTguNzgsInRhcmdldDplbXBsb3llZVBheUNhZ3I6dmFsdWUiOjcsInRhcmdldDplbXBsb3llZVBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6dmFsdWUiOjIuODUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MTUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTptYXgiOjI1Mi42OSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOm1heCI6MTM2Ljg0LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOm1heCI6MzMuNDMsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOm1heCI6My43NH0sIm1ldHJpY0dyb3VwQmFzZXMiOnsiY29tcGFueVNhbGVzIjoicmF0ZSIsInByb2plY3RTYWxlcyI6InJhdGUiLCJsYWJvclByb2R1Y3Rpdml0eSI6InJhdGUiLCJlbXBsb3llZVBheSI6InJhdGUifSwiYXBwbGljYXRpb25DYXRlZ29yeSI6ImdlbmVyYWwiLCJhZGp1c3RlZERyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsInByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwib3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwicHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yNSwib3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMiwicHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsInByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJvdGhlck5vbk9wZXJhdGluZ1JhdGUiOi0wLjAwNSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjowLCJlZmZlY3RpdmVUYXhSYXRlIjowLjMsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQxMDU5NTc2MDIzMzkxNiwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MS4xNzQxODY0OTEwNjQ0NjZlLTE2LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAxOTk4MjEzNTUxMTg3OTg3MywicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwNjM5MDEyNDk3MjI5MzQsInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MTIwNDUxMzMzMTU3NjMsIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNjA1NTE2MjczMDA1MjcsIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4ODEzNjc1MDA5MTcxMTcsIm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwNjA5MzUzOTQzNzE3ODU1LCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIwMjI0ODcyMTY5NDY2NzMsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTY1MTc4NTk0NTIxNzksInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE0OTkwNDgxMzQxMjY1NTUsIm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwicHJvamVjdFBheUdyb3d0aCI6MC4wODkwMDYyMjk5NzUwODAxLCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4ODc3NjE3MTAzMzMwMywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wMjkwNDU0ODIzOTcyMDUwNTUsIm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTc4NDgxNDczMjMwODY2NSwicHJvamVjdFNnYVJhdGVFbmQiOjAuMTA5OTMxODA5MTY0ODQ4MjQsIm90aGVyU2dhUmF0ZUVuZCI6MC4xMDkyNzI1ODk4NzIxMjgyMywicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzNzc4MDU3NjI4NzE2MzIsInVzZWZ1bExpZmUiOjEwLCJpbnZlc3RtZW50IjoyMywic3Vic2lkeSI6Ny42NiwibG9jYWxCZW5jaG1hcmsiOjIzfX0=</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4LCJvcmRpbmFyeUluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsInByZVRheEluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsIm5ldEluY29tZSI6Ny41MX19LHsieWVhciI6MjAyNCwicm9sZSI6InByZXZpb3VzIiwicHJvamVjdCI6eyJzYWxlcyI6NzYsImNvZ3MiOjUxLjY4LCJlbXBsb3llZVBheSI6NS41OSwib2ZmaWNlclBheSI6MC4zOCwiZGVwcmVjaWF0aW9uIjoxLjksIm90aGVyU2dhIjo5LjUsImhlYWRjb3VudCI6OTUsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjUuMzEsImVtcGxveWVlQm9udXMiOjAuMjgsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzQsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40Nywic2dhRGVwcmVjaWF0aW9uIjoxLjQzLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM4fSwib3RoZXIiOnsic2FsZXMiOjY3LjIsImNvZ3MiOjQ1LjcsImVtcGxveWVlUGF5Ijo3LjU0LCJvZmZpY2VyUGF5IjowLjU4LCJkZXByZWNpYXRpb24iOjEuNDQsIm90aGVyU2dhIjo3LjY4LCJoZWFkY291bnQiOjEyNSwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ny4xNiwiZW1wbG95ZWVCb251cyI6MC4zOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41Miwib2ZmaWNlckJvbnVzIjowLjA2LCJjb2dzRGVwcmVjaWF0aW9uIjowLjI5LCJzZ2FEZXByZWNpYXRpb24iOjEuMTUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMjksIm9yZGluYXJ5SW5jb21lIjozLjk2OTk5OTk5OTk5OTk5NywicHJlVGF4SW5jb21lIjozLjk2OTk5OTk5OTk5OTk5NywibmV0SW5jb21lIjo3LjcxfX0seyJ5ZWFyIjoyMDI1LCJyb2xlIjoibGF0ZXN0IiwicHJvamVjdCI6eyJzYWxlcyI6ODAsImNvZ3MiOjU0LjQsImVtcGxveWVlUGF5Ijo2LCJlbXBsb3llZVNhbGFyeSI6NS43LCJlbXBsb3llZUJvbnVzIjowLjMsIm9mZmljZXJQYXkiOjAuNCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNiwib2ZmaWNlckJvbnVzIjowLjA0LCJkZXByZWNpYXRpb24iOjIsImNvZ3NEZXByZWNpYXRpb24iOjAuNSwic2dhRGVwcmVjaWF0aW9uIjoxLjUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuNCwib3RoZXJTZ2EiOjEwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwLCJjb2dzIjo0Ny42LCJlbXBsb3llZVBheSI6OCwiZW1wbG95ZWVTYWxhcnkiOjcuNiwiZW1wbG95ZWVCb251cyI6MC40LCJvZmZpY2VyUGF5IjowLjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTQsIm9mZmljZXJCb251cyI6MC4wNiwiZGVwcmVjaWF0aW9uIjoxLjUsImNvZ3NEZXByZWNpYXRpb24iOjAuMywic2dhRGVwcmVjaWF0aW9uIjoxLjIsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMywib3RoZXJTZ2EiOjgsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjozLjk5OTk5OTk5OTk5OTk5NjQsInByZVRheEluY29tZSI6My45OTk5OTk5OTk5OTk5OTY0LCJuZXRJbmNvbWUiOjcuOTF9fV0sImJhbGFuY2VTaGVldHMiOlt7InllYXIiOjIwMjMsImFzc2V0cyI6MTMyLCJjdXJyZW50QXNzZXRzIjo2NywiY2FzaCI6MjQsImZpeGVkQXNzZXRzIjo2NSwidGFuZ2libGVBc3NldHMiOjUzLCJidWlsZGluZ3MiOjE5LCJtYWNoaW5lcnkiOjI0LCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6Nywic29mdHdhcmUiOjUsImxpYWJpbGl0aWVzIjo3NSwiY3VycmVudExpYWJpbGl0aWVzIjozOSwic2hvcnRUZXJtRGVidCI6MTIsImZpeGVkTGlhYmlsaXRpZXMiOjM2LCJsb25nVGVybURlYnQiOjI5LCJuZXRBc3NldHMiOjU3LCJzaGFyZWhvbGRlckVxdWl0eSI6NTQsImNhcGl0YWwiOjEwLCJjYXBleCI6NX0seyJ5ZWFyIjoyMDI0LCJhc3NldHMiOjE0MywiY3VycmVudEFzc2V0cyI6NzIsImNhc2giOjI1LCJmaXhlZEFzc2V0cyI6NzEsInRhbmdpYmxlQXNzZXRzIjo1OCwiYnVpbGRpbmdzIjoyMCwibWFjaGluZXJ5IjoyOCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjgsInNvZnR3YXJlIjo2LCJsaWFiaWxpdGllcyI6NzksImN1cnJlbnRMaWFiaWxpdGllcyI6NDEsInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozOCwibG9uZ1Rlcm1EZWJ0IjozMSwibmV0QXNzZXRzIjo2NCwic2hhcmVob2xkZXJFcXVpdHkiOjYxLCJjYXBpdGFsIjoxMCwiY2FwZXgiOjh9LHsieWVhciI6MjAyNSwiYXNzZXRzIjoxNTYsImN1cnJlbnRBc3NldHMiOjc4LCJjYXNoIjoyNywiZml4ZWRBc3NldHMiOjc4LCJ0YW5naWJsZUFzc2V0cyI6NjQsImJ1aWxkaW5ncyI6MjIsIm1hY2hpbmVyeSI6MzIsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo5LCJzb2Z0d2FyZSI6NywibGlhYmlsaXRpZXMiOjgzLCJjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJzaG9ydFRlcm1EZWJ0IjoxMSwiZml4ZWRMaWFiaWxpdGllcyI6NDAsImxvbmdUZXJtRGVidCI6MzIsIm5ldEFzc2V0cyI6NzMsInNoYXJlaG9sZGVyRXF1aXR5Ijo3MCwiY2FwaXRhbCI6MTAsImNhcGV4IjoxMH1dLCJmdXR1cmVDYXBleCI6W3sieWVhciI6MjAyNiwidmFsdWUiOjB9LHsieWVhciI6MjAyNywidmFsdWUiOjB9LHsieWVhciI6MjAyOCwidmFsdWUiOjB9LHsieWVhciI6MjAyOSwidmFsdWUiOjB9LHsieWVhciI6MjAzMCwidmFsdWUiOjB9LHsieWVhciI6MjAzMSwidmFsdWUiOjB9XSwiZHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTcyNDYzNzY4MTE1ODYsInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsInByb2plY3RTZ2FSYXRlRW5kIjowLjExLCJvdGhlclNnYVJhdGVFbmQiOjAuMTA5Mjg1NzE0Mjg1NzE0MjgsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6MjMsInN1YnNpZHkiOjcuNjYsImxvY2FsQmVuY2htYXJrIjoyM30sImRyaXZlclJhbmdlcyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjpbLTAuMDUsMC4zXSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6WzAsMC45OV0sIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjpbMCwwLjk5XSwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOlswLDFdLCJvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOlswLDFdLCJwcm9qZWN0T2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjpbMCwxXSwib3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOlswLDFdLCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjpbMCwxXSwib3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOlswLDFdLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOlswLDAuM10sIm90aGVyUmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOlswLDAuM10sInByb2plY3ROb25PcGVyYXRpbmdSYXRlIjpbLTAuNSwwLjVdLCJvdGhlck5vbk9wZXJhdGluZ1JhdGUiOlstMC41LDAuNV0sInByb2plY3RFeHRyYW9yZGluYXJ5UmF0ZSI6Wy0wLjUsMC41XSwib3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6Wy0wLjUsMC41XSwiZWZmZWN0aXZlVGF4UmF0ZSI6WzAsMC42XSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDEuNjY1MzM0NTM2OTM3NzM0OGUtMTZdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkzMjUzMzA1MDE4NDY5MjcsMC4wMjA3MzU5OTQxODMxODkxNjZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlswLjA0MDc2MDg2OTU2NTIxNzE4NCwwLjA0NDM4NDA1Nzk3MTAxNDUyXSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDAwMTM0NTc1NTY5MzU4MTk3MzddLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MTM5NDU3MDIzNzE3NDQzLDAuMDIwNTUzNDU5OTE0NzYzMDk1XSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjAzOTE2NjY2NjY2NjY2NjY4LDAuMDQyNTAwMDAwMDAwMDAwMDldLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbMC4xNSwwLjNdLCJvdGhlclNhbGVzR3Jvd3RoIjpbMC4wNjA3NjA4Njk1NjUyMTcxOSwwLjA2NDM4NDA1Nzk3MTAxNDUzXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMC4wMDUsMC4wMDUxMzQ1NzU1NjkzNTgxOTc1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLjAyNDEzOTQ1NzAyMzcxNzQ0NCwwLjAyNTU1MzQ1OTkxNDc2MzA5Nl0sIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6WzAsMC4wOF0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6WzAuMDQ0MTY2NjY2NjY2NjY2NjgsMC4wNDc1MDAwMDAwMDAwMDAwOV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMC4wODQ5OTk5OTk5OTk5OTk5OSwwLjEzNV0sIm90aGVyU2dhUmF0ZUVuZCI6WzAuMDg5Mjg1NzE0Mjg1NzE0MjcsMC4xMTkyODU3MTQyODU3MTQyN10sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjpbMC4wNDI2MzE1Nzg5NDczNjgzNiwwLjA2NTU1NTU1NTU1NTU1NTU4XSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MTUsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6ODIuNCwibWF4IjoyNTIuNjksInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55UGF5U2NoZWR1bGUiOnsidmFsdWUiOjIsIm1heCI6NywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc1NoYXJlIjp7InZhbHVlIjo2MCwibWF4Ijo5NSwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0NhZ3IiOnsidmFsdWUiOjIyLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjc0LjgsIm1heCI6MTM2Ljg0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MTguNzgsIm1heCI6MzMuNDMsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUNhZ3IiOnsidmFsdWUiOjcsIm1heCI6MTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUluY3JlYXNlIjp7InZhbHVlIjoyLjg1LCJtYXgiOjMuNzQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJpbnZlc3RtZW50U2FsZXNSYXRpbyI6eyJ2YWx1ZSI6MTUsIm1heCI6NzAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvIjp7InZhbHVlIjoyMTMsIm1heCI6MzUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibG9jYWxCZW5jaG1hcmsiOnsidmFsdWUiOjIzLCJtYXgiOjQwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUNhZ3IiOnsidmFsdWUiOjYsIm1heCI6MTAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnsiMjAyOTpvdGhlcjpzYWxlcyI6ODUuMTMsIjIwMjk6cHJvamVjdDo3LTgiOjcuOX0sImZ1dHVyZUlucHV0QmFzaXMiOiJvdGhlciIsImlucHV0VmFsdWVzIjp7ImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xIjoxMzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTMiOjkyLjc1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6MC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMyLjY1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6MC44MiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEwIjowLjA5LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTIiOjExLjY3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjAuNjIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNCI6Mi40NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1IjowLjY0LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTgiOjEwLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTkiOjEwLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjAiOjcuNTEsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yNyI6MjEwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xIjo3MiwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTQiOjIzLjA0LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNiI6Ni43OCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTgiOjUuMTksImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny05IjowLjM2LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTAiOjEuOCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEzIjo5MCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMSI6MTQzLjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0zIjo5Ny4zOCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTQiOjAuNzYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi03IjozNC41MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTkiOjAuODYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMCI6MC4xLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTIiOjEyLjQ3LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTMiOjAuNjYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNCI6Mi41OCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE1IjowLjY3LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTgiOjExLjAxLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTkiOjExLjAxLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjAiOjcuNzEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0yNyI6MjIwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xIjo3NiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0LjMyLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNiI6Ny4wNCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTgiOjUuNTksImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTAiOjEuOSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6MC44LCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTkiOjAuOSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjowLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6Mi43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTUiOjAuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE4IjoxMS4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTkiOjExLjMsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yMCI6Ny45MSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI3IjoyMzAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNCI6MjUuNiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTYiOjcuMywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTgiOjYsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny05IjowLjQsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xMCI6MiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudEFzc2V0cyI6NjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXNoIjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NSwiYmFsYW5jZS1zaGVldDoyMDIzOnRhbmdpYmxlQXNzZXRzIjo1MywiYmFsYW5jZS1zaGVldDoyMDIzOmJ1aWxkaW5ncyI6MTksImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzppbnRhbmdpYmxlQXNzZXRzIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUsImJhbGFuY2Utc2hlZXQ6MjAyMzpsaWFiaWxpdGllcyI6NzUsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50TGlhYmlsaXRpZXMiOjM5LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZExpYWJpbGl0aWVzIjozNiwiYmFsYW5jZS1zaGVldDoyMDIzOmxvbmdUZXJtRGVidCI6MjksImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hhcmVob2xkZXJFcXVpdHkiOjU0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NSwiYmFsYW5jZS1zaGVldDoyMDI0OmFzc2V0cyI6MTQzLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudEFzc2V0cyI6NzIsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNSwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkQXNzZXRzIjo3MSwiYmFsYW5jZS1zaGVldDoyMDI0OnRhbmdpYmxlQXNzZXRzIjo1OCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAsImJhbGFuY2Utc2hlZXQ6MjAyNDptYWNoaW5lcnkiOjI4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c29mdHdhcmUiOjYsImJhbGFuY2Utc2hlZXQ6MjAyNDpsaWFiaWxpdGllcyI6NzksImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZExpYWJpbGl0aWVzIjozOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEsImJhbGFuY2Utc2hlZXQ6MjAyNDpuZXRBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hhcmVob2xkZXJFcXVpdHkiOjYxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBleCI6OCwiYmFsYW5jZS1zaGVldDoyMDI1OmFzc2V0cyI6MTU2LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXNoIjoyNywiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkQXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI1OmJ1aWxkaW5ncyI6MjIsImJhbGFuY2Utc2hlZXQ6MjAyNTptYWNoaW5lcnkiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTppbnRhbmdpYmxlQXNzZXRzIjo5LCJiYWxhbmNlLXNoZWV0OjIwMjU6c29mdHdhcmUiOjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hvcnRUZXJtRGVidCI6MTEsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MCwiYmFsYW5jZS1zaGVldDoyMDI1OmxvbmdUZXJtRGVidCI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpuZXRBc3NldHMiOjczLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBleCI6MTAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC45OSwiZHJpdmVyOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvOjEiOjAuOTksImRyaXZlcjpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwiZHJpdmVyLXJhbmdlOnByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZToxIjoxLCJkcml2ZXI6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJkcml2ZXItcmFuZ2U6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjowLjksImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGU6MSI6MC4zLCJkcml2ZXI6b3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjEiOjAuMywiZHJpdmVyOnByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdE5vbk9wZXJhdGluZ1JhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOnByb2plY3ROb25PcGVyYXRpbmdSYXRlOjEiOjAuNSwiZHJpdmVyOm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJOb25PcGVyYXRpbmdSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpvdGhlck5vbk9wZXJhdGluZ1JhdGU6MSI6MC41LCJkcml2ZXI6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6b3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6ZWZmZWN0aXZlVGF4UmF0ZSI6MC4zLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZTowIjowLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZToxIjowLjYsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjUuNTUxMTE1MTIzMTI1NzgzZS0xNywiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZTowIjowLjAxOTMyNTMzMDUwMTg0NjkyNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA3MzU5OTQxODMxODkxNjYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNTcyNDYzNzY4MTE1ODU0LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZTowIjowLjA0MDc2MDg2OTU2NTIxNzE4NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNDQzODQwNTc5NzEwMTQ1MiwiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjAuMDAwMTM0NTc1NTY5MzU4MTk3MzcsImRyaXZlcjpvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDE5MTM5NDU3MDIzNzE3NDQzLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA1NTM0NTk5MTQ3NjMwOTUsImRyaXZlcjpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZToxIjowLjA4LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjAzOTE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNDI1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MCI6MC4xNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjMsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MCI6MC4wMjQxMzk0NTcwMjM3MTc0NDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDoxIjowLjAyNTU1MzQ1OTkxNDc2MzA5NiwiZHJpdmVyOm90aGVyT2ZmaWNlclBheUdyb3d0aCI6MC4wNDUsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aDoxIjowLjA4LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTgzMzMzMzMzMzMzMzM4NiwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjAiOjAuMDQ0MTY2NjY2NjY2NjY2NjgsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDoxIjowLjA0NzUwMDAwMDAwMDAwMDA5LCJkcml2ZXI6cHJvamVjdFNnYVJhdGVFbmQiOjAuMTEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDowIjowLjA4NDk5OTk5OTk5OTk5OTk5LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MSI6MC4xMzUsImRyaXZlcjpvdGhlclNnYVJhdGVFbmQiOjAuMTA5Mjg1NzE0Mjg1NzE0MjgsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MCI6MC4wODkyODU3MTQyODU3MTQyNywiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDoxIjowLjExOTI4NTcxNDI4NTcxNDI3LCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzODAxMTY5NTkwNjQzMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDowIjowLjA0MjYzMTU3ODk0NzM2ODM2LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MSI6MC4wNjU1NTU1NTU1NTU1NTU1OCwiZHJpdmVyOnVzZWZ1bExpZmUiOjEwLCJkcml2ZXItcmFuZ2U6dXNlZnVsTGlmZTowIjo1LCJkcml2ZXItcmFuZ2U6dXNlZnVsTGlmZToxIjoyMCwiZHJpdmVyOmludmVzdG1lbnQiOjIzLCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDowIjoxNSwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MSI6MjAwLCJkcml2ZXI6c3Vic2lkeSI6Ny42NiwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MCI6MSwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MSI6NTAsImRyaXZlcjpsb2NhbEJlbmNobWFyayI6MjMsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazowIjowLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MSI6MTAwLCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2Fncjp2YWx1ZSI6MTUsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTp2YWx1ZSI6ODIuNCwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTp2YWx1ZSI6MiwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTptYXgiOjcsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTp2YWx1ZSI6NjAsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTptYXgiOjk1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2Fncjp2YWx1ZSI6MjIsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTp2YWx1ZSI6NzQuOCwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2Fncjp2YWx1ZSI6MjEsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6bWF4IjozNSwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTp2YWx1ZSI6MTguNzgsInRhcmdldDplbXBsb3llZVBheUNhZ3I6dmFsdWUiOjcsInRhcmdldDplbXBsb3llZVBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6dmFsdWUiOjIuODUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MTUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTptYXgiOjI1Mi42OSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOm1heCI6MTM2Ljg0LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOm1heCI6MzMuNDMsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOm1heCI6My43NH0sIm1ldHJpY0dyb3VwQmFzZXMiOnsiY29tcGFueVNhbGVzIjoicmF0ZSIsInByb2plY3RTYWxlcyI6InJhdGUiLCJsYWJvclByb2R1Y3Rpdml0eSI6InJhdGUiLCJlbXBsb3llZVBheSI6InJhdGUifSwiYXBwbGljYXRpb25DYXRlZ29yeSI6ImdlbmVyYWwiLCJhZGp1c3RlZERyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsInByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwib3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwicHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yNSwib3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMiwicHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsInByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJvdGhlck5vbk9wZXJhdGluZ1JhdGUiOi0wLjAwNSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjowLCJlZmZlY3RpdmVUYXhSYXRlIjowLjMsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQxMDU5NTc2MDIzMzkxNiwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MS4xNzQxODY0OTEwNjQ0NjZlLTE2LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAxOTk4MjEzNTUxMTg3OTg3MywicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwNjM5MDEyNDk3MjI5MzQsInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MTIwNDUxMzMzMTU3NjMsIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNjA1NTE2MjczMDA1MjcsIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4ODEzNjc1MDA5MTcxMTcsIm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwNjA5MzUzOTQzNzE3ODU1LCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIwMjI0ODcyMTY5NDY2NzMsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTY1MTc4NTk0NTIxNzksInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE0OTkwNDgxMzQxMjY1NTUsIm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwicHJvamVjdFBheUdyb3d0aCI6MC4wODkwMDYyMjk5NzUwODAxLCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4ODc3NjE3MTAzMzMwMywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wMjkwNDU0ODIzOTcyMDUwNTUsIm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTc4NDgxNDczMjMwODY2NSwicHJvamVjdFNnYVJhdGVFbmQiOjAuMTA5OTMxODA5MTY0ODQ4MjQsIm90aGVyU2dhUmF0ZUVuZCI6MC4xMDkyNzI1ODk4NzIxMjgyMywicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzNzc4MDU3NjI4NzE2MzIsInVzZWZ1bExpZmUiOjEwLCJpbnZlc3RtZW50IjoyMywic3Vic2lkeSI6Ny42NiwibG9jYWxCZW5jaG1hcmsiOjIzfX0=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove useful-life depreciation assumption
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -6768,7 +6768,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C292"/>
+  <dimension ref="A1:C289"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="72" customWidth="1"/>
@@ -10038,11 +10038,11 @@
     <row r="218">
       <c r="A218" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:usefulLife:0</t>
+          <t xml:space="preserve">driver:effectiveTaxRate</t>
         </is>
       </c>
       <c r="B218" s="2">
-        <v>5</v>
+        <v>0.3</v>
       </c>
       <c r="C218" s="0" t="inlineStr">
         <is>
@@ -10053,11 +10053,11 @@
     <row r="219">
       <c r="A219" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:usefulLife:1</t>
+          <t xml:space="preserve">driver:investment</t>
         </is>
       </c>
       <c r="B219" s="2">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C219" s="0" t="inlineStr">
         <is>
@@ -10068,11 +10068,11 @@
     <row r="220">
       <c r="A220" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:effectiveTaxRate</t>
+          <t xml:space="preserve">driver:localBenchmark</t>
         </is>
       </c>
       <c r="B220" s="2">
-        <v>0.3</v>
+        <v>23</v>
       </c>
       <c r="C220" s="0" t="inlineStr">
         <is>
@@ -10083,11 +10083,11 @@
     <row r="221">
       <c r="A221" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:investment</t>
+          <t xml:space="preserve">driver:otherCogsDepreciationShare</t>
         </is>
       </c>
       <c r="B221" s="2">
-        <v>23</v>
+        <v>0.2</v>
       </c>
       <c r="C221" s="0" t="inlineStr">
         <is>
@@ -10098,11 +10098,11 @@
     <row r="222">
       <c r="A222" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:localBenchmark</t>
+          <t xml:space="preserve">driver:otherCogsImprovement</t>
         </is>
       </c>
       <c r="B222" s="2">
-        <v>23</v>
+        <v>0.005</v>
       </c>
       <c r="C222" s="0" t="inlineStr">
         <is>
@@ -10113,26 +10113,26 @@
     <row r="223">
       <c r="A223" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherCogsDepreciationShare</t>
+          <t xml:space="preserve">driver:otherCogsImprovementToBase</t>
         </is>
       </c>
       <c r="B223" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="C223" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherCogsImprovement</t>
+          <t xml:space="preserve">driver:otherCogsRateWhenSalesZero</t>
         </is>
       </c>
       <c r="B224" s="2">
-        <v>0.005</v>
+        <v>0.68</v>
       </c>
       <c r="C224" s="0" t="inlineStr">
         <is>
@@ -10143,41 +10143,41 @@
     <row r="225">
       <c r="A225" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherCogsImprovementToBase</t>
+          <t xml:space="preserve">driver:otherEmployeeSalaryShare</t>
         </is>
       </c>
       <c r="B225" s="2">
-        <v>0</v>
+        <v>0.95</v>
       </c>
       <c r="C225" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherCogsRateWhenSalesZero</t>
+          <t xml:space="preserve">driver:otherExtraordinaryRate</t>
         </is>
       </c>
       <c r="B226" s="2">
-        <v>0.68</v>
+        <v>0</v>
       </c>
       <c r="C226" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherEmployeeSalaryShare</t>
+          <t xml:space="preserve">driver:otherHeadcountGrowth</t>
         </is>
       </c>
       <c r="B227" s="2">
-        <v>0.95</v>
+        <v>0.045833333333333386</v>
       </c>
       <c r="C227" s="0" t="inlineStr">
         <is>
@@ -10188,26 +10188,26 @@
     <row r="228">
       <c r="A228" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherExtraordinaryRate</t>
+          <t xml:space="preserve">driver:otherHeadcountGrowthToBase</t>
         </is>
       </c>
       <c r="B228" s="2">
-        <v>0</v>
+        <v>0.04083333333333339</v>
       </c>
       <c r="C228" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherHeadcountGrowth</t>
+          <t xml:space="preserve">driver:otherNonOperatingRate</t>
         </is>
       </c>
       <c r="B229" s="2">
-        <v>0.045833333333333386</v>
+        <v>-0.005</v>
       </c>
       <c r="C229" s="0" t="inlineStr">
         <is>
@@ -10218,11 +10218,11 @@
     <row r="230">
       <c r="A230" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherHeadcountGrowthToBase</t>
+          <t xml:space="preserve">driver:otherOfficerCompensationShare</t>
         </is>
       </c>
       <c r="B230" s="2">
-        <v>0.04083333333333339</v>
+        <v>0.9</v>
       </c>
       <c r="C230" s="0" t="inlineStr">
         <is>
@@ -10233,11 +10233,11 @@
     <row r="231">
       <c r="A231" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherNonOperatingRate</t>
+          <t xml:space="preserve">driver:otherOfficerPayGrowth</t>
         </is>
       </c>
       <c r="B231" s="2">
-        <v>-0.005</v>
+        <v>0.045</v>
       </c>
       <c r="C231" s="0" t="inlineStr">
         <is>
@@ -10248,11 +10248,11 @@
     <row r="232">
       <c r="A232" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherOfficerCompensationShare</t>
+          <t xml:space="preserve">driver:otherOfficerPayGrowthToBase</t>
         </is>
       </c>
       <c r="B232" s="2">
-        <v>0.9</v>
+        <v>0.04</v>
       </c>
       <c r="C232" s="0" t="inlineStr">
         <is>
@@ -10263,11 +10263,11 @@
     <row r="233">
       <c r="A233" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherOfficerPayGrowth</t>
+          <t xml:space="preserve">driver:otherPayGrowth</t>
         </is>
       </c>
       <c r="B233" s="2">
-        <v>0.045</v>
+        <v>0.02484645846924027</v>
       </c>
       <c r="C233" s="0" t="inlineStr">
         <is>
@@ -10278,11 +10278,11 @@
     <row r="234">
       <c r="A234" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherOfficerPayGrowthToBase</t>
+          <t xml:space="preserve">driver:otherPayGrowthToBase</t>
         </is>
       </c>
       <c r="B234" s="2">
-        <v>0.04</v>
+        <v>0.01984645846924027</v>
       </c>
       <c r="C234" s="0" t="inlineStr">
         <is>
@@ -10293,11 +10293,11 @@
     <row r="235">
       <c r="A235" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherPayGrowth</t>
+          <t xml:space="preserve">driver:otherResearchDevelopmentRate</t>
         </is>
       </c>
       <c r="B235" s="2">
-        <v>0.02484645846924027</v>
+        <v>0.004</v>
       </c>
       <c r="C235" s="0" t="inlineStr">
         <is>
@@ -10308,11 +10308,11 @@
     <row r="236">
       <c r="A236" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherPayGrowthToBase</t>
+          <t xml:space="preserve">driver:otherSalesGrowth</t>
         </is>
       </c>
       <c r="B236" s="2">
-        <v>0.01984645846924027</v>
+        <v>0.06257246376811586</v>
       </c>
       <c r="C236" s="0" t="inlineStr">
         <is>
@@ -10323,11 +10323,11 @@
     <row r="237">
       <c r="A237" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherResearchDevelopmentRate</t>
+          <t xml:space="preserve">driver:otherSalesGrowthToBase</t>
         </is>
       </c>
       <c r="B237" s="2">
-        <v>0.004</v>
+        <v>0.042572463768115854</v>
       </c>
       <c r="C237" s="0" t="inlineStr">
         <is>
@@ -10338,26 +10338,26 @@
     <row r="238">
       <c r="A238" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSalesGrowth</t>
+          <t xml:space="preserve">driver:otherSgaImprovementToBase</t>
         </is>
       </c>
       <c r="B238" s="2">
-        <v>0.06257246376811586</v>
+        <v>0</v>
       </c>
       <c r="C238" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSalesGrowthToBase</t>
+          <t xml:space="preserve">driver:otherSgaRateEnd</t>
         </is>
       </c>
       <c r="B239" s="2">
-        <v>0.042572463768115854</v>
+        <v>0.10928571428571428</v>
       </c>
       <c r="C239" s="0" t="inlineStr">
         <is>
@@ -10368,26 +10368,26 @@
     <row r="240">
       <c r="A240" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSgaImprovementToBase</t>
+          <t xml:space="preserve">driver:projectCogsDepreciationShare</t>
         </is>
       </c>
       <c r="B240" s="2">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="C240" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSgaRateEnd</t>
+          <t xml:space="preserve">driver:projectCogsImprovementAfterBase</t>
         </is>
       </c>
       <c r="B241" s="2">
-        <v>0.10928571428571428</v>
+        <v>0.015</v>
       </c>
       <c r="C241" s="0" t="inlineStr">
         <is>
@@ -10398,11 +10398,11 @@
     <row r="242">
       <c r="A242" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectCogsDepreciationShare</t>
+          <t xml:space="preserve">driver:projectCogsImprovementToBase</t>
         </is>
       </c>
       <c r="B242" s="2">
-        <v>0.25</v>
+        <v>5.551115123125783e-17</v>
       </c>
       <c r="C242" s="0" t="inlineStr">
         <is>
@@ -10413,11 +10413,11 @@
     <row r="243">
       <c r="A243" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectCogsImprovementAfterBase</t>
+          <t xml:space="preserve">driver:projectCogsRateWhenSalesZero</t>
         </is>
       </c>
       <c r="B243" s="2">
-        <v>0.015</v>
+        <v>0.68</v>
       </c>
       <c r="C243" s="0" t="inlineStr">
         <is>
@@ -10428,11 +10428,11 @@
     <row r="244">
       <c r="A244" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectCogsImprovementToBase</t>
+          <t xml:space="preserve">driver:projectEmployeeSalaryShare</t>
         </is>
       </c>
       <c r="B244" s="2">
-        <v>5.551115123125783e-17</v>
+        <v>0.95</v>
       </c>
       <c r="C244" s="0" t="inlineStr">
         <is>
@@ -10443,26 +10443,26 @@
     <row r="245">
       <c r="A245" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectCogsRateWhenSalesZero</t>
+          <t xml:space="preserve">driver:projectExtraordinaryRate</t>
         </is>
       </c>
       <c r="B245" s="2">
-        <v>0.68</v>
+        <v>0</v>
       </c>
       <c r="C245" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectEmployeeSalaryShare</t>
+          <t xml:space="preserve">driver:projectHeadcountGrowth</t>
         </is>
       </c>
       <c r="B246" s="2">
-        <v>0.95</v>
+        <v>0.04</v>
       </c>
       <c r="C246" s="0" t="inlineStr">
         <is>
@@ -10473,26 +10473,26 @@
     <row r="247">
       <c r="A247" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectExtraordinaryRate</t>
+          <t xml:space="preserve">driver:projectHeadcountGrowthToBase</t>
         </is>
       </c>
       <c r="B247" s="2">
-        <v>0</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="C247" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectHeadcountGrowth</t>
+          <t xml:space="preserve">driver:projectMarketGrowth</t>
         </is>
       </c>
       <c r="B248" s="2">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="C248" s="0" t="inlineStr">
         <is>
@@ -10503,26 +10503,26 @@
     <row r="249">
       <c r="A249" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectHeadcountGrowthToBase</t>
+          <t xml:space="preserve">driver:projectNonOperatingRate</t>
         </is>
       </c>
       <c r="B249" s="2">
-        <v>0.05409356725146197</v>
+        <v>0</v>
       </c>
       <c r="C249" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectMarketGrowth</t>
+          <t xml:space="preserve">driver:projectOfficerCompensationShare</t>
         </is>
       </c>
       <c r="B250" s="2">
-        <v>0.05</v>
+        <v>0.9</v>
       </c>
       <c r="C250" s="0" t="inlineStr">
         <is>
@@ -10533,26 +10533,26 @@
     <row r="251">
       <c r="A251" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectNonOperatingRate</t>
+          <t xml:space="preserve">driver:projectOfficerPayGrowth</t>
         </is>
       </c>
       <c r="B251" s="2">
-        <v>0</v>
+        <v>0.05380116959064325</v>
       </c>
       <c r="C251" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectOfficerCompensationShare</t>
+          <t xml:space="preserve">driver:projectOfficerPayGrowthToBase</t>
         </is>
       </c>
       <c r="B252" s="2">
-        <v>0.9</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="C252" s="0" t="inlineStr">
         <is>
@@ -10563,11 +10563,11 @@
     <row r="253">
       <c r="A253" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectOfficerPayGrowth</t>
+          <t xml:space="preserve">driver:projectPayGrowth</t>
         </is>
       </c>
       <c r="B253" s="2">
-        <v>0.05380116959064325</v>
+        <v>0.07</v>
       </c>
       <c r="C253" s="0" t="inlineStr">
         <is>
@@ -10578,11 +10578,11 @@
     <row r="254">
       <c r="A254" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectOfficerPayGrowthToBase</t>
+          <t xml:space="preserve">driver:projectPayGrowthToBase</t>
         </is>
       </c>
       <c r="B254" s="2">
-        <v>0.05409356725146197</v>
+        <v>0.020030662342518046</v>
       </c>
       <c r="C254" s="0" t="inlineStr">
         <is>
@@ -10593,11 +10593,11 @@
     <row r="255">
       <c r="A255" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectPayGrowth</t>
+          <t xml:space="preserve">driver:projectResearchDevelopmentRate</t>
         </is>
       </c>
       <c r="B255" s="2">
-        <v>0.07</v>
+        <v>0.005</v>
       </c>
       <c r="C255" s="0" t="inlineStr">
         <is>
@@ -10608,11 +10608,11 @@
     <row r="256">
       <c r="A256" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectPayGrowthToBase</t>
+          <t xml:space="preserve">driver:projectSalesGrowth</t>
         </is>
       </c>
       <c r="B256" s="2">
-        <v>0.020030662342518046</v>
+        <v>0.22</v>
       </c>
       <c r="C256" s="0" t="inlineStr">
         <is>
@@ -10623,11 +10623,11 @@
     <row r="257">
       <c r="A257" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectResearchDevelopmentRate</t>
+          <t xml:space="preserve">driver:projectSalesGrowthToBase</t>
         </is>
       </c>
       <c r="B257" s="2">
-        <v>0.005</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="C257" s="0" t="inlineStr">
         <is>
@@ -10638,26 +10638,26 @@
     <row r="258">
       <c r="A258" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSalesGrowth</t>
+          <t xml:space="preserve">driver:projectSgaImprovementToBase</t>
         </is>
       </c>
       <c r="B258" s="2">
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="C258" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSalesGrowthToBase</t>
+          <t xml:space="preserve">driver:projectSgaRateEnd</t>
         </is>
       </c>
       <c r="B259" s="2">
-        <v>0.05409356725146197</v>
+        <v>0.11</v>
       </c>
       <c r="C259" s="0" t="inlineStr">
         <is>
@@ -10668,26 +10668,26 @@
     <row r="260">
       <c r="A260" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSgaImprovementToBase</t>
+          <t xml:space="preserve">driver:subsidy</t>
         </is>
       </c>
       <c r="B260" s="2">
-        <v>0</v>
+        <v>7.66</v>
       </c>
       <c r="C260" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSgaRateEnd</t>
+          <t xml:space="preserve">target:companyPaySchedule:max</t>
         </is>
       </c>
       <c r="B261" s="2">
-        <v>0.11</v>
+        <v>7</v>
       </c>
       <c r="C261" s="0" t="inlineStr">
         <is>
@@ -10698,11 +10698,11 @@
     <row r="262">
       <c r="A262" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:subsidy</t>
+          <t xml:space="preserve">target:companyPaySchedule:value</t>
         </is>
       </c>
       <c r="B262" s="2">
-        <v>7.66</v>
+        <v>2</v>
       </c>
       <c r="C262" s="0" t="inlineStr">
         <is>
@@ -10713,11 +10713,11 @@
     <row r="263">
       <c r="A263" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:usefulLife</t>
+          <t xml:space="preserve">target:companySalesCagr:max</t>
         </is>
       </c>
       <c r="B263" s="2">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="C263" s="0" t="inlineStr">
         <is>
@@ -10728,11 +10728,11 @@
     <row r="264">
       <c r="A264" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companyPaySchedule:max</t>
+          <t xml:space="preserve">target:companySalesCagr:value</t>
         </is>
       </c>
       <c r="B264" s="2">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C264" s="0" t="inlineStr">
         <is>
@@ -10743,11 +10743,11 @@
     <row r="265">
       <c r="A265" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companyPaySchedule:value</t>
+          <t xml:space="preserve">target:companySalesIncrease:max</t>
         </is>
       </c>
       <c r="B265" s="2">
-        <v>2</v>
+        <v>252.69</v>
       </c>
       <c r="C265" s="0" t="inlineStr">
         <is>
@@ -10758,11 +10758,11 @@
     <row r="266">
       <c r="A266" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesCagr:max</t>
+          <t xml:space="preserve">target:companySalesIncrease:value</t>
         </is>
       </c>
       <c r="B266" s="2">
-        <v>35</v>
+        <v>82.4</v>
       </c>
       <c r="C266" s="0" t="inlineStr">
         <is>
@@ -10773,11 +10773,11 @@
     <row r="267">
       <c r="A267" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesCagr:value</t>
+          <t xml:space="preserve">target:employeePayCagr:max</t>
         </is>
       </c>
       <c r="B267" s="2">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C267" s="0" t="inlineStr">
         <is>
@@ -10788,11 +10788,11 @@
     <row r="268">
       <c r="A268" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesIncrease:max</t>
+          <t xml:space="preserve">target:employeePayCagr:value</t>
         </is>
       </c>
       <c r="B268" s="2">
-        <v>252.69</v>
+        <v>7</v>
       </c>
       <c r="C268" s="0" t="inlineStr">
         <is>
@@ -10803,11 +10803,11 @@
     <row r="269">
       <c r="A269" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesIncrease:value</t>
+          <t xml:space="preserve">target:employeePayIncrease:max</t>
         </is>
       </c>
       <c r="B269" s="2">
-        <v>82.4</v>
+        <v>3.74</v>
       </c>
       <c r="C269" s="0" t="inlineStr">
         <is>
@@ -10818,11 +10818,11 @@
     <row r="270">
       <c r="A270" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayCagr:max</t>
+          <t xml:space="preserve">target:employeePayIncrease:value</t>
         </is>
       </c>
       <c r="B270" s="2">
-        <v>10</v>
+        <v>2.85</v>
       </c>
       <c r="C270" s="0" t="inlineStr">
         <is>
@@ -10833,11 +10833,11 @@
     <row r="271">
       <c r="A271" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayCagr:value</t>
+          <t xml:space="preserve">target:investmentSalesRatio:max</t>
         </is>
       </c>
       <c r="B271" s="2">
-        <v>7</v>
+        <v>70</v>
       </c>
       <c r="C271" s="0" t="inlineStr">
         <is>
@@ -10848,11 +10848,11 @@
     <row r="272">
       <c r="A272" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayIncrease:max</t>
+          <t xml:space="preserve">target:investmentSalesRatio:value</t>
         </is>
       </c>
       <c r="B272" s="2">
-        <v>3.74</v>
+        <v>15</v>
       </c>
       <c r="C272" s="0" t="inlineStr">
         <is>
@@ -10863,11 +10863,11 @@
     <row r="273">
       <c r="A273" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayIncrease:value</t>
+          <t xml:space="preserve">target:laborProductivityCagr:max</t>
         </is>
       </c>
       <c r="B273" s="2">
-        <v>2.85</v>
+        <v>35</v>
       </c>
       <c r="C273" s="0" t="inlineStr">
         <is>
@@ -10878,11 +10878,11 @@
     <row r="274">
       <c r="A274" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:investmentSalesRatio:max</t>
+          <t xml:space="preserve">target:laborProductivityCagr:value</t>
         </is>
       </c>
       <c r="B274" s="2">
-        <v>70</v>
+        <v>21</v>
       </c>
       <c r="C274" s="0" t="inlineStr">
         <is>
@@ -10893,11 +10893,11 @@
     <row r="275">
       <c r="A275" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:investmentSalesRatio:value</t>
+          <t xml:space="preserve">target:localBenchmark:max</t>
         </is>
       </c>
       <c r="B275" s="2">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="C275" s="0" t="inlineStr">
         <is>
@@ -10908,11 +10908,11 @@
     <row r="276">
       <c r="A276" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:laborProductivityCagr:max</t>
+          <t xml:space="preserve">target:localBenchmark:value</t>
         </is>
       </c>
       <c r="B276" s="2">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="C276" s="0" t="inlineStr">
         <is>
@@ -10923,11 +10923,11 @@
     <row r="277">
       <c r="A277" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:laborProductivityCagr:value</t>
+          <t xml:space="preserve">target:officerPayCagr:max</t>
         </is>
       </c>
       <c r="B277" s="2">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C277" s="0" t="inlineStr">
         <is>
@@ -10938,11 +10938,11 @@
     <row r="278">
       <c r="A278" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:localBenchmark:max</t>
+          <t xml:space="preserve">target:officerPayCagr:value</t>
         </is>
       </c>
       <c r="B278" s="2">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="C278" s="0" t="inlineStr">
         <is>
@@ -10953,26 +10953,26 @@
     <row r="279">
       <c r="A279" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:localBenchmark:value</t>
+          <t xml:space="preserve">target:officerPayIncrease:value</t>
         </is>
       </c>
       <c r="B279" s="2">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="C279" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayCagr:max</t>
+          <t xml:space="preserve">target:projectSalesCagr:max</t>
         </is>
       </c>
       <c r="B280" s="2">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="C280" s="0" t="inlineStr">
         <is>
@@ -10983,11 +10983,11 @@
     <row r="281">
       <c r="A281" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayCagr:value</t>
+          <t xml:space="preserve">target:projectSalesCagr:value</t>
         </is>
       </c>
       <c r="B281" s="2">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="C281" s="0" t="inlineStr">
         <is>
@@ -10998,26 +10998,26 @@
     <row r="282">
       <c r="A282" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayIncrease:value</t>
+          <t xml:space="preserve">target:projectSalesIncrease:max</t>
         </is>
       </c>
       <c r="B282" s="2">
-        <v>0</v>
+        <v>136.84</v>
       </c>
       <c r="C282" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesCagr:max</t>
+          <t xml:space="preserve">target:projectSalesIncrease:value</t>
         </is>
       </c>
       <c r="B283" s="2">
-        <v>35</v>
+        <v>74.8</v>
       </c>
       <c r="C283" s="0" t="inlineStr">
         <is>
@@ -11028,11 +11028,11 @@
     <row r="284">
       <c r="A284" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesCagr:value</t>
+          <t xml:space="preserve">target:projectSalesShare:max</t>
         </is>
       </c>
       <c r="B284" s="2">
-        <v>22</v>
+        <v>95</v>
       </c>
       <c r="C284" s="0" t="inlineStr">
         <is>
@@ -11043,11 +11043,11 @@
     <row r="285">
       <c r="A285" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesIncrease:max</t>
+          <t xml:space="preserve">target:projectSalesShare:value</t>
         </is>
       </c>
       <c r="B285" s="2">
-        <v>136.84</v>
+        <v>60</v>
       </c>
       <c r="C285" s="0" t="inlineStr">
         <is>
@@ -11058,11 +11058,11 @@
     <row r="286">
       <c r="A286" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesIncrease:value</t>
+          <t xml:space="preserve">target:valueAddedIncrease:max</t>
         </is>
       </c>
       <c r="B286" s="2">
-        <v>74.8</v>
+        <v>33.43</v>
       </c>
       <c r="C286" s="0" t="inlineStr">
         <is>
@@ -11073,11 +11073,11 @@
     <row r="287">
       <c r="A287" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesShare:max</t>
+          <t xml:space="preserve">target:valueAddedIncrease:value</t>
         </is>
       </c>
       <c r="B287" s="2">
-        <v>95</v>
+        <v>18.78</v>
       </c>
       <c r="C287" s="0" t="inlineStr">
         <is>
@@ -11088,11 +11088,11 @@
     <row r="288">
       <c r="A288" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesShare:value</t>
+          <t xml:space="preserve">target:valueAddedSubsidyRatio:max</t>
         </is>
       </c>
       <c r="B288" s="2">
-        <v>60</v>
+        <v>350</v>
       </c>
       <c r="C288" s="0" t="inlineStr">
         <is>
@@ -11103,58 +11103,13 @@
     <row r="289">
       <c r="A289" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:valueAddedIncrease:max</t>
+          <t xml:space="preserve">target:valueAddedSubsidyRatio:value</t>
         </is>
       </c>
       <c r="B289" s="2">
-        <v>33.43</v>
+        <v>213</v>
       </c>
       <c r="C289" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">入力済み</t>
-        </is>
-      </c>
-    </row>
-    <row r="290">
-      <c r="A290" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">target:valueAddedIncrease:value</t>
-        </is>
-      </c>
-      <c r="B290" s="2">
-        <v>18.78</v>
-      </c>
-      <c r="C290" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">入力済み</t>
-        </is>
-      </c>
-    </row>
-    <row r="291">
-      <c r="A291" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">target:valueAddedSubsidyRatio:max</t>
-        </is>
-      </c>
-      <c r="B291" s="2">
-        <v>350</v>
-      </c>
-      <c r="C291" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">入力済み</t>
-        </is>
-      </c>
-    </row>
-    <row r="292">
-      <c r="A292" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">target:valueAddedSubsidyRatio:value</t>
-        </is>
-      </c>
-      <c r="B292" s="2">
-        <v>213</v>
-      </c>
-      <c r="C292" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">入力済み</t>
         </is>
@@ -11182,7 +11137,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4LCJvcmRpbmFyeUluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsInByZVRheEluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsIm5ldEluY29tZSI6Ny41MX19LHsieWVhciI6MjAyNCwicm9sZSI6InByZXZpb3VzIiwicHJvamVjdCI6eyJzYWxlcyI6NzYsImNvZ3MiOjUxLjY4LCJlbXBsb3llZVBheSI6NS41OSwib2ZmaWNlclBheSI6MC4zOCwiZGVwcmVjaWF0aW9uIjoxLjksIm90aGVyU2dhIjo5LjUsImhlYWRjb3VudCI6OTUsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjUuMzEsImVtcGxveWVlQm9udXMiOjAuMjgsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzQsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40Nywic2dhRGVwcmVjaWF0aW9uIjoxLjQzLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM4fSwib3RoZXIiOnsic2FsZXMiOjY3LjIsImNvZ3MiOjQ1LjcsImVtcGxveWVlUGF5Ijo3LjU0LCJvZmZpY2VyUGF5IjowLjU4LCJkZXByZWNpYXRpb24iOjEuNDQsIm90aGVyU2dhIjo3LjY4LCJoZWFkY291bnQiOjEyNSwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ny4xNiwiZW1wbG95ZWVCb251cyI6MC4zOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41Miwib2ZmaWNlckJvbnVzIjowLjA2LCJjb2dzRGVwcmVjaWF0aW9uIjowLjI5LCJzZ2FEZXByZWNpYXRpb24iOjEuMTUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMjksIm9yZGluYXJ5SW5jb21lIjozLjk2OTk5OTk5OTk5OTk5NywicHJlVGF4SW5jb21lIjozLjk2OTk5OTk5OTk5OTk5NywibmV0SW5jb21lIjo3LjcxfX0seyJ5ZWFyIjoyMDI1LCJyb2xlIjoibGF0ZXN0IiwicHJvamVjdCI6eyJzYWxlcyI6ODAsImNvZ3MiOjU0LjQsImVtcGxveWVlUGF5Ijo2LCJlbXBsb3llZVNhbGFyeSI6NS43LCJlbXBsb3llZUJvbnVzIjowLjMsIm9mZmljZXJQYXkiOjAuNCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNiwib2ZmaWNlckJvbnVzIjowLjA0LCJkZXByZWNpYXRpb24iOjIsImNvZ3NEZXByZWNpYXRpb24iOjAuNSwic2dhRGVwcmVjaWF0aW9uIjoxLjUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuNCwib3RoZXJTZ2EiOjEwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwLCJjb2dzIjo0Ny42LCJlbXBsb3llZVBheSI6OCwiZW1wbG95ZWVTYWxhcnkiOjcuNiwiZW1wbG95ZWVCb251cyI6MC40LCJvZmZpY2VyUGF5IjowLjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTQsIm9mZmljZXJCb251cyI6MC4wNiwiZGVwcmVjaWF0aW9uIjoxLjUsImNvZ3NEZXByZWNpYXRpb24iOjAuMywic2dhRGVwcmVjaWF0aW9uIjoxLjIsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMywib3RoZXJTZ2EiOjgsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjozLjk5OTk5OTk5OTk5OTk5NjQsInByZVRheEluY29tZSI6My45OTk5OTk5OTk5OTk5OTY0LCJuZXRJbmNvbWUiOjcuOTF9fV0sImJhbGFuY2VTaGVldHMiOlt7InllYXIiOjIwMjMsImFzc2V0cyI6MTMyLCJjdXJyZW50QXNzZXRzIjo2NywiY2FzaCI6MjQsImZpeGVkQXNzZXRzIjo2NSwidGFuZ2libGVBc3NldHMiOjUzLCJidWlsZGluZ3MiOjE5LCJtYWNoaW5lcnkiOjI0LCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6Nywic29mdHdhcmUiOjUsImxpYWJpbGl0aWVzIjo3NSwiY3VycmVudExpYWJpbGl0aWVzIjozOSwic2hvcnRUZXJtRGVidCI6MTIsImZpeGVkTGlhYmlsaXRpZXMiOjM2LCJsb25nVGVybURlYnQiOjI5LCJuZXRBc3NldHMiOjU3LCJzaGFyZWhvbGRlckVxdWl0eSI6NTQsImNhcGl0YWwiOjEwLCJjYXBleCI6NX0seyJ5ZWFyIjoyMDI0LCJhc3NldHMiOjE0MywiY3VycmVudEFzc2V0cyI6NzIsImNhc2giOjI1LCJmaXhlZEFzc2V0cyI6NzEsInRhbmdpYmxlQXNzZXRzIjo1OCwiYnVpbGRpbmdzIjoyMCwibWFjaGluZXJ5IjoyOCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjgsInNvZnR3YXJlIjo2LCJsaWFiaWxpdGllcyI6NzksImN1cnJlbnRMaWFiaWxpdGllcyI6NDEsInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozOCwibG9uZ1Rlcm1EZWJ0IjozMSwibmV0QXNzZXRzIjo2NCwic2hhcmVob2xkZXJFcXVpdHkiOjYxLCJjYXBpdGFsIjoxMCwiY2FwZXgiOjh9LHsieWVhciI6MjAyNSwiYXNzZXRzIjoxNTYsImN1cnJlbnRBc3NldHMiOjc4LCJjYXNoIjoyNywiZml4ZWRBc3NldHMiOjc4LCJ0YW5naWJsZUFzc2V0cyI6NjQsImJ1aWxkaW5ncyI6MjIsIm1hY2hpbmVyeSI6MzIsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo5LCJzb2Z0d2FyZSI6NywibGlhYmlsaXRpZXMiOjgzLCJjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJzaG9ydFRlcm1EZWJ0IjoxMSwiZml4ZWRMaWFiaWxpdGllcyI6NDAsImxvbmdUZXJtRGVidCI6MzIsIm5ldEFzc2V0cyI6NzMsInNoYXJlaG9sZGVyRXF1aXR5Ijo3MCwiY2FwaXRhbCI6MTAsImNhcGV4IjoxMH1dLCJmdXR1cmVDYXBleCI6W3sieWVhciI6MjAyNiwidmFsdWUiOjB9LHsieWVhciI6MjAyNywidmFsdWUiOjB9LHsieWVhciI6MjAyOCwidmFsdWUiOjB9LHsieWVhciI6MjAyOSwidmFsdWUiOjB9LHsieWVhciI6MjAzMCwidmFsdWUiOjB9LHsieWVhciI6MjAzMSwidmFsdWUiOjB9XSwiZHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTcyNDYzNzY4MTE1ODYsInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsInByb2plY3RTZ2FSYXRlRW5kIjowLjExLCJvdGhlclNnYVJhdGVFbmQiOjAuMTA5Mjg1NzE0Mjg1NzE0MjgsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJ1c2VmdWxMaWZlIjoxMCwiaW52ZXN0bWVudCI6MjMsInN1YnNpZHkiOjcuNjYsImxvY2FsQmVuY2htYXJrIjoyM30sImRyaXZlclJhbmdlcyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjpbLTAuMDUsMC4zXSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6WzAsMC45OV0sIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjpbMCwwLjk5XSwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOlswLDFdLCJvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOlswLDFdLCJwcm9qZWN0T2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjpbMCwxXSwib3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOlswLDFdLCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjpbMCwxXSwib3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOlswLDFdLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOlswLDAuM10sIm90aGVyUmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOlswLDAuM10sInByb2plY3ROb25PcGVyYXRpbmdSYXRlIjpbLTAuNSwwLjVdLCJvdGhlck5vbk9wZXJhdGluZ1JhdGUiOlstMC41LDAuNV0sInByb2plY3RFeHRyYW9yZGluYXJ5UmF0ZSI6Wy0wLjUsMC41XSwib3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6Wy0wLjUsMC41XSwiZWZmZWN0aXZlVGF4UmF0ZSI6WzAsMC42XSwicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDEuNjY1MzM0NTM2OTM3NzM0OGUtMTZdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkzMjUzMzA1MDE4NDY5MjcsMC4wMjA3MzU5OTQxODMxODkxNjZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlswLjA0MDc2MDg2OTU2NTIxNzE4NCwwLjA0NDM4NDA1Nzk3MTAxNDUyXSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDAwMTM0NTc1NTY5MzU4MTk3MzddLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MTM5NDU3MDIzNzE3NDQzLDAuMDIwNTUzNDU5OTE0NzYzMDk1XSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjAzOTE2NjY2NjY2NjY2NjY4LDAuMDQyNTAwMDAwMDAwMDAwMDldLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbMC4xNSwwLjNdLCJvdGhlclNhbGVzR3Jvd3RoIjpbMC4wNjA3NjA4Njk1NjUyMTcxOSwwLjA2NDM4NDA1Nzk3MTAxNDUzXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMC4wMDUsMC4wMDUxMzQ1NzU1NjkzNTgxOTc1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLjAyNDEzOTQ1NzAyMzcxNzQ0NCwwLjAyNTU1MzQ1OTkxNDc2MzA5Nl0sIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6WzAsMC4wOF0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6WzAuMDQ0MTY2NjY2NjY2NjY2NjgsMC4wNDc1MDAwMDAwMDAwMDAwOV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMC4wODQ5OTk5OTk5OTk5OTk5OSwwLjEzNV0sIm90aGVyU2dhUmF0ZUVuZCI6WzAuMDg5Mjg1NzE0Mjg1NzE0MjcsMC4xMTkyODU3MTQyODU3MTQyN10sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjpbMC4wNDI2MzE1Nzg5NDczNjgzNiwwLjA2NTU1NTU1NTU1NTU1NTU4XSwidXNlZnVsTGlmZSI6WzUsMjBdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MTUsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6ODIuNCwibWF4IjoyNTIuNjksInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55UGF5U2NoZWR1bGUiOnsidmFsdWUiOjIsIm1heCI6NywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc1NoYXJlIjp7InZhbHVlIjo2MCwibWF4Ijo5NSwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0NhZ3IiOnsidmFsdWUiOjIyLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjc0LjgsIm1heCI6MTM2Ljg0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MTguNzgsIm1heCI6MzMuNDMsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUNhZ3IiOnsidmFsdWUiOjcsIm1heCI6MTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUluY3JlYXNlIjp7InZhbHVlIjoyLjg1LCJtYXgiOjMuNzQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJpbnZlc3RtZW50U2FsZXNSYXRpbyI6eyJ2YWx1ZSI6MTUsIm1heCI6NzAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvIjp7InZhbHVlIjoyMTMsIm1heCI6MzUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibG9jYWxCZW5jaG1hcmsiOnsidmFsdWUiOjIzLCJtYXgiOjQwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUNhZ3IiOnsidmFsdWUiOjYsIm1heCI6MTAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnsiMjAyOTpvdGhlcjpzYWxlcyI6ODUuMTMsIjIwMjk6cHJvamVjdDo3LTgiOjcuOX0sImZ1dHVyZUlucHV0QmFzaXMiOiJvdGhlciIsImlucHV0VmFsdWVzIjp7ImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xIjoxMzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTMiOjkyLjc1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6MC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMyLjY1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6MC44MiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEwIjowLjA5LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTIiOjExLjY3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjAuNjIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNCI6Mi40NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1IjowLjY0LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTgiOjEwLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTkiOjEwLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjAiOjcuNTEsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yNyI6MjEwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xIjo3MiwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTQiOjIzLjA0LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNiI6Ni43OCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTgiOjUuMTksImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny05IjowLjM2LCJhY3R1YWw6cHJvamVjdDoyMDIzOlAyLTQiOjAuNDUsImFjdHVhbDpwcm9qZWN0OjIwMjM6UDItMTQiOjEuMzUsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMyI6OTAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEiOjE0My4yLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMyI6OTcuMzgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi00IjowLjc2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNyI6MzQuNTIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi05IjowLjg2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEyIjoxMi40NywiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEzIjowLjY2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTQiOjIuNTgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNSI6MC42NywiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE4IjoxMS4wMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE5IjoxMS4wMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTIwIjo3LjcxLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjciOjIyMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMSI6NzYsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny00IjoyNC4zMiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTYiOjcuMDQsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny04Ijo1LjU5LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctOSI6MC4zOCwiYWN0dWFsOnByb2plY3Q6MjAyNDpQMi00IjowLjQ3LCJhY3R1YWw6cHJvamVjdDoyMDI0OlAyLTE0IjoxLjQzLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTMiOjk1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xIjoxNTAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0zIjoxMDIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi00IjowLjgsImFjdHVhbDpjb21wYW55OjIwMjU6Mi03IjozNi40LCJhY3R1YWw6Y29tcGFueToyMDI1OjItOSI6MC45LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEyIjoxMy4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTMiOjAuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE0IjoyLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNSI6MC43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTgiOjExLjMsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xOSI6MTEuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTIwIjo3LjkxLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjciOjIzMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMSI6ODAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNS42LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6Ny4zLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTkiOjAuNCwiYWN0dWFsOnByb2plY3Q6MjAyNTpQMi00IjowLjUsImFjdHVhbDpwcm9qZWN0OjIwMjU6UDItMTQiOjEuNSwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudEFzc2V0cyI6NjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXNoIjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NSwiYmFsYW5jZS1zaGVldDoyMDIzOnRhbmdpYmxlQXNzZXRzIjo1MywiYmFsYW5jZS1zaGVldDoyMDIzOmJ1aWxkaW5ncyI6MTksImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzppbnRhbmdpYmxlQXNzZXRzIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUsImJhbGFuY2Utc2hlZXQ6MjAyMzpsaWFiaWxpdGllcyI6NzUsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50TGlhYmlsaXRpZXMiOjM5LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZExpYWJpbGl0aWVzIjozNiwiYmFsYW5jZS1zaGVldDoyMDIzOmxvbmdUZXJtRGVidCI6MjksImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hhcmVob2xkZXJFcXVpdHkiOjU0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NSwiYmFsYW5jZS1zaGVldDoyMDI0OmFzc2V0cyI6MTQzLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudEFzc2V0cyI6NzIsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNSwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkQXNzZXRzIjo3MSwiYmFsYW5jZS1zaGVldDoyMDI0OnRhbmdpYmxlQXNzZXRzIjo1OCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAsImJhbGFuY2Utc2hlZXQ6MjAyNDptYWNoaW5lcnkiOjI4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c29mdHdhcmUiOjYsImJhbGFuY2Utc2hlZXQ6MjAyNDpsaWFiaWxpdGllcyI6NzksImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZExpYWJpbGl0aWVzIjozOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEsImJhbGFuY2Utc2hlZXQ6MjAyNDpuZXRBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hhcmVob2xkZXJFcXVpdHkiOjYxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBleCI6OCwiYmFsYW5jZS1zaGVldDoyMDI1OmFzc2V0cyI6MTU2LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXNoIjoyNywiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkQXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI1OmJ1aWxkaW5ncyI6MjIsImJhbGFuY2Utc2hlZXQ6MjAyNTptYWNoaW5lcnkiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTppbnRhbmdpYmxlQXNzZXRzIjo5LCJiYWxhbmNlLXNoZWV0OjIwMjU6c29mdHdhcmUiOjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hvcnRUZXJtRGVidCI6MTEsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MCwiYmFsYW5jZS1zaGVldDoyMDI1OmxvbmdUZXJtRGVidCI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpuZXRBc3NldHMiOjczLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBleCI6MTAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC45OSwiZHJpdmVyOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvOjEiOjAuOTksImRyaXZlcjpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwiZHJpdmVyLXJhbmdlOnByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZToxIjoxLCJkcml2ZXI6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJkcml2ZXItcmFuZ2U6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjowLjksImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGU6MSI6MC4zLCJkcml2ZXI6b3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjEiOjAuMywiZHJpdmVyOnByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdE5vbk9wZXJhdGluZ1JhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOnByb2plY3ROb25PcGVyYXRpbmdSYXRlOjEiOjAuNSwiZHJpdmVyOm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJOb25PcGVyYXRpbmdSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpvdGhlck5vbk9wZXJhdGluZ1JhdGU6MSI6MC41LCJkcml2ZXI6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6b3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6ZWZmZWN0aXZlVGF4UmF0ZSI6MC4zLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZTowIjowLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZToxIjowLjYsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjUuNTUxMTE1MTIzMTI1NzgzZS0xNywiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZTowIjowLjAxOTMyNTMzMDUwMTg0NjkyNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA3MzU5OTQxODMxODkxNjYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNTcyNDYzNzY4MTE1ODU0LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZTowIjowLjA0MDc2MDg2OTU2NTIxNzE4NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNDQzODQwNTc5NzEwMTQ1MiwiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjAuMDAwMTM0NTc1NTY5MzU4MTk3MzcsImRyaXZlcjpvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDE5MTM5NDU3MDIzNzE3NDQzLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA1NTM0NTk5MTQ3NjMwOTUsImRyaXZlcjpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZToxIjowLjA4LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjAzOTE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNDI1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MCI6MC4xNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjMsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MCI6MC4wMjQxMzk0NTcwMjM3MTc0NDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDoxIjowLjAyNTU1MzQ1OTkxNDc2MzA5NiwiZHJpdmVyOm90aGVyT2ZmaWNlclBheUdyb3d0aCI6MC4wNDUsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aDoxIjowLjA4LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTgzMzMzMzMzMzMzMzM4NiwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjAiOjAuMDQ0MTY2NjY2NjY2NjY2NjgsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDoxIjowLjA0NzUwMDAwMDAwMDAwMDA5LCJkcml2ZXI6cHJvamVjdFNnYVJhdGVFbmQiOjAuMTEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDowIjowLjA4NDk5OTk5OTk5OTk5OTk5LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MSI6MC4xMzUsImRyaXZlcjpvdGhlclNnYVJhdGVFbmQiOjAuMTA5Mjg1NzE0Mjg1NzE0MjgsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MCI6MC4wODkyODU3MTQyODU3MTQyNywiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDoxIjowLjExOTI4NTcxNDI4NTcxNDI3LCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzODAxMTY5NTkwNjQzMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDowIjowLjA0MjYzMTU3ODk0NzM2ODM2LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MSI6MC4wNjU1NTU1NTU1NTU1NTU1OCwiZHJpdmVyOnVzZWZ1bExpZmUiOjEwLCJkcml2ZXItcmFuZ2U6dXNlZnVsTGlmZTowIjo1LCJkcml2ZXItcmFuZ2U6dXNlZnVsTGlmZToxIjoyMCwiZHJpdmVyOmludmVzdG1lbnQiOjIzLCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDowIjoxNSwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MSI6MjAwLCJkcml2ZXI6c3Vic2lkeSI6Ny42NiwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MCI6MSwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MSI6NTAsImRyaXZlcjpsb2NhbEJlbmNobWFyayI6MjMsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazowIjowLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MSI6MTAwLCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2Fncjp2YWx1ZSI6MTUsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTp2YWx1ZSI6ODIuNCwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTp2YWx1ZSI6MiwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTptYXgiOjcsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTp2YWx1ZSI6NjAsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTptYXgiOjk1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2Fncjp2YWx1ZSI6MjIsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTp2YWx1ZSI6NzQuOCwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2Fncjp2YWx1ZSI6MjEsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6bWF4IjozNSwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTp2YWx1ZSI6MTguNzgsInRhcmdldDplbXBsb3llZVBheUNhZ3I6dmFsdWUiOjcsInRhcmdldDplbXBsb3llZVBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6dmFsdWUiOjIuODUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MTUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTptYXgiOjI1Mi42OSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOm1heCI6MTM2Ljg0LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOm1heCI6MzMuNDMsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOm1heCI6My43NH0sIm1ldHJpY0dyb3VwQmFzZXMiOnsiY29tcGFueVNhbGVzIjoicmF0ZSIsInByb2plY3RTYWxlcyI6InJhdGUiLCJsYWJvclByb2R1Y3Rpdml0eSI6InJhdGUiLCJlbXBsb3llZVBheSI6InJhdGUifSwiYXBwbGljYXRpb25DYXRlZ29yeSI6ImdlbmVyYWwiLCJhZGp1c3RlZERyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsInByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwib3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwicHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yNSwib3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMiwicHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsInByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJvdGhlck5vbk9wZXJhdGluZ1JhdGUiOi0wLjAwNSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjowLCJlZmZlY3RpdmVUYXhSYXRlIjowLjMsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQxMTgyMzgzMDQwOTM1NSwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MS4xNzQxODY0OTEwNjQ0NjZlLTE2LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzODU2MjA1OTEzMzU2MiwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTIxNTg4ODg3MTgzOTQ1NSwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQxMzg0NDUwMzUzNjE4Nywib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI1Njk3MDU2MzE2MTMxOCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTgxOTg4OTExNDM0OTkxNSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA3OTQ0MTE0MTQ5ODIyMjUsIm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMjAzNzA4MTgxMTU0MTI2OCwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI2MjE3MzU2ODE4MzE4LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNDk1MjgwNjkyMjY2MDg5NSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA4NDgxMjgzMzc0ODY2NTAxLCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NjM3OTU1NTk2MzczNCwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wMjY1MzQwMDY5ODczNjg5OSwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODY4Mzk2ODIxODYwOTA0LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMDk5Nzc1ODM4MTI3MzU1Niwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTMyMTYzMDk2ODAxODY1LCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM3NjI5Njg0Mjg5MjM1OSwidXNlZnVsTGlmZSI6MTAsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9fQ==</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4LCJvcmRpbmFyeUluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsInByZVRheEluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsIm5ldEluY29tZSI6Ny41MX19LHsieWVhciI6MjAyNCwicm9sZSI6InByZXZpb3VzIiwicHJvamVjdCI6eyJzYWxlcyI6NzYsImNvZ3MiOjUxLjY4LCJlbXBsb3llZVBheSI6NS41OSwib2ZmaWNlclBheSI6MC4zOCwiZGVwcmVjaWF0aW9uIjoxLjksIm90aGVyU2dhIjo5LjUsImhlYWRjb3VudCI6OTUsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjUuMzEsImVtcGxveWVlQm9udXMiOjAuMjgsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzQsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40Nywic2dhRGVwcmVjaWF0aW9uIjoxLjQzLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM4fSwib3RoZXIiOnsic2FsZXMiOjY3LjIsImNvZ3MiOjQ1LjcsImVtcGxveWVlUGF5Ijo3LjU0LCJvZmZpY2VyUGF5IjowLjU4LCJkZXByZWNpYXRpb24iOjEuNDQsIm90aGVyU2dhIjo3LjY4LCJoZWFkY291bnQiOjEyNSwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ny4xNiwiZW1wbG95ZWVCb251cyI6MC4zOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41Miwib2ZmaWNlckJvbnVzIjowLjA2LCJjb2dzRGVwcmVjaWF0aW9uIjowLjI5LCJzZ2FEZXByZWNpYXRpb24iOjEuMTUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMjksIm9yZGluYXJ5SW5jb21lIjozLjk2OTk5OTk5OTk5OTk5NywicHJlVGF4SW5jb21lIjozLjk2OTk5OTk5OTk5OTk5NywibmV0SW5jb21lIjo3LjcxfX0seyJ5ZWFyIjoyMDI1LCJyb2xlIjoibGF0ZXN0IiwicHJvamVjdCI6eyJzYWxlcyI6ODAsImNvZ3MiOjU0LjQsImVtcGxveWVlUGF5Ijo2LCJlbXBsb3llZVNhbGFyeSI6NS43LCJlbXBsb3llZUJvbnVzIjowLjMsIm9mZmljZXJQYXkiOjAuNCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNiwib2ZmaWNlckJvbnVzIjowLjA0LCJkZXByZWNpYXRpb24iOjIsImNvZ3NEZXByZWNpYXRpb24iOjAuNSwic2dhRGVwcmVjaWF0aW9uIjoxLjUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuNCwib3RoZXJTZ2EiOjEwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwLCJjb2dzIjo0Ny42LCJlbXBsb3llZVBheSI6OCwiZW1wbG95ZWVTYWxhcnkiOjcuNiwiZW1wbG95ZWVCb251cyI6MC40LCJvZmZpY2VyUGF5IjowLjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTQsIm9mZmljZXJCb251cyI6MC4wNiwiZGVwcmVjaWF0aW9uIjoxLjUsImNvZ3NEZXByZWNpYXRpb24iOjAuMywic2dhRGVwcmVjaWF0aW9uIjoxLjIsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMywib3RoZXJTZ2EiOjgsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjozLjk5OTk5OTk5OTk5OTk5NjQsInByZVRheEluY29tZSI6My45OTk5OTk5OTk5OTk5OTY0LCJuZXRJbmNvbWUiOjcuOTF9fV0sImJhbGFuY2VTaGVldHMiOlt7InllYXIiOjIwMjMsImFzc2V0cyI6MTMyLCJjdXJyZW50QXNzZXRzIjo2NywiY2FzaCI6MjQsImZpeGVkQXNzZXRzIjo2NSwidGFuZ2libGVBc3NldHMiOjUzLCJidWlsZGluZ3MiOjE5LCJtYWNoaW5lcnkiOjI0LCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6Nywic29mdHdhcmUiOjUsImxpYWJpbGl0aWVzIjo3NSwiY3VycmVudExpYWJpbGl0aWVzIjozOSwic2hvcnRUZXJtRGVidCI6MTIsImZpeGVkTGlhYmlsaXRpZXMiOjM2LCJsb25nVGVybURlYnQiOjI5LCJuZXRBc3NldHMiOjU3LCJzaGFyZWhvbGRlckVxdWl0eSI6NTQsImNhcGl0YWwiOjEwLCJjYXBleCI6NX0seyJ5ZWFyIjoyMDI0LCJhc3NldHMiOjE0MywiY3VycmVudEFzc2V0cyI6NzIsImNhc2giOjI1LCJmaXhlZEFzc2V0cyI6NzEsInRhbmdpYmxlQXNzZXRzIjo1OCwiYnVpbGRpbmdzIjoyMCwibWFjaGluZXJ5IjoyOCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjgsInNvZnR3YXJlIjo2LCJsaWFiaWxpdGllcyI6NzksImN1cnJlbnRMaWFiaWxpdGllcyI6NDEsInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozOCwibG9uZ1Rlcm1EZWJ0IjozMSwibmV0QXNzZXRzIjo2NCwic2hhcmVob2xkZXJFcXVpdHkiOjYxLCJjYXBpdGFsIjoxMCwiY2FwZXgiOjh9LHsieWVhciI6MjAyNSwiYXNzZXRzIjoxNTYsImN1cnJlbnRBc3NldHMiOjc4LCJjYXNoIjoyNywiZml4ZWRBc3NldHMiOjc4LCJ0YW5naWJsZUFzc2V0cyI6NjQsImJ1aWxkaW5ncyI6MjIsIm1hY2hpbmVyeSI6MzIsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo5LCJzb2Z0d2FyZSI6NywibGlhYmlsaXRpZXMiOjgzLCJjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJzaG9ydFRlcm1EZWJ0IjoxMSwiZml4ZWRMaWFiaWxpdGllcyI6NDAsImxvbmdUZXJtRGVidCI6MzIsIm5ldEFzc2V0cyI6NzMsInNoYXJlaG9sZGVyRXF1aXR5Ijo3MCwiY2FwaXRhbCI6MTAsImNhcGV4IjoxMH1dLCJmdXR1cmVDYXBleCI6W3sieWVhciI6MjAyNiwidmFsdWUiOjB9LHsieWVhciI6MjAyNywidmFsdWUiOjB9LHsieWVhciI6MjAyOCwidmFsdWUiOjB9LHsieWVhciI6MjAyOSwidmFsdWUiOjB9LHsieWVhciI6MjAzMCwidmFsdWUiOjB9LHsieWVhciI6MjAzMSwidmFsdWUiOjB9XSwiZHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTcyNDYzNzY4MTE1ODYsInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsInByb2plY3RTZ2FSYXRlRW5kIjowLjExLCJvdGhlclNnYVJhdGVFbmQiOjAuMTA5Mjg1NzE0Mjg1NzE0MjgsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJpbnZlc3RtZW50IjoyMywic3Vic2lkeSI6Ny42NiwibG9jYWxCZW5jaG1hcmsiOjIzfSwiZHJpdmVyUmFuZ2VzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOlstMC4wNSwwLjNdLCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjpbMCwwLjk5XSwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOlswLDAuOTldLCJwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOlswLDFdLCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOlswLDFdLCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOlstMC41LDAuNV0sIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6Wy0wLjUsMC41XSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJlZmZlY3RpdmVUYXhSYXRlIjpbMCwwLjZdLCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6WzAsMS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNl0sInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOlswLjAxOTMyNTMzMDUwMTg0NjkyNywwLjAyMDczNTk5NDE4MzE4OTE2Nl0sInByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6WzAuMDQwNzYwODY5NTY1MjE3MTg0LDAuMDQ0Mzg0MDU3OTcxMDE0NTJdLCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6WzAsMC4wMDAxMzQ1NzU1NjkzNTgxOTczN10sIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkxMzk0NTcwMjM3MTc0NDMsMC4wMjA1NTM0NTk5MTQ3NjMwOTVdLCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6WzAuMDM5MTY2NjY2NjY2NjY2NjgsMC4wNDI1MDAwMDAwMDAwMDAwOV0sIm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDBdLCJwcm9qZWN0U2FsZXNHcm93dGgiOlswLjE1LDAuM10sIm90aGVyU2FsZXNHcm93dGgiOlswLjA2MDc2MDg2OTU2NTIxNzE5LDAuMDY0Mzg0MDU3OTcxMDE0NTNdLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjpbMCwwLjAzXSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOlswLjAwNSwwLjAwNTEzNDU3NTU2OTM1ODE5NzVdLCJwcm9qZWN0UGF5R3Jvd3RoIjpbMC4wNSwwLjFdLCJvdGhlclBheUdyb3d0aCI6WzAuMDI0MTM5NDU3MDIzNzE3NDQ0LDAuMDI1NTUzNDU5OTE0NzYzMDk2XSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjpbMCwwLjA4XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6WzAsMC4wOF0sIm90aGVySGVhZGNvdW50R3Jvd3RoIjpbMC4wNDQxNjY2NjY2NjY2NjY2OCwwLjA0NzUwMDAwMDAwMDAwMDA5XSwicHJvamVjdFNnYVJhdGVFbmQiOlswLjA4NDk5OTk5OTk5OTk5OTk5LDAuMTM1XSwib3RoZXJTZ2FSYXRlRW5kIjpbMC4wODkyODU3MTQyODU3MTQyNywwLjExOTI4NTcxNDI4NTcxNDI3XSwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOlswLjA0MjYzMTU3ODk0NzM2ODM2LDAuMDY1NTU1NTU1NTU1NTU1NThdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MTUsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6ODIuNCwibWF4IjoyNTIuNjksInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55UGF5U2NoZWR1bGUiOnsidmFsdWUiOjIsIm1heCI6NywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc1NoYXJlIjp7InZhbHVlIjo2MCwibWF4Ijo5NSwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0NhZ3IiOnsidmFsdWUiOjIyLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjc0LjgsIm1heCI6MTM2Ljg0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MTguNzgsIm1heCI6MzMuNDMsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUNhZ3IiOnsidmFsdWUiOjcsIm1heCI6MTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUluY3JlYXNlIjp7InZhbHVlIjoyLjg1LCJtYXgiOjMuNzQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJpbnZlc3RtZW50U2FsZXNSYXRpbyI6eyJ2YWx1ZSI6MTUsIm1heCI6NzAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvIjp7InZhbHVlIjoyMTMsIm1heCI6MzUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibG9jYWxCZW5jaG1hcmsiOnsidmFsdWUiOjIzLCJtYXgiOjQwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUNhZ3IiOnsidmFsdWUiOjYsIm1heCI6MTAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnsiMjAyOTpvdGhlcjpzYWxlcyI6ODUuMTMsIjIwMjk6cHJvamVjdDo3LTgiOjcuOX0sImZ1dHVyZUlucHV0QmFzaXMiOiJvdGhlciIsImlucHV0VmFsdWVzIjp7ImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xIjoxMzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTMiOjkyLjc1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6MC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMyLjY1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6MC44MiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEwIjowLjA5LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTIiOjExLjY3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjAuNjIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNCI6Mi40NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1IjowLjY0LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTgiOjEwLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTkiOjEwLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjAiOjcuNTEsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yNyI6MjEwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xIjo3MiwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTQiOjIzLjA0LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNiI6Ni43OCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTgiOjUuMTksImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny05IjowLjM2LCJhY3R1YWw6cHJvamVjdDoyMDIzOlAyLTQiOjAuNDUsImFjdHVhbDpwcm9qZWN0OjIwMjM6UDItMTQiOjEuMzUsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMyI6OTAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEiOjE0My4yLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMyI6OTcuMzgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi00IjowLjc2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNyI6MzQuNTIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi05IjowLjg2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEyIjoxMi40NywiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEzIjowLjY2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTQiOjIuNTgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNSI6MC42NywiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE4IjoxMS4wMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE5IjoxMS4wMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTIwIjo3LjcxLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjciOjIyMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMSI6NzYsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny00IjoyNC4zMiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTYiOjcuMDQsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny04Ijo1LjU5LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctOSI6MC4zOCwiYWN0dWFsOnByb2plY3Q6MjAyNDpQMi00IjowLjQ3LCJhY3R1YWw6cHJvamVjdDoyMDI0OlAyLTE0IjoxLjQzLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTMiOjk1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xIjoxNTAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0zIjoxMDIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi00IjowLjgsImFjdHVhbDpjb21wYW55OjIwMjU6Mi03IjozNi40LCJhY3R1YWw6Y29tcGFueToyMDI1OjItOSI6MC45LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEyIjoxMy4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTMiOjAuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE0IjoyLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNSI6MC43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTgiOjExLjMsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xOSI6MTEuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTIwIjo3LjkxLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjciOjIzMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMSI6ODAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNS42LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6Ny4zLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTkiOjAuNCwiYWN0dWFsOnByb2plY3Q6MjAyNTpQMi00IjowLjUsImFjdHVhbDpwcm9qZWN0OjIwMjU6UDItMTQiOjEuNSwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudEFzc2V0cyI6NjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXNoIjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NSwiYmFsYW5jZS1zaGVldDoyMDIzOnRhbmdpYmxlQXNzZXRzIjo1MywiYmFsYW5jZS1zaGVldDoyMDIzOmJ1aWxkaW5ncyI6MTksImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzppbnRhbmdpYmxlQXNzZXRzIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUsImJhbGFuY2Utc2hlZXQ6MjAyMzpsaWFiaWxpdGllcyI6NzUsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50TGlhYmlsaXRpZXMiOjM5LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZExpYWJpbGl0aWVzIjozNiwiYmFsYW5jZS1zaGVldDoyMDIzOmxvbmdUZXJtRGVidCI6MjksImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hhcmVob2xkZXJFcXVpdHkiOjU0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NSwiYmFsYW5jZS1zaGVldDoyMDI0OmFzc2V0cyI6MTQzLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudEFzc2V0cyI6NzIsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNSwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkQXNzZXRzIjo3MSwiYmFsYW5jZS1zaGVldDoyMDI0OnRhbmdpYmxlQXNzZXRzIjo1OCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAsImJhbGFuY2Utc2hlZXQ6MjAyNDptYWNoaW5lcnkiOjI4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c29mdHdhcmUiOjYsImJhbGFuY2Utc2hlZXQ6MjAyNDpsaWFiaWxpdGllcyI6NzksImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZExpYWJpbGl0aWVzIjozOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEsImJhbGFuY2Utc2hlZXQ6MjAyNDpuZXRBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hhcmVob2xkZXJFcXVpdHkiOjYxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBleCI6OCwiYmFsYW5jZS1zaGVldDoyMDI1OmFzc2V0cyI6MTU2LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXNoIjoyNywiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkQXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI1OmJ1aWxkaW5ncyI6MjIsImJhbGFuY2Utc2hlZXQ6MjAyNTptYWNoaW5lcnkiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTppbnRhbmdpYmxlQXNzZXRzIjo5LCJiYWxhbmNlLXNoZWV0OjIwMjU6c29mdHdhcmUiOjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hvcnRUZXJtRGVidCI6MTEsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MCwiYmFsYW5jZS1zaGVldDoyMDI1OmxvbmdUZXJtRGVidCI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpuZXRBc3NldHMiOjczLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBleCI6MTAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC45OSwiZHJpdmVyOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvOjEiOjAuOTksImRyaXZlcjpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwiZHJpdmVyLXJhbmdlOnByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZToxIjoxLCJkcml2ZXI6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJkcml2ZXItcmFuZ2U6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjowLjksImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGU6MSI6MC4zLCJkcml2ZXI6b3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjEiOjAuMywiZHJpdmVyOnByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdE5vbk9wZXJhdGluZ1JhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOnByb2plY3ROb25PcGVyYXRpbmdSYXRlOjEiOjAuNSwiZHJpdmVyOm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJOb25PcGVyYXRpbmdSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpvdGhlck5vbk9wZXJhdGluZ1JhdGU6MSI6MC41LCJkcml2ZXI6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6b3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6ZWZmZWN0aXZlVGF4UmF0ZSI6MC4zLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZTowIjowLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZToxIjowLjYsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjUuNTUxMTE1MTIzMTI1NzgzZS0xNywiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZTowIjowLjAxOTMyNTMzMDUwMTg0NjkyNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA3MzU5OTQxODMxODkxNjYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNTcyNDYzNzY4MTE1ODU0LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZTowIjowLjA0MDc2MDg2OTU2NTIxNzE4NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNDQzODQwNTc5NzEwMTQ1MiwiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjAuMDAwMTM0NTc1NTY5MzU4MTk3MzcsImRyaXZlcjpvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDE5MTM5NDU3MDIzNzE3NDQzLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA1NTM0NTk5MTQ3NjMwOTUsImRyaXZlcjpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZToxIjowLjA4LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjAzOTE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNDI1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MCI6MC4xNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjMsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MCI6MC4wMjQxMzk0NTcwMjM3MTc0NDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDoxIjowLjAyNTU1MzQ1OTkxNDc2MzA5NiwiZHJpdmVyOm90aGVyT2ZmaWNlclBheUdyb3d0aCI6MC4wNDUsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aDoxIjowLjA4LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTgzMzMzMzMzMzMzMzM4NiwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjAiOjAuMDQ0MTY2NjY2NjY2NjY2NjgsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDoxIjowLjA0NzUwMDAwMDAwMDAwMDA5LCJkcml2ZXI6cHJvamVjdFNnYVJhdGVFbmQiOjAuMTEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDowIjowLjA4NDk5OTk5OTk5OTk5OTk5LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MSI6MC4xMzUsImRyaXZlcjpvdGhlclNnYVJhdGVFbmQiOjAuMTA5Mjg1NzE0Mjg1NzE0MjgsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MCI6MC4wODkyODU3MTQyODU3MTQyNywiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDoxIjowLjExOTI4NTcxNDI4NTcxNDI3LCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzODAxMTY5NTkwNjQzMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDowIjowLjA0MjYzMTU3ODk0NzM2ODM2LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MSI6MC4wNjU1NTU1NTU1NTU1NTU1OCwiZHJpdmVyOmludmVzdG1lbnQiOjIzLCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDowIjoxNSwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MSI6MjAwLCJkcml2ZXI6c3Vic2lkeSI6Ny42NiwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MCI6MSwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MSI6NTAsImRyaXZlcjpsb2NhbEJlbmNobWFyayI6MjMsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazowIjowLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MSI6MTAwLCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2Fncjp2YWx1ZSI6MTUsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTp2YWx1ZSI6ODIuNCwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTp2YWx1ZSI6MiwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTptYXgiOjcsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTp2YWx1ZSI6NjAsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTptYXgiOjk1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2Fncjp2YWx1ZSI6MjIsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTp2YWx1ZSI6NzQuOCwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2Fncjp2YWx1ZSI6MjEsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6bWF4IjozNSwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTp2YWx1ZSI6MTguNzgsInRhcmdldDplbXBsb3llZVBheUNhZ3I6dmFsdWUiOjcsInRhcmdldDplbXBsb3llZVBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6dmFsdWUiOjIuODUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MTUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTptYXgiOjI1Mi42OSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOm1heCI6MTM2Ljg0LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOm1heCI6MzMuNDMsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOm1heCI6My43NH0sIm1ldHJpY0dyb3VwQmFzZXMiOnsiY29tcGFueVNhbGVzIjoicmF0ZSIsInByb2plY3RTYWxlcyI6InJhdGUiLCJsYWJvclByb2R1Y3Rpdml0eSI6InJhdGUiLCJlbXBsb3llZVBheSI6InJhdGUifSwiYXBwbGljYXRpb25DYXRlZ29yeSI6ImdlbmVyYWwiLCJhZGp1c3RlZERyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsInByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwib3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwicHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yNSwib3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMiwicHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsInByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJvdGhlck5vbk9wZXJhdGluZ1JhdGUiOi0wLjAwNSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjowLCJlZmZlY3RpdmVUYXhSYXRlIjowLjMsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQxMTgyMzgzMDQwOTM1NSwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MS4xNzQxODY0OTEwNjQ0NjZlLTE2LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzODU2MjA1OTEzMzU2MiwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTIxNTg4ODg3MTgzOTQ1NSwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQxMzg0NDUwMzUzNjE4Nywib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI1Njk3MDU2MzE2MTMxOCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTgxOTg4OTExNDM0OTkxNSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA3OTQ0MTE0MTQ5ODIyMjUsIm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMjAzNzA4MTgxMTU0MTI2OCwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI2MjE3MzU2ODE4MzE4LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNDk1MjgwNjkyMjY2MDg5NSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA4NDgxMjgzMzc0ODY2NTAxLCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NjM3OTU1NTk2MzczNCwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wMjY1MzQwMDY5ODczNjg5OSwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODY4Mzk2ODIxODYwOTA0LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMDk5Nzc1ODM4MTI3MzU1Niwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTMyMTYzMDk2ODAxODY1LCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM3NjI5Njg0Mjg5MjM1OSwiaW52ZXN0bWVudCI6MjMsInN1YnNpZHkiOjcuNjYsImxvY2FsQmVuY2htYXJrIjoyM319</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use SGA improvement points by period
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -1477,10 +1477,10 @@
         <v>46.18</v>
       </c>
       <c r="I9" s="2">
-        <v>50.78999999999999</v>
+        <v>50.8</v>
       </c>
       <c r="J9" s="2">
-        <v>55.97</v>
+        <v>55.96</v>
       </c>
     </row>
     <row r="10">
@@ -1783,10 +1783,10 @@
         <v>18.929999999999986</v>
       </c>
       <c r="I18" s="4">
-        <v>25.099999999999987</v>
+        <v>25.089999999999982</v>
       </c>
       <c r="J18" s="4">
-        <v>32.950000000000024</v>
+        <v>32.96000000000002</v>
       </c>
     </row>
     <row r="19">
@@ -1817,10 +1817,10 @@
         <v>9.48967315019049</v>
       </c>
       <c r="I19" s="2">
-        <v>10.91256901873831</v>
+        <v>10.90822138167905</v>
       </c>
       <c r="J19" s="2">
-        <v>12.367225912997794</v>
+        <v>12.370979244079127</v>
       </c>
     </row>
     <row r="20">
@@ -1851,10 +1851,10 @@
         <v>17.31</v>
       </c>
       <c r="I20" s="4">
-        <v>23.36</v>
+        <v>23.35</v>
       </c>
       <c r="J20" s="4">
-        <v>31.07</v>
+        <v>31.08</v>
       </c>
     </row>
     <row r="21">
@@ -1885,10 +1885,10 @@
         <v>17.31</v>
       </c>
       <c r="I21" s="2">
-        <v>23.36</v>
+        <v>23.35</v>
       </c>
       <c r="J21" s="2">
-        <v>31.07</v>
+        <v>31.08</v>
       </c>
     </row>
     <row r="22">
@@ -1919,7 +1919,7 @@
         <v>12.120000000000001</v>
       </c>
       <c r="I22" s="2">
-        <v>16.36</v>
+        <v>16.35</v>
       </c>
       <c r="J22" s="2">
         <v>21.75</v>
@@ -2055,10 +2055,10 @@
         <v>41.789999999999985</v>
       </c>
       <c r="I26" s="4">
-        <v>49.649999999999984</v>
+        <v>49.63999999999998</v>
       </c>
       <c r="J26" s="4">
-        <v>59.35000000000002</v>
+        <v>59.36000000000002</v>
       </c>
     </row>
     <row r="27">
@@ -2091,10 +2091,10 @@
         <v>20.780346820809203</v>
       </c>
       <c r="I27" s="2">
-        <v>18.808327351040923</v>
+        <v>18.78439818138309</v>
       </c>
       <c r="J27" s="2">
-        <v>19.536757301107844</v>
+        <v>19.580983078162873</v>
       </c>
     </row>
     <row r="28">
@@ -2125,10 +2125,10 @@
         <v>20.949468618407856</v>
       </c>
       <c r="I28" s="2">
-        <v>21.586017999217418</v>
+        <v>21.58167036215816</v>
       </c>
       <c r="J28" s="2">
-        <v>22.27601996772136</v>
+        <v>22.279773298802695</v>
       </c>
     </row>
     <row r="29">
@@ -2367,10 +2367,10 @@
         <v>0.15086642599277972</v>
       </c>
       <c r="I35" s="2">
-        <v>0.17299651567944246</v>
+        <v>0.1729616724738675</v>
       </c>
       <c r="J35" s="2">
-        <v>0.19916107382550344</v>
+        <v>0.1991946308724833</v>
       </c>
     </row>
     <row r="36">
@@ -2401,10 +2401,10 @@
         <v>22.429999999999986</v>
       </c>
       <c r="I36" s="4">
-        <v>28.599999999999987</v>
+        <v>28.589999999999982</v>
       </c>
       <c r="J36" s="4">
-        <v>36.450000000000024</v>
+        <v>36.46000000000002</v>
       </c>
     </row>
     <row r="37">
@@ -2435,10 +2435,10 @@
         <v>11.244235011028668</v>
       </c>
       <c r="I37" s="2">
-        <v>12.434241989478712</v>
+        <v>12.429894352419453</v>
       </c>
       <c r="J37" s="2">
-        <v>13.680891791464934</v>
+        <v>13.684645122546268</v>
       </c>
     </row>
     <row r="38">
@@ -2471,10 +2471,10 @@
         <v>36.18700667880987</v>
       </c>
       <c r="I38" s="2">
-        <v>27.507802050824814</v>
+        <v>27.46321890325458</v>
       </c>
       <c r="J38" s="2">
-        <v>27.447552447552592</v>
+        <v>27.52710738020303</v>
       </c>
     </row>
   </sheetData>
@@ -2811,7 +2811,7 @@
         <v>12.969999999999997</v>
       </c>
       <c r="I8" s="4">
-        <v>18.480000000000004</v>
+        <v>18.470000000000002</v>
       </c>
       <c r="J8" s="4">
         <v>25.61000000000001</v>
@@ -2845,7 +2845,7 @@
         <v>11.34236991692173</v>
       </c>
       <c r="I9" s="2">
-        <v>13.242565388749552</v>
+        <v>13.235399498387675</v>
       </c>
       <c r="J9" s="2">
         <v>15.038167938931302</v>
@@ -3049,7 +3049,7 @@
         <v>23.369999999999997</v>
       </c>
       <c r="I15" s="4">
-        <v>29.800000000000004</v>
+        <v>29.790000000000003</v>
       </c>
       <c r="J15" s="4">
         <v>37.96000000000001</v>
@@ -3085,10 +3085,10 @@
         <v>27.70491803278685</v>
       </c>
       <c r="I16" s="2">
-        <v>27.513906718014592</v>
+        <v>27.47111681643135</v>
       </c>
       <c r="J16" s="2">
-        <v>27.38255033557049</v>
+        <v>27.42531050688153</v>
       </c>
     </row>
     <row r="17">
@@ -3327,7 +3327,7 @@
         <v>0.19314049586776857</v>
       </c>
       <c r="I23" s="2">
-        <v>0.24032258064516132</v>
+        <v>0.240241935483871</v>
       </c>
       <c r="J23" s="2">
         <v>0.2988976377952757</v>
@@ -3849,12 +3849,12 @@
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 22.08 % / 補助 19.75 % / ベース 25.68 %</t>
+          <t xml:space="preserve">全社 22.09 % / 補助 19.76 % / ベース 25.68 %</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 21.01 % / 補助 18.46 % / ベース 25.53 %</t>
+          <t xml:space="preserve">全社 21 % / 補助 18.46 % / ベース 25.52 %</t>
         </is>
       </c>
     </row>
@@ -3916,7 +3916,7 @@
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.37 % / 補助 15.04 % / ベース 7.64 %</t>
+          <t xml:space="preserve">全社 12.37 % / 補助 15.04 % / ベース 7.65 %</t>
         </is>
       </c>
     </row>
@@ -3973,12 +3973,12 @@
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.43 % / 補助 14.68 % / ベース 8.98 %</t>
+          <t xml:space="preserve">全社 12.43 % / 補助 14.67 % / ベース 8.98 %</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.68 % / 補助 16.21 % / ベース 9.2 %</t>
+          <t xml:space="preserve">全社 13.68 % / 補助 16.21 % / ベース 9.21 %</t>
         </is>
       </c>
     </row>
@@ -4035,12 +4035,12 @@
       </c>
       <c r="K10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.3 % / 補助 11.49 % / ベース 10.99 %</t>
+          <t xml:space="preserve">全社 11.3 % / 補助 11.5 % / ベース 10.99 %</t>
         </is>
       </c>
       <c r="L10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.94 % / 補助 11 % / ベース 10.83 %</t>
+          <t xml:space="preserve">全社 10.93 % / 補助 11 % / ベース 10.82 %</t>
         </is>
       </c>
     </row>
@@ -4531,12 +4531,12 @@
       </c>
       <c r="K18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 42.4 % / 補助 31.28 % / ベース 59.09 %</t>
+          <t xml:space="preserve">全社 42.41 % / 補助 31.29 % / ベース 59.09 %</t>
         </is>
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 38.58 % / 補助 27.27 % / ベース 58.67 %</t>
+          <t xml:space="preserve">全社 38.58 % / 補助 27.27 % / ベース 58.64 %</t>
         </is>
       </c>
     </row>
@@ -5218,7 +5218,7 @@
       </c>
       <c r="L29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.41 倍 / 補助 13.81 倍 / ベース 5.89 倍</t>
+          <t xml:space="preserve">全社 10.42 倍 / 補助 13.81 倍 / ベース 5.9 倍</t>
         </is>
       </c>
     </row>
@@ -5590,7 +5590,7 @@
       </c>
       <c r="L35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 7.4 pt</t>
+          <t xml:space="preserve">差 7.39 pt</t>
         </is>
       </c>
     </row>
@@ -5771,12 +5771,12 @@
       </c>
       <c r="K38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 89.3 %</t>
+          <t xml:space="preserve">寄与率 89.29 %</t>
         </is>
       </c>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 90.83 %</t>
+          <t xml:space="preserve">寄与率 90.72 %</t>
         </is>
       </c>
     </row>
@@ -6652,11 +6652,11 @@
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 その他販管費率（事業化報告3年目）</t>
+          <t xml:space="preserve">補助事業 その他販管費率改善ポイント（基準年後）</t>
         </is>
       </c>
       <c r="B38" s="2">
-        <v>11</v>
+        <v>1.5</v>
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
@@ -6664,20 +6664,20 @@
         </is>
       </c>
       <c r="D38" s="2">
-        <v>8.5</v>
+        <v>0</v>
       </c>
       <c r="E38" s="2">
-        <v>13.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 その他販管費率（事業化報告3年目）</t>
+          <t xml:space="preserve">ベース事業 その他販管費率改善ポイント（基準年後）</t>
         </is>
       </c>
       <c r="B39" s="2">
-        <v>10.928571428571427</v>
+        <v>0.5</v>
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
@@ -6685,10 +6685,10 @@
         </is>
       </c>
       <c r="D39" s="2">
-        <v>8.928571428571427</v>
+        <v>0</v>
       </c>
       <c r="E39" s="2">
-        <v>11.928571428571427</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -9382,11 +9382,11 @@
         </is>
       </c>
       <c r="B174" s="2">
-        <v>0.08928571428571427</v>
+        <v>0</v>
       </c>
       <c r="C174" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
@@ -9397,7 +9397,7 @@
         </is>
       </c>
       <c r="B175" s="2">
-        <v>0.11928571428571427</v>
+        <v>0.01</v>
       </c>
       <c r="C175" s="0" t="inlineStr">
         <is>
@@ -9982,11 +9982,11 @@
         </is>
       </c>
       <c r="B214" s="2">
-        <v>0.08499999999999999</v>
+        <v>0</v>
       </c>
       <c r="C214" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
@@ -9997,7 +9997,7 @@
         </is>
       </c>
       <c r="B215" s="2">
-        <v>0.135</v>
+        <v>0.03</v>
       </c>
       <c r="C215" s="0" t="inlineStr">
         <is>
@@ -10357,7 +10357,7 @@
         </is>
       </c>
       <c r="B239" s="2">
-        <v>0.10928571428571428</v>
+        <v>0.005</v>
       </c>
       <c r="C239" s="0" t="inlineStr">
         <is>
@@ -10657,7 +10657,7 @@
         </is>
       </c>
       <c r="B259" s="2">
-        <v>0.11</v>
+        <v>0.015</v>
       </c>
       <c r="C259" s="0" t="inlineStr">
         <is>
@@ -11137,7 +11137,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4LCJvcmRpbmFyeUluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsInByZVRheEluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsIm5ldEluY29tZSI6Ny41MX19LHsieWVhciI6MjAyNCwicm9sZSI6InByZXZpb3VzIiwicHJvamVjdCI6eyJzYWxlcyI6NzYsImNvZ3MiOjUxLjY4LCJlbXBsb3llZVBheSI6NS41OSwib2ZmaWNlclBheSI6MC4zOCwiZGVwcmVjaWF0aW9uIjoxLjksIm90aGVyU2dhIjo5LjUsImhlYWRjb3VudCI6OTUsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjUuMzEsImVtcGxveWVlQm9udXMiOjAuMjgsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzQsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40Nywic2dhRGVwcmVjaWF0aW9uIjoxLjQzLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM4fSwib3RoZXIiOnsic2FsZXMiOjY3LjIsImNvZ3MiOjQ1LjcsImVtcGxveWVlUGF5Ijo3LjU0LCJvZmZpY2VyUGF5IjowLjU4LCJkZXByZWNpYXRpb24iOjEuNDQsIm90aGVyU2dhIjo3LjY4LCJoZWFkY291bnQiOjEyNSwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ny4xNiwiZW1wbG95ZWVCb251cyI6MC4zOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41Miwib2ZmaWNlckJvbnVzIjowLjA2LCJjb2dzRGVwcmVjaWF0aW9uIjowLjI5LCJzZ2FEZXByZWNpYXRpb24iOjEuMTUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMjksIm9yZGluYXJ5SW5jb21lIjozLjk2OTk5OTk5OTk5OTk5NywicHJlVGF4SW5jb21lIjozLjk2OTk5OTk5OTk5OTk5NywibmV0SW5jb21lIjo3LjcxfX0seyJ5ZWFyIjoyMDI1LCJyb2xlIjoibGF0ZXN0IiwicHJvamVjdCI6eyJzYWxlcyI6ODAsImNvZ3MiOjU0LjQsImVtcGxveWVlUGF5Ijo2LCJlbXBsb3llZVNhbGFyeSI6NS43LCJlbXBsb3llZUJvbnVzIjowLjMsIm9mZmljZXJQYXkiOjAuNCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNiwib2ZmaWNlckJvbnVzIjowLjA0LCJkZXByZWNpYXRpb24iOjIsImNvZ3NEZXByZWNpYXRpb24iOjAuNSwic2dhRGVwcmVjaWF0aW9uIjoxLjUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuNCwib3RoZXJTZ2EiOjEwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwLCJjb2dzIjo0Ny42LCJlbXBsb3llZVBheSI6OCwiZW1wbG95ZWVTYWxhcnkiOjcuNiwiZW1wbG95ZWVCb251cyI6MC40LCJvZmZpY2VyUGF5IjowLjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTQsIm9mZmljZXJCb251cyI6MC4wNiwiZGVwcmVjaWF0aW9uIjoxLjUsImNvZ3NEZXByZWNpYXRpb24iOjAuMywic2dhRGVwcmVjaWF0aW9uIjoxLjIsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMywib3RoZXJTZ2EiOjgsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjozLjk5OTk5OTk5OTk5OTk5NjQsInByZVRheEluY29tZSI6My45OTk5OTk5OTk5OTk5OTY0LCJuZXRJbmNvbWUiOjcuOTF9fV0sImJhbGFuY2VTaGVldHMiOlt7InllYXIiOjIwMjMsImFzc2V0cyI6MTMyLCJjdXJyZW50QXNzZXRzIjo2NywiY2FzaCI6MjQsImZpeGVkQXNzZXRzIjo2NSwidGFuZ2libGVBc3NldHMiOjUzLCJidWlsZGluZ3MiOjE5LCJtYWNoaW5lcnkiOjI0LCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6Nywic29mdHdhcmUiOjUsImxpYWJpbGl0aWVzIjo3NSwiY3VycmVudExpYWJpbGl0aWVzIjozOSwic2hvcnRUZXJtRGVidCI6MTIsImZpeGVkTGlhYmlsaXRpZXMiOjM2LCJsb25nVGVybURlYnQiOjI5LCJuZXRBc3NldHMiOjU3LCJzaGFyZWhvbGRlckVxdWl0eSI6NTQsImNhcGl0YWwiOjEwLCJjYXBleCI6NX0seyJ5ZWFyIjoyMDI0LCJhc3NldHMiOjE0MywiY3VycmVudEFzc2V0cyI6NzIsImNhc2giOjI1LCJmaXhlZEFzc2V0cyI6NzEsInRhbmdpYmxlQXNzZXRzIjo1OCwiYnVpbGRpbmdzIjoyMCwibWFjaGluZXJ5IjoyOCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjgsInNvZnR3YXJlIjo2LCJsaWFiaWxpdGllcyI6NzksImN1cnJlbnRMaWFiaWxpdGllcyI6NDEsInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozOCwibG9uZ1Rlcm1EZWJ0IjozMSwibmV0QXNzZXRzIjo2NCwic2hhcmVob2xkZXJFcXVpdHkiOjYxLCJjYXBpdGFsIjoxMCwiY2FwZXgiOjh9LHsieWVhciI6MjAyNSwiYXNzZXRzIjoxNTYsImN1cnJlbnRBc3NldHMiOjc4LCJjYXNoIjoyNywiZml4ZWRBc3NldHMiOjc4LCJ0YW5naWJsZUFzc2V0cyI6NjQsImJ1aWxkaW5ncyI6MjIsIm1hY2hpbmVyeSI6MzIsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo5LCJzb2Z0d2FyZSI6NywibGlhYmlsaXRpZXMiOjgzLCJjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJzaG9ydFRlcm1EZWJ0IjoxMSwiZml4ZWRMaWFiaWxpdGllcyI6NDAsImxvbmdUZXJtRGVidCI6MzIsIm5ldEFzc2V0cyI6NzMsInNoYXJlaG9sZGVyRXF1aXR5Ijo3MCwiY2FwaXRhbCI6MTAsImNhcGV4IjoxMH1dLCJmdXR1cmVDYXBleCI6W3sieWVhciI6MjAyNiwidmFsdWUiOjB9LHsieWVhciI6MjAyNywidmFsdWUiOjB9LHsieWVhciI6MjAyOCwidmFsdWUiOjB9LHsieWVhciI6MjAyOSwidmFsdWUiOjB9LHsieWVhciI6MjAzMCwidmFsdWUiOjB9LHsieWVhciI6MjAzMSwidmFsdWUiOjB9XSwiZHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTcyNDYzNzY4MTE1ODYsInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsInByb2plY3RTZ2FSYXRlRW5kIjowLjExLCJvdGhlclNnYVJhdGVFbmQiOjAuMTA5Mjg1NzE0Mjg1NzE0MjgsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJpbnZlc3RtZW50IjoyMywic3Vic2lkeSI6Ny42NiwibG9jYWxCZW5jaG1hcmsiOjIzfSwiZHJpdmVyUmFuZ2VzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOlstMC4wNSwwLjNdLCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjpbMCwwLjk5XSwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOlswLDAuOTldLCJwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOlswLDFdLCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOlswLDFdLCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOlstMC41LDAuNV0sIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6Wy0wLjUsMC41XSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJlZmZlY3RpdmVUYXhSYXRlIjpbMCwwLjZdLCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6WzAsMS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNl0sInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOlswLjAxOTMyNTMzMDUwMTg0NjkyNywwLjAyMDczNTk5NDE4MzE4OTE2Nl0sInByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6WzAuMDQwNzYwODY5NTY1MjE3MTg0LDAuMDQ0Mzg0MDU3OTcxMDE0NTJdLCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6WzAsMC4wMDAxMzQ1NzU1NjkzNTgxOTczN10sIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkxMzk0NTcwMjM3MTc0NDMsMC4wMjA1NTM0NTk5MTQ3NjMwOTVdLCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6WzAuMDM5MTY2NjY2NjY2NjY2NjgsMC4wNDI1MDAwMDAwMDAwMDAwOV0sIm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDBdLCJwcm9qZWN0U2FsZXNHcm93dGgiOlswLjE1LDAuM10sIm90aGVyU2FsZXNHcm93dGgiOlswLjA2MDc2MDg2OTU2NTIxNzE5LDAuMDY0Mzg0MDU3OTcxMDE0NTNdLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjpbMCwwLjAzXSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOlswLjAwNSwwLjAwNTEzNDU3NTU2OTM1ODE5NzVdLCJwcm9qZWN0UGF5R3Jvd3RoIjpbMC4wNSwwLjFdLCJvdGhlclBheUdyb3d0aCI6WzAuMDI0MTM5NDU3MDIzNzE3NDQ0LDAuMDI1NTUzNDU5OTE0NzYzMDk2XSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjpbMCwwLjA4XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6WzAsMC4wOF0sIm90aGVySGVhZGNvdW50R3Jvd3RoIjpbMC4wNDQxNjY2NjY2NjY2NjY2OCwwLjA0NzUwMDAwMDAwMDAwMDA5XSwicHJvamVjdFNnYVJhdGVFbmQiOlswLjA4NDk5OTk5OTk5OTk5OTk5LDAuMTM1XSwib3RoZXJTZ2FSYXRlRW5kIjpbMC4wODkyODU3MTQyODU3MTQyNywwLjExOTI4NTcxNDI4NTcxNDI3XSwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOlswLjA0MjYzMTU3ODk0NzM2ODM2LDAuMDY1NTU1NTU1NTU1NTU1NThdLCJpbnZlc3RtZW50IjpbMTUsMjAwXSwic3Vic2lkeSI6WzEsNTBdLCJsb2NhbEJlbmNobWFyayI6WzAsMTAwXX0sInRhcmdldHMiOnsiY29tcGFueVNhbGVzQ2FnciI6eyJ2YWx1ZSI6MTUsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6ODIuNCwibWF4IjoyNTIuNjksInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJjb21wYW55UGF5U2NoZWR1bGUiOnsidmFsdWUiOjIsIm1heCI6NywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc1NoYXJlIjp7InZhbHVlIjo2MCwibWF4Ijo5NSwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0NhZ3IiOnsidmFsdWUiOjIyLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjc0LjgsIm1heCI6MTM2Ljg0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MTguNzgsIm1heCI6MzMuNDMsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUNhZ3IiOnsidmFsdWUiOjcsIm1heCI6MTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUluY3JlYXNlIjp7InZhbHVlIjoyLjg1LCJtYXgiOjMuNzQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJpbnZlc3RtZW50U2FsZXNSYXRpbyI6eyJ2YWx1ZSI6MTUsIm1heCI6NzAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvIjp7InZhbHVlIjoyMTMsIm1heCI6MzUwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibG9jYWxCZW5jaG1hcmsiOnsidmFsdWUiOjIzLCJtYXgiOjQwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUNhZ3IiOnsidmFsdWUiOjYsIm1heCI6MTAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5SW5jcmVhc2UiOnsidmFsdWUiOjAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9fSwiZm9yZWNhc3RPdmVycmlkZXMiOnsiMjAyOTpvdGhlcjpzYWxlcyI6ODUuMTMsIjIwMjk6cHJvamVjdDo3LTgiOjcuOX0sImZ1dHVyZUlucHV0QmFzaXMiOiJvdGhlciIsImlucHV0VmFsdWVzIjp7ImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xIjoxMzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTMiOjkyLjc1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6MC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMyLjY1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6MC44MiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEwIjowLjA5LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTIiOjExLjY3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjAuNjIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNCI6Mi40NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1IjowLjY0LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTgiOjEwLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTkiOjEwLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjAiOjcuNTEsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yNyI6MjEwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xIjo3MiwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTQiOjIzLjA0LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNiI6Ni43OCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTgiOjUuMTksImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny05IjowLjM2LCJhY3R1YWw6cHJvamVjdDoyMDIzOlAyLTQiOjAuNDUsImFjdHVhbDpwcm9qZWN0OjIwMjM6UDItMTQiOjEuMzUsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMyI6OTAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEiOjE0My4yLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMyI6OTcuMzgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi00IjowLjc2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNyI6MzQuNTIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi05IjowLjg2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEyIjoxMi40NywiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEzIjowLjY2LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTQiOjIuNTgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNSI6MC42NywiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE4IjoxMS4wMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE5IjoxMS4wMSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTIwIjo3LjcxLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjciOjIyMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMSI6NzYsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny00IjoyNC4zMiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTYiOjcuMDQsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny04Ijo1LjU5LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctOSI6MC4zOCwiYWN0dWFsOnByb2plY3Q6MjAyNDpQMi00IjowLjQ3LCJhY3R1YWw6cHJvamVjdDoyMDI0OlAyLTE0IjoxLjQzLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTMiOjk1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xIjoxNTAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0zIjoxMDIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi00IjowLjgsImFjdHVhbDpjb21wYW55OjIwMjU6Mi03IjozNi40LCJhY3R1YWw6Y29tcGFueToyMDI1OjItOSI6MC45LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTAiOjAuMSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEyIjoxMy4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTMiOjAuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE0IjoyLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNSI6MC43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTgiOjExLjMsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xOSI6MTEuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTIwIjo3LjkxLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjciOjIzMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMSI6ODAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNS42LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6Ny4zLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTkiOjAuNCwiYWN0dWFsOnByb2plY3Q6MjAyNTpQMi00IjowLjUsImFjdHVhbDpwcm9qZWN0OjIwMjU6UDItMTQiOjEuNSwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudEFzc2V0cyI6NjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXNoIjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NSwiYmFsYW5jZS1zaGVldDoyMDIzOnRhbmdpYmxlQXNzZXRzIjo1MywiYmFsYW5jZS1zaGVldDoyMDIzOmJ1aWxkaW5ncyI6MTksImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzppbnRhbmdpYmxlQXNzZXRzIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUsImJhbGFuY2Utc2hlZXQ6MjAyMzpsaWFiaWxpdGllcyI6NzUsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50TGlhYmlsaXRpZXMiOjM5LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZExpYWJpbGl0aWVzIjozNiwiYmFsYW5jZS1zaGVldDoyMDIzOmxvbmdUZXJtRGVidCI6MjksImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3LCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hhcmVob2xkZXJFcXVpdHkiOjU0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NSwiYmFsYW5jZS1zaGVldDoyMDI0OmFzc2V0cyI6MTQzLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudEFzc2V0cyI6NzIsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNSwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkQXNzZXRzIjo3MSwiYmFsYW5jZS1zaGVldDoyMDI0OnRhbmdpYmxlQXNzZXRzIjo1OCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAsImJhbGFuY2Utc2hlZXQ6MjAyNDptYWNoaW5lcnkiOjI4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c29mdHdhcmUiOjYsImJhbGFuY2Utc2hlZXQ6MjAyNDpsaWFiaWxpdGllcyI6NzksImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hvcnRUZXJtRGVidCI6MTIsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZExpYWJpbGl0aWVzIjozOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEsImJhbGFuY2Utc2hlZXQ6MjAyNDpuZXRBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hhcmVob2xkZXJFcXVpdHkiOjYxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBleCI6OCwiYmFsYW5jZS1zaGVldDoyMDI1OmFzc2V0cyI6MTU2LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXNoIjoyNywiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkQXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI1OmJ1aWxkaW5ncyI6MjIsImJhbGFuY2Utc2hlZXQ6MjAyNTptYWNoaW5lcnkiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTppbnRhbmdpYmxlQXNzZXRzIjo5LCJiYWxhbmNlLXNoZWV0OjIwMjU6c29mdHdhcmUiOjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hvcnRUZXJtRGVidCI6MTEsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MCwiYmFsYW5jZS1zaGVldDoyMDI1OmxvbmdUZXJtRGVidCI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpuZXRBc3NldHMiOjczLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwaXRhbCI6MTAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBleCI6MTAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC45OSwiZHJpdmVyOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvOjEiOjAuOTksImRyaXZlcjpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwiZHJpdmVyLXJhbmdlOnByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZToxIjoxLCJkcml2ZXI6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJkcml2ZXItcmFuZ2U6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjowLjksImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGU6MSI6MC4zLCJkcml2ZXI6b3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjEiOjAuMywiZHJpdmVyOnByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdE5vbk9wZXJhdGluZ1JhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOnByb2plY3ROb25PcGVyYXRpbmdSYXRlOjEiOjAuNSwiZHJpdmVyOm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJOb25PcGVyYXRpbmdSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpvdGhlck5vbk9wZXJhdGluZ1JhdGU6MSI6MC41LCJkcml2ZXI6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6b3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6ZWZmZWN0aXZlVGF4UmF0ZSI6MC4zLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZTowIjowLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZToxIjowLjYsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjUuNTUxMTE1MTIzMTI1NzgzZS0xNywiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZTowIjowLjAxOTMyNTMzMDUwMTg0NjkyNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA3MzU5OTQxODMxODkxNjYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNTcyNDYzNzY4MTE1ODU0LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZTowIjowLjA0MDc2MDg2OTU2NTIxNzE4NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNDQzODQwNTc5NzEwMTQ1MiwiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjAuMDAwMTM0NTc1NTY5MzU4MTk3MzcsImRyaXZlcjpvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDE5MTM5NDU3MDIzNzE3NDQzLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA1NTM0NTk5MTQ3NjMwOTUsImRyaXZlcjpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZToxIjowLjA4LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjAzOTE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNDI1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MCI6MC4xNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjMsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MCI6MC4wMjQxMzk0NTcwMjM3MTc0NDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDoxIjowLjAyNTU1MzQ1OTkxNDc2MzA5NiwiZHJpdmVyOm90aGVyT2ZmaWNlclBheUdyb3d0aCI6MC4wNDUsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aDoxIjowLjA4LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTgzMzMzMzMzMzMzMzM4NiwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjAiOjAuMDQ0MTY2NjY2NjY2NjY2NjgsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDoxIjowLjA0NzUwMDAwMDAwMDAwMDA5LCJkcml2ZXI6cHJvamVjdFNnYVJhdGVFbmQiOjAuMTEsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDowIjowLjA4NDk5OTk5OTk5OTk5OTk5LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MSI6MC4xMzUsImRyaXZlcjpvdGhlclNnYVJhdGVFbmQiOjAuMTA5Mjg1NzE0Mjg1NzE0MjgsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MCI6MC4wODkyODU3MTQyODU3MTQyNywiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDoxIjowLjExOTI4NTcxNDI4NTcxNDI3LCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzODAxMTY5NTkwNjQzMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDowIjowLjA0MjYzMTU3ODk0NzM2ODM2LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MSI6MC4wNjU1NTU1NTU1NTU1NTU1OCwiZHJpdmVyOmludmVzdG1lbnQiOjIzLCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDowIjoxNSwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MSI6MjAwLCJkcml2ZXI6c3Vic2lkeSI6Ny42NiwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MCI6MSwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MSI6NTAsImRyaXZlcjpsb2NhbEJlbmNobWFyayI6MjMsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazowIjowLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MSI6MTAwLCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2Fncjp2YWx1ZSI6MTUsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTp2YWx1ZSI6ODIuNCwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTp2YWx1ZSI6MiwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTptYXgiOjcsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTp2YWx1ZSI6NjAsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTptYXgiOjk1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2Fncjp2YWx1ZSI6MjIsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTp2YWx1ZSI6NzQuOCwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2Fncjp2YWx1ZSI6MjEsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6bWF4IjozNSwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTp2YWx1ZSI6MTguNzgsInRhcmdldDplbXBsb3llZVBheUNhZ3I6dmFsdWUiOjcsInRhcmdldDplbXBsb3llZVBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6dmFsdWUiOjIuODUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MTUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTptYXgiOjI1Mi42OSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOm1heCI6MTM2Ljg0LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOm1heCI6MzMuNDMsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOm1heCI6My43NH0sIm1ldHJpY0dyb3VwQmFzZXMiOnsiY29tcGFueVNhbGVzIjoicmF0ZSIsInByb2plY3RTYWxlcyI6InJhdGUiLCJsYWJvclByb2R1Y3Rpdml0eSI6InJhdGUiLCJlbXBsb3llZVBheSI6InJhdGUifSwiYXBwbGljYXRpb25DYXRlZ29yeSI6ImdlbmVyYWwiLCJhZGp1c3RlZERyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsInByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwib3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwicHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yNSwib3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMiwicHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsInByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJvdGhlck5vbk9wZXJhdGluZ1JhdGUiOi0wLjAwNSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjowLCJlZmZlY3RpdmVUYXhSYXRlIjowLjMsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQxMTgyMzgzMDQwOTM1NSwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MS4xNzQxODY0OTEwNjQ0NjZlLTE2LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzODU2MjA1OTEzMzU2MiwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTIxNTg4ODg3MTgzOTQ1NSwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQxMzg0NDUwMzUzNjE4Nywib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI1Njk3MDU2MzE2MTMxOCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTgxOTg4OTExNDM0OTkxNSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA3OTQ0MTE0MTQ5ODIyMjUsIm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMjAzNzA4MTgxMTU0MTI2OCwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI2MjE3MzU2ODE4MzE4LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNDk1MjgwNjkyMjY2MDg5NSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA4NDgxMjgzMzc0ODY2NTAxLCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NjM3OTU1NTk2MzczNCwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wMjY1MzQwMDY5ODczNjg5OSwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODY4Mzk2ODIxODYwOTA0LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4xMDk5Nzc1ODM4MTI3MzU1Niwib3RoZXJTZ2FSYXRlRW5kIjowLjEwOTMyMTYzMDk2ODAxODY1LCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM3NjI5Njg0Mjg5MjM1OSwiaW52ZXN0bWVudCI6MjMsInN1YnNpZHkiOjcuNjYsImxvY2FsQmVuY2htYXJrIjoyM319</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4LCJvcmRpbmFyeUluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsInByZVRheEluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsIm5ldEluY29tZSI6Ny41MX19LHsieWVhciI6MjAyNCwicm9sZSI6InByZXZpb3VzIiwicHJvamVjdCI6eyJzYWxlcyI6NzYsImNvZ3MiOjUxLjY4LCJlbXBsb3llZVBheSI6NS41OSwib2ZmaWNlclBheSI6MC4zOCwiZGVwcmVjaWF0aW9uIjoxLjksIm90aGVyU2dhIjo5LjUsImhlYWRjb3VudCI6OTUsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjUuMzEsImVtcGxveWVlQm9udXMiOjAuMjgsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzQsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40Nywic2dhRGVwcmVjaWF0aW9uIjoxLjQzLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM4fSwib3RoZXIiOnsic2FsZXMiOjY3LjIsImNvZ3MiOjQ1LjcsImVtcGxveWVlUGF5Ijo3LjU0LCJvZmZpY2VyUGF5IjowLjU4LCJkZXByZWNpYXRpb24iOjEuNDQsIm90aGVyU2dhIjo3LjY4LCJoZWFkY291bnQiOjEyNSwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ny4xNiwiZW1wbG95ZWVCb251cyI6MC4zOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41Miwib2ZmaWNlckJvbnVzIjowLjA2LCJjb2dzRGVwcmVjaWF0aW9uIjowLjI5LCJzZ2FEZXByZWNpYXRpb24iOjEuMTUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMjksIm9yZGluYXJ5SW5jb21lIjozLjk2OTk5OTk5OTk5OTk5NywicHJlVGF4SW5jb21lIjozLjk2OTk5OTk5OTk5OTk5NywibmV0SW5jb21lIjo3LjcxfX0seyJ5ZWFyIjoyMDI1LCJyb2xlIjoibGF0ZXN0IiwicHJvamVjdCI6eyJzYWxlcyI6ODAsImNvZ3MiOjU0LjQsImVtcGxveWVlUGF5Ijo2LCJlbXBsb3llZVNhbGFyeSI6NS43LCJlbXBsb3llZUJvbnVzIjowLjMsIm9mZmljZXJQYXkiOjAuNCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNiwib2ZmaWNlckJvbnVzIjowLjA0LCJkZXByZWNpYXRpb24iOjIsImNvZ3NEZXByZWNpYXRpb24iOjAuNSwic2dhRGVwcmVjaWF0aW9uIjoxLjUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuNCwib3RoZXJTZ2EiOjEwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwLCJjb2dzIjo0Ny42LCJlbXBsb3llZVBheSI6OCwiZW1wbG95ZWVTYWxhcnkiOjcuNiwiZW1wbG95ZWVCb251cyI6MC40LCJvZmZpY2VyUGF5IjowLjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTQsIm9mZmljZXJCb251cyI6MC4wNiwiZGVwcmVjaWF0aW9uIjoxLjUsImNvZ3NEZXByZWNpYXRpb24iOjAuMywic2dhRGVwcmVjaWF0aW9uIjoxLjIsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMywib3RoZXJTZ2EiOjgsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjozLjk5OTk5OTk5OTk5OTk5NjQsInByZVRheEluY29tZSI6My45OTk5OTk5OTk5OTk5OTY0LCJuZXRJbmNvbWUiOjcuOTF9fV0sImJhbGFuY2VTaGVldHMiOlt7InllYXIiOjIwMjMsImFzc2V0cyI6MTMyLCJjdXJyZW50QXNzZXRzIjo2NywiY2FzaCI6MjQsImZpeGVkQXNzZXRzIjo2NSwidGFuZ2libGVBc3NldHMiOjUzLCJidWlsZGluZ3MiOjE5LCJtYWNoaW5lcnkiOjI0LCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6Nywic29mdHdhcmUiOjUsImxpYWJpbGl0aWVzIjo3NSwiY3VycmVudExpYWJpbGl0aWVzIjozOSwic2hvcnRUZXJtRGVidCI6MTIsImZpeGVkTGlhYmlsaXRpZXMiOjM2LCJsb25nVGVybURlYnQiOjI5LCJuZXRBc3NldHMiOjU3LCJzaGFyZWhvbGRlckVxdWl0eSI6NTQsImNhcGl0YWwiOjEwLCJjYXBleCI6NX0seyJ5ZWFyIjoyMDI0LCJhc3NldHMiOjE0MywiY3VycmVudEFzc2V0cyI6NzIsImNhc2giOjI1LCJmaXhlZEFzc2V0cyI6NzEsInRhbmdpYmxlQXNzZXRzIjo1OCwiYnVpbGRpbmdzIjoyMCwibWFjaGluZXJ5IjoyOCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjgsInNvZnR3YXJlIjo2LCJsaWFiaWxpdGllcyI6NzksImN1cnJlbnRMaWFiaWxpdGllcyI6NDEsInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozOCwibG9uZ1Rlcm1EZWJ0IjozMSwibmV0QXNzZXRzIjo2NCwic2hhcmVob2xkZXJFcXVpdHkiOjYxLCJjYXBpdGFsIjoxMCwiY2FwZXgiOjh9LHsieWVhciI6MjAyNSwiYXNzZXRzIjoxNTYsImN1cnJlbnRBc3NldHMiOjc4LCJjYXNoIjoyNywiZml4ZWRBc3NldHMiOjc4LCJ0YW5naWJsZUFzc2V0cyI6NjQsImJ1aWxkaW5ncyI6MjIsIm1hY2hpbmVyeSI6MzIsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo5LCJzb2Z0d2FyZSI6NywibGlhYmlsaXRpZXMiOjgzLCJjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJzaG9ydFRlcm1EZWJ0IjoxMSwiZml4ZWRMaWFiaWxpdGllcyI6NDAsImxvbmdUZXJtRGVidCI6MzIsIm5ldEFzc2V0cyI6NzMsInNoYXJlaG9sZGVyRXF1aXR5Ijo3MCwiY2FwaXRhbCI6MTAsImNhcGV4IjoxMH1dLCJmdXR1cmVDYXBleCI6W3sieWVhciI6MjAyNiwidmFsdWUiOjB9LHsieWVhciI6MjAyNywidmFsdWUiOjB9LHsieWVhciI6MjAyOCwidmFsdWUiOjB9LHsieWVhciI6MjAyOSwidmFsdWUiOjB9LHsieWVhciI6MjAzMCwidmFsdWUiOjB9LHsieWVhciI6MjAzMSwidmFsdWUiOjB9XSwiZHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTcyNDYzNzY4MTE1ODYsInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsInByb2plY3RTZ2FSYXRlRW5kIjowLjAxNSwib3RoZXJTZ2FSYXRlRW5kIjowLjAwNSwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzODAxMTY5NTkwNjQzMjUsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOlswLDAuOTldLCJvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6WzAsMC45OV0sInByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlIjpbMCwxXSwib3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlIjpbMCwxXSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6WzAsMV0sIm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjpbMCwxXSwicHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZSI6WzAsMV0sIm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlIjpbMCwxXSwicHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjpbMCwwLjNdLCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjpbMCwwLjNdLCJwcm9qZWN0Tm9uT3BlcmF0aW5nUmF0ZSI6Wy0wLjUsMC41XSwib3RoZXJOb25PcGVyYXRpbmdSYXRlIjpbLTAuNSwwLjVdLCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOlstMC41LDAuNV0sIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOlstMC41LDAuNV0sImVmZmVjdGl2ZVRheFJhdGUiOlswLDAuNl0sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwxLjY2NTMzNDUzNjkzNzczNDhlLTE2XSwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MzI1MzMwNTAxODQ2OTI3LDAuMDIwNzM1OTk0MTgzMTg5MTY2XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDBdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNDA3NjA4Njk1NjUyMTcxODQsMC4wNDQzODQwNTc5NzEwMTQ1Ml0sIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAwMDEzNDU3NTU2OTM1ODE5NzM3XSwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOlswLjAxOTEzOTQ1NzAyMzcxNzQ0MywwLjAyMDU1MzQ1OTkxNDc2MzA5NV0sIm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6WzAsMC4wOF0sIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wMzkxNjY2NjY2NjY2NjY2OCwwLjA0MjUwMDAwMDAwMDAwMDA5XSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RTYWxlc0dyb3d0aCI6WzAuMTUsMC4zXSwib3RoZXJTYWxlc0dyb3d0aCI6WzAuMDYwNzYwODY5NTY1MjE3MTksMC4wNjQzODQwNTc5NzEwMTQ1M10sInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOlswLDAuMDNdLCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6WzAuMDA1LDAuMDA1MTM0NTc1NTY5MzU4MTk3NV0sInByb2plY3RQYXlHcm93dGgiOlswLjA1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMC4wMjQxMzk0NTcwMjM3MTc0NDQsMC4wMjU1NTM0NTk5MTQ3NjMwOTZdLCJvdGhlck9mZmljZXJQYXlHcm93dGgiOlswLDAuMDhdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGgiOlswLjA0NDE2NjY2NjY2NjY2NjY4LDAuMDQ3NTAwMDAwMDAwMDAwMDldLCJwcm9qZWN0U2dhUmF0ZUVuZCI6WzAsMC4wM10sIm90aGVyU2dhUmF0ZUVuZCI6WzAsMC4wMV0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjpbMC4wNDI2MzE1Nzg5NDczNjgzNiwwLjA2NTU1NTU1NTU1NTU1NTU4XSwiaW52ZXN0bWVudCI6WzE1LDIwMF0sInN1YnNpZHkiOlsxLDUwXSwibG9jYWxCZW5jaG1hcmsiOlswLDEwMF19LCJ0YXJnZXRzIjp7ImNvbXBhbnlTYWxlc0NhZ3IiOnsidmFsdWUiOjE1LCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjgyLjQsIm1heCI6MjUyLjY5LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjoyLCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NjAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo3NC44LCJtYXgiOjEzNi44NCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImxhYm9yUHJvZHVjdGl2aXR5Q2FnciI6eyJ2YWx1ZSI6MjEsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkSW5jcmVhc2UiOnsidmFsdWUiOjE4Ljc4LCJtYXgiOjMzLjQzLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6Mi44NSwibWF4IjozLjc0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiaW52ZXN0bWVudFNhbGVzUmF0aW8iOnsidmFsdWUiOjE1LCJtYXgiOjcwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZFN1YnNpZHlSYXRpbyI6eyJ2YWx1ZSI6MjEzLCJtYXgiOjM1MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImxvY2FsQmVuY2htYXJrIjp7InZhbHVlIjoyMywibWF4Ijo0MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlDYWdyIjp7InZhbHVlIjo2LCJtYXgiOjEwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUluY3JlYXNlIjp7InZhbHVlIjowLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfX0sImZvcmVjYXN0T3ZlcnJpZGVzIjp7IjIwMjk6b3RoZXI6c2FsZXMiOjg1LjEzLCIyMDI5OnByb2plY3Q6Ny04Ijo3Ljl9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2LjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mi43NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTQiOjAuNzMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi03IjozMi42NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTkiOjAuODIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMCI6MC4wOSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEyIjoxMS42NywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEzIjowLjYyLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTQiOjIuNDUsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNSI6MC42NCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE4IjoxMC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE5IjoxMC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTIwIjo3LjUxLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjciOjIxMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMSI6NzIsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny00IjoyMy4wNCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjYuNzgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny04Ijo1LjE5LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOSI6MC4zNiwiYWN0dWFsOnByb2plY3Q6MjAyMzpQMi00IjowLjQ1LCJhY3R1YWw6cHJvamVjdDoyMDIzOlAyLTE0IjoxLjM1LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTMiOjkwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xIjoxNDMuMiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTMiOjk3LjM4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNCI6MC43NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTciOjM0LjUyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItOSI6MC44NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMiI6MTIuNDcsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMyI6MC42NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjoyLjU4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTUiOjAuNjcsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xOCI6MTEuMDEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xOSI6MTEuMDEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0yMCI6Ny43MSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTI3IjoyMjAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEiOjc2LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNCI6MjQuMzIsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny02Ijo3LjA0LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctOCI6NS41OSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTkiOjAuMzgsImFjdHVhbDpwcm9qZWN0OjIwMjQ6UDItNCI6MC40NywiYWN0dWFsOnByb2plY3Q6MjAyNDpQMi0xNCI6MS40MywiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6MC44LCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTkiOjAuOSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjowLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6Mi43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTUiOjAuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE4IjoxMS4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTkiOjExLjMsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yMCI6Ny45MSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI3IjoyMzAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNCI6MjUuNiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTYiOjcuMywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTgiOjYsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny05IjowLjQsImFjdHVhbDpwcm9qZWN0OjIwMjU6UDItNCI6MC41LCJhY3R1YWw6cHJvamVjdDoyMDI1OlAyLTE0IjoxLjUsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xMyI6MTAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTQiOjIsImJhbGFuY2Utc2hlZXQ6MjAyMzphc3NldHMiOjEzMiwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRBc3NldHMiOjY3LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FzaCI6MjQsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZEFzc2V0cyI6NjUsImJhbGFuY2Utc2hlZXQ6MjAyMzp0YW5naWJsZUFzc2V0cyI6NTMsImJhbGFuY2Utc2hlZXQ6MjAyMzpidWlsZGluZ3MiOjE5LCJiYWxhbmNlLXNoZWV0OjIwMjM6bWFjaGluZXJ5IjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmxhbmQiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjM6aW50YW5naWJsZUFzc2V0cyI6NywiYmFsYW5jZS1zaGVldDoyMDIzOnNvZnR3YXJlIjo1LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGlhYmlsaXRpZXMiOjc1LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudExpYWJpbGl0aWVzIjozOSwiYmFsYW5jZS1zaGVldDoyMDIzOnNob3J0VGVybURlYnQiOjEyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRMaWFiaWxpdGllcyI6MzYsImJhbGFuY2Utc2hlZXQ6MjAyMzpsb25nVGVybURlYnQiOjI5LCJiYWxhbmNlLXNoZWV0OjIwMjM6bmV0QXNzZXRzIjo1NywiYmFsYW5jZS1zaGVldDoyMDIzOnNoYXJlaG9sZGVyRXF1aXR5Ijo1NCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGl0YWwiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwZXgiOjUsImJhbGFuY2Utc2hlZXQ6MjAyNDphc3NldHMiOjE0MywiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRBc3NldHMiOjcyLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FzaCI6MjUsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZEFzc2V0cyI6NzEsImJhbGFuY2Utc2hlZXQ6MjAyNDp0YW5naWJsZUFzc2V0cyI6NTgsImJhbGFuY2Utc2hlZXQ6MjAyNDpidWlsZGluZ3MiOjIwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bWFjaGluZXJ5IjoyOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxhbmQiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6aW50YW5naWJsZUFzc2V0cyI6OCwiYmFsYW5jZS1zaGVldDoyMDI0OnNvZnR3YXJlIjo2LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGlhYmlsaXRpZXMiOjc5LCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudExpYWJpbGl0aWVzIjo0MSwiYmFsYW5jZS1zaGVldDoyMDI0OnNob3J0VGVybURlYnQiOjEyLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRMaWFiaWxpdGllcyI6MzgsImJhbGFuY2Utc2hlZXQ6MjAyNDpsb25nVGVybURlYnQiOjMxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bmV0QXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI0OnNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGl0YWwiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwZXgiOjgsImJhbGFuY2Utc2hlZXQ6MjAyNTphc3NldHMiOjE1NiwiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRBc3NldHMiOjc4LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FzaCI6MjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTp0YW5naWJsZUFzc2V0cyI6NjQsImJhbGFuY2Utc2hlZXQ6MjAyNTpidWlsZGluZ3MiOjIyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bWFjaGluZXJ5IjozMiwiYmFsYW5jZS1zaGVldDoyMDI1OmxhbmQiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjU6aW50YW5naWJsZUFzc2V0cyI6OSwiYmFsYW5jZS1zaGVldDoyMDI1OnNvZnR3YXJlIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjU6bGlhYmlsaXRpZXMiOjgzLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudExpYWJpbGl0aWVzIjo0MywiYmFsYW5jZS1zaGVldDoyMDI1OnNob3J0VGVybURlYnQiOjExLCJiYWxhbmNlLXNoZWV0OjIwMjU6Zml4ZWRMaWFiaWxpdGllcyI6NDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpsb25nVGVybURlYnQiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bmV0QXNzZXRzIjo3MywiYmFsYW5jZS1zaGVldDoyMDI1OnNoYXJlaG9sZGVyRXF1aXR5Ijo3MCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGl0YWwiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwZXgiOjEwLCJkcml2ZXI6cHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MCI6LTAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjEiOjAuMywiZHJpdmVyOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvOjEiOjAuOTksImRyaXZlcjpvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybzoxIjowLjk5LCJkcml2ZXI6cHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsImRyaXZlci1yYW5nZTpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmU6MSI6MSwiZHJpdmVyOm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwiZHJpdmVyLXJhbmdlOm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlOjEiOjEsImRyaXZlcjpwcm9qZWN0T2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjowLjksImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZToxIjoxLCJkcml2ZXI6b3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMiwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZToxIjoxLCJkcml2ZXI6cHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNSwiZHJpdmVyLXJhbmdlOnByb2plY3RSZXNlYXJjaERldmVsb3BtZW50UmF0ZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjEiOjAuMywiZHJpdmVyOm90aGVyUmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA0LCJkcml2ZXItcmFuZ2U6b3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZToxIjowLjMsImRyaXZlcjpwcm9qZWN0Tm9uT3BlcmF0aW5nUmF0ZSI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3ROb25PcGVyYXRpbmdSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpwcm9qZWN0Tm9uT3BlcmF0aW5nUmF0ZToxIjowLjUsImRyaXZlcjpvdGhlck5vbk9wZXJhdGluZ1JhdGUiOi0wLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyTm9uT3BlcmF0aW5nUmF0ZTowIjotMC41LCJkcml2ZXItcmFuZ2U6b3RoZXJOb25PcGVyYXRpbmdSYXRlOjEiOjAuNSwiZHJpdmVyOnByb2plY3RFeHRyYW9yZGluYXJ5UmF0ZSI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RFeHRyYW9yZGluYXJ5UmF0ZTowIjotMC41LCJkcml2ZXItcmFuZ2U6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlOjEiOjAuNSwiZHJpdmVyOm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImRyaXZlci1yYW5nZTpvdGhlckV4dHJhb3JkaW5hcnlSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpvdGhlckV4dHJhb3JkaW5hcnlSYXRlOjEiOjAuNSwiZHJpdmVyOmVmZmVjdGl2ZVRheFJhdGUiOjAuMywiZHJpdmVyLXJhbmdlOmVmZmVjdGl2ZVRheFJhdGU6MCI6MCwiZHJpdmVyLXJhbmdlOmVmZmVjdGl2ZVRheFJhdGU6MSI6MC42LCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjEuNjY1MzM0NTM2OTM3NzM0OGUtMTYsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkzMjUzMzA1MDE4NDY5MjcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNzM1OTk0MTgzMTg5MTY2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLjAxOTEzOTQ1NzAyMzcxNzQ0MywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNTUzNDU5OTE0NzYzMDk1LCJkcml2ZXI6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wMzkxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDQyNTAwMDAwMDAwMDAwMDksImRyaXZlcjpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjAiOjAuMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MSI6MC4zLCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NzI0NjM3NjgxMTU4NiwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MCI6MC4wNjA3NjA4Njk1NjUyMTcxOSwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MSI6MC4wNjQzODQwNTc5NzEwMTQ1MywiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZToxIjowLjAzLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDoxIjowLjAwNTEzNDU3NTU2OTM1ODE5NzUsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDowIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDoxIjowLjEsImRyaXZlcjpvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjAiOjAuMDI0MTM5NDU3MDIzNzE3NDQ0LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wMjU1NTM0NTk5MTQ3NjMwOTYsImRyaXZlcjpvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGg6MSI6MC4wOCwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjowLjA0NDE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MSI6MC4wNDc1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjAxNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDoxIjowLjAzLCJkcml2ZXI6b3RoZXJTZ2FSYXRlRW5kIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMDEsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAuMDQyNjMxNTc4OTQ3MzY4MzYsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjA2NTU1NTU1NTU1NTU1NTU4LCJkcml2ZXI6aW52ZXN0bWVudCI6MjMsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjAiOjE1LCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDoxIjoyMDAsImRyaXZlcjpzdWJzaWR5Ijo3LjY2LCJkcml2ZXItcmFuZ2U6c3Vic2lkeTowIjoxLCJkcml2ZXItcmFuZ2U6c3Vic2lkeToxIjo1MCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoxNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjo4Mi40LCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjoyLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOm1heCI6NywidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOnZhbHVlIjo2MCwidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOm1heCI6OTUsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOnZhbHVlIjoyMiwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOnZhbHVlIjo3NC44LCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOnZhbHVlIjoyMSwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2FncjptYXgiOjM1LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOnZhbHVlIjoxOC43OCwidGFyZ2V0OmVtcGxveWVlUGF5Q2Fncjp2YWx1ZSI6NywidGFyZ2V0OmVtcGxveWVlUGF5Q2FncjptYXgiOjEwLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlJbmNyZWFzZTp2YWx1ZSI6Mi44NSwidGFyZ2V0OmludmVzdG1lbnRTYWxlc1JhdGlvOnZhbHVlIjoxNSwidGFyZ2V0OmludmVzdG1lbnRTYWxlc1JhdGlvOm1heCI6NzAsInRhcmdldDp2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvOnZhbHVlIjoyMTMsInRhcmdldDp2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvOm1heCI6MzUwLCJ0YXJnZXQ6bG9jYWxCZW5jaG1hcms6dmFsdWUiOjIzLCJ0YXJnZXQ6bG9jYWxCZW5jaG1hcms6bWF4Ijo0MCwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOnZhbHVlIjo2LCJ0YXJnZXQ6b2ZmaWNlclBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0Om9mZmljZXJQYXlJbmNyZWFzZTp2YWx1ZSI6MCwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOm1heCI6MjUyLjY5LCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6bWF4IjoxMzYuODQsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6bWF4IjozMy40MywidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6bWF4IjozLjc0fSwibWV0cmljR3JvdXBCYXNlcyI6eyJjb21wYW55U2FsZXMiOiJyYXRlIiwicHJvamVjdFNhbGVzIjoicmF0ZSIsImxhYm9yUHJvZHVjdGl2aXR5IjoicmF0ZSIsImVtcGxveWVlUGF5IjoicmF0ZSJ9LCJhcHBsaWNhdGlvbkNhdGVnb3J5IjoiZ2VuZXJhbCIsImFkanVzdGVkRHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDExODIzODMwNDA5MzU1LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjoxLjE3NDE4NjQ5MTA2NDQ2NmUtMTYsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDM4NTYyMDU5MTMzNTYyLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1MjE1ODg4ODcxODM5NDU1LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDEzODQ0NTAzNTM2MTg3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU2OTcwNTYzMTYxMzE4LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODE5ODg5MTE0MzQ5OTE1LCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDc5NDQxMTQxNDk4MjIyNSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyMDM3MDgxODExNTQxMjY4LCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjYyMTczNTY4MTgzMTgsInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE0OTUyODA2OTIyNjYwODk1LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDg0ODEyODMzNzQ4NjY1MDEsIm90aGVyUGF5R3Jvd3RoIjowLjAyNDg2Mzc5NTU1OTYzNzM0LCJvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjAyNjUzNDAwNjk4NzM2ODk5LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4NjgzOTY4MjE4NjA5MDQsInByb2plY3RTZ2FSYXRlRW5kIjowLjAxNDk4NjU1MDI4NzY0MTMzOSwib3RoZXJTZ2FSYXRlRW5kIjowLjAwNTAxMTk3MjIyNzQzNDc5MiwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzNzYyOTY4NDI4OTIzNTksImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9fQ==</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use historical cogs rates for forecast bounds
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -204,7 +204,7 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <v>15.474805389539558</v>
+        <v>15.460356409122511</v>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
@@ -234,7 +234,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <v>93.4</v>
+        <v>93.29999999999998</v>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
@@ -264,7 +264,7 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <v>2.002890072409058</v>
+        <v>2.022898486039626</v>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
@@ -294,7 +294,7 @@
         </is>
       </c>
       <c r="B11" s="2">
-        <v>63.919228315129686</v>
+        <v>63.91319040288364</v>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
@@ -324,7 +324,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>22.037045725736924</v>
+        <v>22.022274428397214</v>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
@@ -354,7 +354,7 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <v>76.60000000000001</v>
+        <v>76.53</v>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
@@ -384,7 +384,7 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <v>24.447010059327056</v>
+        <v>24.78660721617638</v>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
@@ -414,7 +414,7 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <v>19.660000000000004</v>
+        <v>19.65</v>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
@@ -444,7 +444,7 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <v>7.017971691139446</v>
+        <v>7.009078296607085</v>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B17" s="2">
-        <v>2.380000000000001</v>
+        <v>2.3</v>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <v>256.6579634464752</v>
+        <v>256.5274151436031</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
@@ -1259,22 +1259,22 @@
         <v>150</v>
       </c>
       <c r="E3" s="4">
-        <v>157.31</v>
+        <v>157.3</v>
       </c>
       <c r="F3" s="4">
-        <v>164.98000000000002</v>
+        <v>164.97</v>
       </c>
       <c r="G3" s="4">
         <v>173.03</v>
       </c>
       <c r="H3" s="4">
-        <v>199.48</v>
+        <v>199.45</v>
       </c>
       <c r="I3" s="4">
-        <v>230.01</v>
+        <v>229.95</v>
       </c>
       <c r="J3" s="4">
-        <v>266.43</v>
+        <v>266.33</v>
       </c>
     </row>
     <row r="4">
@@ -1295,22 +1295,22 @@
         <v>4.748603351955305</v>
       </c>
       <c r="E4" s="2">
-        <v>4.8733333333333295</v>
+        <v>4.866666666666664</v>
       </c>
       <c r="F4" s="2">
-        <v>4.875723094526752</v>
+        <v>4.876033057851226</v>
       </c>
       <c r="G4" s="2">
-        <v>4.879379318705279</v>
+        <v>4.885736800630425</v>
       </c>
       <c r="H4" s="2">
-        <v>15.286366526035945</v>
+        <v>15.269028492168978</v>
       </c>
       <c r="I4" s="2">
-        <v>15.304792460397042</v>
+        <v>15.292053146151918</v>
       </c>
       <c r="J4" s="2">
-        <v>15.834094169818712</v>
+        <v>15.820830615351156</v>
       </c>
     </row>
     <row r="5">
@@ -1332,19 +1332,19 @@
         <v>106.97</v>
       </c>
       <c r="F5" s="2">
-        <v>112.19</v>
+        <v>112.18</v>
       </c>
       <c r="G5" s="2">
         <v>117.66</v>
       </c>
       <c r="H5" s="2">
-        <v>134.37</v>
+        <v>134.36</v>
       </c>
       <c r="I5" s="2">
-        <v>154.12</v>
+        <v>154.07999999999998</v>
       </c>
       <c r="J5" s="2">
-        <v>177.51</v>
+        <v>177.45</v>
       </c>
     </row>
     <row r="6">
@@ -1397,22 +1397,22 @@
         <v>48</v>
       </c>
       <c r="E7" s="4">
-        <v>50.34</v>
+        <v>50.33000000000001</v>
       </c>
       <c r="F7" s="4">
-        <v>52.79000000000002</v>
+        <v>52.78999999999999</v>
       </c>
       <c r="G7" s="4">
         <v>55.370000000000005</v>
       </c>
       <c r="H7" s="4">
-        <v>65.10999999999999</v>
+        <v>65.08999999999997</v>
       </c>
       <c r="I7" s="4">
-        <v>75.88999999999999</v>
+        <v>75.87</v>
       </c>
       <c r="J7" s="4">
-        <v>88.92000000000002</v>
+        <v>88.88</v>
       </c>
     </row>
     <row r="8">
@@ -1431,22 +1431,22 @@
         <v>32</v>
       </c>
       <c r="E8" s="2">
-        <v>32.00050854999682</v>
+        <v>31.996185632549274</v>
       </c>
       <c r="F8" s="2">
-        <v>31.997817917323324</v>
+        <v>31.99975753167242</v>
       </c>
       <c r="G8" s="2">
         <v>32.00023117378489</v>
       </c>
       <c r="H8" s="2">
-        <v>32.63986364547824</v>
+        <v>32.63474555026321</v>
       </c>
       <c r="I8" s="2">
-        <v>32.994217642711185</v>
+        <v>32.99412915851273</v>
       </c>
       <c r="J8" s="2">
-        <v>33.37461997522802</v>
+        <v>33.37213231705027</v>
       </c>
     </row>
     <row r="9">
@@ -1465,22 +1465,22 @@
         <v>36.4</v>
       </c>
       <c r="E9" s="2">
-        <v>38.26</v>
+        <v>38.269999999999996</v>
       </c>
       <c r="F9" s="2">
-        <v>40.26</v>
+        <v>40.28</v>
       </c>
       <c r="G9" s="2">
-        <v>42.400000000000006</v>
+        <v>42.41</v>
       </c>
       <c r="H9" s="2">
         <v>46.18</v>
       </c>
       <c r="I9" s="2">
-        <v>50.8</v>
+        <v>50.75999999999999</v>
       </c>
       <c r="J9" s="2">
-        <v>55.96</v>
+        <v>55.879999999999995</v>
       </c>
     </row>
     <row r="10">
@@ -1601,22 +1601,22 @@
         <v>14</v>
       </c>
       <c r="E13" s="2">
-        <v>14.93</v>
+        <v>14.940000000000001</v>
       </c>
       <c r="F13" s="2">
-        <v>15.92</v>
+        <v>15.94</v>
       </c>
       <c r="G13" s="2">
-        <v>16.990000000000002</v>
+        <v>17</v>
       </c>
       <c r="H13" s="2">
         <v>18.15</v>
       </c>
       <c r="I13" s="2">
-        <v>19.79</v>
+        <v>19.759999999999998</v>
       </c>
       <c r="J13" s="2">
-        <v>21.58</v>
+        <v>21.509999999999998</v>
       </c>
     </row>
     <row r="14">
@@ -1635,22 +1635,22 @@
         <v>13.3</v>
       </c>
       <c r="E14" s="2">
-        <v>14.190000000000001</v>
+        <v>14.2</v>
       </c>
       <c r="F14" s="2">
-        <v>15.120000000000001</v>
+        <v>15.14</v>
       </c>
       <c r="G14" s="2">
-        <v>16.14</v>
+        <v>16.15</v>
       </c>
       <c r="H14" s="2">
         <v>17.59</v>
       </c>
       <c r="I14" s="2">
-        <v>19.18</v>
+        <v>19.15</v>
       </c>
       <c r="J14" s="2">
-        <v>20.93</v>
+        <v>20.85</v>
       </c>
     </row>
     <row r="15">
@@ -1771,22 +1771,22 @@
         <v>11.600000000000001</v>
       </c>
       <c r="E18" s="4">
-        <v>12.080000000000005</v>
+        <v>12.060000000000016</v>
       </c>
       <c r="F18" s="4">
-        <v>12.530000000000012</v>
+        <v>12.509999999999987</v>
       </c>
       <c r="G18" s="4">
-        <v>12.969999999999999</v>
+        <v>12.96</v>
       </c>
       <c r="H18" s="4">
-        <v>18.929999999999986</v>
+        <v>18.909999999999975</v>
       </c>
       <c r="I18" s="4">
-        <v>25.089999999999982</v>
+        <v>25.110000000000007</v>
       </c>
       <c r="J18" s="4">
-        <v>32.96000000000002</v>
+        <v>33.000000000000014</v>
       </c>
     </row>
     <row r="19">
@@ -1805,22 +1805,22 @@
         <v>7.733333333333333</v>
       </c>
       <c r="E19" s="2">
-        <v>7.679104952005597</v>
+        <v>7.666878575969495</v>
       </c>
       <c r="F19" s="2">
-        <v>7.594859983028251</v>
+        <v>7.583196944899065</v>
       </c>
       <c r="G19" s="2">
-        <v>7.495809975148818</v>
+        <v>7.490030630526499</v>
       </c>
       <c r="H19" s="2">
-        <v>9.48967315019049</v>
+        <v>9.481072950614177</v>
       </c>
       <c r="I19" s="2">
-        <v>10.90822138167905</v>
+        <v>10.919765166340511</v>
       </c>
       <c r="J19" s="2">
-        <v>12.370979244079127</v>
+        <v>12.390643187023622</v>
       </c>
     </row>
     <row r="20">
@@ -1839,22 +1839,22 @@
         <v>11.3</v>
       </c>
       <c r="E20" s="4">
-        <v>11.719999999999999</v>
+        <v>11.7</v>
       </c>
       <c r="F20" s="4">
-        <v>12.149999999999999</v>
+        <v>12.129999999999999</v>
       </c>
       <c r="G20" s="4">
-        <v>12.57</v>
+        <v>12.56</v>
       </c>
       <c r="H20" s="4">
-        <v>17.31</v>
+        <v>17.3</v>
       </c>
       <c r="I20" s="4">
-        <v>23.35</v>
+        <v>23.380000000000003</v>
       </c>
       <c r="J20" s="4">
-        <v>31.08</v>
+        <v>31.14</v>
       </c>
     </row>
     <row r="21">
@@ -1873,22 +1873,22 @@
         <v>11.3</v>
       </c>
       <c r="E21" s="2">
-        <v>11.719999999999999</v>
+        <v>11.7</v>
       </c>
       <c r="F21" s="2">
-        <v>12.149999999999999</v>
+        <v>12.129999999999999</v>
       </c>
       <c r="G21" s="2">
-        <v>12.57</v>
+        <v>12.56</v>
       </c>
       <c r="H21" s="2">
-        <v>17.31</v>
+        <v>17.3</v>
       </c>
       <c r="I21" s="2">
-        <v>23.35</v>
+        <v>23.380000000000003</v>
       </c>
       <c r="J21" s="2">
-        <v>31.08</v>
+        <v>31.14</v>
       </c>
     </row>
     <row r="22">
@@ -1907,22 +1907,22 @@
         <v>7.91</v>
       </c>
       <c r="E22" s="2">
-        <v>8.2</v>
+        <v>8.18</v>
       </c>
       <c r="F22" s="2">
-        <v>8.51</v>
+        <v>8.49</v>
       </c>
       <c r="G22" s="2">
-        <v>8.8</v>
+        <v>8.79</v>
       </c>
       <c r="H22" s="2">
-        <v>12.120000000000001</v>
+        <v>12.11</v>
       </c>
       <c r="I22" s="2">
-        <v>16.35</v>
+        <v>16.37</v>
       </c>
       <c r="J22" s="2">
-        <v>21.75</v>
+        <v>21.79</v>
       </c>
     </row>
     <row r="23">
@@ -1941,22 +1941,22 @@
         <v>14</v>
       </c>
       <c r="E23" s="2">
-        <v>14.93</v>
+        <v>14.940000000000001</v>
       </c>
       <c r="F23" s="2">
-        <v>15.92</v>
+        <v>15.94</v>
       </c>
       <c r="G23" s="2">
-        <v>16.990000000000002</v>
+        <v>17</v>
       </c>
       <c r="H23" s="2">
         <v>18.15</v>
       </c>
       <c r="I23" s="2">
-        <v>19.79</v>
+        <v>19.759999999999998</v>
       </c>
       <c r="J23" s="2">
-        <v>21.58</v>
+        <v>21.509999999999998</v>
       </c>
     </row>
     <row r="24">
@@ -2043,22 +2043,22 @@
         <v>30.1</v>
       </c>
       <c r="E26" s="4">
-        <v>31.550000000000004</v>
+        <v>31.540000000000017</v>
       </c>
       <c r="F26" s="4">
-        <v>33.040000000000006</v>
+        <v>33.03999999999999</v>
       </c>
       <c r="G26" s="4">
         <v>34.6</v>
       </c>
       <c r="H26" s="4">
-        <v>41.789999999999985</v>
+        <v>41.769999999999975</v>
       </c>
       <c r="I26" s="4">
-        <v>49.63999999999998</v>
+        <v>49.63</v>
       </c>
       <c r="J26" s="4">
-        <v>59.36000000000002</v>
+        <v>59.33000000000001</v>
       </c>
     </row>
     <row r="27">
@@ -2079,22 +2079,22 @@
         <v>4.768534632788035</v>
       </c>
       <c r="E27" s="2">
-        <v>4.8172757475083205</v>
+        <v>4.7840531561462285</v>
       </c>
       <c r="F27" s="2">
-        <v>4.722662440570535</v>
+        <v>4.755865567533202</v>
       </c>
       <c r="G27" s="2">
-        <v>4.721549636803868</v>
+        <v>4.721549636803912</v>
       </c>
       <c r="H27" s="2">
-        <v>20.780346820809203</v>
+        <v>20.722543352601086</v>
       </c>
       <c r="I27" s="2">
-        <v>18.78439818138309</v>
+        <v>18.817333014125047</v>
       </c>
       <c r="J27" s="2">
-        <v>19.580983078162873</v>
+        <v>19.544630263953277</v>
       </c>
     </row>
     <row r="28">
@@ -2113,22 +2113,22 @@
         <v>20.06666666666667</v>
       </c>
       <c r="E28" s="2">
-        <v>20.055940499650372</v>
+        <v>20.050858232676426</v>
       </c>
       <c r="F28" s="2">
-        <v>20.026669899381744</v>
+        <v>20.027883857671085</v>
       </c>
       <c r="G28" s="2">
         <v>19.99653239322661</v>
       </c>
       <c r="H28" s="2">
-        <v>20.949468618407856</v>
+        <v>20.94259212835296</v>
       </c>
       <c r="I28" s="2">
-        <v>21.58167036215816</v>
+        <v>21.582952815829533</v>
       </c>
       <c r="J28" s="2">
-        <v>22.279773298802695</v>
+        <v>22.276874554124586</v>
       </c>
     </row>
     <row r="29">
@@ -2156,10 +2156,10 @@
         <v>263</v>
       </c>
       <c r="H29" s="2">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="I29" s="2">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="J29" s="2">
         <v>293</v>
@@ -2215,22 +2215,22 @@
         <v>0.06086956521739131</v>
       </c>
       <c r="E31" s="2">
-        <v>0.06220833333333333</v>
+        <v>0.06225000000000001</v>
       </c>
       <c r="F31" s="2">
-        <v>0.06317460317460317</v>
+        <v>0.06325396825396826</v>
       </c>
       <c r="G31" s="2">
-        <v>0.06460076045627378</v>
+        <v>0.06463878326996197</v>
       </c>
       <c r="H31" s="2">
-        <v>0.06672794117647059</v>
+        <v>0.06648351648351648</v>
       </c>
       <c r="I31" s="2">
-        <v>0.070177304964539</v>
+        <v>0.0698233215547703</v>
       </c>
       <c r="J31" s="2">
-        <v>0.0736518771331058</v>
+        <v>0.07341296928327644</v>
       </c>
     </row>
     <row r="32">
@@ -2251,22 +2251,22 @@
         <v>1.9901321235802572</v>
       </c>
       <c r="E32" s="2">
-        <v>2.199404761904744</v>
+        <v>2.267857142857155</v>
       </c>
       <c r="F32" s="2">
-        <v>1.5532803878416823</v>
+        <v>1.6128004079811298</v>
       </c>
       <c r="G32" s="2">
-        <v>2.2574851443529553</v>
+        <v>2.189293500818179</v>
       </c>
       <c r="H32" s="2">
-        <v>3.2928106498632204</v>
+        <v>2.8539107950872777</v>
       </c>
       <c r="I32" s="2">
-        <v>5.169294492311893</v>
+        <v>5.02350845428261</v>
       </c>
       <c r="J32" s="2">
-        <v>4.951133661120943</v>
+        <v>5.141044064611511</v>
       </c>
     </row>
     <row r="33">
@@ -2355,22 +2355,22 @@
         <v>0.12808510638297874</v>
       </c>
       <c r="E35" s="2">
-        <v>0.12877551020408165</v>
+        <v>0.1287346938775511</v>
       </c>
       <c r="F35" s="2">
-        <v>0.1285603112840467</v>
+        <v>0.12856031128404666</v>
       </c>
       <c r="G35" s="2">
         <v>0.1291044776119403</v>
       </c>
       <c r="H35" s="2">
-        <v>0.15086642599277972</v>
+        <v>0.15025179856115098</v>
       </c>
       <c r="I35" s="2">
-        <v>0.1729616724738675</v>
+        <v>0.1723263888888889</v>
       </c>
       <c r="J35" s="2">
-        <v>0.1991946308724833</v>
+        <v>0.19909395973154367</v>
       </c>
     </row>
     <row r="36">
@@ -2389,22 +2389,22 @@
         <v>15.100000000000001</v>
       </c>
       <c r="E36" s="4">
-        <v>15.580000000000005</v>
+        <v>15.560000000000016</v>
       </c>
       <c r="F36" s="4">
-        <v>16.030000000000012</v>
+        <v>16.009999999999987</v>
       </c>
       <c r="G36" s="4">
-        <v>16.47</v>
+        <v>16.46</v>
       </c>
       <c r="H36" s="4">
-        <v>22.429999999999986</v>
+        <v>22.409999999999975</v>
       </c>
       <c r="I36" s="4">
-        <v>28.589999999999982</v>
+        <v>28.610000000000007</v>
       </c>
       <c r="J36" s="4">
-        <v>36.46000000000002</v>
+        <v>36.500000000000014</v>
       </c>
     </row>
     <row r="37">
@@ -2423,22 +2423,22 @@
         <v>10.066666666666668</v>
       </c>
       <c r="E37" s="2">
-        <v>9.904011188099933</v>
+        <v>9.891926255562629</v>
       </c>
       <c r="F37" s="2">
-        <v>9.716329252030555</v>
+        <v>9.704794811177782</v>
       </c>
       <c r="G37" s="2">
-        <v>9.518580592960756</v>
+        <v>9.51280124833844</v>
       </c>
       <c r="H37" s="2">
-        <v>11.244235011028668</v>
+        <v>11.23589872148407</v>
       </c>
       <c r="I37" s="2">
-        <v>12.429894352419453</v>
+        <v>12.441835181561213</v>
       </c>
       <c r="J37" s="2">
-        <v>13.684645122546268</v>
+        <v>13.704802312920068</v>
       </c>
     </row>
     <row r="38">
@@ -2459,22 +2459,22 @@
         <v>3.1420765027322606</v>
       </c>
       <c r="E38" s="2">
-        <v>3.1788079470199015</v>
+        <v>3.0463576158941352</v>
       </c>
       <c r="F38" s="2">
-        <v>2.888318356867825</v>
+        <v>2.8920308483288526</v>
       </c>
       <c r="G38" s="2">
-        <v>2.744853399875158</v>
+        <v>2.810743285446682</v>
       </c>
       <c r="H38" s="2">
-        <v>36.18700667880987</v>
+        <v>36.14823815309827</v>
       </c>
       <c r="I38" s="2">
-        <v>27.46321890325458</v>
+        <v>27.666220437304933</v>
       </c>
       <c r="J38" s="2">
-        <v>27.52710738020303</v>
+        <v>27.57777001048587</v>
       </c>
     </row>
   </sheetData>
@@ -2627,22 +2627,22 @@
         <v>80</v>
       </c>
       <c r="E3" s="4">
-        <v>84.33</v>
+        <v>84.32</v>
       </c>
       <c r="F3" s="4">
-        <v>88.89</v>
+        <v>88.88</v>
       </c>
       <c r="G3" s="4">
-        <v>93.7</v>
+        <v>93.69</v>
       </c>
       <c r="H3" s="4">
-        <v>114.35</v>
+        <v>114.32</v>
       </c>
       <c r="I3" s="4">
-        <v>139.55</v>
+        <v>139.5</v>
       </c>
       <c r="J3" s="4">
-        <v>170.3</v>
+        <v>170.22</v>
       </c>
     </row>
     <row r="4">
@@ -2663,22 +2663,22 @@
         <v>5.263157894736836</v>
       </c>
       <c r="E4" s="2">
-        <v>5.412499999999998</v>
+        <v>5.399999999999983</v>
       </c>
       <c r="F4" s="2">
-        <v>5.407328352899321</v>
+        <v>5.407969639468702</v>
       </c>
       <c r="G4" s="2">
-        <v>5.41118236022049</v>
+        <v>5.41179117911792</v>
       </c>
       <c r="H4" s="2">
-        <v>22.03842049092848</v>
+        <v>22.019425765823453</v>
       </c>
       <c r="I4" s="2">
-        <v>22.03760384783562</v>
+        <v>22.025892232330314</v>
       </c>
       <c r="J4" s="2">
-        <v>22.035112862773197</v>
+        <v>22.021505376344088</v>
       </c>
     </row>
     <row r="5">
@@ -2697,22 +2697,22 @@
         <v>53.333333333333336</v>
       </c>
       <c r="E5" s="2">
-        <v>53.60752653995296</v>
+        <v>53.60457724094086</v>
       </c>
       <c r="F5" s="2">
-        <v>53.87925809188992</v>
+        <v>53.87646238710069</v>
       </c>
       <c r="G5" s="2">
-        <v>54.1524591111368</v>
+        <v>54.146679766514474</v>
       </c>
       <c r="H5" s="2">
-        <v>57.32404251052737</v>
+        <v>57.31762346452744</v>
       </c>
       <c r="I5" s="2">
-        <v>60.67127516194949</v>
+        <v>60.66536203522506</v>
       </c>
       <c r="J5" s="2">
-        <v>63.919228315129686</v>
+        <v>63.91319040288364</v>
       </c>
     </row>
     <row r="6">
@@ -2731,22 +2731,22 @@
         <v>25.6</v>
       </c>
       <c r="E6" s="4">
-        <v>26.989999999999995</v>
+        <v>26.97999999999999</v>
       </c>
       <c r="F6" s="4">
         <v>28.439999999999998</v>
       </c>
       <c r="G6" s="4">
-        <v>29.980000000000004</v>
+        <v>29.979999999999997</v>
       </c>
       <c r="H6" s="4">
-        <v>37.16</v>
+        <v>37.14999999999999</v>
       </c>
       <c r="I6" s="4">
-        <v>46.040000000000006</v>
+        <v>46.03</v>
       </c>
       <c r="J6" s="4">
-        <v>57.040000000000006</v>
+        <v>57.019999999999996</v>
       </c>
     </row>
     <row r="7">
@@ -2765,22 +2765,22 @@
         <v>32</v>
       </c>
       <c r="E7" s="2">
-        <v>32.005217597533495</v>
+        <v>31.997153700189745</v>
       </c>
       <c r="F7" s="2">
-        <v>31.994600067499153</v>
+        <v>31.998199819982</v>
       </c>
       <c r="G7" s="2">
-        <v>31.995731056563503</v>
+        <v>31.999146120183582</v>
       </c>
       <c r="H7" s="2">
-        <v>32.496720594665504</v>
+        <v>32.49650104968509</v>
       </c>
       <c r="I7" s="2">
-        <v>32.99175922608384</v>
+        <v>32.996415770609325</v>
       </c>
       <c r="J7" s="2">
-        <v>33.493834409864945</v>
+        <v>33.49782634238045</v>
       </c>
     </row>
     <row r="8">
@@ -2799,22 +2799,22 @@
         <v>7.300000000000004</v>
       </c>
       <c r="E8" s="4">
-        <v>7.669999999999991</v>
+        <v>7.649999999999988</v>
       </c>
       <c r="F8" s="4">
-        <v>8.039999999999996</v>
+        <v>8.019999999999996</v>
       </c>
       <c r="G8" s="4">
-        <v>8.410000000000004</v>
+        <v>8.389999999999997</v>
       </c>
       <c r="H8" s="4">
-        <v>12.969999999999997</v>
+        <v>12.959999999999992</v>
       </c>
       <c r="I8" s="4">
-        <v>18.470000000000002</v>
+        <v>18.5</v>
       </c>
       <c r="J8" s="4">
-        <v>25.61000000000001</v>
+        <v>25.659999999999997</v>
       </c>
     </row>
     <row r="9">
@@ -2833,22 +2833,22 @@
         <v>9.125000000000005</v>
       </c>
       <c r="E9" s="2">
-        <v>9.095221154986351</v>
+        <v>9.072580645161278</v>
       </c>
       <c r="F9" s="2">
-        <v>9.044886938913258</v>
+        <v>9.02340234023402</v>
       </c>
       <c r="G9" s="2">
-        <v>8.975453575240131</v>
+        <v>8.955064574661113</v>
       </c>
       <c r="H9" s="2">
-        <v>11.34236991692173</v>
+        <v>11.336599020293905</v>
       </c>
       <c r="I9" s="2">
-        <v>13.235399498387675</v>
+        <v>13.261648745519713</v>
       </c>
       <c r="J9" s="2">
-        <v>15.038167938931302</v>
+        <v>15.074609329103511</v>
       </c>
     </row>
     <row r="10">
@@ -2867,22 +2867,22 @@
         <v>6</v>
       </c>
       <c r="E10" s="2">
-        <v>6.44</v>
+        <v>6.45</v>
       </c>
       <c r="F10" s="2">
-        <v>6.91</v>
+        <v>6.93</v>
       </c>
       <c r="G10" s="2">
-        <v>7.42</v>
+        <v>7.44</v>
       </c>
       <c r="H10" s="2">
         <v>7.9</v>
       </c>
       <c r="I10" s="2">
-        <v>8.8</v>
+        <v>8.77</v>
       </c>
       <c r="J10" s="2">
-        <v>9.8</v>
+        <v>9.74</v>
       </c>
     </row>
     <row r="11">
@@ -3037,22 +3037,22 @@
         <v>15.700000000000005</v>
       </c>
       <c r="E15" s="4">
-        <v>16.529999999999994</v>
+        <v>16.51999999999999</v>
       </c>
       <c r="F15" s="4">
         <v>17.389999999999993</v>
       </c>
       <c r="G15" s="4">
-        <v>18.300000000000004</v>
+        <v>18.299999999999997</v>
       </c>
       <c r="H15" s="4">
-        <v>23.369999999999997</v>
+        <v>23.359999999999992</v>
       </c>
       <c r="I15" s="4">
-        <v>29.790000000000003</v>
+        <v>29.79</v>
       </c>
       <c r="J15" s="4">
-        <v>37.96000000000001</v>
+        <v>37.949999999999996</v>
       </c>
     </row>
     <row r="16">
@@ -3073,22 +3073,22 @@
         <v>5.2984574111334615</v>
       </c>
       <c r="E16" s="2">
-        <v>5.286624203821577</v>
+        <v>5.22292993630562</v>
       </c>
       <c r="F16" s="2">
-        <v>5.202661826981236</v>
+        <v>5.266343825665887</v>
       </c>
       <c r="G16" s="2">
-        <v>5.23289246693508</v>
+        <v>5.232892466935035</v>
       </c>
       <c r="H16" s="2">
-        <v>27.70491803278685</v>
+        <v>27.650273224043698</v>
       </c>
       <c r="I16" s="2">
-        <v>27.47111681643135</v>
+        <v>27.525684931506888</v>
       </c>
       <c r="J16" s="2">
-        <v>27.42531050688153</v>
+        <v>27.391742195367552</v>
       </c>
     </row>
     <row r="17">
@@ -3113,13 +3113,13 @@
         <v>111</v>
       </c>
       <c r="G17" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H17" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I17" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J17" s="2">
         <v>125</v>
@@ -3175,22 +3175,22 @@
         <v>0.06</v>
       </c>
       <c r="E19" s="2">
-        <v>0.06133333333333334</v>
+        <v>0.06142857142857143</v>
       </c>
       <c r="F19" s="2">
-        <v>0.062252252252252255</v>
+        <v>0.06243243243243243</v>
       </c>
       <c r="G19" s="2">
-        <v>0.0639655172413793</v>
+        <v>0.06358974358974359</v>
       </c>
       <c r="H19" s="2">
-        <v>0.06638655462184874</v>
+        <v>0.06583333333333334</v>
       </c>
       <c r="I19" s="2">
-        <v>0.07213114754098361</v>
+        <v>0.07130081300813008</v>
       </c>
       <c r="J19" s="2">
-        <v>0.07840000000000001</v>
+        <v>0.07792</v>
       </c>
     </row>
     <row r="20">
@@ -3211,22 +3211,22 @@
         <v>1.9677996422182487</v>
       </c>
       <c r="E20" s="2">
-        <v>2.2222222222222365</v>
+        <v>2.3809523809523947</v>
       </c>
       <c r="F20" s="2">
-        <v>1.4982373678025906</v>
+        <v>1.6341923318667462</v>
       </c>
       <c r="G20" s="2">
-        <v>2.7521333399870063</v>
+        <v>1.8537018537018612</v>
       </c>
       <c r="H20" s="2">
-        <v>3.7849101904912974</v>
+        <v>3.5282258064516236</v>
       </c>
       <c r="I20" s="2">
-        <v>8.653247561734801</v>
+        <v>8.305032417412782</v>
       </c>
       <c r="J20" s="2">
-        <v>8.690909090909106</v>
+        <v>9.283466362599778</v>
       </c>
     </row>
     <row r="21">
@@ -3315,22 +3315,22 @@
         <v>0.15392156862745102</v>
       </c>
       <c r="E23" s="2">
-        <v>0.15448598130841115</v>
+        <v>0.1543925233644859</v>
       </c>
       <c r="F23" s="2">
         <v>0.15389380530973445</v>
       </c>
       <c r="G23" s="2">
-        <v>0.1550847457627119</v>
+        <v>0.153781512605042</v>
       </c>
       <c r="H23" s="2">
-        <v>0.19314049586776857</v>
+        <v>0.1914754098360655</v>
       </c>
       <c r="I23" s="2">
-        <v>0.240241935483871</v>
+        <v>0.23832</v>
       </c>
       <c r="J23" s="2">
-        <v>0.2988976377952757</v>
+        <v>0.29881889763779523</v>
       </c>
     </row>
     <row r="24">
@@ -3643,7 +3643,7 @@
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.87 % / 補助 5.41 % / ベース 4.26 %</t>
+          <t xml:space="preserve">全社 4.87 % / 補助 5.4 % / ベース 4.26 %</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
@@ -3653,22 +3653,22 @@
       </c>
       <c r="I4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.88 % / 補助 5.41 % / ベース 4.26 %</t>
+          <t xml:space="preserve">全社 4.89 % / 補助 5.41 % / ベース 4.27 %</t>
         </is>
       </c>
       <c r="J4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.29 % / 補助 22.04 % / ベース 7.31 %</t>
+          <t xml:space="preserve">全社 15.27 % / 補助 22.02 % / ベース 7.3 %</t>
         </is>
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.3 % / 補助 22.04 % / ベース 6.26 %</t>
+          <t xml:space="preserve">全社 15.29 % / 補助 22.03 % / ベース 6.25 %</t>
         </is>
       </c>
       <c r="L4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.83 % / 補助 22.04 % / ベース 6.27 %</t>
+          <t xml:space="preserve">全社 15.82 % / 補助 22.02 % / ベース 6.26 %</t>
         </is>
       </c>
     </row>
@@ -3705,32 +3705,32 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 68 % / 補助 67.99 % / ベース 68 %</t>
+          <t xml:space="preserve">全社 68 % / 補助 68 % / ベース 68 %</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 68 % / 補助 68.01 % / ベース 68 %</t>
+          <t xml:space="preserve">全社 68 % / 補助 68 % / ベース 68 %</t>
         </is>
       </c>
       <c r="I5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 68 % / 補助 68 % / ベース 67.99 %</t>
+          <t xml:space="preserve">全社 68 % / 補助 68 % / ベース 68 %</t>
         </is>
       </c>
       <c r="J5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 67.36 % / 補助 67.5 % / ベース 67.17 %</t>
+          <t xml:space="preserve">全社 67.37 % / 補助 67.5 % / ベース 67.18 %</t>
         </is>
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 67.01 % / 補助 67.01 % / ベース 67 %</t>
+          <t xml:space="preserve">全社 67.01 % / 補助 67 % / ベース 67.01 %</t>
         </is>
       </c>
       <c r="L5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 66.63 % / 補助 66.51 % / ベース 66.84 %</t>
+          <t xml:space="preserve">全社 66.63 % / 補助 66.5 % / ベース 66.85 %</t>
         </is>
       </c>
     </row>
@@ -3767,32 +3767,32 @@
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32 % / 補助 32.01 % / ベース 32 %</t>
+          <t xml:space="preserve">全社 32 % / 補助 32 % / ベース 32 %</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32 % / 補助 31.99 % / ベース 32 %</t>
+          <t xml:space="preserve">全社 32 % / 補助 32 % / ベース 32 %</t>
         </is>
       </c>
       <c r="I6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32 % / 補助 32 % / ベース 32.01 %</t>
+          <t xml:space="preserve">全社 32 % / 補助 32 % / ベース 32 %</t>
         </is>
       </c>
       <c r="J6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32.64 % / 補助 32.5 % / ベース 32.83 %</t>
+          <t xml:space="preserve">全社 32.63 % / 補助 32.5 % / ベース 32.82 %</t>
         </is>
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32.99 % / 補助 32.99 % / ベース 33 %</t>
+          <t xml:space="preserve">全社 32.99 % / 補助 33 % / ベース 32.99 %</t>
         </is>
       </c>
       <c r="L6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 33.37 % / 補助 33.49 % / ベース 33.16 %</t>
+          <t xml:space="preserve">全社 33.37 % / 補助 33.5 % / ベース 33.15 %</t>
         </is>
       </c>
     </row>
@@ -3829,32 +3829,32 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.32 % / 補助 22.91 % / ベース 25.95 %</t>
+          <t xml:space="preserve">全社 24.33 % / 補助 22.92 % / ベース 25.95 %</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.4 % / 補助 22.95 % / ベース 26.1 %</t>
+          <t xml:space="preserve">全社 24.42 % / 補助 22.97 % / ベース 26.1 %</t>
         </is>
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.5 % / 補助 23.02 % / ベース 26.26 %</t>
+          <t xml:space="preserve">全社 24.51 % / 補助 23.04 % / ベース 26.24 %</t>
         </is>
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 23.15 % / 補助 21.15 % / ベース 25.83 %</t>
+          <t xml:space="preserve">全社 23.15 % / 補助 21.16 % / ベース 25.83 %</t>
         </is>
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 22.09 % / 補助 19.76 % / ベース 25.68 %</t>
+          <t xml:space="preserve">全社 22.07 % / 補助 19.73 % / ベース 25.68 %</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 21 % / 補助 18.46 % / ベース 25.52 %</t>
+          <t xml:space="preserve">全社 20.98 % / 補助 18.42 % / ベース 25.51 %</t>
         </is>
       </c>
     </row>
@@ -3891,32 +3891,32 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.68 % / 補助 9.1 % / ベース 6.04 %</t>
+          <t xml:space="preserve">全社 7.67 % / 補助 9.07 % / ベース 6.04 %</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.59 % / 補助 9.04 % / ベース 5.9 %</t>
+          <t xml:space="preserve">全社 7.58 % / 補助 9.02 % / ベース 5.9 %</t>
         </is>
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.5 % / 補助 8.98 % / ベース 5.75 %</t>
+          <t xml:space="preserve">全社 7.49 % / 補助 8.96 % / ベース 5.76 %</t>
         </is>
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.49 % / 補助 11.34 % / ベース 7 %</t>
+          <t xml:space="preserve">全社 9.48 % / 補助 11.34 % / ベース 6.99 %</t>
         </is>
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.91 % / 補助 13.24 % / ベース 7.32 %</t>
+          <t xml:space="preserve">全社 10.92 % / 補助 13.26 % / ベース 7.31 %</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.37 % / 補助 15.04 % / ベース 7.65 %</t>
+          <t xml:space="preserve">全社 12.39 % / 補助 15.07 % / ベース 7.64 %</t>
         </is>
       </c>
     </row>
@@ -3953,32 +3953,32 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.9 % / 補助 11.47 % / ベース 8.1 %</t>
+          <t xml:space="preserve">全社 9.89 % / 補助 11.44 % / ベース 8.1 %</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.72 % / 補助 11.29 % / ベース 7.87 %</t>
+          <t xml:space="preserve">全社 9.7 % / 補助 11.27 % / ベース 7.87 %</t>
         </is>
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.52 % / 補助 11.11 % / ベース 7.64 %</t>
+          <t xml:space="preserve">全社 9.51 % / 補助 11.09 % / ベース 7.65 %</t>
         </is>
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.24 % / 補助 13.09 % / ベース 8.76 %</t>
+          <t xml:space="preserve">全社 11.24 % / 補助 13.09 % / ベース 8.75 %</t>
         </is>
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.43 % / 補助 14.67 % / ベース 8.98 %</t>
+          <t xml:space="preserve">全社 12.44 % / 補助 14.7 % / ベース 8.97 %</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.68 % / 補助 16.21 % / ベース 9.21 %</t>
+          <t xml:space="preserve">全社 13.7 % / 補助 16.25 % / ベース 9.2 %</t>
         </is>
       </c>
     </row>
@@ -4139,17 +4139,17 @@
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.49 % / 補助 7.64 % / ベース 11.63 %</t>
+          <t xml:space="preserve">全社 9.5 % / 補助 7.65 % / ベース 11.63 %</t>
         </is>
       </c>
       <c r="H12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.65 % / 補助 7.77 % / ベース 11.84 %</t>
+          <t xml:space="preserve">全社 9.66 % / 補助 7.8 % / ベース 11.84 %</t>
         </is>
       </c>
       <c r="I12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.82 % / 補助 7.92 % / ベース 12.06 %</t>
+          <t xml:space="preserve">全社 9.82 % / 補助 7.94 % / ベース 12.05 %</t>
         </is>
       </c>
       <c r="J12" s="0" t="inlineStr">
@@ -4159,12 +4159,12 @@
       </c>
       <c r="K12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.6 % / 補助 6.31 % / ベース 12.15 %</t>
+          <t xml:space="preserve">全社 8.59 % / 補助 6.29 % / ベース 12.15 %</t>
         </is>
       </c>
       <c r="L12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.1 % / 補助 5.75 % / ベース 12.25 %</t>
+          <t xml:space="preserve">全社 8.08 % / 補助 5.72 % / ベース 12.25 %</t>
         </is>
       </c>
     </row>
@@ -4206,7 +4206,7 @@
       </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.66 % / 補助 0.49 % / ベース 0.85 %</t>
+          <t xml:space="preserve">全社 0.66 % / 補助 0.5 % / ベース 0.85 %</t>
         </is>
       </c>
       <c r="I13" s="0" t="inlineStr">
@@ -4263,17 +4263,17 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.15 % / 補助 8.13 % / ベース 12.48 %</t>
+          <t xml:space="preserve">全社 10.16 % / 補助 8.15 % / ベース 12.48 %</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.31 % / 補助 8.27 % / ベース 12.7 %</t>
+          <t xml:space="preserve">全社 10.32 % / 補助 8.29 % / ベース 12.7 %</t>
         </is>
       </c>
       <c r="I14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.48 % / 補助 8.42 % / ベース 12.91 %</t>
+          <t xml:space="preserve">全社 10.48 % / 補助 8.44 % / ベース 12.89 %</t>
         </is>
       </c>
       <c r="J14" s="0" t="inlineStr">
@@ -4283,12 +4283,12 @@
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.15 % / 補助 6.68 % / ベース 12.97 %</t>
+          <t xml:space="preserve">全社 9.14 % / 補助 6.66 % / ベース 12.97 %</t>
         </is>
       </c>
       <c r="L14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.6 % / 補助 6.08 % / ベース 13.06 %</t>
+          <t xml:space="preserve">全社 8.57 % / 補助 6.05 % / ベース 13.05 %</t>
         </is>
       </c>
     </row>
@@ -4340,17 +4340,17 @@
       </c>
       <c r="J15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.067 億円/人 / 補助 0.066 億円/人 / ベース 0.067 億円/人</t>
+          <t xml:space="preserve">全社 0.066 億円/人 / 補助 0.066 億円/人 / ベース 0.067 億円/人</t>
         </is>
       </c>
       <c r="K15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.07 億円/人 / 補助 0.072 億円/人 / ベース 0.069 億円/人</t>
+          <t xml:space="preserve">全社 0.07 億円/人 / 補助 0.071 億円/人 / ベース 0.069 億円/人</t>
         </is>
       </c>
       <c r="L15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.074 億円/人 / 補助 0.078 億円/人 / ベース 0.07 億円/人</t>
+          <t xml:space="preserve">全社 0.073 億円/人 / 補助 0.078 億円/人 / ベース 0.07 億円/人</t>
         </is>
       </c>
     </row>
@@ -4449,32 +4449,32 @@
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.2 % / 補助 2.22 % / ベース 2.19 %</t>
+          <t xml:space="preserve">全社 2.27 % / 補助 2.38 % / ベース 2.19 %</t>
         </is>
       </c>
       <c r="H17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.55 % / 補助 1.5 % / ベース 1.61 %</t>
+          <t xml:space="preserve">全社 1.61 % / 補助 1.63 % / ベース 1.61 %</t>
         </is>
       </c>
       <c r="I17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.26 % / 補助 2.75 % / ベース 1.88 %</t>
+          <t xml:space="preserve">全社 2.19 % / 補助 1.85 % / ベース 2.47 %</t>
         </is>
       </c>
       <c r="J17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.29 % / 補助 3.78 % / ベース 2.91 %</t>
+          <t xml:space="preserve">全社 2.85 % / 補助 3.53 % / ベース 2.31 %</t>
         </is>
       </c>
       <c r="K17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5.17 % / 補助 8.65 % / ベース 2.53 %</t>
+          <t xml:space="preserve">全社 5.02 % / 補助 8.31 % / ベース 2.53 %</t>
         </is>
       </c>
       <c r="L17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.95 % / 補助 8.69 % / ベース 2.08 %</t>
+          <t xml:space="preserve">全社 5.14 % / 補助 9.28 % / ベース 2 %</t>
         </is>
       </c>
     </row>
@@ -4511,32 +4511,32 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 50.62 % / 補助 41.5 % / ベース 60.65 %</t>
+          <t xml:space="preserve">全社 50.67 % / 補助 41.59 % / ベース 60.65 %</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 51.48 % / 補助 42.27 % / ベース 61.73 %</t>
+          <t xml:space="preserve">全社 51.54 % / 補助 42.38 % / ベース 61.73 %</t>
         </is>
       </c>
       <c r="I18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 52.4 % / 補助 43.11 % / ベース 62.82 %</t>
+          <t xml:space="preserve">全社 52.43 % / 補助 43.22 % / ベース 62.76 %</t>
         </is>
       </c>
       <c r="J18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 46.33 % / 補助 35.94 % / ベース 59.5 %</t>
+          <t xml:space="preserve">全社 46.35 % / 補助 35.96 % / ベース 59.53 %</t>
         </is>
       </c>
       <c r="K18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 42.41 % / 補助 31.29 % / ベース 59.09 %</t>
+          <t xml:space="preserve">全社 42.35 % / 補助 31.18 % / ベース 59.12 %</t>
         </is>
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 38.58 % / 補助 27.27 % / ベース 58.64 %</t>
+          <t xml:space="preserve">全社 38.48 % / 補助 27.11 % / ベース 58.65 %</t>
         </is>
       </c>
     </row>
@@ -4645,17 +4645,17 @@
       </c>
       <c r="I20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.658 億円/人 / 補助 0.808 億円/人 / ベース 0.54 億円/人</t>
+          <t xml:space="preserve">全社 0.658 億円/人 / 補助 0.801 億円/人 / ベース 0.543 億円/人</t>
         </is>
       </c>
       <c r="J20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.733 億円/人 / 補助 0.961 億円/人 / ベース 0.556 億円/人</t>
+          <t xml:space="preserve">全社 0.731 億円/人 / 補助 0.953 億円/人 / ベース 0.556 億円/人</t>
         </is>
       </c>
       <c r="K20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.816 億円/人 / 補助 1.144 億円/人 / ベース 0.565 億円/人</t>
+          <t xml:space="preserve">全社 0.813 億円/人 / 補助 1.134 億円/人 / ベース 0.565 億円/人</t>
         </is>
       </c>
       <c r="L20" s="0" t="inlineStr">
@@ -4707,22 +4707,22 @@
       </c>
       <c r="I21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.049 億円/人 / 補助 0.073 億円/人 / ベース 0.031 億円/人</t>
+          <t xml:space="preserve">全社 0.049 億円/人 / 補助 0.072 億円/人 / ベース 0.031 億円/人</t>
         </is>
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.07 億円/人 / 補助 0.109 億円/人 / ベース 0.039 億円/人</t>
+          <t xml:space="preserve">全社 0.069 億円/人 / 補助 0.108 億円/人 / ベース 0.039 億円/人</t>
         </is>
       </c>
       <c r="K21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.089 億円/人 / 補助 0.151 億円/人 / ベース 0.041 億円/人</t>
+          <t xml:space="preserve">全社 0.089 億円/人 / 補助 0.15 億円/人 / ベース 0.041 億円/人</t>
         </is>
       </c>
       <c r="L21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.112 億円/人 / 補助 0.205 億円/人 / ベース 0.044 億円/人</t>
+          <t xml:space="preserve">全社 0.113 億円/人 / 補助 0.205 億円/人 / ベース 0.044 億円/人</t>
         </is>
       </c>
     </row>
@@ -4769,17 +4769,17 @@
       </c>
       <c r="I22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.129 億円/人 / 補助 0.155 億円/人 / ベース 0.109 億円/人</t>
+          <t xml:space="preserve">全社 0.129 億円/人 / 補助 0.154 億円/人 / ベース 0.109 億円/人</t>
         </is>
       </c>
       <c r="J22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.151 億円/人 / 補助 0.193 億円/人 / ベース 0.118 億円/人</t>
+          <t xml:space="preserve">全社 0.15 億円/人 / 補助 0.191 億円/人 / ベース 0.118 億円/人</t>
         </is>
       </c>
       <c r="K22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.173 億円/人 / 補助 0.24 億円/人 / ベース 0.122 億円/人</t>
+          <t xml:space="preserve">全社 0.172 億円/人 / 補助 0.238 億円/人 / ベース 0.122 億円/人</t>
         </is>
       </c>
       <c r="L22" s="0" t="inlineStr">
@@ -4831,22 +4831,22 @@
       </c>
       <c r="I23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.37 % / 補助 4.5 % / ベース 4.26 %</t>
+          <t xml:space="preserve">全社 4.37 % / 補助 5.41 % / ベース 3.55 %</t>
         </is>
       </c>
       <c r="J23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.42 % / 補助 2.59 % / ベース 4.08 %</t>
+          <t xml:space="preserve">全社 3.8 % / 補助 2.56 % / ベース 4.79 %</t>
         </is>
       </c>
       <c r="K23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.68 % / 補助 2.52 % / ベース 4.58 %</t>
+          <t xml:space="preserve">全社 3.66 % / 補助 2.5 % / ベース 4.58 %</t>
         </is>
       </c>
       <c r="L23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.9 % / 補助 2.46 % / ベース 5 %</t>
+          <t xml:space="preserve">全社 3.53 % / 補助 1.63 % / ベース 5 %</t>
         </is>
       </c>
     </row>
@@ -4883,7 +4883,7 @@
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.53 pt / 補助 0.41 pt / ベース 0.41 pt</t>
+          <t xml:space="preserve">全社 0.52 pt / 補助 0.4 pt / ベース 0.41 pt</t>
         </is>
       </c>
       <c r="H24" s="0" t="inlineStr">
@@ -4893,22 +4893,22 @@
       </c>
       <c r="I24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.51 pt / 補助 0.91 pt / ベース 0 pt</t>
+          <t xml:space="preserve">全社 0.52 pt / 補助 0.01 pt / ベース 0.73 pt</t>
         </is>
       </c>
       <c r="J24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.86 pt / 補助 19.45 pt / ベース 3.23 pt</t>
+          <t xml:space="preserve">全社 11.47 pt / 補助 19.46 pt / ベース 2.5 pt</t>
         </is>
       </c>
       <c r="K24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.63 pt / 補助 19.52 pt / ベース 1.69 pt</t>
+          <t xml:space="preserve">全社 11.63 pt / 補助 19.53 pt / ベース 1.67 pt</t>
         </is>
       </c>
       <c r="L24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.93 pt / 補助 19.58 pt / ベース 1.27 pt</t>
+          <t xml:space="preserve">全社 12.29 pt / 補助 20.4 pt / ベース 1.26 pt</t>
         </is>
       </c>
     </row>
@@ -5007,7 +5007,7 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.22 % / 補助 2.37 % / ベース 2.06 %</t>
+          <t xml:space="preserve">全社 2.23 % / 補助 2.37 % / ベース 2.06 %</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
@@ -5193,32 +5193,32 @@
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.45 倍 / 補助 4.83 倍 / ベース 3.94 倍</t>
+          <t xml:space="preserve">全社 4.45 倍 / 補助 4.82 倍 / ベース 3.94 倍</t>
         </is>
       </c>
       <c r="H29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.58 倍 / 補助 5.02 倍 / ベース 3.99 倍</t>
+          <t xml:space="preserve">全社 4.57 倍 / 補助 5.01 倍 / ベース 3.99 倍</t>
         </is>
       </c>
       <c r="I29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.71 倍 / 補助 5.21 倍 / ベース 4.04 倍</t>
+          <t xml:space="preserve">全社 4.7 倍 / 補助 5.19 倍 / ベース 4.05 倍</t>
         </is>
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.41 倍 / 補助 7.48 倍 / ベース 4.97 倍</t>
+          <t xml:space="preserve">全社 6.4 倍 / 補助 7.48 倍 / ベース 4.97 倍</t>
         </is>
       </c>
       <c r="K29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.17 倍 / 補助 10.24 倍 / ベース 5.41 倍</t>
+          <t xml:space="preserve">全社 8.17 倍 / 補助 10.25 倍 / ベース 5.41 倍</t>
         </is>
       </c>
       <c r="L29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.42 倍 / 補助 13.81 倍 / ベース 5.9 倍</t>
+          <t xml:space="preserve">全社 10.43 倍 / 補助 13.83 倍 / ベース 5.89 倍</t>
         </is>
       </c>
     </row>
@@ -5379,7 +5379,7 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 53.61 %</t>
+          <t xml:space="preserve">構成比 53.6 %</t>
         </is>
       </c>
       <c r="H32" s="0" t="inlineStr">
@@ -5404,7 +5404,7 @@
       </c>
       <c r="L32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 63.92 %</t>
+          <t xml:space="preserve">構成比 63.91 %</t>
         </is>
       </c>
     </row>
@@ -5441,32 +5441,32 @@
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">補助 5.4 % / ベース 4.26 %</t>
+        </is>
+      </c>
+      <c r="H33" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">補助 5.41 % / ベース 4.26 %</t>
         </is>
       </c>
-      <c r="H33" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">補助 5.41 % / ベース 4.26 %</t>
-        </is>
-      </c>
       <c r="I33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 5.41 % / ベース 4.26 %</t>
+          <t xml:space="preserve">補助 5.41 % / ベース 4.27 %</t>
         </is>
       </c>
       <c r="J33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 22.04 % / ベース 7.31 %</t>
+          <t xml:space="preserve">補助 22.02 % / ベース 7.3 %</t>
         </is>
       </c>
       <c r="K33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 22.04 % / ベース 6.26 %</t>
+          <t xml:space="preserve">補助 22.03 % / ベース 6.25 %</t>
         </is>
       </c>
       <c r="L33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 22.04 % / ベース 6.27 %</t>
+          <t xml:space="preserve">補助 22.02 % / ベース 6.26 %</t>
         </is>
       </c>
     </row>
@@ -5503,32 +5503,32 @@
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">差 -0 pt</t>
+        </is>
+      </c>
+      <c r="H34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">差 0 pt</t>
+        </is>
+      </c>
+      <c r="I34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">差 0 pt</t>
+        </is>
+      </c>
+      <c r="J34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">差 0.32 pt</t>
+        </is>
+      </c>
+      <c r="K34" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">差 -0.01 pt</t>
         </is>
       </c>
-      <c r="H34" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">差 0.01 pt</t>
-        </is>
-      </c>
-      <c r="I34" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">差 0.01 pt</t>
-        </is>
-      </c>
-      <c r="J34" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">差 0.34 pt</t>
-        </is>
-      </c>
-      <c r="K34" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">差 0.01 pt</t>
-        </is>
-      </c>
       <c r="L34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -0.33 pt</t>
+          <t xml:space="preserve">差 -0.35 pt</t>
         </is>
       </c>
     </row>
@@ -5565,32 +5565,32 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 3.05 pt</t>
+          <t xml:space="preserve">差 3.03 pt</t>
         </is>
       </c>
       <c r="H35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 3.14 pt</t>
+          <t xml:space="preserve">差 3.12 pt</t>
         </is>
       </c>
       <c r="I35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 3.23 pt</t>
+          <t xml:space="preserve">差 3.2 pt</t>
         </is>
       </c>
       <c r="J35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 4.34 pt</t>
+          <t xml:space="preserve">差 4.35 pt</t>
         </is>
       </c>
       <c r="K35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 5.92 pt</t>
+          <t xml:space="preserve">差 5.95 pt</t>
         </is>
       </c>
       <c r="L35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 7.39 pt</t>
+          <t xml:space="preserve">差 7.44 pt</t>
         </is>
       </c>
     </row>
@@ -5637,17 +5637,17 @@
       </c>
       <c r="I36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.808 億円/人 / ベース 0.54 億円/人</t>
+          <t xml:space="preserve">補助 0.801 億円/人 / ベース 0.543 億円/人</t>
         </is>
       </c>
       <c r="J36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.961 億円/人 / ベース 0.556 億円/人</t>
+          <t xml:space="preserve">補助 0.953 億円/人 / ベース 0.556 億円/人</t>
         </is>
       </c>
       <c r="K36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 1.144 億円/人 / ベース 0.565 億円/人</t>
+          <t xml:space="preserve">補助 1.134 億円/人 / ベース 0.565 億円/人</t>
         </is>
       </c>
       <c r="L36" s="0" t="inlineStr">
@@ -5709,7 +5709,7 @@
       </c>
       <c r="K37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 0.072 億円/人 / ベース 0.069 億円/人</t>
+          <t xml:space="preserve">補助 0.071 億円/人 / ベース 0.069 億円/人</t>
         </is>
       </c>
       <c r="L37" s="0" t="inlineStr">
@@ -5751,7 +5751,7 @@
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 77.08 %</t>
+          <t xml:space="preserve">寄与率 76.09 %</t>
         </is>
       </c>
       <c r="H38" s="0" t="inlineStr">
@@ -5761,22 +5761,22 @@
       </c>
       <c r="I38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 84.09 %</t>
+          <t xml:space="preserve">寄与率 82.22 %</t>
         </is>
       </c>
       <c r="J38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 76.51 %</t>
+          <t xml:space="preserve">寄与率 76.81 %</t>
         </is>
       </c>
       <c r="K38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 89.29 %</t>
+          <t xml:space="preserve">寄与率 89.35 %</t>
         </is>
       </c>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 90.72 %</t>
+          <t xml:space="preserve">寄与率 90.75 %</t>
         </is>
       </c>
     </row>
@@ -5878,7 +5878,7 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 原価率（売上実績が0の場合の開始水準）</t>
+          <t xml:space="preserve">補助事業 原価率</t>
         </is>
       </c>
       <c r="B4" s="2">
@@ -5889,21 +5889,17 @@
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D4" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E4" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="D4" s="2">
+        <v>66</v>
+      </c>
+      <c r="E4" s="2">
+        <v>70</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 原価率（売上実績が0の場合の開始水準）</t>
+          <t xml:space="preserve">ベース事業 原価率</t>
         </is>
       </c>
       <c r="B5" s="2">
@@ -5914,15 +5910,11 @@
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D5" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E5" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="D5" s="2">
+        <v>66</v>
+      </c>
+      <c r="E5" s="2">
+        <v>70</v>
       </c>
     </row>
     <row r="6">
@@ -8932,11 +8924,11 @@
         </is>
       </c>
       <c r="B144" s="2">
-        <v>0</v>
+        <v>0.66</v>
       </c>
       <c r="C144" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
@@ -8947,7 +8939,7 @@
         </is>
       </c>
       <c r="B145" s="2">
-        <v>0.99</v>
+        <v>0.7</v>
       </c>
       <c r="C145" s="0" t="inlineStr">
         <is>
@@ -9502,11 +9494,11 @@
         </is>
       </c>
       <c r="B182" s="2">
-        <v>0</v>
+        <v>0.66</v>
       </c>
       <c r="C182" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
@@ -9517,7 +9509,7 @@
         </is>
       </c>
       <c r="B183" s="2">
-        <v>0.99</v>
+        <v>0.7</v>
       </c>
       <c r="C183" s="0" t="inlineStr">
         <is>
@@ -11137,7 +11129,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4LCJvcmRpbmFyeUluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsInByZVRheEluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsIm5ldEluY29tZSI6Ny41MX19LHsieWVhciI6MjAyNCwicm9sZSI6InByZXZpb3VzIiwicHJvamVjdCI6eyJzYWxlcyI6NzYsImNvZ3MiOjUxLjY4LCJlbXBsb3llZVBheSI6NS41OSwib2ZmaWNlclBheSI6MC4zOCwiZGVwcmVjaWF0aW9uIjoxLjksIm90aGVyU2dhIjo5LjUsImhlYWRjb3VudCI6OTUsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjUuMzEsImVtcGxveWVlQm9udXMiOjAuMjgsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzQsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40Nywic2dhRGVwcmVjaWF0aW9uIjoxLjQzLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM4fSwib3RoZXIiOnsic2FsZXMiOjY3LjIsImNvZ3MiOjQ1LjcsImVtcGxveWVlUGF5Ijo3LjU0LCJvZmZpY2VyUGF5IjowLjU4LCJkZXByZWNpYXRpb24iOjEuNDQsIm90aGVyU2dhIjo3LjY4LCJoZWFkY291bnQiOjEyNSwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ny4xNiwiZW1wbG95ZWVCb251cyI6MC4zOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41Miwib2ZmaWNlckJvbnVzIjowLjA2LCJjb2dzRGVwcmVjaWF0aW9uIjowLjI5LCJzZ2FEZXByZWNpYXRpb24iOjEuMTUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMjksIm9yZGluYXJ5SW5jb21lIjozLjk2OTk5OTk5OTk5OTk5NywicHJlVGF4SW5jb21lIjozLjk2OTk5OTk5OTk5OTk5NywibmV0SW5jb21lIjo3LjcxfX0seyJ5ZWFyIjoyMDI1LCJyb2xlIjoibGF0ZXN0IiwicHJvamVjdCI6eyJzYWxlcyI6ODAsImNvZ3MiOjU0LjQsImVtcGxveWVlUGF5Ijo2LCJlbXBsb3llZVNhbGFyeSI6NS43LCJlbXBsb3llZUJvbnVzIjowLjMsIm9mZmljZXJQYXkiOjAuNCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNiwib2ZmaWNlckJvbnVzIjowLjA0LCJkZXByZWNpYXRpb24iOjIsImNvZ3NEZXByZWNpYXRpb24iOjAuNSwic2dhRGVwcmVjaWF0aW9uIjoxLjUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuNCwib3RoZXJTZ2EiOjEwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwLCJjb2dzIjo0Ny42LCJlbXBsb3llZVBheSI6OCwiZW1wbG95ZWVTYWxhcnkiOjcuNiwiZW1wbG95ZWVCb251cyI6MC40LCJvZmZpY2VyUGF5IjowLjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTQsIm9mZmljZXJCb251cyI6MC4wNiwiZGVwcmVjaWF0aW9uIjoxLjUsImNvZ3NEZXByZWNpYXRpb24iOjAuMywic2dhRGVwcmVjaWF0aW9uIjoxLjIsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMywib3RoZXJTZ2EiOjgsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjozLjk5OTk5OTk5OTk5OTk5NjQsInByZVRheEluY29tZSI6My45OTk5OTk5OTk5OTk5OTY0LCJuZXRJbmNvbWUiOjcuOTF9fV0sImJhbGFuY2VTaGVldHMiOlt7InllYXIiOjIwMjMsImFzc2V0cyI6MTMyLCJjdXJyZW50QXNzZXRzIjo2NywiY2FzaCI6MjQsImZpeGVkQXNzZXRzIjo2NSwidGFuZ2libGVBc3NldHMiOjUzLCJidWlsZGluZ3MiOjE5LCJtYWNoaW5lcnkiOjI0LCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6Nywic29mdHdhcmUiOjUsImxpYWJpbGl0aWVzIjo3NSwiY3VycmVudExpYWJpbGl0aWVzIjozOSwic2hvcnRUZXJtRGVidCI6MTIsImZpeGVkTGlhYmlsaXRpZXMiOjM2LCJsb25nVGVybURlYnQiOjI5LCJuZXRBc3NldHMiOjU3LCJzaGFyZWhvbGRlckVxdWl0eSI6NTQsImNhcGl0YWwiOjEwLCJjYXBleCI6NX0seyJ5ZWFyIjoyMDI0LCJhc3NldHMiOjE0MywiY3VycmVudEFzc2V0cyI6NzIsImNhc2giOjI1LCJmaXhlZEFzc2V0cyI6NzEsInRhbmdpYmxlQXNzZXRzIjo1OCwiYnVpbGRpbmdzIjoyMCwibWFjaGluZXJ5IjoyOCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjgsInNvZnR3YXJlIjo2LCJsaWFiaWxpdGllcyI6NzksImN1cnJlbnRMaWFiaWxpdGllcyI6NDEsInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozOCwibG9uZ1Rlcm1EZWJ0IjozMSwibmV0QXNzZXRzIjo2NCwic2hhcmVob2xkZXJFcXVpdHkiOjYxLCJjYXBpdGFsIjoxMCwiY2FwZXgiOjh9LHsieWVhciI6MjAyNSwiYXNzZXRzIjoxNTYsImN1cnJlbnRBc3NldHMiOjc4LCJjYXNoIjoyNywiZml4ZWRBc3NldHMiOjc4LCJ0YW5naWJsZUFzc2V0cyI6NjQsImJ1aWxkaW5ncyI6MjIsIm1hY2hpbmVyeSI6MzIsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo5LCJzb2Z0d2FyZSI6NywibGlhYmlsaXRpZXMiOjgzLCJjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJzaG9ydFRlcm1EZWJ0IjoxMSwiZml4ZWRMaWFiaWxpdGllcyI6NDAsImxvbmdUZXJtRGVidCI6MzIsIm5ldEFzc2V0cyI6NzMsInNoYXJlaG9sZGVyRXF1aXR5Ijo3MCwiY2FwaXRhbCI6MTAsImNhcGV4IjoxMH1dLCJmdXR1cmVDYXBleCI6W3sieWVhciI6MjAyNiwidmFsdWUiOjB9LHsieWVhciI6MjAyNywidmFsdWUiOjB9LHsieWVhciI6MjAyOCwidmFsdWUiOjB9LHsieWVhciI6MjAyOSwidmFsdWUiOjB9LHsieWVhciI6MjAzMCwidmFsdWUiOjB9LHsieWVhciI6MjAzMSwidmFsdWUiOjB9XSwiZHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTcyNDYzNzY4MTE1ODYsInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsInByb2plY3RTZ2FSYXRlRW5kIjowLjAxNSwib3RoZXJTZ2FSYXRlRW5kIjowLjAwNSwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzODAxMTY5NTkwNjQzMjUsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOlswLDAuOTldLCJvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6WzAsMC45OV0sInByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlIjpbMCwxXSwib3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlIjpbMCwxXSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6WzAsMV0sIm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjpbMCwxXSwicHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZSI6WzAsMV0sIm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlIjpbMCwxXSwicHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjpbMCwwLjNdLCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjpbMCwwLjNdLCJwcm9qZWN0Tm9uT3BlcmF0aW5nUmF0ZSI6Wy0wLjUsMC41XSwib3RoZXJOb25PcGVyYXRpbmdSYXRlIjpbLTAuNSwwLjVdLCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOlstMC41LDAuNV0sIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOlstMC41LDAuNV0sImVmZmVjdGl2ZVRheFJhdGUiOlswLDAuNl0sInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwxLjY2NTMzNDUzNjkzNzczNDhlLTE2XSwicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MzI1MzMwNTAxODQ2OTI3LDAuMDIwNzM1OTk0MTgzMTg5MTY2XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDBdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6WzAuMDUxMTY5NTkwNjQzMjc0NzU0LDAuMDU3MDE3NTQzODU5NjQ5MTldLCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjpbMC4wNDA3NjA4Njk1NjUyMTcxODQsMC4wNDQzODQwNTc5NzEwMTQ1Ml0sIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjpbMCwwLjAwMDEzNDU3NTU2OTM1ODE5NzM3XSwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOlswLjAxOTEzOTQ1NzAyMzcxNzQ0MywwLjAyMDU1MzQ1OTkxNDc2MzA5NV0sIm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6WzAsMC4wOF0sIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wMzkxNjY2NjY2NjY2NjY2OCwwLjA0MjUwMDAwMDAwMDAwMDA5XSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RTYWxlc0dyb3d0aCI6WzAuMTUsMC4zXSwib3RoZXJTYWxlc0dyb3d0aCI6WzAuMDYwNzYwODY5NTY1MjE3MTksMC4wNjQzODQwNTc5NzEwMTQ1M10sInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOlswLDAuMDNdLCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6WzAuMDA1LDAuMDA1MTM0NTc1NTY5MzU4MTk3NV0sInByb2plY3RQYXlHcm93dGgiOlswLjA1LDAuMV0sIm90aGVyUGF5R3Jvd3RoIjpbMC4wMjQxMzk0NTcwMjM3MTc0NDQsMC4wMjU1NTM0NTk5MTQ3NjMwOTZdLCJvdGhlck9mZmljZXJQYXlHcm93dGgiOlswLDAuMDhdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGgiOlswLjA0NDE2NjY2NjY2NjY2NjY4LDAuMDQ3NTAwMDAwMDAwMDAwMDldLCJwcm9qZWN0U2dhUmF0ZUVuZCI6WzAsMC4wM10sIm90aGVyU2dhUmF0ZUVuZCI6WzAsMC4wMV0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjpbMC4wNDI2MzE1Nzg5NDczNjgzNiwwLjA2NTU1NTU1NTU1NTU1NTU4XSwiaW52ZXN0bWVudCI6WzE1LDIwMF0sInN1YnNpZHkiOlsxLDUwXSwibG9jYWxCZW5jaG1hcmsiOlswLDEwMF19LCJ0YXJnZXRzIjp7ImNvbXBhbnlTYWxlc0NhZ3IiOnsidmFsdWUiOjE1LCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjgyLjQsIm1heCI6MjUyLjY5LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjoyLCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NjAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo3NC44LCJtYXgiOjEzNi44NCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImxhYm9yUHJvZHVjdGl2aXR5Q2FnciI6eyJ2YWx1ZSI6MjEsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJ2YWx1ZUFkZGVkSW5jcmVhc2UiOnsidmFsdWUiOjE4Ljc4LCJtYXgiOjMzLjQzLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6Mi44NSwibWF4IjozLjc0LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiaW52ZXN0bWVudFNhbGVzUmF0aW8iOnsidmFsdWUiOjE1LCJtYXgiOjcwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZFN1YnNpZHlSYXRpbyI6eyJ2YWx1ZSI6MjEzLCJtYXgiOjM1MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImxvY2FsQmVuY2htYXJrIjp7InZhbHVlIjoyMywibWF4Ijo0MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlDYWdyIjp7InZhbHVlIjo2LCJtYXgiOjEwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUluY3JlYXNlIjp7InZhbHVlIjowLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfX0sImZvcmVjYXN0T3ZlcnJpZGVzIjp7IjIwMjk6b3RoZXI6c2FsZXMiOjg1LjEzLCIyMDI5OnByb2plY3Q6Ny04Ijo3Ljl9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2LjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mi43NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTQiOjAuNzMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi03IjozMi42NSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTkiOjAuODIsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMCI6MC4wOSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEyIjoxMS42NywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEzIjowLjYyLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTQiOjIuNDUsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNSI6MC42NCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE4IjoxMC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE5IjoxMC43MywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTIwIjo3LjUxLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjciOjIxMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMSI6NzIsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny00IjoyMy4wNCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjYuNzgsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny04Ijo1LjE5LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOSI6MC4zNiwiYWN0dWFsOnByb2plY3Q6MjAyMzpQMi00IjowLjQ1LCJhY3R1YWw6cHJvamVjdDoyMDIzOlAyLTE0IjoxLjM1LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTMiOjkwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xIjoxNDMuMiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTMiOjk3LjM4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItNCI6MC43NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTciOjM0LjUyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItOSI6MC44NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMiI6MTIuNDcsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMyI6MC42NiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjoyLjU4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTUiOjAuNjcsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xOCI6MTEuMDEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xOSI6MTEuMDEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0yMCI6Ny43MSwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTI3IjoyMjAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEiOjc2LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNCI6MjQuMzIsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny02Ijo3LjA0LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctOCI6NS41OSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTkiOjAuMzgsImFjdHVhbDpwcm9qZWN0OjIwMjQ6UDItNCI6MC40NywiYWN0dWFsOnByb2plY3Q6MjAyNDpQMi0xNCI6MS40MywiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTEzIjo5NSwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMSI6MTUwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6MC44LCJhY3R1YWw6Y29tcGFueToyMDI1OjItNyI6MzYuNCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTkiOjAuOSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEwIjowLjEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjowLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNCI6Mi43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTUiOjAuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE4IjoxMS4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTkiOjExLjMsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yMCI6Ny45MSwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI3IjoyMzAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNCI6MjUuNiwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTYiOjcuMywiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTgiOjYsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny05IjowLjQsImFjdHVhbDpwcm9qZWN0OjIwMjU6UDItNCI6MC41LCJhY3R1YWw6cHJvamVjdDoyMDI1OlAyLTE0IjoxLjUsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xMyI6MTAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTQiOjIsImJhbGFuY2Utc2hlZXQ6MjAyMzphc3NldHMiOjEzMiwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRBc3NldHMiOjY3LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FzaCI6MjQsImJhbGFuY2Utc2hlZXQ6MjAyMzpmaXhlZEFzc2V0cyI6NjUsImJhbGFuY2Utc2hlZXQ6MjAyMzp0YW5naWJsZUFzc2V0cyI6NTMsImJhbGFuY2Utc2hlZXQ6MjAyMzpidWlsZGluZ3MiOjE5LCJiYWxhbmNlLXNoZWV0OjIwMjM6bWFjaGluZXJ5IjoyNCwiYmFsYW5jZS1zaGVldDoyMDIzOmxhbmQiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjM6aW50YW5naWJsZUFzc2V0cyI6NywiYmFsYW5jZS1zaGVldDoyMDIzOnNvZnR3YXJlIjo1LCJiYWxhbmNlLXNoZWV0OjIwMjM6bGlhYmlsaXRpZXMiOjc1LCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudExpYWJpbGl0aWVzIjozOSwiYmFsYW5jZS1zaGVldDoyMDIzOnNob3J0VGVybURlYnQiOjEyLCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRMaWFiaWxpdGllcyI6MzYsImJhbGFuY2Utc2hlZXQ6MjAyMzpsb25nVGVybURlYnQiOjI5LCJiYWxhbmNlLXNoZWV0OjIwMjM6bmV0QXNzZXRzIjo1NywiYmFsYW5jZS1zaGVldDoyMDIzOnNoYXJlaG9sZGVyRXF1aXR5Ijo1NCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGl0YWwiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwZXgiOjUsImJhbGFuY2Utc2hlZXQ6MjAyNDphc3NldHMiOjE0MywiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRBc3NldHMiOjcyLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FzaCI6MjUsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZEFzc2V0cyI6NzEsImJhbGFuY2Utc2hlZXQ6MjAyNDp0YW5naWJsZUFzc2V0cyI6NTgsImJhbGFuY2Utc2hlZXQ6MjAyNDpidWlsZGluZ3MiOjIwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bWFjaGluZXJ5IjoyOCwiYmFsYW5jZS1zaGVldDoyMDI0OmxhbmQiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6aW50YW5naWJsZUFzc2V0cyI6OCwiYmFsYW5jZS1zaGVldDoyMDI0OnNvZnR3YXJlIjo2LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGlhYmlsaXRpZXMiOjc5LCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudExpYWJpbGl0aWVzIjo0MSwiYmFsYW5jZS1zaGVldDoyMDI0OnNob3J0VGVybURlYnQiOjEyLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRMaWFiaWxpdGllcyI6MzgsImJhbGFuY2Utc2hlZXQ6MjAyNDpsb25nVGVybURlYnQiOjMxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bmV0QXNzZXRzIjo2NCwiYmFsYW5jZS1zaGVldDoyMDI0OnNoYXJlaG9sZGVyRXF1aXR5Ijo2MSwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGl0YWwiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwZXgiOjgsImJhbGFuY2Utc2hlZXQ6MjAyNTphc3NldHMiOjE1NiwiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRBc3NldHMiOjc4LCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FzaCI6MjcsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZEFzc2V0cyI6NzgsImJhbGFuY2Utc2hlZXQ6MjAyNTp0YW5naWJsZUFzc2V0cyI6NjQsImJhbGFuY2Utc2hlZXQ6MjAyNTpidWlsZGluZ3MiOjIyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bWFjaGluZXJ5IjozMiwiYmFsYW5jZS1zaGVldDoyMDI1OmxhbmQiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjU6aW50YW5naWJsZUFzc2V0cyI6OSwiYmFsYW5jZS1zaGVldDoyMDI1OnNvZnR3YXJlIjo3LCJiYWxhbmNlLXNoZWV0OjIwMjU6bGlhYmlsaXRpZXMiOjgzLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudExpYWJpbGl0aWVzIjo0MywiYmFsYW5jZS1zaGVldDoyMDI1OnNob3J0VGVybURlYnQiOjExLCJiYWxhbmNlLXNoZWV0OjIwMjU6Zml4ZWRMaWFiaWxpdGllcyI6NDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpsb25nVGVybURlYnQiOjMyLCJiYWxhbmNlLXNoZWV0OjIwMjU6bmV0QXNzZXRzIjo3MywiYmFsYW5jZS1zaGVldDoyMDI1OnNoYXJlaG9sZGVyRXF1aXR5Ijo3MCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGl0YWwiOjEwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwZXgiOjEwLCJkcml2ZXI6cHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MCI6LTAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjEiOjAuMywiZHJpdmVyOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvOjEiOjAuOTksImRyaXZlcjpvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybzoxIjowLjk5LCJkcml2ZXI6cHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsImRyaXZlci1yYW5nZTpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmU6MSI6MSwiZHJpdmVyOm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwiZHJpdmVyLXJhbmdlOm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlOjEiOjEsImRyaXZlcjpwcm9qZWN0T2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjowLjksImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZToxIjoxLCJkcml2ZXI6b3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMiwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZToxIjoxLCJkcml2ZXI6cHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNSwiZHJpdmVyLXJhbmdlOnByb2plY3RSZXNlYXJjaERldmVsb3BtZW50UmF0ZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjEiOjAuMywiZHJpdmVyOm90aGVyUmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA0LCJkcml2ZXItcmFuZ2U6b3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZToxIjowLjMsImRyaXZlcjpwcm9qZWN0Tm9uT3BlcmF0aW5nUmF0ZSI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3ROb25PcGVyYXRpbmdSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpwcm9qZWN0Tm9uT3BlcmF0aW5nUmF0ZToxIjowLjUsImRyaXZlcjpvdGhlck5vbk9wZXJhdGluZ1JhdGUiOi0wLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyTm9uT3BlcmF0aW5nUmF0ZTowIjotMC41LCJkcml2ZXItcmFuZ2U6b3RoZXJOb25PcGVyYXRpbmdSYXRlOjEiOjAuNSwiZHJpdmVyOnByb2plY3RFeHRyYW9yZGluYXJ5UmF0ZSI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RFeHRyYW9yZGluYXJ5UmF0ZTowIjotMC41LCJkcml2ZXItcmFuZ2U6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlOjEiOjAuNSwiZHJpdmVyOm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImRyaXZlci1yYW5nZTpvdGhlckV4dHJhb3JkaW5hcnlSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpvdGhlckV4dHJhb3JkaW5hcnlSYXRlOjEiOjAuNSwiZHJpdmVyOmVmZmVjdGl2ZVRheFJhdGUiOjAuMywiZHJpdmVyLXJhbmdlOmVmZmVjdGl2ZVRheFJhdGU6MCI6MCwiZHJpdmVyLXJhbmdlOmVmZmVjdGl2ZVRheFJhdGU6MSI6MC42LCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjEuNjY1MzM0NTM2OTM3NzM0OGUtMTYsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkzMjUzMzA1MDE4NDY5MjcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNzM1OTk0MTgzMTg5MTY2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLjAxOTEzOTQ1NzAyMzcxNzQ0MywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNTUzNDU5OTE0NzYzMDk1LCJkcml2ZXI6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wMzkxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDQyNTAwMDAwMDAwMDAwMDksImRyaXZlcjpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjAiOjAuMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MSI6MC4zLCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NzI0NjM3NjgxMTU4NiwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MCI6MC4wNjA3NjA4Njk1NjUyMTcxOSwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MSI6MC4wNjQzODQwNTc5NzEwMTQ1MywiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZToxIjowLjAzLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDoxIjowLjAwNTEzNDU3NTU2OTM1ODE5NzUsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDowIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDoxIjowLjEsImRyaXZlcjpvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjAiOjAuMDI0MTM5NDU3MDIzNzE3NDQ0LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wMjU1NTM0NTk5MTQ3NjMwOTYsImRyaXZlcjpvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGg6MSI6MC4wOCwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjowLjA0NDE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MSI6MC4wNDc1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjAxNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDoxIjowLjAzLCJkcml2ZXI6b3RoZXJTZ2FSYXRlRW5kIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMDEsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAuMDQyNjMxNTc4OTQ3MzY4MzYsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjA2NTU1NTU1NTU1NTU1NTU4LCJkcml2ZXI6aW52ZXN0bWVudCI6MjMsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjAiOjE1LCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDoxIjoyMDAsImRyaXZlcjpzdWJzaWR5Ijo3LjY2LCJkcml2ZXItcmFuZ2U6c3Vic2lkeTowIjoxLCJkcml2ZXItcmFuZ2U6c3Vic2lkeToxIjo1MCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoxNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjo4Mi40LCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjoyLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOm1heCI6NywidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOnZhbHVlIjo2MCwidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOm1heCI6OTUsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOnZhbHVlIjoyMiwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOnZhbHVlIjo3NC44LCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOnZhbHVlIjoyMSwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2FncjptYXgiOjM1LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOnZhbHVlIjoxOC43OCwidGFyZ2V0OmVtcGxveWVlUGF5Q2Fncjp2YWx1ZSI6NywidGFyZ2V0OmVtcGxveWVlUGF5Q2FncjptYXgiOjEwLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlJbmNyZWFzZTp2YWx1ZSI6Mi44NSwidGFyZ2V0OmludmVzdG1lbnRTYWxlc1JhdGlvOnZhbHVlIjoxNSwidGFyZ2V0OmludmVzdG1lbnRTYWxlc1JhdGlvOm1heCI6NzAsInRhcmdldDp2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvOnZhbHVlIjoyMTMsInRhcmdldDp2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvOm1heCI6MzUwLCJ0YXJnZXQ6bG9jYWxCZW5jaG1hcms6dmFsdWUiOjIzLCJ0YXJnZXQ6bG9jYWxCZW5jaG1hcms6bWF4Ijo0MCwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOnZhbHVlIjo2LCJ0YXJnZXQ6b2ZmaWNlclBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0Om9mZmljZXJQYXlJbmNyZWFzZTp2YWx1ZSI6MCwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOm1heCI6MjUyLjY5LCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6bWF4IjoxMzYuODQsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6bWF4IjozMy40MywidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6bWF4IjozLjc0fSwibWV0cmljR3JvdXBCYXNlcyI6eyJjb21wYW55U2FsZXMiOiJyYXRlIiwicHJvamVjdFNhbGVzIjoicmF0ZSIsImxhYm9yUHJvZHVjdGl2aXR5IjoicmF0ZSIsImVtcGxveWVlUGF5IjoicmF0ZSJ9LCJhcHBsaWNhdGlvbkNhdGVnb3J5IjoiZ2VuZXJhbCIsImFkanVzdGVkRHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDExODIzODMwNDA5MzU1LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjoxLjE3NDE4NjQ5MTA2NDQ2NmUtMTYsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDM4NTYyMDU5MTMzNTYyLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1MjE1ODg4ODcxODM5NDU1LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDEzODQ0NTAzNTM2MTg3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU2OTcwNTYzMTYxMzE4LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODE5ODg5MTE0MzQ5OTE1LCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDc5NDQxMTQxNDk4MjIyNSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyMDM3MDgxODExNTQxMjY4LCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjYyMTczNTY4MTgzMTgsInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE0OTUyODA2OTIyNjYwODk1LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDg0ODEyODMzNzQ4NjY1MDEsIm90aGVyUGF5R3Jvd3RoIjowLjAyNDg2Mzc5NTU1OTYzNzM0LCJvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjAyNjUzNDAwNjk4NzM2ODk5LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4NjgzOTY4MjE4NjA5MDQsInByb2plY3RTZ2FSYXRlRW5kIjowLjAxNDk4NjU1MDI4NzY0MTMzOSwib3RoZXJTZ2FSYXRlRW5kIjowLjAwNTAxMTk3MjIyNzQzNDc5MiwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzNzYyOTY4NDI4OTIzNTksImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9fQ==</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MiwiY29ncyI6NDguOTYsImVtcGxveWVlUGF5Ijo1LjE5LCJvZmZpY2VyUGF5IjowLjM2LCJkZXByZWNpYXRpb24iOjEuOCwib3RoZXJTZ2EiOjksImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQuOTMsImVtcGxveWVlQm9udXMiOjAuMjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzIsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40NSwic2dhRGVwcmVjaWF0aW9uIjoxLjM1LCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM2fSwib3RoZXIiOnsic2FsZXMiOjY0LjQsImNvZ3MiOjQzLjc5LCJlbXBsb3llZVBheSI6Ny4xLCJvZmZpY2VyUGF5IjowLjU1LCJkZXByZWNpYXRpb24iOjEuMzgsIm90aGVyU2dhIjo3LjM2LCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ni43NCwiZW1wbG95ZWVCb251cyI6MC4zNiwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41LCJvZmZpY2VyQm9udXMiOjAuMDUsImNvZ3NEZXByZWNpYXRpb24iOjAuMjgsInNnYURlcHJlY2lhdGlvbiI6MS4xLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjI4LCJvcmRpbmFyeUluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsInByZVRheEluY29tZSI6My45NTAwMDAwMDAwMDAwMDMsIm5ldEluY29tZSI6Ny41MX19LHsieWVhciI6MjAyNCwicm9sZSI6InByZXZpb3VzIiwicHJvamVjdCI6eyJzYWxlcyI6NzYsImNvZ3MiOjUxLjY4LCJlbXBsb3llZVBheSI6NS41OSwib2ZmaWNlclBheSI6MC4zOCwiZGVwcmVjaWF0aW9uIjoxLjksIm90aGVyU2dhIjo5LjUsImhlYWRjb3VudCI6OTUsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjUuMzEsImVtcGxveWVlQm9udXMiOjAuMjgsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuMzQsIm9mZmljZXJCb251cyI6MC4wNCwiY29nc0RlcHJlY2lhdGlvbiI6MC40Nywic2dhRGVwcmVjaWF0aW9uIjoxLjQzLCJyZXNlYXJjaERldmVsb3BtZW50IjowLjM4fSwib3RoZXIiOnsic2FsZXMiOjY3LjIsImNvZ3MiOjQ1LjcsImVtcGxveWVlUGF5Ijo3LjU0LCJvZmZpY2VyUGF5IjowLjU4LCJkZXByZWNpYXRpb24iOjEuNDQsIm90aGVyU2dhIjo3LjY4LCJoZWFkY291bnQiOjEyNSwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Ny4xNiwiZW1wbG95ZWVCb251cyI6MC4zOCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC41Miwib2ZmaWNlckJvbnVzIjowLjA2LCJjb2dzRGVwcmVjaWF0aW9uIjowLjI5LCJzZ2FEZXByZWNpYXRpb24iOjEuMTUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMjksIm9yZGluYXJ5SW5jb21lIjozLjk2OTk5OTk5OTk5OTk5NywicHJlVGF4SW5jb21lIjozLjk2OTk5OTk5OTk5OTk5NywibmV0SW5jb21lIjo3LjcxfX0seyJ5ZWFyIjoyMDI1LCJyb2xlIjoibGF0ZXN0IiwicHJvamVjdCI6eyJzYWxlcyI6ODAsImNvZ3MiOjU0LjQsImVtcGxveWVlUGF5Ijo2LCJlbXBsb3llZVNhbGFyeSI6NS43LCJlbXBsb3llZUJvbnVzIjowLjMsIm9mZmljZXJQYXkiOjAuNCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MC4zNiwib2ZmaWNlckJvbnVzIjowLjA0LCJkZXByZWNpYXRpb24iOjIsImNvZ3NEZXByZWNpYXRpb24iOjAuNSwic2dhRGVwcmVjaWF0aW9uIjoxLjUsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuNCwib3RoZXJTZ2EiOjEwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwLCJjb2dzIjo0Ny42LCJlbXBsb3llZVBheSI6OCwiZW1wbG95ZWVTYWxhcnkiOjcuNiwiZW1wbG95ZWVCb251cyI6MC40LCJvZmZpY2VyUGF5IjowLjYsIm9mZmljZXJDb21wZW5zYXRpb24iOjAuNTQsIm9mZmljZXJCb251cyI6MC4wNiwiZGVwcmVjaWF0aW9uIjoxLjUsImNvZ3NEZXByZWNpYXRpb24iOjAuMywic2dhRGVwcmVjaWF0aW9uIjoxLjIsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjAuMywib3RoZXJTZ2EiOjgsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjozLjk5OTk5OTk5OTk5OTk5NjQsInByZVRheEluY29tZSI6My45OTk5OTk5OTk5OTk5OTY0LCJuZXRJbmNvbWUiOjcuOTF9fV0sImJhbGFuY2VTaGVldHMiOlt7InllYXIiOjIwMjMsImFzc2V0cyI6MTMyLCJjdXJyZW50QXNzZXRzIjo2NywiY2FzaCI6MjQsImZpeGVkQXNzZXRzIjo2NSwidGFuZ2libGVBc3NldHMiOjUzLCJidWlsZGluZ3MiOjE5LCJtYWNoaW5lcnkiOjI0LCJsYW5kIjoxMCwiaW50YW5naWJsZUFzc2V0cyI6Nywic29mdHdhcmUiOjUsImxpYWJpbGl0aWVzIjo3NSwiY3VycmVudExpYWJpbGl0aWVzIjozOSwic2hvcnRUZXJtRGVidCI6MTIsImZpeGVkTGlhYmlsaXRpZXMiOjM2LCJsb25nVGVybURlYnQiOjI5LCJuZXRBc3NldHMiOjU3LCJzaGFyZWhvbGRlckVxdWl0eSI6NTQsImNhcGl0YWwiOjEwLCJjYXBleCI6NX0seyJ5ZWFyIjoyMDI0LCJhc3NldHMiOjE0MywiY3VycmVudEFzc2V0cyI6NzIsImNhc2giOjI1LCJmaXhlZEFzc2V0cyI6NzEsInRhbmdpYmxlQXNzZXRzIjo1OCwiYnVpbGRpbmdzIjoyMCwibWFjaGluZXJ5IjoyOCwibGFuZCI6MTAsImludGFuZ2libGVBc3NldHMiOjgsInNvZnR3YXJlIjo2LCJsaWFiaWxpdGllcyI6NzksImN1cnJlbnRMaWFiaWxpdGllcyI6NDEsInNob3J0VGVybURlYnQiOjEyLCJmaXhlZExpYWJpbGl0aWVzIjozOCwibG9uZ1Rlcm1EZWJ0IjozMSwibmV0QXNzZXRzIjo2NCwic2hhcmVob2xkZXJFcXVpdHkiOjYxLCJjYXBpdGFsIjoxMCwiY2FwZXgiOjh9LHsieWVhciI6MjAyNSwiYXNzZXRzIjoxNTYsImN1cnJlbnRBc3NldHMiOjc4LCJjYXNoIjoyNywiZml4ZWRBc3NldHMiOjc4LCJ0YW5naWJsZUFzc2V0cyI6NjQsImJ1aWxkaW5ncyI6MjIsIm1hY2hpbmVyeSI6MzIsImxhbmQiOjEwLCJpbnRhbmdpYmxlQXNzZXRzIjo5LCJzb2Z0d2FyZSI6NywibGlhYmlsaXRpZXMiOjgzLCJjdXJyZW50TGlhYmlsaXRpZXMiOjQzLCJzaG9ydFRlcm1EZWJ0IjoxMSwiZml4ZWRMaWFiaWxpdGllcyI6NDAsImxvbmdUZXJtRGVidCI6MzIsIm5ldEFzc2V0cyI6NzMsInNoYXJlaG9sZGVyRXF1aXR5Ijo3MCwiY2FwaXRhbCI6MTAsImNhcGV4IjoxMH1dLCJmdXR1cmVDYXBleCI6W3sieWVhciI6MjAyNiwidmFsdWUiOjB9LHsieWVhciI6MjAyNywidmFsdWUiOjB9LHsieWVhciI6MjAyOCwidmFsdWUiOjB9LHsieWVhciI6MjAyOSwidmFsdWUiOjB9LHsieWVhciI6MjAzMCwidmFsdWUiOjB9LHsieWVhciI6MjAzMSwidmFsdWUiOjB9XSwiZHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTcyNDYzNzY4MTE1ODYsInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDcsIm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsInByb2plY3RTZ2FSYXRlRW5kIjowLjAxNSwib3RoZXJTZ2FSYXRlRW5kIjowLjAwNSwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzODAxMTY5NTkwNjQzMjUsImludmVzdG1lbnQiOjIzLCJzdWJzaWR5Ijo3LjY2LCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOlswLjY2LDAuN10sIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjpbMC42NiwwLjddLCJwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOlswLDFdLCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOlswLDFdLCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOlstMC41LDAuNV0sIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6Wy0wLjUsMC41XSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJlZmZlY3RpdmVUYXhSYXRlIjpbMCwwLjZdLCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6WzAsMS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNl0sInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOlswLjAxOTMyNTMzMDUwMTg0NjkyNywwLjAyMDczNTk5NDE4MzE4OTE2Nl0sInByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6WzAuMDQwNzYwODY5NTY1MjE3MTg0LDAuMDQ0Mzg0MDU3OTcxMDE0NTJdLCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6WzAsMC4wMDAxMzQ1NzU1NjkzNTgxOTczN10sIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkxMzk0NTcwMjM3MTc0NDMsMC4wMjA1NTM0NTk5MTQ3NjMwOTVdLCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6WzAuMDM5MTY2NjY2NjY2NjY2NjgsMC4wNDI1MDAwMDAwMDAwMDAwOV0sIm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDBdLCJwcm9qZWN0U2FsZXNHcm93dGgiOlswLjE1LDAuM10sIm90aGVyU2FsZXNHcm93dGgiOlswLjA2MDc2MDg2OTU2NTIxNzE5LDAuMDY0Mzg0MDU3OTcxMDE0NTNdLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjpbMCwwLjAzXSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOlswLjAwNSwwLjAwNTEzNDU3NTU2OTM1ODE5NzVdLCJwcm9qZWN0UGF5R3Jvd3RoIjpbMC4wNSwwLjFdLCJvdGhlclBheUdyb3d0aCI6WzAuMDI0MTM5NDU3MDIzNzE3NDQ0LDAuMDI1NTUzNDU5OTE0NzYzMDk2XSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjpbMCwwLjA4XSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6WzAsMC4wOF0sIm90aGVySGVhZGNvdW50R3Jvd3RoIjpbMC4wNDQxNjY2NjY2NjY2NjY2OCwwLjA0NzUwMDAwMDAwMDAwMDA5XSwicHJvamVjdFNnYVJhdGVFbmQiOlswLDAuMDNdLCJvdGhlclNnYVJhdGVFbmQiOlswLDAuMDFdLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6WzAuMDQyNjMxNTc4OTQ3MzY4MzYsMC4wNjU1NTU1NTU1NTU1NTU1OF0sImludmVzdG1lbnQiOlsxNSwyMDBdLCJzdWJzaWR5IjpbMSw1MF0sImxvY2FsQmVuY2htYXJrIjpbMCwxMDBdfSwidGFyZ2V0cyI6eyJjb21wYW55U2FsZXNDYWdyIjp7InZhbHVlIjoxNSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo4Mi40LCJtYXgiOjI1Mi42OSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlQYXlTY2hlZHVsZSI6eyJ2YWx1ZSI6MiwibWF4Ijo3LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzU2hhcmUiOnsidmFsdWUiOjYwLCJtYXgiOjk1LCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzQ2FnciI6eyJ2YWx1ZSI6MjIsIm1heCI6MzUsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNJbmNyZWFzZSI6eyJ2YWx1ZSI6NzQuOCwibWF4IjoxMzYuODQsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsYWJvclByb2R1Y3Rpdml0eUNhZ3IiOnsidmFsdWUiOjIxLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZEluY3JlYXNlIjp7InZhbHVlIjoxOC43OCwibWF4IjozMy40MywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5Q2FnciI6eyJ2YWx1ZSI6NywibWF4IjoxMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImVtcGxveWVlUGF5SW5jcmVhc2UiOnsidmFsdWUiOjIuODUsIm1heCI6My43NCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjoxNSwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX19LCJmb3JlY2FzdE92ZXJyaWRlcyI6eyIyMDI5Om90aGVyOnNhbGVzIjo4NS4xMywiMjAyOTpwcm9qZWN0OjctOCI6Ny45fSwiZnV0dXJlSW5wdXRCYXNpcyI6Im90aGVyIiwiaW5wdXRWYWx1ZXMiOnsiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEiOjEzNi40LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMyI6OTIuNzUsImFjdHVhbDpjb21wYW55OjIwMjM6Mi00IjowLjczLCJhY3R1YWw6Y29tcGFueToyMDIzOjItNyI6MzIuNjUsImFjdHVhbDpjb21wYW55OjIwMjM6Mi05IjowLjgyLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTAiOjAuMDksImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMiI6MTEuNjcsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMyI6MC42MiwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE0IjoyLjQ1LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTUiOjAuNjQsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xOCI6MTAuNzMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xOSI6MTAuNzMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yMCI6Ny41MSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTI3IjoyMTAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEiOjcyLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNCI6MjMuMDQsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny02Ijo2Ljc4LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOCI6NS4xOSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTkiOjAuMzYsImFjdHVhbDpwcm9qZWN0OjIwMjM6UDItNCI6MC40NSwiYWN0dWFsOnByb2plY3Q6MjAyMzpQMi0xNCI6MS4zNSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEzIjo5MCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMSI6MTQzLjIsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0zIjo5Ny4zOCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTQiOjAuNzYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi03IjozNC41MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTkiOjAuODYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMCI6MC4xLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTIiOjEyLjQ3LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTMiOjAuNjYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNCI6Mi41OCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE1IjowLjY3LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTgiOjExLjAxLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTkiOjExLjAxLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjAiOjcuNzEsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0yNyI6MjIwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xIjo3NiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0LjMyLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNiI6Ny4wNCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTgiOjUuNTksImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjowLjM4LCJhY3R1YWw6cHJvamVjdDoyMDI0OlAyLTQiOjAuNDcsImFjdHVhbDpwcm9qZWN0OjIwMjQ6UDItMTQiOjEuNDMsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xMyI6OTUsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEiOjE1MCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTMiOjEwMiwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTQiOjAuOCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTciOjM2LjQsImFjdHVhbDpjb21wYW55OjIwMjU6Mi05IjowLjksImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMCI6MC4xLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTIiOjEzLjMsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMyI6MC43LCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTQiOjIuNywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE1IjowLjcsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xOCI6MTEuMywiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE5IjoxMS4zLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjAiOjcuOTEsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yNyI6MjMwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xIjo4MCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTQiOjI1LjYsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny02Ijo3LjMsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny04Ijo2LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOSI6MC40LCJhY3R1YWw6cHJvamVjdDoyMDI1OlAyLTQiOjAuNSwiYWN0dWFsOnByb2plY3Q6MjAyNTpQMi0xNCI6MS41LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTMiOjEwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTE0IjoyLCJiYWxhbmNlLXNoZWV0OjIwMjM6YXNzZXRzIjoxMzIsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NywiYmFsYW5jZS1zaGVldDoyMDIzOmNhc2giOjI0LCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRBc3NldHMiOjY1LCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzLCJiYWxhbmNlLXNoZWV0OjIwMjM6YnVpbGRpbmdzIjoxOSwiYmFsYW5jZS1zaGVldDoyMDIzOm1hY2hpbmVyeSI6MjQsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmludGFuZ2libGVBc3NldHMiOjcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzb2Z0d2FyZSI6NSwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NSwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRMaWFiaWxpdGllcyI6MzksImJhbGFuY2Utc2hlZXQ6MjAyMzpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2LCJiYWxhbmNlLXNoZWV0OjIwMjM6bG9uZ1Rlcm1EZWJ0IjoyOSwiYmFsYW5jZS1zaGVldDoyMDIzOm5ldEFzc2V0cyI6NTcsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGV4Ijo1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50QXNzZXRzIjo3MiwiYmFsYW5jZS1zaGVldDoyMDI0OmNhc2giOjI1LCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxLCJiYWxhbmNlLXNoZWV0OjIwMjQ6dGFuZ2libGVBc3NldHMiOjU4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6YnVpbGRpbmdzIjoyMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmludGFuZ2libGVBc3NldHMiOjgsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NiwiYmFsYW5jZS1zaGVldDoyMDI0OmxpYWJpbGl0aWVzIjo3OSwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRMaWFiaWxpdGllcyI6NDEsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMiwiYmFsYW5jZS1zaGVldDoyMDI0OmZpeGVkTGlhYmlsaXRpZXMiOjM4LCJiYWxhbmNlLXNoZWV0OjIwMjQ6bG9uZ1Rlcm1EZWJ0IjozMSwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaGFyZWhvbGRlckVxdWl0eSI6NjEsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4LCJiYWxhbmNlLXNoZWV0OjIwMjU6YXNzZXRzIjoxNTYsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50QXNzZXRzIjo3OCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3LCJiYWxhbmNlLXNoZWV0OjIwMjU6Zml4ZWRBc3NldHMiOjc4LCJiYWxhbmNlLXNoZWV0OjIwMjU6dGFuZ2libGVBc3NldHMiOjY0LCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMiwiYmFsYW5jZS1zaGVldDoyMDI1Om1hY2hpbmVyeSI6MzIsImJhbGFuY2Utc2hlZXQ6MjAyNTpsYW5kIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjksImJhbGFuY2Utc2hlZXQ6MjAyNTpzb2Z0d2FyZSI6NywiYmFsYW5jZS1zaGVldDoyMDI1OmxpYWJpbGl0aWVzIjo4MywiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaG9ydFRlcm1EZWJ0IjoxMSwiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkTGlhYmlsaXRpZXMiOjQwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMiwiYmFsYW5jZS1zaGVldDoyMDI1Om5ldEFzc2V0cyI6NzMsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaGFyZWhvbGRlckVxdWl0eSI6NzAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGV4IjoxMCwiZHJpdmVyOnByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDoxIjowLjMsImRyaXZlcjpwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybzowIjowLjY2LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybzoxIjowLjcsImRyaXZlcjpvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvOjAiOjAuNjYsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybzoxIjowLjcsImRyaXZlcjpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwiZHJpdmVyLXJhbmdlOnByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZToxIjoxLCJkcml2ZXI6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJkcml2ZXItcmFuZ2U6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjowLjksImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGU6MSI6MC4zLCJkcml2ZXI6b3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjEiOjAuMywiZHJpdmVyOnByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdE5vbk9wZXJhdGluZ1JhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOnByb2plY3ROb25PcGVyYXRpbmdSYXRlOjEiOjAuNSwiZHJpdmVyOm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJOb25PcGVyYXRpbmdSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpvdGhlck5vbk9wZXJhdGluZ1JhdGU6MSI6MC41LCJkcml2ZXI6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6b3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6ZWZmZWN0aXZlVGF4UmF0ZSI6MC4zLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZTowIjowLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZToxIjowLjYsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjUuNTUxMTE1MTIzMTI1NzgzZS0xNywiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZTowIjowLjAxOTMyNTMzMDUwMTg0NjkyNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA3MzU5OTQxODMxODkxNjYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNTcyNDYzNzY4MTE1ODU0LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZTowIjowLjA0MDc2MDg2OTU2NTIxNzE4NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNDQzODQwNTc5NzEwMTQ1MiwiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjAuMDAwMTM0NTc1NTY5MzU4MTk3MzcsImRyaXZlcjpvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDE5MTM5NDU3MDIzNzE3NDQzLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA1NTM0NTk5MTQ3NjMwOTUsImRyaXZlcjpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZToxIjowLjA4LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjAzOTE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNDI1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MCI6MC4xNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjMsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MCI6MC4wMjQxMzk0NTcwMjM3MTc0NDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDoxIjowLjAyNTU1MzQ1OTkxNDc2MzA5NiwiZHJpdmVyOm90aGVyT2ZmaWNlclBheUdyb3d0aCI6MC4wNDUsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aDoxIjowLjA4LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTgzMzMzMzMzMzMzMzM4NiwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjAiOjAuMDQ0MTY2NjY2NjY2NjY2NjgsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDoxIjowLjA0NzUwMDAwMDAwMDAwMDA5LCJkcml2ZXI6cHJvamVjdFNnYVJhdGVFbmQiOjAuMDE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjEiOjAuMDMsImRyaXZlcjpvdGhlclNnYVJhdGVFbmQiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MSI6MC4wMSwiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MCI6MC4wNDI2MzE1Nzg5NDczNjgzNiwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjEiOjAuMDY1NTU1NTU1NTU1NTU1NTgsImRyaXZlcjppbnZlc3RtZW50IjoyMywiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUsImRyaXZlci1yYW5nZTppbnZlc3RtZW50OjEiOjIwMCwiZHJpdmVyOnN1YnNpZHkiOjcuNjYsImRyaXZlci1yYW5nZTpzdWJzaWR5OjAiOjEsImRyaXZlci1yYW5nZTpzdWJzaWR5OjEiOjUwLCJkcml2ZXI6bG9jYWxCZW5jaG1hcmsiOjIzLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MCI6MCwiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjEiOjEwMCwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6dmFsdWUiOjE1LCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6dmFsdWUiOjgyLjQsInRhcmdldDpjb21wYW55UGF5U2NoZWR1bGU6dmFsdWUiOjIsInRhcmdldDpjb21wYW55UGF5U2NoZWR1bGU6bWF4Ijo3LCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6dmFsdWUiOjYwLCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6bWF4Ijo5NSwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6dmFsdWUiOjIyLCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6dmFsdWUiOjc0LjgsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6dmFsdWUiOjIxLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOm1heCI6MzUsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6dmFsdWUiOjE4Ljc4LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOnZhbHVlIjo3LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOm1heCI6MTAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOnZhbHVlIjoyLjg1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86dmFsdWUiOjE1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86bWF4Ijo3MCwidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86dmFsdWUiOjIxMywidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86bWF4IjozNTAsInRhcmdldDpsb2NhbEJlbmNobWFyazp2YWx1ZSI6MjMsInRhcmdldDpsb2NhbEJlbmNobWFyazptYXgiOjQwLCJ0YXJnZXQ6b2ZmaWNlclBheUNhZ3I6dmFsdWUiOjYsInRhcmdldDpvZmZpY2VyUGF5Q2FncjptYXgiOjEwLCJ0YXJnZXQ6b2ZmaWNlclBheUluY3JlYXNlOnZhbHVlIjowLCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6bWF4IjoyNTIuNjksInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTptYXgiOjEzNi44NCwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTptYXgiOjMzLjQzLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlJbmNyZWFzZTptYXgiOjMuNzR9LCJtZXRyaWNHcm91cEJhc2VzIjp7ImNvbXBhbnlTYWxlcyI6InJhdGUiLCJwcm9qZWN0U2FsZXMiOiJyYXRlIiwibGFib3JQcm9kdWN0aXZpdHkiOiJyYXRlIiwiZW1wbG95ZWVQYXkiOiJyYXRlIn0sImFwcGxpY2F0aW9uQ2F0ZWdvcnkiOiJnZW5lcmFsIiwiYWRqdXN0ZWREcml2ZXJzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsInByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgwMDI4NDA0NTQyOTk2MSwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgwMDUyNDc2MjMzNTg5OSwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA1MDE2NDQ3MzY4NDE5NCwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MS4xNzQxODY0OTEwNjQ0NjZlLTE2LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDA3NDY3NTA0OTM3NTkyNywicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTM0MDkwNjM0NzUwMTQwMywicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQxMjg3NTYxMTg3OTAzNiwib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI2MjAwODk1NTgzMTQ1OSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTgzMDU4MTAwNzY2NTk1LCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDU4MTAxNDY2NTA4MTMxLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIwMjEyOTI5MTQ1MzYxNTYsIm90aGVyU2FsZXNHcm93dGgiOjAuMDYyNTQyMzQxMDg0MDY4MjMsInByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE0OTk0NTMxODYxODcyNTUxLCJvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsInByb2plY3RQYXlHcm93dGgiOjAuMDg0NjU3MDI3NjgwNzMxLCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4ODAyMTk0MDI2MDIzMywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wMjM0OTc4NDU2NjU1NDI1NSwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODcyODIxNjY3NjA0OTg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wMTQ5OTk3MzcyMjE1OTkxMDYsIm90aGVyU2dhUmF0ZUVuZCI6MC4wMDUwMjY1MjM0NDMxNzAyNzEsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1Mzc5NTIyMjczNjgwNjY1LCJpbnZlc3RtZW50IjoyMywic3Vic2lkeSI6Ny42NiwibG9jYWxCZW5jaG1hcmsiOjIzfX0=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Model annual cogs rate transitions
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -384,7 +384,7 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <v>25.077299690268575</v>
+        <v>27.83033380160913</v>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
@@ -414,7 +414,7 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <v>1963420.9999999995</v>
+        <v>2219470.9999999995</v>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <v>256.3212793733681</v>
+        <v>289.7481723237597</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
@@ -1338,13 +1338,13 @@
         <v>11765868</v>
       </c>
       <c r="H5" s="2">
-        <v>13433135</v>
+        <v>13503917</v>
       </c>
       <c r="I5" s="2">
-        <v>15403258</v>
+        <v>15317999</v>
       </c>
       <c r="J5" s="2">
-        <v>17736579</v>
+        <v>17432946</v>
       </c>
     </row>
     <row r="6">
@@ -1406,13 +1406,13 @@
         <v>5536879</v>
       </c>
       <c r="H7" s="4">
-        <v>6510222</v>
+        <v>6439440</v>
       </c>
       <c r="I7" s="4">
-        <v>7587065.969999999</v>
+        <v>7672324.969999999</v>
       </c>
       <c r="J7" s="4">
-        <v>8887231.75</v>
+        <v>9190864.75</v>
       </c>
     </row>
     <row r="8">
@@ -1440,13 +1440,13 @@
         <v>31.999999768822835</v>
       </c>
       <c r="H8" s="2">
-        <v>32.643561462596296</v>
+        <v>32.28864628958906</v>
       </c>
       <c r="I8" s="2">
-        <v>33.00112682144165</v>
+        <v>33.37197414012778</v>
       </c>
       <c r="J8" s="2">
-        <v>33.38076518591539</v>
+        <v>34.52122176011186</v>
       </c>
     </row>
     <row r="9">
@@ -1780,13 +1780,13 @@
         <v>1297150</v>
       </c>
       <c r="H18" s="4">
-        <v>1892515</v>
+        <v>1821733</v>
       </c>
       <c r="I18" s="4">
-        <v>2516058.799999999</v>
+        <v>2601317.799999999</v>
       </c>
       <c r="J18" s="4">
-        <v>3308236.7699999996</v>
+        <v>3611869.7699999996</v>
       </c>
     </row>
     <row r="19">
@@ -1814,13 +1814,13 @@
         <v>7.496786492919304</v>
       </c>
       <c r="H19" s="2">
-        <v>9.489450547367728</v>
+        <v>9.134535374360494</v>
       </c>
       <c r="I19" s="2">
-        <v>10.94399019032179</v>
+        <v>11.314837509007921</v>
       </c>
       <c r="J19" s="2">
-        <v>12.425857444167717</v>
+        <v>13.566314018364181</v>
       </c>
     </row>
     <row r="20">
@@ -1848,13 +1848,13 @@
         <v>1257482</v>
       </c>
       <c r="H20" s="4">
-        <v>1737685</v>
+        <v>1666903</v>
       </c>
       <c r="I20" s="4">
-        <v>2350316</v>
+        <v>2435575</v>
       </c>
       <c r="J20" s="4">
-        <v>3130771</v>
+        <v>3434404</v>
       </c>
     </row>
     <row r="21">
@@ -1882,13 +1882,13 @@
         <v>1257482</v>
       </c>
       <c r="H21" s="2">
-        <v>1737685</v>
+        <v>1666903</v>
       </c>
       <c r="I21" s="2">
-        <v>2350316</v>
+        <v>2435575</v>
       </c>
       <c r="J21" s="2">
-        <v>3130771</v>
+        <v>3434404</v>
       </c>
     </row>
     <row r="22">
@@ -1916,13 +1916,13 @@
         <v>880237</v>
       </c>
       <c r="H22" s="2">
-        <v>1216380</v>
+        <v>1166832</v>
       </c>
       <c r="I22" s="2">
-        <v>1645221</v>
+        <v>1704903</v>
       </c>
       <c r="J22" s="2">
-        <v>2191540</v>
+        <v>2404083</v>
       </c>
     </row>
     <row r="23">
@@ -2052,13 +2052,13 @@
         <v>3460459</v>
       </c>
       <c r="H26" s="4">
-        <v>4178279</v>
+        <v>4107497</v>
       </c>
       <c r="I26" s="4">
-        <v>4963855.969999999</v>
+        <v>5049114.969999999</v>
       </c>
       <c r="J26" s="4">
-        <v>5932265.75</v>
+        <v>6235898.75</v>
       </c>
     </row>
     <row r="27">
@@ -2088,13 +2088,13 @@
         <v>4.7439697723573815</v>
       </c>
       <c r="H27" s="2">
-        <v>20.74349096463792</v>
+        <v>18.69803976871276</v>
       </c>
       <c r="I27" s="2">
-        <v>18.801448395379982</v>
+        <v>22.92437389485613</v>
       </c>
       <c r="J27" s="2">
-        <v>19.509223995473857</v>
+        <v>23.504788206476547</v>
       </c>
     </row>
     <row r="28">
@@ -2122,13 +2122,13 @@
         <v>19.99947753960686</v>
       </c>
       <c r="H28" s="2">
-        <v>20.950730611701932</v>
+        <v>20.595815438694697</v>
       </c>
       <c r="I28" s="2">
-        <v>21.591065773920015</v>
+        <v>21.961913092606146</v>
       </c>
       <c r="J28" s="2">
-        <v>22.28180558262119</v>
+        <v>23.422262156817652</v>
       </c>
     </row>
     <row r="29">
@@ -2364,13 +2364,13 @@
         <v>12912.160447761195</v>
       </c>
       <c r="H35" s="2">
-        <v>15138.692028985508</v>
+        <v>14882.235507246376</v>
       </c>
       <c r="I35" s="2">
-        <v>17356.139755244752</v>
+        <v>17654.248146853144</v>
       </c>
       <c r="J35" s="2">
-        <v>20041.438344594593</v>
+        <v>21067.225506756757</v>
       </c>
     </row>
     <row r="36">
@@ -2398,13 +2398,13 @@
         <v>1647150</v>
       </c>
       <c r="H36" s="4">
-        <v>2242515</v>
+        <v>2171733</v>
       </c>
       <c r="I36" s="4">
-        <v>2866058.799999999</v>
+        <v>2951317.799999999</v>
       </c>
       <c r="J36" s="4">
-        <v>3658236.7699999996</v>
+        <v>3961869.7699999996</v>
       </c>
     </row>
     <row r="37">
@@ -2432,13 +2432,13 @@
         <v>9.519586687593593</v>
       </c>
       <c r="H37" s="2">
-        <v>11.244420886614023</v>
+        <v>10.889505713606791</v>
       </c>
       <c r="I37" s="2">
-        <v>12.466369781217134</v>
+        <v>12.837217099903263</v>
       </c>
       <c r="J37" s="2">
-        <v>13.740470154145756</v>
+        <v>14.880926728342219</v>
       </c>
     </row>
     <row r="38">
@@ -2468,13 +2468,13 @@
         <v>2.8427467189470645</v>
       </c>
       <c r="H38" s="2">
-        <v>36.14515982150988</v>
+        <v>31.847919133047988</v>
       </c>
       <c r="I38" s="2">
-        <v>27.805557599391694</v>
+        <v>35.896898928183106</v>
       </c>
       <c r="J38" s="2">
-        <v>27.6399761930914</v>
+        <v>34.2407032546614</v>
       </c>
     </row>
   </sheetData>
@@ -2740,13 +2740,13 @@
         <v>2998121</v>
       </c>
       <c r="H6" s="4">
-        <v>3715418</v>
+        <v>3658685</v>
       </c>
       <c r="I6" s="4">
-        <v>4602592</v>
+        <v>4672923</v>
       </c>
       <c r="J6" s="4">
-        <v>5700296</v>
+        <v>5956346</v>
       </c>
     </row>
     <row r="7">
@@ -2774,13 +2774,13 @@
         <v>31.99999701146179</v>
       </c>
       <c r="H7" s="2">
-        <v>32.50482902677493</v>
+        <v>32.00849282310255</v>
       </c>
       <c r="I7" s="2">
-        <v>33.00517889489181</v>
+        <v>33.50952236849465</v>
       </c>
       <c r="J7" s="2">
-        <v>33.50552318685166</v>
+        <v>35.01054840168144</v>
       </c>
     </row>
     <row r="8">
@@ -2808,13 +2808,13 @@
         <v>841473</v>
       </c>
       <c r="H8" s="4">
-        <v>1297205</v>
+        <v>1240472</v>
       </c>
       <c r="I8" s="4">
-        <v>1854476.83</v>
+        <v>1924807.83</v>
       </c>
       <c r="J8" s="4">
-        <v>2575001.0199999996</v>
+        <v>2831051.0199999996</v>
       </c>
     </row>
     <row r="9">
@@ -2842,13 +2842,13 @@
         <v>8.981336472152321</v>
       </c>
       <c r="H9" s="2">
-        <v>11.348770646446125</v>
+        <v>10.852434442773747</v>
       </c>
       <c r="I9" s="2">
-        <v>13.298449988741535</v>
+        <v>13.802793462344374</v>
       </c>
       <c r="J9" s="2">
-        <v>15.135487066246501</v>
+        <v>16.640512281076283</v>
       </c>
     </row>
     <row r="10">
@@ -3046,13 +3046,13 @@
         <v>1830134</v>
       </c>
       <c r="H15" s="4">
-        <v>2336568</v>
+        <v>2279835</v>
       </c>
       <c r="I15" s="4">
-        <v>2979051</v>
+        <v>3049382</v>
       </c>
       <c r="J15" s="4">
-        <v>3793554.9999999995</v>
+        <v>4049604.9999999995</v>
       </c>
     </row>
     <row r="16">
@@ -3082,13 +3082,13 @@
         <v>5.251552921839475</v>
       </c>
       <c r="H16" s="2">
-        <v>27.671962818023154</v>
+        <v>24.57202587351528</v>
       </c>
       <c r="I16" s="2">
-        <v>27.496867200098606</v>
+        <v>33.75450416367851</v>
       </c>
       <c r="J16" s="2">
-        <v>27.34105592687066</v>
+        <v>32.80084292489427</v>
       </c>
     </row>
     <row r="17">
@@ -3324,13 +3324,13 @@
         <v>15509.610169491525</v>
       </c>
       <c r="H23" s="2">
-        <v>19471.4</v>
+        <v>18998.625</v>
       </c>
       <c r="I23" s="2">
-        <v>24219.926829268294</v>
+        <v>24791.72357723577</v>
       </c>
       <c r="J23" s="2">
-        <v>30348.439999999995</v>
+        <v>32396.839999999997</v>
       </c>
     </row>
     <row r="24">
@@ -3720,17 +3720,17 @@
       </c>
       <c r="J5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 67.36 % / 補助 67.5 % / ベース 67.17 %</t>
+          <t xml:space="preserve">全社 67.71 % / 補助 67.99 % / ベース 67.34 %</t>
         </is>
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 67 % / 補助 66.99 % / ベース 67.01 %</t>
+          <t xml:space="preserve">全社 66.63 % / 補助 66.49 % / ベース 66.84 %</t>
         </is>
       </c>
       <c r="L5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 66.62 % / 補助 66.49 % / ベース 66.84 %</t>
+          <t xml:space="preserve">全社 65.48 % / 補助 64.99 % / ベース 66.34 %</t>
         </is>
       </c>
     </row>
@@ -3782,17 +3782,17 @@
       </c>
       <c r="J6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32.64 % / 補助 32.5 % / ベース 32.83 %</t>
+          <t xml:space="preserve">全社 32.29 % / 補助 32.01 % / ベース 32.66 %</t>
         </is>
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 33 % / 補助 33.01 % / ベース 32.99 %</t>
+          <t xml:space="preserve">全社 33.37 % / 補助 33.51 % / ベース 33.16 %</t>
         </is>
       </c>
       <c r="L6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 33.38 % / 補助 33.51 % / ベース 33.16 %</t>
+          <t xml:space="preserve">全社 34.52 % / 補助 35.01 % / ベース 33.66 %</t>
         </is>
       </c>
     </row>
@@ -3906,17 +3906,17 @@
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.49 % / 補助 11.35 % / ベース 6.99 %</t>
+          <t xml:space="preserve">全社 9.13 % / 補助 10.85 % / ベース 6.83 %</t>
         </is>
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.94 % / 補助 13.3 % / ベース 7.31 %</t>
+          <t xml:space="preserve">全社 11.31 % / 補助 13.8 % / ベース 7.48 %</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.43 % / 補助 15.14 % / ベース 7.63 %</t>
+          <t xml:space="preserve">全社 13.57 % / 補助 16.64 % / ベース 8.12 %</t>
         </is>
       </c>
     </row>
@@ -3968,17 +3968,17 @@
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.24 % / 補助 13.1 % / ベース 8.75 %</t>
+          <t xml:space="preserve">全社 10.89 % / 補助 12.6 % / ベース 8.59 %</t>
         </is>
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.47 % / 補助 14.73 % / ベース 8.97 %</t>
+          <t xml:space="preserve">全社 12.84 % / 補助 15.24 % / ベース 9.14 %</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.74 % / 補助 16.31 % / ベース 9.19 %</t>
+          <t xml:space="preserve">全社 14.88 % / 補助 17.82 % / ベース 9.69 %</t>
         </is>
       </c>
     </row>
@@ -4526,17 +4526,17 @@
       </c>
       <c r="J18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 46.33 % / 補助 35.92 % / ベース 59.53 %</t>
+          <t xml:space="preserve">全社 47.13 % / 補助 36.82 % / ベース 59.99 %</t>
         </is>
       </c>
       <c r="K18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 42.26 % / 補助 31.04 % / ベース 59.11 %</t>
+          <t xml:space="preserve">全社 41.55 % / 補助 30.32 % / ベース 58.67 %</t>
         </is>
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 38.33 % / 補助 26.85 % / ベース 58.7 %</t>
+          <t xml:space="preserve">全社 36.47 % / 補助 25.15 % / ベース 57.42 %</t>
         </is>
       </c>
     </row>
@@ -4712,17 +4712,17 @@
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6,983.45 千円/人 / 補助 10,993.26 千円/人 / ベース 3,890.92 千円/人</t>
+          <t xml:space="preserve">全社 6,722.26 千円/人 / 補助 10,512.47 千円/人 / ベース 3,799.09 千円/人</t>
         </is>
       </c>
       <c r="K21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8,953.95 千円/人 / 補助 15,326.25 千円/人 / ベース 4,134.89 千円/人</t>
+          <t xml:space="preserve">全社 9,257.36 千円/人 / 補助 15,907.5 千円/人 / ベース 4,228.19 千円/人</t>
         </is>
       </c>
       <c r="L21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11,368.51 千円/人 / 補助 20,934.97 千円/人 / ベース 4,364.5 千円/人</t>
+          <t xml:space="preserve">全社 12,411.92 千円/人 / 補助 23,016.67 千円/人 / ベース 4,647.73 千円/人</t>
         </is>
       </c>
     </row>
@@ -4774,17 +4774,17 @@
       </c>
       <c r="J22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15,138.69 千円/人 / 補助 19,471.4 千円/人 / ベース 11,805.84 千円/人</t>
+          <t xml:space="preserve">全社 14,882.24 千円/人 / 補助 18,998.63 千円/人 / ベース 11,715.78 千円/人</t>
         </is>
       </c>
       <c r="K22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 17,356.14 千円/人 / 補助 24,219.93 千円/人 / ベース 12,176.72 千円/人</t>
+          <t xml:space="preserve">全社 17,654.25 千円/人 / 補助 24,791.72 千円/人 / ベース 12,268.3 千円/人</t>
         </is>
       </c>
       <c r="L22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 20,041.44 千円/人 / 補助 30,348.44 千円/人 / ベース 12,507.08 千円/人</t>
+          <t xml:space="preserve">全社 21,067.23 千円/人 / 補助 32,396.84 千円/人 / ベース 12,785.34 千円/人</t>
         </is>
       </c>
     </row>
@@ -5208,17 +5208,17 @@
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.41 倍 / 補助 7.49 倍 / ベース 4.97 倍</t>
+          <t xml:space="preserve">全社 6.2 倍 / 補助 7.2 倍 / ベース 4.88 倍</t>
         </is>
       </c>
       <c r="K29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.19 倍 / 補助 10.27 倍 / ベース 5.41 倍</t>
+          <t xml:space="preserve">全社 8.43 倍 / 補助 10.62 倍 / ベース 5.51 倍</t>
         </is>
       </c>
       <c r="L29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.45 倍 / 補助 13.88 倍 / ベース 5.89 倍</t>
+          <t xml:space="preserve">全社 11.32 倍 / 補助 15.16 倍 / ベース 6.21 倍</t>
         </is>
       </c>
     </row>
@@ -5518,17 +5518,17 @@
       </c>
       <c r="J34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 0.33 pt</t>
+          <t xml:space="preserve">差 0.66 pt</t>
         </is>
       </c>
       <c r="K34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -0.01 pt</t>
+          <t xml:space="preserve">差 -0.35 pt</t>
         </is>
       </c>
       <c r="L34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -0.35 pt</t>
+          <t xml:space="preserve">差 -1.36 pt</t>
         </is>
       </c>
     </row>
@@ -5580,17 +5580,17 @@
       </c>
       <c r="J35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 4.36 pt</t>
+          <t xml:space="preserve">差 4.02 pt</t>
         </is>
       </c>
       <c r="K35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 5.98 pt</t>
+          <t xml:space="preserve">差 6.32 pt</t>
         </is>
       </c>
       <c r="L35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 7.51 pt</t>
+          <t xml:space="preserve">差 8.52 pt</t>
         </is>
       </c>
     </row>
@@ -5766,17 +5766,17 @@
       </c>
       <c r="J38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 76.55 %</t>
+          <t xml:space="preserve">寄与率 76.06 %</t>
         </is>
       </c>
       <c r="K38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 89.37 %</t>
+          <t xml:space="preserve">寄与率 87.78 %</t>
         </is>
       </c>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 90.95 %</t>
+          <t xml:space="preserve">寄与率 89.68 %</t>
         </is>
       </c>
     </row>
@@ -5878,7 +5878,7 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 原価率</t>
+          <t xml:space="preserve">補助事業 原価率（基準年後初年度）</t>
         </is>
       </c>
       <c r="B4" s="2">
@@ -5899,7 +5899,7 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 原価率</t>
+          <t xml:space="preserve">ベース事業 原価率（基準年後初年度）</t>
         </is>
       </c>
       <c r="B5" s="2">
@@ -5920,7 +5920,7 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 原価率（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 原価率（設備導入期間初年度）</t>
         </is>
       </c>
       <c r="B6" s="2">
@@ -5941,7 +5941,7 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 原価率（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 原価率（設備導入期間初年度）</t>
         </is>
       </c>
       <c r="B7" s="2">
@@ -6308,7 +6308,7 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 原価率改善ポイント（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 原価率 年当たり改善ポイント（設備導入期間）</t>
         </is>
       </c>
       <c r="B22" s="2">
@@ -6434,7 +6434,7 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 原価率改善ポイント（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 原価率 年当たり改善ポイント（設備導入期間）</t>
         </is>
       </c>
       <c r="B28" s="2">
@@ -6585,7 +6585,7 @@
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 原価率改善ポイント（基準年度後）</t>
+          <t xml:space="preserve">補助事業 原価率 年当たり改善ポイント（基準年後）</t>
         </is>
       </c>
       <c r="B35" s="2">
@@ -6606,7 +6606,7 @@
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 原価率改善ポイント（基準年度後）</t>
+          <t xml:space="preserve">ベース事業 原価率 年当たり改善ポイント（基準年後）</t>
         </is>
       </c>
       <c r="B36" s="2">
@@ -11401,7 +11401,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsIm1vbmV5VW5pdCI6IuWNg+WGhiIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MjAwMDAwLCJjb2dzIjo0ODk2MDAwLCJlbXBsb3llZVBheSI6NTE5MDMxLCJvZmZpY2VyUGF5IjozNjAwMCwiZGVwcmVjaWF0aW9uIjoxODAwMDAsIm90aGVyU2dhIjo5MDAwMDAsImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQ5MzA3OSwiZW1wbG95ZWVCb251cyI6MjU5NTIsIm9mZmljZXJDb21wZW5zYXRpb24iOjMyNDAwLCJvZmZpY2VyQm9udXMiOjM2MDAsImNvZ3NEZXByZWNpYXRpb24iOjQ1MDAwLCJzZ2FEZXByZWNpYXRpb24iOjEzNTAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6MzYwMDB9LCJvdGhlciI6eyJzYWxlcyI6NjQ0MDAwMCwiY29ncyI6NDM3OTIwMCwiZW1wbG95ZWVQYXkiOjcwOTc4Niwib2ZmaWNlclBheSI6NTUyMDAsImRlcHJlY2lhdGlvbiI6MTM4MDAwLCJvdGhlclNnYSI6NzM2MDAwLCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Njc0Mjk3LCJlbXBsb3llZUJvbnVzIjozNTQ4OSwib2ZmaWNlckNvbXBlbnNhdGlvbiI6NDk2ODAsIm9mZmljZXJCb251cyI6NTUyMCwiY29nc0RlcHJlY2lhdGlvbiI6Mjc2MDAsInNnYURlcHJlY2lhdGlvbiI6MTEwNDAwLCJyZXNlYXJjaERldmVsb3BtZW50IjoyNzYwMCwib3JkaW5hcnlJbmNvbWUiOjM5NDUzNCwicHJlVGF4SW5jb21lIjozOTQ1MzQsIm5ldEluY29tZSI6NzUwNzUyLjF9fSx7InllYXIiOjIwMjQsInJvbGUiOiJwcmV2aW91cyIsInByb2plY3QiOnsic2FsZXMiOjc2MDAwMDAsImNvZ3MiOjUxNjgwMDAsImVtcGxveWVlUGF5Ijo1NTg4MjQsIm9mZmljZXJQYXkiOjM4MDAwLCJkZXByZWNpYXRpb24iOjE5MDAwMCwib3RoZXJTZ2EiOjk1MDAwMCwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NTMwODgzLCJlbXBsb3llZUJvbnVzIjoyNzk0MSwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MzQyMDAsIm9mZmljZXJCb251cyI6MzgwMCwiY29nc0RlcHJlY2lhdGlvbiI6NDc1MDAsInNnYURlcHJlY2lhdGlvbiI6MTQyNTAwLCJyZXNlYXJjaERldmVsb3BtZW50IjozODAwMH0sIm90aGVyIjp7InNhbGVzIjo2NzIwMDAwLCJjb2dzIjo0NTY5NjAwLCJlbXBsb3llZVBheSI6NzU0MTQ4LCJvZmZpY2VyUGF5Ijo1NzYwMCwiZGVwcmVjaWF0aW9uIjoxNDQwMDAsIm90aGVyU2dhIjo3NjgwMDAsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3MTY0NDEsImVtcGxveWVlQm9udXMiOjM3NzA3LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjo1MTg0MCwib2ZmaWNlckJvbnVzIjo1NzYwLCJjb2dzRGVwcmVjaWF0aW9uIjoyODgwMCwic2dhRGVwcmVjaWF0aW9uIjoxMTUyMDAsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjI4ODAwLCJvcmRpbmFyeUluY29tZSI6Mzk4MDEyLCJwcmVUYXhJbmNvbWUiOjM5ODAxMiwibmV0SW5jb21lIjo3NzE4ODEuNn19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwMDAwMDAsImNvZ3MiOjU0NDAwMDAsImVtcGxveWVlUGF5Ijo2MDAwMDAsImVtcGxveWVlU2FsYXJ5Ijo1NzAwMDAsImVtcGxveWVlQm9udXMiOjMwMDAwLCJvZmZpY2VyUGF5Ijo0MDAwMCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MzYwMDAsIm9mZmljZXJCb251cyI6NDAwMCwiZGVwcmVjaWF0aW9uIjoyMDAwMDAsImNvZ3NEZXByZWNpYXRpb24iOjUwMDAwLCJzZ2FEZXByZWNpYXRpb24iOjE1MDAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6NDAwMDAsIm90aGVyU2dhIjoxMDAwMDAwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwMDAwMDAsImNvZ3MiOjQ3NjAwMDAsImVtcGxveWVlUGF5Ijo4MDAwMDAsImVtcGxveWVlU2FsYXJ5Ijo3NjAwMDAsImVtcGxveWVlQm9udXMiOjQwMDAwLCJvZmZpY2VyUGF5Ijo2MDAwMCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6NTQwMDAsIm9mZmljZXJCb251cyI6NjAwMCwiZGVwcmVjaWF0aW9uIjoxNTAwMDAsImNvZ3NEZXByZWNpYXRpb24iOjMwMDAwLCJzZ2FEZXByZWNpYXRpb24iOjEyMDAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6MzAwMDAsIm90aGVyU2dhIjo4MDAwMDAsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjo0MDAwMDAsInByZVRheEluY29tZSI6NDAwMDAwLCJuZXRJbmNvbWUiOjc5MTAwMH19XSwiYmFsYW5jZVNoZWV0cyI6W3sieWVhciI6MjAyMywiYXNzZXRzIjoxMzIwMDAwMCwiY3VycmVudEFzc2V0cyI6NjcwMDAwMCwiY2FzaCI6MjQwMDAwMCwiZml4ZWRBc3NldHMiOjY1MDAwMDAsInRhbmdpYmxlQXNzZXRzIjo1MzAwMDAwLCJidWlsZGluZ3MiOjE5MDAwMDAsIm1hY2hpbmVyeSI6MjQwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6NzAwMDAwLCJzb2Z0d2FyZSI6NTAwMDAwLCJsaWFiaWxpdGllcyI6NzUwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjozOTAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjozNjAwMDAwLCJsb25nVGVybURlYnQiOjI5MDAwMDAsIm5ldEFzc2V0cyI6NTcwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjU0MDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4Ijo1MDAwMDB9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMwMDAwMCwiY3VycmVudEFzc2V0cyI6NzIwMDAwMCwiY2FzaCI6MjUwMDAwMCwiZml4ZWRBc3NldHMiOjcxMDAwMDAsInRhbmdpYmxlQXNzZXRzIjo1ODAwMDAwLCJidWlsZGluZ3MiOjIwMDAwMDAsIm1hY2hpbmVyeSI6MjgwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6ODAwMDAwLCJzb2Z0d2FyZSI6NjAwMDAwLCJsaWFiaWxpdGllcyI6NzkwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjo0MTAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjozODAwMDAwLCJsb25nVGVybURlYnQiOjMxMDAwMDAsIm5ldEFzc2V0cyI6NjQwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjYxMDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4Ijo4MDAwMDB9LHsieWVhciI6MjAyNSwiYXNzZXRzIjoxNTYwMDAwMCwiY3VycmVudEFzc2V0cyI6NzgwMDAwMCwiY2FzaCI6MjcwMDAwMCwiZml4ZWRBc3NldHMiOjc4MDAwMDAsInRhbmdpYmxlQXNzZXRzIjo2NDAwMDAwLCJidWlsZGluZ3MiOjIyMDAwMDAsIm1hY2hpbmVyeSI6MzIwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6OTAwMDAwLCJzb2Z0d2FyZSI6NzAwMDAwLCJsaWFiaWxpdGllcyI6ODMwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjo0MzAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMTAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjo0MDAwMDAwLCJsb25nVGVybURlYnQiOjMyMDAwMDAsIm5ldEFzc2V0cyI6NzMwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjcwMDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4IjoxMDAwMDAwfV0sImZ1dHVyZUNhcGV4IjpbeyJ5ZWFyIjoyMDI2LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI4LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI5LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMwLCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMxLCJ2YWx1ZSI6MH1dLCJkcml2ZXJzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsInByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJwcm9qZWN0Q29nc1JhdGVUb0Jhc2UiOjAuNjgsIm90aGVyQ29nc1JhdGVUb0Jhc2UiOjAuNjgsInByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwib3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwicHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yNSwib3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMiwicHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsInByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJvdGhlck5vbk9wZXJhdGluZ1JhdGUiOi0wLjAwNSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjowLCJlZmZlY3RpdmVUYXhSYXRlIjowLjMsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdEZpcnN0WWVhclNhbGVzIjowLCJwcm9qZWN0QmFzZVllYXJTYWxlcyI6MCwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6NS41NTExMTUxMjMxMjU3ODNlLTE3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5Nywib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI1NzI0NjM3NjgxMTU4NTQsIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wMTUsIm90aGVyU2dhUmF0ZUVuZCI6MC4wMDUsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJpbnZlc3RtZW50IjoyMzAwMDAwLCJzdWJzaWR5Ijo3NjYwMDAsImxvY2FsQmVuY2htYXJrIjoyM30sImRyaXZlclJhbmdlcyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjpbLTAuMDUsMC4zXSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6WzAuNjYsMC43XSwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOlswLjY2LDAuN10sInByb2plY3RDb2dzUmF0ZVRvQmFzZSI6WzAuNjgsMC42OF0sIm90aGVyQ29nc1JhdGVUb0Jhc2UiOlswLjY4LDAuNjhdLCJwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOlswLDFdLCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOlswLDFdLCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOlstMC41LDAuNV0sIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6Wy0wLjUsMC41XSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJlZmZlY3RpdmVUYXhSYXRlIjpbMCwwLjZdLCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwicHJvamVjdEZpcnN0WWVhclNhbGVzIjpbMCwxMDAwMDAwMDAwMF0sInByb2plY3RCYXNlWWVhclNhbGVzIjpbMCwxMDAwMDAwMDAwMF0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDEuNjY1MzM0NTM2OTM3NzM0OGUtMTZdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkzMjUzMzA1MDE4NDY5MjcsMC4wMjA3MzU5OTQxODMxODkxNjZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlswLjA0MDc2MDg2OTU2NTIxNzE4NCwwLjA0NDM4NDA1Nzk3MTAxNDUyXSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDAwMTM0NTc1NTY5MzU4MTk3MzddLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MTM5NDU3MDIzNzE3NDQzLDAuMDIwNTUzNDU5OTE0NzYzMDk1XSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjAzOTE2NjY2NjY2NjY2NjY4LDAuMDQyNTAwMDAwMDAwMDAwMDldLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbMC4xNSwwLjNdLCJvdGhlclNhbGVzR3Jvd3RoIjpbMC4wNjA3NjA4Njk1NjUyMTcxOSwwLjA2NDM4NDA1Nzk3MTAxNDUzXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMC4wMDUsMC4wMDUxMzQ1NzU1NjkzNTgxOTc1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLjAyNDEzOTQ1NzAyMzcxNzQ0NCwwLjAyNTU1MzQ1OTkxNDc2MzA5Nl0sIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6WzAsMC4wOF0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6WzAuMDQ0MTY2NjY2NjY2NjY2NjgsMC4wNDc1MDAwMDAwMDAwMDAwOV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMCwwLjAzXSwib3RoZXJTZ2FSYXRlRW5kIjpbMCwwLjAxXSwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOlswLjA0MjYzMTU3ODk0NzM2ODM2LDAuMDY1NTU1NTU1NTU1NTU1NThdLCJpbnZlc3RtZW50IjpbMTUwMDAwMCwyMDAwMDAwMF0sInN1YnNpZHkiOlsxMDAwMDAsNTAwMDAwMF0sImxvY2FsQmVuY2htYXJrIjpbMCwxMDBdfSwidGFyZ2V0cyI6eyJjb21wYW55U2FsZXNDYWdyIjp7InZhbHVlIjoxNSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo4MjQwMDAwLCJtYXgiOjI1MjY5MDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjoyLCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NjAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo3NDgwMDAwLCJtYXgiOjEzNjg0MDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MTg3ODAwMCwibWF4IjozMzQzMDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6Mjg1MDAwLCJtYXgiOjM3NDAwMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjoxNSwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX19LCJmb3JlY2FzdE92ZXJyaWRlcyI6eyIyMDI5Om90aGVyOnNhbGVzIjo4NTEzMDAwLCIyMDI5OnByb2plY3Q6Ny04Ijo3OTAwMDB9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2NDAwMDAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mjc1MjAwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6NzI2MDAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi03IjozMjY1MDE3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6ODIwODAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMCI6OTEyMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEyIjoxMTY3Mzc2LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjYxNDQxLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTQiOjI0NTQwMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1Ijo2MzYwMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE4IjoxMDcyNTAzLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTkiOjEwNzI1MDMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yMCI6NzUwNzUyLjEsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yNyI6MjEwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xIjo3MjAwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNCI6MjMwNDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjY3Nzk2OSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTgiOjUxOTAzMSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTkiOjM2MDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOlAyLTQiOjQ1MDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOlAyLTE0IjoxMzUwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMyI6OTAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEiOjE0MzIwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMyI6OTczNzYwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTQiOjc2MzAwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItNyI6MzQ1MTA3MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTkiOjg2MDQwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTAiOjk1NjAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMiI6MTI0NzMyNCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEzIjo2NTY0OCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjoyNTc3MDAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNSI6NjY4MDAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xOCI6MTEwMjY4OCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE5IjoxMTAyNjg4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjAiOjc3MTg4MS42LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjciOjIyMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMSI6NzYwMDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0MzIwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny02Ijo3MDQ2NzYsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny04Ijo1NTg4MjQsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjozODAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDpQMi00Ijo0NzUwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDpQMi0xNCI6MTQyNTAwLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTMiOjk1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xIjoxNTAwMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTMiOjEwMjAwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6ODAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi03IjozNjQwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItOSI6OTAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMCI6MTAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMzMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjo3MDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE0IjoyNzAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNSI6NzAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xOCI6MTEzMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE5IjoxMTMwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjAiOjc5MTAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI3IjoyMzAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwMDAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNTYwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6NzMwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NjAwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOSI6NDAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6UDItNCI6NTAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6UDItMTQiOjE1MDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FzaCI6MjQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpidWlsZGluZ3MiOjE5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6aW50YW5naWJsZUFzc2V0cyI6NzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudExpYWJpbGl0aWVzIjozOTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpsb25nVGVybURlYnQiOjI5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGl0YWwiOjEwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRBc3NldHMiOjcyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDp0YW5naWJsZUFzc2V0cyI6NTgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmxhbmQiOjEwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGlhYmlsaXRpZXMiOjc5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRMaWFiaWxpdGllcyI6MzgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OnNoYXJlaG9sZGVyRXF1aXR5Ijo2MTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTphc3NldHMiOjE1NjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZEFzc2V0cyI6NzgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bWFjaGluZXJ5IjozMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjkwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OnNvZnR3YXJlIjo3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OnNob3J0VGVybURlYnQiOjExMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bmV0QXNzZXRzIjo3MzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwZXgiOjEwMDAwMDAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MC42NiwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC43LCJkcml2ZXI6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybzowIjowLjY2LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC43LCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlVG9CYXNlIjowLjY4LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NSYXRlVG9CYXNlOjAiOjAuNjgsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc1JhdGVUb0Jhc2U6MSI6MC42OCwiZHJpdmVyOm90aGVyQ29nc1JhdGVUb0Jhc2UiOjAuNjgsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlVG9CYXNlOjAiOjAuNjgsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlVG9CYXNlOjEiOjAuNjgsImRyaXZlcjpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwiZHJpdmVyLXJhbmdlOnByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZToxIjoxLCJkcml2ZXI6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJkcml2ZXItcmFuZ2U6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjowLjksImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGU6MSI6MC4zLCJkcml2ZXI6b3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjEiOjAuMywiZHJpdmVyOnByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdE5vbk9wZXJhdGluZ1JhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOnByb2plY3ROb25PcGVyYXRpbmdSYXRlOjEiOjAuNSwiZHJpdmVyOm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJOb25PcGVyYXRpbmdSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpvdGhlck5vbk9wZXJhdGluZ1JhdGU6MSI6MC41LCJkcml2ZXI6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6b3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6ZWZmZWN0aXZlVGF4UmF0ZSI6MC4zLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZTowIjowLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZToxIjowLjYsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RGaXJzdFllYXJTYWxlcyI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RGaXJzdFllYXJTYWxlczowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEZpcnN0WWVhclNhbGVzOjEiOjEwMDAwMDAwMDAwLCJkcml2ZXI6cHJvamVjdEJhc2VZZWFyU2FsZXMiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0QmFzZVllYXJTYWxlczowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEJhc2VZZWFyU2FsZXM6MSI6MTAwMDAwMDAwMDAsImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjEuNjY1MzM0NTM2OTM3NzM0OGUtMTYsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkzMjUzMzA1MDE4NDY5MjcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNzM1OTk0MTgzMTg5MTY2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLjAxOTEzOTQ1NzAyMzcxNzQ0MywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNTUzNDU5OTE0NzYzMDk1LCJkcml2ZXI6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wMzkxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDQyNTAwMDAwMDAwMDAwMDksImRyaXZlcjpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjAiOjAuMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MSI6MC4zLCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NzI0NjM3NjgxMTU4NiwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MCI6MC4wNjA3NjA4Njk1NjUyMTcxOSwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MSI6MC4wNjQzODQwNTc5NzEwMTQ1MywiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZToxIjowLjAzLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDoxIjowLjAwNTEzNDU3NTU2OTM1ODE5NzUsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDowIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDoxIjowLjEsImRyaXZlcjpvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjAiOjAuMDI0MTM5NDU3MDIzNzE3NDQ0LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wMjU1NTM0NTk5MTQ3NjMwOTYsImRyaXZlcjpvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGg6MSI6MC4wOCwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjowLjA0NDE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MSI6MC4wNDc1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjAxNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDoxIjowLjAzLCJkcml2ZXI6b3RoZXJTZ2FSYXRlRW5kIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMDEsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAuMDQyNjMxNTc4OTQ3MzY4MzYsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjA2NTU1NTU1NTU1NTU1NTU4LCJkcml2ZXI6aW52ZXN0bWVudCI6MjMwMDAwMCwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUwMDAwMCwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MSI6MjAwMDAwMDAsImRyaXZlcjpzdWJzaWR5Ijo3NjYwMDAsImRyaXZlci1yYW5nZTpzdWJzaWR5OjAiOjEwMDAwMCwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MSI6NTAwMDAwMCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoxNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjo4MjQwMDAwLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjoyLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOm1heCI6NywidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOnZhbHVlIjo2MCwidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOm1heCI6OTUsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOnZhbHVlIjoyMiwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOnZhbHVlIjo3NDgwMDAwLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOnZhbHVlIjoyMSwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2FncjptYXgiOjM1LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOnZhbHVlIjoxODc4MDAwLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOnZhbHVlIjo3LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOm1heCI6MTAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOnZhbHVlIjoyODUwMDAsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MTUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTptYXgiOjI1MjY5MDAwLCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6bWF4IjoxMzY4NDAwMCwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTptYXgiOjMzNDMwMDAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOm1heCI6Mzc0MDAwfSwibWV0cmljR3JvdXBCYXNlcyI6eyJjb21wYW55U2FsZXMiOiJyYXRlIiwicHJvamVjdFNhbGVzIjoicmF0ZSIsImxhYm9yUHJvZHVjdGl2aXR5IjoicmF0ZSIsImVtcGxveWVlUGF5IjoicmF0ZSJ9LCJhcHBsaWNhdGlvbkNhdGVnb3J5IjoiZ2VuZXJhbCIsImFkanVzdGVkRHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY3OTk1NTA3Mjk3OTcwNzksIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4MDAwOTM1MzYzNDAxMzIsInByb2plY3RDb2dzUmF0ZVRvQmFzZSI6MC42OCwib3RoZXJDb2dzUmF0ZVRvQmFzZSI6MC42OCwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA3MDcyMzY4NDIxMDUxLCJwcm9qZWN0Rmlyc3RZZWFyU2FsZXMiOjAsInByb2plY3RCYXNlWWVhclNhbGVzIjowLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjoxLjMzNzU5NjcwMDA2ODM4ODdlLTE2LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDA0NzAwOTU3NDk0MjI0LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1MjE5MjI1ODM4MTk5Mjk4LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA0OTgyMDkxOTA3OTY4Niwib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI2MTYwNTg0NTI3Njc5OCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg2NDI2Njc5MjM0NzY0OCwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA5MzA4MjU0MjAwMTQ2NSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyMDAwMjEzNjI4OTg4NjM4LCJvdGhl</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsIm1vbmV5VW5pdCI6IuWNg+WGhiIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MjAwMDAwLCJjb2dzIjo0ODk2MDAwLCJlbXBsb3llZVBheSI6NTE5MDMxLCJvZmZpY2VyUGF5IjozNjAwMCwiZGVwcmVjaWF0aW9uIjoxODAwMDAsIm90aGVyU2dhIjo5MDAwMDAsImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQ5MzA3OSwiZW1wbG95ZWVCb251cyI6MjU5NTIsIm9mZmljZXJDb21wZW5zYXRpb24iOjMyNDAwLCJvZmZpY2VyQm9udXMiOjM2MDAsImNvZ3NEZXByZWNpYXRpb24iOjQ1MDAwLCJzZ2FEZXByZWNpYXRpb24iOjEzNTAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6MzYwMDB9LCJvdGhlciI6eyJzYWxlcyI6NjQ0MDAwMCwiY29ncyI6NDM3OTIwMCwiZW1wbG95ZWVQYXkiOjcwOTc4Niwib2ZmaWNlclBheSI6NTUyMDAsImRlcHJlY2lhdGlvbiI6MTM4MDAwLCJvdGhlclNnYSI6NzM2MDAwLCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Njc0Mjk3LCJlbXBsb3llZUJvbnVzIjozNTQ4OSwib2ZmaWNlckNvbXBlbnNhdGlvbiI6NDk2ODAsIm9mZmljZXJCb251cyI6NTUyMCwiY29nc0RlcHJlY2lhdGlvbiI6Mjc2MDAsInNnYURlcHJlY2lhdGlvbiI6MTEwNDAwLCJyZXNlYXJjaERldmVsb3BtZW50IjoyNzYwMCwib3JkaW5hcnlJbmNvbWUiOjM5NDUzNCwicHJlVGF4SW5jb21lIjozOTQ1MzQsIm5ldEluY29tZSI6NzUwNzUyLjF9fSx7InllYXIiOjIwMjQsInJvbGUiOiJwcmV2aW91cyIsInByb2plY3QiOnsic2FsZXMiOjc2MDAwMDAsImNvZ3MiOjUxNjgwMDAsImVtcGxveWVlUGF5Ijo1NTg4MjQsIm9mZmljZXJQYXkiOjM4MDAwLCJkZXByZWNpYXRpb24iOjE5MDAwMCwib3RoZXJTZ2EiOjk1MDAwMCwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NTMwODgzLCJlbXBsb3llZUJvbnVzIjoyNzk0MSwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MzQyMDAsIm9mZmljZXJCb251cyI6MzgwMCwiY29nc0RlcHJlY2lhdGlvbiI6NDc1MDAsInNnYURlcHJlY2lhdGlvbiI6MTQyNTAwLCJyZXNlYXJjaERldmVsb3BtZW50IjozODAwMH0sIm90aGVyIjp7InNhbGVzIjo2NzIwMDAwLCJjb2dzIjo0NTY5NjAwLCJlbXBsb3llZVBheSI6NzU0MTQ4LCJvZmZpY2VyUGF5Ijo1NzYwMCwiZGVwcmVjaWF0aW9uIjoxNDQwMDAsIm90aGVyU2dhIjo3NjgwMDAsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3MTY0NDEsImVtcGxveWVlQm9udXMiOjM3NzA3LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjo1MTg0MCwib2ZmaWNlckJvbnVzIjo1NzYwLCJjb2dzRGVwcmVjaWF0aW9uIjoyODgwMCwic2dhRGVwcmVjaWF0aW9uIjoxMTUyMDAsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjI4ODAwLCJvcmRpbmFyeUluY29tZSI6Mzk4MDEyLCJwcmVUYXhJbmNvbWUiOjM5ODAxMiwibmV0SW5jb21lIjo3NzE4ODEuNn19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwMDAwMDAsImNvZ3MiOjU0NDAwMDAsImVtcGxveWVlUGF5Ijo2MDAwMDAsImVtcGxveWVlU2FsYXJ5Ijo1NzAwMDAsImVtcGxveWVlQm9udXMiOjMwMDAwLCJvZmZpY2VyUGF5Ijo0MDAwMCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MzYwMDAsIm9mZmljZXJCb251cyI6NDAwMCwiZGVwcmVjaWF0aW9uIjoyMDAwMDAsImNvZ3NEZXByZWNpYXRpb24iOjUwMDAwLCJzZ2FEZXByZWNpYXRpb24iOjE1MDAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6NDAwMDAsIm90aGVyU2dhIjoxMDAwMDAwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwMDAwMDAsImNvZ3MiOjQ3NjAwMDAsImVtcGxveWVlUGF5Ijo4MDAwMDAsImVtcGxveWVlU2FsYXJ5Ijo3NjAwMDAsImVtcGxveWVlQm9udXMiOjQwMDAwLCJvZmZpY2VyUGF5Ijo2MDAwMCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6NTQwMDAsIm9mZmljZXJCb251cyI6NjAwMCwiZGVwcmVjaWF0aW9uIjoxNTAwMDAsImNvZ3NEZXByZWNpYXRpb24iOjMwMDAwLCJzZ2FEZXByZWNpYXRpb24iOjEyMDAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6MzAwMDAsIm90aGVyU2dhIjo4MDAwMDAsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjo0MDAwMDAsInByZVRheEluY29tZSI6NDAwMDAwLCJuZXRJbmNvbWUiOjc5MTAwMH19XSwiYmFsYW5jZVNoZWV0cyI6W3sieWVhciI6MjAyMywiYXNzZXRzIjoxMzIwMDAwMCwiY3VycmVudEFzc2V0cyI6NjcwMDAwMCwiY2FzaCI6MjQwMDAwMCwiZml4ZWRBc3NldHMiOjY1MDAwMDAsInRhbmdpYmxlQXNzZXRzIjo1MzAwMDAwLCJidWlsZGluZ3MiOjE5MDAwMDAsIm1hY2hpbmVyeSI6MjQwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6NzAwMDAwLCJzb2Z0d2FyZSI6NTAwMDAwLCJsaWFiaWxpdGllcyI6NzUwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjozOTAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjozNjAwMDAwLCJsb25nVGVybURlYnQiOjI5MDAwMDAsIm5ldEFzc2V0cyI6NTcwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjU0MDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4Ijo1MDAwMDB9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMwMDAwMCwiY3VycmVudEFzc2V0cyI6NzIwMDAwMCwiY2FzaCI6MjUwMDAwMCwiZml4ZWRBc3NldHMiOjcxMDAwMDAsInRhbmdpYmxlQXNzZXRzIjo1ODAwMDAwLCJidWlsZGluZ3MiOjIwMDAwMDAsIm1hY2hpbmVyeSI6MjgwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6ODAwMDAwLCJzb2Z0d2FyZSI6NjAwMDAwLCJsaWFiaWxpdGllcyI6NzkwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjo0MTAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjozODAwMDAwLCJsb25nVGVybURlYnQiOjMxMDAwMDAsIm5ldEFzc2V0cyI6NjQwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjYxMDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4Ijo4MDAwMDB9LHsieWVhciI6MjAyNSwiYXNzZXRzIjoxNTYwMDAwMCwiY3VycmVudEFzc2V0cyI6NzgwMDAwMCwiY2FzaCI6MjcwMDAwMCwiZml4ZWRBc3NldHMiOjc4MDAwMDAsInRhbmdpYmxlQXNzZXRzIjo2NDAwMDAwLCJidWlsZGluZ3MiOjIyMDAwMDAsIm1hY2hpbmVyeSI6MzIwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6OTAwMDAwLCJzb2Z0d2FyZSI6NzAwMDAwLCJsaWFiaWxpdGllcyI6ODMwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjo0MzAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMTAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjo0MDAwMDAwLCJsb25nVGVybURlYnQiOjMyMDAwMDAsIm5ldEFzc2V0cyI6NzMwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjcwMDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4IjoxMDAwMDAwfV0sImZ1dHVyZUNhcGV4IjpbeyJ5ZWFyIjoyMDI2LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI4LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI5LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMwLCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMxLCJ2YWx1ZSI6MH1dLCJkcml2ZXJzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsInByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJwcm9qZWN0Q29nc1JhdGVUb0Jhc2UiOjAuNjgsIm90aGVyQ29nc1JhdGVUb0Jhc2UiOjAuNjgsInByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwib3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwicHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yNSwib3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMiwicHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsInByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJvdGhlck5vbk9wZXJhdGluZ1JhdGUiOi0wLjAwNSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjowLCJlZmZlY3RpdmVUYXhSYXRlIjowLjMsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdEZpcnN0WWVhclNhbGVzIjowLCJwcm9qZWN0QmFzZVllYXJTYWxlcyI6MCwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6NS41NTExMTUxMjMxMjU3ODNlLTE3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5Nywib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI1NzI0NjM3NjgxMTU4NTQsIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wMTUsIm90aGVyU2dhUmF0ZUVuZCI6MC4wMDUsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJpbnZlc3RtZW50IjoyMzAwMDAwLCJzdWJzaWR5Ijo3NjYwMDAsImxvY2FsQmVuY2htYXJrIjoyM30sImRyaXZlclJhbmdlcyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjpbLTAuMDUsMC4zXSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6WzAuNjYsMC43XSwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOlswLjY2LDAuN10sInByb2plY3RDb2dzUmF0ZVRvQmFzZSI6WzAuNjgsMC42OF0sIm90aGVyQ29nc1JhdGVUb0Jhc2UiOlswLjY4LDAuNjhdLCJwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOlswLDFdLCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOlswLDFdLCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOlstMC41LDAuNV0sIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6Wy0wLjUsMC41XSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJlZmZlY3RpdmVUYXhSYXRlIjpbMCwwLjZdLCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwicHJvamVjdEZpcnN0WWVhclNhbGVzIjpbMCwxMDAwMDAwMDAwMF0sInByb2plY3RCYXNlWWVhclNhbGVzIjpbMCwxMDAwMDAwMDAwMF0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDEuNjY1MzM0NTM2OTM3NzM0OGUtMTZdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkzMjUzMzA1MDE4NDY5MjcsMC4wMjA3MzU5OTQxODMxODkxNjZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlswLjA0MDc2MDg2OTU2NTIxNzE4NCwwLjA0NDM4NDA1Nzk3MTAxNDUyXSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDAwMTM0NTc1NTY5MzU4MTk3MzddLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MTM5NDU3MDIzNzE3NDQzLDAuMDIwNTUzNDU5OTE0NzYzMDk1XSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjAzOTE2NjY2NjY2NjY2NjY4LDAuMDQyNTAwMDAwMDAwMDAwMDldLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbMC4xNSwwLjNdLCJvdGhlclNhbGVzR3Jvd3RoIjpbMC4wNjA3NjA4Njk1NjUyMTcxOSwwLjA2NDM4NDA1Nzk3MTAxNDUzXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMC4wMDUsMC4wMDUxMzQ1NzU1NjkzNTgxOTc1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLjAyNDEzOTQ1NzAyMzcxNzQ0NCwwLjAyNTU1MzQ1OTkxNDc2MzA5Nl0sIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6WzAsMC4wOF0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6WzAuMDQ0MTY2NjY2NjY2NjY2NjgsMC4wNDc1MDAwMDAwMDAwMDAwOV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMCwwLjAzXSwib3RoZXJTZ2FSYXRlRW5kIjpbMCwwLjAxXSwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOlswLjA0MjYzMTU3ODk0NzM2ODM2LDAuMDY1NTU1NTU1NTU1NTU1NThdLCJpbnZlc3RtZW50IjpbMTUwMDAwMCwyMDAwMDAwMF0sInN1YnNpZHkiOlsxMDAwMDAsNTAwMDAwMF0sImxvY2FsQmVuY2htYXJrIjpbMCwxMDBdfSwidGFyZ2V0cyI6eyJjb21wYW55U2FsZXNDYWdyIjp7InZhbHVlIjoxNSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo4MjQwMDAwLCJtYXgiOjI1MjY5MDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjoyLCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NjAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo3NDgwMDAwLCJtYXgiOjEzNjg0MDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MTg3ODAwMCwibWF4IjozMzQzMDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6Mjg1MDAwLCJtYXgiOjM3NDAwMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjoxNSwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX19LCJmb3JlY2FzdE92ZXJyaWRlcyI6eyIyMDI5Om90aGVyOnNhbGVzIjo4NTEzMDAwLCIyMDI5OnByb2plY3Q6Ny04Ijo3OTAwMDB9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2NDAwMDAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mjc1MjAwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6NzI2MDAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi03IjozMjY1MDE3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6ODIwODAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMCI6OTEyMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEyIjoxMTY3Mzc2LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjYxNDQxLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTQiOjI0NTQwMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1Ijo2MzYwMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE4IjoxMDcyNTAzLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTkiOjEwNzI1MDMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yMCI6NzUwNzUyLjEsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yNyI6MjEwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xIjo3MjAwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNCI6MjMwNDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjY3Nzk2OSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTgiOjUxOTAzMSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTkiOjM2MDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOlAyLTQiOjQ1MDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOlAyLTE0IjoxMzUwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMyI6OTAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEiOjE0MzIwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMyI6OTczNzYwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTQiOjc2MzAwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItNyI6MzQ1MTA3MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTkiOjg2MDQwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTAiOjk1NjAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMiI6MTI0NzMyNCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEzIjo2NTY0OCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjoyNTc3MDAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNSI6NjY4MDAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xOCI6MTEwMjY4OCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE5IjoxMTAyNjg4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjAiOjc3MTg4MS42LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjciOjIyMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMSI6NzYwMDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0MzIwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny02Ijo3MDQ2NzYsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny04Ijo1NTg4MjQsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjozODAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDpQMi00Ijo0NzUwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDpQMi0xNCI6MTQyNTAwLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTMiOjk1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xIjoxNTAwMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTMiOjEwMjAwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6ODAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi03IjozNjQwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItOSI6OTAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMCI6MTAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMzMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjo3MDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE0IjoyNzAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNSI6NzAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xOCI6MTEzMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE5IjoxMTMwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjAiOjc5MTAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI3IjoyMzAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwMDAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNTYwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6NzMwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NjAwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOSI6NDAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6UDItNCI6NTAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6UDItMTQiOjE1MDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FzaCI6MjQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpidWlsZGluZ3MiOjE5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6aW50YW5naWJsZUFzc2V0cyI6NzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudExpYWJpbGl0aWVzIjozOTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpsb25nVGVybURlYnQiOjI5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGl0YWwiOjEwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRBc3NldHMiOjcyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDp0YW5naWJsZUFzc2V0cyI6NTgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmxhbmQiOjEwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGlhYmlsaXRpZXMiOjc5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRMaWFiaWxpdGllcyI6MzgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OnNoYXJlaG9sZGVyRXF1aXR5Ijo2MTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTphc3NldHMiOjE1NjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZEFzc2V0cyI6NzgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bWFjaGluZXJ5IjozMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjkwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OnNvZnR3YXJlIjo3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OnNob3J0VGVybURlYnQiOjExMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bmV0QXNzZXRzIjo3MzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwZXgiOjEwMDAwMDAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MC42NiwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC43LCJkcml2ZXI6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybzowIjowLjY2LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC43LCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlVG9CYXNlIjowLjY4LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NSYXRlVG9CYXNlOjAiOjAuNjgsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc1JhdGVUb0Jhc2U6MSI6MC42OCwiZHJpdmVyOm90aGVyQ29nc1JhdGVUb0Jhc2UiOjAuNjgsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlVG9CYXNlOjAiOjAuNjgsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlVG9CYXNlOjEiOjAuNjgsImRyaXZlcjpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwiZHJpdmVyLXJhbmdlOnByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZToxIjoxLCJkcml2ZXI6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJkcml2ZXItcmFuZ2U6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjowLjksImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGU6MSI6MC4zLCJkcml2ZXI6b3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjEiOjAuMywiZHJpdmVyOnByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdE5vbk9wZXJhdGluZ1JhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOnByb2plY3ROb25PcGVyYXRpbmdSYXRlOjEiOjAuNSwiZHJpdmVyOm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJOb25PcGVyYXRpbmdSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpvdGhlck5vbk9wZXJhdGluZ1JhdGU6MSI6MC41LCJkcml2ZXI6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6b3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6ZWZmZWN0aXZlVGF4UmF0ZSI6MC4zLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZTowIjowLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZToxIjowLjYsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RGaXJzdFllYXJTYWxlcyI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RGaXJzdFllYXJTYWxlczowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEZpcnN0WWVhclNhbGVzOjEiOjEwMDAwMDAwMDAwLCJkcml2ZXI6cHJvamVjdEJhc2VZZWFyU2FsZXMiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0QmFzZVllYXJTYWxlczowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEJhc2VZZWFyU2FsZXM6MSI6MTAwMDAwMDAwMDAsImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjEuNjY1MzM0NTM2OTM3NzM0OGUtMTYsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkzMjUzMzA1MDE4NDY5MjcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNzM1OTk0MTgzMTg5MTY2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLjAxOTEzOTQ1NzAyMzcxNzQ0MywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNTUzNDU5OTE0NzYzMDk1LCJkcml2ZXI6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wMzkxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDQyNTAwMDAwMDAwMDAwMDksImRyaXZlcjpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjAiOjAuMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MSI6MC4zLCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NzI0NjM3NjgxMTU4NiwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MCI6MC4wNjA3NjA4Njk1NjUyMTcxOSwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MSI6MC4wNjQzODQwNTc5NzEwMTQ1MywiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZToxIjowLjAzLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDoxIjowLjAwNTEzNDU3NTU2OTM1ODE5NzUsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDowIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDoxIjowLjEsImRyaXZlcjpvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjAiOjAuMDI0MTM5NDU3MDIzNzE3NDQ0LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wMjU1NTM0NTk5MTQ3NjMwOTYsImRyaXZlcjpvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGg6MSI6MC4wOCwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjowLjA0NDE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MSI6MC4wNDc1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjAxNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDoxIjowLjAzLCJkcml2ZXI6b3RoZXJTZ2FSYXRlRW5kIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMDEsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAuMDQyNjMxNTc4OTQ3MzY4MzYsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjA2NTU1NTU1NTU1NTU1NTU4LCJkcml2ZXI6aW52ZXN0bWVudCI6MjMwMDAwMCwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUwMDAwMCwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MSI6MjAwMDAwMDAsImRyaXZlcjpzdWJzaWR5Ijo3NjYwMDAsImRyaXZlci1yYW5nZTpzdWJzaWR5OjAiOjEwMDAwMCwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MSI6NTAwMDAwMCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoxNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjo4MjQwMDAwLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjoyLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOm1heCI6NywidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOnZhbHVlIjo2MCwidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOm1heCI6OTUsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOnZhbHVlIjoyMiwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOnZhbHVlIjo3NDgwMDAwLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOnZhbHVlIjoyMSwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2FncjptYXgiOjM1LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOnZhbHVlIjoxODc4MDAwLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOnZhbHVlIjo3LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOm1heCI6MTAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOnZhbHVlIjoyODUwMDAsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MTUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTptYXgiOjI1MjY5MDAwLCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6bWF4IjoxMzY4NDAwMCwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTptYXgiOjMzNDMwMDAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOm1heCI6Mzc0MDAwfSwibWV0cmljR3JvdXBCYXNlcyI6eyJjb21wYW55U2FsZXMiOiJyYXRlIiwicHJvamVjdFNhbGVzIjoicmF0ZSIsImxhYm9yUHJvZHVjdGl2aXR5IjoicmF0ZSIsImVtcGxveWVlUGF5IjoicmF0ZSJ9LCJhcHBsaWNhdGlvbkNhdGVnb3J5IjoiZ2VuZXJhbCIsImFkanVzdGVkRHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY3OTkxNTA3Mjk3OTcwODEsIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4MDAwOTM1MzYzNDAxMzIsInByb2plY3RDb2dzUmF0ZVRvQmFzZSI6MC42OCwib3RoZXJDb2dzUmF0ZVRvQmFzZSI6MC42OCwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA3MDcyMzY4NDIxMDUxLCJwcm9qZWN0Rmlyc3RZZWFyU2FsZXMiOjAsInByb2plY3RCYXNlWWVhclNhbGVzIjowLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjoxLjMzNzU5NjcwMDA2ODM4ODdlLTE2LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDA0NzAwOTU3NDk0MjI0LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1MjE5MjI1ODM4MTk5Mjk4LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA0OTgyMDkxOTA3OTY4Niwib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI2MTYwNTg0NTI3Njc5OCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg2NDI2Njc5MjM0NzY0OCwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA5MzA4MjU0MjAwMTQ2NSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyMDAwMjEzNjI4OTg4NjM4LCJvdGhl</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Warn on excessive annual cogs improvements
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -1338,13 +1338,13 @@
         <v>11765868</v>
       </c>
       <c r="H5" s="2">
-        <v>13503917</v>
+        <v>13503580</v>
       </c>
       <c r="I5" s="2">
-        <v>15317999</v>
+        <v>15317641</v>
       </c>
       <c r="J5" s="2">
-        <v>17432946</v>
+        <v>17432565</v>
       </c>
     </row>
     <row r="6">
@@ -1406,13 +1406,13 @@
         <v>5536879</v>
       </c>
       <c r="H7" s="4">
-        <v>6439440</v>
+        <v>6439777</v>
       </c>
       <c r="I7" s="4">
-        <v>7672324.969999999</v>
+        <v>7672682.969999999</v>
       </c>
       <c r="J7" s="4">
-        <v>9190864.75</v>
+        <v>9191245.75</v>
       </c>
     </row>
     <row r="8">
@@ -1440,13 +1440,13 @@
         <v>31.999999768822835</v>
       </c>
       <c r="H8" s="2">
-        <v>32.28864628958906</v>
+        <v>32.29033607531571</v>
       </c>
       <c r="I8" s="2">
-        <v>33.37197414012778</v>
+        <v>33.37353131696647</v>
       </c>
       <c r="J8" s="2">
-        <v>34.52122176011186</v>
+        <v>34.52265280994758</v>
       </c>
     </row>
     <row r="9">
@@ -1780,13 +1780,13 @@
         <v>1297150</v>
       </c>
       <c r="H18" s="4">
-        <v>1821733</v>
+        <v>1822070</v>
       </c>
       <c r="I18" s="4">
-        <v>2601317.799999999</v>
+        <v>2601675.799999999</v>
       </c>
       <c r="J18" s="4">
-        <v>3611869.7699999996</v>
+        <v>3612250.7699999996</v>
       </c>
     </row>
     <row r="19">
@@ -1814,13 +1814,13 @@
         <v>7.496786492919304</v>
       </c>
       <c r="H19" s="2">
-        <v>9.134535374360494</v>
+        <v>9.136225160087141</v>
       </c>
       <c r="I19" s="2">
-        <v>11.314837509007921</v>
+        <v>11.316394685846609</v>
       </c>
       <c r="J19" s="2">
-        <v>13.566314018364181</v>
+        <v>13.5677450681999</v>
       </c>
     </row>
     <row r="20">
@@ -1848,13 +1848,13 @@
         <v>1257482</v>
       </c>
       <c r="H20" s="4">
-        <v>1666903</v>
+        <v>1667240</v>
       </c>
       <c r="I20" s="4">
-        <v>2435575</v>
+        <v>2435933</v>
       </c>
       <c r="J20" s="4">
-        <v>3434404</v>
+        <v>3434785</v>
       </c>
     </row>
     <row r="21">
@@ -1882,13 +1882,13 @@
         <v>1257482</v>
       </c>
       <c r="H21" s="2">
-        <v>1666903</v>
+        <v>1667240</v>
       </c>
       <c r="I21" s="2">
-        <v>2435575</v>
+        <v>2435933</v>
       </c>
       <c r="J21" s="2">
-        <v>3434404</v>
+        <v>3434785</v>
       </c>
     </row>
     <row r="22">
@@ -1916,13 +1916,13 @@
         <v>880237</v>
       </c>
       <c r="H22" s="2">
-        <v>1166832</v>
+        <v>1167068</v>
       </c>
       <c r="I22" s="2">
-        <v>1704903</v>
+        <v>1705153</v>
       </c>
       <c r="J22" s="2">
-        <v>2404083</v>
+        <v>2404350</v>
       </c>
     </row>
     <row r="23">
@@ -2052,13 +2052,13 @@
         <v>3460459</v>
       </c>
       <c r="H26" s="4">
-        <v>4107497</v>
+        <v>4107834</v>
       </c>
       <c r="I26" s="4">
-        <v>5049114.969999999</v>
+        <v>5049472.969999999</v>
       </c>
       <c r="J26" s="4">
-        <v>6235898.75</v>
+        <v>6236279.75</v>
       </c>
     </row>
     <row r="27">
@@ -2088,13 +2088,13 @@
         <v>4.7439697723573815</v>
       </c>
       <c r="H27" s="2">
-        <v>18.69803976871276</v>
+        <v>18.707778361194283</v>
       </c>
       <c r="I27" s="2">
-        <v>22.92437389485613</v>
+        <v>22.92300443494062</v>
       </c>
       <c r="J27" s="2">
-        <v>23.504788206476547</v>
+        <v>23.503577245607097</v>
       </c>
     </row>
     <row r="28">
@@ -2122,13 +2122,13 @@
         <v>19.99947753960686</v>
       </c>
       <c r="H28" s="2">
-        <v>20.595815438694697</v>
+        <v>20.597505224421344</v>
       </c>
       <c r="I28" s="2">
-        <v>21.961913092606146</v>
+        <v>21.963470269444834</v>
       </c>
       <c r="J28" s="2">
-        <v>23.422262156817652</v>
+        <v>23.423693206653372</v>
       </c>
     </row>
     <row r="29">
@@ -2364,13 +2364,13 @@
         <v>12912.160447761195</v>
       </c>
       <c r="H35" s="2">
-        <v>14882.235507246376</v>
+        <v>14883.45652173913</v>
       </c>
       <c r="I35" s="2">
-        <v>17654.248146853144</v>
+        <v>17655.49989510489</v>
       </c>
       <c r="J35" s="2">
-        <v>21067.225506756757</v>
+        <v>21068.51266891892</v>
       </c>
     </row>
     <row r="36">
@@ -2398,13 +2398,13 @@
         <v>1647150</v>
       </c>
       <c r="H36" s="4">
-        <v>2171733</v>
+        <v>2172070</v>
       </c>
       <c r="I36" s="4">
-        <v>2951317.799999999</v>
+        <v>2951675.799999999</v>
       </c>
       <c r="J36" s="4">
-        <v>3961869.7699999996</v>
+        <v>3962250.7699999996</v>
       </c>
     </row>
     <row r="37">
@@ -2432,13 +2432,13 @@
         <v>9.519586687593593</v>
       </c>
       <c r="H37" s="2">
-        <v>10.889505713606791</v>
+        <v>10.891195499333438</v>
       </c>
       <c r="I37" s="2">
-        <v>12.837217099903263</v>
+        <v>12.838774276741951</v>
       </c>
       <c r="J37" s="2">
-        <v>14.880926728342219</v>
+        <v>14.88235777817794</v>
       </c>
     </row>
     <row r="38">
@@ -2468,13 +2468,13 @@
         <v>2.8427467189470645</v>
       </c>
       <c r="H38" s="2">
-        <v>31.847919133047988</v>
+        <v>31.868378714749724</v>
       </c>
       <c r="I38" s="2">
-        <v>35.896898928183106</v>
+        <v>35.89229628879358</v>
       </c>
       <c r="J38" s="2">
-        <v>34.2407032546614</v>
+        <v>34.23732951972573</v>
       </c>
     </row>
   </sheetData>
@@ -3720,7 +3720,7 @@
       </c>
       <c r="J5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 67.71 % / 補助 67.99 % / ベース 67.34 %</t>
+          <t xml:space="preserve">全社 67.71 % / 補助 67.99 % / ベース 67.33 %</t>
         </is>
       </c>
       <c r="K5" s="0" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="J6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 32.29 % / 補助 32.01 % / ベース 32.66 %</t>
+          <t xml:space="preserve">全社 32.29 % / 補助 32.01 % / ベース 32.67 %</t>
         </is>
       </c>
       <c r="K6" s="0" t="inlineStr">
@@ -3906,17 +3906,17 @@
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.13 % / 補助 10.85 % / ベース 6.83 %</t>
+          <t xml:space="preserve">全社 9.14 % / 補助 10.85 % / ベース 6.83 %</t>
         </is>
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.31 % / 補助 13.8 % / ベース 7.48 %</t>
+          <t xml:space="preserve">全社 11.32 % / 補助 13.8 % / ベース 7.48 %</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.57 % / 補助 16.64 % / ベース 8.12 %</t>
+          <t xml:space="preserve">全社 13.57 % / 補助 16.64 % / ベース 8.13 %</t>
         </is>
       </c>
     </row>
@@ -4526,17 +4526,17 @@
       </c>
       <c r="J18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 47.13 % / 補助 36.82 % / ベース 59.99 %</t>
+          <t xml:space="preserve">全社 47.12 % / 補助 36.82 % / ベース 59.98 %</t>
         </is>
       </c>
       <c r="K18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 41.55 % / 補助 30.32 % / ベース 58.67 %</t>
+          <t xml:space="preserve">全社 41.54 % / 補助 30.32 % / ベース 58.66 %</t>
         </is>
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 36.47 % / 補助 25.15 % / ベース 57.42 %</t>
+          <t xml:space="preserve">全社 36.46 % / 補助 25.15 % / ベース 57.41 %</t>
         </is>
       </c>
     </row>
@@ -4712,17 +4712,17 @@
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6,722.26 千円/人 / 補助 10,512.47 千円/人 / ベース 3,799.09 千円/人</t>
+          <t xml:space="preserve">全社 6,723.51 千円/人 / 補助 10,512.47 千円/人 / ベース 3,801.29 千円/人</t>
         </is>
       </c>
       <c r="K21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9,257.36 千円/人 / 補助 15,907.5 千円/人 / ベース 4,228.19 千円/人</t>
+          <t xml:space="preserve">全社 9,258.63 千円/人 / 補助 15,907.5 千円/人 / ベース 4,230.42 千円/人</t>
         </is>
       </c>
       <c r="L21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12,411.92 千円/人 / 補助 23,016.67 千円/人 / ベース 4,647.73 千円/人</t>
+          <t xml:space="preserve">全社 12,413.23 千円/人 / 補助 23,016.67 千円/人 / ベース 4,650 千円/人</t>
         </is>
       </c>
     </row>
@@ -4774,17 +4774,17 @@
       </c>
       <c r="J22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 14,882.24 千円/人 / 補助 18,998.63 千円/人 / ベース 11,715.78 千円/人</t>
+          <t xml:space="preserve">全社 14,883.46 千円/人 / 補助 18,998.63 千円/人 / ベース 11,717.94 千円/人</t>
         </is>
       </c>
       <c r="K22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 17,654.25 千円/人 / 補助 24,791.72 千円/人 / ベース 12,268.3 千円/人</t>
+          <t xml:space="preserve">全社 17,655.5 千円/人 / 補助 24,791.72 千円/人 / ベース 12,270.5 千円/人</t>
         </is>
       </c>
       <c r="L22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 21,067.23 千円/人 / 補助 32,396.84 千円/人 / ベース 12,785.34 千円/人</t>
+          <t xml:space="preserve">全社 21,068.51 千円/人 / 補助 32,396.84 千円/人 / ベース 12,787.57 千円/人</t>
         </is>
       </c>
     </row>
@@ -5208,7 +5208,7 @@
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.2 倍 / 補助 7.2 倍 / ベース 4.88 倍</t>
+          <t xml:space="preserve">全社 6.21 倍 / 補助 7.2 倍 / ベース 4.88 倍</t>
         </is>
       </c>
       <c r="K29" s="0" t="inlineStr">
@@ -5528,7 +5528,7 @@
       </c>
       <c r="L34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 -1.36 pt</t>
+          <t xml:space="preserve">差 -1.35 pt</t>
         </is>
       </c>
     </row>
@@ -5590,7 +5590,7 @@
       </c>
       <c r="L35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 8.52 pt</t>
+          <t xml:space="preserve">差 8.51 pt</t>
         </is>
       </c>
     </row>
@@ -5766,7 +5766,7 @@
       </c>
       <c r="J38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 76.06 %</t>
+          <t xml:space="preserve">寄与率 76.01 %</t>
         </is>
       </c>
       <c r="K38" s="0" t="inlineStr">
@@ -11401,7 +11401,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsIm1vbmV5VW5pdCI6IuWNg+WGhiIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MjAwMDAwLCJjb2dzIjo0ODk2MDAwLCJlbXBsb3llZVBheSI6NTE5MDMxLCJvZmZpY2VyUGF5IjozNjAwMCwiZGVwcmVjaWF0aW9uIjoxODAwMDAsIm90aGVyU2dhIjo5MDAwMDAsImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQ5MzA3OSwiZW1wbG95ZWVCb251cyI6MjU5NTIsIm9mZmljZXJDb21wZW5zYXRpb24iOjMyNDAwLCJvZmZpY2VyQm9udXMiOjM2MDAsImNvZ3NEZXByZWNpYXRpb24iOjQ1MDAwLCJzZ2FEZXByZWNpYXRpb24iOjEzNTAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6MzYwMDB9LCJvdGhlciI6eyJzYWxlcyI6NjQ0MDAwMCwiY29ncyI6NDM3OTIwMCwiZW1wbG95ZWVQYXkiOjcwOTc4Niwib2ZmaWNlclBheSI6NTUyMDAsImRlcHJlY2lhdGlvbiI6MTM4MDAwLCJvdGhlclNnYSI6NzM2MDAwLCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Njc0Mjk3LCJlbXBsb3llZUJvbnVzIjozNTQ4OSwib2ZmaWNlckNvbXBlbnNhdGlvbiI6NDk2ODAsIm9mZmljZXJCb251cyI6NTUyMCwiY29nc0RlcHJlY2lhdGlvbiI6Mjc2MDAsInNnYURlcHJlY2lhdGlvbiI6MTEwNDAwLCJyZXNlYXJjaERldmVsb3BtZW50IjoyNzYwMCwib3JkaW5hcnlJbmNvbWUiOjM5NDUzNCwicHJlVGF4SW5jb21lIjozOTQ1MzQsIm5ldEluY29tZSI6NzUwNzUyLjF9fSx7InllYXIiOjIwMjQsInJvbGUiOiJwcmV2aW91cyIsInByb2plY3QiOnsic2FsZXMiOjc2MDAwMDAsImNvZ3MiOjUxNjgwMDAsImVtcGxveWVlUGF5Ijo1NTg4MjQsIm9mZmljZXJQYXkiOjM4MDAwLCJkZXByZWNpYXRpb24iOjE5MDAwMCwib3RoZXJTZ2EiOjk1MDAwMCwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NTMwODgzLCJlbXBsb3llZUJvbnVzIjoyNzk0MSwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MzQyMDAsIm9mZmljZXJCb251cyI6MzgwMCwiY29nc0RlcHJlY2lhdGlvbiI6NDc1MDAsInNnYURlcHJlY2lhdGlvbiI6MTQyNTAwLCJyZXNlYXJjaERldmVsb3BtZW50IjozODAwMH0sIm90aGVyIjp7InNhbGVzIjo2NzIwMDAwLCJjb2dzIjo0NTY5NjAwLCJlbXBsb3llZVBheSI6NzU0MTQ4LCJvZmZpY2VyUGF5Ijo1NzYwMCwiZGVwcmVjaWF0aW9uIjoxNDQwMDAsIm90aGVyU2dhIjo3NjgwMDAsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3MTY0NDEsImVtcGxveWVlQm9udXMiOjM3NzA3LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjo1MTg0MCwib2ZmaWNlckJvbnVzIjo1NzYwLCJjb2dzRGVwcmVjaWF0aW9uIjoyODgwMCwic2dhRGVwcmVjaWF0aW9uIjoxMTUyMDAsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjI4ODAwLCJvcmRpbmFyeUluY29tZSI6Mzk4MDEyLCJwcmVUYXhJbmNvbWUiOjM5ODAxMiwibmV0SW5jb21lIjo3NzE4ODEuNn19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwMDAwMDAsImNvZ3MiOjU0NDAwMDAsImVtcGxveWVlUGF5Ijo2MDAwMDAsImVtcGxveWVlU2FsYXJ5Ijo1NzAwMDAsImVtcGxveWVlQm9udXMiOjMwMDAwLCJvZmZpY2VyUGF5Ijo0MDAwMCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MzYwMDAsIm9mZmljZXJCb251cyI6NDAwMCwiZGVwcmVjaWF0aW9uIjoyMDAwMDAsImNvZ3NEZXByZWNpYXRpb24iOjUwMDAwLCJzZ2FEZXByZWNpYXRpb24iOjE1MDAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6NDAwMDAsIm90aGVyU2dhIjoxMDAwMDAwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwMDAwMDAsImNvZ3MiOjQ3NjAwMDAsImVtcGxveWVlUGF5Ijo4MDAwMDAsImVtcGxveWVlU2FsYXJ5Ijo3NjAwMDAsImVtcGxveWVlQm9udXMiOjQwMDAwLCJvZmZpY2VyUGF5Ijo2MDAwMCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6NTQwMDAsIm9mZmljZXJCb251cyI6NjAwMCwiZGVwcmVjaWF0aW9uIjoxNTAwMDAsImNvZ3NEZXByZWNpYXRpb24iOjMwMDAwLCJzZ2FEZXByZWNpYXRpb24iOjEyMDAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6MzAwMDAsIm90aGVyU2dhIjo4MDAwMDAsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjo0MDAwMDAsInByZVRheEluY29tZSI6NDAwMDAwLCJuZXRJbmNvbWUiOjc5MTAwMH19XSwiYmFsYW5jZVNoZWV0cyI6W3sieWVhciI6MjAyMywiYXNzZXRzIjoxMzIwMDAwMCwiY3VycmVudEFzc2V0cyI6NjcwMDAwMCwiY2FzaCI6MjQwMDAwMCwiZml4ZWRBc3NldHMiOjY1MDAwMDAsInRhbmdpYmxlQXNzZXRzIjo1MzAwMDAwLCJidWlsZGluZ3MiOjE5MDAwMDAsIm1hY2hpbmVyeSI6MjQwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6NzAwMDAwLCJzb2Z0d2FyZSI6NTAwMDAwLCJsaWFiaWxpdGllcyI6NzUwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjozOTAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjozNjAwMDAwLCJsb25nVGVybURlYnQiOjI5MDAwMDAsIm5ldEFzc2V0cyI6NTcwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjU0MDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4Ijo1MDAwMDB9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMwMDAwMCwiY3VycmVudEFzc2V0cyI6NzIwMDAwMCwiY2FzaCI6MjUwMDAwMCwiZml4ZWRBc3NldHMiOjcxMDAwMDAsInRhbmdpYmxlQXNzZXRzIjo1ODAwMDAwLCJidWlsZGluZ3MiOjIwMDAwMDAsIm1hY2hpbmVyeSI6MjgwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6ODAwMDAwLCJzb2Z0d2FyZSI6NjAwMDAwLCJsaWFiaWxpdGllcyI6NzkwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjo0MTAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjozODAwMDAwLCJsb25nVGVybURlYnQiOjMxMDAwMDAsIm5ldEFzc2V0cyI6NjQwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjYxMDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4Ijo4MDAwMDB9LHsieWVhciI6MjAyNSwiYXNzZXRzIjoxNTYwMDAwMCwiY3VycmVudEFzc2V0cyI6NzgwMDAwMCwiY2FzaCI6MjcwMDAwMCwiZml4ZWRBc3NldHMiOjc4MDAwMDAsInRhbmdpYmxlQXNzZXRzIjo2NDAwMDAwLCJidWlsZGluZ3MiOjIyMDAwMDAsIm1hY2hpbmVyeSI6MzIwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6OTAwMDAwLCJzb2Z0d2FyZSI6NzAwMDAwLCJsaWFiaWxpdGllcyI6ODMwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjo0MzAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMTAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjo0MDAwMDAwLCJsb25nVGVybURlYnQiOjMyMDAwMDAsIm5ldEFzc2V0cyI6NzMwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjcwMDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4IjoxMDAwMDAwfV0sImZ1dHVyZUNhcGV4IjpbeyJ5ZWFyIjoyMDI2LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI4LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI5LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMwLCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMxLCJ2YWx1ZSI6MH1dLCJkcml2ZXJzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsInByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJwcm9qZWN0Q29nc1JhdGVUb0Jhc2UiOjAuNjgsIm90aGVyQ29nc1JhdGVUb0Jhc2UiOjAuNjgsInByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwib3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwicHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yNSwib3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMiwicHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsInByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJvdGhlck5vbk9wZXJhdGluZ1JhdGUiOi0wLjAwNSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjowLCJlZmZlY3RpdmVUYXhSYXRlIjowLjMsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdEZpcnN0WWVhclNhbGVzIjowLCJwcm9qZWN0QmFzZVllYXJTYWxlcyI6MCwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6NS41NTExMTUxMjMxMjU3ODNlLTE3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5Nywib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI1NzI0NjM3NjgxMTU4NTQsIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wMTUsIm90aGVyU2dhUmF0ZUVuZCI6MC4wMDUsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJpbnZlc3RtZW50IjoyMzAwMDAwLCJzdWJzaWR5Ijo3NjYwMDAsImxvY2FsQmVuY2htYXJrIjoyM30sImRyaXZlclJhbmdlcyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjpbLTAuMDUsMC4zXSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6WzAuNjYsMC43XSwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOlswLjY2LDAuN10sInByb2plY3RDb2dzUmF0ZVRvQmFzZSI6WzAuNjgsMC42OF0sIm90aGVyQ29nc1JhdGVUb0Jhc2UiOlswLjY4LDAuNjhdLCJwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOlswLDFdLCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOlswLDFdLCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOlstMC41LDAuNV0sIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6Wy0wLjUsMC41XSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJlZmZlY3RpdmVUYXhSYXRlIjpbMCwwLjZdLCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwicHJvamVjdEZpcnN0WWVhclNhbGVzIjpbMCwxMDAwMDAwMDAwMF0sInByb2plY3RCYXNlWWVhclNhbGVzIjpbMCwxMDAwMDAwMDAwMF0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDEuNjY1MzM0NTM2OTM3NzM0OGUtMTZdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkzMjUzMzA1MDE4NDY5MjcsMC4wMjA3MzU5OTQxODMxODkxNjZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlswLjA0MDc2MDg2OTU2NTIxNzE4NCwwLjA0NDM4NDA1Nzk3MTAxNDUyXSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDAwMTM0NTc1NTY5MzU4MTk3MzddLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MTM5NDU3MDIzNzE3NDQzLDAuMDIwNTUzNDU5OTE0NzYzMDk1XSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjAzOTE2NjY2NjY2NjY2NjY4LDAuMDQyNTAwMDAwMDAwMDAwMDldLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbMC4xNSwwLjNdLCJvdGhlclNhbGVzR3Jvd3RoIjpbMC4wNjA3NjA4Njk1NjUyMTcxOSwwLjA2NDM4NDA1Nzk3MTAxNDUzXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMC4wMDUsMC4wMDUxMzQ1NzU1NjkzNTgxOTc1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLjAyNDEzOTQ1NzAyMzcxNzQ0NCwwLjAyNTU1MzQ1OTkxNDc2MzA5Nl0sIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6WzAsMC4wOF0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6WzAuMDQ0MTY2NjY2NjY2NjY2NjgsMC4wNDc1MDAwMDAwMDAwMDAwOV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMCwwLjAzXSwib3RoZXJTZ2FSYXRlRW5kIjpbMCwwLjAxXSwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOlswLjA0MjYzMTU3ODk0NzM2ODM2LDAuMDY1NTU1NTU1NTU1NTU1NThdLCJpbnZlc3RtZW50IjpbMTUwMDAwMCwyMDAwMDAwMF0sInN1YnNpZHkiOlsxMDAwMDAsNTAwMDAwMF0sImxvY2FsQmVuY2htYXJrIjpbMCwxMDBdfSwidGFyZ2V0cyI6eyJjb21wYW55U2FsZXNDYWdyIjp7InZhbHVlIjoxNSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo4MjQwMDAwLCJtYXgiOjI1MjY5MDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjoyLCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NjAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo3NDgwMDAwLCJtYXgiOjEzNjg0MDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MTg3ODAwMCwibWF4IjozMzQzMDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6Mjg1MDAwLCJtYXgiOjM3NDAwMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjoxNSwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX19LCJmb3JlY2FzdE92ZXJyaWRlcyI6eyIyMDI5Om90aGVyOnNhbGVzIjo4NTEzMDAwLCIyMDI5OnByb2plY3Q6Ny04Ijo3OTAwMDB9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2NDAwMDAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mjc1MjAwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6NzI2MDAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi03IjozMjY1MDE3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6ODIwODAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMCI6OTEyMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEyIjoxMTY3Mzc2LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjYxNDQxLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTQiOjI0NTQwMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1Ijo2MzYwMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE4IjoxMDcyNTAzLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTkiOjEwNzI1MDMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yMCI6NzUwNzUyLjEsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yNyI6MjEwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xIjo3MjAwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNCI6MjMwNDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjY3Nzk2OSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTgiOjUxOTAzMSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTkiOjM2MDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOlAyLTQiOjQ1MDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOlAyLTE0IjoxMzUwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMyI6OTAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEiOjE0MzIwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMyI6OTczNzYwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTQiOjc2MzAwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItNyI6MzQ1MTA3MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTkiOjg2MDQwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTAiOjk1NjAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMiI6MTI0NzMyNCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEzIjo2NTY0OCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjoyNTc3MDAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNSI6NjY4MDAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xOCI6MTEwMjY4OCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE5IjoxMTAyNjg4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjAiOjc3MTg4MS42LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjciOjIyMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMSI6NzYwMDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0MzIwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny02Ijo3MDQ2NzYsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny04Ijo1NTg4MjQsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjozODAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDpQMi00Ijo0NzUwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDpQMi0xNCI6MTQyNTAwLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTMiOjk1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xIjoxNTAwMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTMiOjEwMjAwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6ODAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi03IjozNjQwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItOSI6OTAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMCI6MTAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMzMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjo3MDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE0IjoyNzAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNSI6NzAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xOCI6MTEzMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE5IjoxMTMwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjAiOjc5MTAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI3IjoyMzAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwMDAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNTYwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6NzMwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NjAwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOSI6NDAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6UDItNCI6NTAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6UDItMTQiOjE1MDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FzaCI6MjQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpidWlsZGluZ3MiOjE5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6aW50YW5naWJsZUFzc2V0cyI6NzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudExpYWJpbGl0aWVzIjozOTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpsb25nVGVybURlYnQiOjI5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGl0YWwiOjEwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRBc3NldHMiOjcyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDp0YW5naWJsZUFzc2V0cyI6NTgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmxhbmQiOjEwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGlhYmlsaXRpZXMiOjc5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRMaWFiaWxpdGllcyI6MzgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OnNoYXJlaG9sZGVyRXF1aXR5Ijo2MTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTphc3NldHMiOjE1NjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZEFzc2V0cyI6NzgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bWFjaGluZXJ5IjozMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjkwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OnNvZnR3YXJlIjo3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OnNob3J0VGVybURlYnQiOjExMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bmV0QXNzZXRzIjo3MzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwZXgiOjEwMDAwMDAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MC42NiwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC43LCJkcml2ZXI6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybzowIjowLjY2LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC43LCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlVG9CYXNlIjowLjY4LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NSYXRlVG9CYXNlOjAiOjAuNjgsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc1JhdGVUb0Jhc2U6MSI6MC42OCwiZHJpdmVyOm90aGVyQ29nc1JhdGVUb0Jhc2UiOjAuNjgsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlVG9CYXNlOjAiOjAuNjgsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlVG9CYXNlOjEiOjAuNjgsImRyaXZlcjpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwiZHJpdmVyLXJhbmdlOnByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZToxIjoxLCJkcml2ZXI6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJkcml2ZXItcmFuZ2U6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjowLjksImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGU6MSI6MC4zLCJkcml2ZXI6b3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjEiOjAuMywiZHJpdmVyOnByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdE5vbk9wZXJhdGluZ1JhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOnByb2plY3ROb25PcGVyYXRpbmdSYXRlOjEiOjAuNSwiZHJpdmVyOm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJOb25PcGVyYXRpbmdSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpvdGhlck5vbk9wZXJhdGluZ1JhdGU6MSI6MC41LCJkcml2ZXI6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6b3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6ZWZmZWN0aXZlVGF4UmF0ZSI6MC4zLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZTowIjowLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZToxIjowLjYsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RGaXJzdFllYXJTYWxlcyI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RGaXJzdFllYXJTYWxlczowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEZpcnN0WWVhclNhbGVzOjEiOjEwMDAwMDAwMDAwLCJkcml2ZXI6cHJvamVjdEJhc2VZZWFyU2FsZXMiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0QmFzZVllYXJTYWxlczowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEJhc2VZZWFyU2FsZXM6MSI6MTAwMDAwMDAwMDAsImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjEuNjY1MzM0NTM2OTM3NzM0OGUtMTYsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkzMjUzMzA1MDE4NDY5MjcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNzM1OTk0MTgzMTg5MTY2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLjAxOTEzOTQ1NzAyMzcxNzQ0MywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNTUzNDU5OTE0NzYzMDk1LCJkcml2ZXI6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wMzkxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDQyNTAwMDAwMDAwMDAwMDksImRyaXZlcjpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjAiOjAuMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MSI6MC4zLCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NzI0NjM3NjgxMTU4NiwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MCI6MC4wNjA3NjA4Njk1NjUyMTcxOSwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MSI6MC4wNjQzODQwNTc5NzEwMTQ1MywiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZToxIjowLjAzLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDoxIjowLjAwNTEzNDU3NTU2OTM1ODE5NzUsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDowIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDoxIjowLjEsImRyaXZlcjpvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjAiOjAuMDI0MTM5NDU3MDIzNzE3NDQ0LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wMjU1NTM0NTk5MTQ3NjMwOTYsImRyaXZlcjpvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGg6MSI6MC4wOCwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjowLjA0NDE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MSI6MC4wNDc1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjAxNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDoxIjowLjAzLCJkcml2ZXI6b3RoZXJTZ2FSYXRlRW5kIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMDEsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAuMDQyNjMxNTc4OTQ3MzY4MzYsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjA2NTU1NTU1NTU1NTU1NTU4LCJkcml2ZXI6aW52ZXN0bWVudCI6MjMwMDAwMCwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUwMDAwMCwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MSI6MjAwMDAwMDAsImRyaXZlcjpzdWJzaWR5Ijo3NjYwMDAsImRyaXZlci1yYW5nZTpzdWJzaWR5OjAiOjEwMDAwMCwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MSI6NTAwMDAwMCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoxNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjo4MjQwMDAwLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjoyLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOm1heCI6NywidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOnZhbHVlIjo2MCwidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOm1heCI6OTUsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOnZhbHVlIjoyMiwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOnZhbHVlIjo3NDgwMDAwLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOnZhbHVlIjoyMSwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2FncjptYXgiOjM1LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOnZhbHVlIjoxODc4MDAwLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOnZhbHVlIjo3LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOm1heCI6MTAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOnZhbHVlIjoyODUwMDAsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MTUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTptYXgiOjI1MjY5MDAwLCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6bWF4IjoxMzY4NDAwMCwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTptYXgiOjMzNDMwMDAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOm1heCI6Mzc0MDAwfSwibWV0cmljR3JvdXBCYXNlcyI6eyJjb21wYW55U2FsZXMiOiJyYXRlIiwicHJvamVjdFNhbGVzIjoicmF0ZSIsImxhYm9yUHJvZHVjdGl2aXR5IjoicmF0ZSIsImVtcGxveWVlUGF5IjoicmF0ZSJ9LCJhcHBsaWNhdGlvbkNhdGVnb3J5IjoiZ2VuZXJhbCIsImFkanVzdGVkRHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY3OTkxNTA3Mjk3OTcwODEsIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4MDAwOTM1MzYzNDAxMzIsInByb2plY3RDb2dzUmF0ZVRvQmFzZSI6MC42OCwib3RoZXJDb2dzUmF0ZVRvQmFzZSI6MC42OCwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA3MDcyMzY4NDIxMDUxLCJwcm9qZWN0Rmlyc3RZZWFyU2FsZXMiOjAsInByb2plY3RCYXNlWWVhclNhbGVzIjowLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjoxLjMzNzU5NjcwMDA2ODM4ODdlLTE2LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDA0NzAwOTU3NDk0MjI0LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1MjE5MjI1ODM4MTk5Mjk4LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA0OTgyMDkxOTA3OTY4Niwib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI2MTYwNTg0NTI3Njc5OCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg2NDI2Njc5MjM0NzY0OCwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA5MzA4MjU0MjAwMTQ2NSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyMDAwMjEzNjI4OTg4NjM4LCJvdGhl</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsIm1vbmV5VW5pdCI6IuWNg+WGhiIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MjAwMDAwLCJjb2dzIjo0ODk2MDAwLCJlbXBsb3llZVBheSI6NTE5MDMxLCJvZmZpY2VyUGF5IjozNjAwMCwiZGVwcmVjaWF0aW9uIjoxODAwMDAsIm90aGVyU2dhIjo5MDAwMDAsImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQ5MzA3OSwiZW1wbG95ZWVCb251cyI6MjU5NTIsIm9mZmljZXJDb21wZW5zYXRpb24iOjMyNDAwLCJvZmZpY2VyQm9udXMiOjM2MDAsImNvZ3NEZXByZWNpYXRpb24iOjQ1MDAwLCJzZ2FEZXByZWNpYXRpb24iOjEzNTAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6MzYwMDB9LCJvdGhlciI6eyJzYWxlcyI6NjQ0MDAwMCwiY29ncyI6NDM3OTIwMCwiZW1wbG95ZWVQYXkiOjcwOTc4Niwib2ZmaWNlclBheSI6NTUyMDAsImRlcHJlY2lhdGlvbiI6MTM4MDAwLCJvdGhlclNnYSI6NzM2MDAwLCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Njc0Mjk3LCJlbXBsb3llZUJvbnVzIjozNTQ4OSwib2ZmaWNlckNvbXBlbnNhdGlvbiI6NDk2ODAsIm9mZmljZXJCb251cyI6NTUyMCwiY29nc0RlcHJlY2lhdGlvbiI6Mjc2MDAsInNnYURlcHJlY2lhdGlvbiI6MTEwNDAwLCJyZXNlYXJjaERldmVsb3BtZW50IjoyNzYwMCwib3JkaW5hcnlJbmNvbWUiOjM5NDUzNCwicHJlVGF4SW5jb21lIjozOTQ1MzQsIm5ldEluY29tZSI6NzUwNzUyLjF9fSx7InllYXIiOjIwMjQsInJvbGUiOiJwcmV2aW91cyIsInByb2plY3QiOnsic2FsZXMiOjc2MDAwMDAsImNvZ3MiOjUxNjgwMDAsImVtcGxveWVlUGF5Ijo1NTg4MjQsIm9mZmljZXJQYXkiOjM4MDAwLCJkZXByZWNpYXRpb24iOjE5MDAwMCwib3RoZXJTZ2EiOjk1MDAwMCwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NTMwODgzLCJlbXBsb3llZUJvbnVzIjoyNzk0MSwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MzQyMDAsIm9mZmljZXJCb251cyI6MzgwMCwiY29nc0RlcHJlY2lhdGlvbiI6NDc1MDAsInNnYURlcHJlY2lhdGlvbiI6MTQyNTAwLCJyZXNlYXJjaERldmVsb3BtZW50IjozODAwMH0sIm90aGVyIjp7InNhbGVzIjo2NzIwMDAwLCJjb2dzIjo0NTY5NjAwLCJlbXBsb3llZVBheSI6NzU0MTQ4LCJvZmZpY2VyUGF5Ijo1NzYwMCwiZGVwcmVjaWF0aW9uIjoxNDQwMDAsIm90aGVyU2dhIjo3NjgwMDAsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3MTY0NDEsImVtcGxveWVlQm9udXMiOjM3NzA3LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjo1MTg0MCwib2ZmaWNlckJvbnVzIjo1NzYwLCJjb2dzRGVwcmVjaWF0aW9uIjoyODgwMCwic2dhRGVwcmVjaWF0aW9uIjoxMTUyMDAsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjI4ODAwLCJvcmRpbmFyeUluY29tZSI6Mzk4MDEyLCJwcmVUYXhJbmNvbWUiOjM5ODAxMiwibmV0SW5jb21lIjo3NzE4ODEuNn19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwMDAwMDAsImNvZ3MiOjU0NDAwMDAsImVtcGxveWVlUGF5Ijo2MDAwMDAsImVtcGxveWVlU2FsYXJ5Ijo1NzAwMDAsImVtcGxveWVlQm9udXMiOjMwMDAwLCJvZmZpY2VyUGF5Ijo0MDAwMCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MzYwMDAsIm9mZmljZXJCb251cyI6NDAwMCwiZGVwcmVjaWF0aW9uIjoyMDAwMDAsImNvZ3NEZXByZWNpYXRpb24iOjUwMDAwLCJzZ2FEZXByZWNpYXRpb24iOjE1MDAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6NDAwMDAsIm90aGVyU2dhIjoxMDAwMDAwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwMDAwMDAsImNvZ3MiOjQ3NjAwMDAsImVtcGxveWVlUGF5Ijo4MDAwMDAsImVtcGxveWVlU2FsYXJ5Ijo3NjAwMDAsImVtcGxveWVlQm9udXMiOjQwMDAwLCJvZmZpY2VyUGF5Ijo2MDAwMCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6NTQwMDAsIm9mZmljZXJCb251cyI6NjAwMCwiZGVwcmVjaWF0aW9uIjoxNTAwMDAsImNvZ3NEZXByZWNpYXRpb24iOjMwMDAwLCJzZ2FEZXByZWNpYXRpb24iOjEyMDAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6MzAwMDAsIm90aGVyU2dhIjo4MDAwMDAsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjo0MDAwMDAsInByZVRheEluY29tZSI6NDAwMDAwLCJuZXRJbmNvbWUiOjc5MTAwMH19XSwiYmFsYW5jZVNoZWV0cyI6W3sieWVhciI6MjAyMywiYXNzZXRzIjoxMzIwMDAwMCwiY3VycmVudEFzc2V0cyI6NjcwMDAwMCwiY2FzaCI6MjQwMDAwMCwiZml4ZWRBc3NldHMiOjY1MDAwMDAsInRhbmdpYmxlQXNzZXRzIjo1MzAwMDAwLCJidWlsZGluZ3MiOjE5MDAwMDAsIm1hY2hpbmVyeSI6MjQwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6NzAwMDAwLCJzb2Z0d2FyZSI6NTAwMDAwLCJsaWFiaWxpdGllcyI6NzUwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjozOTAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjozNjAwMDAwLCJsb25nVGVybURlYnQiOjI5MDAwMDAsIm5ldEFzc2V0cyI6NTcwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjU0MDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4Ijo1MDAwMDB9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMwMDAwMCwiY3VycmVudEFzc2V0cyI6NzIwMDAwMCwiY2FzaCI6MjUwMDAwMCwiZml4ZWRBc3NldHMiOjcxMDAwMDAsInRhbmdpYmxlQXNzZXRzIjo1ODAwMDAwLCJidWlsZGluZ3MiOjIwMDAwMDAsIm1hY2hpbmVyeSI6MjgwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6ODAwMDAwLCJzb2Z0d2FyZSI6NjAwMDAwLCJsaWFiaWxpdGllcyI6NzkwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjo0MTAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjozODAwMDAwLCJsb25nVGVybURlYnQiOjMxMDAwMDAsIm5ldEFzc2V0cyI6NjQwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjYxMDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4Ijo4MDAwMDB9LHsieWVhciI6MjAyNSwiYXNzZXRzIjoxNTYwMDAwMCwiY3VycmVudEFzc2V0cyI6NzgwMDAwMCwiY2FzaCI6MjcwMDAwMCwiZml4ZWRBc3NldHMiOjc4MDAwMDAsInRhbmdpYmxlQXNzZXRzIjo2NDAwMDAwLCJidWlsZGluZ3MiOjIyMDAwMDAsIm1hY2hpbmVyeSI6MzIwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6OTAwMDAwLCJzb2Z0d2FyZSI6NzAwMDAwLCJsaWFiaWxpdGllcyI6ODMwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjo0MzAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMTAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjo0MDAwMDAwLCJsb25nVGVybURlYnQiOjMyMDAwMDAsIm5ldEFzc2V0cyI6NzMwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjcwMDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4IjoxMDAwMDAwfV0sImZ1dHVyZUNhcGV4IjpbeyJ5ZWFyIjoyMDI2LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI4LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI5LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMwLCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMxLCJ2YWx1ZSI6MH1dLCJkcml2ZXJzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsInByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJwcm9qZWN0Q29nc1JhdGVUb0Jhc2UiOjAuNjgsIm90aGVyQ29nc1JhdGVUb0Jhc2UiOjAuNjgsInByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwib3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwicHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yNSwib3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMiwicHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsInByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJvdGhlck5vbk9wZXJhdGluZ1JhdGUiOi0wLjAwNSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjowLCJlZmZlY3RpdmVUYXhSYXRlIjowLjMsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdEZpcnN0WWVhclNhbGVzIjowLCJwcm9qZWN0QmFzZVllYXJTYWxlcyI6MCwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6NS41NTExMTUxMjMxMjU3ODNlLTE3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5Nywib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI1NzI0NjM3NjgxMTU4NTQsIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wMTUsIm90aGVyU2dhUmF0ZUVuZCI6MC4wMDUsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJpbnZlc3RtZW50IjoyMzAwMDAwLCJzdWJzaWR5Ijo3NjYwMDAsImxvY2FsQmVuY2htYXJrIjoyM30sImRyaXZlclJhbmdlcyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjpbLTAuMDUsMC4zXSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6WzAuNjYsMC43XSwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOlswLjY2LDAuN10sInByb2plY3RDb2dzUmF0ZVRvQmFzZSI6WzAuNjgsMC42OF0sIm90aGVyQ29nc1JhdGVUb0Jhc2UiOlswLjY4LDAuNjhdLCJwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOlswLDFdLCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOlswLDFdLCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOlstMC41LDAuNV0sIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6Wy0wLjUsMC41XSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJlZmZlY3RpdmVUYXhSYXRlIjpbMCwwLjZdLCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwicHJvamVjdEZpcnN0WWVhclNhbGVzIjpbMCwxMDAwMDAwMDAwMF0sInByb2plY3RCYXNlWWVhclNhbGVzIjpbMCwxMDAwMDAwMDAwMF0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDEuNjY1MzM0NTM2OTM3NzM0OGUtMTZdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkzMjUzMzA1MDE4NDY5MjcsMC4wMjA3MzU5OTQxODMxODkxNjZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlswLjA0MDc2MDg2OTU2NTIxNzE4NCwwLjA0NDM4NDA1Nzk3MTAxNDUyXSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDAwMTM0NTc1NTY5MzU4MTk3MzddLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MTM5NDU3MDIzNzE3NDQzLDAuMDIwNTUzNDU5OTE0NzYzMDk1XSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjAzOTE2NjY2NjY2NjY2NjY4LDAuMDQyNTAwMDAwMDAwMDAwMDldLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbMC4xNSwwLjNdLCJvdGhlclNhbGVzR3Jvd3RoIjpbMC4wNjA3NjA4Njk1NjUyMTcxOSwwLjA2NDM4NDA1Nzk3MTAxNDUzXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMC4wMDUsMC4wMDUxMzQ1NzU1NjkzNTgxOTc1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLjAyNDEzOTQ1NzAyMzcxNzQ0NCwwLjAyNTU1MzQ1OTkxNDc2MzA5Nl0sIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6WzAsMC4wOF0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6WzAuMDQ0MTY2NjY2NjY2NjY2NjgsMC4wNDc1MDAwMDAwMDAwMDAwOV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMCwwLjAzXSwib3RoZXJTZ2FSYXRlRW5kIjpbMCwwLjAxXSwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOlswLjA0MjYzMTU3ODk0NzM2ODM2LDAuMDY1NTU1NTU1NTU1NTU1NThdLCJpbnZlc3RtZW50IjpbMTUwMDAwMCwyMDAwMDAwMF0sInN1YnNpZHkiOlsxMDAwMDAsNTAwMDAwMF0sImxvY2FsQmVuY2htYXJrIjpbMCwxMDBdfSwidGFyZ2V0cyI6eyJjb21wYW55U2FsZXNDYWdyIjp7InZhbHVlIjoxNSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo4MjQwMDAwLCJtYXgiOjI1MjY5MDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjoyLCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NjAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo3NDgwMDAwLCJtYXgiOjEzNjg0MDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MTg3ODAwMCwibWF4IjozMzQzMDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6Mjg1MDAwLCJtYXgiOjM3NDAwMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjoxNSwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX19LCJmb3JlY2FzdE92ZXJyaWRlcyI6eyIyMDI5Om90aGVyOnNhbGVzIjo4NTEzMDAwLCIyMDI5OnByb2plY3Q6Ny04Ijo3OTAwMDB9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2NDAwMDAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mjc1MjAwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6NzI2MDAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi03IjozMjY1MDE3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6ODIwODAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMCI6OTEyMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEyIjoxMTY3Mzc2LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjYxNDQxLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTQiOjI0NTQwMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1Ijo2MzYwMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE4IjoxMDcyNTAzLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTkiOjEwNzI1MDMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yMCI6NzUwNzUyLjEsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yNyI6MjEwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xIjo3MjAwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNCI6MjMwNDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjY3Nzk2OSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTgiOjUxOTAzMSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTkiOjM2MDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOlAyLTQiOjQ1MDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOlAyLTE0IjoxMzUwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMyI6OTAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEiOjE0MzIwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMyI6OTczNzYwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTQiOjc2MzAwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItNyI6MzQ1MTA3MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTkiOjg2MDQwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTAiOjk1NjAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMiI6MTI0NzMyNCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEzIjo2NTY0OCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjoyNTc3MDAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNSI6NjY4MDAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xOCI6MTEwMjY4OCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE5IjoxMTAyNjg4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjAiOjc3MTg4MS42LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjciOjIyMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMSI6NzYwMDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0MzIwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny02Ijo3MDQ2NzYsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny04Ijo1NTg4MjQsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjozODAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDpQMi00Ijo0NzUwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDpQMi0xNCI6MTQyNTAwLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTMiOjk1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xIjoxNTAwMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTMiOjEwMjAwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6ODAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi03IjozNjQwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItOSI6OTAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMCI6MTAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMzMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjo3MDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE0IjoyNzAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNSI6NzAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xOCI6MTEzMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE5IjoxMTMwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjAiOjc5MTAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI3IjoyMzAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwMDAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNTYwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6NzMwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NjAwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOSI6NDAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6UDItNCI6NTAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6UDItMTQiOjE1MDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FzaCI6MjQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpidWlsZGluZ3MiOjE5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6aW50YW5naWJsZUFzc2V0cyI6NzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudExpYWJpbGl0aWVzIjozOTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpsb25nVGVybURlYnQiOjI5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGl0YWwiOjEwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRBc3NldHMiOjcyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDp0YW5naWJsZUFzc2V0cyI6NTgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmxhbmQiOjEwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGlhYmlsaXRpZXMiOjc5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRMaWFiaWxpdGllcyI6MzgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OnNoYXJlaG9sZGVyRXF1aXR5Ijo2MTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTphc3NldHMiOjE1NjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZEFzc2V0cyI6NzgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bWFjaGluZXJ5IjozMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjkwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OnNvZnR3YXJlIjo3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OnNob3J0VGVybURlYnQiOjExMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bmV0QXNzZXRzIjo3MzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwZXgiOjEwMDAwMDAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MC42NiwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC43LCJkcml2ZXI6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybzowIjowLjY2LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC43LCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlVG9CYXNlIjowLjY4LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NSYXRlVG9CYXNlOjAiOjAuNjgsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc1JhdGVUb0Jhc2U6MSI6MC42OCwiZHJpdmVyOm90aGVyQ29nc1JhdGVUb0Jhc2UiOjAuNjgsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlVG9CYXNlOjAiOjAuNjgsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlVG9CYXNlOjEiOjAuNjgsImRyaXZlcjpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwiZHJpdmVyLXJhbmdlOnByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZToxIjoxLCJkcml2ZXI6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJkcml2ZXItcmFuZ2U6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjowLjksImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGU6MSI6MC4zLCJkcml2ZXI6b3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjEiOjAuMywiZHJpdmVyOnByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdE5vbk9wZXJhdGluZ1JhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOnByb2plY3ROb25PcGVyYXRpbmdSYXRlOjEiOjAuNSwiZHJpdmVyOm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJOb25PcGVyYXRpbmdSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpvdGhlck5vbk9wZXJhdGluZ1JhdGU6MSI6MC41LCJkcml2ZXI6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6b3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6ZWZmZWN0aXZlVGF4UmF0ZSI6MC4zLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZTowIjowLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZToxIjowLjYsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RGaXJzdFllYXJTYWxlcyI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RGaXJzdFllYXJTYWxlczowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEZpcnN0WWVhclNhbGVzOjEiOjEwMDAwMDAwMDAwLCJkcml2ZXI6cHJvamVjdEJhc2VZZWFyU2FsZXMiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0QmFzZVllYXJTYWxlczowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEJhc2VZZWFyU2FsZXM6MSI6MTAwMDAwMDAwMDAsImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjEuNjY1MzM0NTM2OTM3NzM0OGUtMTYsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkzMjUzMzA1MDE4NDY5MjcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNzM1OTk0MTgzMTg5MTY2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLjAxOTEzOTQ1NzAyMzcxNzQ0MywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNTUzNDU5OTE0NzYzMDk1LCJkcml2ZXI6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wMzkxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDQyNTAwMDAwMDAwMDAwMDksImRyaXZlcjpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjAiOjAuMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MSI6MC4zLCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NzI0NjM3NjgxMTU4NiwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MCI6MC4wNjA3NjA4Njk1NjUyMTcxOSwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MSI6MC4wNjQzODQwNTc5NzEwMTQ1MywiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZToxIjowLjAzLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDoxIjowLjAwNTEzNDU3NTU2OTM1ODE5NzUsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDowIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDoxIjowLjEsImRyaXZlcjpvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjAiOjAuMDI0MTM5NDU3MDIzNzE3NDQ0LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wMjU1NTM0NTk5MTQ3NjMwOTYsImRyaXZlcjpvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGg6MSI6MC4wOCwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjowLjA0NDE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MSI6MC4wNDc1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjAxNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDoxIjowLjAzLCJkcml2ZXI6b3RoZXJTZ2FSYXRlRW5kIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMDEsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAuMDQyNjMxNTc4OTQ3MzY4MzYsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjA2NTU1NTU1NTU1NTU1NTU4LCJkcml2ZXI6aW52ZXN0bWVudCI6MjMwMDAwMCwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUwMDAwMCwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MSI6MjAwMDAwMDAsImRyaXZlcjpzdWJzaWR5Ijo3NjYwMDAsImRyaXZlci1yYW5nZTpzdWJzaWR5OjAiOjEwMDAwMCwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MSI6NTAwMDAwMCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoxNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjo4MjQwMDAwLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjoyLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOm1heCI6NywidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOnZhbHVlIjo2MCwidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOm1heCI6OTUsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOnZhbHVlIjoyMiwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOnZhbHVlIjo3NDgwMDAwLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOnZhbHVlIjoyMSwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2FncjptYXgiOjM1LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOnZhbHVlIjoxODc4MDAwLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOnZhbHVlIjo3LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOm1heCI6MTAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOnZhbHVlIjoyODUwMDAsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MTUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTptYXgiOjI1MjY5MDAwLCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6bWF4IjoxMzY4NDAwMCwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTptYXgiOjMzNDMwMDAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOm1heCI6Mzc0MDAwfSwibWV0cmljR3JvdXBCYXNlcyI6eyJjb21wYW55U2FsZXMiOiJyYXRlIiwicHJvamVjdFNhbGVzIjoicmF0ZSIsImxhYm9yUHJvZHVjdGl2aXR5IjoicmF0ZSIsImVtcGxveWVlUGF5IjoicmF0ZSJ9LCJhcHBsaWNhdGlvbkNhdGVnb3J5IjoiZ2VuZXJhbCIsImFkanVzdGVkRHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY3OTkxNTA3Mjk3OTcwODEsIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY3OTk2OTM1MzYzNDAxMzMsInByb2plY3RDb2dzUmF0ZVRvQmFzZSI6MC42OCwib3RoZXJDb2dzUmF0ZVRvQmFzZSI6MC42OCwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA3MDcyMzY4NDIxMDUxLCJwcm9qZWN0Rmlyc3RZZWFyU2FsZXMiOjAsInByb2plY3RCYXNlWWVhclNhbGVzIjowLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjoxLjMzNzU5NjcwMDA2ODM4ODdlLTE2LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDA0NzAwOTU3NDk0MjI0LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1MjE5MjI1ODM4MTk5Mjk4LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA0OTgyMDkxOTA3OTY4Niwib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI2MTYwNTg0NTI3Njc5OCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg2NDI2Njc5MjM0NzY0OCwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA5MzA4MjU0MjAwMTQ2NSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyMDAwMjEzNjI4OTg4NjM4LCJvdGhl</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Forecast depreciation from latest expense ratios
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -204,7 +204,7 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <v>15.44763837519807</v>
+        <v>15.474852079230983</v>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
@@ -234,7 +234,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <v>9321063.75</v>
+        <v>9339895.75</v>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
@@ -294,7 +294,7 @@
         </is>
       </c>
       <c r="B11" s="2">
-        <v>63.90146083802072</v>
+        <v>63.92697661345926</v>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
@@ -324,7 +324,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>22.000214756484016</v>
+        <v>22.04521290118877</v>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
@@ -354,7 +354,7 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <v>7643875</v>
+        <v>7662707</v>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
@@ -384,7 +384,7 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <v>27.83033380160913</v>
+        <v>28.208408977597756</v>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
@@ -414,7 +414,7 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <v>2219470.9999999995</v>
+        <v>2266054.9999999995</v>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <v>289.7481723237597</v>
+        <v>295.8296344647519</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
@@ -1268,13 +1268,13 @@
         <v>17302747</v>
       </c>
       <c r="H3" s="4">
-        <v>19943357</v>
+        <v>19947574</v>
       </c>
       <c r="I3" s="4">
-        <v>22990323.97</v>
+        <v>23000613.97</v>
       </c>
       <c r="J3" s="4">
-        <v>26623810.75</v>
+        <v>26642642.75</v>
       </c>
     </row>
     <row r="4">
@@ -1304,13 +1304,13 @@
         <v>4.878742144662529</v>
       </c>
       <c r="H4" s="2">
-        <v>15.261218348739657</v>
+        <v>15.285590201370924</v>
       </c>
       <c r="I4" s="2">
-        <v>15.278104734323318</v>
+        <v>15.30531968448894</v>
       </c>
       <c r="J4" s="2">
-        <v>15.804417479028675</v>
+        <v>15.834485047878921</v>
       </c>
     </row>
     <row r="5">
@@ -1338,13 +1338,13 @@
         <v>11765868</v>
       </c>
       <c r="H5" s="2">
-        <v>13503580</v>
+        <v>13506447</v>
       </c>
       <c r="I5" s="2">
-        <v>15317641</v>
+        <v>15324483</v>
       </c>
       <c r="J5" s="2">
-        <v>17432565</v>
+        <v>17444804</v>
       </c>
     </row>
     <row r="6">
@@ -1363,22 +1363,22 @@
         <v>80000</v>
       </c>
       <c r="E6" s="2">
-        <v>80000</v>
+        <v>83982</v>
       </c>
       <c r="F6" s="2">
-        <v>80000</v>
+        <v>88164</v>
       </c>
       <c r="G6" s="2">
-        <v>80000</v>
+        <v>92558</v>
       </c>
       <c r="H6" s="2">
-        <v>80000</v>
+        <v>107582</v>
       </c>
       <c r="I6" s="2">
-        <v>80000</v>
+        <v>123387</v>
       </c>
       <c r="J6" s="2">
-        <v>80000</v>
+        <v>141920</v>
       </c>
     </row>
     <row r="7">
@@ -1406,13 +1406,13 @@
         <v>5536879</v>
       </c>
       <c r="H7" s="4">
-        <v>6439777</v>
+        <v>6441127</v>
       </c>
       <c r="I7" s="4">
-        <v>7672682.969999999</v>
+        <v>7676130.969999999</v>
       </c>
       <c r="J7" s="4">
-        <v>9191245.75</v>
+        <v>9197838.75</v>
       </c>
     </row>
     <row r="8">
@@ -1440,13 +1440,13 @@
         <v>31.999999768822835</v>
       </c>
       <c r="H8" s="2">
-        <v>32.29033607531571</v>
+        <v>32.29027750442234</v>
       </c>
       <c r="I8" s="2">
-        <v>33.37353131696647</v>
+        <v>33.373591591998704</v>
       </c>
       <c r="J8" s="2">
-        <v>34.52265280994758</v>
+        <v>34.52299697258824</v>
       </c>
     </row>
     <row r="9">
@@ -1465,22 +1465,22 @@
         <v>3640000</v>
       </c>
       <c r="E9" s="2">
-        <v>3827340</v>
+        <v>3842514</v>
       </c>
       <c r="F9" s="2">
-        <v>4027695</v>
+        <v>4059082</v>
       </c>
       <c r="G9" s="2">
-        <v>4239729</v>
+        <v>4288284</v>
       </c>
       <c r="H9" s="2">
-        <v>4617707</v>
+        <v>4701324</v>
       </c>
       <c r="I9" s="2">
-        <v>5071007.17</v>
+        <v>5194247.17</v>
       </c>
       <c r="J9" s="2">
-        <v>5578994.98</v>
+        <v>5747021.98</v>
       </c>
     </row>
     <row r="10">
@@ -1703,22 +1703,22 @@
         <v>270000</v>
       </c>
       <c r="E16" s="2">
-        <v>270000</v>
+        <v>285174</v>
       </c>
       <c r="F16" s="2">
-        <v>270000</v>
+        <v>301387</v>
       </c>
       <c r="G16" s="2">
-        <v>270000</v>
+        <v>318555</v>
       </c>
       <c r="H16" s="2">
-        <v>270000</v>
+        <v>352862</v>
       </c>
       <c r="I16" s="2">
-        <v>270000</v>
+        <v>391446</v>
       </c>
       <c r="J16" s="2">
-        <v>270000</v>
+        <v>434839</v>
       </c>
     </row>
     <row r="17">
@@ -1746,13 +1746,13 @@
         <v>78580</v>
       </c>
       <c r="H17" s="2">
-        <v>90871</v>
+        <v>90892</v>
       </c>
       <c r="I17" s="2">
-        <v>105552</v>
+        <v>105604</v>
       </c>
       <c r="J17" s="2">
-        <v>123132</v>
+        <v>123226</v>
       </c>
     </row>
     <row r="18">
@@ -1771,22 +1771,22 @@
         <v>1160000</v>
       </c>
       <c r="E18" s="4">
-        <v>1206541</v>
+        <v>1191367</v>
       </c>
       <c r="F18" s="4">
-        <v>1251620</v>
+        <v>1220233</v>
       </c>
       <c r="G18" s="4">
-        <v>1297150</v>
+        <v>1248595</v>
       </c>
       <c r="H18" s="4">
-        <v>1822070</v>
+        <v>1739803</v>
       </c>
       <c r="I18" s="4">
-        <v>2601675.799999999</v>
+        <v>2481883.799999999</v>
       </c>
       <c r="J18" s="4">
-        <v>3612250.7699999996</v>
+        <v>3450816.7699999996</v>
       </c>
     </row>
     <row r="19">
@@ -1805,22 +1805,22 @@
         <v>7.733333333333333</v>
       </c>
       <c r="E19" s="2">
-        <v>7.669889754405316</v>
+        <v>7.573429785673756</v>
       </c>
       <c r="F19" s="2">
-        <v>7.586560171231915</v>
+        <v>7.396311242567899</v>
       </c>
       <c r="G19" s="2">
-        <v>7.496786492919304</v>
+        <v>7.2161663116267025</v>
       </c>
       <c r="H19" s="2">
-        <v>9.136225160087141</v>
+        <v>8.721877657904665</v>
       </c>
       <c r="I19" s="2">
-        <v>11.316394685846609</v>
+        <v>10.790511084778661</v>
       </c>
       <c r="J19" s="2">
-        <v>13.5677450681999</v>
+        <v>12.95223151239379</v>
       </c>
     </row>
     <row r="20">
@@ -1839,22 +1839,22 @@
         <v>1130000</v>
       </c>
       <c r="E20" s="4">
-        <v>1170049</v>
+        <v>1154875</v>
       </c>
       <c r="F20" s="4">
-        <v>1213573</v>
+        <v>1182186</v>
       </c>
       <c r="G20" s="4">
-        <v>1257482</v>
+        <v>1208927</v>
       </c>
       <c r="H20" s="4">
-        <v>1667240</v>
+        <v>1584973</v>
       </c>
       <c r="I20" s="4">
-        <v>2435933</v>
+        <v>2316141</v>
       </c>
       <c r="J20" s="4">
-        <v>3434785</v>
+        <v>3273351</v>
       </c>
     </row>
     <row r="21">
@@ -1873,22 +1873,22 @@
         <v>1130000</v>
       </c>
       <c r="E21" s="2">
-        <v>1170049</v>
+        <v>1154875</v>
       </c>
       <c r="F21" s="2">
-        <v>1213573</v>
+        <v>1182186</v>
       </c>
       <c r="G21" s="2">
-        <v>1257482</v>
+        <v>1208927</v>
       </c>
       <c r="H21" s="2">
-        <v>1667240</v>
+        <v>1584973</v>
       </c>
       <c r="I21" s="2">
-        <v>2435933</v>
+        <v>2316141</v>
       </c>
       <c r="J21" s="2">
-        <v>3434785</v>
+        <v>3273351</v>
       </c>
     </row>
     <row r="22">
@@ -1907,22 +1907,22 @@
         <v>791000</v>
       </c>
       <c r="E22" s="2">
-        <v>819035</v>
+        <v>808413</v>
       </c>
       <c r="F22" s="2">
-        <v>849501</v>
+        <v>827530</v>
       </c>
       <c r="G22" s="2">
-        <v>880237</v>
+        <v>846249</v>
       </c>
       <c r="H22" s="2">
-        <v>1167068</v>
+        <v>1109481</v>
       </c>
       <c r="I22" s="2">
-        <v>1705153</v>
+        <v>1621299</v>
       </c>
       <c r="J22" s="2">
-        <v>2404350</v>
+        <v>2291346</v>
       </c>
     </row>
     <row r="23">
@@ -2009,22 +2009,22 @@
         <v>350000</v>
       </c>
       <c r="E25" s="2">
-        <v>350000</v>
+        <v>369156</v>
       </c>
       <c r="F25" s="2">
-        <v>350000</v>
+        <v>389551</v>
       </c>
       <c r="G25" s="2">
-        <v>350000</v>
+        <v>411113</v>
       </c>
       <c r="H25" s="2">
-        <v>350000</v>
+        <v>460444</v>
       </c>
       <c r="I25" s="2">
-        <v>350000</v>
+        <v>514833</v>
       </c>
       <c r="J25" s="2">
-        <v>350000</v>
+        <v>576759</v>
       </c>
     </row>
     <row r="26">
@@ -2043,22 +2043,22 @@
         <v>3010000</v>
       </c>
       <c r="E26" s="4">
-        <v>3154361</v>
+        <v>3158343</v>
       </c>
       <c r="F26" s="4">
-        <v>3303731</v>
+        <v>3311895</v>
       </c>
       <c r="G26" s="4">
-        <v>3460459</v>
+        <v>3473017</v>
       </c>
       <c r="H26" s="4">
-        <v>4107834</v>
+        <v>4136011</v>
       </c>
       <c r="I26" s="4">
-        <v>5049472.969999999</v>
+        <v>5094513.969999999</v>
       </c>
       <c r="J26" s="4">
-        <v>6236279.75</v>
+        <v>6301604.75</v>
       </c>
     </row>
     <row r="27">
@@ -2079,22 +2079,22 @@
         <v>4.735724973033162</v>
       </c>
       <c r="E27" s="2">
-        <v>4.796046511627905</v>
+        <v>4.928338870431892</v>
       </c>
       <c r="F27" s="2">
-        <v>4.735348934380057</v>
+        <v>4.8617898689281125</v>
       </c>
       <c r="G27" s="2">
-        <v>4.7439697723573815</v>
+        <v>4.864948918972378</v>
       </c>
       <c r="H27" s="2">
-        <v>18.707778361194283</v>
+        <v>19.089857607952965</v>
       </c>
       <c r="I27" s="2">
-        <v>22.92300443494062</v>
+        <v>23.174574970907933</v>
       </c>
       <c r="J27" s="2">
-        <v>23.503577245607097</v>
+        <v>23.693934045684873</v>
       </c>
     </row>
     <row r="28">
@@ -2113,22 +2113,22 @@
         <v>20.066666666666666</v>
       </c>
       <c r="E28" s="2">
-        <v>20.05203396784337</v>
+        <v>20.0773472402494</v>
       </c>
       <c r="F28" s="2">
-        <v>20.025210543986343</v>
+        <v>20.074695752945882</v>
       </c>
       <c r="G28" s="2">
-        <v>19.99947753960686</v>
+        <v>20.072055610591775</v>
       </c>
       <c r="H28" s="2">
-        <v>20.597505224421344</v>
+        <v>20.73440609870654</v>
       </c>
       <c r="I28" s="2">
-        <v>21.963470269444834</v>
+        <v>22.149469473488143</v>
       </c>
       <c r="J28" s="2">
-        <v>23.423693206653372</v>
+        <v>23.652326119187254</v>
       </c>
     </row>
     <row r="29">
@@ -2355,22 +2355,22 @@
         <v>12808.510638297872</v>
       </c>
       <c r="E35" s="2">
-        <v>12874.942857142858</v>
+        <v>12891.195918367346</v>
       </c>
       <c r="F35" s="2">
-        <v>12854.984435797665</v>
+        <v>12886.750972762646</v>
       </c>
       <c r="G35" s="2">
-        <v>12912.160447761195</v>
+        <v>12959.018656716418</v>
       </c>
       <c r="H35" s="2">
-        <v>14883.45652173913</v>
+        <v>14985.547101449276</v>
       </c>
       <c r="I35" s="2">
-        <v>17655.49989510489</v>
+        <v>17812.985909090905</v>
       </c>
       <c r="J35" s="2">
-        <v>21068.51266891892</v>
+        <v>21289.205236486487</v>
       </c>
     </row>
     <row r="36">
@@ -2389,22 +2389,22 @@
         <v>1510000</v>
       </c>
       <c r="E36" s="4">
-        <v>1556541</v>
+        <v>1560523</v>
       </c>
       <c r="F36" s="4">
-        <v>1601620</v>
+        <v>1609784</v>
       </c>
       <c r="G36" s="4">
-        <v>1647150</v>
+        <v>1659708</v>
       </c>
       <c r="H36" s="4">
-        <v>2172070</v>
+        <v>2200247</v>
       </c>
       <c r="I36" s="4">
-        <v>2951675.799999999</v>
+        <v>2996716.799999999</v>
       </c>
       <c r="J36" s="4">
-        <v>3962250.7699999996</v>
+        <v>4027575.7699999996</v>
       </c>
     </row>
     <row r="37">
@@ -2423,22 +2423,22 @@
         <v>10.066666666666666</v>
       </c>
       <c r="E37" s="2">
-        <v>9.894813245643377</v>
+        <v>9.920126518049406</v>
       </c>
       <c r="F37" s="2">
-        <v>9.708047571506096</v>
+        <v>9.757532780465635</v>
       </c>
       <c r="G37" s="2">
-        <v>9.519586687593593</v>
+        <v>9.592164758578507</v>
       </c>
       <c r="H37" s="2">
-        <v>10.891195499333438</v>
+        <v>11.030148327811693</v>
       </c>
       <c r="I37" s="2">
-        <v>12.838774276741951</v>
+        <v>13.028855681455529</v>
       </c>
       <c r="J37" s="2">
-        <v>14.88235777817794</v>
+        <v>15.117028020803227</v>
       </c>
     </row>
     <row r="38">
@@ -2459,22 +2459,22 @@
         <v>3.0486007228415657</v>
       </c>
       <c r="E38" s="2">
-        <v>3.0821854304635687</v>
+        <v>3.345894039735109</v>
       </c>
       <c r="F38" s="2">
-        <v>2.896101034280507</v>
+        <v>3.156698106980804</v>
       </c>
       <c r="G38" s="2">
-        <v>2.8427467189470645</v>
+        <v>3.1012856383216603</v>
       </c>
       <c r="H38" s="2">
-        <v>31.868378714749724</v>
+        <v>32.568319246518065</v>
       </c>
       <c r="I38" s="2">
-        <v>35.89229628879358</v>
+        <v>36.1991085546304</v>
       </c>
       <c r="J38" s="2">
-        <v>34.23732951972573</v>
+        <v>34.3996126026991</v>
       </c>
     </row>
   </sheetData>
@@ -2636,13 +2636,13 @@
         <v>9369129</v>
       </c>
       <c r="H3" s="4">
-        <v>11430357</v>
+        <v>11434574</v>
       </c>
       <c r="I3" s="4">
-        <v>13945060</v>
+        <v>13955350</v>
       </c>
       <c r="J3" s="4">
-        <v>17013004</v>
+        <v>17031836</v>
       </c>
     </row>
     <row r="4">
@@ -2672,13 +2672,13 @@
         <v>5.407063784852406</v>
       </c>
       <c r="H4" s="2">
-        <v>22.000209411141626</v>
+        <v>22.045218931236832</v>
       </c>
       <c r="I4" s="2">
-        <v>22.000213991566486</v>
+        <v>22.04521130389292</v>
       </c>
       <c r="J4" s="2">
-        <v>22.0002208667442</v>
+        <v>22.045208468436826</v>
       </c>
     </row>
     <row r="5">
@@ -2706,13 +2706,13 @@
         <v>54.14821704322441</v>
       </c>
       <c r="H5" s="2">
-        <v>57.3141071485608</v>
+        <v>57.32313112361433</v>
       </c>
       <c r="I5" s="2">
-        <v>60.6562135366029</v>
+        <v>60.673815134683565</v>
       </c>
       <c r="J5" s="2">
-        <v>63.90146083802072</v>
+        <v>63.92697661345926</v>
       </c>
     </row>
     <row r="6">
@@ -2740,13 +2740,13 @@
         <v>2998121</v>
       </c>
       <c r="H6" s="4">
-        <v>3658685</v>
+        <v>3660035</v>
       </c>
       <c r="I6" s="4">
-        <v>4672923</v>
+        <v>4676371</v>
       </c>
       <c r="J6" s="4">
-        <v>5956346</v>
+        <v>5962939</v>
       </c>
     </row>
     <row r="7">
@@ -2774,13 +2774,13 @@
         <v>31.99999701146179</v>
       </c>
       <c r="H7" s="2">
-        <v>32.00849282310255</v>
+        <v>32.00849458842979</v>
       </c>
       <c r="I7" s="2">
-        <v>33.50952236849465</v>
+        <v>33.50952143801481</v>
       </c>
       <c r="J7" s="2">
-        <v>35.01054840168144</v>
+        <v>35.01054730682001</v>
       </c>
     </row>
     <row r="8">
@@ -2799,22 +2799,22 @@
         <v>730000</v>
       </c>
       <c r="E8" s="4">
-        <v>766054</v>
+        <v>756914</v>
       </c>
       <c r="F8" s="4">
-        <v>803213</v>
+        <v>784364</v>
       </c>
       <c r="G8" s="4">
-        <v>841473</v>
+        <v>812308</v>
       </c>
       <c r="H8" s="4">
-        <v>1240472</v>
+        <v>1185861</v>
       </c>
       <c r="I8" s="4">
-        <v>1924807.83</v>
+        <v>1841433.83</v>
       </c>
       <c r="J8" s="4">
-        <v>2831051.0199999996</v>
+        <v>2715324.0199999996</v>
       </c>
     </row>
     <row r="9">
@@ -2833,22 +2833,22 @@
         <v>9.125</v>
       </c>
       <c r="E9" s="2">
-        <v>9.084470847900866</v>
+        <v>8.976081539118699</v>
       </c>
       <c r="F9" s="2">
-        <v>9.036520248981805</v>
+        <v>8.824460222347453</v>
       </c>
       <c r="G9" s="2">
-        <v>8.981336472152321</v>
+        <v>8.670048197649963</v>
       </c>
       <c r="H9" s="2">
-        <v>10.852434442773747</v>
+        <v>10.370836727279913</v>
       </c>
       <c r="I9" s="2">
-        <v>13.802793462344374</v>
+        <v>13.195181991136016</v>
       </c>
       <c r="J9" s="2">
-        <v>16.640512281076283</v>
+        <v>15.94263836265215</v>
       </c>
     </row>
     <row r="10">
@@ -2935,22 +2935,22 @@
         <v>50000</v>
       </c>
       <c r="E12" s="2">
-        <v>50000</v>
+        <v>52704</v>
       </c>
       <c r="F12" s="2">
-        <v>50000</v>
+        <v>55553</v>
       </c>
       <c r="G12" s="2">
-        <v>50000</v>
+        <v>58557</v>
       </c>
       <c r="H12" s="2">
-        <v>50000</v>
+        <v>71457</v>
       </c>
       <c r="I12" s="2">
-        <v>50000</v>
+        <v>85285</v>
       </c>
       <c r="J12" s="2">
-        <v>50000</v>
+        <v>101736</v>
       </c>
     </row>
     <row r="13">
@@ -2969,22 +2969,22 @@
         <v>150000</v>
       </c>
       <c r="E13" s="2">
-        <v>150000</v>
+        <v>159140</v>
       </c>
       <c r="F13" s="2">
-        <v>150000</v>
+        <v>168849</v>
       </c>
       <c r="G13" s="2">
-        <v>150000</v>
+        <v>179165</v>
       </c>
       <c r="H13" s="2">
-        <v>150000</v>
+        <v>205206</v>
       </c>
       <c r="I13" s="2">
-        <v>150000</v>
+        <v>235028</v>
       </c>
       <c r="J13" s="2">
-        <v>150000</v>
+        <v>269132</v>
       </c>
     </row>
     <row r="14">
@@ -3003,22 +3003,22 @@
         <v>200000</v>
       </c>
       <c r="E14" s="2">
-        <v>200000</v>
+        <v>211844</v>
       </c>
       <c r="F14" s="2">
-        <v>200000</v>
+        <v>224402</v>
       </c>
       <c r="G14" s="2">
-        <v>200000</v>
+        <v>237722</v>
       </c>
       <c r="H14" s="2">
-        <v>200000</v>
+        <v>276663</v>
       </c>
       <c r="I14" s="2">
-        <v>200000</v>
+        <v>320313</v>
       </c>
       <c r="J14" s="2">
-        <v>200000</v>
+        <v>370868</v>
       </c>
     </row>
     <row r="15">
@@ -3037,22 +3037,22 @@
         <v>1570000</v>
       </c>
       <c r="E15" s="4">
-        <v>1652187</v>
+        <v>1654891</v>
       </c>
       <c r="F15" s="4">
-        <v>1738819</v>
+        <v>1744372</v>
       </c>
       <c r="G15" s="4">
-        <v>1830134</v>
+        <v>1838691</v>
       </c>
       <c r="H15" s="4">
-        <v>2279835</v>
+        <v>2301887</v>
       </c>
       <c r="I15" s="4">
-        <v>3049382</v>
+        <v>3086321</v>
       </c>
       <c r="J15" s="4">
-        <v>4049604.9999999995</v>
+        <v>4104745.9999999995</v>
       </c>
     </row>
     <row r="16">
@@ -3073,22 +3073,22 @@
         <v>5.263157894736836</v>
       </c>
       <c r="E16" s="2">
-        <v>5.234840764331206</v>
+        <v>5.407070063694275</v>
       </c>
       <c r="F16" s="2">
-        <v>5.243474255638136</v>
+        <v>5.407063063367912</v>
       </c>
       <c r="G16" s="2">
-        <v>5.251552921839475</v>
+        <v>5.40704620344743</v>
       </c>
       <c r="H16" s="2">
-        <v>24.57202587351528</v>
+        <v>25.191617297305523</v>
       </c>
       <c r="I16" s="2">
-        <v>33.75450416367851</v>
+        <v>34.07786741920869</v>
       </c>
       <c r="J16" s="2">
-        <v>32.80084292489427</v>
+        <v>32.998025804833645</v>
       </c>
     </row>
     <row r="17">
@@ -3315,22 +3315,22 @@
         <v>15392.156862745098</v>
       </c>
       <c r="E23" s="2">
-        <v>15441</v>
+        <v>15466.271028037383</v>
       </c>
       <c r="F23" s="2">
-        <v>15387.778761061947</v>
+        <v>15436.920353982301</v>
       </c>
       <c r="G23" s="2">
-        <v>15509.610169491525</v>
+        <v>15582.127118644068</v>
       </c>
       <c r="H23" s="2">
-        <v>18998.625</v>
+        <v>19182.391666666666</v>
       </c>
       <c r="I23" s="2">
-        <v>24791.72357723577</v>
+        <v>25092.040650406503</v>
       </c>
       <c r="J23" s="2">
-        <v>32396.839999999997</v>
+        <v>32837.96799999999</v>
       </c>
     </row>
     <row r="24">
@@ -3658,17 +3658,17 @@
       </c>
       <c r="J4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.26 % / 補助 22 % / ベース 7.3 %</t>
+          <t xml:space="preserve">全社 15.29 % / 補助 22.05 % / ベース 7.3 %</t>
         </is>
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.28 % / 補助 22 % / ベース 6.25 %</t>
+          <t xml:space="preserve">全社 15.31 % / 補助 22.05 % / ベース 6.25 %</t>
         </is>
       </c>
       <c r="L4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15.8 % / 補助 22 % / ベース 6.25 %</t>
+          <t xml:space="preserve">全社 15.83 % / 補助 22.05 % / ベース 6.25 %</t>
         </is>
       </c>
     </row>
@@ -3829,32 +3829,32 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.33 % / 補助 22.92 % / ベース 25.96 %</t>
+          <t xml:space="preserve">全社 24.43 % / 補助 23.02 % / ベース 26.05 %</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.41 % / 補助 22.96 % / ベース 26.11 %</t>
+          <t xml:space="preserve">全社 24.6 % / 補助 23.18 % / ベース 26.27 %</t>
         </is>
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 24.5 % / 補助 23.02 % / ベース 26.26 %</t>
+          <t xml:space="preserve">全社 24.78 % / 補助 23.33 % / ベース 26.5 %</t>
         </is>
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 23.15 % / 補助 21.16 % / ベース 25.84 %</t>
+          <t xml:space="preserve">全社 23.57 % / 補助 21.64 % / ベース 26.16 %</t>
         </is>
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 22.06 % / 補助 19.71 % / ベース 25.68 %</t>
+          <t xml:space="preserve">全社 22.58 % / 補助 20.31 % / ベース 26.08 %</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 20.95 % / 補助 18.37 % / ベース 25.53 %</t>
+          <t xml:space="preserve">全社 21.57 % / 補助 19.07 % / ベース 26.01 %</t>
         </is>
       </c>
     </row>
@@ -3891,32 +3891,32 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.67 % / 補助 9.08 % / ベース 6.04 %</t>
+          <t xml:space="preserve">全社 7.57 % / 補助 8.98 % / ベース 5.95 %</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.59 % / 補助 9.04 % / ベース 5.89 %</t>
+          <t xml:space="preserve">全社 7.4 % / 補助 8.82 % / ベース 5.73 %</t>
         </is>
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7.5 % / 補助 8.98 % / ベース 5.74 %</t>
+          <t xml:space="preserve">全社 7.22 % / 補助 8.67 % / ベース 5.5 %</t>
         </is>
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.14 % / 補助 10.85 % / ベース 6.83 %</t>
+          <t xml:space="preserve">全社 8.72 % / 補助 10.37 % / ベース 6.51 %</t>
         </is>
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.32 % / 補助 13.8 % / ベース 7.48 %</t>
+          <t xml:space="preserve">全社 10.79 % / 補助 13.2 % / ベース 7.08 %</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.57 % / 補助 16.64 % / ベース 8.13 %</t>
+          <t xml:space="preserve">全社 12.95 % / 補助 15.94 % / ベース 7.65 %</t>
         </is>
       </c>
     </row>
@@ -3953,32 +3953,32 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.89 % / 補助 11.46 % / ベース 8.09 %</t>
+          <t xml:space="preserve">全社 9.92 % / 補助 11.49 % / ベース 8.11 %</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.71 % / 補助 11.29 % / ベース 7.86 %</t>
+          <t xml:space="preserve">全社 9.76 % / 補助 11.35 % / ベース 7.9 %</t>
         </is>
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.52 % / 補助 11.12 % / ベース 7.63 %</t>
+          <t xml:space="preserve">全社 9.59 % / 補助 11.21 % / ベース 7.68 %</t>
         </is>
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.89 % / 補助 12.6 % / ベース 8.59 %</t>
+          <t xml:space="preserve">全社 11.03 % / 補助 12.79 % / ベース 8.67 %</t>
         </is>
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.84 % / 補助 15.24 % / ベース 9.14 %</t>
+          <t xml:space="preserve">全社 13.03 % / 補助 15.49 % / ベース 9.23 %</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 14.88 % / 補助 17.82 % / ベース 9.69 %</t>
+          <t xml:space="preserve">全社 15.12 % / 補助 18.12 % / ベース 9.8 %</t>
         </is>
       </c>
     </row>
@@ -4040,7 +4040,7 @@
       </c>
       <c r="L10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.94 % / 補助 11 % / ベース 10.82 %</t>
+          <t xml:space="preserve">全社 10.94 % / 補助 11.01 % / ベース 10.82 %</t>
         </is>
       </c>
     </row>
@@ -4154,17 +4154,17 @@
       </c>
       <c r="J12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.11 % / 補助 6.91 % / ベース 12.05 %</t>
+          <t xml:space="preserve">全社 9.1 % / 補助 6.91 % / ベース 12.05 %</t>
         </is>
       </c>
       <c r="K12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.58 % / 補助 6.26 % / ベース 12.16 %</t>
+          <t xml:space="preserve">全社 8.57 % / 補助 6.25 % / ベース 12.16 %</t>
         </is>
       </c>
       <c r="L12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.05 % / 補助 5.66 % / ベース 12.26 %</t>
+          <t xml:space="preserve">全社 8.04 % / 補助 5.66 % / ベース 12.26 %</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
       </c>
       <c r="L13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.5 % / 補助 0.32 % / ベース 0.8 %</t>
+          <t xml:space="preserve">全社 0.49 % / 補助 0.32 % / ベース 0.8 %</t>
         </is>
       </c>
     </row>
@@ -4278,7 +4278,7 @@
       </c>
       <c r="J14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.71 % / 補助 7.34 % / ベース 12.88 %</t>
+          <t xml:space="preserve">全社 9.7 % / 補助 7.34 % / ベース 12.88 %</t>
         </is>
       </c>
       <c r="K14" s="0" t="inlineStr">
@@ -4288,7 +4288,7 @@
       </c>
       <c r="L14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.54 % / 補助 5.99 % / ベース 13.06 %</t>
+          <t xml:space="preserve">全社 8.54 % / 補助 5.98 % / ベース 13.06 %</t>
         </is>
       </c>
     </row>
@@ -4511,32 +4511,32 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 50.65 % / 補助 41.53 % / ベース 60.69 %</t>
+          <t xml:space="preserve">全社 50.59 % / 補助 41.46 % / ベース 60.64 %</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 51.52 % / 補助 42.3 % / ベース 61.76 %</t>
+          <t xml:space="preserve">全社 51.39 % / 補助 42.17 % / ベース 61.66 %</t>
         </is>
       </c>
       <c r="I18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 52.4 % / 補助 43.09 % / ベース 62.85 %</t>
+          <t xml:space="preserve">全社 52.21 % / 補助 42.89 % / ベース 62.7 %</t>
         </is>
       </c>
       <c r="J18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 47.12 % / 補助 36.82 % / ベース 59.98 %</t>
+          <t xml:space="preserve">全社 46.8 % / 補助 36.46 % / ベース 59.78 %</t>
         </is>
       </c>
       <c r="K18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 41.54 % / 補助 30.32 % / ベース 58.66 %</t>
+          <t xml:space="preserve">全社 41.18 % / 補助 29.96 % / ベース 58.42 %</t>
         </is>
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 36.46 % / 補助 25.15 % / ベース 57.41 %</t>
+          <t xml:space="preserve">全社 36.09 % / 補助 24.81 % / ベース 57.15 %</t>
         </is>
       </c>
     </row>
@@ -4650,17 +4650,17 @@
       </c>
       <c r="J20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 73,591.72 千円/人 / 補助 96,867.43 千円/人 / ベース 55,640.52 千円/人</t>
+          <t xml:space="preserve">全社 73,607.28 千円/人 / 補助 96,903.17 千円/人 / ベース 55,640.52 千円/人</t>
         </is>
       </c>
       <c r="K20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 81,816.1 千円/人 / 補助 115,248.43 千円/人 / ベース 56,532.9 千円/人</t>
+          <t xml:space="preserve">全社 81,852.72 千円/人 / 補助 115,333.47 千円/人 / ベース 56,532.9 千円/人</t>
         </is>
       </c>
       <c r="L20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 91,490.76 千円/人 / 補助 138,317.11 千円/人 / ベース 57,207.18 千円/人</t>
+          <t xml:space="preserve">全社 91,555.47 千円/人 / 補助 138,470.21 千円/人 / ベース 57,207.18 千円/人</t>
         </is>
       </c>
     </row>
@@ -4697,32 +4697,32 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5,027.25 千円/人 / 補助 7,295.75 千円/人 / ベース 3,262.87 千円/人</t>
+          <t xml:space="preserve">全社 4,964.03 千円/人 / 補助 7,208.7 千円/人 / ベース 3,218.17 千円/人</t>
         </is>
       </c>
       <c r="H21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4,966.75 千円/人 / 補助 7,236.15 千円/人 / ベース 3,180.19 千円/人</t>
+          <t xml:space="preserve">全社 4,842.19 千円/人 / 補助 7,066.34 千円/人 / ベース 3,091.27 千円/人</t>
         </is>
       </c>
       <c r="I21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4,932.13 千円/人 / 補助 7,254.08 千円/人 / ベース 3,099.84 千円/人</t>
+          <t xml:space="preserve">全社 4,747.51 千円/人 / 補助 7,002.66 千円/人 / ベース 2,967.94 千円/人</t>
         </is>
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6,723.51 千円/人 / 補助 10,512.47 千円/人 / ベース 3,801.29 千円/人</t>
+          <t xml:space="preserve">全社 6,419.94 千円/人 / 補助 10,049.67 千円/人 / ベース 3,620.54 千円/人</t>
         </is>
       </c>
       <c r="K21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9,258.63 千円/人 / 補助 15,907.5 千円/人 / ベース 4,230.42 千円/人</t>
+          <t xml:space="preserve">全社 8,832.33 千円/人 / 補助 15,218.46 千円/人 / ベース 4,002.81 千円/人</t>
         </is>
       </c>
       <c r="L21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12,413.23 千円/人 / 補助 23,016.67 千円/人 / ベース 4,650 千円/人</t>
+          <t xml:space="preserve">全社 11,858.48 千円/人 / 補助 22,075.81 千円/人 / ベース 4,377.93 千円/人</t>
         </is>
       </c>
     </row>
@@ -4759,32 +4759,32 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12,874.94 千円/人 / 補助 15,441 千円/人 / ベース 10,885.32 千円/人</t>
+          <t xml:space="preserve">全社 12,891.2 千円/人 / 補助 15,466.27 千円/人 / ベース 10,894.58 千円/人</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12,854.98 千円/人 / 補助 15,387.78 千円/人 / ベース 10,867.44 千円/人</t>
+          <t xml:space="preserve">全社 12,886.75 千円/人 / 補助 15,436.92 千円/人 / ベース 10,885.58 千円/人</t>
         </is>
       </c>
       <c r="I22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12,912.16 千円/人 / 補助 15,509.61 千円/人 / ベース 10,868.83 千円/人</t>
+          <t xml:space="preserve">全社 12,959.02 千円/人 / 補助 15,582.13 千円/人 / ベース 10,895.51 千円/人</t>
         </is>
       </c>
       <c r="J22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 14,883.46 千円/人 / 補助 18,998.63 千円/人 / ベース 11,717.94 千円/人</t>
+          <t xml:space="preserve">全社 14,985.55 千円/人 / 補助 19,182.39 千円/人 / ベース 11,757.21 千円/人</t>
         </is>
       </c>
       <c r="K22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 17,655.5 千円/人 / 補助 24,791.72 千円/人 / ベース 12,270.5 千円/人</t>
+          <t xml:space="preserve">全社 17,812.99 千円/人 / 補助 25,092.04 千円/人 / ベース 12,320.2 千円/人</t>
         </is>
       </c>
       <c r="L22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 21,068.51 千円/人 / 補助 32,396.84 千円/人 / ベース 12,787.57 千円/人</t>
+          <t xml:space="preserve">全社 21,289.21 千円/人 / 補助 32,837.97 千円/人 / ベース 12,847.13 千円/人</t>
         </is>
       </c>
     </row>
@@ -4898,17 +4898,17 @@
       </c>
       <c r="J24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.22 pt / 補助 20.28 pt / ベース 3.22 pt</t>
+          <t xml:space="preserve">全社 12.24 pt / 補助 20.32 pt / ベース 3.22 pt</t>
         </is>
       </c>
       <c r="K24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.59 pt / 補助 19.46 pt / ベース 1.68 pt</t>
+          <t xml:space="preserve">全社 11.62 pt / 補助 19.5 pt / ベース 1.68 pt</t>
         </is>
       </c>
       <c r="L24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.25 pt / 補助 20.35 pt / ベース 1.25 pt</t>
+          <t xml:space="preserve">全社 12.28 pt / 補助 20.39 pt / ベース 1.25 pt</t>
         </is>
       </c>
     </row>
@@ -5007,32 +5007,32 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.22 % / 補助 2.37 % / ベース 2.06 %</t>
+          <t xml:space="preserve">全社 2.35 % / 補助 2.51 % / ベース 2.16 %</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.12 % / 補助 2.25 % / ベース 1.97 %</t>
+          <t xml:space="preserve">全社 2.36 % / 補助 2.52 % / ベース 2.17 %</t>
         </is>
       </c>
       <c r="I26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 2.02 % / 補助 2.13 % / ベース 1.89 %</t>
+          <t xml:space="preserve">全社 2.38 % / 補助 2.54 % / ベース 2.19 %</t>
         </is>
       </c>
       <c r="J26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.75 % / 補助 1.75 % / ベース 1.76 %</t>
+          <t xml:space="preserve">全社 2.31 % / 補助 2.42 % / ベース 2.16 %</t>
         </is>
       </c>
       <c r="K26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.52 % / 補助 1.43 % / ベース 1.66 %</t>
+          <t xml:space="preserve">全社 2.24 % / 補助 2.3 % / ベース 2.15 %</t>
         </is>
       </c>
       <c r="L26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 1.31 % / 補助 1.18 % / ベース 1.56 %</t>
+          <t xml:space="preserve">全社 2.16 % / 補助 2.18 % / ベース 2.14 %</t>
         </is>
       </c>
     </row>
@@ -5193,32 +5193,32 @@
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.45 倍 / 補助 4.83 倍 / ベース 3.94 倍</t>
+          <t xml:space="preserve">全社 4.23 倍 / 補助 4.57 倍 / ベース 3.76 倍</t>
         </is>
       </c>
       <c r="H29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.58 倍 / 補助 5.02 倍 / ベース 3.99 倍</t>
+          <t xml:space="preserve">全社 4.13 倍 / 補助 4.5 倍 / ベース 3.64 倍</t>
         </is>
       </c>
       <c r="I29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.71 倍 / 補助 5.21 倍 / ベース 4.04 倍</t>
+          <t xml:space="preserve">全社 4.04 倍 / 補助 4.42 倍 / ベース 3.52 倍</t>
         </is>
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6.21 倍 / 補助 7.2 倍 / ベース 4.88 倍</t>
+          <t xml:space="preserve">全社 4.78 倍 / 補助 5.29 倍 / ベース 4.01 倍</t>
         </is>
       </c>
       <c r="K29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.43 倍 / 補助 10.62 倍 / ベース 5.51 倍</t>
+          <t xml:space="preserve">全社 5.82 倍 / 補助 6.75 倍 / ベース 4.29 倍</t>
         </is>
       </c>
       <c r="L29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.32 倍 / 補助 15.16 倍 / ベース 6.21 倍</t>
+          <t xml:space="preserve">全社 6.98 倍 / 補助 8.32 倍 / ベース 4.57 倍</t>
         </is>
       </c>
     </row>
@@ -5394,17 +5394,17 @@
       </c>
       <c r="J32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 57.31 %</t>
+          <t xml:space="preserve">構成比 57.32 %</t>
         </is>
       </c>
       <c r="K32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 60.66 %</t>
+          <t xml:space="preserve">構成比 60.67 %</t>
         </is>
       </c>
       <c r="L32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">構成比 63.9 %</t>
+          <t xml:space="preserve">構成比 63.93 %</t>
         </is>
       </c>
     </row>
@@ -5456,17 +5456,17 @@
       </c>
       <c r="J33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 22 % / ベース 7.3 %</t>
+          <t xml:space="preserve">補助 22.05 % / ベース 7.3 %</t>
         </is>
       </c>
       <c r="K33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 22 % / ベース 6.25 %</t>
+          <t xml:space="preserve">補助 22.05 % / ベース 6.25 %</t>
         </is>
       </c>
       <c r="L33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 22 % / ベース 6.25 %</t>
+          <t xml:space="preserve">補助 22.05 % / ベース 6.25 %</t>
         </is>
       </c>
     </row>
@@ -5565,32 +5565,32 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 3.05 pt</t>
+          <t xml:space="preserve">差 3.02 pt</t>
         </is>
       </c>
       <c r="H35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 3.14 pt</t>
+          <t xml:space="preserve">差 3.1 pt</t>
         </is>
       </c>
       <c r="I35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 3.24 pt</t>
+          <t xml:space="preserve">差 3.17 pt</t>
         </is>
       </c>
       <c r="J35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 4.02 pt</t>
+          <t xml:space="preserve">差 3.86 pt</t>
         </is>
       </c>
       <c r="K35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 6.32 pt</t>
+          <t xml:space="preserve">差 6.11 pt</t>
         </is>
       </c>
       <c r="L35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 8.51 pt</t>
+          <t xml:space="preserve">差 8.29 pt</t>
         </is>
       </c>
     </row>
@@ -5642,17 +5642,17 @@
       </c>
       <c r="J36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 96,867.43 千円/人 / ベース 55,640.52 千円/人</t>
+          <t xml:space="preserve">補助 96,903.17 千円/人 / ベース 55,640.52 千円/人</t>
         </is>
       </c>
       <c r="K36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 115,248.43 千円/人 / ベース 56,532.9 千円/人</t>
+          <t xml:space="preserve">補助 115,333.47 千円/人 / ベース 56,532.9 千円/人</t>
         </is>
       </c>
       <c r="L36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 138,317.11 千円/人 / ベース 57,207.18 千円/人</t>
+          <t xml:space="preserve">補助 138,470.21 千円/人 / ベース 57,207.18 千円/人</t>
         </is>
       </c>
     </row>
@@ -5751,32 +5751,32 @@
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 77.47 %</t>
+          <t xml:space="preserve">寄与率 85.8 %</t>
         </is>
       </c>
       <c r="H38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 82.43 %</t>
+          <t xml:space="preserve">寄与率 95.09 %</t>
         </is>
       </c>
       <c r="I38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 84.03 %</t>
+          <t xml:space="preserve">寄与率 98.53 %</t>
         </is>
       </c>
       <c r="J38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 76.01 %</t>
+          <t xml:space="preserve">寄与率 76.05 %</t>
         </is>
       </c>
       <c r="K38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 87.78 %</t>
+          <t xml:space="preserve">寄与率 88.34 %</t>
         </is>
       </c>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 89.68 %</t>
+          <t xml:space="preserve">寄与率 90.19 %</t>
         </is>
       </c>
     </row>
@@ -6635,7 +6635,7 @@
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">—</t>
+          <t xml:space="preserve">制度下限5.0%/年（基準年→事業化報告3年目）</t>
         </is>
       </c>
       <c r="D37" s="2">
@@ -11401,14 +11401,14 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsIm1vbmV5VW5pdCI6IuWNg+WGhiIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MjAwMDAwLCJjb2dzIjo0ODk2MDAwLCJlbXBsb3llZVBheSI6NTE5MDMxLCJvZmZpY2VyUGF5IjozNjAwMCwiZGVwcmVjaWF0aW9uIjoxODAwMDAsIm90aGVyU2dhIjo5MDAwMDAsImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQ5MzA3OSwiZW1wbG95ZWVCb251cyI6MjU5NTIsIm9mZmljZXJDb21wZW5zYXRpb24iOjMyNDAwLCJvZmZpY2VyQm9udXMiOjM2MDAsImNvZ3NEZXByZWNpYXRpb24iOjQ1MDAwLCJzZ2FEZXByZWNpYXRpb24iOjEzNTAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6MzYwMDB9LCJvdGhlciI6eyJzYWxlcyI6NjQ0MDAwMCwiY29ncyI6NDM3OTIwMCwiZW1wbG95ZWVQYXkiOjcwOTc4Niwib2ZmaWNlclBheSI6NTUyMDAsImRlcHJlY2lhdGlvbiI6MTM4MDAwLCJvdGhlclNnYSI6NzM2MDAwLCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Njc0Mjk3LCJlbXBsb3llZUJvbnVzIjozNTQ4OSwib2ZmaWNlckNvbXBlbnNhdGlvbiI6NDk2ODAsIm9mZmljZXJCb251cyI6NTUyMCwiY29nc0RlcHJlY2lhdGlvbiI6Mjc2MDAsInNnYURlcHJlY2lhdGlvbiI6MTEwNDAwLCJyZXNlYXJjaERldmVsb3BtZW50IjoyNzYwMCwib3JkaW5hcnlJbmNvbWUiOjM5NDUzNCwicHJlVGF4SW5jb21lIjozOTQ1MzQsIm5ldEluY29tZSI6NzUwNzUyLjF9fSx7InllYXIiOjIwMjQsInJvbGUiOiJwcmV2aW91cyIsInByb2plY3QiOnsic2FsZXMiOjc2MDAwMDAsImNvZ3MiOjUxNjgwMDAsImVtcGxveWVlUGF5Ijo1NTg4MjQsIm9mZmljZXJQYXkiOjM4MDAwLCJkZXByZWNpYXRpb24iOjE5MDAwMCwib3RoZXJTZ2EiOjk1MDAwMCwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NTMwODgzLCJlbXBsb3llZUJvbnVzIjoyNzk0MSwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MzQyMDAsIm9mZmljZXJCb251cyI6MzgwMCwiY29nc0RlcHJlY2lhdGlvbiI6NDc1MDAsInNnYURlcHJlY2lhdGlvbiI6MTQyNTAwLCJyZXNlYXJjaERldmVsb3BtZW50IjozODAwMH0sIm90aGVyIjp7InNhbGVzIjo2NzIwMDAwLCJjb2dzIjo0NTY5NjAwLCJlbXBsb3llZVBheSI6NzU0MTQ4LCJvZmZpY2VyUGF5Ijo1NzYwMCwiZGVwcmVjaWF0aW9uIjoxNDQwMDAsIm90aGVyU2dhIjo3NjgwMDAsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3MTY0NDEsImVtcGxveWVlQm9udXMiOjM3NzA3LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjo1MTg0MCwib2ZmaWNlckJvbnVzIjo1NzYwLCJjb2dzRGVwcmVjaWF0aW9uIjoyODgwMCwic2dhRGVwcmVjaWF0aW9uIjoxMTUyMDAsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjI4ODAwLCJvcmRpbmFyeUluY29tZSI6Mzk4MDEyLCJwcmVUYXhJbmNvbWUiOjM5ODAxMiwibmV0SW5jb21lIjo3NzE4ODEuNn19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwMDAwMDAsImNvZ3MiOjU0NDAwMDAsImVtcGxveWVlUGF5Ijo2MDAwMDAsImVtcGxveWVlU2FsYXJ5Ijo1NzAwMDAsImVtcGxveWVlQm9udXMiOjMwMDAwLCJvZmZpY2VyUGF5Ijo0MDAwMCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MzYwMDAsIm9mZmljZXJCb251cyI6NDAwMCwiZGVwcmVjaWF0aW9uIjoyMDAwMDAsImNvZ3NEZXByZWNpYXRpb24iOjUwMDAwLCJzZ2FEZXByZWNpYXRpb24iOjE1MDAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6NDAwMDAsIm90aGVyU2dhIjoxMDAwMDAwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwMDAwMDAsImNvZ3MiOjQ3NjAwMDAsImVtcGxveWVlUGF5Ijo4MDAwMDAsImVtcGxveWVlU2FsYXJ5Ijo3NjAwMDAsImVtcGxveWVlQm9udXMiOjQwMDAwLCJvZmZpY2VyUGF5Ijo2MDAwMCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6NTQwMDAsIm9mZmljZXJCb251cyI6NjAwMCwiZGVwcmVjaWF0aW9uIjoxNTAwMDAsImNvZ3NEZXByZWNpYXRpb24iOjMwMDAwLCJzZ2FEZXByZWNpYXRpb24iOjEyMDAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6MzAwMDAsIm90aGVyU2dhIjo4MDAwMDAsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjo0MDAwMDAsInByZVRheEluY29tZSI6NDAwMDAwLCJuZXRJbmNvbWUiOjc5MTAwMH19XSwiYmFsYW5jZVNoZWV0cyI6W3sieWVhciI6MjAyMywiYXNzZXRzIjoxMzIwMDAwMCwiY3VycmVudEFzc2V0cyI6NjcwMDAwMCwiY2FzaCI6MjQwMDAwMCwiZml4ZWRBc3NldHMiOjY1MDAwMDAsInRhbmdpYmxlQXNzZXRzIjo1MzAwMDAwLCJidWlsZGluZ3MiOjE5MDAwMDAsIm1hY2hpbmVyeSI6MjQwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6NzAwMDAwLCJzb2Z0d2FyZSI6NTAwMDAwLCJsaWFiaWxpdGllcyI6NzUwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjozOTAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjozNjAwMDAwLCJsb25nVGVybURlYnQiOjI5MDAwMDAsIm5ldEFzc2V0cyI6NTcwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjU0MDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4Ijo1MDAwMDB9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMwMDAwMCwiY3VycmVudEFzc2V0cyI6NzIwMDAwMCwiY2FzaCI6MjUwMDAwMCwiZml4ZWRBc3NldHMiOjcxMDAwMDAsInRhbmdpYmxlQXNzZXRzIjo1ODAwMDAwLCJidWlsZGluZ3MiOjIwMDAwMDAsIm1hY2hpbmVyeSI6MjgwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6ODAwMDAwLCJzb2Z0d2FyZSI6NjAwMDAwLCJsaWFiaWxpdGllcyI6NzkwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjo0MTAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjozODAwMDAwLCJsb25nVGVybURlYnQiOjMxMDAwMDAsIm5ldEFzc2V0cyI6NjQwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjYxMDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4Ijo4MDAwMDB9LHsieWVhciI6MjAyNSwiYXNzZXRzIjoxNTYwMDAwMCwiY3VycmVudEFzc2V0cyI6NzgwMDAwMCwiY2FzaCI6MjcwMDAwMCwiZml4ZWRBc3NldHMiOjc4MDAwMDAsInRhbmdpYmxlQXNzZXRzIjo2NDAwMDAwLCJidWlsZGluZ3MiOjIyMDAwMDAsIm1hY2hpbmVyeSI6MzIwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6OTAwMDAwLCJzb2Z0d2FyZSI6NzAwMDAwLCJsaWFiaWxpdGllcyI6ODMwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjo0MzAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMTAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjo0MDAwMDAwLCJsb25nVGVybURlYnQiOjMyMDAwMDAsIm5ldEFzc2V0cyI6NzMwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjcwMDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4IjoxMDAwMDAwfV0sImZ1dHVyZUNhcGV4IjpbeyJ5ZWFyIjoyMDI2LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI4LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI5LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMwLCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMxLCJ2YWx1ZSI6MH1dLCJkcml2ZXJzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsInByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJwcm9qZWN0Q29nc1JhdGVUb0Jhc2UiOjAuNjgsIm90aGVyQ29nc1JhdGVUb0Jhc2UiOjAuNjgsInByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwib3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwicHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yNSwib3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMiwicHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsInByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJvdGhlck5vbk9wZXJhdGluZ1JhdGUiOi0wLjAwNSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjowLCJlZmZlY3RpdmVUYXhSYXRlIjowLjMsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdEZpcnN0WWVhclNhbGVzIjowLCJwcm9qZWN0QmFzZVllYXJTYWxlcyI6MCwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6NS41NTExMTUxMjMxMjU3ODNlLTE3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5Nywib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI1NzI0NjM3NjgxMTU4NTQsIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wMTUsIm90aGVyU2dhUmF0ZUVuZCI6MC4wMDUsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJpbnZlc3RtZW50IjoyMzAwMDAwLCJzdWJzaWR5Ijo3NjYwMDAsImxvY2FsQmVuY2htYXJrIjoyM30sImRyaXZlclJhbmdlcyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjpbLTAuMDUsMC4zXSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6WzAuNjYsMC43XSwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOlswLjY2LDAuN10sInByb2plY3RDb2dzUmF0ZVRvQmFzZSI6WzAuNjgsMC42OF0sIm90aGVyQ29nc1JhdGVUb0Jhc2UiOlswLjY4LDAuNjhdLCJwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOlswLDFdLCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOlswLDFdLCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOlstMC41LDAuNV0sIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6Wy0wLjUsMC41XSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJlZmZlY3RpdmVUYXhSYXRlIjpbMCwwLjZdLCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwicHJvamVjdEZpcnN0WWVhclNhbGVzIjpbMCwxMDAwMDAwMDAwMF0sInByb2plY3RCYXNlWWVhclNhbGVzIjpbMCwxMDAwMDAwMDAwMF0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDEuNjY1MzM0NTM2OTM3NzM0OGUtMTZdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkzMjUzMzA1MDE4NDY5MjcsMC4wMjA3MzU5OTQxODMxODkxNjZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlswLjA0MDc2MDg2OTU2NTIxNzE4NCwwLjA0NDM4NDA1Nzk3MTAxNDUyXSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDAwMTM0NTc1NTY5MzU4MTk3MzddLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MTM5NDU3MDIzNzE3NDQzLDAuMDIwNTUzNDU5OTE0NzYzMDk1XSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjAzOTE2NjY2NjY2NjY2NjY4LDAuMDQyNTAwMDAwMDAwMDAwMDldLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbMC4xNSwwLjNdLCJvdGhlclNhbGVzR3Jvd3RoIjpbMC4wNjA3NjA4Njk1NjUyMTcxOSwwLjA2NDM4NDA1Nzk3MTAxNDUzXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMC4wMDUsMC4wMDUxMzQ1NzU1NjkzNTgxOTc1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLjAyNDEzOTQ1NzAyMzcxNzQ0NCwwLjAyNTU1MzQ1OTkxNDc2MzA5Nl0sIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6WzAsMC4wOF0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6WzAuMDQ0MTY2NjY2NjY2NjY2NjgsMC4wNDc1MDAwMDAwMDAwMDAwOV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMCwwLjAzXSwib3RoZXJTZ2FSYXRlRW5kIjpbMCwwLjAxXSwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOlswLjA0MjYzMTU3ODk0NzM2ODM2LDAuMDY1NTU1NTU1NTU1NTU1NThdLCJpbnZlc3RtZW50IjpbMTUwMDAwMCwyMDAwMDAwMF0sInN1YnNpZHkiOlsxMDAwMDAsNTAwMDAwMF0sImxvY2FsQmVuY2htYXJrIjpbMCwxMDBdfSwidGFyZ2V0cyI6eyJjb21wYW55U2FsZXNDYWdyIjp7InZhbHVlIjoxNSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo4MjQwMDAwLCJtYXgiOjI1MjY5MDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjoyLCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NjAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo3NDgwMDAwLCJtYXgiOjEzNjg0MDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MTg3ODAwMCwibWF4IjozMzQzMDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6Mjg1MDAwLCJtYXgiOjM3NDAwMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjoxNSwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX19LCJmb3JlY2FzdE92ZXJyaWRlcyI6eyIyMDI5Om90aGVyOnNhbGVzIjo4NTEzMDAwLCIyMDI5OnByb2plY3Q6Ny04Ijo3OTAwMDB9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2NDAwMDAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mjc1MjAwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6NzI2MDAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi03IjozMjY1MDE3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6ODIwODAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMCI6OTEyMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEyIjoxMTY3Mzc2LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjYxNDQxLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTQiOjI0NTQwMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1Ijo2MzYwMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE4IjoxMDcyNTAzLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTkiOjEwNzI1MDMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yMCI6NzUwNzUyLjEsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yNyI6MjEwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xIjo3MjAwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNCI6MjMwNDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjY3Nzk2OSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTgiOjUxOTAzMSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTkiOjM2MDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOlAyLTQiOjQ1MDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOlAyLTE0IjoxMzUwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMyI6OTAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEiOjE0MzIwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMyI6OTczNzYwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTQiOjc2MzAwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItNyI6MzQ1MTA3MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTkiOjg2MDQwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTAiOjk1NjAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMiI6MTI0NzMyNCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEzIjo2NTY0OCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjoyNTc3MDAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNSI6NjY4MDAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xOCI6MTEwMjY4OCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE5IjoxMTAyNjg4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjAiOjc3MTg4MS42LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjciOjIyMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMSI6NzYwMDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0MzIwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny02Ijo3MDQ2NzYsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny04Ijo1NTg4MjQsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjozODAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDpQMi00Ijo0NzUwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDpQMi0xNCI6MTQyNTAwLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTMiOjk1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xIjoxNTAwMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTMiOjEwMjAwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6ODAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi03IjozNjQwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItOSI6OTAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMCI6MTAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMzMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjo3MDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE0IjoyNzAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNSI6NzAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xOCI6MTEzMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE5IjoxMTMwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjAiOjc5MTAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI3IjoyMzAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwMDAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNTYwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6NzMwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NjAwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOSI6NDAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6UDItNCI6NTAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6UDItMTQiOjE1MDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FzaCI6MjQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpidWlsZGluZ3MiOjE5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6aW50YW5naWJsZUFzc2V0cyI6NzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudExpYWJpbGl0aWVzIjozOTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpsb25nVGVybURlYnQiOjI5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGl0YWwiOjEwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRBc3NldHMiOjcyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDp0YW5naWJsZUFzc2V0cyI6NTgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmxhbmQiOjEwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGlhYmlsaXRpZXMiOjc5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRMaWFiaWxpdGllcyI6MzgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OnNoYXJlaG9sZGVyRXF1aXR5Ijo2MTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTphc3NldHMiOjE1NjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZEFzc2V0cyI6NzgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bWFjaGluZXJ5IjozMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjkwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OnNvZnR3YXJlIjo3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OnNob3J0VGVybURlYnQiOjExMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bmV0QXNzZXRzIjo3MzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwZXgiOjEwMDAwMDAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MC42NiwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC43LCJkcml2ZXI6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybzowIjowLjY2LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC43LCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlVG9CYXNlIjowLjY4LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NSYXRlVG9CYXNlOjAiOjAuNjgsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc1JhdGVUb0Jhc2U6MSI6MC42OCwiZHJpdmVyOm90aGVyQ29nc1JhdGVUb0Jhc2UiOjAuNjgsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlVG9CYXNlOjAiOjAuNjgsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlVG9CYXNlOjEiOjAuNjgsImRyaXZlcjpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwiZHJpdmVyLXJhbmdlOnByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZToxIjoxLCJkcml2ZXI6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJkcml2ZXItcmFuZ2U6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjowLjksImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGU6MSI6MC4zLCJkcml2ZXI6b3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjEiOjAuMywiZHJpdmVyOnByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdE5vbk9wZXJhdGluZ1JhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOnByb2plY3ROb25PcGVyYXRpbmdSYXRlOjEiOjAuNSwiZHJpdmVyOm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJOb25PcGVyYXRpbmdSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpvdGhlck5vbk9wZXJhdGluZ1JhdGU6MSI6MC41LCJkcml2ZXI6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6b3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6ZWZmZWN0aXZlVGF4UmF0ZSI6MC4zLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZTowIjowLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZToxIjowLjYsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RGaXJzdFllYXJTYWxlcyI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RGaXJzdFllYXJTYWxlczowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEZpcnN0WWVhclNhbGVzOjEiOjEwMDAwMDAwMDAwLCJkcml2ZXI6cHJvamVjdEJhc2VZZWFyU2FsZXMiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0QmFzZVllYXJTYWxlczowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEJhc2VZZWFyU2FsZXM6MSI6MTAwMDAwMDAwMDAsImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjEuNjY1MzM0NTM2OTM3NzM0OGUtMTYsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkzMjUzMzA1MDE4NDY5MjcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNzM1OTk0MTgzMTg5MTY2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLjAxOTEzOTQ1NzAyMzcxNzQ0MywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNTUzNDU5OTE0NzYzMDk1LCJkcml2ZXI6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wMzkxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDQyNTAwMDAwMDAwMDAwMDksImRyaXZlcjpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjAiOjAuMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MSI6MC4zLCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NzI0NjM3NjgxMTU4NiwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MCI6MC4wNjA3NjA4Njk1NjUyMTcxOSwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MSI6MC4wNjQzODQwNTc5NzEwMTQ1MywiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZToxIjowLjAzLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDoxIjowLjAwNTEzNDU3NTU2OTM1ODE5NzUsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDowIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDoxIjowLjEsImRyaXZlcjpvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjAiOjAuMDI0MTM5NDU3MDIzNzE3NDQ0LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wMjU1NTM0NTk5MTQ3NjMwOTYsImRyaXZlcjpvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGg6MSI6MC4wOCwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjowLjA0NDE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MSI6MC4wNDc1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjAxNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDoxIjowLjAzLCJkcml2ZXI6b3RoZXJTZ2FSYXRlRW5kIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMDEsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAuMDQyNjMxNTc4OTQ3MzY4MzYsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjA2NTU1NTU1NTU1NTU1NTU4LCJkcml2ZXI6aW52ZXN0bWVudCI6MjMwMDAwMCwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUwMDAwMCwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MSI6MjAwMDAwMDAsImRyaXZlcjpzdWJzaWR5Ijo3NjYwMDAsImRyaXZlci1yYW5nZTpzdWJzaWR5OjAiOjEwMDAwMCwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MSI6NTAwMDAwMCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoxNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjo4MjQwMDAwLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjoyLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOm1heCI6NywidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOnZhbHVlIjo2MCwidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOm1heCI6OTUsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOnZhbHVlIjoyMiwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOnZhbHVlIjo3NDgwMDAwLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOnZhbHVlIjoyMSwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2FncjptYXgiOjM1LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOnZhbHVlIjoxODc4MDAwLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOnZhbHVlIjo3LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOm1heCI6MTAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOnZhbHVlIjoyODUwMDAsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MTUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTptYXgiOjI1MjY5MDAwLCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6bWF4IjoxMzY4NDAwMCwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTptYXgiOjMzNDMwMDAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOm1heCI6Mzc0MDAwfSwibWV0cmljR3JvdXBCYXNlcyI6eyJjb21wYW55U2FsZXMiOiJyYXRlIiwicHJvamVjdFNhbGVzIjoicmF0ZSIsImxhYm9yUHJvZHVjdGl2aXR5IjoicmF0ZSIsImVtcGxveWVlUGF5IjoicmF0ZSJ9LCJhcHBsaWNhdGlvbkNhdGVnb3J5IjoiZ2VuZXJhbCIsImFkanVzdGVkRHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY3OTkxNTA3Mjk3OTcwODEsIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY3OTk2OTM1MzYzNDAxMzMsInByb2plY3RDb2dzUmF0ZVRvQmFzZSI6MC42OCwib3RoZXJDb2dzUmF0ZVRvQmFzZSI6MC42OCwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA3MDcyMzY4NDIxMDUxLCJwcm9qZWN0Rmlyc3RZZWFyU2FsZXMiOjAsInByb2plY3RCYXNlWWVhclNhbGVzIjowLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjoxLjMzNzU5NjcwMDA2ODM4ODdlLTE2LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDA0NzAwOTU3NDk0MjI0LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1MjE5MjI1ODM4MTk5Mjk4LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA0OTgyMDkxOTA3OTY4Niwib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI2MTYwNTg0NTI3Njc5OCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg2NDI2Njc5MjM0NzY0OCwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA5MzA4MjU0MjAwMTQ2NSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyMDAwMjEzNjI4OTg4NjM4LCJvdGhl</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsIm1vbmV5VW5pdCI6IuWNg+WGhiIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOaPkOahiOioiOeUu+OCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MjAwMDAwLCJjb2dzIjo0ODk2MDAwLCJlbXBsb3llZVBheSI6NTE5MDMxLCJvZmZpY2VyUGF5IjozNjAwMCwiZGVwcmVjaWF0aW9uIjoxODAwMDAsIm90aGVyU2dhIjo5MDAwMDAsImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQ5MzA3OSwiZW1wbG95ZWVCb251cyI6MjU5NTIsIm9mZmljZXJDb21wZW5zYXRpb24iOjMyNDAwLCJvZmZpY2VyQm9udXMiOjM2MDAsImNvZ3NEZXByZWNpYXRpb24iOjQ1MDAwLCJzZ2FEZXByZWNpYXRpb24iOjEzNTAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6MzYwMDB9LCJvdGhlciI6eyJzYWxlcyI6NjQ0MDAwMCwiY29ncyI6NDM3OTIwMCwiZW1wbG95ZWVQYXkiOjcwOTc4Niwib2ZmaWNlclBheSI6NTUyMDAsImRlcHJlY2lhdGlvbiI6MTM4MDAwLCJvdGhlclNnYSI6NzM2MDAwLCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Njc0Mjk3LCJlbXBsb3llZUJvbnVzIjozNTQ4OSwib2ZmaWNlckNvbXBlbnNhdGlvbiI6NDk2ODAsIm9mZmljZXJCb251cyI6NTUyMCwiY29nc0RlcHJlY2lhdGlvbiI6Mjc2MDAsInNnYURlcHJlY2lhdGlvbiI6MTEwNDAwLCJyZXNlYXJjaERldmVsb3BtZW50IjoyNzYwMCwib3JkaW5hcnlJbmNvbWUiOjM5NDUzNCwicHJlVGF4SW5jb21lIjozOTQ1MzQsIm5ldEluY29tZSI6NzUwNzUyLjF9fSx7InllYXIiOjIwMjQsInJvbGUiOiJwcmV2aW91cyIsInByb2plY3QiOnsic2FsZXMiOjc2MDAwMDAsImNvZ3MiOjUxNjgwMDAsImVtcGxveWVlUGF5Ijo1NTg4MjQsIm9mZmljZXJQYXkiOjM4MDAwLCJkZXByZWNpYXRpb24iOjE5MDAwMCwib3RoZXJTZ2EiOjk1MDAwMCwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NTMwODgzLCJlbXBsb3llZUJvbnVzIjoyNzk0MSwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MzQyMDAsIm9mZmljZXJCb251cyI6MzgwMCwiY29nc0RlcHJlY2lhdGlvbiI6NDc1MDAsInNnYURlcHJlY2lhdGlvbiI6MTQyNTAwLCJyZXNlYXJjaERldmVsb3BtZW50IjozODAwMH0sIm90aGVyIjp7InNhbGVzIjo2NzIwMDAwLCJjb2dzIjo0NTY5NjAwLCJlbXBsb3llZVBheSI6NzU0MTQ4LCJvZmZpY2VyUGF5Ijo1NzYwMCwiZGVwcmVjaWF0aW9uIjoxNDQwMDAsIm90aGVyU2dhIjo3NjgwMDAsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3MTY0NDEsImVtcGxveWVlQm9udXMiOjM3NzA3LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjo1MTg0MCwib2ZmaWNlckJvbnVzIjo1NzYwLCJjb2dzRGVwcmVjaWF0aW9uIjoyODgwMCwic2dhRGVwcmVjaWF0aW9uIjoxMTUyMDAsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjI4ODAwLCJvcmRpbmFyeUluY29tZSI6Mzk4MDEyLCJwcmVUYXhJbmNvbWUiOjM5ODAxMiwibmV0SW5jb21lIjo3NzE4ODEuNn19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwMDAwMDAsImNvZ3MiOjU0NDAwMDAsImVtcGxveWVlUGF5Ijo2MDAwMDAsImVtcGxveWVlU2FsYXJ5Ijo1NzAwMDAsImVtcGxveWVlQm9udXMiOjMwMDAwLCJvZmZpY2VyUGF5Ijo0MDAwMCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MzYwMDAsIm9mZmljZXJCb251cyI6NDAwMCwiZGVwcmVjaWF0aW9uIjoyMDAwMDAsImNvZ3NEZXByZWNpYXRpb24iOjUwMDAwLCJzZ2FEZXByZWNpYXRpb24iOjE1MDAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6NDAwMDAsIm90aGVyU2dhIjoxMDAwMDAwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwMDAwMDAsImNvZ3MiOjQ3NjAwMDAsImVtcGxveWVlUGF5Ijo4MDAwMDAsImVtcGxveWVlU2FsYXJ5Ijo3NjAwMDAsImVtcGxveWVlQm9udXMiOjQwMDAwLCJvZmZpY2VyUGF5Ijo2MDAwMCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6NTQwMDAsIm9mZmljZXJCb251cyI6NjAwMCwiZGVwcmVjaWF0aW9uIjoxNTAwMDAsImNvZ3NEZXByZWNpYXRpb24iOjMwMDAwLCJzZ2FEZXByZWNpYXRpb24iOjEyMDAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6MzAwMDAsIm90aGVyU2dhIjo4MDAwMDAsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjo0MDAwMDAsInByZVRheEluY29tZSI6NDAwMDAwLCJuZXRJbmNvbWUiOjc5MTAwMH19XSwiYmFsYW5jZVNoZWV0cyI6W3sieWVhciI6MjAyMywiYXNzZXRzIjoxMzIwMDAwMCwiY3VycmVudEFzc2V0cyI6NjcwMDAwMCwiY2FzaCI6MjQwMDAwMCwiZml4ZWRBc3NldHMiOjY1MDAwMDAsInRhbmdpYmxlQXNzZXRzIjo1MzAwMDAwLCJidWlsZGluZ3MiOjE5MDAwMDAsIm1hY2hpbmVyeSI6MjQwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6NzAwMDAwLCJzb2Z0d2FyZSI6NTAwMDAwLCJsaWFiaWxpdGllcyI6NzUwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjozOTAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjozNjAwMDAwLCJsb25nVGVybURlYnQiOjI5MDAwMDAsIm5ldEFzc2V0cyI6NTcwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjU0MDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4Ijo1MDAwMDB9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMwMDAwMCwiY3VycmVudEFzc2V0cyI6NzIwMDAwMCwiY2FzaCI6MjUwMDAwMCwiZml4ZWRBc3NldHMiOjcxMDAwMDAsInRhbmdpYmxlQXNzZXRzIjo1ODAwMDAwLCJidWlsZGluZ3MiOjIwMDAwMDAsIm1hY2hpbmVyeSI6MjgwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6ODAwMDAwLCJzb2Z0d2FyZSI6NjAwMDAwLCJsaWFiaWxpdGllcyI6NzkwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjo0MTAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjozODAwMDAwLCJsb25nVGVybURlYnQiOjMxMDAwMDAsIm5ldEFzc2V0cyI6NjQwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjYxMDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4Ijo4MDAwMDB9LHsieWVhciI6MjAyNSwiYXNzZXRzIjoxNTYwMDAwMCwiY3VycmVudEFzc2V0cyI6NzgwMDAwMCwiY2FzaCI6MjcwMDAwMCwiZml4ZWRBc3NldHMiOjc4MDAwMDAsInRhbmdpYmxlQXNzZXRzIjo2NDAwMDAwLCJidWlsZGluZ3MiOjIyMDAwMDAsIm1hY2hpbmVyeSI6MzIwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6OTAwMDAwLCJzb2Z0d2FyZSI6NzAwMDAwLCJsaWFiaWxpdGllcyI6ODMwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjo0MzAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMTAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjo0MDAwMDAwLCJsb25nVGVybURlYnQiOjMyMDAwMDAsIm5ldEFzc2V0cyI6NzMwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjcwMDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4IjoxMDAwMDAwfV0sImZ1dHVyZUNhcGV4IjpbeyJ5ZWFyIjoyMDI2LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI4LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI5LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMwLCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMxLCJ2YWx1ZSI6MH1dLCJkcml2ZXJzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsInByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJwcm9qZWN0Q29nc1JhdGVUb0Jhc2UiOjAuNjgsIm90aGVyQ29nc1JhdGVUb0Jhc2UiOjAuNjgsInByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwib3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwicHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yNSwib3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMiwicHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsInByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJvdGhlck5vbk9wZXJhdGluZ1JhdGUiOi0wLjAwNSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjowLCJlZmZlY3RpdmVUYXhSYXRlIjowLjMsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdEZpcnN0WWVhclNhbGVzIjowLCJwcm9qZWN0QmFzZVllYXJTYWxlcyI6MCwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6NS41NTExMTUxMjMxMjU3ODNlLTE3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5Nywib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI1NzI0NjM3NjgxMTU4NTQsIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wMTUsIm90aGVyU2dhUmF0ZUVuZCI6MC4wMDUsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJpbnZlc3RtZW50IjoyMzAwMDAwLCJzdWJzaWR5Ijo3NjYwMDAsImxvY2FsQmVuY2htYXJrIjoyM30sImRyaXZlclJhbmdlcyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjpbLTAuMDUsMC4zXSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6WzAuNjYsMC43XSwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOlswLjY2LDAuN10sInByb2plY3RDb2dzUmF0ZVRvQmFzZSI6WzAuNjgsMC42OF0sIm90aGVyQ29nc1JhdGVUb0Jhc2UiOlswLjY4LDAuNjhdLCJwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOlswLDFdLCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOlswLDFdLCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOlstMC41LDAuNV0sIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6Wy0wLjUsMC41XSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJlZmZlY3RpdmVUYXhSYXRlIjpbMCwwLjZdLCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwicHJvamVjdEZpcnN0WWVhclNhbGVzIjpbMCwxMDAwMDAwMDAwMF0sInByb2plY3RCYXNlWWVhclNhbGVzIjpbMCwxMDAwMDAwMDAwMF0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDEuNjY1MzM0NTM2OTM3NzM0OGUtMTZdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkzMjUzMzA1MDE4NDY5MjcsMC4wMjA3MzU5OTQxODMxODkxNjZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlswLjA0MDc2MDg2OTU2NTIxNzE4NCwwLjA0NDM4NDA1Nzk3MTAxNDUyXSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDAwMTM0NTc1NTY5MzU4MTk3MzddLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MTM5NDU3MDIzNzE3NDQzLDAuMDIwNTUzNDU5OTE0NzYzMDk1XSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjAzOTE2NjY2NjY2NjY2NjY4LDAuMDQyNTAwMDAwMDAwMDAwMDldLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbMC4xNSwwLjNdLCJvdGhlclNhbGVzR3Jvd3RoIjpbMC4wNjA3NjA4Njk1NjUyMTcxOSwwLjA2NDM4NDA1Nzk3MTAxNDUzXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMC4wMDUsMC4wMDUxMzQ1NzU1NjkzNTgxOTc1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLjAyNDEzOTQ1NzAyMzcxNzQ0NCwwLjAyNTU1MzQ1OTkxNDc2MzA5Nl0sIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6WzAsMC4wOF0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6WzAuMDQ0MTY2NjY2NjY2NjY2NjgsMC4wNDc1MDAwMDAwMDAwMDAwOV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMCwwLjAzXSwib3RoZXJTZ2FSYXRlRW5kIjpbMCwwLjAxXSwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOlswLjA0MjYzMTU3ODk0NzM2ODM2LDAuMDY1NTU1NTU1NTU1NTU1NThdLCJpbnZlc3RtZW50IjpbMTUwMDAwMCwyMDAwMDAwMF0sInN1YnNpZHkiOlsxMDAwMDAsNTAwMDAwMF0sImxvY2FsQmVuY2htYXJrIjpbMCwxMDBdfSwidGFyZ2V0cyI6eyJjb21wYW55U2FsZXNDYWdyIjp7InZhbHVlIjoxNSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo4MjQwMDAwLCJtYXgiOjI1MjY5MDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjoyLCJtYXgiOjcsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNTaGFyZSI6eyJ2YWx1ZSI6NjAsIm1heCI6OTUsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJwcm9qZWN0U2FsZXNDYWdyIjp7InZhbHVlIjoyMiwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo3NDgwMDAwLCJtYXgiOjEzNjg0MDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwibGFib3JQcm9kdWN0aXZpdHlDYWdyIjp7InZhbHVlIjoyMSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRJbmNyZWFzZSI6eyJ2YWx1ZSI6MTg3ODAwMCwibWF4IjozMzQzMDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlDYWdyIjp7InZhbHVlIjo3LCJtYXgiOjEwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiZW1wbG95ZWVQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6Mjg1MDAwLCJtYXgiOjM3NDAwMCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImludmVzdG1lbnRTYWxlc1JhdGlvIjp7InZhbHVlIjoxNSwibWF4Ijo3MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInZhbHVlQWRkZWRTdWJzaWR5UmF0aW8iOnsidmFsdWUiOjIxMywibWF4IjozNTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsb2NhbEJlbmNobWFyayI6eyJ2YWx1ZSI6MjMsIm1heCI6NDAsInBvbGljeSI6Im1vbml0b3IiLCJ3ZWlnaHQiOjF9LCJvZmZpY2VyUGF5Q2FnciI6eyJ2YWx1ZSI6NiwibWF4IjoxMCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlJbmNyZWFzZSI6eyJ2YWx1ZSI6MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX19LCJmb3JlY2FzdE92ZXJyaWRlcyI6eyIyMDI5Om90aGVyOnNhbGVzIjo4NTEzMDAwLCIyMDI5OnByb2plY3Q6Ny04Ijo3OTAwMDB9LCJmdXR1cmVJbnB1dEJhc2lzIjoib3RoZXIiLCJpbnB1dFZhbHVlcyI6eyJhY3R1YWw6Y29tcGFueToyMDIzOjItMSI6MTM2NDAwMDAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0zIjo5Mjc1MjAwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItNCI6NzI2MDAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi03IjozMjY1MDE3LCJhY3R1YWw6Y29tcGFueToyMDIzOjItOSI6ODIwODAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMCI6OTEyMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEyIjoxMTY3Mzc2LCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTMiOjYxNDQxLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTQiOjI0NTQwMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE1Ijo2MzYwMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTE4IjoxMDcyNTAzLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTkiOjEwNzI1MDMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yMCI6NzUwNzUyLjEsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yNyI6MjEwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xIjo3MjAwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNCI6MjMwNDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTYiOjY3Nzk2OSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTgiOjUxOTAzMSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTkiOjM2MDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOlAyLTQiOjQ1MDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOlAyLTE0IjoxMzUwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xMyI6OTAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEiOjE0MzIwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMyI6OTczNzYwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTQiOjc2MzAwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItNyI6MzQ1MTA3MiwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTkiOjg2MDQwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTAiOjk1NjAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMiI6MTI0NzMyNCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEzIjo2NTY0OCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE0IjoyNTc3MDAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xNSI6NjY4MDAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xOCI6MTEwMjY4OCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE5IjoxMTAyNjg4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjAiOjc3MTg4MS42LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjciOjIyMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMSI6NzYwMDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTQiOjI0MzIwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny02Ijo3MDQ2NzYsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny04Ijo1NTg4MjQsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny05IjozODAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDpQMi00Ijo0NzUwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDpQMi0xNCI6MTQyNTAwLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTMiOjk1LCJhY3R1YWw6cHJvamVjdDoyMDI0OjctMTQiOjIsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xIjoxNTAwMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTMiOjEwMjAwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItNCI6ODAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi03IjozNjQwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItOSI6OTAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMCI6MTAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xMiI6MTMzMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEzIjo3MDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE0IjoyNzAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xNSI6NzAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0xOCI6MTEzMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE5IjoxMTMwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjAiOjc5MTAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI3IjoyMzAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEiOjgwMDAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny00IjoyNTYwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctNiI6NzMwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOCI6NjAwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctOSI6NDAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6UDItNCI6NTAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6UDItMTQiOjE1MDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTEzIjoxMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny0xNCI6MiwiYmFsYW5jZS1zaGVldDoyMDIzOmFzc2V0cyI6MTMyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50QXNzZXRzIjo2NzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FzaCI6MjQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkQXNzZXRzIjo2NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6dGFuZ2libGVBc3NldHMiOjUzMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpidWlsZGluZ3MiOjE5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzptYWNoaW5lcnkiOjI0MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpsYW5kIjoxMDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6aW50YW5naWJsZUFzc2V0cyI6NzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6c29mdHdhcmUiOjUwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmxpYWJpbGl0aWVzIjo3NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y3VycmVudExpYWJpbGl0aWVzIjozOTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6c2hvcnRUZXJtRGVidCI6MTIwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmZpeGVkTGlhYmlsaXRpZXMiOjM2MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpsb25nVGVybURlYnQiOjI5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpuZXRBc3NldHMiOjU3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaGFyZWhvbGRlckVxdWl0eSI6NTQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGl0YWwiOjEwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXBleCI6NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6YXNzZXRzIjoxNDMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRBc3NldHMiOjcyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXNoIjoyNTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRBc3NldHMiOjcxMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDp0YW5naWJsZUFzc2V0cyI6NTgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmJ1aWxkaW5ncyI6MjAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0Om1hY2hpbmVyeSI6MjgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmxhbmQiOjEwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDppbnRhbmdpYmxlQXNzZXRzIjo4MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpzb2Z0d2FyZSI6NjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGlhYmlsaXRpZXMiOjc5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjdXJyZW50TGlhYmlsaXRpZXMiOjQxMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Zml4ZWRMaWFiaWxpdGllcyI6MzgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmxvbmdUZXJtRGVidCI6MzEwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0Om5ldEFzc2V0cyI6NjQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OnNoYXJlaG9sZGVyRXF1aXR5Ijo2MTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwaXRhbCI6MTAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhcGV4Ijo4MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTphc3NldHMiOjE1NjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudEFzc2V0cyI6NzgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhc2giOjI3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZEFzc2V0cyI6NzgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OnRhbmdpYmxlQXNzZXRzIjo2NDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6YnVpbGRpbmdzIjoyMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bWFjaGluZXJ5IjozMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bGFuZCI6MTAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmludGFuZ2libGVBc3NldHMiOjkwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OnNvZnR3YXJlIjo3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpsaWFiaWxpdGllcyI6ODMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmN1cnJlbnRMaWFiaWxpdGllcyI6NDMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OnNob3J0VGVybURlYnQiOjExMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpmaXhlZExpYWJpbGl0aWVzIjo0MDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bG9uZ1Rlcm1EZWJ0IjozMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6bmV0QXNzZXRzIjo3MzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hhcmVob2xkZXJFcXVpdHkiOjcwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBpdGFsIjoxMDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FwZXgiOjEwMDAwMDAsImRyaXZlcjpwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDowIjotMC4wNSwiZHJpdmVyLXJhbmdlOnByb2plY3RNYXJrZXRHcm93dGg6MSI6MC4zLCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MCI6MC42NiwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC43LCJkcml2ZXI6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybzowIjowLjY2LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm86MSI6MC43LCJkcml2ZXI6cHJvamVjdENvZ3NSYXRlVG9CYXNlIjowLjY4LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NSYXRlVG9CYXNlOjAiOjAuNjgsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc1JhdGVUb0Jhc2U6MSI6MC42OCwiZHJpdmVyOm90aGVyQ29nc1JhdGVUb0Jhc2UiOjAuNjgsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlVG9CYXNlOjAiOjAuNjgsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlVG9CYXNlOjEiOjAuNjgsImRyaXZlcjpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwiZHJpdmVyLXJhbmdlOnByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZToxIjoxLCJkcml2ZXI6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJkcml2ZXItcmFuZ2U6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjowLjksImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGU6MSI6MC4zLCJkcml2ZXI6b3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjEiOjAuMywiZHJpdmVyOnByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdE5vbk9wZXJhdGluZ1JhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOnByb2plY3ROb25PcGVyYXRpbmdSYXRlOjEiOjAuNSwiZHJpdmVyOm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJOb25PcGVyYXRpbmdSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpvdGhlck5vbk9wZXJhdGluZ1JhdGU6MSI6MC41LCJkcml2ZXI6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6b3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6ZWZmZWN0aXZlVGF4UmF0ZSI6MC4zLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZTowIjowLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZToxIjowLjYsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RGaXJzdFllYXJTYWxlcyI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RGaXJzdFllYXJTYWxlczowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEZpcnN0WWVhclNhbGVzOjEiOjEwMDAwMDAwMDAwLCJkcml2ZXI6cHJvamVjdEJhc2VZZWFyU2FsZXMiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0QmFzZVllYXJTYWxlczowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEJhc2VZZWFyU2FsZXM6MSI6MTAwMDAwMDAwMDAsImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjEuNjY1MzM0NTM2OTM3NzM0OGUtMTYsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkzMjUzMzA1MDE4NDY5MjcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNzM1OTk0MTgzMTg5MTY2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLjAxOTEzOTQ1NzAyMzcxNzQ0MywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNTUzNDU5OTE0NzYzMDk1LCJkcml2ZXI6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wMzkxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDQyNTAwMDAwMDAwMDAwMDksImRyaXZlcjpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjAiOjAuMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MSI6MC4zLCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NzI0NjM3NjgxMTU4NiwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MCI6MC4wNjA3NjA4Njk1NjUyMTcxOSwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MSI6MC4wNjQzODQwNTc5NzEwMTQ1MywiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZToxIjowLjAzLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDoxIjowLjAwNTEzNDU3NTU2OTM1ODE5NzUsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDowIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDoxIjowLjEsImRyaXZlcjpvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjAiOjAuMDI0MTM5NDU3MDIzNzE3NDQ0LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wMjU1NTM0NTk5MTQ3NjMwOTYsImRyaXZlcjpvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGg6MSI6MC4wOCwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjowLjA0NDE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MSI6MC4wNDc1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjAxNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDoxIjowLjAzLCJkcml2ZXI6b3RoZXJTZ2FSYXRlRW5kIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMDEsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAuMDQyNjMxNTc4OTQ3MzY4MzYsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjA2NTU1NTU1NTU1NTU1NTU4LCJkcml2ZXI6aW52ZXN0bWVudCI6MjMwMDAwMCwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUwMDAwMCwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MSI6MjAwMDAwMDAsImRyaXZlcjpzdWJzaWR5Ijo3NjYwMDAsImRyaXZlci1yYW5nZTpzdWJzaWR5OjAiOjEwMDAwMCwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MSI6NTAwMDAwMCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoxNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjo4MjQwMDAwLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjoyLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOm1heCI6NywidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOnZhbHVlIjo2MCwidGFyZ2V0OnByb2plY3RTYWxlc1NoYXJlOm1heCI6OTUsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOnZhbHVlIjoyMiwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOnZhbHVlIjo3NDgwMDAwLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOnZhbHVlIjoyMSwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2FncjptYXgiOjM1LCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOnZhbHVlIjoxODc4MDAwLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOnZhbHVlIjo3LCJ0YXJnZXQ6ZW1wbG95ZWVQYXlDYWdyOm1heCI6MTAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOnZhbHVlIjoyODUwMDAsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzp2YWx1ZSI6MTUsInRhcmdldDppbnZlc3RtZW50U2FsZXNSYXRpbzptYXgiOjcwLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzp2YWx1ZSI6MjEzLCJ0YXJnZXQ6dmFsdWVBZGRlZFN1YnNpZHlSYXRpbzptYXgiOjM1MCwidGFyZ2V0OmxvY2FsQmVuY2htYXJrOnZhbHVlIjoyMywidGFyZ2V0OmxvY2FsQmVuY2htYXJrOm1heCI6NDAsInRhcmdldDpvZmZpY2VyUGF5Q2Fncjp2YWx1ZSI6NiwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOm1heCI6MTAsInRhcmdldDpvZmZpY2VyUGF5SW5jcmVhc2U6dmFsdWUiOjAsInRhcmdldDpjb21wYW55U2FsZXNJbmNyZWFzZTptYXgiOjI1MjY5MDAwLCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6bWF4IjoxMzY4NDAwMCwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTptYXgiOjMzNDMwMDAsInRhcmdldDplbXBsb3llZVBheUluY3JlYXNlOm1heCI6Mzc0MDAwfSwibWV0cmljR3JvdXBCYXNlcyI6eyJjb21wYW55U2FsZXMiOiJyYXRlIiwicHJvamVjdFNhbGVzIjoicmF0ZSIsImxhYm9yUHJvZHVjdGl2aXR5IjoicmF0ZSIsImVtcGxveWVlUGF5IjoicmF0ZSJ9LCJhcHBsaWNhdGlvbkNhdGVnb3J5IjoiZ2VuZXJhbCIsImFkanVzdGVkRHJpdmVycyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjowLjA1LCJwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY3OTkxNTA3Mjk3OTcwODEsIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY3OTk2OTM1MzYzNDAxMzMsInByb2plY3RDb2dzUmF0ZVRvQmFzZSI6MC42OCwib3RoZXJDb2dzUmF0ZVRvQmFzZSI6MC42OCwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA3MDcyMzY4NDIxMDUxLCJwcm9qZWN0Rmlyc3RZZWFyU2FsZXMiOjAsInByb2plY3RCYXNlWWVhclNhbGVzIjowLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjoxLjMzNzU5NjcwMDA2ODM4ODdlLTE2LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDA0NzAwOTU3NDk0MjI0LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1MjE5MjI1ODM4MTk5Mjk4LCJwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA1NDA0OTgyMDkxOTA3OTY4Niwib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI2MTYwNTg0NTI3Njc5OCwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjAsIm90aGVyUGF5R3Jvd3RoVG9CYXNlIjowLjAxOTg2NDI2Njc5MjM0NzY0OCwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA5MzA4MjU0MjAwMTQ2NSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyMDQ1MjEzNjI4OTg4NjM5LCJvdGhl</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">clNhbGVzR3Jvd3RoIjowLjA2MjUyMzYxODc5MjY4NTk2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNTAxMDI4MjE4MjIwOTA4MSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA4MTg1Mjk5NTQzNzQxMzIzLCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4MTgxOTk2Mzg3MDk4OTcsIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6MC4wNDUsInByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDIwOTMzNjQ1MjQ5MTU4NzksIm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTgzNTU4ODEzNTY3NTI5LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wMTQ5ODU1NTIzMjkyNTEzNjEsIm90aGVyU2dhUmF0ZUVuZCI6MC4wMDQ5ODc2OTI2MzQ3MTE0NDgsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1Mzc5NjY0NTQ2MTMxNTI2LCJpbnZlc3RtZW50IjoyMzAwMDAwLCJzdWJzaWR5Ijo3NjYwMDAsImxvY2FsQmVuY2htYXJrIjoyM319</t>
+          <t xml:space="preserve">clNhbGVzR3Jvd3RoIjowLjA2MjUyMzYxODc5MjY4NTk2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNTAxMDI4MjE4MjIwOTA4MSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA4MTg1Mjk5NTQzNzQxMzIzLCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4MTgxOTk2Mzg3MDk4OTcsIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6MC4wNDUsInByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDIwOTMzNjQ1MjQ5MTU4NzksIm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTgzNTU4ODEzNTY3NTI5LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wMTQ5MjU1NTIzMjkyNTEzNiwib3RoZXJTZ2FSYXRlRW5kIjowLjAwNDk4NzY5MjYzNDcxMTQ0OCwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOjAuMDUzNzk2NjQ1NDYxMzE1MjYsImludmVzdG1lbnQiOjIzMDAwMDAsInN1YnNpZHkiOjc2NjAwMCwibG9jYWxCZW5jaG1hcmsiOjIzfX0=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Populate payroll totals in sample proposals
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル.xlsx
@@ -8233,7 +8233,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C298"/>
+  <dimension ref="A1:C304"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="72" customWidth="1"/>
@@ -8413,11 +8413,11 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2023:2-27</t>
+          <t xml:space="preserve">actual:company:2023:2-21</t>
         </is>
       </c>
       <c r="B12" s="2">
-        <v>210</v>
+        <v>1228817</v>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
@@ -8428,11 +8428,11 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2023:2-28</t>
+          <t xml:space="preserve">actual:company:2023:2-22</t>
         </is>
       </c>
       <c r="B13" s="2">
-        <v>5</v>
+        <v>91200</v>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
@@ -8443,11 +8443,11 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2023:2-3</t>
+          <t xml:space="preserve">actual:company:2023:2-27</t>
         </is>
       </c>
       <c r="B14" s="2">
-        <v>9275200</v>
+        <v>210</v>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
@@ -8458,11 +8458,11 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2023:2-4</t>
+          <t xml:space="preserve">actual:company:2023:2-28</t>
         </is>
       </c>
       <c r="B15" s="2">
-        <v>72600</v>
+        <v>5</v>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
@@ -8473,11 +8473,11 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2023:2-7</t>
+          <t xml:space="preserve">actual:company:2023:2-3</t>
         </is>
       </c>
       <c r="B16" s="2">
-        <v>3265017</v>
+        <v>9275200</v>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
@@ -8488,11 +8488,11 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2023:2-9</t>
+          <t xml:space="preserve">actual:company:2023:2-4</t>
         </is>
       </c>
       <c r="B17" s="2">
-        <v>82080</v>
+        <v>72600</v>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
@@ -8503,11 +8503,11 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-1</t>
+          <t xml:space="preserve">actual:company:2023:2-7</t>
         </is>
       </c>
       <c r="B18" s="2">
-        <v>14320000</v>
+        <v>3265017</v>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
@@ -8518,11 +8518,11 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-10</t>
+          <t xml:space="preserve">actual:company:2023:2-9</t>
         </is>
       </c>
       <c r="B19" s="2">
-        <v>9560</v>
+        <v>82080</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
@@ -8533,11 +8533,11 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-12</t>
+          <t xml:space="preserve">actual:company:2024:2-1</t>
         </is>
       </c>
       <c r="B20" s="2">
-        <v>1247324</v>
+        <v>14320000</v>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
@@ -8548,11 +8548,11 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-13</t>
+          <t xml:space="preserve">actual:company:2024:2-10</t>
         </is>
       </c>
       <c r="B21" s="2">
-        <v>65648</v>
+        <v>9560</v>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
@@ -8563,11 +8563,11 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-14</t>
+          <t xml:space="preserve">actual:company:2024:2-12</t>
         </is>
       </c>
       <c r="B22" s="2">
-        <v>257700</v>
+        <v>1247324</v>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
@@ -8578,11 +8578,11 @@
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-15</t>
+          <t xml:space="preserve">actual:company:2024:2-13</t>
         </is>
       </c>
       <c r="B23" s="2">
-        <v>66800</v>
+        <v>65648</v>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
@@ -8593,11 +8593,11 @@
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-18</t>
+          <t xml:space="preserve">actual:company:2024:2-14</t>
         </is>
       </c>
       <c r="B24" s="2">
-        <v>1102688</v>
+        <v>257700</v>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
@@ -8608,11 +8608,11 @@
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-19</t>
+          <t xml:space="preserve">actual:company:2024:2-15</t>
         </is>
       </c>
       <c r="B25" s="2">
-        <v>1102688</v>
+        <v>66800</v>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
@@ -8623,11 +8623,11 @@
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-20</t>
+          <t xml:space="preserve">actual:company:2024:2-18</t>
         </is>
       </c>
       <c r="B26" s="2">
-        <v>771881.6</v>
+        <v>1102688</v>
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
@@ -8638,11 +8638,11 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-27</t>
+          <t xml:space="preserve">actual:company:2024:2-19</t>
         </is>
       </c>
       <c r="B27" s="2">
-        <v>220</v>
+        <v>1102688</v>
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
@@ -8653,11 +8653,11 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-28</t>
+          <t xml:space="preserve">actual:company:2024:2-20</t>
         </is>
       </c>
       <c r="B28" s="2">
-        <v>5</v>
+        <v>771881.6</v>
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
@@ -8668,11 +8668,11 @@
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-3</t>
+          <t xml:space="preserve">actual:company:2024:2-21</t>
         </is>
       </c>
       <c r="B29" s="2">
-        <v>9737600</v>
+        <v>1312972</v>
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
@@ -8683,11 +8683,11 @@
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-4</t>
+          <t xml:space="preserve">actual:company:2024:2-22</t>
         </is>
       </c>
       <c r="B30" s="2">
-        <v>76300</v>
+        <v>95600</v>
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
@@ -8698,11 +8698,11 @@
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-7</t>
+          <t xml:space="preserve">actual:company:2024:2-27</t>
         </is>
       </c>
       <c r="B31" s="2">
-        <v>3451072</v>
+        <v>220</v>
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
@@ -8713,11 +8713,11 @@
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2024:2-9</t>
+          <t xml:space="preserve">actual:company:2024:2-28</t>
         </is>
       </c>
       <c r="B32" s="2">
-        <v>86040</v>
+        <v>5</v>
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
@@ -8728,11 +8728,11 @@
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-1</t>
+          <t xml:space="preserve">actual:company:2024:2-3</t>
         </is>
       </c>
       <c r="B33" s="2">
-        <v>15000000</v>
+        <v>9737600</v>
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
@@ -8743,11 +8743,11 @@
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-10</t>
+          <t xml:space="preserve">actual:company:2024:2-4</t>
         </is>
       </c>
       <c r="B34" s="2">
-        <v>10000</v>
+        <v>76300</v>
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
@@ -8758,11 +8758,11 @@
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-12</t>
+          <t xml:space="preserve">actual:company:2024:2-7</t>
         </is>
       </c>
       <c r="B35" s="2">
-        <v>1330000</v>
+        <v>3451072</v>
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
@@ -8773,11 +8773,11 @@
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-13</t>
+          <t xml:space="preserve">actual:company:2024:2-9</t>
         </is>
       </c>
       <c r="B36" s="2">
-        <v>70000</v>
+        <v>86040</v>
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
@@ -8788,11 +8788,11 @@
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-14</t>
+          <t xml:space="preserve">actual:company:2025:2-1</t>
         </is>
       </c>
       <c r="B37" s="2">
-        <v>270000</v>
+        <v>15000000</v>
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
@@ -8803,11 +8803,11 @@
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-15</t>
+          <t xml:space="preserve">actual:company:2025:2-10</t>
         </is>
       </c>
       <c r="B38" s="2">
-        <v>70000</v>
+        <v>10000</v>
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
@@ -8818,11 +8818,11 @@
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-18</t>
+          <t xml:space="preserve">actual:company:2025:2-12</t>
         </is>
       </c>
       <c r="B39" s="2">
-        <v>1130000</v>
+        <v>1330000</v>
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
@@ -8833,11 +8833,11 @@
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-19</t>
+          <t xml:space="preserve">actual:company:2025:2-13</t>
         </is>
       </c>
       <c r="B40" s="2">
-        <v>1130000</v>
+        <v>70000</v>
       </c>
       <c r="C40" s="0" t="inlineStr">
         <is>
@@ -8848,11 +8848,11 @@
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-20</t>
+          <t xml:space="preserve">actual:company:2025:2-14</t>
         </is>
       </c>
       <c r="B41" s="2">
-        <v>791000</v>
+        <v>270000</v>
       </c>
       <c r="C41" s="0" t="inlineStr">
         <is>
@@ -8863,11 +8863,11 @@
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-27</t>
+          <t xml:space="preserve">actual:company:2025:2-15</t>
         </is>
       </c>
       <c r="B42" s="2">
-        <v>230</v>
+        <v>70000</v>
       </c>
       <c r="C42" s="0" t="inlineStr">
         <is>
@@ -8878,11 +8878,11 @@
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-28</t>
+          <t xml:space="preserve">actual:company:2025:2-18</t>
         </is>
       </c>
       <c r="B43" s="2">
-        <v>5</v>
+        <v>1130000</v>
       </c>
       <c r="C43" s="0" t="inlineStr">
         <is>
@@ -8893,11 +8893,11 @@
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-3</t>
+          <t xml:space="preserve">actual:company:2025:2-19</t>
         </is>
       </c>
       <c r="B44" s="2">
-        <v>10200000</v>
+        <v>1130000</v>
       </c>
       <c r="C44" s="0" t="inlineStr">
         <is>
@@ -8908,11 +8908,11 @@
     <row r="45">
       <c r="A45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-4</t>
+          <t xml:space="preserve">actual:company:2025:2-20</t>
         </is>
       </c>
       <c r="B45" s="2">
-        <v>80000</v>
+        <v>791000</v>
       </c>
       <c r="C45" s="0" t="inlineStr">
         <is>
@@ -8923,11 +8923,11 @@
     <row r="46">
       <c r="A46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-7</t>
+          <t xml:space="preserve">actual:company:2025:2-21</t>
         </is>
       </c>
       <c r="B46" s="2">
-        <v>3640000</v>
+        <v>1400000</v>
       </c>
       <c r="C46" s="0" t="inlineStr">
         <is>
@@ -8938,11 +8938,11 @@
     <row r="47">
       <c r="A47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:company:2025:2-9</t>
+          <t xml:space="preserve">actual:company:2025:2-22</t>
         </is>
       </c>
       <c r="B47" s="2">
-        <v>90000</v>
+        <v>100000</v>
       </c>
       <c r="C47" s="0" t="inlineStr">
         <is>
@@ -8953,11 +8953,11 @@
     <row r="48">
       <c r="A48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2023:7-1</t>
+          <t xml:space="preserve">actual:company:2025:2-27</t>
         </is>
       </c>
       <c r="B48" s="2">
-        <v>7200000</v>
+        <v>230</v>
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
@@ -8968,11 +8968,11 @@
     <row r="49">
       <c r="A49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2023:7-10</t>
+          <t xml:space="preserve">actual:company:2025:2-28</t>
         </is>
       </c>
       <c r="B49" s="2">
-        <v>180000</v>
+        <v>5</v>
       </c>
       <c r="C49" s="0" t="inlineStr">
         <is>
@@ -8983,11 +8983,11 @@
     <row r="50">
       <c r="A50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2023:7-13</t>
+          <t xml:space="preserve">actual:company:2025:2-3</t>
         </is>
       </c>
       <c r="B50" s="2">
-        <v>90</v>
+        <v>10200000</v>
       </c>
       <c r="C50" s="0" t="inlineStr">
         <is>
@@ -8998,11 +8998,11 @@
     <row r="51">
       <c r="A51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2023:7-14</t>
+          <t xml:space="preserve">actual:company:2025:2-4</t>
         </is>
       </c>
       <c r="B51" s="2">
-        <v>2</v>
+        <v>80000</v>
       </c>
       <c r="C51" s="0" t="inlineStr">
         <is>
@@ -9013,11 +9013,11 @@
     <row r="52">
       <c r="A52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2023:7-4</t>
+          <t xml:space="preserve">actual:company:2025:2-7</t>
         </is>
       </c>
       <c r="B52" s="2">
-        <v>2304000</v>
+        <v>3640000</v>
       </c>
       <c r="C52" s="0" t="inlineStr">
         <is>
@@ -9028,11 +9028,11 @@
     <row r="53">
       <c r="A53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2023:7-6</t>
+          <t xml:space="preserve">actual:company:2025:2-9</t>
         </is>
       </c>
       <c r="B53" s="2">
-        <v>677969</v>
+        <v>90000</v>
       </c>
       <c r="C53" s="0" t="inlineStr">
         <is>
@@ -9043,11 +9043,11 @@
     <row r="54">
       <c r="A54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2023:7-8</t>
+          <t xml:space="preserve">actual:project:2023:7-1</t>
         </is>
       </c>
       <c r="B54" s="2">
-        <v>519031</v>
+        <v>7200000</v>
       </c>
       <c r="C54" s="0" t="inlineStr">
         <is>
@@ -9058,11 +9058,11 @@
     <row r="55">
       <c r="A55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2023:7-9</t>
+          <t xml:space="preserve">actual:project:2023:7-10</t>
         </is>
       </c>
       <c r="B55" s="2">
-        <v>36000</v>
+        <v>180000</v>
       </c>
       <c r="C55" s="0" t="inlineStr">
         <is>
@@ -9073,11 +9073,11 @@
     <row r="56">
       <c r="A56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2024:7-1</t>
+          <t xml:space="preserve">actual:project:2023:7-13</t>
         </is>
       </c>
       <c r="B56" s="2">
-        <v>7600000</v>
+        <v>90</v>
       </c>
       <c r="C56" s="0" t="inlineStr">
         <is>
@@ -9088,11 +9088,11 @@
     <row r="57">
       <c r="A57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2024:7-10</t>
+          <t xml:space="preserve">actual:project:2023:7-14</t>
         </is>
       </c>
       <c r="B57" s="2">
-        <v>190000</v>
+        <v>2</v>
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
@@ -9103,11 +9103,11 @@
     <row r="58">
       <c r="A58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2024:7-13</t>
+          <t xml:space="preserve">actual:project:2023:7-4</t>
         </is>
       </c>
       <c r="B58" s="2">
-        <v>95</v>
+        <v>2304000</v>
       </c>
       <c r="C58" s="0" t="inlineStr">
         <is>
@@ -9118,11 +9118,11 @@
     <row r="59">
       <c r="A59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2024:7-14</t>
+          <t xml:space="preserve">actual:project:2023:7-6</t>
         </is>
       </c>
       <c r="B59" s="2">
-        <v>2</v>
+        <v>677969</v>
       </c>
       <c r="C59" s="0" t="inlineStr">
         <is>
@@ -9133,11 +9133,11 @@
     <row r="60">
       <c r="A60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2024:7-4</t>
+          <t xml:space="preserve">actual:project:2023:7-8</t>
         </is>
       </c>
       <c r="B60" s="2">
-        <v>2432000</v>
+        <v>519031</v>
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
@@ -9148,11 +9148,11 @@
     <row r="61">
       <c r="A61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2024:7-6</t>
+          <t xml:space="preserve">actual:project:2023:7-9</t>
         </is>
       </c>
       <c r="B61" s="2">
-        <v>704676</v>
+        <v>36000</v>
       </c>
       <c r="C61" s="0" t="inlineStr">
         <is>
@@ -9163,11 +9163,11 @@
     <row r="62">
       <c r="A62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">actual:project:2024:7-8</t>
+          <t xml:space="preserve">actual:project